<commit_message>
Workspace konfiguriert und Pläne aktualisiert
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6438ED1D-8E3D-40BE-96D5-43AB19769829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F447247-391A-4F79-93FA-5EE3BAC58BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
@@ -953,7 +953,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1024,6 +1024,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1133,7 +1139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1221,51 +1227,52 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1584,7 +1591,7 @@
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="62" t="s">
+      <c r="G1" s="59" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="54"/>
@@ -1593,7 +1600,7 @@
       <c r="K1" s="54"/>
       <c r="L1" s="54"/>
       <c r="M1" s="54"/>
-      <c r="N1" s="62" t="s">
+      <c r="N1" s="59" t="s">
         <v>2</v>
       </c>
       <c r="O1" s="54"/>
@@ -1602,7 +1609,7 @@
       <c r="R1" s="54"/>
       <c r="S1" s="54"/>
       <c r="T1" s="54"/>
-      <c r="U1" s="62" t="s">
+      <c r="U1" s="59" t="s">
         <v>3</v>
       </c>
       <c r="V1" s="54"/>
@@ -1611,7 +1618,7 @@
       <c r="Y1" s="54"/>
       <c r="Z1" s="54"/>
       <c r="AA1" s="54"/>
-      <c r="AB1" s="69" t="s">
+      <c r="AB1" s="60" t="s">
         <v>4</v>
       </c>
       <c r="AC1" s="54"/>
@@ -1620,7 +1627,7 @@
       <c r="AF1" s="54"/>
       <c r="AG1" s="54"/>
       <c r="AH1" s="54"/>
-      <c r="AI1" s="62" t="s">
+      <c r="AI1" s="59" t="s">
         <v>5</v>
       </c>
       <c r="AJ1" s="54"/>
@@ -1629,7 +1636,7 @@
       <c r="AM1" s="54"/>
       <c r="AN1" s="54"/>
       <c r="AO1" s="54"/>
-      <c r="AP1" s="62" t="s">
+      <c r="AP1" s="59" t="s">
         <v>6</v>
       </c>
       <c r="AQ1" s="54"/>
@@ -1638,7 +1645,7 @@
       <c r="AT1" s="54"/>
       <c r="AU1" s="54"/>
       <c r="AV1" s="54"/>
-      <c r="AW1" s="62" t="s">
+      <c r="AW1" s="59" t="s">
         <v>7</v>
       </c>
       <c r="AX1" s="54"/>
@@ -1647,7 +1654,7 @@
       <c r="BA1" s="54"/>
       <c r="BB1" s="54"/>
       <c r="BC1" s="54"/>
-      <c r="BD1" s="62" t="s">
+      <c r="BD1" s="59" t="s">
         <v>8</v>
       </c>
       <c r="BE1" s="54"/>
@@ -1656,7 +1663,7 @@
       <c r="BH1" s="54"/>
       <c r="BI1" s="54"/>
       <c r="BJ1" s="54"/>
-      <c r="BK1" s="62" t="s">
+      <c r="BK1" s="59" t="s">
         <v>9</v>
       </c>
       <c r="BL1" s="54"/>
@@ -1665,7 +1672,7 @@
       <c r="BO1" s="54"/>
       <c r="BP1" s="54"/>
       <c r="BQ1" s="54"/>
-      <c r="BR1" s="62" t="s">
+      <c r="BR1" s="59" t="s">
         <v>10</v>
       </c>
       <c r="BS1" s="54"/>
@@ -1674,7 +1681,7 @@
       <c r="BV1" s="54"/>
       <c r="BW1" s="54"/>
       <c r="BX1" s="54"/>
-      <c r="BY1" s="62" t="s">
+      <c r="BY1" s="59" t="s">
         <v>11</v>
       </c>
       <c r="BZ1" s="54"/>
@@ -1683,7 +1690,7 @@
       <c r="CC1" s="54"/>
       <c r="CD1" s="54"/>
       <c r="CE1" s="54"/>
-      <c r="CF1" s="62" t="s">
+      <c r="CF1" s="59" t="s">
         <v>12</v>
       </c>
       <c r="CG1" s="54"/>
@@ -1692,7 +1699,7 @@
       <c r="CJ1" s="54"/>
       <c r="CK1" s="54"/>
       <c r="CL1" s="54"/>
-      <c r="CM1" s="62" t="s">
+      <c r="CM1" s="59" t="s">
         <v>13</v>
       </c>
       <c r="CN1" s="54"/>
@@ -1701,7 +1708,7 @@
       <c r="CQ1" s="54"/>
       <c r="CR1" s="54"/>
       <c r="CS1" s="54"/>
-      <c r="CT1" s="62" t="s">
+      <c r="CT1" s="59" t="s">
         <v>14</v>
       </c>
       <c r="CU1" s="54"/>
@@ -1710,7 +1717,7 @@
       <c r="CX1" s="54"/>
       <c r="CY1" s="54"/>
       <c r="CZ1" s="54"/>
-      <c r="DA1" s="62" t="s">
+      <c r="DA1" s="59" t="s">
         <v>15</v>
       </c>
       <c r="DB1" s="54"/>
@@ -1719,7 +1726,7 @@
       <c r="DE1" s="54"/>
       <c r="DF1" s="54"/>
       <c r="DG1" s="54"/>
-      <c r="DH1" s="62" t="s">
+      <c r="DH1" s="59" t="s">
         <v>16</v>
       </c>
       <c r="DI1" s="54"/>
@@ -1728,7 +1735,7 @@
       <c r="DL1" s="54"/>
       <c r="DM1" s="54"/>
       <c r="DN1" s="54"/>
-      <c r="DO1" s="62" t="s">
+      <c r="DO1" s="59" t="s">
         <v>17</v>
       </c>
       <c r="DP1" s="54"/>
@@ -1737,7 +1744,7 @@
       <c r="DS1" s="54"/>
       <c r="DT1" s="54"/>
       <c r="DU1" s="54"/>
-      <c r="DV1" s="62" t="s">
+      <c r="DV1" s="59" t="s">
         <v>18</v>
       </c>
       <c r="DW1" s="54"/>
@@ -1746,7 +1753,7 @@
       <c r="DZ1" s="54"/>
       <c r="EA1" s="54"/>
       <c r="EB1" s="54"/>
-      <c r="EC1" s="62" t="s">
+      <c r="EC1" s="59" t="s">
         <v>19</v>
       </c>
       <c r="ED1" s="54"/>
@@ -1755,7 +1762,7 @@
       <c r="EG1" s="54"/>
       <c r="EH1" s="54"/>
       <c r="EI1" s="54"/>
-      <c r="EJ1" s="62" t="s">
+      <c r="EJ1" s="59" t="s">
         <v>20</v>
       </c>
       <c r="EK1" s="54"/>
@@ -1764,7 +1771,7 @@
       <c r="EN1" s="54"/>
       <c r="EO1" s="54"/>
       <c r="EP1" s="54"/>
-      <c r="EQ1" s="62" t="s">
+      <c r="EQ1" s="59" t="s">
         <v>21</v>
       </c>
       <c r="ER1" s="54"/>
@@ -1773,7 +1780,7 @@
       <c r="EU1" s="54"/>
       <c r="EV1" s="54"/>
       <c r="EW1" s="54"/>
-      <c r="EX1" s="62" t="s">
+      <c r="EX1" s="59" t="s">
         <v>22</v>
       </c>
       <c r="EY1" s="54"/>
@@ -1782,7 +1789,7 @@
       <c r="FB1" s="54"/>
       <c r="FC1" s="54"/>
       <c r="FD1" s="54"/>
-      <c r="FE1" s="62" t="s">
+      <c r="FE1" s="59" t="s">
         <v>23</v>
       </c>
       <c r="FF1" s="54"/>
@@ -1791,7 +1798,7 @@
       <c r="FI1" s="54"/>
       <c r="FJ1" s="54"/>
       <c r="FK1" s="54"/>
-      <c r="FL1" s="62" t="s">
+      <c r="FL1" s="59" t="s">
         <v>24</v>
       </c>
       <c r="FM1" s="54"/>
@@ -1800,7 +1807,7 @@
       <c r="FP1" s="54"/>
       <c r="FQ1" s="54"/>
       <c r="FR1" s="54"/>
-      <c r="FS1" s="62" t="s">
+      <c r="FS1" s="59" t="s">
         <v>25</v>
       </c>
       <c r="FT1" s="54"/>
@@ -1809,7 +1816,7 @@
       <c r="FW1" s="54"/>
       <c r="FX1" s="54"/>
       <c r="FY1" s="54"/>
-      <c r="FZ1" s="62" t="s">
+      <c r="FZ1" s="59" t="s">
         <v>26</v>
       </c>
       <c r="GA1" s="54"/>
@@ -1818,7 +1825,7 @@
       <c r="GD1" s="54"/>
       <c r="GE1" s="54"/>
       <c r="GF1" s="54"/>
-      <c r="GG1" s="62" t="s">
+      <c r="GG1" s="59" t="s">
         <v>27</v>
       </c>
       <c r="GH1" s="54"/>
@@ -1827,7 +1834,7 @@
       <c r="GK1" s="54"/>
       <c r="GL1" s="54"/>
       <c r="GM1" s="54"/>
-      <c r="GN1" s="62" t="s">
+      <c r="GN1" s="59" t="s">
         <v>28</v>
       </c>
       <c r="GO1" s="54"/>
@@ -1836,7 +1843,7 @@
       <c r="GR1" s="54"/>
       <c r="GS1" s="54"/>
       <c r="GT1" s="54"/>
-      <c r="GU1" s="62" t="s">
+      <c r="GU1" s="59" t="s">
         <v>29</v>
       </c>
       <c r="GV1" s="54"/>
@@ -1845,7 +1852,7 @@
       <c r="GY1" s="54"/>
       <c r="GZ1" s="54"/>
       <c r="HA1" s="54"/>
-      <c r="HB1" s="62" t="s">
+      <c r="HB1" s="59" t="s">
         <v>30</v>
       </c>
       <c r="HC1" s="54"/>
@@ -1854,7 +1861,7 @@
       <c r="HF1" s="54"/>
       <c r="HG1" s="54"/>
       <c r="HH1" s="54"/>
-      <c r="HI1" s="62" t="s">
+      <c r="HI1" s="59" t="s">
         <v>31</v>
       </c>
       <c r="HJ1" s="54"/>
@@ -1863,7 +1870,7 @@
       <c r="HM1" s="54"/>
       <c r="HN1" s="54"/>
       <c r="HO1" s="54"/>
-      <c r="HP1" s="62" t="s">
+      <c r="HP1" s="59" t="s">
         <v>32</v>
       </c>
       <c r="HQ1" s="54"/>
@@ -3438,20 +3445,20 @@
       <c r="HR4" s="7"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="56" t="s">
+      <c r="B5" s="65"/>
+      <c r="C5" s="63" t="s">
         <v>46</v>
       </c>
       <c r="D5" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E5" s="67" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="63"/>
+      <c r="F5" s="61"/>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
       <c r="I5" s="11"/>
@@ -3674,14 +3681,14 @@
       <c r="HR5" s="11"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="57"/>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
       <c r="D6" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="11"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
@@ -3904,18 +3911,18 @@
       <c r="HR6" s="11"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="57"/>
-      <c r="B7" s="64"/>
-      <c r="C7" s="56" t="s">
+      <c r="A7" s="62"/>
+      <c r="B7" s="65"/>
+      <c r="C7" s="63" t="s">
         <v>50</v>
       </c>
       <c r="D7" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="66" t="s">
+      <c r="E7" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="63"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="11"/>
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
@@ -4138,14 +4145,14 @@
       <c r="HR7" s="11"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="57"/>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
+      <c r="A8" s="62"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
       <c r="D8" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
@@ -4368,18 +4375,18 @@
       <c r="HR8" s="11"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="57"/>
-      <c r="B9" s="64"/>
-      <c r="C9" s="56" t="s">
+      <c r="A9" s="62"/>
+      <c r="B9" s="65"/>
+      <c r="C9" s="63" t="s">
         <v>52</v>
       </c>
       <c r="D9" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="66" t="s">
+      <c r="E9" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="63"/>
+      <c r="F9" s="61"/>
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -4602,14 +4609,14 @@
       <c r="HR9" s="11"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="57"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
       <c r="D10" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -4832,18 +4839,18 @@
       <c r="HR10" s="11"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="57"/>
-      <c r="B11" s="64"/>
-      <c r="C11" s="56" t="s">
+      <c r="A11" s="62"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="63" t="s">
         <v>54</v>
       </c>
       <c r="D11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="66" t="s">
+      <c r="E11" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="63"/>
+      <c r="F11" s="61"/>
       <c r="G11" s="11"/>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
@@ -5066,14 +5073,14 @@
       <c r="HR11" s="11"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="57"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
+      <c r="A12" s="62"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
       <c r="D12" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="57"/>
-      <c r="F12" s="57"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
@@ -5296,18 +5303,18 @@
       <c r="HR12" s="11"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="57"/>
-      <c r="B13" s="64"/>
-      <c r="C13" s="56" t="s">
+      <c r="A13" s="62"/>
+      <c r="B13" s="65"/>
+      <c r="C13" s="63" t="s">
         <v>56</v>
       </c>
       <c r="D13" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="66" t="s">
+      <c r="E13" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="63"/>
+      <c r="F13" s="61"/>
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -5530,14 +5537,14 @@
       <c r="HR13" s="11"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="57"/>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
+      <c r="A14" s="62"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
       <c r="D14" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -5760,18 +5767,18 @@
       <c r="HR14" s="11"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="57"/>
-      <c r="B15" s="64"/>
-      <c r="C15" s="56" t="s">
+      <c r="A15" s="62"/>
+      <c r="B15" s="65"/>
+      <c r="C15" s="63" t="s">
         <v>58</v>
       </c>
       <c r="D15" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="66" t="s">
+      <c r="E15" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="63"/>
+      <c r="F15" s="61"/>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -5994,14 +6001,14 @@
       <c r="HR15" s="11"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="57"/>
-      <c r="B16" s="57"/>
-      <c r="C16" s="57"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
       <c r="D16" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
@@ -6224,18 +6231,18 @@
       <c r="HR16" s="11"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="57"/>
-      <c r="B17" s="64"/>
-      <c r="C17" s="56" t="s">
+      <c r="A17" s="62"/>
+      <c r="B17" s="65"/>
+      <c r="C17" s="63" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="66" t="s">
+      <c r="E17" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="63"/>
+      <c r="F17" s="61"/>
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
@@ -6458,14 +6465,14 @@
       <c r="HR17" s="11"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="57"/>
-      <c r="B18" s="57"/>
-      <c r="C18" s="57"/>
+      <c r="A18" s="62"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
       <c r="D18" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="57"/>
-      <c r="F18" s="57"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
@@ -6688,18 +6695,18 @@
       <c r="HR18" s="11"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="57"/>
-      <c r="B19" s="64"/>
-      <c r="C19" s="56" t="s">
+      <c r="A19" s="62"/>
+      <c r="B19" s="65"/>
+      <c r="C19" s="63" t="s">
         <v>62</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="66" t="s">
+      <c r="E19" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="63"/>
+      <c r="F19" s="61"/>
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
@@ -6922,14 +6929,14 @@
       <c r="HR19" s="11"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="57"/>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
+      <c r="A20" s="62"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
       <c r="D20" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="11"/>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
@@ -7152,18 +7159,18 @@
       <c r="HR20" s="11"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="57"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="56" t="s">
+      <c r="A21" s="62"/>
+      <c r="B21" s="65"/>
+      <c r="C21" s="63" t="s">
         <v>64</v>
       </c>
       <c r="D21" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="66" t="s">
+      <c r="E21" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="63"/>
+      <c r="F21" s="61"/>
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
@@ -7386,14 +7393,14 @@
       <c r="HR21" s="11"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="65"/>
-      <c r="B22" s="65"/>
-      <c r="C22" s="65"/>
+      <c r="A22" s="68"/>
+      <c r="B22" s="68"/>
+      <c r="C22" s="68"/>
       <c r="D22" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="65"/>
-      <c r="F22" s="65"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="68"/>
       <c r="G22" s="44"/>
       <c r="H22" s="44"/>
       <c r="I22" s="44"/>
@@ -7616,22 +7623,22 @@
       <c r="HR22" s="44"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="53" t="s">
+      <c r="A23" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="57" t="s">
         <v>68</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="58" t="s">
+      <c r="E23" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="60" t="s">
+      <c r="F23" s="58" t="s">
         <v>70</v>
       </c>
       <c r="G23" s="11"/>
@@ -8087,19 +8094,19 @@
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="54"/>
-      <c r="B25" s="59" t="s">
+      <c r="B25" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="57" t="s">
         <v>72</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="58" t="s">
+      <c r="E25" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="F25" s="60" t="s">
+      <c r="F25" s="58" t="s">
         <v>70</v>
       </c>
       <c r="G25" s="11"/>
@@ -8553,19 +8560,19 @@
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="54"/>
-      <c r="B27" s="59" t="s">
+      <c r="B27" s="55" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="66" t="s">
         <v>75</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E27" s="58" t="s">
+      <c r="E27" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="F27" s="60"/>
+      <c r="F27" s="58"/>
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
@@ -9018,22 +9025,22 @@
       <c r="HR28" s="11"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="53" t="s">
+      <c r="A29" s="64" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="59" t="s">
+      <c r="B29" s="55" t="s">
         <v>78</v>
       </c>
-      <c r="C29" s="55" t="s">
+      <c r="C29" s="57" t="s">
         <v>79</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E29" s="58" t="s">
+      <c r="E29" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="F29" s="60" t="s">
+      <c r="F29" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="11"/>
@@ -9489,19 +9496,19 @@
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="54"/>
-      <c r="B31" s="59" t="s">
+      <c r="B31" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="55" t="s">
+      <c r="C31" s="57" t="s">
         <v>82</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E31" s="58" t="s">
+      <c r="E31" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="F31" s="60" t="s">
+      <c r="F31" s="58" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="11"/>
@@ -9956,19 +9963,19 @@
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="54"/>
-      <c r="B33" s="59" t="s">
+      <c r="B33" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="55" t="s">
+      <c r="C33" s="57" t="s">
         <v>85</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E33" s="58" t="s">
+      <c r="E33" s="56" t="s">
         <v>86</v>
       </c>
-      <c r="F33" s="60" t="s">
+      <c r="F33" s="58" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="11"/>
@@ -10230,7 +10237,7 @@
       <c r="AG34" s="13"/>
       <c r="AH34" s="14"/>
       <c r="AI34" s="11"/>
-      <c r="AJ34" s="11"/>
+      <c r="AJ34" s="70"/>
       <c r="AK34" s="11"/>
       <c r="AL34" s="11"/>
       <c r="AM34" s="12"/>
@@ -10424,19 +10431,19 @@
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="54"/>
-      <c r="B35" s="59" t="s">
+      <c r="B35" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="C35" s="55" t="s">
+      <c r="C35" s="57" t="s">
         <v>88</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="58" t="s">
+      <c r="E35" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="F35" s="60" t="s">
+      <c r="F35" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="11"/>
@@ -10892,19 +10899,19 @@
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="54"/>
-      <c r="B37" s="59" t="s">
+      <c r="B37" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="55" t="s">
+      <c r="C37" s="57" t="s">
         <v>91</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="58" t="s">
+      <c r="E37" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="F37" s="60" t="s">
+      <c r="F37" s="58" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="11"/>
@@ -11360,19 +11367,19 @@
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="54"/>
-      <c r="B39" s="59" t="s">
+      <c r="B39" s="55" t="s">
         <v>93</v>
       </c>
-      <c r="C39" s="55" t="s">
+      <c r="C39" s="57" t="s">
         <v>94</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E39" s="58" t="s">
+      <c r="E39" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="F39" s="60" t="s">
+      <c r="F39" s="58" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="11"/>
@@ -11827,22 +11834,22 @@
       <c r="HR40" s="11"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="53" t="s">
+      <c r="A41" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="B41" s="59" t="s">
+      <c r="B41" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="C41" s="55" t="s">
+      <c r="C41" s="57" t="s">
         <v>98</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E41" s="58" t="s">
+      <c r="E41" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="F41" s="60" t="s">
+      <c r="F41" s="58" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="11"/>
@@ -12298,19 +12305,19 @@
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="54"/>
-      <c r="B43" s="59" t="s">
+      <c r="B43" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="C43" s="55" t="s">
+      <c r="C43" s="57" t="s">
         <v>101</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E43" s="58" t="s">
+      <c r="E43" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="F43" s="60" t="s">
+      <c r="F43" s="58" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="11"/>
@@ -12764,19 +12771,19 @@
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="54"/>
-      <c r="B45" s="59" t="s">
+      <c r="B45" s="55" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="55" t="s">
+      <c r="C45" s="57" t="s">
         <v>104</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E45" s="58" t="s">
+      <c r="E45" s="56" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="60" t="s">
+      <c r="F45" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="11"/>
@@ -13230,22 +13237,22 @@
       <c r="HR46" s="11"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="53" t="s">
+      <c r="A47" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="B47" s="59" t="s">
+      <c r="B47" s="55" t="s">
         <v>107</v>
       </c>
-      <c r="C47" s="55" t="s">
+      <c r="C47" s="57" t="s">
         <v>108</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E47" s="58" t="s">
+      <c r="E47" s="56" t="s">
         <v>109</v>
       </c>
-      <c r="F47" s="60" t="s">
+      <c r="F47" s="58" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="11"/>
@@ -13701,19 +13708,19 @@
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="54"/>
-      <c r="B49" s="59" t="s">
+      <c r="B49" s="55" t="s">
         <v>110</v>
       </c>
-      <c r="C49" s="55" t="s">
+      <c r="C49" s="57" t="s">
         <v>111</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E49" s="58" t="s">
+      <c r="E49" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="F49" s="60" t="s">
+      <c r="F49" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="11"/>
@@ -14168,22 +14175,22 @@
       <c r="HR50" s="11"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53" t="s">
+      <c r="A51" s="64" t="s">
         <v>113</v>
       </c>
-      <c r="B51" s="59" t="s">
+      <c r="B51" s="55" t="s">
         <v>114</v>
       </c>
-      <c r="C51" s="55" t="s">
+      <c r="C51" s="57" t="s">
         <v>115</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E51" s="58" t="s">
+      <c r="E51" s="56" t="s">
         <v>116</v>
       </c>
-      <c r="F51" s="60" t="s">
+      <c r="F51" s="58" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="11"/>
@@ -14639,19 +14646,19 @@
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="54"/>
-      <c r="B53" s="59" t="s">
+      <c r="B53" s="55" t="s">
         <v>117</v>
       </c>
-      <c r="C53" s="55" t="s">
+      <c r="C53" s="57" t="s">
         <v>118</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E53" s="58" t="s">
+      <c r="E53" s="56" t="s">
         <v>119</v>
       </c>
-      <c r="F53" s="60" t="s">
+      <c r="F53" s="58" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="11"/>
@@ -15106,22 +15113,22 @@
       <c r="HR54" s="11"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="53" t="s">
+      <c r="A55" s="64" t="s">
         <v>120</v>
       </c>
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="55" t="s">
         <v>121</v>
       </c>
-      <c r="C55" s="55" t="s">
+      <c r="C55" s="57" t="s">
         <v>122</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E55" s="58" t="s">
+      <c r="E55" s="56" t="s">
         <v>123</v>
       </c>
-      <c r="F55" s="60" t="s">
+      <c r="F55" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="11"/>
@@ -15577,19 +15584,19 @@
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="54"/>
-      <c r="B57" s="59" t="s">
+      <c r="B57" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="C57" s="55" t="s">
+      <c r="C57" s="57" t="s">
         <v>125</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E57" s="58" t="s">
+      <c r="E57" s="56" t="s">
         <v>126</v>
       </c>
-      <c r="F57" s="60" t="s">
+      <c r="F57" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="11"/>
@@ -16045,19 +16052,19 @@
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="54"/>
-      <c r="B59" s="59" t="s">
+      <c r="B59" s="55" t="s">
         <v>127</v>
       </c>
-      <c r="C59" s="55" t="s">
+      <c r="C59" s="57" t="s">
         <v>128</v>
       </c>
       <c r="D59" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E59" s="58" t="s">
+      <c r="E59" s="56" t="s">
         <v>129</v>
       </c>
-      <c r="F59" s="60" t="s">
+      <c r="F59" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="11"/>
@@ -16513,19 +16520,19 @@
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="54"/>
-      <c r="B61" s="59" t="s">
+      <c r="B61" s="55" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="55" t="s">
+      <c r="C61" s="57" t="s">
         <v>131</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="58" t="s">
+      <c r="E61" s="56" t="s">
         <v>132</v>
       </c>
-      <c r="F61" s="60" t="s">
+      <c r="F61" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="11"/>
@@ -16981,19 +16988,19 @@
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="54"/>
-      <c r="B63" s="59" t="s">
+      <c r="B63" s="55" t="s">
         <v>133</v>
       </c>
-      <c r="C63" s="55" t="s">
+      <c r="C63" s="57" t="s">
         <v>134</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E63" s="58" t="s">
+      <c r="E63" s="56" t="s">
         <v>135</v>
       </c>
-      <c r="F63" s="60" t="s">
+      <c r="F63" s="58" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="11"/>
@@ -17449,19 +17456,19 @@
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="54"/>
-      <c r="B65" s="59" t="s">
+      <c r="B65" s="55" t="s">
         <v>136</v>
       </c>
-      <c r="C65" s="55" t="s">
+      <c r="C65" s="57" t="s">
         <v>137</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E65" s="58" t="s">
+      <c r="E65" s="56" t="s">
         <v>138</v>
       </c>
-      <c r="F65" s="60" t="s">
+      <c r="F65" s="58" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="11"/>
@@ -17916,22 +17923,22 @@
       <c r="HR66" s="11"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="53" t="s">
+      <c r="A67" s="64" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="59" t="s">
+      <c r="B67" s="55" t="s">
         <v>140</v>
       </c>
-      <c r="C67" s="55" t="s">
+      <c r="C67" s="57" t="s">
         <v>141</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E67" s="58" t="s">
+      <c r="E67" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="F67" s="60" t="s">
+      <c r="F67" s="58" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="11"/>
@@ -18387,19 +18394,19 @@
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="54"/>
-      <c r="B69" s="59" t="s">
+      <c r="B69" s="55" t="s">
         <v>143</v>
       </c>
-      <c r="C69" s="55" t="s">
+      <c r="C69" s="57" t="s">
         <v>144</v>
       </c>
       <c r="D69" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E69" s="58" t="s">
+      <c r="E69" s="56" t="s">
         <v>145</v>
       </c>
-      <c r="F69" s="60" t="s">
+      <c r="F69" s="58" t="s">
         <v>70</v>
       </c>
       <c r="G69" s="11"/>
@@ -18855,19 +18862,19 @@
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="54"/>
-      <c r="B71" s="59" t="s">
+      <c r="B71" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="C71" s="55" t="s">
+      <c r="C71" s="57" t="s">
         <v>147</v>
       </c>
       <c r="D71" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E71" s="58" t="s">
+      <c r="E71" s="56" t="s">
         <v>148</v>
       </c>
-      <c r="F71" s="60" t="s">
+      <c r="F71" s="58" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="11"/>
@@ -19323,19 +19330,19 @@
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="54"/>
-      <c r="B73" s="59" t="s">
+      <c r="B73" s="55" t="s">
         <v>149</v>
       </c>
-      <c r="C73" s="55" t="s">
+      <c r="C73" s="57" t="s">
         <v>150</v>
       </c>
       <c r="D73" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E73" s="58" t="s">
+      <c r="E73" s="56" t="s">
         <v>151</v>
       </c>
-      <c r="F73" s="60" t="s">
+      <c r="F73" s="58" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="11"/>
@@ -19791,19 +19798,19 @@
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="54"/>
-      <c r="B75" s="59" t="s">
+      <c r="B75" s="55" t="s">
         <v>152</v>
       </c>
-      <c r="C75" s="55" t="s">
+      <c r="C75" s="57" t="s">
         <v>153</v>
       </c>
       <c r="D75" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E75" s="58" t="s">
+      <c r="E75" s="56" t="s">
         <v>154</v>
       </c>
-      <c r="F75" s="60" t="s">
+      <c r="F75" s="58" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="11"/>
@@ -20259,19 +20266,19 @@
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="54"/>
-      <c r="B77" s="59" t="s">
+      <c r="B77" s="55" t="s">
         <v>155</v>
       </c>
-      <c r="C77" s="55" t="s">
+      <c r="C77" s="57" t="s">
         <v>156</v>
       </c>
       <c r="D77" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E77" s="58" t="s">
+      <c r="E77" s="56" t="s">
         <v>157</v>
       </c>
-      <c r="F77" s="60" t="s">
+      <c r="F77" s="58" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="11"/>
@@ -20726,22 +20733,22 @@
       <c r="HR78" s="11"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="53" t="s">
+      <c r="A79" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="B79" s="59" t="s">
+      <c r="B79" s="55" t="s">
         <v>159</v>
       </c>
-      <c r="C79" s="61" t="s">
+      <c r="C79" s="53" t="s">
         <v>160</v>
       </c>
       <c r="D79" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E79" s="58" t="s">
+      <c r="E79" s="56" t="s">
         <v>161</v>
       </c>
-      <c r="F79" s="60" t="s">
+      <c r="F79" s="58" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="11"/>
@@ -21197,19 +21204,19 @@
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="54"/>
-      <c r="B81" s="59" t="s">
+      <c r="B81" s="55" t="s">
         <v>162</v>
       </c>
-      <c r="C81" s="61" t="s">
+      <c r="C81" s="53" t="s">
         <v>163</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E81" s="58" t="s">
+      <c r="E81" s="56" t="s">
         <v>164</v>
       </c>
-      <c r="F81" s="60" t="s">
+      <c r="F81" s="58" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="11"/>
@@ -21665,19 +21672,19 @@
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="54"/>
-      <c r="B83" s="59" t="s">
+      <c r="B83" s="55" t="s">
         <v>165</v>
       </c>
-      <c r="C83" s="55" t="s">
+      <c r="C83" s="57" t="s">
         <v>166</v>
       </c>
       <c r="D83" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E83" s="58" t="s">
+      <c r="E83" s="56" t="s">
         <v>167</v>
       </c>
-      <c r="F83" s="60" t="s">
+      <c r="F83" s="58" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="11"/>
@@ -22133,19 +22140,19 @@
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="54"/>
-      <c r="B85" s="59" t="s">
+      <c r="B85" s="55" t="s">
         <v>168</v>
       </c>
-      <c r="C85" s="67" t="s">
+      <c r="C85" s="66" t="s">
         <v>169</v>
       </c>
       <c r="D85" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E85" s="58" t="s">
+      <c r="E85" s="56" t="s">
         <v>170</v>
       </c>
-      <c r="F85" s="60"/>
+      <c r="F85" s="58"/>
       <c r="G85" s="11"/>
       <c r="H85" s="11"/>
       <c r="I85" s="11"/>
@@ -22599,6 +22606,187 @@
     </row>
   </sheetData>
   <mergeCells count="205">
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
     <mergeCell ref="C79:C80"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="E79:E80"/>
@@ -22623,187 +22811,6 @@
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="AP1:AV1"/>
     <mergeCell ref="E59:E60"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="B65:B66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added workspace file and further notes for methodology
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F447247-391A-4F79-93FA-5EE3BAC58BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD3D7FB-2299-468F-B1F8-07BD8610318F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1227,6 +1227,7 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1272,7 +1273,6 @@
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1591,290 +1591,290 @@
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="59" t="s">
+      <c r="G1" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="59" t="s">
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="54"/>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="59" t="s">
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="54"/>
-      <c r="W1" s="54"/>
-      <c r="X1" s="54"/>
-      <c r="Y1" s="54"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="60" t="s">
+      <c r="V1" s="55"/>
+      <c r="W1" s="55"/>
+      <c r="X1" s="55"/>
+      <c r="Y1" s="55"/>
+      <c r="Z1" s="55"/>
+      <c r="AA1" s="55"/>
+      <c r="AB1" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="54"/>
-      <c r="AD1" s="54"/>
-      <c r="AE1" s="54"/>
-      <c r="AF1" s="54"/>
-      <c r="AG1" s="54"/>
-      <c r="AH1" s="54"/>
-      <c r="AI1" s="59" t="s">
+      <c r="AC1" s="55"/>
+      <c r="AD1" s="55"/>
+      <c r="AE1" s="55"/>
+      <c r="AF1" s="55"/>
+      <c r="AG1" s="55"/>
+      <c r="AH1" s="55"/>
+      <c r="AI1" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="54"/>
-      <c r="AK1" s="54"/>
-      <c r="AL1" s="54"/>
-      <c r="AM1" s="54"/>
-      <c r="AN1" s="54"/>
-      <c r="AO1" s="54"/>
-      <c r="AP1" s="59" t="s">
+      <c r="AJ1" s="55"/>
+      <c r="AK1" s="55"/>
+      <c r="AL1" s="55"/>
+      <c r="AM1" s="55"/>
+      <c r="AN1" s="55"/>
+      <c r="AO1" s="55"/>
+      <c r="AP1" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="54"/>
-      <c r="AR1" s="54"/>
-      <c r="AS1" s="54"/>
-      <c r="AT1" s="54"/>
-      <c r="AU1" s="54"/>
-      <c r="AV1" s="54"/>
-      <c r="AW1" s="59" t="s">
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="55"/>
+      <c r="AS1" s="55"/>
+      <c r="AT1" s="55"/>
+      <c r="AU1" s="55"/>
+      <c r="AV1" s="55"/>
+      <c r="AW1" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="54"/>
-      <c r="AY1" s="54"/>
-      <c r="AZ1" s="54"/>
-      <c r="BA1" s="54"/>
-      <c r="BB1" s="54"/>
-      <c r="BC1" s="54"/>
-      <c r="BD1" s="59" t="s">
+      <c r="AX1" s="55"/>
+      <c r="AY1" s="55"/>
+      <c r="AZ1" s="55"/>
+      <c r="BA1" s="55"/>
+      <c r="BB1" s="55"/>
+      <c r="BC1" s="55"/>
+      <c r="BD1" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="54"/>
-      <c r="BF1" s="54"/>
-      <c r="BG1" s="54"/>
-      <c r="BH1" s="54"/>
-      <c r="BI1" s="54"/>
-      <c r="BJ1" s="54"/>
-      <c r="BK1" s="59" t="s">
+      <c r="BE1" s="55"/>
+      <c r="BF1" s="55"/>
+      <c r="BG1" s="55"/>
+      <c r="BH1" s="55"/>
+      <c r="BI1" s="55"/>
+      <c r="BJ1" s="55"/>
+      <c r="BK1" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="54"/>
-      <c r="BM1" s="54"/>
-      <c r="BN1" s="54"/>
-      <c r="BO1" s="54"/>
-      <c r="BP1" s="54"/>
-      <c r="BQ1" s="54"/>
-      <c r="BR1" s="59" t="s">
+      <c r="BL1" s="55"/>
+      <c r="BM1" s="55"/>
+      <c r="BN1" s="55"/>
+      <c r="BO1" s="55"/>
+      <c r="BP1" s="55"/>
+      <c r="BQ1" s="55"/>
+      <c r="BR1" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="54"/>
-      <c r="BT1" s="54"/>
-      <c r="BU1" s="54"/>
-      <c r="BV1" s="54"/>
-      <c r="BW1" s="54"/>
-      <c r="BX1" s="54"/>
-      <c r="BY1" s="59" t="s">
+      <c r="BS1" s="55"/>
+      <c r="BT1" s="55"/>
+      <c r="BU1" s="55"/>
+      <c r="BV1" s="55"/>
+      <c r="BW1" s="55"/>
+      <c r="BX1" s="55"/>
+      <c r="BY1" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="54"/>
-      <c r="CA1" s="54"/>
-      <c r="CB1" s="54"/>
-      <c r="CC1" s="54"/>
-      <c r="CD1" s="54"/>
-      <c r="CE1" s="54"/>
-      <c r="CF1" s="59" t="s">
+      <c r="BZ1" s="55"/>
+      <c r="CA1" s="55"/>
+      <c r="CB1" s="55"/>
+      <c r="CC1" s="55"/>
+      <c r="CD1" s="55"/>
+      <c r="CE1" s="55"/>
+      <c r="CF1" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="54"/>
-      <c r="CH1" s="54"/>
-      <c r="CI1" s="54"/>
-      <c r="CJ1" s="54"/>
-      <c r="CK1" s="54"/>
-      <c r="CL1" s="54"/>
-      <c r="CM1" s="59" t="s">
+      <c r="CG1" s="55"/>
+      <c r="CH1" s="55"/>
+      <c r="CI1" s="55"/>
+      <c r="CJ1" s="55"/>
+      <c r="CK1" s="55"/>
+      <c r="CL1" s="55"/>
+      <c r="CM1" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="54"/>
-      <c r="CO1" s="54"/>
-      <c r="CP1" s="54"/>
-      <c r="CQ1" s="54"/>
-      <c r="CR1" s="54"/>
-      <c r="CS1" s="54"/>
-      <c r="CT1" s="59" t="s">
+      <c r="CN1" s="55"/>
+      <c r="CO1" s="55"/>
+      <c r="CP1" s="55"/>
+      <c r="CQ1" s="55"/>
+      <c r="CR1" s="55"/>
+      <c r="CS1" s="55"/>
+      <c r="CT1" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="54"/>
-      <c r="CV1" s="54"/>
-      <c r="CW1" s="54"/>
-      <c r="CX1" s="54"/>
-      <c r="CY1" s="54"/>
-      <c r="CZ1" s="54"/>
-      <c r="DA1" s="59" t="s">
+      <c r="CU1" s="55"/>
+      <c r="CV1" s="55"/>
+      <c r="CW1" s="55"/>
+      <c r="CX1" s="55"/>
+      <c r="CY1" s="55"/>
+      <c r="CZ1" s="55"/>
+      <c r="DA1" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="54"/>
-      <c r="DC1" s="54"/>
-      <c r="DD1" s="54"/>
-      <c r="DE1" s="54"/>
-      <c r="DF1" s="54"/>
-      <c r="DG1" s="54"/>
-      <c r="DH1" s="59" t="s">
+      <c r="DB1" s="55"/>
+      <c r="DC1" s="55"/>
+      <c r="DD1" s="55"/>
+      <c r="DE1" s="55"/>
+      <c r="DF1" s="55"/>
+      <c r="DG1" s="55"/>
+      <c r="DH1" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="54"/>
-      <c r="DJ1" s="54"/>
-      <c r="DK1" s="54"/>
-      <c r="DL1" s="54"/>
-      <c r="DM1" s="54"/>
-      <c r="DN1" s="54"/>
-      <c r="DO1" s="59" t="s">
+      <c r="DI1" s="55"/>
+      <c r="DJ1" s="55"/>
+      <c r="DK1" s="55"/>
+      <c r="DL1" s="55"/>
+      <c r="DM1" s="55"/>
+      <c r="DN1" s="55"/>
+      <c r="DO1" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="54"/>
-      <c r="DQ1" s="54"/>
-      <c r="DR1" s="54"/>
-      <c r="DS1" s="54"/>
-      <c r="DT1" s="54"/>
-      <c r="DU1" s="54"/>
-      <c r="DV1" s="59" t="s">
+      <c r="DP1" s="55"/>
+      <c r="DQ1" s="55"/>
+      <c r="DR1" s="55"/>
+      <c r="DS1" s="55"/>
+      <c r="DT1" s="55"/>
+      <c r="DU1" s="55"/>
+      <c r="DV1" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="54"/>
-      <c r="DX1" s="54"/>
-      <c r="DY1" s="54"/>
-      <c r="DZ1" s="54"/>
-      <c r="EA1" s="54"/>
-      <c r="EB1" s="54"/>
-      <c r="EC1" s="59" t="s">
+      <c r="DW1" s="55"/>
+      <c r="DX1" s="55"/>
+      <c r="DY1" s="55"/>
+      <c r="DZ1" s="55"/>
+      <c r="EA1" s="55"/>
+      <c r="EB1" s="55"/>
+      <c r="EC1" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="54"/>
-      <c r="EE1" s="54"/>
-      <c r="EF1" s="54"/>
-      <c r="EG1" s="54"/>
-      <c r="EH1" s="54"/>
-      <c r="EI1" s="54"/>
-      <c r="EJ1" s="59" t="s">
+      <c r="ED1" s="55"/>
+      <c r="EE1" s="55"/>
+      <c r="EF1" s="55"/>
+      <c r="EG1" s="55"/>
+      <c r="EH1" s="55"/>
+      <c r="EI1" s="55"/>
+      <c r="EJ1" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="54"/>
-      <c r="EL1" s="54"/>
-      <c r="EM1" s="54"/>
-      <c r="EN1" s="54"/>
-      <c r="EO1" s="54"/>
-      <c r="EP1" s="54"/>
-      <c r="EQ1" s="59" t="s">
+      <c r="EK1" s="55"/>
+      <c r="EL1" s="55"/>
+      <c r="EM1" s="55"/>
+      <c r="EN1" s="55"/>
+      <c r="EO1" s="55"/>
+      <c r="EP1" s="55"/>
+      <c r="EQ1" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="54"/>
-      <c r="ES1" s="54"/>
-      <c r="ET1" s="54"/>
-      <c r="EU1" s="54"/>
-      <c r="EV1" s="54"/>
-      <c r="EW1" s="54"/>
-      <c r="EX1" s="59" t="s">
+      <c r="ER1" s="55"/>
+      <c r="ES1" s="55"/>
+      <c r="ET1" s="55"/>
+      <c r="EU1" s="55"/>
+      <c r="EV1" s="55"/>
+      <c r="EW1" s="55"/>
+      <c r="EX1" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="54"/>
-      <c r="EZ1" s="54"/>
-      <c r="FA1" s="54"/>
-      <c r="FB1" s="54"/>
-      <c r="FC1" s="54"/>
-      <c r="FD1" s="54"/>
-      <c r="FE1" s="59" t="s">
+      <c r="EY1" s="55"/>
+      <c r="EZ1" s="55"/>
+      <c r="FA1" s="55"/>
+      <c r="FB1" s="55"/>
+      <c r="FC1" s="55"/>
+      <c r="FD1" s="55"/>
+      <c r="FE1" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="54"/>
-      <c r="FG1" s="54"/>
-      <c r="FH1" s="54"/>
-      <c r="FI1" s="54"/>
-      <c r="FJ1" s="54"/>
-      <c r="FK1" s="54"/>
-      <c r="FL1" s="59" t="s">
+      <c r="FF1" s="55"/>
+      <c r="FG1" s="55"/>
+      <c r="FH1" s="55"/>
+      <c r="FI1" s="55"/>
+      <c r="FJ1" s="55"/>
+      <c r="FK1" s="55"/>
+      <c r="FL1" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="54"/>
-      <c r="FN1" s="54"/>
-      <c r="FO1" s="54"/>
-      <c r="FP1" s="54"/>
-      <c r="FQ1" s="54"/>
-      <c r="FR1" s="54"/>
-      <c r="FS1" s="59" t="s">
+      <c r="FM1" s="55"/>
+      <c r="FN1" s="55"/>
+      <c r="FO1" s="55"/>
+      <c r="FP1" s="55"/>
+      <c r="FQ1" s="55"/>
+      <c r="FR1" s="55"/>
+      <c r="FS1" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="54"/>
-      <c r="FU1" s="54"/>
-      <c r="FV1" s="54"/>
-      <c r="FW1" s="54"/>
-      <c r="FX1" s="54"/>
-      <c r="FY1" s="54"/>
-      <c r="FZ1" s="59" t="s">
+      <c r="FT1" s="55"/>
+      <c r="FU1" s="55"/>
+      <c r="FV1" s="55"/>
+      <c r="FW1" s="55"/>
+      <c r="FX1" s="55"/>
+      <c r="FY1" s="55"/>
+      <c r="FZ1" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="54"/>
-      <c r="GB1" s="54"/>
-      <c r="GC1" s="54"/>
-      <c r="GD1" s="54"/>
-      <c r="GE1" s="54"/>
-      <c r="GF1" s="54"/>
-      <c r="GG1" s="59" t="s">
+      <c r="GA1" s="55"/>
+      <c r="GB1" s="55"/>
+      <c r="GC1" s="55"/>
+      <c r="GD1" s="55"/>
+      <c r="GE1" s="55"/>
+      <c r="GF1" s="55"/>
+      <c r="GG1" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="54"/>
-      <c r="GI1" s="54"/>
-      <c r="GJ1" s="54"/>
-      <c r="GK1" s="54"/>
-      <c r="GL1" s="54"/>
-      <c r="GM1" s="54"/>
-      <c r="GN1" s="59" t="s">
+      <c r="GH1" s="55"/>
+      <c r="GI1" s="55"/>
+      <c r="GJ1" s="55"/>
+      <c r="GK1" s="55"/>
+      <c r="GL1" s="55"/>
+      <c r="GM1" s="55"/>
+      <c r="GN1" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="54"/>
-      <c r="GP1" s="54"/>
-      <c r="GQ1" s="54"/>
-      <c r="GR1" s="54"/>
-      <c r="GS1" s="54"/>
-      <c r="GT1" s="54"/>
-      <c r="GU1" s="59" t="s">
+      <c r="GO1" s="55"/>
+      <c r="GP1" s="55"/>
+      <c r="GQ1" s="55"/>
+      <c r="GR1" s="55"/>
+      <c r="GS1" s="55"/>
+      <c r="GT1" s="55"/>
+      <c r="GU1" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="54"/>
-      <c r="GW1" s="54"/>
-      <c r="GX1" s="54"/>
-      <c r="GY1" s="54"/>
-      <c r="GZ1" s="54"/>
-      <c r="HA1" s="54"/>
-      <c r="HB1" s="59" t="s">
+      <c r="GV1" s="55"/>
+      <c r="GW1" s="55"/>
+      <c r="GX1" s="55"/>
+      <c r="GY1" s="55"/>
+      <c r="GZ1" s="55"/>
+      <c r="HA1" s="55"/>
+      <c r="HB1" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="54"/>
-      <c r="HD1" s="54"/>
-      <c r="HE1" s="54"/>
-      <c r="HF1" s="54"/>
-      <c r="HG1" s="54"/>
-      <c r="HH1" s="54"/>
-      <c r="HI1" s="59" t="s">
+      <c r="HC1" s="55"/>
+      <c r="HD1" s="55"/>
+      <c r="HE1" s="55"/>
+      <c r="HF1" s="55"/>
+      <c r="HG1" s="55"/>
+      <c r="HH1" s="55"/>
+      <c r="HI1" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="54"/>
-      <c r="HK1" s="54"/>
-      <c r="HL1" s="54"/>
-      <c r="HM1" s="54"/>
-      <c r="HN1" s="54"/>
-      <c r="HO1" s="54"/>
-      <c r="HP1" s="59" t="s">
+      <c r="HJ1" s="55"/>
+      <c r="HK1" s="55"/>
+      <c r="HL1" s="55"/>
+      <c r="HM1" s="55"/>
+      <c r="HN1" s="55"/>
+      <c r="HO1" s="55"/>
+      <c r="HP1" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="54"/>
-      <c r="HR1" s="54"/>
+      <c r="HQ1" s="55"/>
+      <c r="HR1" s="55"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="1" t="s">
@@ -3445,20 +3445,20 @@
       <c r="HR4" s="7"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="70" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="63" t="s">
+      <c r="B5" s="66"/>
+      <c r="C5" s="64" t="s">
         <v>46</v>
       </c>
       <c r="D5" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="67" t="s">
+      <c r="E5" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="61"/>
+      <c r="F5" s="62"/>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
       <c r="I5" s="11"/>
@@ -3681,14 +3681,14 @@
       <c r="HR5" s="11"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="62"/>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
+      <c r="A6" s="63"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
       <c r="D6" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
       <c r="G6" s="11"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
@@ -3911,18 +3911,18 @@
       <c r="HR6" s="11"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="62"/>
-      <c r="B7" s="65"/>
-      <c r="C7" s="63" t="s">
+      <c r="A7" s="63"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="64" t="s">
         <v>50</v>
       </c>
       <c r="D7" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="67" t="s">
+      <c r="E7" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="61"/>
+      <c r="F7" s="62"/>
       <c r="G7" s="11"/>
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
@@ -4145,14 +4145,14 @@
       <c r="HR7" s="11"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="62"/>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
+      <c r="A8" s="63"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
       <c r="D8" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
@@ -4375,18 +4375,18 @@
       <c r="HR8" s="11"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="62"/>
-      <c r="B9" s="65"/>
-      <c r="C9" s="63" t="s">
+      <c r="A9" s="63"/>
+      <c r="B9" s="66"/>
+      <c r="C9" s="64" t="s">
         <v>52</v>
       </c>
       <c r="D9" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="67" t="s">
+      <c r="E9" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="61"/>
+      <c r="F9" s="62"/>
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -4609,14 +4609,14 @@
       <c r="HR9" s="11"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
+      <c r="A10" s="63"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="63"/>
       <c r="D10" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -4839,18 +4839,18 @@
       <c r="HR10" s="11"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="62"/>
-      <c r="B11" s="65"/>
-      <c r="C11" s="63" t="s">
+      <c r="A11" s="63"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="64" t="s">
         <v>54</v>
       </c>
       <c r="D11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="67" t="s">
+      <c r="E11" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="61"/>
+      <c r="F11" s="62"/>
       <c r="G11" s="11"/>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
@@ -5073,14 +5073,14 @@
       <c r="HR11" s="11"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="62"/>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
+      <c r="A12" s="63"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
       <c r="D12" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
@@ -5303,18 +5303,18 @@
       <c r="HR12" s="11"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="63" t="s">
+      <c r="A13" s="63"/>
+      <c r="B13" s="66"/>
+      <c r="C13" s="64" t="s">
         <v>56</v>
       </c>
       <c r="D13" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="67" t="s">
+      <c r="E13" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="61"/>
+      <c r="F13" s="62"/>
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -5537,14 +5537,14 @@
       <c r="HR13" s="11"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="62"/>
-      <c r="B14" s="62"/>
-      <c r="C14" s="62"/>
+      <c r="A14" s="63"/>
+      <c r="B14" s="63"/>
+      <c r="C14" s="63"/>
       <c r="D14" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
+      <c r="E14" s="63"/>
+      <c r="F14" s="63"/>
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -5767,18 +5767,18 @@
       <c r="HR14" s="11"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="62"/>
-      <c r="B15" s="65"/>
-      <c r="C15" s="63" t="s">
+      <c r="A15" s="63"/>
+      <c r="B15" s="66"/>
+      <c r="C15" s="64" t="s">
         <v>58</v>
       </c>
       <c r="D15" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="67" t="s">
+      <c r="E15" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="61"/>
+      <c r="F15" s="62"/>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -6001,14 +6001,14 @@
       <c r="HR15" s="11"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="62"/>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
+      <c r="A16" s="63"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="63"/>
       <c r="D16" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="63"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
@@ -6231,18 +6231,18 @@
       <c r="HR16" s="11"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="62"/>
-      <c r="B17" s="65"/>
-      <c r="C17" s="63" t="s">
+      <c r="A17" s="63"/>
+      <c r="B17" s="66"/>
+      <c r="C17" s="64" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="67" t="s">
+      <c r="E17" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="61"/>
+      <c r="F17" s="62"/>
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
@@ -6465,14 +6465,14 @@
       <c r="HR17" s="11"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="62"/>
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
+      <c r="A18" s="63"/>
+      <c r="B18" s="63"/>
+      <c r="C18" s="63"/>
       <c r="D18" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
@@ -6695,18 +6695,18 @@
       <c r="HR18" s="11"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="62"/>
-      <c r="B19" s="65"/>
-      <c r="C19" s="63" t="s">
+      <c r="A19" s="63"/>
+      <c r="B19" s="66"/>
+      <c r="C19" s="64" t="s">
         <v>62</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="67" t="s">
+      <c r="E19" s="68" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="61"/>
+      <c r="F19" s="62"/>
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
@@ -6929,14 +6929,14 @@
       <c r="HR19" s="11"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="62"/>
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
+      <c r="A20" s="63"/>
+      <c r="B20" s="63"/>
+      <c r="C20" s="63"/>
       <c r="D20" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
       <c r="G20" s="11"/>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
@@ -7159,18 +7159,18 @@
       <c r="HR20" s="11"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="62"/>
-      <c r="B21" s="65"/>
-      <c r="C21" s="63" t="s">
+      <c r="A21" s="63"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="64" t="s">
         <v>64</v>
       </c>
       <c r="D21" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="67" t="s">
+      <c r="E21" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="61"/>
+      <c r="F21" s="62"/>
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
@@ -7393,14 +7393,14 @@
       <c r="HR21" s="11"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="68"/>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
+      <c r="A22" s="69"/>
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
       <c r="D22" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
+      <c r="E22" s="69"/>
+      <c r="F22" s="69"/>
       <c r="G22" s="44"/>
       <c r="H22" s="44"/>
       <c r="I22" s="44"/>
@@ -7623,22 +7623,22 @@
       <c r="HR22" s="44"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="64" t="s">
+      <c r="A23" s="65" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="57" t="s">
+      <c r="C23" s="58" t="s">
         <v>68</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="56" t="s">
+      <c r="E23" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="58" t="s">
+      <c r="F23" s="59" t="s">
         <v>70</v>
       </c>
       <c r="G23" s="11"/>
@@ -7863,14 +7863,14 @@
       <c r="HR23" s="11"/>
     </row>
     <row r="24" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="54"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="54"/>
+      <c r="A24" s="55"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
       <c r="D24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
       <c r="G24" s="11"/>
       <c r="H24" s="11"/>
       <c r="I24" s="11"/>
@@ -8093,20 +8093,20 @@
       <c r="HR24" s="11"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="54"/>
-      <c r="B25" s="55" t="s">
+      <c r="A25" s="55"/>
+      <c r="B25" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="C25" s="57" t="s">
+      <c r="C25" s="58" t="s">
         <v>72</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="56" t="s">
+      <c r="E25" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="F25" s="58" t="s">
+      <c r="F25" s="59" t="s">
         <v>70</v>
       </c>
       <c r="G25" s="11"/>
@@ -8329,14 +8329,14 @@
       <c r="HS25" s="11"/>
     </row>
     <row r="26" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="54"/>
-      <c r="B26" s="54"/>
-      <c r="C26" s="54"/>
+      <c r="A26" s="55"/>
+      <c r="B26" s="55"/>
+      <c r="C26" s="55"/>
       <c r="D26" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="55"/>
       <c r="G26" s="11"/>
       <c r="H26" s="11"/>
       <c r="I26" s="11"/>
@@ -8373,7 +8373,7 @@
       <c r="AN26" s="13"/>
       <c r="AO26" s="14"/>
       <c r="AP26" s="11"/>
-      <c r="AQ26" s="11"/>
+      <c r="AQ26" s="52"/>
       <c r="AR26" s="11"/>
       <c r="AS26" s="11"/>
       <c r="AT26" s="12"/>
@@ -8559,20 +8559,20 @@
       <c r="HR26" s="11"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="54"/>
-      <c r="B27" s="55" t="s">
+      <c r="A27" s="55"/>
+      <c r="B27" s="56" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="66" t="s">
+      <c r="C27" s="67" t="s">
         <v>75</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E27" s="56" t="s">
+      <c r="E27" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="F27" s="58"/>
+      <c r="F27" s="59"/>
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
@@ -8795,14 +8795,14 @@
       <c r="HR27" s="11"/>
     </row>
     <row r="28" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="54"/>
-      <c r="B28" s="54"/>
-      <c r="C28" s="54"/>
+      <c r="A28" s="55"/>
+      <c r="B28" s="55"/>
+      <c r="C28" s="55"/>
       <c r="D28" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
       <c r="G28" s="11"/>
       <c r="H28" s="11"/>
       <c r="I28" s="11"/>
@@ -8834,7 +8834,6 @@
       <c r="AI28" s="11"/>
       <c r="AJ28" s="11"/>
       <c r="AK28" s="11"/>
-      <c r="AL28" s="11"/>
       <c r="AM28" s="12"/>
       <c r="AN28" s="13"/>
       <c r="AO28" s="14"/>
@@ -9025,22 +9024,22 @@
       <c r="HR28" s="11"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="64" t="s">
+      <c r="A29" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="55" t="s">
+      <c r="B29" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C29" s="57" t="s">
+      <c r="C29" s="58" t="s">
         <v>79</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E29" s="56" t="s">
+      <c r="E29" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="F29" s="58" t="s">
+      <c r="F29" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="11"/>
@@ -9074,7 +9073,6 @@
       <c r="AI29" s="11"/>
       <c r="AJ29" s="22"/>
       <c r="AK29" s="11"/>
-      <c r="AL29" s="11"/>
       <c r="AM29" s="12"/>
       <c r="AN29" s="13"/>
       <c r="AO29" s="14"/>
@@ -9265,14 +9263,14 @@
       <c r="HR29" s="11"/>
     </row>
     <row r="30" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="54"/>
-      <c r="B30" s="54"/>
-      <c r="C30" s="54"/>
+      <c r="A30" s="55"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
       <c r="D30" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="54"/>
-      <c r="F30" s="54"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
@@ -9304,7 +9302,7 @@
       <c r="AI30" s="11"/>
       <c r="AJ30" s="11"/>
       <c r="AK30" s="11"/>
-      <c r="AL30" s="11"/>
+      <c r="AL30" s="52"/>
       <c r="AM30" s="12"/>
       <c r="AN30" s="13"/>
       <c r="AO30" s="14"/>
@@ -9495,20 +9493,20 @@
       <c r="HR30" s="11"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="54"/>
-      <c r="B31" s="55" t="s">
+      <c r="A31" s="55"/>
+      <c r="B31" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="57" t="s">
+      <c r="C31" s="58" t="s">
         <v>82</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E31" s="56" t="s">
+      <c r="E31" s="57" t="s">
         <v>83</v>
       </c>
-      <c r="F31" s="58" t="s">
+      <c r="F31" s="59" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="11"/>
@@ -9542,6 +9540,7 @@
       <c r="AI31" s="11"/>
       <c r="AJ31" s="11"/>
       <c r="AK31" s="22"/>
+      <c r="AL31" s="11"/>
       <c r="AM31" s="12"/>
       <c r="AN31" s="13"/>
       <c r="AO31" s="14"/>
@@ -9732,14 +9731,14 @@
       <c r="HR31" s="11"/>
     </row>
     <row r="32" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="54"/>
-      <c r="B32" s="54"/>
-      <c r="C32" s="54"/>
+      <c r="A32" s="55"/>
+      <c r="B32" s="55"/>
+      <c r="C32" s="55"/>
       <c r="D32" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E32" s="54"/>
-      <c r="F32" s="54"/>
+      <c r="E32" s="55"/>
+      <c r="F32" s="55"/>
       <c r="G32" s="11"/>
       <c r="H32" s="11"/>
       <c r="I32" s="11"/>
@@ -9771,9 +9770,8 @@
       <c r="AI32" s="11"/>
       <c r="AJ32" s="11"/>
       <c r="AK32" s="11"/>
-      <c r="AL32" s="11"/>
       <c r="AM32" s="12"/>
-      <c r="AN32" s="13"/>
+      <c r="AN32" s="52"/>
       <c r="AO32" s="14"/>
       <c r="AP32" s="11"/>
       <c r="AQ32" s="11"/>
@@ -9962,20 +9960,20 @@
       <c r="HR32" s="11"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="54"/>
-      <c r="B33" s="55" t="s">
+      <c r="A33" s="55"/>
+      <c r="B33" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="57" t="s">
+      <c r="C33" s="58" t="s">
         <v>85</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E33" s="56" t="s">
+      <c r="E33" s="57" t="s">
         <v>86</v>
       </c>
-      <c r="F33" s="58" t="s">
+      <c r="F33" s="59" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="11"/>
@@ -10200,14 +10198,14 @@
       <c r="HR33" s="11"/>
     </row>
     <row r="34" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="54"/>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
+      <c r="A34" s="55"/>
+      <c r="B34" s="55"/>
+      <c r="C34" s="55"/>
       <c r="D34" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
+      <c r="E34" s="55"/>
+      <c r="F34" s="55"/>
       <c r="G34" s="11"/>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
@@ -10237,12 +10235,12 @@
       <c r="AG34" s="13"/>
       <c r="AH34" s="14"/>
       <c r="AI34" s="11"/>
-      <c r="AJ34" s="70"/>
-      <c r="AK34" s="11"/>
+      <c r="AJ34" s="53"/>
+      <c r="AK34" s="53"/>
       <c r="AL34" s="11"/>
       <c r="AM34" s="12"/>
-      <c r="AN34" s="13"/>
-      <c r="AO34" s="14"/>
+      <c r="AN34" s="53"/>
+      <c r="AO34" s="53"/>
       <c r="AP34" s="11"/>
       <c r="AQ34" s="11"/>
       <c r="AR34" s="11"/>
@@ -10430,20 +10428,20 @@
       <c r="HR34" s="11"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="54"/>
-      <c r="B35" s="55" t="s">
+      <c r="A35" s="55"/>
+      <c r="B35" s="56" t="s">
         <v>87</v>
       </c>
-      <c r="C35" s="57" t="s">
+      <c r="C35" s="58" t="s">
         <v>88</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E35" s="56" t="s">
+      <c r="E35" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="F35" s="58" t="s">
+      <c r="F35" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="11"/>
@@ -10668,14 +10666,14 @@
       <c r="HR35" s="11"/>
     </row>
     <row r="36" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="54"/>
-      <c r="B36" s="54"/>
-      <c r="C36" s="54"/>
+      <c r="A36" s="55"/>
+      <c r="B36" s="55"/>
+      <c r="C36" s="55"/>
       <c r="D36" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
       <c r="G36" s="11"/>
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
@@ -10898,20 +10896,20 @@
       <c r="HR36" s="11"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="54"/>
-      <c r="B37" s="55" t="s">
+      <c r="A37" s="55"/>
+      <c r="B37" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="57" t="s">
+      <c r="C37" s="58" t="s">
         <v>91</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="56" t="s">
+      <c r="E37" s="57" t="s">
         <v>92</v>
       </c>
-      <c r="F37" s="58" t="s">
+      <c r="F37" s="59" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="11"/>
@@ -11136,14 +11134,14 @@
       <c r="HR37" s="11"/>
     </row>
     <row r="38" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="54"/>
-      <c r="B38" s="54"/>
-      <c r="C38" s="54"/>
+      <c r="A38" s="55"/>
+      <c r="B38" s="55"/>
+      <c r="C38" s="55"/>
       <c r="D38" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
+      <c r="E38" s="55"/>
+      <c r="F38" s="55"/>
       <c r="G38" s="11"/>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
@@ -11366,20 +11364,20 @@
       <c r="HR38" s="11"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="54"/>
-      <c r="B39" s="55" t="s">
+      <c r="A39" s="55"/>
+      <c r="B39" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="C39" s="57" t="s">
+      <c r="C39" s="58" t="s">
         <v>94</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E39" s="56" t="s">
+      <c r="E39" s="57" t="s">
         <v>95</v>
       </c>
-      <c r="F39" s="58" t="s">
+      <c r="F39" s="59" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="11"/>
@@ -11604,14 +11602,14 @@
       <c r="HR39" s="11"/>
     </row>
     <row r="40" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="54"/>
-      <c r="B40" s="54"/>
-      <c r="C40" s="54"/>
+      <c r="A40" s="55"/>
+      <c r="B40" s="55"/>
+      <c r="C40" s="55"/>
       <c r="D40" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
       <c r="G40" s="11"/>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
@@ -11834,22 +11832,22 @@
       <c r="HR40" s="11"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="64" t="s">
+      <c r="A41" s="65" t="s">
         <v>96</v>
       </c>
-      <c r="B41" s="55" t="s">
+      <c r="B41" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="C41" s="57" t="s">
+      <c r="C41" s="58" t="s">
         <v>98</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E41" s="56" t="s">
+      <c r="E41" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="F41" s="58" t="s">
+      <c r="F41" s="59" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="11"/>
@@ -12074,14 +12072,14 @@
       <c r="HR41" s="11"/>
     </row>
     <row r="42" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="54"/>
-      <c r="B42" s="54"/>
-      <c r="C42" s="54"/>
+      <c r="A42" s="55"/>
+      <c r="B42" s="55"/>
+      <c r="C42" s="55"/>
       <c r="D42" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
+      <c r="E42" s="55"/>
+      <c r="F42" s="55"/>
       <c r="G42" s="11"/>
       <c r="H42" s="11"/>
       <c r="I42" s="11"/>
@@ -12304,20 +12302,20 @@
       <c r="HR42" s="11"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="54"/>
-      <c r="B43" s="55" t="s">
+      <c r="A43" s="55"/>
+      <c r="B43" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="C43" s="57" t="s">
+      <c r="C43" s="58" t="s">
         <v>101</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E43" s="56" t="s">
+      <c r="E43" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="F43" s="58" t="s">
+      <c r="F43" s="59" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="11"/>
@@ -12540,14 +12538,14 @@
       <c r="HR43" s="11"/>
     </row>
     <row r="44" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="54"/>
-      <c r="B44" s="54"/>
-      <c r="C44" s="54"/>
+      <c r="A44" s="55"/>
+      <c r="B44" s="55"/>
+      <c r="C44" s="55"/>
       <c r="D44" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E44" s="54"/>
-      <c r="F44" s="54"/>
+      <c r="E44" s="55"/>
+      <c r="F44" s="55"/>
       <c r="G44" s="11"/>
       <c r="H44" s="11"/>
       <c r="I44" s="11"/>
@@ -12770,20 +12768,20 @@
       <c r="HR44" s="11"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="54"/>
-      <c r="B45" s="55" t="s">
+      <c r="A45" s="55"/>
+      <c r="B45" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="57" t="s">
+      <c r="C45" s="58" t="s">
         <v>104</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E45" s="56" t="s">
+      <c r="E45" s="57" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="58" t="s">
+      <c r="F45" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="11"/>
@@ -13007,14 +13005,14 @@
       <c r="HR45" s="11"/>
     </row>
     <row r="46" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="54"/>
-      <c r="B46" s="54"/>
-      <c r="C46" s="54"/>
+      <c r="A46" s="55"/>
+      <c r="B46" s="55"/>
+      <c r="C46" s="55"/>
       <c r="D46" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E46" s="54"/>
-      <c r="F46" s="54"/>
+      <c r="E46" s="55"/>
+      <c r="F46" s="55"/>
       <c r="G46" s="11"/>
       <c r="H46" s="11"/>
       <c r="I46" s="11"/>
@@ -13048,8 +13046,7 @@
       <c r="AK46" s="11"/>
       <c r="AL46" s="11"/>
       <c r="AM46" s="12"/>
-      <c r="AN46" s="13"/>
-      <c r="AO46" s="14"/>
+      <c r="AO46" s="52"/>
       <c r="AP46" s="11"/>
       <c r="AQ46" s="11"/>
       <c r="AR46" s="11"/>
@@ -13237,22 +13234,22 @@
       <c r="HR46" s="11"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="B47" s="55" t="s">
+      <c r="B47" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="C47" s="57" t="s">
+      <c r="C47" s="58" t="s">
         <v>108</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E47" s="56" t="s">
+      <c r="E47" s="57" t="s">
         <v>109</v>
       </c>
-      <c r="F47" s="58" t="s">
+      <c r="F47" s="59" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="11"/>
@@ -13477,14 +13474,14 @@
       <c r="HR47" s="11"/>
     </row>
     <row r="48" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="54"/>
-      <c r="B48" s="54"/>
-      <c r="C48" s="54"/>
+      <c r="A48" s="55"/>
+      <c r="B48" s="55"/>
+      <c r="C48" s="55"/>
       <c r="D48" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E48" s="54"/>
-      <c r="F48" s="54"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
@@ -13707,20 +13704,20 @@
       <c r="HR48" s="11"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="54"/>
-      <c r="B49" s="55" t="s">
+      <c r="A49" s="55"/>
+      <c r="B49" s="56" t="s">
         <v>110</v>
       </c>
-      <c r="C49" s="57" t="s">
+      <c r="C49" s="58" t="s">
         <v>111</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E49" s="56" t="s">
+      <c r="E49" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="F49" s="58" t="s">
+      <c r="F49" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="11"/>
@@ -13945,14 +13942,14 @@
       <c r="HR49" s="11"/>
     </row>
     <row r="50" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="54"/>
-      <c r="B50" s="54"/>
-      <c r="C50" s="54"/>
+      <c r="A50" s="55"/>
+      <c r="B50" s="55"/>
+      <c r="C50" s="55"/>
       <c r="D50" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E50" s="54"/>
-      <c r="F50" s="54"/>
+      <c r="E50" s="55"/>
+      <c r="F50" s="55"/>
       <c r="G50" s="11"/>
       <c r="H50" s="11"/>
       <c r="I50" s="11"/>
@@ -14175,22 +14172,22 @@
       <c r="HR50" s="11"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="64" t="s">
+      <c r="A51" s="65" t="s">
         <v>113</v>
       </c>
-      <c r="B51" s="55" t="s">
+      <c r="B51" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="C51" s="57" t="s">
+      <c r="C51" s="58" t="s">
         <v>115</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E51" s="56" t="s">
+      <c r="E51" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="F51" s="58" t="s">
+      <c r="F51" s="59" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="11"/>
@@ -14415,14 +14412,14 @@
       <c r="HR51" s="11"/>
     </row>
     <row r="52" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="54"/>
-      <c r="B52" s="54"/>
-      <c r="C52" s="54"/>
+      <c r="A52" s="55"/>
+      <c r="B52" s="55"/>
+      <c r="C52" s="55"/>
       <c r="D52" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E52" s="54"/>
-      <c r="F52" s="54"/>
+      <c r="E52" s="55"/>
+      <c r="F52" s="55"/>
       <c r="G52" s="11"/>
       <c r="H52" s="11"/>
       <c r="I52" s="11"/>
@@ -14645,20 +14642,20 @@
       <c r="HR52" s="11"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="54"/>
-      <c r="B53" s="55" t="s">
+      <c r="A53" s="55"/>
+      <c r="B53" s="56" t="s">
         <v>117</v>
       </c>
-      <c r="C53" s="57" t="s">
+      <c r="C53" s="58" t="s">
         <v>118</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E53" s="56" t="s">
+      <c r="E53" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="F53" s="58" t="s">
+      <c r="F53" s="59" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="11"/>
@@ -14883,14 +14880,14 @@
       <c r="HR53" s="11"/>
     </row>
     <row r="54" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="54"/>
-      <c r="B54" s="54"/>
-      <c r="C54" s="54"/>
+      <c r="A54" s="55"/>
+      <c r="B54" s="55"/>
+      <c r="C54" s="55"/>
       <c r="D54" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
+      <c r="E54" s="55"/>
+      <c r="F54" s="55"/>
       <c r="G54" s="11"/>
       <c r="H54" s="11"/>
       <c r="I54" s="11"/>
@@ -15113,22 +15110,22 @@
       <c r="HR54" s="11"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="64" t="s">
+      <c r="A55" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="B55" s="55" t="s">
+      <c r="B55" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="C55" s="57" t="s">
+      <c r="C55" s="58" t="s">
         <v>122</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E55" s="56" t="s">
+      <c r="E55" s="57" t="s">
         <v>123</v>
       </c>
-      <c r="F55" s="58" t="s">
+      <c r="F55" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="11"/>
@@ -15353,14 +15350,14 @@
       <c r="HR55" s="11"/>
     </row>
     <row r="56" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="54"/>
-      <c r="B56" s="54"/>
-      <c r="C56" s="54"/>
+      <c r="A56" s="55"/>
+      <c r="B56" s="55"/>
+      <c r="C56" s="55"/>
       <c r="D56" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E56" s="54"/>
-      <c r="F56" s="54"/>
+      <c r="E56" s="55"/>
+      <c r="F56" s="55"/>
       <c r="G56" s="11"/>
       <c r="H56" s="11"/>
       <c r="I56" s="11"/>
@@ -15583,20 +15580,20 @@
       <c r="HR56" s="11"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="54"/>
-      <c r="B57" s="55" t="s">
+      <c r="A57" s="55"/>
+      <c r="B57" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C57" s="57" t="s">
+      <c r="C57" s="58" t="s">
         <v>125</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E57" s="56" t="s">
+      <c r="E57" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="F57" s="58" t="s">
+      <c r="F57" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="11"/>
@@ -15821,14 +15818,14 @@
       <c r="HR57" s="11"/>
     </row>
     <row r="58" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="54"/>
-      <c r="B58" s="54"/>
-      <c r="C58" s="54"/>
+      <c r="A58" s="55"/>
+      <c r="B58" s="55"/>
+      <c r="C58" s="55"/>
       <c r="D58" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E58" s="54"/>
-      <c r="F58" s="54"/>
+      <c r="E58" s="55"/>
+      <c r="F58" s="55"/>
       <c r="G58" s="11"/>
       <c r="H58" s="11"/>
       <c r="I58" s="11"/>
@@ -16051,20 +16048,20 @@
       <c r="HR58" s="11"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="54"/>
-      <c r="B59" s="55" t="s">
+      <c r="A59" s="55"/>
+      <c r="B59" s="56" t="s">
         <v>127</v>
       </c>
-      <c r="C59" s="57" t="s">
+      <c r="C59" s="58" t="s">
         <v>128</v>
       </c>
       <c r="D59" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E59" s="56" t="s">
+      <c r="E59" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="F59" s="58" t="s">
+      <c r="F59" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="11"/>
@@ -16289,14 +16286,14 @@
       <c r="HR59" s="11"/>
     </row>
     <row r="60" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="54"/>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
+      <c r="A60" s="55"/>
+      <c r="B60" s="55"/>
+      <c r="C60" s="55"/>
       <c r="D60" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
+      <c r="E60" s="55"/>
+      <c r="F60" s="55"/>
       <c r="G60" s="11"/>
       <c r="H60" s="11"/>
       <c r="I60" s="11"/>
@@ -16519,20 +16516,20 @@
       <c r="HR60" s="11"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="54"/>
-      <c r="B61" s="55" t="s">
+      <c r="A61" s="55"/>
+      <c r="B61" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="57" t="s">
+      <c r="C61" s="58" t="s">
         <v>131</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="56" t="s">
+      <c r="E61" s="57" t="s">
         <v>132</v>
       </c>
-      <c r="F61" s="58" t="s">
+      <c r="F61" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="11"/>
@@ -16757,14 +16754,14 @@
       <c r="HR61" s="11"/>
     </row>
     <row r="62" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="54"/>
-      <c r="B62" s="54"/>
-      <c r="C62" s="54"/>
+      <c r="A62" s="55"/>
+      <c r="B62" s="55"/>
+      <c r="C62" s="55"/>
       <c r="D62" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
+      <c r="E62" s="55"/>
+      <c r="F62" s="55"/>
       <c r="G62" s="11"/>
       <c r="H62" s="11"/>
       <c r="I62" s="11"/>
@@ -16987,20 +16984,20 @@
       <c r="HR62" s="11"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="54"/>
-      <c r="B63" s="55" t="s">
+      <c r="A63" s="55"/>
+      <c r="B63" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="C63" s="57" t="s">
+      <c r="C63" s="58" t="s">
         <v>134</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E63" s="56" t="s">
+      <c r="E63" s="57" t="s">
         <v>135</v>
       </c>
-      <c r="F63" s="58" t="s">
+      <c r="F63" s="59" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="11"/>
@@ -17225,14 +17222,14 @@
       <c r="HR63" s="11"/>
     </row>
     <row r="64" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="54"/>
-      <c r="B64" s="54"/>
-      <c r="C64" s="54"/>
+      <c r="A64" s="55"/>
+      <c r="B64" s="55"/>
+      <c r="C64" s="55"/>
       <c r="D64" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E64" s="54"/>
-      <c r="F64" s="54"/>
+      <c r="E64" s="55"/>
+      <c r="F64" s="55"/>
       <c r="G64" s="11"/>
       <c r="H64" s="11"/>
       <c r="I64" s="11"/>
@@ -17455,20 +17452,20 @@
       <c r="HR64" s="11"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="54"/>
-      <c r="B65" s="55" t="s">
+      <c r="A65" s="55"/>
+      <c r="B65" s="56" t="s">
         <v>136</v>
       </c>
-      <c r="C65" s="57" t="s">
+      <c r="C65" s="58" t="s">
         <v>137</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E65" s="56" t="s">
+      <c r="E65" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="F65" s="58" t="s">
+      <c r="F65" s="59" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="11"/>
@@ -17693,14 +17690,14 @@
       <c r="HR65" s="11"/>
     </row>
     <row r="66" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="54"/>
-      <c r="B66" s="54"/>
-      <c r="C66" s="54"/>
+      <c r="A66" s="55"/>
+      <c r="B66" s="55"/>
+      <c r="C66" s="55"/>
       <c r="D66" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E66" s="54"/>
-      <c r="F66" s="54"/>
+      <c r="E66" s="55"/>
+      <c r="F66" s="55"/>
       <c r="G66" s="11"/>
       <c r="H66" s="11"/>
       <c r="I66" s="11"/>
@@ -17923,22 +17920,22 @@
       <c r="HR66" s="11"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="64" t="s">
+      <c r="A67" s="65" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="55" t="s">
+      <c r="B67" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="C67" s="57" t="s">
+      <c r="C67" s="58" t="s">
         <v>141</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E67" s="56" t="s">
+      <c r="E67" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="F67" s="58" t="s">
+      <c r="F67" s="59" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="11"/>
@@ -18163,14 +18160,14 @@
       <c r="HR67" s="11"/>
     </row>
     <row r="68" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="54"/>
-      <c r="B68" s="54"/>
-      <c r="C68" s="54"/>
+      <c r="A68" s="55"/>
+      <c r="B68" s="55"/>
+      <c r="C68" s="55"/>
       <c r="D68" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E68" s="54"/>
-      <c r="F68" s="54"/>
+      <c r="E68" s="55"/>
+      <c r="F68" s="55"/>
       <c r="G68" s="11"/>
       <c r="H68" s="11"/>
       <c r="I68" s="11"/>
@@ -18393,20 +18390,20 @@
       <c r="HR68" s="11"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="54"/>
-      <c r="B69" s="55" t="s">
+      <c r="A69" s="55"/>
+      <c r="B69" s="56" t="s">
         <v>143</v>
       </c>
-      <c r="C69" s="57" t="s">
+      <c r="C69" s="58" t="s">
         <v>144</v>
       </c>
       <c r="D69" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E69" s="56" t="s">
+      <c r="E69" s="57" t="s">
         <v>145</v>
       </c>
-      <c r="F69" s="58" t="s">
+      <c r="F69" s="59" t="s">
         <v>70</v>
       </c>
       <c r="G69" s="11"/>
@@ -18631,14 +18628,14 @@
       <c r="HR69" s="11"/>
     </row>
     <row r="70" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="54"/>
-      <c r="B70" s="54"/>
-      <c r="C70" s="54"/>
+      <c r="A70" s="55"/>
+      <c r="B70" s="55"/>
+      <c r="C70" s="55"/>
       <c r="D70" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E70" s="54"/>
-      <c r="F70" s="54"/>
+      <c r="E70" s="55"/>
+      <c r="F70" s="55"/>
       <c r="G70" s="11"/>
       <c r="H70" s="11"/>
       <c r="I70" s="11"/>
@@ -18861,20 +18858,20 @@
       <c r="HR70" s="11"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="54"/>
-      <c r="B71" s="55" t="s">
+      <c r="A71" s="55"/>
+      <c r="B71" s="56" t="s">
         <v>146</v>
       </c>
-      <c r="C71" s="57" t="s">
+      <c r="C71" s="58" t="s">
         <v>147</v>
       </c>
       <c r="D71" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E71" s="56" t="s">
+      <c r="E71" s="57" t="s">
         <v>148</v>
       </c>
-      <c r="F71" s="58" t="s">
+      <c r="F71" s="59" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="11"/>
@@ -19099,14 +19096,14 @@
       <c r="HR71" s="11"/>
     </row>
     <row r="72" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="54"/>
-      <c r="B72" s="54"/>
-      <c r="C72" s="54"/>
+      <c r="A72" s="55"/>
+      <c r="B72" s="55"/>
+      <c r="C72" s="55"/>
       <c r="D72" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E72" s="54"/>
-      <c r="F72" s="54"/>
+      <c r="E72" s="55"/>
+      <c r="F72" s="55"/>
       <c r="G72" s="11"/>
       <c r="H72" s="11"/>
       <c r="I72" s="11"/>
@@ -19329,20 +19326,20 @@
       <c r="HR72" s="11"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="54"/>
-      <c r="B73" s="55" t="s">
+      <c r="A73" s="55"/>
+      <c r="B73" s="56" t="s">
         <v>149</v>
       </c>
-      <c r="C73" s="57" t="s">
+      <c r="C73" s="58" t="s">
         <v>150</v>
       </c>
       <c r="D73" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E73" s="56" t="s">
+      <c r="E73" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="F73" s="58" t="s">
+      <c r="F73" s="59" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="11"/>
@@ -19567,14 +19564,14 @@
       <c r="HR73" s="11"/>
     </row>
     <row r="74" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="54"/>
-      <c r="B74" s="54"/>
-      <c r="C74" s="54"/>
+      <c r="A74" s="55"/>
+      <c r="B74" s="55"/>
+      <c r="C74" s="55"/>
       <c r="D74" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E74" s="54"/>
-      <c r="F74" s="54"/>
+      <c r="E74" s="55"/>
+      <c r="F74" s="55"/>
       <c r="G74" s="11"/>
       <c r="H74" s="11"/>
       <c r="I74" s="11"/>
@@ -19797,20 +19794,20 @@
       <c r="HR74" s="11"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="54"/>
-      <c r="B75" s="55" t="s">
+      <c r="A75" s="55"/>
+      <c r="B75" s="56" t="s">
         <v>152</v>
       </c>
-      <c r="C75" s="57" t="s">
+      <c r="C75" s="58" t="s">
         <v>153</v>
       </c>
       <c r="D75" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E75" s="56" t="s">
+      <c r="E75" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="F75" s="58" t="s">
+      <c r="F75" s="59" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="11"/>
@@ -20035,14 +20032,14 @@
       <c r="HR75" s="11"/>
     </row>
     <row r="76" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="54"/>
-      <c r="B76" s="54"/>
-      <c r="C76" s="54"/>
+      <c r="A76" s="55"/>
+      <c r="B76" s="55"/>
+      <c r="C76" s="55"/>
       <c r="D76" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E76" s="54"/>
-      <c r="F76" s="54"/>
+      <c r="E76" s="55"/>
+      <c r="F76" s="55"/>
       <c r="G76" s="11"/>
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
@@ -20265,20 +20262,20 @@
       <c r="HR76" s="11"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="54"/>
-      <c r="B77" s="55" t="s">
+      <c r="A77" s="55"/>
+      <c r="B77" s="56" t="s">
         <v>155</v>
       </c>
-      <c r="C77" s="57" t="s">
+      <c r="C77" s="58" t="s">
         <v>156</v>
       </c>
       <c r="D77" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E77" s="56" t="s">
+      <c r="E77" s="57" t="s">
         <v>157</v>
       </c>
-      <c r="F77" s="58" t="s">
+      <c r="F77" s="59" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="11"/>
@@ -20503,14 +20500,14 @@
       <c r="HR77" s="11"/>
     </row>
     <row r="78" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="54"/>
-      <c r="B78" s="54"/>
-      <c r="C78" s="54"/>
+      <c r="A78" s="55"/>
+      <c r="B78" s="55"/>
+      <c r="C78" s="55"/>
       <c r="D78" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E78" s="54"/>
-      <c r="F78" s="54"/>
+      <c r="E78" s="55"/>
+      <c r="F78" s="55"/>
       <c r="G78" s="11"/>
       <c r="H78" s="11"/>
       <c r="I78" s="11"/>
@@ -20733,22 +20730,22 @@
       <c r="HR78" s="11"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="64" t="s">
+      <c r="A79" s="65" t="s">
         <v>158</v>
       </c>
-      <c r="B79" s="55" t="s">
+      <c r="B79" s="56" t="s">
         <v>159</v>
       </c>
-      <c r="C79" s="53" t="s">
+      <c r="C79" s="54" t="s">
         <v>160</v>
       </c>
       <c r="D79" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E79" s="56" t="s">
+      <c r="E79" s="57" t="s">
         <v>161</v>
       </c>
-      <c r="F79" s="58" t="s">
+      <c r="F79" s="59" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="11"/>
@@ -20973,14 +20970,14 @@
       <c r="HR79" s="11"/>
     </row>
     <row r="80" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="54"/>
-      <c r="B80" s="54"/>
-      <c r="C80" s="54"/>
+      <c r="A80" s="55"/>
+      <c r="B80" s="55"/>
+      <c r="C80" s="55"/>
       <c r="D80" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E80" s="54"/>
-      <c r="F80" s="54"/>
+      <c r="E80" s="55"/>
+      <c r="F80" s="55"/>
       <c r="G80" s="11"/>
       <c r="H80" s="11"/>
       <c r="I80" s="11"/>
@@ -21203,20 +21200,20 @@
       <c r="HR80" s="11"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="54"/>
-      <c r="B81" s="55" t="s">
+      <c r="A81" s="55"/>
+      <c r="B81" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="C81" s="53" t="s">
+      <c r="C81" s="54" t="s">
         <v>163</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E81" s="56" t="s">
+      <c r="E81" s="57" t="s">
         <v>164</v>
       </c>
-      <c r="F81" s="58" t="s">
+      <c r="F81" s="59" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="11"/>
@@ -21441,14 +21438,14 @@
       <c r="HR81" s="11"/>
     </row>
     <row r="82" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="54"/>
-      <c r="B82" s="54"/>
-      <c r="C82" s="54"/>
+      <c r="A82" s="55"/>
+      <c r="B82" s="55"/>
+      <c r="C82" s="55"/>
       <c r="D82" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E82" s="54"/>
-      <c r="F82" s="54"/>
+      <c r="E82" s="55"/>
+      <c r="F82" s="55"/>
       <c r="G82" s="11"/>
       <c r="H82" s="11"/>
       <c r="I82" s="11"/>
@@ -21671,20 +21668,20 @@
       <c r="HR82" s="11"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="54"/>
-      <c r="B83" s="55" t="s">
+      <c r="A83" s="55"/>
+      <c r="B83" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="C83" s="57" t="s">
+      <c r="C83" s="58" t="s">
         <v>166</v>
       </c>
       <c r="D83" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E83" s="56" t="s">
+      <c r="E83" s="57" t="s">
         <v>167</v>
       </c>
-      <c r="F83" s="58" t="s">
+      <c r="F83" s="59" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="11"/>
@@ -21909,14 +21906,14 @@
       <c r="HR83" s="11"/>
     </row>
     <row r="84" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="54"/>
-      <c r="B84" s="54"/>
-      <c r="C84" s="54"/>
+      <c r="A84" s="55"/>
+      <c r="B84" s="55"/>
+      <c r="C84" s="55"/>
       <c r="D84" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E84" s="54"/>
-      <c r="F84" s="54"/>
+      <c r="E84" s="55"/>
+      <c r="F84" s="55"/>
       <c r="G84" s="11"/>
       <c r="H84" s="11"/>
       <c r="I84" s="11"/>
@@ -22139,20 +22136,20 @@
       <c r="HR84" s="11"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="54"/>
-      <c r="B85" s="55" t="s">
+      <c r="A85" s="55"/>
+      <c r="B85" s="56" t="s">
         <v>168</v>
       </c>
-      <c r="C85" s="66" t="s">
+      <c r="C85" s="67" t="s">
         <v>169</v>
       </c>
       <c r="D85" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E85" s="56" t="s">
+      <c r="E85" s="57" t="s">
         <v>170</v>
       </c>
-      <c r="F85" s="58"/>
+      <c r="F85" s="59"/>
       <c r="G85" s="11"/>
       <c r="H85" s="11"/>
       <c r="I85" s="11"/>
@@ -22375,14 +22372,14 @@
       <c r="HR85" s="23"/>
     </row>
     <row r="86" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="54"/>
-      <c r="B86" s="54"/>
-      <c r="C86" s="54"/>
+      <c r="A86" s="55"/>
+      <c r="B86" s="55"/>
+      <c r="C86" s="55"/>
       <c r="D86" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E86" s="54"/>
-      <c r="F86" s="54"/>
+      <c r="E86" s="55"/>
+      <c r="F86" s="55"/>
       <c r="G86" s="11"/>
       <c r="H86" s="11"/>
       <c r="I86" s="11"/>
@@ -22606,7 +22603,6 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="B65:B66"/>
     <mergeCell ref="FS1:FY1"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="C37:C38"/>
@@ -22615,6 +22611,12 @@
     <mergeCell ref="B41:B42"/>
     <mergeCell ref="F69:F70"/>
     <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
     <mergeCell ref="E85:E86"/>
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="B85:B86"/>
@@ -22632,17 +22634,12 @@
     <mergeCell ref="C67:C68"/>
     <mergeCell ref="C61:C62"/>
     <mergeCell ref="E43:E44"/>
-    <mergeCell ref="E17:E18"/>
     <mergeCell ref="B47:B48"/>
-    <mergeCell ref="F25:F26"/>
     <mergeCell ref="C33:C34"/>
     <mergeCell ref="E33:E34"/>
-    <mergeCell ref="E19:E20"/>
     <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C9:C10"/>
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="E35:E36"/>
-    <mergeCell ref="E9:E10"/>
     <mergeCell ref="C83:C84"/>
     <mergeCell ref="E83:E84"/>
     <mergeCell ref="B81:B82"/>
@@ -22692,7 +22689,6 @@
     <mergeCell ref="F67:F68"/>
     <mergeCell ref="C53:C54"/>
     <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E39:E40"/>
     <mergeCell ref="B73:B74"/>
     <mergeCell ref="G1:M1"/>
     <mergeCell ref="C59:C60"/>
@@ -22715,6 +22711,7 @@
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="BD1:BJ1"/>
     <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
     <mergeCell ref="F83:F84"/>
     <mergeCell ref="E55:E56"/>
     <mergeCell ref="E13:E14"/>

</xml_diff>

<commit_message>
Konsultation abgehalten; Methodik ausgearbeitet, Vorlage für Thesis erhalten
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30ECF1DF-A614-4567-953C-0CEA0931F63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86F4B1B-EA88-4513-BCC0-E9BB17578C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
     <sheet name="Pakete &amp; Leitfragen" sheetId="2" r:id="rId2"/>
     <sheet name="Legende &amp; Regeln" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -1259,53 +1270,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1626,290 +1637,290 @@
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="70" t="s">
+      <c r="G1" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
-      <c r="N1" s="70" t="s">
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="65"/>
-      <c r="P1" s="65"/>
-      <c r="Q1" s="65"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="65"/>
-      <c r="T1" s="65"/>
-      <c r="U1" s="70" t="s">
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="65"/>
-      <c r="W1" s="65"/>
-      <c r="X1" s="65"/>
-      <c r="Y1" s="65"/>
-      <c r="Z1" s="65"/>
-      <c r="AA1" s="65"/>
-      <c r="AB1" s="71" t="s">
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="65"/>
-      <c r="AD1" s="65"/>
-      <c r="AE1" s="65"/>
-      <c r="AF1" s="65"/>
-      <c r="AG1" s="65"/>
-      <c r="AH1" s="65"/>
-      <c r="AI1" s="70" t="s">
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="65"/>
-      <c r="AK1" s="65"/>
-      <c r="AL1" s="65"/>
-      <c r="AM1" s="65"/>
-      <c r="AN1" s="65"/>
-      <c r="AO1" s="65"/>
-      <c r="AP1" s="70" t="s">
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="65"/>
-      <c r="AR1" s="65"/>
-      <c r="AS1" s="65"/>
-      <c r="AT1" s="65"/>
-      <c r="AU1" s="65"/>
-      <c r="AV1" s="65"/>
-      <c r="AW1" s="70" t="s">
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67"/>
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="65"/>
-      <c r="AY1" s="65"/>
-      <c r="AZ1" s="65"/>
-      <c r="BA1" s="65"/>
-      <c r="BB1" s="65"/>
-      <c r="BC1" s="65"/>
-      <c r="BD1" s="70" t="s">
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67"/>
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="67"/>
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67"/>
+      <c r="BD1" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="65"/>
-      <c r="BF1" s="65"/>
-      <c r="BG1" s="65"/>
-      <c r="BH1" s="65"/>
-      <c r="BI1" s="65"/>
-      <c r="BJ1" s="65"/>
-      <c r="BK1" s="70" t="s">
+      <c r="BE1" s="67"/>
+      <c r="BF1" s="67"/>
+      <c r="BG1" s="67"/>
+      <c r="BH1" s="67"/>
+      <c r="BI1" s="67"/>
+      <c r="BJ1" s="67"/>
+      <c r="BK1" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="65"/>
-      <c r="BM1" s="65"/>
-      <c r="BN1" s="65"/>
-      <c r="BO1" s="65"/>
-      <c r="BP1" s="65"/>
-      <c r="BQ1" s="65"/>
-      <c r="BR1" s="70" t="s">
+      <c r="BL1" s="67"/>
+      <c r="BM1" s="67"/>
+      <c r="BN1" s="67"/>
+      <c r="BO1" s="67"/>
+      <c r="BP1" s="67"/>
+      <c r="BQ1" s="67"/>
+      <c r="BR1" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="65"/>
-      <c r="BT1" s="65"/>
-      <c r="BU1" s="65"/>
-      <c r="BV1" s="65"/>
-      <c r="BW1" s="65"/>
-      <c r="BX1" s="65"/>
-      <c r="BY1" s="70" t="s">
+      <c r="BS1" s="67"/>
+      <c r="BT1" s="67"/>
+      <c r="BU1" s="67"/>
+      <c r="BV1" s="67"/>
+      <c r="BW1" s="67"/>
+      <c r="BX1" s="67"/>
+      <c r="BY1" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="65"/>
-      <c r="CA1" s="65"/>
-      <c r="CB1" s="65"/>
-      <c r="CC1" s="65"/>
-      <c r="CD1" s="65"/>
-      <c r="CE1" s="65"/>
-      <c r="CF1" s="70" t="s">
+      <c r="BZ1" s="67"/>
+      <c r="CA1" s="67"/>
+      <c r="CB1" s="67"/>
+      <c r="CC1" s="67"/>
+      <c r="CD1" s="67"/>
+      <c r="CE1" s="67"/>
+      <c r="CF1" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="65"/>
-      <c r="CH1" s="65"/>
-      <c r="CI1" s="65"/>
-      <c r="CJ1" s="65"/>
-      <c r="CK1" s="65"/>
-      <c r="CL1" s="65"/>
-      <c r="CM1" s="70" t="s">
+      <c r="CG1" s="67"/>
+      <c r="CH1" s="67"/>
+      <c r="CI1" s="67"/>
+      <c r="CJ1" s="67"/>
+      <c r="CK1" s="67"/>
+      <c r="CL1" s="67"/>
+      <c r="CM1" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="65"/>
-      <c r="CO1" s="65"/>
-      <c r="CP1" s="65"/>
-      <c r="CQ1" s="65"/>
-      <c r="CR1" s="65"/>
-      <c r="CS1" s="65"/>
-      <c r="CT1" s="70" t="s">
+      <c r="CN1" s="67"/>
+      <c r="CO1" s="67"/>
+      <c r="CP1" s="67"/>
+      <c r="CQ1" s="67"/>
+      <c r="CR1" s="67"/>
+      <c r="CS1" s="67"/>
+      <c r="CT1" s="66" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="65"/>
-      <c r="CV1" s="65"/>
-      <c r="CW1" s="65"/>
-      <c r="CX1" s="65"/>
-      <c r="CY1" s="65"/>
-      <c r="CZ1" s="65"/>
-      <c r="DA1" s="70" t="s">
+      <c r="CU1" s="67"/>
+      <c r="CV1" s="67"/>
+      <c r="CW1" s="67"/>
+      <c r="CX1" s="67"/>
+      <c r="CY1" s="67"/>
+      <c r="CZ1" s="67"/>
+      <c r="DA1" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="65"/>
-      <c r="DC1" s="65"/>
-      <c r="DD1" s="65"/>
-      <c r="DE1" s="65"/>
-      <c r="DF1" s="65"/>
-      <c r="DG1" s="65"/>
-      <c r="DH1" s="70" t="s">
+      <c r="DB1" s="67"/>
+      <c r="DC1" s="67"/>
+      <c r="DD1" s="67"/>
+      <c r="DE1" s="67"/>
+      <c r="DF1" s="67"/>
+      <c r="DG1" s="67"/>
+      <c r="DH1" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="65"/>
-      <c r="DJ1" s="65"/>
-      <c r="DK1" s="65"/>
-      <c r="DL1" s="65"/>
-      <c r="DM1" s="65"/>
-      <c r="DN1" s="65"/>
-      <c r="DO1" s="70" t="s">
+      <c r="DI1" s="67"/>
+      <c r="DJ1" s="67"/>
+      <c r="DK1" s="67"/>
+      <c r="DL1" s="67"/>
+      <c r="DM1" s="67"/>
+      <c r="DN1" s="67"/>
+      <c r="DO1" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="65"/>
-      <c r="DQ1" s="65"/>
-      <c r="DR1" s="65"/>
-      <c r="DS1" s="65"/>
-      <c r="DT1" s="65"/>
-      <c r="DU1" s="65"/>
-      <c r="DV1" s="70" t="s">
+      <c r="DP1" s="67"/>
+      <c r="DQ1" s="67"/>
+      <c r="DR1" s="67"/>
+      <c r="DS1" s="67"/>
+      <c r="DT1" s="67"/>
+      <c r="DU1" s="67"/>
+      <c r="DV1" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="65"/>
-      <c r="DX1" s="65"/>
-      <c r="DY1" s="65"/>
-      <c r="DZ1" s="65"/>
-      <c r="EA1" s="65"/>
-      <c r="EB1" s="65"/>
-      <c r="EC1" s="70" t="s">
+      <c r="DW1" s="67"/>
+      <c r="DX1" s="67"/>
+      <c r="DY1" s="67"/>
+      <c r="DZ1" s="67"/>
+      <c r="EA1" s="67"/>
+      <c r="EB1" s="67"/>
+      <c r="EC1" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="65"/>
-      <c r="EE1" s="65"/>
-      <c r="EF1" s="65"/>
-      <c r="EG1" s="65"/>
-      <c r="EH1" s="65"/>
-      <c r="EI1" s="65"/>
-      <c r="EJ1" s="70" t="s">
+      <c r="ED1" s="67"/>
+      <c r="EE1" s="67"/>
+      <c r="EF1" s="67"/>
+      <c r="EG1" s="67"/>
+      <c r="EH1" s="67"/>
+      <c r="EI1" s="67"/>
+      <c r="EJ1" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="65"/>
-      <c r="EL1" s="65"/>
-      <c r="EM1" s="65"/>
-      <c r="EN1" s="65"/>
-      <c r="EO1" s="65"/>
-      <c r="EP1" s="65"/>
-      <c r="EQ1" s="70" t="s">
+      <c r="EK1" s="67"/>
+      <c r="EL1" s="67"/>
+      <c r="EM1" s="67"/>
+      <c r="EN1" s="67"/>
+      <c r="EO1" s="67"/>
+      <c r="EP1" s="67"/>
+      <c r="EQ1" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="65"/>
-      <c r="ES1" s="65"/>
-      <c r="ET1" s="65"/>
-      <c r="EU1" s="65"/>
-      <c r="EV1" s="65"/>
-      <c r="EW1" s="65"/>
-      <c r="EX1" s="70" t="s">
+      <c r="ER1" s="67"/>
+      <c r="ES1" s="67"/>
+      <c r="ET1" s="67"/>
+      <c r="EU1" s="67"/>
+      <c r="EV1" s="67"/>
+      <c r="EW1" s="67"/>
+      <c r="EX1" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="65"/>
-      <c r="EZ1" s="65"/>
-      <c r="FA1" s="65"/>
-      <c r="FB1" s="65"/>
-      <c r="FC1" s="65"/>
-      <c r="FD1" s="65"/>
-      <c r="FE1" s="70" t="s">
+      <c r="EY1" s="67"/>
+      <c r="EZ1" s="67"/>
+      <c r="FA1" s="67"/>
+      <c r="FB1" s="67"/>
+      <c r="FC1" s="67"/>
+      <c r="FD1" s="67"/>
+      <c r="FE1" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="65"/>
-      <c r="FG1" s="65"/>
-      <c r="FH1" s="65"/>
-      <c r="FI1" s="65"/>
-      <c r="FJ1" s="65"/>
-      <c r="FK1" s="65"/>
-      <c r="FL1" s="70" t="s">
+      <c r="FF1" s="67"/>
+      <c r="FG1" s="67"/>
+      <c r="FH1" s="67"/>
+      <c r="FI1" s="67"/>
+      <c r="FJ1" s="67"/>
+      <c r="FK1" s="67"/>
+      <c r="FL1" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="65"/>
-      <c r="FN1" s="65"/>
-      <c r="FO1" s="65"/>
-      <c r="FP1" s="65"/>
-      <c r="FQ1" s="65"/>
-      <c r="FR1" s="65"/>
-      <c r="FS1" s="70" t="s">
+      <c r="FM1" s="67"/>
+      <c r="FN1" s="67"/>
+      <c r="FO1" s="67"/>
+      <c r="FP1" s="67"/>
+      <c r="FQ1" s="67"/>
+      <c r="FR1" s="67"/>
+      <c r="FS1" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="65"/>
-      <c r="FU1" s="65"/>
-      <c r="FV1" s="65"/>
-      <c r="FW1" s="65"/>
-      <c r="FX1" s="65"/>
-      <c r="FY1" s="65"/>
-      <c r="FZ1" s="70" t="s">
+      <c r="FT1" s="67"/>
+      <c r="FU1" s="67"/>
+      <c r="FV1" s="67"/>
+      <c r="FW1" s="67"/>
+      <c r="FX1" s="67"/>
+      <c r="FY1" s="67"/>
+      <c r="FZ1" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="65"/>
-      <c r="GB1" s="65"/>
-      <c r="GC1" s="65"/>
-      <c r="GD1" s="65"/>
-      <c r="GE1" s="65"/>
-      <c r="GF1" s="65"/>
-      <c r="GG1" s="70" t="s">
+      <c r="GA1" s="67"/>
+      <c r="GB1" s="67"/>
+      <c r="GC1" s="67"/>
+      <c r="GD1" s="67"/>
+      <c r="GE1" s="67"/>
+      <c r="GF1" s="67"/>
+      <c r="GG1" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="65"/>
-      <c r="GI1" s="65"/>
-      <c r="GJ1" s="65"/>
-      <c r="GK1" s="65"/>
-      <c r="GL1" s="65"/>
-      <c r="GM1" s="65"/>
-      <c r="GN1" s="70" t="s">
+      <c r="GH1" s="67"/>
+      <c r="GI1" s="67"/>
+      <c r="GJ1" s="67"/>
+      <c r="GK1" s="67"/>
+      <c r="GL1" s="67"/>
+      <c r="GM1" s="67"/>
+      <c r="GN1" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="65"/>
-      <c r="GP1" s="65"/>
-      <c r="GQ1" s="65"/>
-      <c r="GR1" s="65"/>
-      <c r="GS1" s="65"/>
-      <c r="GT1" s="65"/>
-      <c r="GU1" s="70" t="s">
+      <c r="GO1" s="67"/>
+      <c r="GP1" s="67"/>
+      <c r="GQ1" s="67"/>
+      <c r="GR1" s="67"/>
+      <c r="GS1" s="67"/>
+      <c r="GT1" s="67"/>
+      <c r="GU1" s="66" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="65"/>
-      <c r="GW1" s="65"/>
-      <c r="GX1" s="65"/>
-      <c r="GY1" s="65"/>
-      <c r="GZ1" s="65"/>
-      <c r="HA1" s="65"/>
-      <c r="HB1" s="70" t="s">
+      <c r="GV1" s="67"/>
+      <c r="GW1" s="67"/>
+      <c r="GX1" s="67"/>
+      <c r="GY1" s="67"/>
+      <c r="GZ1" s="67"/>
+      <c r="HA1" s="67"/>
+      <c r="HB1" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="65"/>
-      <c r="HD1" s="65"/>
-      <c r="HE1" s="65"/>
-      <c r="HF1" s="65"/>
-      <c r="HG1" s="65"/>
-      <c r="HH1" s="65"/>
-      <c r="HI1" s="70" t="s">
+      <c r="HC1" s="67"/>
+      <c r="HD1" s="67"/>
+      <c r="HE1" s="67"/>
+      <c r="HF1" s="67"/>
+      <c r="HG1" s="67"/>
+      <c r="HH1" s="67"/>
+      <c r="HI1" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="65"/>
-      <c r="HK1" s="65"/>
-      <c r="HL1" s="65"/>
-      <c r="HM1" s="65"/>
-      <c r="HN1" s="65"/>
-      <c r="HO1" s="65"/>
-      <c r="HP1" s="70" t="s">
+      <c r="HJ1" s="67"/>
+      <c r="HK1" s="67"/>
+      <c r="HL1" s="67"/>
+      <c r="HM1" s="67"/>
+      <c r="HN1" s="67"/>
+      <c r="HO1" s="67"/>
+      <c r="HP1" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="65"/>
-      <c r="HR1" s="65"/>
+      <c r="HQ1" s="67"/>
+      <c r="HR1" s="67"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="1" t="s">
@@ -3480,20 +3491,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="76"/>
-      <c r="C5" s="74" t="s">
+      <c r="B5" s="77"/>
+      <c r="C5" s="70" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="78" t="s">
+      <c r="E5" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="72"/>
+      <c r="F5" s="79"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3715,14 +3726,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="73"/>
-      <c r="B6" s="73"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="71"/>
+      <c r="C6" s="71"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
+      <c r="E6" s="71"/>
+      <c r="F6" s="71"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3944,18 +3955,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="73"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="74" t="s">
+      <c r="A7" s="71"/>
+      <c r="B7" s="77"/>
+      <c r="C7" s="70" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="78" t="s">
+      <c r="E7" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="72"/>
+      <c r="F7" s="79"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -4177,14 +4188,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="73"/>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
+      <c r="A8" s="71"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="71"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="71"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4406,18 +4417,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="73"/>
-      <c r="B9" s="76"/>
-      <c r="C9" s="74" t="s">
+      <c r="A9" s="71"/>
+      <c r="B9" s="77"/>
+      <c r="C9" s="70" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="78" t="s">
+      <c r="E9" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="72"/>
+      <c r="F9" s="79"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4639,14 +4650,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="73"/>
-      <c r="B10" s="73"/>
-      <c r="C10" s="73"/>
+      <c r="A10" s="71"/>
+      <c r="B10" s="71"/>
+      <c r="C10" s="71"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="73"/>
-      <c r="F10" s="73"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="71"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4868,18 +4879,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="73"/>
-      <c r="B11" s="76"/>
-      <c r="C11" s="74" t="s">
+      <c r="A11" s="71"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="70" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="78" t="s">
+      <c r="E11" s="75" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="72"/>
+      <c r="F11" s="79"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -5101,14 +5112,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="73"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
+      <c r="A12" s="71"/>
+      <c r="B12" s="71"/>
+      <c r="C12" s="71"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
+      <c r="E12" s="71"/>
+      <c r="F12" s="71"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5330,18 +5341,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="73"/>
-      <c r="B13" s="76"/>
-      <c r="C13" s="74" t="s">
+      <c r="A13" s="71"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="70" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="78" t="s">
+      <c r="E13" s="75" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="72"/>
+      <c r="F13" s="79"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5563,14 +5574,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="73"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
+      <c r="A14" s="71"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5792,18 +5803,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="73"/>
-      <c r="B15" s="76"/>
-      <c r="C15" s="74" t="s">
+      <c r="A15" s="71"/>
+      <c r="B15" s="77"/>
+      <c r="C15" s="70" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="78" t="s">
+      <c r="E15" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="72"/>
+      <c r="F15" s="79"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -6025,14 +6036,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="73"/>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
+      <c r="A16" s="71"/>
+      <c r="B16" s="71"/>
+      <c r="C16" s="71"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="73"/>
-      <c r="F16" s="73"/>
+      <c r="E16" s="71"/>
+      <c r="F16" s="71"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6254,18 +6265,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="73"/>
-      <c r="B17" s="76"/>
-      <c r="C17" s="74" t="s">
+      <c r="A17" s="71"/>
+      <c r="B17" s="77"/>
+      <c r="C17" s="70" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="78" t="s">
+      <c r="E17" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="72"/>
+      <c r="F17" s="79"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6487,14 +6498,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="73"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
+      <c r="A18" s="71"/>
+      <c r="B18" s="71"/>
+      <c r="C18" s="71"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
+      <c r="E18" s="71"/>
+      <c r="F18" s="71"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6716,18 +6727,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="73"/>
-      <c r="B19" s="76"/>
-      <c r="C19" s="74" t="s">
+      <c r="A19" s="71"/>
+      <c r="B19" s="77"/>
+      <c r="C19" s="70" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="78" t="s">
+      <c r="E19" s="75" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="72"/>
+      <c r="F19" s="79"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6949,14 +6960,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="73"/>
-      <c r="B20" s="73"/>
-      <c r="C20" s="73"/>
+      <c r="A20" s="71"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="73"/>
-      <c r="F20" s="73"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="71"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -7178,18 +7189,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="73"/>
-      <c r="B21" s="76"/>
-      <c r="C21" s="74" t="s">
+      <c r="A21" s="71"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="70" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="78" t="s">
+      <c r="E21" s="75" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="72"/>
+      <c r="F21" s="79"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7411,14 +7422,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="79"/>
-      <c r="B22" s="79"/>
-      <c r="C22" s="79"/>
+      <c r="A22" s="78"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="78"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="79"/>
-      <c r="F22" s="79"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="78"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7641,22 +7652,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="73" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="68" t="s">
+      <c r="C23" s="69" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="67" t="s">
+      <c r="E23" s="72" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="69" t="s">
+      <c r="F23" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7881,14 +7892,14 @@
       <c r="HR23" s="8"/>
     </row>
     <row r="24" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="65"/>
-      <c r="B24" s="65"/>
-      <c r="C24" s="65"/>
+      <c r="A24" s="67"/>
+      <c r="B24" s="67"/>
+      <c r="C24" s="67"/>
       <c r="D24" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="65"/>
-      <c r="F24" s="65"/>
+      <c r="E24" s="67"/>
+      <c r="F24" s="67"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
@@ -7924,8 +7935,8 @@
       <c r="AM24" s="9"/>
       <c r="AN24" s="10"/>
       <c r="AO24" s="11"/>
-      <c r="AP24" s="81"/>
-      <c r="AQ24" s="82"/>
+      <c r="AP24" s="64"/>
+      <c r="AQ24" s="65"/>
       <c r="AR24" s="8"/>
       <c r="AS24" s="8"/>
       <c r="AT24" s="9"/>
@@ -8111,20 +8122,20 @@
       <c r="HR24" s="8"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="65"/>
-      <c r="B25" s="66" t="s">
+      <c r="A25" s="67"/>
+      <c r="B25" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="68" t="s">
+      <c r="C25" s="69" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="67" t="s">
+      <c r="E25" s="72" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="69" t="s">
+      <c r="F25" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8340,14 +8351,14 @@
       <c r="HS25" s="8"/>
     </row>
     <row r="26" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="65"/>
-      <c r="B26" s="65"/>
-      <c r="C26" s="65"/>
+      <c r="A26" s="67"/>
+      <c r="B26" s="67"/>
+      <c r="C26" s="67"/>
       <c r="D26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="65"/>
-      <c r="F26" s="65"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="67"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
@@ -8569,20 +8580,20 @@
       <c r="HR26" s="8"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="65"/>
-      <c r="B27" s="66" t="s">
+      <c r="A27" s="67"/>
+      <c r="B27" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="77" t="s">
+      <c r="C27" s="80" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="67" t="s">
+      <c r="E27" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="69"/>
+      <c r="F27" s="74"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8620,14 +8631,13 @@
       <c r="AO27" s="11"/>
       <c r="AQ27" s="8"/>
       <c r="AR27" s="8"/>
-      <c r="AS27" s="17"/>
       <c r="AT27" s="9"/>
       <c r="AU27" s="10"/>
       <c r="AV27" s="11"/>
       <c r="AW27" s="8"/>
       <c r="AX27" s="8"/>
       <c r="AY27" s="8"/>
-      <c r="AZ27" s="8"/>
+      <c r="AZ27" s="17"/>
       <c r="BA27" s="9"/>
       <c r="BB27" s="10"/>
       <c r="BC27" s="11"/>
@@ -8804,14 +8814,14 @@
       <c r="HR27" s="8"/>
     </row>
     <row r="28" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="65"/>
-      <c r="B28" s="65"/>
-      <c r="C28" s="65"/>
+      <c r="A28" s="67"/>
+      <c r="B28" s="67"/>
+      <c r="C28" s="67"/>
       <c r="D28" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="65"/>
-      <c r="F28" s="65"/>
+      <c r="E28" s="67"/>
+      <c r="F28" s="67"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
@@ -8855,7 +8865,7 @@
       <c r="AW28" s="8"/>
       <c r="AX28" s="8"/>
       <c r="AY28" s="8"/>
-      <c r="AZ28" s="8"/>
+      <c r="AZ28" s="43"/>
       <c r="BA28" s="9"/>
       <c r="BB28" s="10"/>
       <c r="BC28" s="11"/>
@@ -9032,22 +9042,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="75" t="s">
+      <c r="A29" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="66" t="s">
+      <c r="B29" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="68" t="s">
+      <c r="C29" s="69" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="67" t="s">
+      <c r="E29" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="69" t="s">
+      <c r="F29" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9270,14 +9280,14 @@
       <c r="HR29" s="8"/>
     </row>
     <row r="30" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="65"/>
-      <c r="B30" s="65"/>
-      <c r="C30" s="65"/>
+      <c r="A30" s="67"/>
+      <c r="B30" s="67"/>
+      <c r="C30" s="67"/>
       <c r="D30" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="65"/>
-      <c r="F30" s="65"/>
+      <c r="E30" s="67"/>
+      <c r="F30" s="67"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
@@ -9499,20 +9509,20 @@
       <c r="HR30" s="8"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="65"/>
-      <c r="B31" s="66" t="s">
+      <c r="A31" s="67"/>
+      <c r="B31" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="68" t="s">
+      <c r="C31" s="69" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="67" t="s">
+      <c r="E31" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="69" t="s">
+      <c r="F31" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9736,14 +9746,14 @@
       <c r="HR31" s="8"/>
     </row>
     <row r="32" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="65"/>
-      <c r="B32" s="65"/>
-      <c r="C32" s="65"/>
+      <c r="A32" s="67"/>
+      <c r="B32" s="67"/>
+      <c r="C32" s="67"/>
       <c r="D32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="65"/>
-      <c r="F32" s="65"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="67"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="8"/>
@@ -9965,20 +9975,20 @@
       <c r="HR32" s="8"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="65"/>
-      <c r="B33" s="66" t="s">
+      <c r="A33" s="67"/>
+      <c r="B33" s="73" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="69" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="67" t="s">
+      <c r="E33" s="72" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="69" t="s">
+      <c r="F33" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -10202,14 +10212,14 @@
       <c r="HR33" s="8"/>
     </row>
     <row r="34" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="65"/>
-      <c r="B34" s="65"/>
-      <c r="C34" s="65"/>
+      <c r="A34" s="67"/>
+      <c r="B34" s="67"/>
+      <c r="C34" s="67"/>
       <c r="D34" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="65"/>
-      <c r="F34" s="65"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="67"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
@@ -10431,20 +10441,20 @@
       <c r="HR34" s="8"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="65"/>
-      <c r="B35" s="66" t="s">
+      <c r="A35" s="67"/>
+      <c r="B35" s="73" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="68" t="s">
+      <c r="C35" s="69" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="67" t="s">
+      <c r="E35" s="72" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="69" t="s">
+      <c r="F35" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10668,14 +10678,14 @@
       <c r="HR35" s="8"/>
     </row>
     <row r="36" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="65"/>
-      <c r="B36" s="65"/>
-      <c r="C36" s="65"/>
+      <c r="A36" s="67"/>
+      <c r="B36" s="67"/>
+      <c r="C36" s="67"/>
       <c r="D36" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="65"/>
-      <c r="F36" s="65"/>
+      <c r="E36" s="67"/>
+      <c r="F36" s="67"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
@@ -10897,20 +10907,20 @@
       <c r="HR36" s="8"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="65"/>
-      <c r="B37" s="66" t="s">
+      <c r="A37" s="67"/>
+      <c r="B37" s="73" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="68" t="s">
+      <c r="C37" s="69" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="67" t="s">
+      <c r="E37" s="72" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="69" t="s">
+      <c r="F37" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -11134,14 +11144,14 @@
       <c r="HR37" s="8"/>
     </row>
     <row r="38" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="65"/>
-      <c r="B38" s="65"/>
-      <c r="C38" s="65"/>
+      <c r="A38" s="67"/>
+      <c r="B38" s="67"/>
+      <c r="C38" s="67"/>
       <c r="D38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
+      <c r="E38" s="67"/>
+      <c r="F38" s="67"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
@@ -11363,20 +11373,20 @@
       <c r="HR38" s="8"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="65"/>
-      <c r="B39" s="66" t="s">
+      <c r="A39" s="67"/>
+      <c r="B39" s="73" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="69" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="67" t="s">
+      <c r="E39" s="72" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="69" t="s">
+      <c r="F39" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11600,14 +11610,14 @@
       <c r="HR39" s="8"/>
     </row>
     <row r="40" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="65"/>
-      <c r="B40" s="65"/>
-      <c r="C40" s="65"/>
+      <c r="A40" s="67"/>
+      <c r="B40" s="67"/>
+      <c r="C40" s="67"/>
       <c r="D40" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="65"/>
-      <c r="F40" s="65"/>
+      <c r="E40" s="67"/>
+      <c r="F40" s="67"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
@@ -11829,22 +11839,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="75" t="s">
+      <c r="A41" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="66" t="s">
+      <c r="B41" s="73" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="69" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="67" t="s">
+      <c r="E41" s="72" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="69" t="s">
+      <c r="F41" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -12068,14 +12078,14 @@
       <c r="HR41" s="8"/>
     </row>
     <row r="42" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="65"/>
-      <c r="B42" s="65"/>
-      <c r="C42" s="65"/>
+      <c r="A42" s="67"/>
+      <c r="B42" s="67"/>
+      <c r="C42" s="67"/>
       <c r="D42" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="65"/>
-      <c r="F42" s="65"/>
+      <c r="E42" s="67"/>
+      <c r="F42" s="67"/>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="8"/>
@@ -12297,20 +12307,20 @@
       <c r="HR42" s="8"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="65"/>
-      <c r="B43" s="66" t="s">
+      <c r="A43" s="67"/>
+      <c r="B43" s="73" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="68" t="s">
+      <c r="C43" s="69" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="67" t="s">
+      <c r="E43" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="69" t="s">
+      <c r="F43" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12533,14 +12543,14 @@
       <c r="HR43" s="8"/>
     </row>
     <row r="44" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="65"/>
-      <c r="B44" s="65"/>
-      <c r="C44" s="65"/>
+      <c r="A44" s="67"/>
+      <c r="B44" s="67"/>
+      <c r="C44" s="67"/>
       <c r="D44" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="65"/>
-      <c r="F44" s="65"/>
+      <c r="E44" s="67"/>
+      <c r="F44" s="67"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="8"/>
@@ -12578,7 +12588,7 @@
       <c r="AO44" s="11"/>
       <c r="AP44" s="43"/>
       <c r="AQ44" s="8"/>
-      <c r="AR44" s="8"/>
+      <c r="AR44" s="44"/>
       <c r="AS44" s="8"/>
       <c r="AT44" s="9"/>
       <c r="AU44" s="10"/>
@@ -12763,20 +12773,20 @@
       <c r="HR44" s="8"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="65"/>
-      <c r="B45" s="66" t="s">
+      <c r="A45" s="67"/>
+      <c r="B45" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="69" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="67" t="s">
+      <c r="E45" s="72" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="69" t="s">
+      <c r="F45" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12999,14 +13009,14 @@
       <c r="HR45" s="8"/>
     </row>
     <row r="46" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="65"/>
-      <c r="B46" s="65"/>
-      <c r="C46" s="65"/>
+      <c r="A46" s="67"/>
+      <c r="B46" s="67"/>
+      <c r="C46" s="67"/>
       <c r="D46" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="65"/>
-      <c r="F46" s="65"/>
+      <c r="E46" s="67"/>
+      <c r="F46" s="67"/>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="8"/>
@@ -13228,22 +13238,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="75" t="s">
+      <c r="A47" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="66" t="s">
+      <c r="B47" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="69" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="67" t="s">
+      <c r="E47" s="72" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="69" t="s">
+      <c r="F47" s="74" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13467,14 +13477,14 @@
       <c r="HR47" s="8"/>
     </row>
     <row r="48" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="65"/>
-      <c r="B48" s="65"/>
-      <c r="C48" s="65"/>
+      <c r="A48" s="67"/>
+      <c r="B48" s="67"/>
+      <c r="C48" s="67"/>
       <c r="D48" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="65"/>
-      <c r="F48" s="65"/>
+      <c r="E48" s="67"/>
+      <c r="F48" s="67"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
@@ -13696,20 +13706,20 @@
       <c r="HR48" s="8"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="65"/>
-      <c r="B49" s="66" t="s">
+      <c r="A49" s="67"/>
+      <c r="B49" s="73" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="68" t="s">
+      <c r="C49" s="69" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="67" t="s">
+      <c r="E49" s="72" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="69" t="s">
+      <c r="F49" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13933,14 +13943,14 @@
       <c r="HR49" s="8"/>
     </row>
     <row r="50" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="65"/>
-      <c r="B50" s="65"/>
-      <c r="C50" s="65"/>
+      <c r="A50" s="67"/>
+      <c r="B50" s="67"/>
+      <c r="C50" s="67"/>
       <c r="D50" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="65"/>
-      <c r="F50" s="65"/>
+      <c r="E50" s="67"/>
+      <c r="F50" s="67"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
@@ -14162,22 +14172,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="68" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="66" t="s">
+      <c r="B51" s="73" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="68" t="s">
+      <c r="C51" s="69" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="67" t="s">
+      <c r="E51" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="69" t="s">
+      <c r="F51" s="74" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14401,14 +14411,14 @@
       <c r="HR51" s="8"/>
     </row>
     <row r="52" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="65"/>
-      <c r="B52" s="65"/>
-      <c r="C52" s="65"/>
+      <c r="A52" s="67"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="67"/>
       <c r="D52" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="65"/>
-      <c r="F52" s="65"/>
+      <c r="E52" s="67"/>
+      <c r="F52" s="67"/>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="8"/>
@@ -14630,20 +14640,20 @@
       <c r="HR52" s="8"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="65"/>
-      <c r="B53" s="66" t="s">
+      <c r="A53" s="67"/>
+      <c r="B53" s="73" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="68" t="s">
+      <c r="C53" s="69" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="67" t="s">
+      <c r="E53" s="72" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="69" t="s">
+      <c r="F53" s="74" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14867,14 +14877,14 @@
       <c r="HR53" s="8"/>
     </row>
     <row r="54" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="65"/>
-      <c r="B54" s="65"/>
-      <c r="C54" s="65"/>
+      <c r="A54" s="67"/>
+      <c r="B54" s="67"/>
+      <c r="C54" s="67"/>
       <c r="D54" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="65"/>
-      <c r="F54" s="65"/>
+      <c r="E54" s="67"/>
+      <c r="F54" s="67"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
@@ -15096,22 +15106,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="75" t="s">
+      <c r="A55" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="66" t="s">
+      <c r="B55" s="73" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="68" t="s">
+      <c r="C55" s="69" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="67" t="s">
+      <c r="E55" s="72" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="69" t="s">
+      <c r="F55" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -15335,14 +15345,14 @@
       <c r="HR55" s="8"/>
     </row>
     <row r="56" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="65"/>
-      <c r="B56" s="65"/>
-      <c r="C56" s="65"/>
+      <c r="A56" s="67"/>
+      <c r="B56" s="67"/>
+      <c r="C56" s="67"/>
       <c r="D56" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="65"/>
-      <c r="F56" s="65"/>
+      <c r="E56" s="67"/>
+      <c r="F56" s="67"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
@@ -15564,20 +15574,20 @@
       <c r="HR56" s="8"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="65"/>
-      <c r="B57" s="66" t="s">
+      <c r="A57" s="67"/>
+      <c r="B57" s="73" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="68" t="s">
+      <c r="C57" s="69" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="67" t="s">
+      <c r="E57" s="72" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="69" t="s">
+      <c r="F57" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15801,14 +15811,14 @@
       <c r="HR57" s="8"/>
     </row>
     <row r="58" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="65"/>
-      <c r="B58" s="65"/>
-      <c r="C58" s="65"/>
+      <c r="A58" s="67"/>
+      <c r="B58" s="67"/>
+      <c r="C58" s="67"/>
       <c r="D58" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="65"/>
-      <c r="F58" s="65"/>
+      <c r="E58" s="67"/>
+      <c r="F58" s="67"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
@@ -16030,20 +16040,20 @@
       <c r="HR58" s="8"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="65"/>
-      <c r="B59" s="66" t="s">
+      <c r="A59" s="67"/>
+      <c r="B59" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="68" t="s">
+      <c r="C59" s="69" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="67" t="s">
+      <c r="E59" s="72" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="69" t="s">
+      <c r="F59" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -16267,14 +16277,14 @@
       <c r="HR59" s="8"/>
     </row>
     <row r="60" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="65"/>
-      <c r="B60" s="65"/>
-      <c r="C60" s="65"/>
+      <c r="A60" s="67"/>
+      <c r="B60" s="67"/>
+      <c r="C60" s="67"/>
       <c r="D60" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="65"/>
-      <c r="F60" s="65"/>
+      <c r="E60" s="67"/>
+      <c r="F60" s="67"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
@@ -16496,20 +16506,20 @@
       <c r="HR60" s="8"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="65"/>
-      <c r="B61" s="66" t="s">
+      <c r="A61" s="67"/>
+      <c r="B61" s="73" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="68" t="s">
+      <c r="C61" s="69" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="67" t="s">
+      <c r="E61" s="72" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="69" t="s">
+      <c r="F61" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16733,14 +16743,14 @@
       <c r="HR61" s="8"/>
     </row>
     <row r="62" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="65"/>
-      <c r="B62" s="65"/>
-      <c r="C62" s="65"/>
+      <c r="A62" s="67"/>
+      <c r="B62" s="67"/>
+      <c r="C62" s="67"/>
       <c r="D62" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="65"/>
-      <c r="F62" s="65"/>
+      <c r="E62" s="67"/>
+      <c r="F62" s="67"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
       <c r="I62" s="8"/>
@@ -16962,20 +16972,20 @@
       <c r="HR62" s="8"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="65"/>
-      <c r="B63" s="66" t="s">
+      <c r="A63" s="67"/>
+      <c r="B63" s="73" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="68" t="s">
+      <c r="C63" s="69" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="67" t="s">
+      <c r="E63" s="72" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="69" t="s">
+      <c r="F63" s="74" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -17199,14 +17209,14 @@
       <c r="HR63" s="8"/>
     </row>
     <row r="64" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="65"/>
-      <c r="B64" s="65"/>
-      <c r="C64" s="65"/>
+      <c r="A64" s="67"/>
+      <c r="B64" s="67"/>
+      <c r="C64" s="67"/>
       <c r="D64" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="65"/>
-      <c r="F64" s="65"/>
+      <c r="E64" s="67"/>
+      <c r="F64" s="67"/>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
@@ -17428,20 +17438,20 @@
       <c r="HR64" s="8"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="65"/>
-      <c r="B65" s="66" t="s">
+      <c r="A65" s="67"/>
+      <c r="B65" s="73" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="68" t="s">
+      <c r="C65" s="69" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="67" t="s">
+      <c r="E65" s="72" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="69" t="s">
+      <c r="F65" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17665,14 +17675,14 @@
       <c r="HR65" s="8"/>
     </row>
     <row r="66" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="65"/>
-      <c r="B66" s="65"/>
-      <c r="C66" s="65"/>
+      <c r="A66" s="67"/>
+      <c r="B66" s="67"/>
+      <c r="C66" s="67"/>
       <c r="D66" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="65"/>
-      <c r="F66" s="65"/>
+      <c r="E66" s="67"/>
+      <c r="F66" s="67"/>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
@@ -17894,22 +17904,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="75" t="s">
+      <c r="A67" s="68" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="66" t="s">
+      <c r="B67" s="73" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="68" t="s">
+      <c r="C67" s="69" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="67" t="s">
+      <c r="E67" s="72" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="69" t="s">
+      <c r="F67" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -18133,14 +18143,14 @@
       <c r="HR67" s="8"/>
     </row>
     <row r="68" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="65"/>
-      <c r="B68" s="65"/>
-      <c r="C68" s="65"/>
+      <c r="A68" s="67"/>
+      <c r="B68" s="67"/>
+      <c r="C68" s="67"/>
       <c r="D68" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="65"/>
-      <c r="F68" s="65"/>
+      <c r="E68" s="67"/>
+      <c r="F68" s="67"/>
       <c r="G68" s="8"/>
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
@@ -18362,20 +18372,20 @@
       <c r="HR68" s="8"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="65"/>
-      <c r="B69" s="66" t="s">
+      <c r="A69" s="67"/>
+      <c r="B69" s="73" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="68" t="s">
+      <c r="C69" s="69" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="67" t="s">
+      <c r="E69" s="72" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="69" t="s">
+      <c r="F69" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18600,14 +18610,14 @@
       <c r="HR69" s="8"/>
     </row>
     <row r="70" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="65"/>
-      <c r="B70" s="65"/>
-      <c r="C70" s="65"/>
+      <c r="A70" s="67"/>
+      <c r="B70" s="67"/>
+      <c r="C70" s="67"/>
       <c r="D70" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="65"/>
-      <c r="F70" s="65"/>
+      <c r="E70" s="67"/>
+      <c r="F70" s="67"/>
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
       <c r="I70" s="8"/>
@@ -18829,20 +18839,20 @@
       <c r="HR70" s="8"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="65"/>
-      <c r="B71" s="66" t="s">
+      <c r="A71" s="67"/>
+      <c r="B71" s="73" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="68" t="s">
+      <c r="C71" s="69" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="67" t="s">
+      <c r="E71" s="72" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="69" t="s">
+      <c r="F71" s="74" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -19066,14 +19076,14 @@
       <c r="HR71" s="8"/>
     </row>
     <row r="72" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="65"/>
-      <c r="B72" s="65"/>
-      <c r="C72" s="65"/>
+      <c r="A72" s="67"/>
+      <c r="B72" s="67"/>
+      <c r="C72" s="67"/>
       <c r="D72" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="65"/>
-      <c r="F72" s="65"/>
+      <c r="E72" s="67"/>
+      <c r="F72" s="67"/>
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
@@ -19295,20 +19305,20 @@
       <c r="HR72" s="8"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="65"/>
-      <c r="B73" s="66" t="s">
+      <c r="A73" s="67"/>
+      <c r="B73" s="73" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="68" t="s">
+      <c r="C73" s="69" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="67" t="s">
+      <c r="E73" s="72" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="69" t="s">
+      <c r="F73" s="74" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19532,14 +19542,14 @@
       <c r="HR73" s="8"/>
     </row>
     <row r="74" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="65"/>
-      <c r="B74" s="65"/>
-      <c r="C74" s="65"/>
+      <c r="A74" s="67"/>
+      <c r="B74" s="67"/>
+      <c r="C74" s="67"/>
       <c r="D74" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="65"/>
-      <c r="F74" s="65"/>
+      <c r="E74" s="67"/>
+      <c r="F74" s="67"/>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>
@@ -19761,20 +19771,20 @@
       <c r="HR74" s="8"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="65"/>
-      <c r="B75" s="66" t="s">
+      <c r="A75" s="67"/>
+      <c r="B75" s="73" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="68" t="s">
+      <c r="C75" s="69" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="67" t="s">
+      <c r="E75" s="72" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="69" t="s">
+      <c r="F75" s="74" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19998,14 +20008,14 @@
       <c r="HR75" s="8"/>
     </row>
     <row r="76" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="65"/>
-      <c r="B76" s="65"/>
-      <c r="C76" s="65"/>
+      <c r="A76" s="67"/>
+      <c r="B76" s="67"/>
+      <c r="C76" s="67"/>
       <c r="D76" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="65"/>
-      <c r="F76" s="65"/>
+      <c r="E76" s="67"/>
+      <c r="F76" s="67"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
       <c r="I76" s="8"/>
@@ -20227,20 +20237,20 @@
       <c r="HR76" s="8"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="65"/>
-      <c r="B77" s="66" t="s">
+      <c r="A77" s="67"/>
+      <c r="B77" s="73" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="68" t="s">
+      <c r="C77" s="69" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="67" t="s">
+      <c r="E77" s="72" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="69" t="s">
+      <c r="F77" s="74" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20464,14 +20474,14 @@
       <c r="HR77" s="8"/>
     </row>
     <row r="78" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="65"/>
-      <c r="B78" s="65"/>
-      <c r="C78" s="65"/>
+      <c r="A78" s="67"/>
+      <c r="B78" s="67"/>
+      <c r="C78" s="67"/>
       <c r="D78" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="65"/>
-      <c r="F78" s="65"/>
+      <c r="E78" s="67"/>
+      <c r="F78" s="67"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
       <c r="I78" s="8"/>
@@ -20693,22 +20703,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="75" t="s">
+      <c r="A79" s="68" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="66" t="s">
+      <c r="B79" s="73" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="64" t="s">
+      <c r="C79" s="76" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="67" t="s">
+      <c r="E79" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="69" t="s">
+      <c r="F79" s="74" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20932,14 +20942,14 @@
       <c r="HR79" s="8"/>
     </row>
     <row r="80" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="65"/>
-      <c r="B80" s="65"/>
-      <c r="C80" s="65"/>
+      <c r="A80" s="67"/>
+      <c r="B80" s="67"/>
+      <c r="C80" s="67"/>
       <c r="D80" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="65"/>
-      <c r="F80" s="65"/>
+      <c r="E80" s="67"/>
+      <c r="F80" s="67"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
       <c r="I80" s="8"/>
@@ -21161,20 +21171,20 @@
       <c r="HR80" s="8"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="65"/>
-      <c r="B81" s="66" t="s">
+      <c r="A81" s="67"/>
+      <c r="B81" s="73" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="64" t="s">
+      <c r="C81" s="76" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="67" t="s">
+      <c r="E81" s="72" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="69" t="s">
+      <c r="F81" s="74" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -21398,14 +21408,14 @@
       <c r="HR81" s="8"/>
     </row>
     <row r="82" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="65"/>
-      <c r="B82" s="65"/>
-      <c r="C82" s="65"/>
+      <c r="A82" s="67"/>
+      <c r="B82" s="67"/>
+      <c r="C82" s="67"/>
       <c r="D82" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="65"/>
-      <c r="F82" s="65"/>
+      <c r="E82" s="67"/>
+      <c r="F82" s="67"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
       <c r="I82" s="8"/>
@@ -21627,20 +21637,20 @@
       <c r="HR82" s="8"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="65"/>
-      <c r="B83" s="66" t="s">
+      <c r="A83" s="67"/>
+      <c r="B83" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="68" t="s">
+      <c r="C83" s="69" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="67" t="s">
+      <c r="E83" s="72" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="69" t="s">
+      <c r="F83" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21864,14 +21874,14 @@
       <c r="HR83" s="8"/>
     </row>
     <row r="84" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="65"/>
-      <c r="B84" s="65"/>
-      <c r="C84" s="65"/>
+      <c r="A84" s="67"/>
+      <c r="B84" s="67"/>
+      <c r="C84" s="67"/>
       <c r="D84" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="65"/>
-      <c r="F84" s="65"/>
+      <c r="E84" s="67"/>
+      <c r="F84" s="67"/>
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
@@ -22093,20 +22103,20 @@
       <c r="HR84" s="8"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="65"/>
-      <c r="B85" s="66" t="s">
+      <c r="A85" s="67"/>
+      <c r="B85" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="77" t="s">
+      <c r="C85" s="80" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="67" t="s">
+      <c r="E85" s="72" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="69"/>
+      <c r="F85" s="74"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -22328,14 +22338,14 @@
       <c r="HR85" s="17"/>
     </row>
     <row r="86" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="65"/>
-      <c r="B86" s="65"/>
-      <c r="C86" s="65"/>
+      <c r="A86" s="67"/>
+      <c r="B86" s="67"/>
+      <c r="C86" s="67"/>
       <c r="D86" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="65"/>
-      <c r="F86" s="65"/>
+      <c r="E86" s="67"/>
+      <c r="F86" s="67"/>
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
@@ -22558,20 +22568,173 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="GU1:HA1"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
     <mergeCell ref="E85:E86"/>
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="B85:B86"/>
@@ -22596,173 +22759,20 @@
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="GU1:HA1"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Profiling auf gpu ausgewertet
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86F4B1B-EA88-4513-BCC0-E9BB17578C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4742DE79-2CBF-406F-A180-C1578FC8EC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
@@ -1042,7 +1042,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1125,8 +1125,8 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
@@ -1134,8 +1134,8 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="hair">
@@ -1143,31 +1143,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1259,6 +1239,57 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1266,57 +1297,9 @@
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1629,298 +1612,300 @@
     <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
     <col min="7" max="41" width="2.140625" customWidth="1"/>
-    <col min="42" max="42" width="2.140625" style="60" customWidth="1"/>
-    <col min="43" max="226" width="2.140625" customWidth="1"/>
+    <col min="42" max="42" width="2.140625" style="57" customWidth="1"/>
+    <col min="43" max="45" width="2.140625" customWidth="1"/>
+    <col min="46" max="46" width="2.140625" style="83" customWidth="1"/>
+    <col min="47" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="66" t="s">
+      <c r="G1" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="66" t="s">
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="66" t="s">
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="82" t="s">
+      <c r="V1" s="59"/>
+      <c r="W1" s="59"/>
+      <c r="X1" s="59"/>
+      <c r="Y1" s="59"/>
+      <c r="Z1" s="59"/>
+      <c r="AA1" s="59"/>
+      <c r="AB1" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67"/>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="67"/>
-      <c r="AI1" s="66" t="s">
+      <c r="AC1" s="59"/>
+      <c r="AD1" s="59"/>
+      <c r="AE1" s="59"/>
+      <c r="AF1" s="59"/>
+      <c r="AG1" s="59"/>
+      <c r="AH1" s="59"/>
+      <c r="AI1" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="67"/>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="66" t="s">
+      <c r="AJ1" s="59"/>
+      <c r="AK1" s="59"/>
+      <c r="AL1" s="59"/>
+      <c r="AM1" s="59"/>
+      <c r="AN1" s="59"/>
+      <c r="AO1" s="59"/>
+      <c r="AP1" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="67"/>
-      <c r="AU1" s="67"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="66" t="s">
+      <c r="AQ1" s="59"/>
+      <c r="AR1" s="59"/>
+      <c r="AS1" s="59"/>
+      <c r="AT1" s="59"/>
+      <c r="AU1" s="59"/>
+      <c r="AV1" s="59"/>
+      <c r="AW1" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="67"/>
-      <c r="AY1" s="67"/>
-      <c r="AZ1" s="67"/>
-      <c r="BA1" s="67"/>
-      <c r="BB1" s="67"/>
-      <c r="BC1" s="67"/>
-      <c r="BD1" s="66" t="s">
+      <c r="AX1" s="59"/>
+      <c r="AY1" s="59"/>
+      <c r="AZ1" s="59"/>
+      <c r="BA1" s="59"/>
+      <c r="BB1" s="59"/>
+      <c r="BC1" s="59"/>
+      <c r="BD1" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="67"/>
-      <c r="BF1" s="67"/>
-      <c r="BG1" s="67"/>
-      <c r="BH1" s="67"/>
-      <c r="BI1" s="67"/>
-      <c r="BJ1" s="67"/>
-      <c r="BK1" s="66" t="s">
+      <c r="BE1" s="59"/>
+      <c r="BF1" s="59"/>
+      <c r="BG1" s="59"/>
+      <c r="BH1" s="59"/>
+      <c r="BI1" s="59"/>
+      <c r="BJ1" s="59"/>
+      <c r="BK1" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="67"/>
-      <c r="BM1" s="67"/>
-      <c r="BN1" s="67"/>
-      <c r="BO1" s="67"/>
-      <c r="BP1" s="67"/>
-      <c r="BQ1" s="67"/>
-      <c r="BR1" s="66" t="s">
+      <c r="BL1" s="59"/>
+      <c r="BM1" s="59"/>
+      <c r="BN1" s="59"/>
+      <c r="BO1" s="59"/>
+      <c r="BP1" s="59"/>
+      <c r="BQ1" s="59"/>
+      <c r="BR1" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="67"/>
-      <c r="BT1" s="67"/>
-      <c r="BU1" s="67"/>
-      <c r="BV1" s="67"/>
-      <c r="BW1" s="67"/>
-      <c r="BX1" s="67"/>
-      <c r="BY1" s="66" t="s">
+      <c r="BS1" s="59"/>
+      <c r="BT1" s="59"/>
+      <c r="BU1" s="59"/>
+      <c r="BV1" s="59"/>
+      <c r="BW1" s="59"/>
+      <c r="BX1" s="59"/>
+      <c r="BY1" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="67"/>
-      <c r="CA1" s="67"/>
-      <c r="CB1" s="67"/>
-      <c r="CC1" s="67"/>
-      <c r="CD1" s="67"/>
-      <c r="CE1" s="67"/>
-      <c r="CF1" s="66" t="s">
+      <c r="BZ1" s="59"/>
+      <c r="CA1" s="59"/>
+      <c r="CB1" s="59"/>
+      <c r="CC1" s="59"/>
+      <c r="CD1" s="59"/>
+      <c r="CE1" s="59"/>
+      <c r="CF1" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="67"/>
-      <c r="CH1" s="67"/>
-      <c r="CI1" s="67"/>
-      <c r="CJ1" s="67"/>
-      <c r="CK1" s="67"/>
-      <c r="CL1" s="67"/>
-      <c r="CM1" s="66" t="s">
+      <c r="CG1" s="59"/>
+      <c r="CH1" s="59"/>
+      <c r="CI1" s="59"/>
+      <c r="CJ1" s="59"/>
+      <c r="CK1" s="59"/>
+      <c r="CL1" s="59"/>
+      <c r="CM1" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="67"/>
-      <c r="CO1" s="67"/>
-      <c r="CP1" s="67"/>
-      <c r="CQ1" s="67"/>
-      <c r="CR1" s="67"/>
-      <c r="CS1" s="67"/>
-      <c r="CT1" s="66" t="s">
+      <c r="CN1" s="59"/>
+      <c r="CO1" s="59"/>
+      <c r="CP1" s="59"/>
+      <c r="CQ1" s="59"/>
+      <c r="CR1" s="59"/>
+      <c r="CS1" s="59"/>
+      <c r="CT1" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="67"/>
-      <c r="CV1" s="67"/>
-      <c r="CW1" s="67"/>
-      <c r="CX1" s="67"/>
-      <c r="CY1" s="67"/>
-      <c r="CZ1" s="67"/>
-      <c r="DA1" s="66" t="s">
+      <c r="CU1" s="59"/>
+      <c r="CV1" s="59"/>
+      <c r="CW1" s="59"/>
+      <c r="CX1" s="59"/>
+      <c r="CY1" s="59"/>
+      <c r="CZ1" s="59"/>
+      <c r="DA1" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="67"/>
-      <c r="DC1" s="67"/>
-      <c r="DD1" s="67"/>
-      <c r="DE1" s="67"/>
-      <c r="DF1" s="67"/>
-      <c r="DG1" s="67"/>
-      <c r="DH1" s="66" t="s">
+      <c r="DB1" s="59"/>
+      <c r="DC1" s="59"/>
+      <c r="DD1" s="59"/>
+      <c r="DE1" s="59"/>
+      <c r="DF1" s="59"/>
+      <c r="DG1" s="59"/>
+      <c r="DH1" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="67"/>
-      <c r="DJ1" s="67"/>
-      <c r="DK1" s="67"/>
-      <c r="DL1" s="67"/>
-      <c r="DM1" s="67"/>
-      <c r="DN1" s="67"/>
-      <c r="DO1" s="66" t="s">
+      <c r="DI1" s="59"/>
+      <c r="DJ1" s="59"/>
+      <c r="DK1" s="59"/>
+      <c r="DL1" s="59"/>
+      <c r="DM1" s="59"/>
+      <c r="DN1" s="59"/>
+      <c r="DO1" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="67"/>
-      <c r="DQ1" s="67"/>
-      <c r="DR1" s="67"/>
-      <c r="DS1" s="67"/>
-      <c r="DT1" s="67"/>
-      <c r="DU1" s="67"/>
-      <c r="DV1" s="66" t="s">
+      <c r="DP1" s="59"/>
+      <c r="DQ1" s="59"/>
+      <c r="DR1" s="59"/>
+      <c r="DS1" s="59"/>
+      <c r="DT1" s="59"/>
+      <c r="DU1" s="59"/>
+      <c r="DV1" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="67"/>
-      <c r="DX1" s="67"/>
-      <c r="DY1" s="67"/>
-      <c r="DZ1" s="67"/>
-      <c r="EA1" s="67"/>
-      <c r="EB1" s="67"/>
-      <c r="EC1" s="66" t="s">
+      <c r="DW1" s="59"/>
+      <c r="DX1" s="59"/>
+      <c r="DY1" s="59"/>
+      <c r="DZ1" s="59"/>
+      <c r="EA1" s="59"/>
+      <c r="EB1" s="59"/>
+      <c r="EC1" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="67"/>
-      <c r="EE1" s="67"/>
-      <c r="EF1" s="67"/>
-      <c r="EG1" s="67"/>
-      <c r="EH1" s="67"/>
-      <c r="EI1" s="67"/>
-      <c r="EJ1" s="66" t="s">
+      <c r="ED1" s="59"/>
+      <c r="EE1" s="59"/>
+      <c r="EF1" s="59"/>
+      <c r="EG1" s="59"/>
+      <c r="EH1" s="59"/>
+      <c r="EI1" s="59"/>
+      <c r="EJ1" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="67"/>
-      <c r="EL1" s="67"/>
-      <c r="EM1" s="67"/>
-      <c r="EN1" s="67"/>
-      <c r="EO1" s="67"/>
-      <c r="EP1" s="67"/>
-      <c r="EQ1" s="66" t="s">
+      <c r="EK1" s="59"/>
+      <c r="EL1" s="59"/>
+      <c r="EM1" s="59"/>
+      <c r="EN1" s="59"/>
+      <c r="EO1" s="59"/>
+      <c r="EP1" s="59"/>
+      <c r="EQ1" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="67"/>
-      <c r="ES1" s="67"/>
-      <c r="ET1" s="67"/>
-      <c r="EU1" s="67"/>
-      <c r="EV1" s="67"/>
-      <c r="EW1" s="67"/>
-      <c r="EX1" s="66" t="s">
+      <c r="ER1" s="59"/>
+      <c r="ES1" s="59"/>
+      <c r="ET1" s="59"/>
+      <c r="EU1" s="59"/>
+      <c r="EV1" s="59"/>
+      <c r="EW1" s="59"/>
+      <c r="EX1" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="67"/>
-      <c r="EZ1" s="67"/>
-      <c r="FA1" s="67"/>
-      <c r="FB1" s="67"/>
-      <c r="FC1" s="67"/>
-      <c r="FD1" s="67"/>
-      <c r="FE1" s="66" t="s">
+      <c r="EY1" s="59"/>
+      <c r="EZ1" s="59"/>
+      <c r="FA1" s="59"/>
+      <c r="FB1" s="59"/>
+      <c r="FC1" s="59"/>
+      <c r="FD1" s="59"/>
+      <c r="FE1" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="67"/>
-      <c r="FG1" s="67"/>
-      <c r="FH1" s="67"/>
-      <c r="FI1" s="67"/>
-      <c r="FJ1" s="67"/>
-      <c r="FK1" s="67"/>
-      <c r="FL1" s="66" t="s">
+      <c r="FF1" s="59"/>
+      <c r="FG1" s="59"/>
+      <c r="FH1" s="59"/>
+      <c r="FI1" s="59"/>
+      <c r="FJ1" s="59"/>
+      <c r="FK1" s="59"/>
+      <c r="FL1" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="67"/>
-      <c r="FN1" s="67"/>
-      <c r="FO1" s="67"/>
-      <c r="FP1" s="67"/>
-      <c r="FQ1" s="67"/>
-      <c r="FR1" s="67"/>
-      <c r="FS1" s="66" t="s">
+      <c r="FM1" s="59"/>
+      <c r="FN1" s="59"/>
+      <c r="FO1" s="59"/>
+      <c r="FP1" s="59"/>
+      <c r="FQ1" s="59"/>
+      <c r="FR1" s="59"/>
+      <c r="FS1" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="67"/>
-      <c r="FU1" s="67"/>
-      <c r="FV1" s="67"/>
-      <c r="FW1" s="67"/>
-      <c r="FX1" s="67"/>
-      <c r="FY1" s="67"/>
-      <c r="FZ1" s="66" t="s">
+      <c r="FT1" s="59"/>
+      <c r="FU1" s="59"/>
+      <c r="FV1" s="59"/>
+      <c r="FW1" s="59"/>
+      <c r="FX1" s="59"/>
+      <c r="FY1" s="59"/>
+      <c r="FZ1" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="67"/>
-      <c r="GB1" s="67"/>
-      <c r="GC1" s="67"/>
-      <c r="GD1" s="67"/>
-      <c r="GE1" s="67"/>
-      <c r="GF1" s="67"/>
-      <c r="GG1" s="66" t="s">
+      <c r="GA1" s="59"/>
+      <c r="GB1" s="59"/>
+      <c r="GC1" s="59"/>
+      <c r="GD1" s="59"/>
+      <c r="GE1" s="59"/>
+      <c r="GF1" s="59"/>
+      <c r="GG1" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="67"/>
-      <c r="GI1" s="67"/>
-      <c r="GJ1" s="67"/>
-      <c r="GK1" s="67"/>
-      <c r="GL1" s="67"/>
-      <c r="GM1" s="67"/>
-      <c r="GN1" s="66" t="s">
+      <c r="GH1" s="59"/>
+      <c r="GI1" s="59"/>
+      <c r="GJ1" s="59"/>
+      <c r="GK1" s="59"/>
+      <c r="GL1" s="59"/>
+      <c r="GM1" s="59"/>
+      <c r="GN1" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="67"/>
-      <c r="GP1" s="67"/>
-      <c r="GQ1" s="67"/>
-      <c r="GR1" s="67"/>
-      <c r="GS1" s="67"/>
-      <c r="GT1" s="67"/>
-      <c r="GU1" s="66" t="s">
+      <c r="GO1" s="59"/>
+      <c r="GP1" s="59"/>
+      <c r="GQ1" s="59"/>
+      <c r="GR1" s="59"/>
+      <c r="GS1" s="59"/>
+      <c r="GT1" s="59"/>
+      <c r="GU1" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="67"/>
-      <c r="GW1" s="67"/>
-      <c r="GX1" s="67"/>
-      <c r="GY1" s="67"/>
-      <c r="GZ1" s="67"/>
-      <c r="HA1" s="67"/>
-      <c r="HB1" s="66" t="s">
+      <c r="GV1" s="59"/>
+      <c r="GW1" s="59"/>
+      <c r="GX1" s="59"/>
+      <c r="GY1" s="59"/>
+      <c r="GZ1" s="59"/>
+      <c r="HA1" s="59"/>
+      <c r="HB1" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="67"/>
-      <c r="HD1" s="67"/>
-      <c r="HE1" s="67"/>
-      <c r="HF1" s="67"/>
-      <c r="HG1" s="67"/>
-      <c r="HH1" s="67"/>
-      <c r="HI1" s="66" t="s">
+      <c r="HC1" s="59"/>
+      <c r="HD1" s="59"/>
+      <c r="HE1" s="59"/>
+      <c r="HF1" s="59"/>
+      <c r="HG1" s="59"/>
+      <c r="HH1" s="59"/>
+      <c r="HI1" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="67"/>
-      <c r="HK1" s="67"/>
-      <c r="HL1" s="67"/>
-      <c r="HM1" s="67"/>
-      <c r="HN1" s="67"/>
-      <c r="HO1" s="67"/>
-      <c r="HP1" s="66" t="s">
+      <c r="HJ1" s="59"/>
+      <c r="HK1" s="59"/>
+      <c r="HL1" s="59"/>
+      <c r="HM1" s="59"/>
+      <c r="HN1" s="59"/>
+      <c r="HO1" s="59"/>
+      <c r="HP1" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="67"/>
-      <c r="HR1" s="67"/>
+      <c r="HQ1" s="59"/>
+      <c r="HR1" s="59"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="1" t="s">
@@ -2031,7 +2016,7 @@
       <c r="AO2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AP2" s="57" t="s">
+      <c r="AP2" s="77" t="s">
         <v>34</v>
       </c>
       <c r="AQ2" s="2" t="s">
@@ -2043,7 +2028,7 @@
       <c r="AS2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AT2" s="2" t="s">
+      <c r="AT2" s="78" t="s">
         <v>36</v>
       </c>
       <c r="AU2" s="2" t="s">
@@ -2696,7 +2681,7 @@
       <c r="AO3" s="3">
         <v>46285</v>
       </c>
-      <c r="AP3" s="58">
+      <c r="AP3" s="50">
         <v>46286</v>
       </c>
       <c r="AQ3" s="3">
@@ -2708,7 +2693,7 @@
       <c r="AS3" s="3">
         <v>46289</v>
       </c>
-      <c r="AT3" s="3">
+      <c r="AT3" s="79">
         <v>46290</v>
       </c>
       <c r="AU3" s="3">
@@ -3304,11 +3289,11 @@
       <c r="AM4" s="5"/>
       <c r="AN4" s="5"/>
       <c r="AO4" s="5"/>
-      <c r="AP4" s="59"/>
+      <c r="AP4" s="51"/>
       <c r="AQ4" s="5"/>
       <c r="AR4" s="5"/>
       <c r="AS4" s="5"/>
-      <c r="AT4" s="5"/>
+      <c r="AT4" s="80"/>
       <c r="AU4" s="5"/>
       <c r="AV4" s="5"/>
       <c r="AW4" s="5"/>
@@ -3491,20 +3476,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="74" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="70" t="s">
+      <c r="B5" s="70"/>
+      <c r="C5" s="68" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="75" t="s">
+      <c r="E5" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="79"/>
+      <c r="F5" s="66"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3539,11 +3524,11 @@
       <c r="AL5" s="8"/>
       <c r="AM5" s="9"/>
       <c r="AN5" s="10"/>
-      <c r="AO5" s="11"/>
+      <c r="AO5" s="47"/>
       <c r="AQ5" s="8"/>
       <c r="AR5" s="8"/>
       <c r="AS5" s="8"/>
-      <c r="AT5" s="9"/>
+      <c r="AT5" s="81"/>
       <c r="AU5" s="10"/>
       <c r="AV5" s="11"/>
       <c r="AW5" s="8"/>
@@ -3726,14 +3711,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="71"/>
-      <c r="B6" s="71"/>
-      <c r="C6" s="71"/>
+      <c r="A6" s="67"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3768,11 +3753,11 @@
       <c r="AL6" s="8"/>
       <c r="AM6" s="9"/>
       <c r="AN6" s="10"/>
-      <c r="AO6" s="11"/>
+      <c r="AO6" s="47"/>
       <c r="AQ6" s="8"/>
       <c r="AR6" s="8"/>
       <c r="AS6" s="8"/>
-      <c r="AT6" s="9"/>
+      <c r="AT6" s="81"/>
       <c r="AU6" s="10"/>
       <c r="AV6" s="11"/>
       <c r="AW6" s="8"/>
@@ -3955,18 +3940,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="71"/>
-      <c r="B7" s="77"/>
-      <c r="C7" s="70" t="s">
+      <c r="A7" s="67"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="68" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="75" t="s">
+      <c r="E7" s="72" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="79"/>
+      <c r="F7" s="66"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -4001,11 +3986,11 @@
       <c r="AL7" s="8"/>
       <c r="AM7" s="9"/>
       <c r="AN7" s="10"/>
-      <c r="AO7" s="11"/>
+      <c r="AO7" s="47"/>
       <c r="AQ7" s="8"/>
       <c r="AR7" s="8"/>
       <c r="AS7" s="8"/>
-      <c r="AT7" s="9"/>
+      <c r="AT7" s="81"/>
       <c r="AU7" s="10"/>
       <c r="AV7" s="11"/>
       <c r="AW7" s="8"/>
@@ -4188,14 +4173,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="71"/>
-      <c r="B8" s="71"/>
-      <c r="C8" s="71"/>
+      <c r="A8" s="67"/>
+      <c r="B8" s="67"/>
+      <c r="C8" s="67"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4230,11 +4215,11 @@
       <c r="AL8" s="8"/>
       <c r="AM8" s="9"/>
       <c r="AN8" s="10"/>
-      <c r="AO8" s="11"/>
+      <c r="AO8" s="47"/>
       <c r="AQ8" s="8"/>
       <c r="AR8" s="8"/>
       <c r="AS8" s="8"/>
-      <c r="AT8" s="9"/>
+      <c r="AT8" s="81"/>
       <c r="AU8" s="10"/>
       <c r="AV8" s="11"/>
       <c r="AW8" s="8"/>
@@ -4417,18 +4402,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="71"/>
-      <c r="B9" s="77"/>
-      <c r="C9" s="70" t="s">
+      <c r="A9" s="67"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="68" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="75" t="s">
+      <c r="E9" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="79"/>
+      <c r="F9" s="66"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4463,11 +4448,11 @@
       <c r="AL9" s="8"/>
       <c r="AM9" s="9"/>
       <c r="AN9" s="10"/>
-      <c r="AO9" s="11"/>
+      <c r="AO9" s="47"/>
       <c r="AQ9" s="8"/>
       <c r="AR9" s="8"/>
       <c r="AS9" s="8"/>
-      <c r="AT9" s="9"/>
+      <c r="AT9" s="81"/>
       <c r="AU9" s="10"/>
       <c r="AV9" s="11"/>
       <c r="AW9" s="8"/>
@@ -4650,14 +4635,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="71"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
+      <c r="A10" s="67"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="67"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="71"/>
-      <c r="F10" s="71"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="67"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4692,11 +4677,11 @@
       <c r="AL10" s="8"/>
       <c r="AM10" s="9"/>
       <c r="AN10" s="10"/>
-      <c r="AO10" s="11"/>
+      <c r="AO10" s="47"/>
       <c r="AQ10" s="8"/>
       <c r="AR10" s="8"/>
       <c r="AS10" s="8"/>
-      <c r="AT10" s="9"/>
+      <c r="AT10" s="81"/>
       <c r="AU10" s="10"/>
       <c r="AV10" s="11"/>
       <c r="AW10" s="8"/>
@@ -4879,18 +4864,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="71"/>
-      <c r="B11" s="77"/>
-      <c r="C11" s="70" t="s">
+      <c r="A11" s="67"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="68" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="75" t="s">
+      <c r="E11" s="72" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="79"/>
+      <c r="F11" s="66"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -4925,11 +4910,11 @@
       <c r="AL11" s="8"/>
       <c r="AM11" s="9"/>
       <c r="AN11" s="10"/>
-      <c r="AO11" s="11"/>
+      <c r="AO11" s="47"/>
       <c r="AQ11" s="8"/>
       <c r="AR11" s="8"/>
       <c r="AS11" s="8"/>
-      <c r="AT11" s="9"/>
+      <c r="AT11" s="81"/>
       <c r="AU11" s="10"/>
       <c r="AV11" s="11"/>
       <c r="AW11" s="8"/>
@@ -5112,14 +5097,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="71"/>
-      <c r="B12" s="71"/>
-      <c r="C12" s="71"/>
+      <c r="A12" s="67"/>
+      <c r="B12" s="67"/>
+      <c r="C12" s="67"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="71"/>
-      <c r="F12" s="71"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="67"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5154,11 +5139,11 @@
       <c r="AL12" s="8"/>
       <c r="AM12" s="9"/>
       <c r="AN12" s="10"/>
-      <c r="AO12" s="11"/>
+      <c r="AO12" s="47"/>
       <c r="AQ12" s="8"/>
       <c r="AR12" s="8"/>
       <c r="AS12" s="8"/>
-      <c r="AT12" s="9"/>
+      <c r="AT12" s="81"/>
       <c r="AU12" s="10"/>
       <c r="AV12" s="11"/>
       <c r="AW12" s="8"/>
@@ -5341,18 +5326,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="71"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="70" t="s">
+      <c r="A13" s="67"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="68" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="75" t="s">
+      <c r="E13" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="79"/>
+      <c r="F13" s="66"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5387,11 +5372,11 @@
       <c r="AL13" s="8"/>
       <c r="AM13" s="9"/>
       <c r="AN13" s="10"/>
-      <c r="AO13" s="11"/>
+      <c r="AO13" s="47"/>
       <c r="AQ13" s="8"/>
       <c r="AR13" s="8"/>
       <c r="AS13" s="8"/>
-      <c r="AT13" s="9"/>
+      <c r="AT13" s="81"/>
       <c r="AU13" s="10"/>
       <c r="AV13" s="11"/>
       <c r="AW13" s="8"/>
@@ -5574,14 +5559,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="71"/>
-      <c r="B14" s="71"/>
-      <c r="C14" s="71"/>
+      <c r="A14" s="67"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="67"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="71"/>
-      <c r="F14" s="71"/>
+      <c r="E14" s="67"/>
+      <c r="F14" s="67"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5616,11 +5601,11 @@
       <c r="AL14" s="8"/>
       <c r="AM14" s="9"/>
       <c r="AN14" s="10"/>
-      <c r="AO14" s="11"/>
+      <c r="AO14" s="47"/>
       <c r="AQ14" s="8"/>
       <c r="AR14" s="8"/>
       <c r="AS14" s="8"/>
-      <c r="AT14" s="9"/>
+      <c r="AT14" s="81"/>
       <c r="AU14" s="10"/>
       <c r="AV14" s="11"/>
       <c r="AW14" s="8"/>
@@ -5803,18 +5788,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="71"/>
-      <c r="B15" s="77"/>
-      <c r="C15" s="70" t="s">
+      <c r="A15" s="67"/>
+      <c r="B15" s="70"/>
+      <c r="C15" s="68" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="75" t="s">
+      <c r="E15" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="79"/>
+      <c r="F15" s="66"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -5849,11 +5834,11 @@
       <c r="AL15" s="8"/>
       <c r="AM15" s="9"/>
       <c r="AN15" s="10"/>
-      <c r="AO15" s="11"/>
+      <c r="AO15" s="47"/>
       <c r="AQ15" s="8"/>
       <c r="AR15" s="8"/>
       <c r="AS15" s="8"/>
-      <c r="AT15" s="9"/>
+      <c r="AT15" s="81"/>
       <c r="AU15" s="10"/>
       <c r="AV15" s="11"/>
       <c r="AW15" s="8"/>
@@ -6036,14 +6021,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="71"/>
-      <c r="B16" s="71"/>
-      <c r="C16" s="71"/>
+      <c r="A16" s="67"/>
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="71"/>
-      <c r="F16" s="71"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6078,11 +6063,11 @@
       <c r="AL16" s="8"/>
       <c r="AM16" s="9"/>
       <c r="AN16" s="10"/>
-      <c r="AO16" s="11"/>
+      <c r="AO16" s="47"/>
       <c r="AQ16" s="8"/>
       <c r="AR16" s="8"/>
       <c r="AS16" s="8"/>
-      <c r="AT16" s="9"/>
+      <c r="AT16" s="81"/>
       <c r="AU16" s="10"/>
       <c r="AV16" s="11"/>
       <c r="AW16" s="8"/>
@@ -6265,18 +6250,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="71"/>
-      <c r="B17" s="77"/>
-      <c r="C17" s="70" t="s">
+      <c r="A17" s="67"/>
+      <c r="B17" s="70"/>
+      <c r="C17" s="68" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="75" t="s">
+      <c r="E17" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="79"/>
+      <c r="F17" s="66"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6311,11 +6296,11 @@
       <c r="AL17" s="8"/>
       <c r="AM17" s="9"/>
       <c r="AN17" s="10"/>
-      <c r="AO17" s="11"/>
+      <c r="AO17" s="47"/>
       <c r="AQ17" s="8"/>
       <c r="AR17" s="8"/>
       <c r="AS17" s="8"/>
-      <c r="AT17" s="9"/>
+      <c r="AT17" s="81"/>
       <c r="AU17" s="10"/>
       <c r="AV17" s="11"/>
       <c r="AW17" s="8"/>
@@ -6498,14 +6483,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="71"/>
-      <c r="B18" s="71"/>
-      <c r="C18" s="71"/>
+      <c r="A18" s="67"/>
+      <c r="B18" s="67"/>
+      <c r="C18" s="67"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="71"/>
-      <c r="F18" s="71"/>
+      <c r="E18" s="67"/>
+      <c r="F18" s="67"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6540,11 +6525,11 @@
       <c r="AL18" s="8"/>
       <c r="AM18" s="9"/>
       <c r="AN18" s="10"/>
-      <c r="AO18" s="11"/>
+      <c r="AO18" s="47"/>
       <c r="AQ18" s="8"/>
       <c r="AR18" s="8"/>
       <c r="AS18" s="8"/>
-      <c r="AT18" s="9"/>
+      <c r="AT18" s="81"/>
       <c r="AU18" s="10"/>
       <c r="AV18" s="11"/>
       <c r="AW18" s="8"/>
@@ -6727,18 +6712,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="71"/>
-      <c r="B19" s="77"/>
-      <c r="C19" s="70" t="s">
+      <c r="A19" s="67"/>
+      <c r="B19" s="70"/>
+      <c r="C19" s="68" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="75" t="s">
+      <c r="E19" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="79"/>
+      <c r="F19" s="66"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6773,11 +6758,11 @@
       <c r="AL19" s="8"/>
       <c r="AM19" s="9"/>
       <c r="AN19" s="10"/>
-      <c r="AO19" s="11"/>
+      <c r="AO19" s="47"/>
       <c r="AQ19" s="8"/>
       <c r="AR19" s="8"/>
       <c r="AS19" s="8"/>
-      <c r="AT19" s="9"/>
+      <c r="AT19" s="81"/>
       <c r="AU19" s="10"/>
       <c r="AV19" s="11"/>
       <c r="AW19" s="8"/>
@@ -6960,14 +6945,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="71"/>
-      <c r="B20" s="71"/>
-      <c r="C20" s="71"/>
+      <c r="A20" s="67"/>
+      <c r="B20" s="67"/>
+      <c r="C20" s="67"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="71"/>
-      <c r="F20" s="71"/>
+      <c r="E20" s="67"/>
+      <c r="F20" s="67"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -7002,11 +6987,11 @@
       <c r="AL20" s="8"/>
       <c r="AM20" s="9"/>
       <c r="AN20" s="10"/>
-      <c r="AO20" s="11"/>
+      <c r="AO20" s="47"/>
       <c r="AQ20" s="8"/>
       <c r="AR20" s="8"/>
       <c r="AS20" s="8"/>
-      <c r="AT20" s="9"/>
+      <c r="AT20" s="81"/>
       <c r="AU20" s="10"/>
       <c r="AV20" s="11"/>
       <c r="AW20" s="8"/>
@@ -7189,18 +7174,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="71"/>
-      <c r="B21" s="77"/>
-      <c r="C21" s="70" t="s">
+      <c r="A21" s="67"/>
+      <c r="B21" s="70"/>
+      <c r="C21" s="68" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="75" t="s">
+      <c r="E21" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="79"/>
+      <c r="F21" s="66"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7235,11 +7220,11 @@
       <c r="AL21" s="8"/>
       <c r="AM21" s="9"/>
       <c r="AN21" s="10"/>
-      <c r="AO21" s="11"/>
+      <c r="AO21" s="47"/>
       <c r="AQ21" s="8"/>
       <c r="AR21" s="8"/>
       <c r="AS21" s="8"/>
-      <c r="AT21" s="9"/>
+      <c r="AT21" s="81"/>
       <c r="AU21" s="10"/>
       <c r="AV21" s="11"/>
       <c r="AW21" s="8"/>
@@ -7422,14 +7407,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="78"/>
-      <c r="B22" s="78"/>
-      <c r="C22" s="78"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="73"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="78"/>
-      <c r="F22" s="78"/>
+      <c r="E22" s="73"/>
+      <c r="F22" s="73"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7464,12 +7449,11 @@
       <c r="AL22" s="38"/>
       <c r="AM22" s="39"/>
       <c r="AN22" s="40"/>
-      <c r="AO22" s="41"/>
-      <c r="AP22" s="61"/>
+      <c r="AO22" s="48"/>
       <c r="AQ22" s="38"/>
       <c r="AR22" s="38"/>
       <c r="AS22" s="38"/>
-      <c r="AT22" s="39"/>
+      <c r="AT22" s="82"/>
       <c r="AU22" s="40"/>
       <c r="AV22" s="41"/>
       <c r="AW22" s="38"/>
@@ -7652,22 +7636,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="68" t="s">
+      <c r="A23" s="69" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="73" t="s">
+      <c r="B23" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="69" t="s">
+      <c r="C23" s="62" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="72" t="s">
+      <c r="E23" s="61" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="74" t="s">
+      <c r="F23" s="63" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7704,12 +7688,12 @@
       <c r="AL23" s="8"/>
       <c r="AM23" s="9"/>
       <c r="AN23" s="10"/>
-      <c r="AO23" s="11"/>
-      <c r="AP23" s="62"/>
+      <c r="AO23" s="47"/>
+      <c r="AP23" s="54"/>
       <c r="AQ23" s="8"/>
       <c r="AR23" s="8"/>
       <c r="AS23" s="8"/>
-      <c r="AT23" s="9"/>
+      <c r="AT23" s="81"/>
       <c r="AU23" s="10"/>
       <c r="AV23" s="11"/>
       <c r="AW23" s="16"/>
@@ -7892,14 +7876,14 @@
       <c r="HR23" s="8"/>
     </row>
     <row r="24" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="67"/>
-      <c r="B24" s="67"/>
-      <c r="C24" s="67"/>
+      <c r="A24" s="59"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="59"/>
       <c r="D24" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="67"/>
-      <c r="F24" s="67"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
@@ -7934,12 +7918,12 @@
       <c r="AL24" s="8"/>
       <c r="AM24" s="9"/>
       <c r="AN24" s="10"/>
-      <c r="AO24" s="11"/>
-      <c r="AP24" s="64"/>
-      <c r="AQ24" s="65"/>
+      <c r="AO24" s="47"/>
+      <c r="AP24" s="56"/>
+      <c r="AQ24" s="8"/>
       <c r="AR24" s="8"/>
       <c r="AS24" s="8"/>
-      <c r="AT24" s="9"/>
+      <c r="AT24" s="81"/>
       <c r="AU24" s="10"/>
       <c r="AV24" s="11"/>
       <c r="AW24" s="8"/>
@@ -8122,20 +8106,20 @@
       <c r="HR24" s="8"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="67"/>
-      <c r="B25" s="73" t="s">
+      <c r="A25" s="59"/>
+      <c r="B25" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="69" t="s">
+      <c r="C25" s="62" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="72" t="s">
+      <c r="E25" s="61" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="74" t="s">
+      <c r="F25" s="63" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8169,11 +8153,11 @@
       <c r="AL25" s="16"/>
       <c r="AM25" s="9"/>
       <c r="AN25" s="10"/>
-      <c r="AO25" s="11"/>
+      <c r="AO25" s="47"/>
       <c r="AQ25" s="8"/>
       <c r="AR25" s="8"/>
       <c r="AS25" s="8"/>
-      <c r="AT25" s="9"/>
+      <c r="AT25" s="81"/>
       <c r="AU25" s="10"/>
       <c r="AV25" s="11"/>
       <c r="AW25" s="8"/>
@@ -8351,14 +8335,14 @@
       <c r="HS25" s="8"/>
     </row>
     <row r="26" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="67"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="67"/>
+      <c r="A26" s="59"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
       <c r="D26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
@@ -8393,11 +8377,11 @@
       <c r="AL26" s="8"/>
       <c r="AM26" s="9"/>
       <c r="AN26" s="10"/>
-      <c r="AO26" s="11"/>
+      <c r="AO26" s="47"/>
       <c r="AQ26" s="44"/>
       <c r="AR26" s="8"/>
       <c r="AS26" s="8"/>
-      <c r="AT26" s="9"/>
+      <c r="AT26" s="81"/>
       <c r="AU26" s="10"/>
       <c r="AV26" s="11"/>
       <c r="AW26" s="8"/>
@@ -8580,20 +8564,20 @@
       <c r="HR26" s="8"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="67"/>
-      <c r="B27" s="73" t="s">
+      <c r="A27" s="59"/>
+      <c r="B27" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="80" t="s">
+      <c r="C27" s="71" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="72" t="s">
+      <c r="E27" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="74"/>
+      <c r="F27" s="63"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8628,10 +8612,10 @@
       <c r="AL27" s="8"/>
       <c r="AM27" s="9"/>
       <c r="AN27" s="10"/>
-      <c r="AO27" s="11"/>
+      <c r="AO27" s="47"/>
       <c r="AQ27" s="8"/>
       <c r="AR27" s="8"/>
-      <c r="AT27" s="9"/>
+      <c r="AT27" s="81"/>
       <c r="AU27" s="10"/>
       <c r="AV27" s="11"/>
       <c r="AW27" s="8"/>
@@ -8814,14 +8798,14 @@
       <c r="HR27" s="8"/>
     </row>
     <row r="28" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="67"/>
-      <c r="B28" s="67"/>
-      <c r="C28" s="67"/>
+      <c r="A28" s="59"/>
+      <c r="B28" s="59"/>
+      <c r="C28" s="59"/>
       <c r="D28" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="67"/>
-      <c r="F28" s="67"/>
+      <c r="E28" s="59"/>
+      <c r="F28" s="59"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
@@ -8855,11 +8839,11 @@
       <c r="AK28" s="8"/>
       <c r="AM28" s="9"/>
       <c r="AN28" s="10"/>
-      <c r="AO28" s="11"/>
+      <c r="AO28" s="47"/>
       <c r="AQ28" s="8"/>
       <c r="AR28" s="8"/>
       <c r="AS28" s="8"/>
-      <c r="AT28" s="9"/>
+      <c r="AT28" s="81"/>
       <c r="AU28" s="10"/>
       <c r="AV28" s="11"/>
       <c r="AW28" s="8"/>
@@ -9042,22 +9026,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="73" t="s">
+      <c r="B29" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="69" t="s">
+      <c r="C29" s="62" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="72" t="s">
+      <c r="E29" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="74" t="s">
+      <c r="F29" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9093,11 +9077,11 @@
       <c r="AK29" s="8"/>
       <c r="AM29" s="9"/>
       <c r="AN29" s="10"/>
-      <c r="AO29" s="11"/>
+      <c r="AO29" s="47"/>
       <c r="AQ29" s="8"/>
       <c r="AR29" s="8"/>
       <c r="AS29" s="8"/>
-      <c r="AT29" s="9"/>
+      <c r="AT29" s="81"/>
       <c r="AU29" s="10"/>
       <c r="AV29" s="11"/>
       <c r="AW29" s="8"/>
@@ -9280,14 +9264,14 @@
       <c r="HR29" s="8"/>
     </row>
     <row r="30" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="67"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="67"/>
+      <c r="A30" s="59"/>
+      <c r="B30" s="59"/>
+      <c r="C30" s="59"/>
       <c r="D30" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="67"/>
-      <c r="F30" s="67"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="59"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
@@ -9322,11 +9306,11 @@
       <c r="AL30" s="44"/>
       <c r="AM30" s="9"/>
       <c r="AN30" s="10"/>
-      <c r="AO30" s="11"/>
+      <c r="AO30" s="47"/>
       <c r="AQ30" s="8"/>
       <c r="AR30" s="8"/>
       <c r="AS30" s="8"/>
-      <c r="AT30" s="9"/>
+      <c r="AT30" s="81"/>
       <c r="AU30" s="10"/>
       <c r="AV30" s="11"/>
       <c r="AW30" s="8"/>
@@ -9509,20 +9493,20 @@
       <c r="HR30" s="8"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="67"/>
-      <c r="B31" s="73" t="s">
+      <c r="A31" s="59"/>
+      <c r="B31" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="69" t="s">
+      <c r="C31" s="62" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="72" t="s">
+      <c r="E31" s="61" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="74" t="s">
+      <c r="F31" s="63" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9559,11 +9543,11 @@
       <c r="AL31" s="8"/>
       <c r="AM31" s="9"/>
       <c r="AN31" s="10"/>
-      <c r="AO31" s="11"/>
+      <c r="AO31" s="47"/>
       <c r="AQ31" s="8"/>
       <c r="AR31" s="8"/>
       <c r="AS31" s="8"/>
-      <c r="AT31" s="9"/>
+      <c r="AT31" s="81"/>
       <c r="AU31" s="10"/>
       <c r="AV31" s="11"/>
       <c r="AW31" s="8"/>
@@ -9746,14 +9730,14 @@
       <c r="HR31" s="8"/>
     </row>
     <row r="32" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="67"/>
-      <c r="B32" s="67"/>
-      <c r="C32" s="67"/>
+      <c r="A32" s="59"/>
+      <c r="B32" s="59"/>
+      <c r="C32" s="59"/>
       <c r="D32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="67"/>
-      <c r="F32" s="67"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="8"/>
@@ -9787,12 +9771,12 @@
       <c r="AK32" s="8"/>
       <c r="AM32" s="9"/>
       <c r="AN32" s="10"/>
-      <c r="AO32" s="11"/>
-      <c r="AP32" s="44"/>
+      <c r="AO32" s="47"/>
+      <c r="AP32" s="76"/>
       <c r="AQ32" s="8"/>
       <c r="AR32" s="8"/>
       <c r="AS32" s="8"/>
-      <c r="AT32" s="9"/>
+      <c r="AT32" s="81"/>
       <c r="AU32" s="10"/>
       <c r="AV32" s="11"/>
       <c r="AW32" s="8"/>
@@ -9975,20 +9959,20 @@
       <c r="HR32" s="8"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="67"/>
-      <c r="B33" s="73" t="s">
+      <c r="A33" s="59"/>
+      <c r="B33" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="69" t="s">
+      <c r="C33" s="62" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="72" t="s">
+      <c r="E33" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="74" t="s">
+      <c r="F33" s="63" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -10025,11 +10009,11 @@
       <c r="AL33" s="8"/>
       <c r="AM33" s="9"/>
       <c r="AN33" s="10"/>
-      <c r="AO33" s="11"/>
+      <c r="AO33" s="47"/>
       <c r="AQ33" s="8"/>
       <c r="AR33" s="16"/>
       <c r="AS33" s="16"/>
-      <c r="AT33" s="9"/>
+      <c r="AT33" s="81"/>
       <c r="AU33" s="10"/>
       <c r="AV33" s="11"/>
       <c r="AW33" s="8"/>
@@ -10212,14 +10196,14 @@
       <c r="HR33" s="8"/>
     </row>
     <row r="34" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="67"/>
-      <c r="B34" s="67"/>
-      <c r="C34" s="67"/>
+      <c r="A34" s="59"/>
+      <c r="B34" s="59"/>
+      <c r="C34" s="59"/>
       <c r="D34" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="67"/>
-      <c r="F34" s="67"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
@@ -10254,11 +10238,11 @@
       <c r="AL34" s="8"/>
       <c r="AM34" s="9"/>
       <c r="AN34" s="45"/>
-      <c r="AO34" s="45"/>
+      <c r="AO34" s="75"/>
       <c r="AQ34" s="8"/>
       <c r="AR34" s="8"/>
       <c r="AS34" s="8"/>
-      <c r="AT34" s="9"/>
+      <c r="AT34" s="81"/>
       <c r="AU34" s="10"/>
       <c r="AV34" s="11"/>
       <c r="AW34" s="8"/>
@@ -10441,20 +10425,20 @@
       <c r="HR34" s="8"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="67"/>
-      <c r="B35" s="73" t="s">
+      <c r="A35" s="59"/>
+      <c r="B35" s="60" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="69" t="s">
+      <c r="C35" s="62" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="72" t="s">
+      <c r="E35" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="74" t="s">
+      <c r="F35" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10491,11 +10475,11 @@
       <c r="AL35" s="8"/>
       <c r="AM35" s="9"/>
       <c r="AN35" s="10"/>
-      <c r="AO35" s="11"/>
+      <c r="AO35" s="47"/>
       <c r="AQ35" s="8"/>
       <c r="AR35" s="8"/>
       <c r="AS35" s="8"/>
-      <c r="AT35" s="9"/>
+      <c r="AT35" s="81"/>
       <c r="AU35" s="10"/>
       <c r="AV35" s="11"/>
       <c r="AW35" s="8"/>
@@ -10678,14 +10662,14 @@
       <c r="HR35" s="8"/>
     </row>
     <row r="36" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="67"/>
-      <c r="B36" s="67"/>
-      <c r="C36" s="67"/>
+      <c r="A36" s="59"/>
+      <c r="B36" s="59"/>
+      <c r="C36" s="59"/>
       <c r="D36" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="67"/>
-      <c r="F36" s="67"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="59"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
@@ -10720,11 +10704,11 @@
       <c r="AL36" s="8"/>
       <c r="AM36" s="9"/>
       <c r="AN36" s="10"/>
-      <c r="AO36" s="11"/>
+      <c r="AO36" s="47"/>
       <c r="AQ36" s="8"/>
       <c r="AR36" s="8"/>
       <c r="AS36" s="8"/>
-      <c r="AT36" s="9"/>
+      <c r="AT36" s="81"/>
       <c r="AU36" s="10"/>
       <c r="AV36" s="11"/>
       <c r="AW36" s="8"/>
@@ -10907,20 +10891,20 @@
       <c r="HR36" s="8"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="67"/>
-      <c r="B37" s="73" t="s">
+      <c r="A37" s="59"/>
+      <c r="B37" s="60" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="69" t="s">
+      <c r="C37" s="62" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="72" t="s">
+      <c r="E37" s="61" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="74" t="s">
+      <c r="F37" s="63" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -10957,11 +10941,11 @@
       <c r="AL37" s="8"/>
       <c r="AM37" s="9"/>
       <c r="AN37" s="10"/>
-      <c r="AO37" s="11"/>
+      <c r="AO37" s="47"/>
       <c r="AQ37" s="8"/>
       <c r="AR37" s="8"/>
       <c r="AS37" s="8"/>
-      <c r="AT37" s="9"/>
+      <c r="AT37" s="81"/>
       <c r="AU37" s="10"/>
       <c r="AV37" s="11"/>
       <c r="AW37" s="8"/>
@@ -11144,14 +11128,14 @@
       <c r="HR37" s="8"/>
     </row>
     <row r="38" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="67"/>
-      <c r="B38" s="67"/>
-      <c r="C38" s="67"/>
+      <c r="A38" s="59"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="59"/>
       <c r="D38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="67"/>
-      <c r="F38" s="67"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="59"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
@@ -11186,11 +11170,11 @@
       <c r="AL38" s="8"/>
       <c r="AM38" s="9"/>
       <c r="AN38" s="10"/>
-      <c r="AO38" s="11"/>
+      <c r="AO38" s="47"/>
       <c r="AQ38" s="8"/>
       <c r="AR38" s="8"/>
       <c r="AS38" s="8"/>
-      <c r="AT38" s="9"/>
+      <c r="AT38" s="81"/>
       <c r="AU38" s="10"/>
       <c r="AV38" s="11"/>
       <c r="AW38" s="8"/>
@@ -11373,20 +11357,20 @@
       <c r="HR38" s="8"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="67"/>
-      <c r="B39" s="73" t="s">
+      <c r="A39" s="59"/>
+      <c r="B39" s="60" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="69" t="s">
+      <c r="C39" s="62" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="72" t="s">
+      <c r="E39" s="61" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="74" t="s">
+      <c r="F39" s="63" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11423,11 +11407,11 @@
       <c r="AL39" s="8"/>
       <c r="AM39" s="9"/>
       <c r="AN39" s="10"/>
-      <c r="AO39" s="11"/>
+      <c r="AO39" s="47"/>
       <c r="AQ39" s="8"/>
       <c r="AR39" s="8"/>
       <c r="AS39" s="8"/>
-      <c r="AT39" s="9"/>
+      <c r="AT39" s="81"/>
       <c r="AU39" s="10"/>
       <c r="AV39" s="11"/>
       <c r="AW39" s="8"/>
@@ -11610,14 +11594,14 @@
       <c r="HR39" s="8"/>
     </row>
     <row r="40" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="67"/>
-      <c r="B40" s="67"/>
-      <c r="C40" s="67"/>
+      <c r="A40" s="59"/>
+      <c r="B40" s="59"/>
+      <c r="C40" s="59"/>
       <c r="D40" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="67"/>
-      <c r="F40" s="67"/>
+      <c r="E40" s="59"/>
+      <c r="F40" s="59"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
@@ -11652,11 +11636,11 @@
       <c r="AL40" s="8"/>
       <c r="AM40" s="9"/>
       <c r="AN40" s="10"/>
-      <c r="AO40" s="11"/>
+      <c r="AO40" s="47"/>
       <c r="AQ40" s="8"/>
       <c r="AR40" s="8"/>
       <c r="AS40" s="8"/>
-      <c r="AT40" s="9"/>
+      <c r="AT40" s="81"/>
       <c r="AU40" s="10"/>
       <c r="AV40" s="11"/>
       <c r="AW40" s="8"/>
@@ -11839,22 +11823,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="68" t="s">
+      <c r="A41" s="69" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="73" t="s">
+      <c r="B41" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="69" t="s">
+      <c r="C41" s="62" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="72" t="s">
+      <c r="E41" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="74" t="s">
+      <c r="F41" s="63" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -11891,11 +11875,11 @@
       <c r="AL41" s="8"/>
       <c r="AM41" s="9"/>
       <c r="AN41" s="10"/>
-      <c r="AO41" s="11"/>
+      <c r="AO41" s="47"/>
       <c r="AQ41" s="8"/>
       <c r="AR41" s="8"/>
       <c r="AS41" s="8"/>
-      <c r="AT41" s="9"/>
+      <c r="AT41" s="81"/>
       <c r="AU41" s="10"/>
       <c r="AV41" s="11"/>
       <c r="AW41" s="8"/>
@@ -12078,14 +12062,14 @@
       <c r="HR41" s="8"/>
     </row>
     <row r="42" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="67"/>
-      <c r="B42" s="67"/>
-      <c r="C42" s="67"/>
+      <c r="A42" s="59"/>
+      <c r="B42" s="59"/>
+      <c r="C42" s="59"/>
       <c r="D42" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="67"/>
-      <c r="F42" s="67"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="59"/>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="8"/>
@@ -12120,11 +12104,11 @@
       <c r="AL42" s="8"/>
       <c r="AM42" s="9"/>
       <c r="AN42" s="10"/>
-      <c r="AO42" s="11"/>
+      <c r="AO42" s="47"/>
       <c r="AQ42" s="8"/>
       <c r="AR42" s="8"/>
       <c r="AS42" s="8"/>
-      <c r="AT42" s="9"/>
+      <c r="AT42" s="81"/>
       <c r="AU42" s="10"/>
       <c r="AV42" s="11"/>
       <c r="AW42" s="8"/>
@@ -12307,20 +12291,20 @@
       <c r="HR42" s="8"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="67"/>
-      <c r="B43" s="73" t="s">
+      <c r="A43" s="59"/>
+      <c r="B43" s="60" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="69" t="s">
+      <c r="C43" s="62" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="72" t="s">
+      <c r="E43" s="61" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="74" t="s">
+      <c r="F43" s="63" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12355,12 +12339,12 @@
       <c r="AL43" s="8"/>
       <c r="AM43" s="9"/>
       <c r="AN43" s="10"/>
-      <c r="AO43" s="11"/>
-      <c r="AP43" s="63"/>
+      <c r="AO43" s="47"/>
+      <c r="AP43" s="52"/>
       <c r="AQ43" s="7"/>
       <c r="AR43" s="8"/>
       <c r="AS43" s="8"/>
-      <c r="AT43" s="9"/>
+      <c r="AT43" s="81"/>
       <c r="AU43" s="10"/>
       <c r="AV43" s="11"/>
       <c r="AW43" s="8"/>
@@ -12543,14 +12527,14 @@
       <c r="HR43" s="8"/>
     </row>
     <row r="44" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="67"/>
-      <c r="B44" s="67"/>
-      <c r="C44" s="67"/>
+      <c r="A44" s="59"/>
+      <c r="B44" s="59"/>
+      <c r="C44" s="59"/>
       <c r="D44" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="67"/>
-      <c r="F44" s="67"/>
+      <c r="E44" s="59"/>
+      <c r="F44" s="59"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="8"/>
@@ -12585,12 +12569,12 @@
       <c r="AL44" s="8"/>
       <c r="AM44" s="9"/>
       <c r="AN44" s="10"/>
-      <c r="AO44" s="11"/>
-      <c r="AP44" s="43"/>
+      <c r="AO44" s="47"/>
+      <c r="AP44" s="56"/>
       <c r="AQ44" s="8"/>
       <c r="AR44" s="44"/>
-      <c r="AS44" s="8"/>
-      <c r="AT44" s="9"/>
+      <c r="AS44" s="44"/>
+      <c r="AT44" s="81"/>
       <c r="AU44" s="10"/>
       <c r="AV44" s="11"/>
       <c r="AW44" s="8"/>
@@ -12773,20 +12757,20 @@
       <c r="HR44" s="8"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="67"/>
-      <c r="B45" s="73" t="s">
+      <c r="A45" s="59"/>
+      <c r="B45" s="60" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="69" t="s">
+      <c r="C45" s="62" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="72" t="s">
+      <c r="E45" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="74" t="s">
+      <c r="F45" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12823,10 +12807,10 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="9"/>
       <c r="AN45" s="10"/>
-      <c r="AO45" s="11"/>
+      <c r="AO45" s="47"/>
       <c r="AR45" s="8"/>
       <c r="AS45" s="8"/>
-      <c r="AT45" s="9"/>
+      <c r="AT45" s="81"/>
       <c r="AU45" s="10"/>
       <c r="AV45" s="11"/>
       <c r="AW45" s="7"/>
@@ -13009,14 +12993,14 @@
       <c r="HR45" s="8"/>
     </row>
     <row r="46" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="67"/>
-      <c r="B46" s="67"/>
-      <c r="C46" s="67"/>
+      <c r="A46" s="59"/>
+      <c r="B46" s="59"/>
+      <c r="C46" s="59"/>
       <c r="D46" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="67"/>
-      <c r="F46" s="67"/>
+      <c r="E46" s="59"/>
+      <c r="F46" s="59"/>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="8"/>
@@ -13051,11 +13035,11 @@
       <c r="AL46" s="8"/>
       <c r="AM46" s="9"/>
       <c r="AN46" s="10"/>
-      <c r="AO46" s="44"/>
+      <c r="AO46" s="76"/>
       <c r="AQ46" s="8"/>
       <c r="AR46" s="8"/>
       <c r="AS46" s="8"/>
-      <c r="AT46" s="9"/>
+      <c r="AT46" s="81"/>
       <c r="AU46" s="10"/>
       <c r="AV46" s="11"/>
       <c r="AW46" s="8"/>
@@ -13238,22 +13222,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="68" t="s">
+      <c r="A47" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="73" t="s">
+      <c r="B47" s="60" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="69" t="s">
+      <c r="C47" s="62" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="72" t="s">
+      <c r="E47" s="61" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="74" t="s">
+      <c r="F47" s="63" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13290,11 +13274,11 @@
       <c r="AL47" s="8"/>
       <c r="AM47" s="9"/>
       <c r="AN47" s="10"/>
-      <c r="AO47" s="11"/>
+      <c r="AO47" s="47"/>
       <c r="AQ47" s="8"/>
       <c r="AR47" s="8"/>
       <c r="AS47" s="8"/>
-      <c r="AT47" s="9"/>
+      <c r="AT47" s="81"/>
       <c r="AU47" s="10"/>
       <c r="AV47" s="11"/>
       <c r="AW47" s="8"/>
@@ -13477,14 +13461,14 @@
       <c r="HR47" s="8"/>
     </row>
     <row r="48" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="67"/>
-      <c r="B48" s="67"/>
-      <c r="C48" s="67"/>
+      <c r="A48" s="59"/>
+      <c r="B48" s="59"/>
+      <c r="C48" s="59"/>
       <c r="D48" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="67"/>
-      <c r="F48" s="67"/>
+      <c r="E48" s="59"/>
+      <c r="F48" s="59"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
@@ -13519,11 +13503,11 @@
       <c r="AL48" s="8"/>
       <c r="AM48" s="9"/>
       <c r="AN48" s="10"/>
-      <c r="AO48" s="11"/>
+      <c r="AO48" s="47"/>
       <c r="AQ48" s="8"/>
       <c r="AR48" s="8"/>
       <c r="AS48" s="8"/>
-      <c r="AT48" s="9"/>
+      <c r="AT48" s="81"/>
       <c r="AU48" s="10"/>
       <c r="AV48" s="11"/>
       <c r="AW48" s="8"/>
@@ -13706,20 +13690,20 @@
       <c r="HR48" s="8"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="67"/>
-      <c r="B49" s="73" t="s">
+      <c r="A49" s="59"/>
+      <c r="B49" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="69" t="s">
+      <c r="C49" s="62" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="72" t="s">
+      <c r="E49" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="74" t="s">
+      <c r="F49" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13756,11 +13740,11 @@
       <c r="AL49" s="8"/>
       <c r="AM49" s="9"/>
       <c r="AN49" s="10"/>
-      <c r="AO49" s="11"/>
+      <c r="AO49" s="47"/>
       <c r="AQ49" s="8"/>
       <c r="AR49" s="8"/>
       <c r="AS49" s="8"/>
-      <c r="AT49" s="9"/>
+      <c r="AT49" s="81"/>
       <c r="AU49" s="10"/>
       <c r="AV49" s="11"/>
       <c r="AW49" s="8"/>
@@ -13943,14 +13927,14 @@
       <c r="HR49" s="8"/>
     </row>
     <row r="50" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="67"/>
-      <c r="B50" s="67"/>
-      <c r="C50" s="67"/>
+      <c r="A50" s="59"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="59"/>
       <c r="D50" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="67"/>
-      <c r="F50" s="67"/>
+      <c r="E50" s="59"/>
+      <c r="F50" s="59"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
@@ -13985,11 +13969,11 @@
       <c r="AL50" s="8"/>
       <c r="AM50" s="9"/>
       <c r="AN50" s="10"/>
-      <c r="AO50" s="11"/>
+      <c r="AO50" s="47"/>
       <c r="AQ50" s="8"/>
       <c r="AR50" s="8"/>
       <c r="AS50" s="8"/>
-      <c r="AT50" s="9"/>
+      <c r="AT50" s="81"/>
       <c r="AU50" s="10"/>
       <c r="AV50" s="11"/>
       <c r="AW50" s="8"/>
@@ -14172,22 +14156,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="68" t="s">
+      <c r="A51" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="73" t="s">
+      <c r="B51" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="69" t="s">
+      <c r="C51" s="62" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="72" t="s">
+      <c r="E51" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="74" t="s">
+      <c r="F51" s="63" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14224,11 +14208,11 @@
       <c r="AL51" s="8"/>
       <c r="AM51" s="9"/>
       <c r="AN51" s="10"/>
-      <c r="AO51" s="11"/>
+      <c r="AO51" s="47"/>
       <c r="AQ51" s="8"/>
       <c r="AR51" s="8"/>
       <c r="AS51" s="8"/>
-      <c r="AT51" s="9"/>
+      <c r="AT51" s="81"/>
       <c r="AU51" s="10"/>
       <c r="AV51" s="11"/>
       <c r="AW51" s="8"/>
@@ -14411,14 +14395,14 @@
       <c r="HR51" s="8"/>
     </row>
     <row r="52" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="67"/>
-      <c r="B52" s="67"/>
-      <c r="C52" s="67"/>
+      <c r="A52" s="59"/>
+      <c r="B52" s="59"/>
+      <c r="C52" s="59"/>
       <c r="D52" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="67"/>
-      <c r="F52" s="67"/>
+      <c r="E52" s="59"/>
+      <c r="F52" s="59"/>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="8"/>
@@ -14453,11 +14437,11 @@
       <c r="AL52" s="8"/>
       <c r="AM52" s="9"/>
       <c r="AN52" s="10"/>
-      <c r="AO52" s="11"/>
+      <c r="AO52" s="47"/>
       <c r="AQ52" s="8"/>
       <c r="AR52" s="8"/>
       <c r="AS52" s="8"/>
-      <c r="AT52" s="9"/>
+      <c r="AT52" s="81"/>
       <c r="AU52" s="10"/>
       <c r="AV52" s="11"/>
       <c r="AW52" s="8"/>
@@ -14640,20 +14624,20 @@
       <c r="HR52" s="8"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="67"/>
-      <c r="B53" s="73" t="s">
+      <c r="A53" s="59"/>
+      <c r="B53" s="60" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="69" t="s">
+      <c r="C53" s="62" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="72" t="s">
+      <c r="E53" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="74" t="s">
+      <c r="F53" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14690,11 +14674,11 @@
       <c r="AL53" s="8"/>
       <c r="AM53" s="9"/>
       <c r="AN53" s="10"/>
-      <c r="AO53" s="11"/>
+      <c r="AO53" s="47"/>
       <c r="AQ53" s="8"/>
       <c r="AR53" s="8"/>
       <c r="AS53" s="8"/>
-      <c r="AT53" s="9"/>
+      <c r="AT53" s="81"/>
       <c r="AU53" s="10"/>
       <c r="AV53" s="11"/>
       <c r="AW53" s="8"/>
@@ -14877,14 +14861,14 @@
       <c r="HR53" s="8"/>
     </row>
     <row r="54" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="67"/>
-      <c r="B54" s="67"/>
-      <c r="C54" s="67"/>
+      <c r="A54" s="59"/>
+      <c r="B54" s="59"/>
+      <c r="C54" s="59"/>
       <c r="D54" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="67"/>
-      <c r="F54" s="67"/>
+      <c r="E54" s="59"/>
+      <c r="F54" s="59"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
@@ -14919,11 +14903,11 @@
       <c r="AL54" s="8"/>
       <c r="AM54" s="9"/>
       <c r="AN54" s="10"/>
-      <c r="AO54" s="11"/>
+      <c r="AO54" s="47"/>
       <c r="AQ54" s="8"/>
       <c r="AR54" s="8"/>
       <c r="AS54" s="8"/>
-      <c r="AT54" s="9"/>
+      <c r="AT54" s="81"/>
       <c r="AU54" s="10"/>
       <c r="AV54" s="11"/>
       <c r="AW54" s="8"/>
@@ -15106,22 +15090,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="68" t="s">
+      <c r="A55" s="69" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="73" t="s">
+      <c r="B55" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="69" t="s">
+      <c r="C55" s="62" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="72" t="s">
+      <c r="E55" s="61" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="74" t="s">
+      <c r="F55" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -15158,11 +15142,11 @@
       <c r="AL55" s="8"/>
       <c r="AM55" s="9"/>
       <c r="AN55" s="10"/>
-      <c r="AO55" s="11"/>
+      <c r="AO55" s="47"/>
       <c r="AQ55" s="8"/>
       <c r="AR55" s="8"/>
       <c r="AS55" s="8"/>
-      <c r="AT55" s="9"/>
+      <c r="AT55" s="81"/>
       <c r="AU55" s="10"/>
       <c r="AV55" s="11"/>
       <c r="AW55" s="8"/>
@@ -15345,14 +15329,14 @@
       <c r="HR55" s="8"/>
     </row>
     <row r="56" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="67"/>
-      <c r="B56" s="67"/>
-      <c r="C56" s="67"/>
+      <c r="A56" s="59"/>
+      <c r="B56" s="59"/>
+      <c r="C56" s="59"/>
       <c r="D56" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="67"/>
-      <c r="F56" s="67"/>
+      <c r="E56" s="59"/>
+      <c r="F56" s="59"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
@@ -15387,11 +15371,11 @@
       <c r="AL56" s="8"/>
       <c r="AM56" s="9"/>
       <c r="AN56" s="10"/>
-      <c r="AO56" s="11"/>
+      <c r="AO56" s="47"/>
       <c r="AQ56" s="8"/>
       <c r="AR56" s="8"/>
       <c r="AS56" s="8"/>
-      <c r="AT56" s="9"/>
+      <c r="AT56" s="81"/>
       <c r="AU56" s="10"/>
       <c r="AV56" s="11"/>
       <c r="AW56" s="8"/>
@@ -15574,20 +15558,20 @@
       <c r="HR56" s="8"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="67"/>
-      <c r="B57" s="73" t="s">
+      <c r="A57" s="59"/>
+      <c r="B57" s="60" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="69" t="s">
+      <c r="C57" s="62" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="72" t="s">
+      <c r="E57" s="61" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="74" t="s">
+      <c r="F57" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15624,11 +15608,11 @@
       <c r="AL57" s="8"/>
       <c r="AM57" s="9"/>
       <c r="AN57" s="10"/>
-      <c r="AO57" s="11"/>
+      <c r="AO57" s="47"/>
       <c r="AQ57" s="8"/>
       <c r="AR57" s="8"/>
       <c r="AS57" s="8"/>
-      <c r="AT57" s="9"/>
+      <c r="AT57" s="81"/>
       <c r="AU57" s="10"/>
       <c r="AV57" s="11"/>
       <c r="AW57" s="8"/>
@@ -15811,14 +15795,14 @@
       <c r="HR57" s="8"/>
     </row>
     <row r="58" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="67"/>
-      <c r="B58" s="67"/>
-      <c r="C58" s="67"/>
+      <c r="A58" s="59"/>
+      <c r="B58" s="59"/>
+      <c r="C58" s="59"/>
       <c r="D58" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="67"/>
-      <c r="F58" s="67"/>
+      <c r="E58" s="59"/>
+      <c r="F58" s="59"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
@@ -15853,11 +15837,11 @@
       <c r="AL58" s="8"/>
       <c r="AM58" s="9"/>
       <c r="AN58" s="10"/>
-      <c r="AO58" s="11"/>
+      <c r="AO58" s="47"/>
       <c r="AQ58" s="8"/>
       <c r="AR58" s="8"/>
       <c r="AS58" s="8"/>
-      <c r="AT58" s="9"/>
+      <c r="AT58" s="81"/>
       <c r="AU58" s="10"/>
       <c r="AV58" s="11"/>
       <c r="AW58" s="8"/>
@@ -16040,20 +16024,20 @@
       <c r="HR58" s="8"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="67"/>
-      <c r="B59" s="73" t="s">
+      <c r="A59" s="59"/>
+      <c r="B59" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="69" t="s">
+      <c r="C59" s="62" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="72" t="s">
+      <c r="E59" s="61" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="74" t="s">
+      <c r="F59" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -16090,11 +16074,11 @@
       <c r="AL59" s="8"/>
       <c r="AM59" s="9"/>
       <c r="AN59" s="10"/>
-      <c r="AO59" s="11"/>
+      <c r="AO59" s="47"/>
       <c r="AQ59" s="8"/>
       <c r="AR59" s="8"/>
       <c r="AS59" s="8"/>
-      <c r="AT59" s="9"/>
+      <c r="AT59" s="81"/>
       <c r="AU59" s="10"/>
       <c r="AV59" s="11"/>
       <c r="AW59" s="8"/>
@@ -16277,14 +16261,14 @@
       <c r="HR59" s="8"/>
     </row>
     <row r="60" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="67"/>
-      <c r="B60" s="67"/>
-      <c r="C60" s="67"/>
+      <c r="A60" s="59"/>
+      <c r="B60" s="59"/>
+      <c r="C60" s="59"/>
       <c r="D60" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="67"/>
-      <c r="F60" s="67"/>
+      <c r="E60" s="59"/>
+      <c r="F60" s="59"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
@@ -16319,11 +16303,11 @@
       <c r="AL60" s="8"/>
       <c r="AM60" s="9"/>
       <c r="AN60" s="10"/>
-      <c r="AO60" s="11"/>
+      <c r="AO60" s="47"/>
       <c r="AQ60" s="8"/>
       <c r="AR60" s="8"/>
       <c r="AS60" s="8"/>
-      <c r="AT60" s="9"/>
+      <c r="AT60" s="81"/>
       <c r="AU60" s="10"/>
       <c r="AV60" s="11"/>
       <c r="AW60" s="8"/>
@@ -16506,20 +16490,20 @@
       <c r="HR60" s="8"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="67"/>
-      <c r="B61" s="73" t="s">
+      <c r="A61" s="59"/>
+      <c r="B61" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="69" t="s">
+      <c r="C61" s="62" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="72" t="s">
+      <c r="E61" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="74" t="s">
+      <c r="F61" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16556,11 +16540,11 @@
       <c r="AL61" s="8"/>
       <c r="AM61" s="9"/>
       <c r="AN61" s="10"/>
-      <c r="AO61" s="11"/>
+      <c r="AO61" s="47"/>
       <c r="AQ61" s="8"/>
       <c r="AR61" s="8"/>
       <c r="AS61" s="8"/>
-      <c r="AT61" s="9"/>
+      <c r="AT61" s="81"/>
       <c r="AU61" s="10"/>
       <c r="AV61" s="11"/>
       <c r="AW61" s="8"/>
@@ -16743,14 +16727,14 @@
       <c r="HR61" s="8"/>
     </row>
     <row r="62" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="67"/>
-      <c r="B62" s="67"/>
-      <c r="C62" s="67"/>
+      <c r="A62" s="59"/>
+      <c r="B62" s="59"/>
+      <c r="C62" s="59"/>
       <c r="D62" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="67"/>
-      <c r="F62" s="67"/>
+      <c r="E62" s="59"/>
+      <c r="F62" s="59"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
       <c r="I62" s="8"/>
@@ -16785,11 +16769,11 @@
       <c r="AL62" s="8"/>
       <c r="AM62" s="9"/>
       <c r="AN62" s="10"/>
-      <c r="AO62" s="11"/>
+      <c r="AO62" s="47"/>
       <c r="AQ62" s="8"/>
       <c r="AR62" s="8"/>
       <c r="AS62" s="8"/>
-      <c r="AT62" s="9"/>
+      <c r="AT62" s="81"/>
       <c r="AU62" s="10"/>
       <c r="AV62" s="11"/>
       <c r="AW62" s="8"/>
@@ -16972,20 +16956,20 @@
       <c r="HR62" s="8"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="67"/>
-      <c r="B63" s="73" t="s">
+      <c r="A63" s="59"/>
+      <c r="B63" s="60" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="69" t="s">
+      <c r="C63" s="62" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="72" t="s">
+      <c r="E63" s="61" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="74" t="s">
+      <c r="F63" s="63" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -17022,11 +17006,11 @@
       <c r="AL63" s="8"/>
       <c r="AM63" s="9"/>
       <c r="AN63" s="10"/>
-      <c r="AO63" s="11"/>
+      <c r="AO63" s="47"/>
       <c r="AQ63" s="8"/>
       <c r="AR63" s="8"/>
       <c r="AS63" s="8"/>
-      <c r="AT63" s="9"/>
+      <c r="AT63" s="81"/>
       <c r="AU63" s="10"/>
       <c r="AV63" s="11"/>
       <c r="AW63" s="8"/>
@@ -17209,14 +17193,14 @@
       <c r="HR63" s="8"/>
     </row>
     <row r="64" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="67"/>
-      <c r="B64" s="67"/>
-      <c r="C64" s="67"/>
+      <c r="A64" s="59"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="59"/>
       <c r="D64" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="67"/>
-      <c r="F64" s="67"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
@@ -17251,11 +17235,11 @@
       <c r="AL64" s="8"/>
       <c r="AM64" s="9"/>
       <c r="AN64" s="10"/>
-      <c r="AO64" s="11"/>
+      <c r="AO64" s="47"/>
       <c r="AQ64" s="8"/>
       <c r="AR64" s="8"/>
       <c r="AS64" s="8"/>
-      <c r="AT64" s="9"/>
+      <c r="AT64" s="81"/>
       <c r="AU64" s="10"/>
       <c r="AV64" s="11"/>
       <c r="AW64" s="8"/>
@@ -17438,20 +17422,20 @@
       <c r="HR64" s="8"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="67"/>
-      <c r="B65" s="73" t="s">
+      <c r="A65" s="59"/>
+      <c r="B65" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="69" t="s">
+      <c r="C65" s="62" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="72" t="s">
+      <c r="E65" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="74" t="s">
+      <c r="F65" s="63" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17488,11 +17472,11 @@
       <c r="AL65" s="8"/>
       <c r="AM65" s="9"/>
       <c r="AN65" s="10"/>
-      <c r="AO65" s="11"/>
+      <c r="AO65" s="47"/>
       <c r="AQ65" s="8"/>
       <c r="AR65" s="8"/>
       <c r="AS65" s="8"/>
-      <c r="AT65" s="9"/>
+      <c r="AT65" s="81"/>
       <c r="AU65" s="10"/>
       <c r="AV65" s="11"/>
       <c r="AW65" s="8"/>
@@ -17675,14 +17659,14 @@
       <c r="HR65" s="8"/>
     </row>
     <row r="66" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="67"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67"/>
+      <c r="A66" s="59"/>
+      <c r="B66" s="59"/>
+      <c r="C66" s="59"/>
       <c r="D66" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="67"/>
-      <c r="F66" s="67"/>
+      <c r="E66" s="59"/>
+      <c r="F66" s="59"/>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
@@ -17717,11 +17701,11 @@
       <c r="AL66" s="8"/>
       <c r="AM66" s="9"/>
       <c r="AN66" s="10"/>
-      <c r="AO66" s="11"/>
+      <c r="AO66" s="47"/>
       <c r="AQ66" s="8"/>
       <c r="AR66" s="8"/>
       <c r="AS66" s="8"/>
-      <c r="AT66" s="9"/>
+      <c r="AT66" s="81"/>
       <c r="AU66" s="10"/>
       <c r="AV66" s="11"/>
       <c r="AW66" s="8"/>
@@ -17904,22 +17888,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="68" t="s">
+      <c r="A67" s="69" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="73" t="s">
+      <c r="B67" s="60" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="69" t="s">
+      <c r="C67" s="62" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="72" t="s">
+      <c r="E67" s="61" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="74" t="s">
+      <c r="F67" s="63" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -17956,11 +17940,11 @@
       <c r="AL67" s="8"/>
       <c r="AM67" s="9"/>
       <c r="AN67" s="10"/>
-      <c r="AO67" s="11"/>
+      <c r="AO67" s="47"/>
       <c r="AQ67" s="8"/>
       <c r="AR67" s="7"/>
       <c r="AS67" s="8"/>
-      <c r="AT67" s="9"/>
+      <c r="AT67" s="81"/>
       <c r="AU67" s="10"/>
       <c r="AV67" s="11"/>
       <c r="AW67" s="8"/>
@@ -18143,14 +18127,14 @@
       <c r="HR67" s="8"/>
     </row>
     <row r="68" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="67"/>
-      <c r="B68" s="67"/>
-      <c r="C68" s="67"/>
+      <c r="A68" s="59"/>
+      <c r="B68" s="59"/>
+      <c r="C68" s="59"/>
       <c r="D68" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="67"/>
-      <c r="F68" s="67"/>
+      <c r="E68" s="59"/>
+      <c r="F68" s="59"/>
       <c r="G68" s="8"/>
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
@@ -18185,11 +18169,11 @@
       <c r="AL68" s="8"/>
       <c r="AM68" s="9"/>
       <c r="AN68" s="10"/>
-      <c r="AO68" s="11"/>
+      <c r="AO68" s="47"/>
       <c r="AQ68" s="8"/>
       <c r="AR68" s="8"/>
       <c r="AS68" s="8"/>
-      <c r="AT68" s="9"/>
+      <c r="AT68" s="81"/>
       <c r="AU68" s="10"/>
       <c r="AV68" s="11"/>
       <c r="AW68" s="8"/>
@@ -18372,20 +18356,20 @@
       <c r="HR68" s="8"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="67"/>
-      <c r="B69" s="73" t="s">
+      <c r="A69" s="59"/>
+      <c r="B69" s="60" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="69" t="s">
+      <c r="C69" s="62" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="72" t="s">
+      <c r="E69" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="74" t="s">
+      <c r="F69" s="63" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18422,12 +18406,12 @@
       <c r="AL69" s="16"/>
       <c r="AM69" s="9"/>
       <c r="AN69" s="10"/>
-      <c r="AO69" s="11"/>
-      <c r="AP69" s="62"/>
+      <c r="AO69" s="47"/>
+      <c r="AP69" s="54"/>
       <c r="AQ69" s="16"/>
       <c r="AR69" s="16"/>
       <c r="AS69" s="16"/>
-      <c r="AT69" s="9"/>
+      <c r="AT69" s="81"/>
       <c r="AU69" s="10"/>
       <c r="AV69" s="11"/>
       <c r="AW69" s="16"/>
@@ -18610,14 +18594,14 @@
       <c r="HR69" s="8"/>
     </row>
     <row r="70" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="67"/>
-      <c r="B70" s="67"/>
-      <c r="C70" s="67"/>
+      <c r="A70" s="59"/>
+      <c r="B70" s="59"/>
+      <c r="C70" s="59"/>
       <c r="D70" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="67"/>
-      <c r="F70" s="67"/>
+      <c r="E70" s="59"/>
+      <c r="F70" s="59"/>
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
       <c r="I70" s="8"/>
@@ -18652,11 +18636,11 @@
       <c r="AL70" s="8"/>
       <c r="AM70" s="9"/>
       <c r="AN70" s="10"/>
-      <c r="AO70" s="11"/>
+      <c r="AO70" s="47"/>
       <c r="AQ70" s="8"/>
       <c r="AR70" s="8"/>
       <c r="AS70" s="8"/>
-      <c r="AT70" s="9"/>
+      <c r="AT70" s="81"/>
       <c r="AU70" s="10"/>
       <c r="AV70" s="11"/>
       <c r="AW70" s="8"/>
@@ -18839,20 +18823,20 @@
       <c r="HR70" s="8"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="67"/>
-      <c r="B71" s="73" t="s">
+      <c r="A71" s="59"/>
+      <c r="B71" s="60" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="69" t="s">
+      <c r="C71" s="62" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="72" t="s">
+      <c r="E71" s="61" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="74" t="s">
+      <c r="F71" s="63" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -18889,11 +18873,11 @@
       <c r="AL71" s="8"/>
       <c r="AM71" s="9"/>
       <c r="AN71" s="10"/>
-      <c r="AO71" s="11"/>
+      <c r="AO71" s="47"/>
       <c r="AQ71" s="8"/>
       <c r="AR71" s="8"/>
       <c r="AS71" s="8"/>
-      <c r="AT71" s="9"/>
+      <c r="AT71" s="81"/>
       <c r="AU71" s="10"/>
       <c r="AV71" s="11"/>
       <c r="AW71" s="8"/>
@@ -19076,14 +19060,14 @@
       <c r="HR71" s="8"/>
     </row>
     <row r="72" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="67"/>
-      <c r="B72" s="67"/>
-      <c r="C72" s="67"/>
+      <c r="A72" s="59"/>
+      <c r="B72" s="59"/>
+      <c r="C72" s="59"/>
       <c r="D72" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="67"/>
-      <c r="F72" s="67"/>
+      <c r="E72" s="59"/>
+      <c r="F72" s="59"/>
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
@@ -19118,11 +19102,11 @@
       <c r="AL72" s="8"/>
       <c r="AM72" s="9"/>
       <c r="AN72" s="10"/>
-      <c r="AO72" s="11"/>
+      <c r="AO72" s="47"/>
       <c r="AQ72" s="8"/>
       <c r="AR72" s="8"/>
       <c r="AS72" s="8"/>
-      <c r="AT72" s="9"/>
+      <c r="AT72" s="81"/>
       <c r="AU72" s="10"/>
       <c r="AV72" s="11"/>
       <c r="AW72" s="8"/>
@@ -19305,20 +19289,20 @@
       <c r="HR72" s="8"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="67"/>
-      <c r="B73" s="73" t="s">
+      <c r="A73" s="59"/>
+      <c r="B73" s="60" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="69" t="s">
+      <c r="C73" s="62" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="72" t="s">
+      <c r="E73" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="74" t="s">
+      <c r="F73" s="63" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19355,11 +19339,11 @@
       <c r="AL73" s="8"/>
       <c r="AM73" s="9"/>
       <c r="AN73" s="10"/>
-      <c r="AO73" s="11"/>
+      <c r="AO73" s="47"/>
       <c r="AQ73" s="8"/>
       <c r="AR73" s="8"/>
       <c r="AS73" s="8"/>
-      <c r="AT73" s="9"/>
+      <c r="AT73" s="81"/>
       <c r="AU73" s="10"/>
       <c r="AV73" s="11"/>
       <c r="AW73" s="8"/>
@@ -19542,14 +19526,14 @@
       <c r="HR73" s="8"/>
     </row>
     <row r="74" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="67"/>
-      <c r="B74" s="67"/>
-      <c r="C74" s="67"/>
+      <c r="A74" s="59"/>
+      <c r="B74" s="59"/>
+      <c r="C74" s="59"/>
       <c r="D74" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="67"/>
-      <c r="F74" s="67"/>
+      <c r="E74" s="59"/>
+      <c r="F74" s="59"/>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>
@@ -19584,11 +19568,11 @@
       <c r="AL74" s="8"/>
       <c r="AM74" s="9"/>
       <c r="AN74" s="10"/>
-      <c r="AO74" s="11"/>
+      <c r="AO74" s="47"/>
       <c r="AQ74" s="8"/>
       <c r="AR74" s="8"/>
       <c r="AS74" s="8"/>
-      <c r="AT74" s="9"/>
+      <c r="AT74" s="81"/>
       <c r="AU74" s="10"/>
       <c r="AV74" s="11"/>
       <c r="AW74" s="8"/>
@@ -19771,20 +19755,20 @@
       <c r="HR74" s="8"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="67"/>
-      <c r="B75" s="73" t="s">
+      <c r="A75" s="59"/>
+      <c r="B75" s="60" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="69" t="s">
+      <c r="C75" s="62" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="72" t="s">
+      <c r="E75" s="61" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="74" t="s">
+      <c r="F75" s="63" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19821,11 +19805,11 @@
       <c r="AL75" s="8"/>
       <c r="AM75" s="9"/>
       <c r="AN75" s="10"/>
-      <c r="AO75" s="11"/>
+      <c r="AO75" s="47"/>
       <c r="AQ75" s="8"/>
       <c r="AR75" s="8"/>
       <c r="AS75" s="8"/>
-      <c r="AT75" s="9"/>
+      <c r="AT75" s="81"/>
       <c r="AU75" s="10"/>
       <c r="AV75" s="11"/>
       <c r="AW75" s="8"/>
@@ -20008,14 +19992,14 @@
       <c r="HR75" s="8"/>
     </row>
     <row r="76" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="67"/>
-      <c r="B76" s="67"/>
-      <c r="C76" s="67"/>
+      <c r="A76" s="59"/>
+      <c r="B76" s="59"/>
+      <c r="C76" s="59"/>
       <c r="D76" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="67"/>
-      <c r="F76" s="67"/>
+      <c r="E76" s="59"/>
+      <c r="F76" s="59"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
       <c r="I76" s="8"/>
@@ -20050,11 +20034,11 @@
       <c r="AL76" s="8"/>
       <c r="AM76" s="9"/>
       <c r="AN76" s="10"/>
-      <c r="AO76" s="11"/>
+      <c r="AO76" s="47"/>
       <c r="AQ76" s="8"/>
       <c r="AR76" s="8"/>
       <c r="AS76" s="8"/>
-      <c r="AT76" s="9"/>
+      <c r="AT76" s="81"/>
       <c r="AU76" s="10"/>
       <c r="AV76" s="11"/>
       <c r="AW76" s="8"/>
@@ -20237,20 +20221,20 @@
       <c r="HR76" s="8"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="67"/>
-      <c r="B77" s="73" t="s">
+      <c r="A77" s="59"/>
+      <c r="B77" s="60" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="69" t="s">
+      <c r="C77" s="62" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="72" t="s">
+      <c r="E77" s="61" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="74" t="s">
+      <c r="F77" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20287,11 +20271,11 @@
       <c r="AL77" s="8"/>
       <c r="AM77" s="9"/>
       <c r="AN77" s="10"/>
-      <c r="AO77" s="11"/>
+      <c r="AO77" s="47"/>
       <c r="AQ77" s="8"/>
       <c r="AR77" s="8"/>
       <c r="AS77" s="8"/>
-      <c r="AT77" s="9"/>
+      <c r="AT77" s="81"/>
       <c r="AU77" s="10"/>
       <c r="AV77" s="11"/>
       <c r="AW77" s="8"/>
@@ -20474,14 +20458,14 @@
       <c r="HR77" s="8"/>
     </row>
     <row r="78" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="67"/>
-      <c r="B78" s="67"/>
-      <c r="C78" s="67"/>
+      <c r="A78" s="59"/>
+      <c r="B78" s="59"/>
+      <c r="C78" s="59"/>
       <c r="D78" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="67"/>
-      <c r="F78" s="67"/>
+      <c r="E78" s="59"/>
+      <c r="F78" s="59"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
       <c r="I78" s="8"/>
@@ -20516,11 +20500,11 @@
       <c r="AL78" s="8"/>
       <c r="AM78" s="9"/>
       <c r="AN78" s="10"/>
-      <c r="AO78" s="11"/>
+      <c r="AO78" s="47"/>
       <c r="AQ78" s="8"/>
       <c r="AR78" s="8"/>
       <c r="AS78" s="8"/>
-      <c r="AT78" s="9"/>
+      <c r="AT78" s="81"/>
       <c r="AU78" s="10"/>
       <c r="AV78" s="11"/>
       <c r="AW78" s="8"/>
@@ -20703,22 +20687,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="68" t="s">
+      <c r="A79" s="69" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="73" t="s">
+      <c r="B79" s="60" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="76" t="s">
+      <c r="C79" s="58" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="72" t="s">
+      <c r="E79" s="61" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="74" t="s">
+      <c r="F79" s="63" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20755,11 +20739,11 @@
       <c r="AL79" s="8"/>
       <c r="AM79" s="9"/>
       <c r="AN79" s="10"/>
-      <c r="AO79" s="11"/>
+      <c r="AO79" s="47"/>
       <c r="AQ79" s="8"/>
       <c r="AR79" s="8"/>
       <c r="AS79" s="8"/>
-      <c r="AT79" s="9"/>
+      <c r="AT79" s="81"/>
       <c r="AU79" s="10"/>
       <c r="AV79" s="11"/>
       <c r="AW79" s="8"/>
@@ -20942,14 +20926,14 @@
       <c r="HR79" s="8"/>
     </row>
     <row r="80" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="67"/>
-      <c r="B80" s="67"/>
-      <c r="C80" s="67"/>
+      <c r="A80" s="59"/>
+      <c r="B80" s="59"/>
+      <c r="C80" s="59"/>
       <c r="D80" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="67"/>
-      <c r="F80" s="67"/>
+      <c r="E80" s="59"/>
+      <c r="F80" s="59"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
       <c r="I80" s="8"/>
@@ -20984,11 +20968,11 @@
       <c r="AL80" s="8"/>
       <c r="AM80" s="9"/>
       <c r="AN80" s="10"/>
-      <c r="AO80" s="11"/>
+      <c r="AO80" s="47"/>
       <c r="AQ80" s="8"/>
       <c r="AR80" s="8"/>
       <c r="AS80" s="8"/>
-      <c r="AT80" s="9"/>
+      <c r="AT80" s="81"/>
       <c r="AU80" s="10"/>
       <c r="AV80" s="11"/>
       <c r="AW80" s="8"/>
@@ -21171,20 +21155,20 @@
       <c r="HR80" s="8"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="67"/>
-      <c r="B81" s="73" t="s">
+      <c r="A81" s="59"/>
+      <c r="B81" s="60" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="76" t="s">
+      <c r="C81" s="58" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="72" t="s">
+      <c r="E81" s="61" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="74" t="s">
+      <c r="F81" s="63" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -21221,11 +21205,11 @@
       <c r="AL81" s="8"/>
       <c r="AM81" s="9"/>
       <c r="AN81" s="10"/>
-      <c r="AO81" s="11"/>
+      <c r="AO81" s="47"/>
       <c r="AQ81" s="8"/>
       <c r="AR81" s="8"/>
       <c r="AS81" s="8"/>
-      <c r="AT81" s="9"/>
+      <c r="AT81" s="81"/>
       <c r="AU81" s="10"/>
       <c r="AV81" s="11"/>
       <c r="AW81" s="8"/>
@@ -21408,14 +21392,14 @@
       <c r="HR81" s="8"/>
     </row>
     <row r="82" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="67"/>
-      <c r="B82" s="67"/>
-      <c r="C82" s="67"/>
+      <c r="A82" s="59"/>
+      <c r="B82" s="59"/>
+      <c r="C82" s="59"/>
       <c r="D82" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="67"/>
-      <c r="F82" s="67"/>
+      <c r="E82" s="59"/>
+      <c r="F82" s="59"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
       <c r="I82" s="8"/>
@@ -21450,11 +21434,11 @@
       <c r="AL82" s="8"/>
       <c r="AM82" s="9"/>
       <c r="AN82" s="10"/>
-      <c r="AO82" s="11"/>
+      <c r="AO82" s="47"/>
       <c r="AQ82" s="8"/>
       <c r="AR82" s="8"/>
       <c r="AS82" s="8"/>
-      <c r="AT82" s="9"/>
+      <c r="AT82" s="81"/>
       <c r="AU82" s="10"/>
       <c r="AV82" s="11"/>
       <c r="AW82" s="8"/>
@@ -21637,20 +21621,20 @@
       <c r="HR82" s="8"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="67"/>
-      <c r="B83" s="73" t="s">
+      <c r="A83" s="59"/>
+      <c r="B83" s="60" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="69" t="s">
+      <c r="C83" s="62" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="72" t="s">
+      <c r="E83" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="74" t="s">
+      <c r="F83" s="63" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21687,11 +21671,11 @@
       <c r="AL83" s="8"/>
       <c r="AM83" s="9"/>
       <c r="AN83" s="10"/>
-      <c r="AO83" s="11"/>
+      <c r="AO83" s="47"/>
       <c r="AQ83" s="8"/>
       <c r="AR83" s="8"/>
       <c r="AS83" s="8"/>
-      <c r="AT83" s="9"/>
+      <c r="AT83" s="81"/>
       <c r="AU83" s="10"/>
       <c r="AV83" s="11"/>
       <c r="AW83" s="8"/>
@@ -21874,14 +21858,14 @@
       <c r="HR83" s="8"/>
     </row>
     <row r="84" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="67"/>
-      <c r="B84" s="67"/>
-      <c r="C84" s="67"/>
+      <c r="A84" s="59"/>
+      <c r="B84" s="59"/>
+      <c r="C84" s="59"/>
       <c r="D84" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="67"/>
-      <c r="F84" s="67"/>
+      <c r="E84" s="59"/>
+      <c r="F84" s="59"/>
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
@@ -21916,11 +21900,11 @@
       <c r="AL84" s="8"/>
       <c r="AM84" s="9"/>
       <c r="AN84" s="10"/>
-      <c r="AO84" s="11"/>
+      <c r="AO84" s="47"/>
       <c r="AQ84" s="8"/>
       <c r="AR84" s="8"/>
       <c r="AS84" s="8"/>
-      <c r="AT84" s="9"/>
+      <c r="AT84" s="81"/>
       <c r="AU84" s="10"/>
       <c r="AV84" s="11"/>
       <c r="AW84" s="8"/>
@@ -22103,20 +22087,20 @@
       <c r="HR84" s="8"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="67"/>
-      <c r="B85" s="73" t="s">
+      <c r="A85" s="59"/>
+      <c r="B85" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="80" t="s">
+      <c r="C85" s="71" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="72" t="s">
+      <c r="E85" s="61" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="74"/>
+      <c r="F85" s="63"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -22151,11 +22135,11 @@
       <c r="AL85" s="8"/>
       <c r="AM85" s="9"/>
       <c r="AN85" s="10"/>
-      <c r="AO85" s="11"/>
+      <c r="AO85" s="47"/>
       <c r="AQ85" s="8"/>
       <c r="AR85" s="8"/>
       <c r="AS85" s="8"/>
-      <c r="AT85" s="9"/>
+      <c r="AT85" s="81"/>
       <c r="AU85" s="10"/>
       <c r="AV85" s="11"/>
       <c r="AW85" s="8"/>
@@ -22338,14 +22322,14 @@
       <c r="HR85" s="17"/>
     </row>
     <row r="86" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="67"/>
-      <c r="B86" s="67"/>
-      <c r="C86" s="67"/>
+      <c r="A86" s="59"/>
+      <c r="B86" s="59"/>
+      <c r="C86" s="59"/>
       <c r="D86" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="67"/>
-      <c r="F86" s="67"/>
+      <c r="E86" s="59"/>
+      <c r="F86" s="59"/>
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
@@ -22380,11 +22364,11 @@
       <c r="AL86" s="8"/>
       <c r="AM86" s="9"/>
       <c r="AN86" s="10"/>
-      <c r="AO86" s="11"/>
+      <c r="AO86" s="47"/>
       <c r="AQ86" s="8"/>
       <c r="AR86" s="8"/>
       <c r="AS86" s="8"/>
-      <c r="AT86" s="9"/>
+      <c r="AT86" s="81"/>
       <c r="AU86" s="10"/>
       <c r="AV86" s="11"/>
       <c r="AW86" s="8"/>
@@ -22568,6 +22552,187 @@
     </row>
   </sheetData>
   <mergeCells count="205">
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
     <mergeCell ref="C79:C80"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="E79:E80"/>
@@ -22592,187 +22757,6 @@
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="AP1:AV1"/>
     <mergeCell ref="E59:E60"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ersten Draft für Intro, Methodologie und Motivation erstellt
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8502F956-9277-4D55-9E71-9982CE897119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{555DB17D-D7C6-4413-8180-244C296AC2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1255,58 +1255,58 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1623,298 +1623,299 @@
     <col min="43" max="45" width="2.140625" customWidth="1"/>
     <col min="46" max="46" width="2.140625" style="58" customWidth="1"/>
     <col min="47" max="48" width="2.140625" customWidth="1"/>
-    <col min="49" max="49" width="2.140625" style="66" customWidth="1"/>
-    <col min="50" max="226" width="2.140625" customWidth="1"/>
+    <col min="49" max="49" width="2.140625" style="67" customWidth="1"/>
+    <col min="50" max="50" width="2.140625" style="66" customWidth="1"/>
+    <col min="51" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="67" t="s">
+      <c r="G1" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="67" t="s">
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="67" t="s">
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="75"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="83" t="s">
+      <c r="V1" s="75"/>
+      <c r="W1" s="75"/>
+      <c r="X1" s="75"/>
+      <c r="Y1" s="75"/>
+      <c r="Z1" s="75"/>
+      <c r="AA1" s="75"/>
+      <c r="AB1" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="68"/>
-      <c r="AD1" s="68"/>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="68"/>
-      <c r="AG1" s="68"/>
-      <c r="AH1" s="68"/>
-      <c r="AI1" s="67" t="s">
+      <c r="AC1" s="75"/>
+      <c r="AD1" s="75"/>
+      <c r="AE1" s="75"/>
+      <c r="AF1" s="75"/>
+      <c r="AG1" s="75"/>
+      <c r="AH1" s="75"/>
+      <c r="AI1" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="68"/>
-      <c r="AK1" s="68"/>
-      <c r="AL1" s="68"/>
-      <c r="AM1" s="68"/>
-      <c r="AN1" s="68"/>
-      <c r="AO1" s="68"/>
-      <c r="AP1" s="67" t="s">
+      <c r="AJ1" s="75"/>
+      <c r="AK1" s="75"/>
+      <c r="AL1" s="75"/>
+      <c r="AM1" s="75"/>
+      <c r="AN1" s="75"/>
+      <c r="AO1" s="75"/>
+      <c r="AP1" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="68"/>
-      <c r="AR1" s="68"/>
-      <c r="AS1" s="68"/>
-      <c r="AT1" s="68"/>
-      <c r="AU1" s="68"/>
-      <c r="AV1" s="68"/>
-      <c r="AW1" s="67" t="s">
+      <c r="AQ1" s="75"/>
+      <c r="AR1" s="75"/>
+      <c r="AS1" s="75"/>
+      <c r="AT1" s="75"/>
+      <c r="AU1" s="75"/>
+      <c r="AV1" s="75"/>
+      <c r="AW1" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="68"/>
-      <c r="AY1" s="68"/>
-      <c r="AZ1" s="68"/>
-      <c r="BA1" s="68"/>
-      <c r="BB1" s="68"/>
-      <c r="BC1" s="68"/>
-      <c r="BD1" s="67" t="s">
+      <c r="AX1" s="75"/>
+      <c r="AY1" s="75"/>
+      <c r="AZ1" s="75"/>
+      <c r="BA1" s="75"/>
+      <c r="BB1" s="75"/>
+      <c r="BC1" s="75"/>
+      <c r="BD1" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="68"/>
-      <c r="BF1" s="68"/>
-      <c r="BG1" s="68"/>
-      <c r="BH1" s="68"/>
-      <c r="BI1" s="68"/>
-      <c r="BJ1" s="68"/>
-      <c r="BK1" s="67" t="s">
+      <c r="BE1" s="75"/>
+      <c r="BF1" s="75"/>
+      <c r="BG1" s="75"/>
+      <c r="BH1" s="75"/>
+      <c r="BI1" s="75"/>
+      <c r="BJ1" s="75"/>
+      <c r="BK1" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="68"/>
-      <c r="BM1" s="68"/>
-      <c r="BN1" s="68"/>
-      <c r="BO1" s="68"/>
-      <c r="BP1" s="68"/>
-      <c r="BQ1" s="68"/>
-      <c r="BR1" s="67" t="s">
+      <c r="BL1" s="75"/>
+      <c r="BM1" s="75"/>
+      <c r="BN1" s="75"/>
+      <c r="BO1" s="75"/>
+      <c r="BP1" s="75"/>
+      <c r="BQ1" s="75"/>
+      <c r="BR1" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="68"/>
-      <c r="BT1" s="68"/>
-      <c r="BU1" s="68"/>
-      <c r="BV1" s="68"/>
-      <c r="BW1" s="68"/>
-      <c r="BX1" s="68"/>
-      <c r="BY1" s="67" t="s">
+      <c r="BS1" s="75"/>
+      <c r="BT1" s="75"/>
+      <c r="BU1" s="75"/>
+      <c r="BV1" s="75"/>
+      <c r="BW1" s="75"/>
+      <c r="BX1" s="75"/>
+      <c r="BY1" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="68"/>
-      <c r="CA1" s="68"/>
-      <c r="CB1" s="68"/>
-      <c r="CC1" s="68"/>
-      <c r="CD1" s="68"/>
-      <c r="CE1" s="68"/>
-      <c r="CF1" s="67" t="s">
+      <c r="BZ1" s="75"/>
+      <c r="CA1" s="75"/>
+      <c r="CB1" s="75"/>
+      <c r="CC1" s="75"/>
+      <c r="CD1" s="75"/>
+      <c r="CE1" s="75"/>
+      <c r="CF1" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="68"/>
-      <c r="CH1" s="68"/>
-      <c r="CI1" s="68"/>
-      <c r="CJ1" s="68"/>
-      <c r="CK1" s="68"/>
-      <c r="CL1" s="68"/>
-      <c r="CM1" s="67" t="s">
+      <c r="CG1" s="75"/>
+      <c r="CH1" s="75"/>
+      <c r="CI1" s="75"/>
+      <c r="CJ1" s="75"/>
+      <c r="CK1" s="75"/>
+      <c r="CL1" s="75"/>
+      <c r="CM1" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="68"/>
-      <c r="CO1" s="68"/>
-      <c r="CP1" s="68"/>
-      <c r="CQ1" s="68"/>
-      <c r="CR1" s="68"/>
-      <c r="CS1" s="68"/>
-      <c r="CT1" s="67" t="s">
+      <c r="CN1" s="75"/>
+      <c r="CO1" s="75"/>
+      <c r="CP1" s="75"/>
+      <c r="CQ1" s="75"/>
+      <c r="CR1" s="75"/>
+      <c r="CS1" s="75"/>
+      <c r="CT1" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="68"/>
-      <c r="CV1" s="68"/>
-      <c r="CW1" s="68"/>
-      <c r="CX1" s="68"/>
-      <c r="CY1" s="68"/>
-      <c r="CZ1" s="68"/>
-      <c r="DA1" s="67" t="s">
+      <c r="CU1" s="75"/>
+      <c r="CV1" s="75"/>
+      <c r="CW1" s="75"/>
+      <c r="CX1" s="75"/>
+      <c r="CY1" s="75"/>
+      <c r="CZ1" s="75"/>
+      <c r="DA1" s="80" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="68"/>
-      <c r="DC1" s="68"/>
-      <c r="DD1" s="68"/>
-      <c r="DE1" s="68"/>
-      <c r="DF1" s="68"/>
-      <c r="DG1" s="68"/>
-      <c r="DH1" s="67" t="s">
+      <c r="DB1" s="75"/>
+      <c r="DC1" s="75"/>
+      <c r="DD1" s="75"/>
+      <c r="DE1" s="75"/>
+      <c r="DF1" s="75"/>
+      <c r="DG1" s="75"/>
+      <c r="DH1" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="68"/>
-      <c r="DJ1" s="68"/>
-      <c r="DK1" s="68"/>
-      <c r="DL1" s="68"/>
-      <c r="DM1" s="68"/>
-      <c r="DN1" s="68"/>
-      <c r="DO1" s="67" t="s">
+      <c r="DI1" s="75"/>
+      <c r="DJ1" s="75"/>
+      <c r="DK1" s="75"/>
+      <c r="DL1" s="75"/>
+      <c r="DM1" s="75"/>
+      <c r="DN1" s="75"/>
+      <c r="DO1" s="80" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="68"/>
-      <c r="DQ1" s="68"/>
-      <c r="DR1" s="68"/>
-      <c r="DS1" s="68"/>
-      <c r="DT1" s="68"/>
-      <c r="DU1" s="68"/>
-      <c r="DV1" s="67" t="s">
+      <c r="DP1" s="75"/>
+      <c r="DQ1" s="75"/>
+      <c r="DR1" s="75"/>
+      <c r="DS1" s="75"/>
+      <c r="DT1" s="75"/>
+      <c r="DU1" s="75"/>
+      <c r="DV1" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="68"/>
-      <c r="DX1" s="68"/>
-      <c r="DY1" s="68"/>
-      <c r="DZ1" s="68"/>
-      <c r="EA1" s="68"/>
-      <c r="EB1" s="68"/>
-      <c r="EC1" s="67" t="s">
+      <c r="DW1" s="75"/>
+      <c r="DX1" s="75"/>
+      <c r="DY1" s="75"/>
+      <c r="DZ1" s="75"/>
+      <c r="EA1" s="75"/>
+      <c r="EB1" s="75"/>
+      <c r="EC1" s="80" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="68"/>
-      <c r="EE1" s="68"/>
-      <c r="EF1" s="68"/>
-      <c r="EG1" s="68"/>
-      <c r="EH1" s="68"/>
-      <c r="EI1" s="68"/>
-      <c r="EJ1" s="67" t="s">
+      <c r="ED1" s="75"/>
+      <c r="EE1" s="75"/>
+      <c r="EF1" s="75"/>
+      <c r="EG1" s="75"/>
+      <c r="EH1" s="75"/>
+      <c r="EI1" s="75"/>
+      <c r="EJ1" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="68"/>
-      <c r="EL1" s="68"/>
-      <c r="EM1" s="68"/>
-      <c r="EN1" s="68"/>
-      <c r="EO1" s="68"/>
-      <c r="EP1" s="68"/>
-      <c r="EQ1" s="67" t="s">
+      <c r="EK1" s="75"/>
+      <c r="EL1" s="75"/>
+      <c r="EM1" s="75"/>
+      <c r="EN1" s="75"/>
+      <c r="EO1" s="75"/>
+      <c r="EP1" s="75"/>
+      <c r="EQ1" s="80" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="68"/>
-      <c r="ES1" s="68"/>
-      <c r="ET1" s="68"/>
-      <c r="EU1" s="68"/>
-      <c r="EV1" s="68"/>
-      <c r="EW1" s="68"/>
-      <c r="EX1" s="67" t="s">
+      <c r="ER1" s="75"/>
+      <c r="ES1" s="75"/>
+      <c r="ET1" s="75"/>
+      <c r="EU1" s="75"/>
+      <c r="EV1" s="75"/>
+      <c r="EW1" s="75"/>
+      <c r="EX1" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="68"/>
-      <c r="EZ1" s="68"/>
-      <c r="FA1" s="68"/>
-      <c r="FB1" s="68"/>
-      <c r="FC1" s="68"/>
-      <c r="FD1" s="68"/>
-      <c r="FE1" s="67" t="s">
+      <c r="EY1" s="75"/>
+      <c r="EZ1" s="75"/>
+      <c r="FA1" s="75"/>
+      <c r="FB1" s="75"/>
+      <c r="FC1" s="75"/>
+      <c r="FD1" s="75"/>
+      <c r="FE1" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="68"/>
-      <c r="FG1" s="68"/>
-      <c r="FH1" s="68"/>
-      <c r="FI1" s="68"/>
-      <c r="FJ1" s="68"/>
-      <c r="FK1" s="68"/>
-      <c r="FL1" s="67" t="s">
+      <c r="FF1" s="75"/>
+      <c r="FG1" s="75"/>
+      <c r="FH1" s="75"/>
+      <c r="FI1" s="75"/>
+      <c r="FJ1" s="75"/>
+      <c r="FK1" s="75"/>
+      <c r="FL1" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="68"/>
-      <c r="FN1" s="68"/>
-      <c r="FO1" s="68"/>
-      <c r="FP1" s="68"/>
-      <c r="FQ1" s="68"/>
-      <c r="FR1" s="68"/>
-      <c r="FS1" s="67" t="s">
+      <c r="FM1" s="75"/>
+      <c r="FN1" s="75"/>
+      <c r="FO1" s="75"/>
+      <c r="FP1" s="75"/>
+      <c r="FQ1" s="75"/>
+      <c r="FR1" s="75"/>
+      <c r="FS1" s="80" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="68"/>
-      <c r="FU1" s="68"/>
-      <c r="FV1" s="68"/>
-      <c r="FW1" s="68"/>
-      <c r="FX1" s="68"/>
-      <c r="FY1" s="68"/>
-      <c r="FZ1" s="67" t="s">
+      <c r="FT1" s="75"/>
+      <c r="FU1" s="75"/>
+      <c r="FV1" s="75"/>
+      <c r="FW1" s="75"/>
+      <c r="FX1" s="75"/>
+      <c r="FY1" s="75"/>
+      <c r="FZ1" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="68"/>
-      <c r="GB1" s="68"/>
-      <c r="GC1" s="68"/>
-      <c r="GD1" s="68"/>
-      <c r="GE1" s="68"/>
-      <c r="GF1" s="68"/>
-      <c r="GG1" s="67" t="s">
+      <c r="GA1" s="75"/>
+      <c r="GB1" s="75"/>
+      <c r="GC1" s="75"/>
+      <c r="GD1" s="75"/>
+      <c r="GE1" s="75"/>
+      <c r="GF1" s="75"/>
+      <c r="GG1" s="80" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="68"/>
-      <c r="GI1" s="68"/>
-      <c r="GJ1" s="68"/>
-      <c r="GK1" s="68"/>
-      <c r="GL1" s="68"/>
-      <c r="GM1" s="68"/>
-      <c r="GN1" s="67" t="s">
+      <c r="GH1" s="75"/>
+      <c r="GI1" s="75"/>
+      <c r="GJ1" s="75"/>
+      <c r="GK1" s="75"/>
+      <c r="GL1" s="75"/>
+      <c r="GM1" s="75"/>
+      <c r="GN1" s="80" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="68"/>
-      <c r="GP1" s="68"/>
-      <c r="GQ1" s="68"/>
-      <c r="GR1" s="68"/>
-      <c r="GS1" s="68"/>
-      <c r="GT1" s="68"/>
-      <c r="GU1" s="67" t="s">
+      <c r="GO1" s="75"/>
+      <c r="GP1" s="75"/>
+      <c r="GQ1" s="75"/>
+      <c r="GR1" s="75"/>
+      <c r="GS1" s="75"/>
+      <c r="GT1" s="75"/>
+      <c r="GU1" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="68"/>
-      <c r="GW1" s="68"/>
-      <c r="GX1" s="68"/>
-      <c r="GY1" s="68"/>
-      <c r="GZ1" s="68"/>
-      <c r="HA1" s="68"/>
-      <c r="HB1" s="67" t="s">
+      <c r="GV1" s="75"/>
+      <c r="GW1" s="75"/>
+      <c r="GX1" s="75"/>
+      <c r="GY1" s="75"/>
+      <c r="GZ1" s="75"/>
+      <c r="HA1" s="75"/>
+      <c r="HB1" s="80" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="68"/>
-      <c r="HD1" s="68"/>
-      <c r="HE1" s="68"/>
-      <c r="HF1" s="68"/>
-      <c r="HG1" s="68"/>
-      <c r="HH1" s="68"/>
-      <c r="HI1" s="67" t="s">
+      <c r="HC1" s="75"/>
+      <c r="HD1" s="75"/>
+      <c r="HE1" s="75"/>
+      <c r="HF1" s="75"/>
+      <c r="HG1" s="75"/>
+      <c r="HH1" s="75"/>
+      <c r="HI1" s="80" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="68"/>
-      <c r="HK1" s="68"/>
-      <c r="HL1" s="68"/>
-      <c r="HM1" s="68"/>
-      <c r="HN1" s="68"/>
-      <c r="HO1" s="68"/>
-      <c r="HP1" s="67" t="s">
+      <c r="HJ1" s="75"/>
+      <c r="HK1" s="75"/>
+      <c r="HL1" s="75"/>
+      <c r="HM1" s="75"/>
+      <c r="HN1" s="75"/>
+      <c r="HO1" s="75"/>
+      <c r="HP1" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="68"/>
-      <c r="HR1" s="68"/>
+      <c r="HQ1" s="75"/>
+      <c r="HR1" s="75"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="1" t="s">
@@ -2046,10 +2047,10 @@
       <c r="AV2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AW2" s="63" t="s">
+      <c r="AW2" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="AX2" s="2" t="s">
+      <c r="AX2" s="63" t="s">
         <v>35</v>
       </c>
       <c r="AY2" s="2" t="s">
@@ -2711,10 +2712,10 @@
       <c r="AV3" s="3">
         <v>46292</v>
       </c>
-      <c r="AW3" s="64">
+      <c r="AW3" s="50">
         <v>46293</v>
       </c>
-      <c r="AX3" s="3">
+      <c r="AX3" s="64">
         <v>46294</v>
       </c>
       <c r="AY3" s="3">
@@ -3305,8 +3306,8 @@
       <c r="AT4" s="51"/>
       <c r="AU4" s="5"/>
       <c r="AV4" s="5"/>
-      <c r="AW4" s="65"/>
-      <c r="AX4" s="5"/>
+      <c r="AW4" s="51"/>
+      <c r="AX4" s="65"/>
       <c r="AY4" s="5"/>
       <c r="AZ4" s="5"/>
       <c r="BA4" s="5"/>
@@ -3485,20 +3486,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="82" t="s">
+      <c r="A5" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="78"/>
-      <c r="C5" s="71" t="s">
+      <c r="B5" s="86"/>
+      <c r="C5" s="84" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="76" t="s">
+      <c r="E5" s="88" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="80"/>
+      <c r="F5" s="82"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3537,10 +3538,9 @@
       <c r="AQ5" s="8"/>
       <c r="AR5" s="8"/>
       <c r="AS5" s="58"/>
-      <c r="AT5" s="84"/>
+      <c r="AT5" s="68"/>
       <c r="AU5" s="10"/>
-      <c r="AV5" s="11"/>
-      <c r="AX5" s="8"/>
+      <c r="AV5" s="47"/>
       <c r="AY5" s="8"/>
       <c r="AZ5" s="8"/>
       <c r="BA5" s="9"/>
@@ -3719,14 +3719,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="72"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="72"/>
+      <c r="A6" s="83"/>
+      <c r="B6" s="83"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="72"/>
-      <c r="F6" s="72"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="83"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3765,10 +3765,9 @@
       <c r="AQ6" s="8"/>
       <c r="AR6" s="8"/>
       <c r="AS6" s="58"/>
-      <c r="AT6" s="84"/>
+      <c r="AT6" s="68"/>
       <c r="AU6" s="10"/>
-      <c r="AV6" s="11"/>
-      <c r="AX6" s="8"/>
+      <c r="AV6" s="47"/>
       <c r="AY6" s="8"/>
       <c r="AZ6" s="8"/>
       <c r="BA6" s="9"/>
@@ -3947,18 +3946,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="72"/>
-      <c r="B7" s="78"/>
-      <c r="C7" s="71" t="s">
+      <c r="A7" s="83"/>
+      <c r="B7" s="86"/>
+      <c r="C7" s="84" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="76" t="s">
+      <c r="E7" s="88" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="80"/>
+      <c r="F7" s="82"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -3997,10 +3996,9 @@
       <c r="AQ7" s="8"/>
       <c r="AR7" s="8"/>
       <c r="AS7" s="58"/>
-      <c r="AT7" s="84"/>
+      <c r="AT7" s="68"/>
       <c r="AU7" s="10"/>
-      <c r="AV7" s="11"/>
-      <c r="AX7" s="8"/>
+      <c r="AV7" s="47"/>
       <c r="AY7" s="8"/>
       <c r="AZ7" s="8"/>
       <c r="BA7" s="9"/>
@@ -4179,14 +4177,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="72"/>
-      <c r="B8" s="72"/>
-      <c r="C8" s="72"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="83"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="72"/>
-      <c r="F8" s="72"/>
+      <c r="E8" s="83"/>
+      <c r="F8" s="83"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4225,10 +4223,9 @@
       <c r="AQ8" s="8"/>
       <c r="AR8" s="8"/>
       <c r="AS8" s="58"/>
-      <c r="AT8" s="84"/>
+      <c r="AT8" s="68"/>
       <c r="AU8" s="10"/>
-      <c r="AV8" s="11"/>
-      <c r="AX8" s="8"/>
+      <c r="AV8" s="47"/>
       <c r="AY8" s="8"/>
       <c r="AZ8" s="8"/>
       <c r="BA8" s="9"/>
@@ -4407,18 +4404,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="78"/>
-      <c r="C9" s="71" t="s">
+      <c r="A9" s="83"/>
+      <c r="B9" s="86"/>
+      <c r="C9" s="84" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="76" t="s">
+      <c r="E9" s="88" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="80"/>
+      <c r="F9" s="82"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4457,10 +4454,9 @@
       <c r="AQ9" s="8"/>
       <c r="AR9" s="8"/>
       <c r="AS9" s="58"/>
-      <c r="AT9" s="84"/>
+      <c r="AT9" s="68"/>
       <c r="AU9" s="10"/>
-      <c r="AV9" s="11"/>
-      <c r="AX9" s="8"/>
+      <c r="AV9" s="47"/>
       <c r="AY9" s="8"/>
       <c r="AZ9" s="8"/>
       <c r="BA9" s="9"/>
@@ -4639,14 +4635,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="72"/>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
+      <c r="A10" s="83"/>
+      <c r="B10" s="83"/>
+      <c r="C10" s="83"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="72"/>
-      <c r="F10" s="72"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4685,10 +4681,9 @@
       <c r="AQ10" s="8"/>
       <c r="AR10" s="8"/>
       <c r="AS10" s="58"/>
-      <c r="AT10" s="84"/>
+      <c r="AT10" s="68"/>
       <c r="AU10" s="10"/>
-      <c r="AV10" s="11"/>
-      <c r="AX10" s="8"/>
+      <c r="AV10" s="47"/>
       <c r="AY10" s="8"/>
       <c r="AZ10" s="8"/>
       <c r="BA10" s="9"/>
@@ -4867,18 +4862,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="72"/>
-      <c r="B11" s="78"/>
-      <c r="C11" s="71" t="s">
+      <c r="A11" s="83"/>
+      <c r="B11" s="86"/>
+      <c r="C11" s="84" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="76" t="s">
+      <c r="E11" s="88" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="80"/>
+      <c r="F11" s="82"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -4917,10 +4912,9 @@
       <c r="AQ11" s="8"/>
       <c r="AR11" s="8"/>
       <c r="AS11" s="58"/>
-      <c r="AT11" s="84"/>
+      <c r="AT11" s="68"/>
       <c r="AU11" s="10"/>
-      <c r="AV11" s="11"/>
-      <c r="AX11" s="8"/>
+      <c r="AV11" s="47"/>
       <c r="AY11" s="8"/>
       <c r="AZ11" s="8"/>
       <c r="BA11" s="9"/>
@@ -5099,14 +5093,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="72"/>
-      <c r="C12" s="72"/>
+      <c r="A12" s="83"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="83"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5145,10 +5139,9 @@
       <c r="AQ12" s="8"/>
       <c r="AR12" s="8"/>
       <c r="AS12" s="58"/>
-      <c r="AT12" s="84"/>
+      <c r="AT12" s="68"/>
       <c r="AU12" s="10"/>
-      <c r="AV12" s="11"/>
-      <c r="AX12" s="8"/>
+      <c r="AV12" s="47"/>
       <c r="AY12" s="8"/>
       <c r="AZ12" s="8"/>
       <c r="BA12" s="9"/>
@@ -5327,18 +5320,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="78"/>
-      <c r="C13" s="71" t="s">
+      <c r="A13" s="83"/>
+      <c r="B13" s="86"/>
+      <c r="C13" s="84" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="76" t="s">
+      <c r="E13" s="88" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="80"/>
+      <c r="F13" s="82"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5377,10 +5370,9 @@
       <c r="AQ13" s="8"/>
       <c r="AR13" s="8"/>
       <c r="AS13" s="58"/>
-      <c r="AT13" s="84"/>
+      <c r="AT13" s="68"/>
       <c r="AU13" s="10"/>
-      <c r="AV13" s="11"/>
-      <c r="AX13" s="8"/>
+      <c r="AV13" s="47"/>
       <c r="AY13" s="8"/>
       <c r="AZ13" s="8"/>
       <c r="BA13" s="9"/>
@@ -5559,14 +5551,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="72"/>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
+      <c r="A14" s="83"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5605,10 +5597,9 @@
       <c r="AQ14" s="8"/>
       <c r="AR14" s="8"/>
       <c r="AS14" s="58"/>
-      <c r="AT14" s="84"/>
+      <c r="AT14" s="68"/>
       <c r="AU14" s="10"/>
-      <c r="AV14" s="11"/>
-      <c r="AX14" s="8"/>
+      <c r="AV14" s="47"/>
       <c r="AY14" s="8"/>
       <c r="AZ14" s="8"/>
       <c r="BA14" s="9"/>
@@ -5787,18 +5778,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="72"/>
-      <c r="B15" s="78"/>
-      <c r="C15" s="71" t="s">
+      <c r="A15" s="83"/>
+      <c r="B15" s="86"/>
+      <c r="C15" s="84" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="76" t="s">
+      <c r="E15" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="80"/>
+      <c r="F15" s="82"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -5837,10 +5828,9 @@
       <c r="AQ15" s="8"/>
       <c r="AR15" s="8"/>
       <c r="AS15" s="58"/>
-      <c r="AT15" s="84"/>
+      <c r="AT15" s="68"/>
       <c r="AU15" s="10"/>
-      <c r="AV15" s="11"/>
-      <c r="AX15" s="8"/>
+      <c r="AV15" s="47"/>
       <c r="AY15" s="8"/>
       <c r="AZ15" s="8"/>
       <c r="BA15" s="9"/>
@@ -6019,14 +6009,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="72"/>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
+      <c r="A16" s="83"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="83"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6065,10 +6055,9 @@
       <c r="AQ16" s="8"/>
       <c r="AR16" s="8"/>
       <c r="AS16" s="58"/>
-      <c r="AT16" s="84"/>
+      <c r="AT16" s="68"/>
       <c r="AU16" s="10"/>
-      <c r="AV16" s="11"/>
-      <c r="AX16" s="8"/>
+      <c r="AV16" s="47"/>
       <c r="AY16" s="8"/>
       <c r="AZ16" s="8"/>
       <c r="BA16" s="9"/>
@@ -6247,18 +6236,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="72"/>
-      <c r="B17" s="78"/>
-      <c r="C17" s="71" t="s">
+      <c r="A17" s="83"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="84" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="76" t="s">
+      <c r="E17" s="88" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="80"/>
+      <c r="F17" s="82"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6297,10 +6286,9 @@
       <c r="AQ17" s="8"/>
       <c r="AR17" s="8"/>
       <c r="AS17" s="58"/>
-      <c r="AT17" s="84"/>
+      <c r="AT17" s="68"/>
       <c r="AU17" s="10"/>
-      <c r="AV17" s="11"/>
-      <c r="AX17" s="8"/>
+      <c r="AV17" s="47"/>
       <c r="AY17" s="8"/>
       <c r="AZ17" s="8"/>
       <c r="BA17" s="9"/>
@@ -6479,14 +6467,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="72"/>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
+      <c r="A18" s="83"/>
+      <c r="B18" s="83"/>
+      <c r="C18" s="83"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
+      <c r="E18" s="83"/>
+      <c r="F18" s="83"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6525,10 +6513,9 @@
       <c r="AQ18" s="8"/>
       <c r="AR18" s="8"/>
       <c r="AS18" s="58"/>
-      <c r="AT18" s="84"/>
+      <c r="AT18" s="68"/>
       <c r="AU18" s="10"/>
-      <c r="AV18" s="11"/>
-      <c r="AX18" s="8"/>
+      <c r="AV18" s="47"/>
       <c r="AY18" s="8"/>
       <c r="AZ18" s="8"/>
       <c r="BA18" s="9"/>
@@ -6707,18 +6694,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
-      <c r="B19" s="78"/>
-      <c r="C19" s="71" t="s">
+      <c r="A19" s="83"/>
+      <c r="B19" s="86"/>
+      <c r="C19" s="84" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="76" t="s">
+      <c r="E19" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="80"/>
+      <c r="F19" s="82"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6757,10 +6744,9 @@
       <c r="AQ19" s="8"/>
       <c r="AR19" s="8"/>
       <c r="AS19" s="58"/>
-      <c r="AT19" s="84"/>
+      <c r="AT19" s="68"/>
       <c r="AU19" s="10"/>
-      <c r="AV19" s="11"/>
-      <c r="AX19" s="8"/>
+      <c r="AV19" s="47"/>
       <c r="AY19" s="8"/>
       <c r="AZ19" s="8"/>
       <c r="BA19" s="9"/>
@@ -6939,14 +6925,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="72"/>
-      <c r="B20" s="72"/>
-      <c r="C20" s="72"/>
+      <c r="A20" s="83"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="83"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="72"/>
-      <c r="F20" s="72"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -6985,10 +6971,9 @@
       <c r="AQ20" s="8"/>
       <c r="AR20" s="8"/>
       <c r="AS20" s="58"/>
-      <c r="AT20" s="84"/>
+      <c r="AT20" s="68"/>
       <c r="AU20" s="10"/>
-      <c r="AV20" s="11"/>
-      <c r="AX20" s="8"/>
+      <c r="AV20" s="47"/>
       <c r="AY20" s="8"/>
       <c r="AZ20" s="8"/>
       <c r="BA20" s="9"/>
@@ -7167,18 +7152,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
-      <c r="B21" s="78"/>
-      <c r="C21" s="71" t="s">
+      <c r="A21" s="83"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="84" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="76" t="s">
+      <c r="E21" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="80"/>
+      <c r="F21" s="82"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7217,10 +7202,9 @@
       <c r="AQ21" s="8"/>
       <c r="AR21" s="8"/>
       <c r="AS21" s="58"/>
-      <c r="AT21" s="84"/>
+      <c r="AT21" s="68"/>
       <c r="AU21" s="10"/>
-      <c r="AV21" s="11"/>
-      <c r="AX21" s="8"/>
+      <c r="AV21" s="47"/>
       <c r="AY21" s="8"/>
       <c r="AZ21" s="8"/>
       <c r="BA21" s="9"/>
@@ -7399,14 +7383,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="79"/>
-      <c r="B22" s="79"/>
-      <c r="C22" s="79"/>
+      <c r="A22" s="89"/>
+      <c r="B22" s="89"/>
+      <c r="C22" s="89"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="79"/>
-      <c r="F22" s="79"/>
+      <c r="E22" s="89"/>
+      <c r="F22" s="89"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7445,11 +7429,10 @@
       <c r="AQ22" s="38"/>
       <c r="AR22" s="38"/>
       <c r="AS22" s="59"/>
-      <c r="AT22" s="84"/>
+      <c r="AT22" s="68"/>
       <c r="AU22" s="40"/>
-      <c r="AV22" s="41"/>
-      <c r="AW22" s="85"/>
-      <c r="AX22" s="38"/>
+      <c r="AV22" s="48"/>
+      <c r="AX22" s="69"/>
       <c r="AY22" s="38"/>
       <c r="AZ22" s="38"/>
       <c r="BA22" s="39"/>
@@ -7628,22 +7611,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="69" t="s">
+      <c r="A23" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="74" t="s">
+      <c r="B23" s="76" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="70" t="s">
+      <c r="C23" s="78" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="73" t="s">
+      <c r="E23" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="75" t="s">
+      <c r="F23" s="79" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7685,11 +7668,10 @@
       <c r="AQ23" s="8"/>
       <c r="AR23" s="8"/>
       <c r="AS23" s="58"/>
-      <c r="AT23" s="84"/>
+      <c r="AT23" s="68"/>
       <c r="AU23" s="10"/>
-      <c r="AV23" s="11"/>
-      <c r="AW23" s="86"/>
-      <c r="AX23" s="8"/>
+      <c r="AV23" s="47"/>
+      <c r="AW23" s="54"/>
       <c r="AY23" s="8"/>
       <c r="AZ23" s="8"/>
       <c r="BA23" s="9"/>
@@ -7868,14 +7850,14 @@
       <c r="HR23" s="8"/>
     </row>
     <row r="24" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="68"/>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
+      <c r="A24" s="75"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="75"/>
       <c r="D24" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
+      <c r="E24" s="75"/>
+      <c r="F24" s="75"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
@@ -7915,11 +7897,10 @@
       <c r="AQ24" s="8"/>
       <c r="AR24" s="8"/>
       <c r="AS24" s="58"/>
-      <c r="AT24" s="84"/>
+      <c r="AT24" s="68"/>
       <c r="AU24" s="10"/>
-      <c r="AV24" s="11"/>
-      <c r="AW24" s="88"/>
-      <c r="AX24" s="8"/>
+      <c r="AV24" s="47"/>
+      <c r="AW24" s="56"/>
       <c r="AY24" s="8"/>
       <c r="AZ24" s="8"/>
       <c r="BA24" s="9"/>
@@ -8098,20 +8079,20 @@
       <c r="HR24" s="8"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="68"/>
-      <c r="B25" s="74" t="s">
+      <c r="A25" s="75"/>
+      <c r="B25" s="76" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="70" t="s">
+      <c r="C25" s="78" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="73" t="s">
+      <c r="E25" s="77" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="75" t="s">
+      <c r="F25" s="79" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8149,10 +8130,9 @@
       <c r="AQ25" s="8"/>
       <c r="AR25" s="8"/>
       <c r="AS25" s="58"/>
-      <c r="AT25" s="84"/>
+      <c r="AT25" s="68"/>
       <c r="AU25" s="10"/>
-      <c r="AV25" s="11"/>
-      <c r="AX25" s="8"/>
+      <c r="AV25" s="47"/>
       <c r="AY25" s="8"/>
       <c r="BA25" s="9"/>
       <c r="BB25" s="10"/>
@@ -8326,14 +8306,14 @@
       <c r="HS25" s="8"/>
     </row>
     <row r="26" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="68"/>
-      <c r="B26" s="68"/>
-      <c r="C26" s="68"/>
+      <c r="A26" s="75"/>
+      <c r="B26" s="75"/>
+      <c r="C26" s="75"/>
       <c r="D26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="68"/>
-      <c r="F26" s="68"/>
+      <c r="E26" s="75"/>
+      <c r="F26" s="75"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
@@ -8372,10 +8352,9 @@
       <c r="AQ26" s="44"/>
       <c r="AR26" s="8"/>
       <c r="AS26" s="58"/>
-      <c r="AT26" s="84"/>
+      <c r="AT26" s="68"/>
       <c r="AU26" s="10"/>
-      <c r="AV26" s="11"/>
-      <c r="AX26" s="8"/>
+      <c r="AV26" s="47"/>
       <c r="AY26" s="8"/>
       <c r="AZ26" s="8"/>
       <c r="BA26" s="9"/>
@@ -8554,20 +8533,20 @@
       <c r="HR26" s="8"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="68"/>
-      <c r="B27" s="74" t="s">
+      <c r="A27" s="75"/>
+      <c r="B27" s="76" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="81" t="s">
+      <c r="C27" s="87" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="73" t="s">
+      <c r="E27" s="77" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="75"/>
+      <c r="F27" s="79"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8605,10 +8584,9 @@
       <c r="AO27" s="47"/>
       <c r="AQ27" s="8"/>
       <c r="AR27" s="8"/>
-      <c r="AT27" s="84"/>
+      <c r="AT27" s="68"/>
       <c r="AU27" s="10"/>
-      <c r="AV27" s="11"/>
-      <c r="AX27" s="8"/>
+      <c r="AV27" s="47"/>
       <c r="AY27" s="8"/>
       <c r="AZ27" s="17"/>
       <c r="BA27" s="9"/>
@@ -8787,14 +8765,14 @@
       <c r="HR27" s="8"/>
     </row>
     <row r="28" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="68"/>
-      <c r="B28" s="68"/>
-      <c r="C28" s="68"/>
+      <c r="A28" s="75"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
       <c r="D28" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="68"/>
-      <c r="F28" s="68"/>
+      <c r="E28" s="75"/>
+      <c r="F28" s="75"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
@@ -8832,10 +8810,9 @@
       <c r="AQ28" s="8"/>
       <c r="AR28" s="8"/>
       <c r="AS28" s="58"/>
-      <c r="AT28" s="84"/>
+      <c r="AT28" s="68"/>
       <c r="AU28" s="10"/>
-      <c r="AV28" s="11"/>
-      <c r="AX28" s="8"/>
+      <c r="AV28" s="47"/>
       <c r="AY28" s="8"/>
       <c r="AZ28" s="43"/>
       <c r="BA28" s="9"/>
@@ -9014,22 +8991,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="69" t="s">
+      <c r="A29" s="85" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="74" t="s">
+      <c r="B29" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="70" t="s">
+      <c r="C29" s="78" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="73" t="s">
+      <c r="E29" s="77" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="75" t="s">
+      <c r="F29" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9069,10 +9046,9 @@
       <c r="AQ29" s="8"/>
       <c r="AR29" s="8"/>
       <c r="AS29" s="58"/>
-      <c r="AT29" s="84"/>
+      <c r="AT29" s="68"/>
       <c r="AU29" s="10"/>
-      <c r="AV29" s="11"/>
-      <c r="AX29" s="8"/>
+      <c r="AV29" s="47"/>
       <c r="AY29" s="8"/>
       <c r="AZ29" s="8"/>
       <c r="BA29" s="9"/>
@@ -9251,14 +9227,14 @@
       <c r="HR29" s="8"/>
     </row>
     <row r="30" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="68"/>
-      <c r="B30" s="68"/>
-      <c r="C30" s="68"/>
+      <c r="A30" s="75"/>
+      <c r="B30" s="75"/>
+      <c r="C30" s="75"/>
       <c r="D30" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="68"/>
-      <c r="F30" s="68"/>
+      <c r="E30" s="75"/>
+      <c r="F30" s="75"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
@@ -9297,10 +9273,9 @@
       <c r="AQ30" s="8"/>
       <c r="AR30" s="8"/>
       <c r="AS30" s="58"/>
-      <c r="AT30" s="84"/>
+      <c r="AT30" s="68"/>
       <c r="AU30" s="10"/>
-      <c r="AV30" s="11"/>
-      <c r="AX30" s="8"/>
+      <c r="AV30" s="47"/>
       <c r="AY30" s="8"/>
       <c r="AZ30" s="8"/>
       <c r="BA30" s="9"/>
@@ -9479,20 +9454,20 @@
       <c r="HR30" s="8"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="68"/>
-      <c r="B31" s="74" t="s">
+      <c r="A31" s="75"/>
+      <c r="B31" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="70" t="s">
+      <c r="C31" s="78" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="73" t="s">
+      <c r="E31" s="77" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="75" t="s">
+      <c r="F31" s="79" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9533,10 +9508,9 @@
       <c r="AQ31" s="8"/>
       <c r="AR31" s="8"/>
       <c r="AS31" s="58"/>
-      <c r="AT31" s="84"/>
+      <c r="AT31" s="68"/>
       <c r="AU31" s="10"/>
-      <c r="AV31" s="11"/>
-      <c r="AX31" s="8"/>
+      <c r="AV31" s="47"/>
       <c r="AY31" s="8"/>
       <c r="AZ31" s="8"/>
       <c r="BA31" s="9"/>
@@ -9715,14 +9689,14 @@
       <c r="HR31" s="8"/>
     </row>
     <row r="32" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="68"/>
-      <c r="B32" s="68"/>
-      <c r="C32" s="68"/>
+      <c r="A32" s="75"/>
+      <c r="B32" s="75"/>
+      <c r="C32" s="75"/>
       <c r="D32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="68"/>
-      <c r="F32" s="68"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="8"/>
@@ -9761,10 +9735,9 @@
       <c r="AQ32" s="8"/>
       <c r="AR32" s="8"/>
       <c r="AS32" s="58"/>
-      <c r="AT32" s="84"/>
+      <c r="AT32" s="68"/>
       <c r="AU32" s="10"/>
-      <c r="AV32" s="11"/>
-      <c r="AX32" s="8"/>
+      <c r="AV32" s="47"/>
       <c r="AY32" s="8"/>
       <c r="AZ32" s="8"/>
       <c r="BA32" s="9"/>
@@ -9943,20 +9916,20 @@
       <c r="HR32" s="8"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="68"/>
-      <c r="B33" s="74" t="s">
+      <c r="A33" s="75"/>
+      <c r="B33" s="76" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="70" t="s">
+      <c r="C33" s="78" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="73" t="s">
+      <c r="E33" s="77" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="75" t="s">
+      <c r="F33" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -9997,10 +9970,9 @@
       <c r="AQ33" s="8"/>
       <c r="AR33" s="16"/>
       <c r="AS33" s="54"/>
-      <c r="AT33" s="84"/>
+      <c r="AT33" s="68"/>
       <c r="AU33" s="10"/>
-      <c r="AV33" s="11"/>
-      <c r="AX33" s="8"/>
+      <c r="AV33" s="47"/>
       <c r="AY33" s="16"/>
       <c r="AZ33" s="8"/>
       <c r="BA33" s="9"/>
@@ -10179,14 +10151,14 @@
       <c r="HR33" s="8"/>
     </row>
     <row r="34" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="68"/>
-      <c r="B34" s="68"/>
-      <c r="C34" s="68"/>
+      <c r="A34" s="75"/>
+      <c r="B34" s="75"/>
+      <c r="C34" s="75"/>
       <c r="D34" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
+      <c r="E34" s="75"/>
+      <c r="F34" s="75"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
@@ -10225,10 +10197,9 @@
       <c r="AQ34" s="8"/>
       <c r="AR34" s="8"/>
       <c r="AS34" s="58"/>
-      <c r="AT34" s="84"/>
+      <c r="AT34" s="68"/>
       <c r="AU34" s="10"/>
-      <c r="AV34" s="90"/>
-      <c r="AX34" s="8"/>
+      <c r="AV34" s="60"/>
       <c r="AY34" s="8"/>
       <c r="AZ34" s="8"/>
       <c r="BA34" s="9"/>
@@ -10407,20 +10378,20 @@
       <c r="HR34" s="8"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="68"/>
-      <c r="B35" s="74" t="s">
+      <c r="A35" s="75"/>
+      <c r="B35" s="76" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="70" t="s">
+      <c r="C35" s="78" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="73" t="s">
+      <c r="E35" s="77" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="75" t="s">
+      <c r="F35" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10461,10 +10432,9 @@
       <c r="AQ35" s="8"/>
       <c r="AR35" s="8"/>
       <c r="AS35" s="58"/>
-      <c r="AT35" s="84"/>
+      <c r="AT35" s="68"/>
       <c r="AU35" s="10"/>
-      <c r="AV35" s="11"/>
-      <c r="AX35" s="8"/>
+      <c r="AV35" s="47"/>
       <c r="AY35" s="8"/>
       <c r="AZ35" s="8"/>
       <c r="BA35" s="9"/>
@@ -10643,14 +10613,14 @@
       <c r="HR35" s="8"/>
     </row>
     <row r="36" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="68"/>
-      <c r="B36" s="68"/>
-      <c r="C36" s="68"/>
+      <c r="A36" s="75"/>
+      <c r="B36" s="75"/>
+      <c r="C36" s="75"/>
       <c r="D36" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="68"/>
-      <c r="F36" s="68"/>
+      <c r="E36" s="75"/>
+      <c r="F36" s="75"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
@@ -10689,10 +10659,9 @@
       <c r="AQ36" s="8"/>
       <c r="AR36" s="8"/>
       <c r="AS36" s="58"/>
-      <c r="AT36" s="84"/>
+      <c r="AT36" s="68"/>
       <c r="AU36" s="10"/>
-      <c r="AV36" s="11"/>
-      <c r="AX36" s="8"/>
+      <c r="AV36" s="47"/>
       <c r="AY36" s="8"/>
       <c r="AZ36" s="8"/>
       <c r="BA36" s="9"/>
@@ -10871,20 +10840,20 @@
       <c r="HR36" s="8"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="68"/>
-      <c r="B37" s="74" t="s">
+      <c r="A37" s="75"/>
+      <c r="B37" s="76" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="70" t="s">
+      <c r="C37" s="78" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="73" t="s">
+      <c r="E37" s="77" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="75" t="s">
+      <c r="F37" s="79" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -10925,10 +10894,9 @@
       <c r="AQ37" s="8"/>
       <c r="AR37" s="8"/>
       <c r="AS37" s="58"/>
-      <c r="AT37" s="84"/>
+      <c r="AT37" s="68"/>
       <c r="AU37" s="10"/>
-      <c r="AV37" s="11"/>
-      <c r="AX37" s="8"/>
+      <c r="AV37" s="47"/>
       <c r="AY37" s="8"/>
       <c r="AZ37" s="8"/>
       <c r="BA37" s="9"/>
@@ -11107,14 +11075,14 @@
       <c r="HR37" s="8"/>
     </row>
     <row r="38" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="68"/>
-      <c r="B38" s="68"/>
-      <c r="C38" s="68"/>
+      <c r="A38" s="75"/>
+      <c r="B38" s="75"/>
+      <c r="C38" s="75"/>
       <c r="D38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="68"/>
-      <c r="F38" s="68"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
@@ -11153,10 +11121,9 @@
       <c r="AQ38" s="8"/>
       <c r="AR38" s="8"/>
       <c r="AS38" s="58"/>
-      <c r="AT38" s="84"/>
+      <c r="AT38" s="68"/>
       <c r="AU38" s="10"/>
-      <c r="AV38" s="11"/>
-      <c r="AX38" s="8"/>
+      <c r="AV38" s="47"/>
       <c r="AY38" s="8"/>
       <c r="AZ38" s="8"/>
       <c r="BA38" s="9"/>
@@ -11335,20 +11302,20 @@
       <c r="HR38" s="8"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="68"/>
-      <c r="B39" s="74" t="s">
+      <c r="A39" s="75"/>
+      <c r="B39" s="76" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="70" t="s">
+      <c r="C39" s="78" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="73" t="s">
+      <c r="E39" s="77" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="75" t="s">
+      <c r="F39" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11389,10 +11356,9 @@
       <c r="AQ39" s="8"/>
       <c r="AR39" s="8"/>
       <c r="AS39" s="58"/>
-      <c r="AT39" s="84"/>
+      <c r="AT39" s="68"/>
       <c r="AU39" s="10"/>
-      <c r="AV39" s="11"/>
-      <c r="AX39" s="8"/>
+      <c r="AV39" s="47"/>
       <c r="AY39" s="8"/>
       <c r="AZ39" s="8"/>
       <c r="BA39" s="9"/>
@@ -11571,14 +11537,14 @@
       <c r="HR39" s="8"/>
     </row>
     <row r="40" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="68"/>
-      <c r="B40" s="68"/>
-      <c r="C40" s="68"/>
+      <c r="A40" s="75"/>
+      <c r="B40" s="75"/>
+      <c r="C40" s="75"/>
       <c r="D40" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="68"/>
-      <c r="F40" s="68"/>
+      <c r="E40" s="75"/>
+      <c r="F40" s="75"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
@@ -11617,10 +11583,9 @@
       <c r="AQ40" s="8"/>
       <c r="AR40" s="8"/>
       <c r="AS40" s="58"/>
-      <c r="AT40" s="84"/>
+      <c r="AT40" s="68"/>
       <c r="AU40" s="10"/>
-      <c r="AV40" s="11"/>
-      <c r="AX40" s="8"/>
+      <c r="AV40" s="47"/>
       <c r="AY40" s="8"/>
       <c r="AZ40" s="8"/>
       <c r="BA40" s="9"/>
@@ -11799,22 +11764,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="69" t="s">
+      <c r="A41" s="85" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="74" t="s">
+      <c r="B41" s="76" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="70" t="s">
+      <c r="C41" s="78" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="73" t="s">
+      <c r="E41" s="77" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="75" t="s">
+      <c r="F41" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -11855,10 +11820,9 @@
       <c r="AQ41" s="8"/>
       <c r="AR41" s="8"/>
       <c r="AS41" s="58"/>
-      <c r="AT41" s="84"/>
+      <c r="AT41" s="68"/>
       <c r="AU41" s="10"/>
-      <c r="AV41" s="11"/>
-      <c r="AX41" s="8"/>
+      <c r="AV41" s="47"/>
       <c r="AY41" s="8"/>
       <c r="AZ41" s="8"/>
       <c r="BA41" s="9"/>
@@ -12037,14 +12001,14 @@
       <c r="HR41" s="8"/>
     </row>
     <row r="42" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="68"/>
-      <c r="B42" s="68"/>
-      <c r="C42" s="68"/>
+      <c r="A42" s="75"/>
+      <c r="B42" s="75"/>
+      <c r="C42" s="75"/>
       <c r="D42" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="68"/>
-      <c r="F42" s="68"/>
+      <c r="E42" s="75"/>
+      <c r="F42" s="75"/>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="8"/>
@@ -12083,10 +12047,9 @@
       <c r="AQ42" s="8"/>
       <c r="AR42" s="8"/>
       <c r="AS42" s="58"/>
-      <c r="AT42" s="84"/>
+      <c r="AT42" s="68"/>
       <c r="AU42" s="10"/>
-      <c r="AV42" s="11"/>
-      <c r="AX42" s="8"/>
+      <c r="AV42" s="47"/>
       <c r="AY42" s="8"/>
       <c r="AZ42" s="8"/>
       <c r="BA42" s="9"/>
@@ -12265,20 +12228,20 @@
       <c r="HR42" s="8"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="68"/>
-      <c r="B43" s="74" t="s">
+      <c r="A43" s="75"/>
+      <c r="B43" s="76" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="70" t="s">
+      <c r="C43" s="78" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="73" t="s">
+      <c r="E43" s="77" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="75" t="s">
+      <c r="F43" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12318,10 +12281,9 @@
       <c r="AQ43" s="7"/>
       <c r="AR43" s="8"/>
       <c r="AS43" s="58"/>
-      <c r="AT43" s="84"/>
+      <c r="AT43" s="68"/>
       <c r="AU43" s="10"/>
-      <c r="AV43" s="11"/>
-      <c r="AX43" s="8"/>
+      <c r="AV43" s="47"/>
       <c r="AY43" s="8"/>
       <c r="AZ43" s="8"/>
       <c r="BA43" s="9"/>
@@ -12500,14 +12462,14 @@
       <c r="HR43" s="8"/>
     </row>
     <row r="44" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="68"/>
-      <c r="B44" s="68"/>
-      <c r="C44" s="68"/>
+      <c r="A44" s="75"/>
+      <c r="B44" s="75"/>
+      <c r="C44" s="75"/>
       <c r="D44" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="68"/>
-      <c r="F44" s="68"/>
+      <c r="E44" s="75"/>
+      <c r="F44" s="75"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="8"/>
@@ -12547,10 +12509,10 @@
       <c r="AQ44" s="8"/>
       <c r="AR44" s="44"/>
       <c r="AS44" s="61"/>
-      <c r="AT44" s="84"/>
+      <c r="AT44" s="68"/>
       <c r="AU44" s="10"/>
-      <c r="AV44" s="11"/>
-      <c r="AX44" s="8"/>
+      <c r="AV44" s="47"/>
+      <c r="AX44" s="73"/>
       <c r="AY44" s="8"/>
       <c r="AZ44" s="8"/>
       <c r="BA44" s="9"/>
@@ -12729,20 +12691,20 @@
       <c r="HR44" s="8"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="68"/>
-      <c r="B45" s="74" t="s">
+      <c r="A45" s="75"/>
+      <c r="B45" s="76" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="70" t="s">
+      <c r="C45" s="78" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="73" t="s">
+      <c r="E45" s="77" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="75" t="s">
+      <c r="F45" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12782,11 +12744,10 @@
       <c r="AO45" s="47"/>
       <c r="AR45" s="8"/>
       <c r="AS45" s="58"/>
-      <c r="AT45" s="84"/>
+      <c r="AT45" s="68"/>
       <c r="AU45" s="10"/>
-      <c r="AV45" s="11"/>
-      <c r="AW45" s="87"/>
-      <c r="AX45" s="8"/>
+      <c r="AV45" s="47"/>
+      <c r="AW45" s="52"/>
       <c r="AY45" s="8"/>
       <c r="AZ45" s="8"/>
       <c r="BA45" s="9"/>
@@ -12965,14 +12926,14 @@
       <c r="HR45" s="8"/>
     </row>
     <row r="46" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="68"/>
-      <c r="B46" s="68"/>
-      <c r="C46" s="68"/>
+      <c r="A46" s="75"/>
+      <c r="B46" s="75"/>
+      <c r="C46" s="75"/>
       <c r="D46" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="68"/>
-      <c r="F46" s="68"/>
+      <c r="E46" s="75"/>
+      <c r="F46" s="75"/>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="8"/>
@@ -13011,11 +12972,10 @@
       <c r="AQ46" s="8"/>
       <c r="AR46" s="8"/>
       <c r="AS46" s="58"/>
-      <c r="AT46" s="84"/>
+      <c r="AT46" s="68"/>
       <c r="AU46" s="10"/>
-      <c r="AV46" s="11"/>
-      <c r="AW46" s="88"/>
-      <c r="AX46" s="8"/>
+      <c r="AV46" s="47"/>
+      <c r="AW46" s="56"/>
       <c r="AY46" s="8"/>
       <c r="AZ46" s="8"/>
       <c r="BA46" s="9"/>
@@ -13194,22 +13154,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="69" t="s">
+      <c r="A47" s="85" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="74" t="s">
+      <c r="B47" s="76" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="70" t="s">
+      <c r="C47" s="78" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="73" t="s">
+      <c r="E47" s="77" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="75" t="s">
+      <c r="F47" s="79" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13250,10 +13210,10 @@
       <c r="AQ47" s="8"/>
       <c r="AR47" s="8"/>
       <c r="AS47" s="58"/>
-      <c r="AT47" s="84"/>
+      <c r="AT47" s="68"/>
       <c r="AU47" s="10"/>
-      <c r="AV47" s="11"/>
-      <c r="AX47" s="7"/>
+      <c r="AV47" s="47"/>
+      <c r="AX47" s="71"/>
       <c r="AY47" s="7"/>
       <c r="AZ47" s="7"/>
       <c r="BA47" s="9"/>
@@ -13432,14 +13392,14 @@
       <c r="HR47" s="8"/>
     </row>
     <row r="48" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="68"/>
-      <c r="B48" s="68"/>
-      <c r="C48" s="68"/>
+      <c r="A48" s="75"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
       <c r="D48" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="68"/>
-      <c r="F48" s="68"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
@@ -13478,10 +13438,9 @@
       <c r="AQ48" s="8"/>
       <c r="AR48" s="8"/>
       <c r="AS48" s="58"/>
-      <c r="AT48" s="84"/>
+      <c r="AT48" s="68"/>
       <c r="AU48" s="10"/>
-      <c r="AV48" s="11"/>
-      <c r="AX48" s="8"/>
+      <c r="AV48" s="47"/>
       <c r="AY48" s="8"/>
       <c r="AZ48" s="8"/>
       <c r="BA48" s="9"/>
@@ -13660,20 +13619,20 @@
       <c r="HR48" s="8"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="68"/>
-      <c r="B49" s="74" t="s">
+      <c r="A49" s="75"/>
+      <c r="B49" s="76" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="70" t="s">
+      <c r="C49" s="78" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="73" t="s">
+      <c r="E49" s="77" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="75" t="s">
+      <c r="F49" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13714,10 +13673,9 @@
       <c r="AQ49" s="8"/>
       <c r="AR49" s="8"/>
       <c r="AS49" s="58"/>
-      <c r="AT49" s="84"/>
+      <c r="AT49" s="68"/>
       <c r="AU49" s="10"/>
-      <c r="AV49" s="11"/>
-      <c r="AX49" s="8"/>
+      <c r="AV49" s="47"/>
       <c r="AY49" s="8"/>
       <c r="AZ49" s="8"/>
       <c r="BA49" s="9"/>
@@ -13896,14 +13854,14 @@
       <c r="HR49" s="8"/>
     </row>
     <row r="50" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="68"/>
-      <c r="B50" s="68"/>
-      <c r="C50" s="68"/>
+      <c r="A50" s="75"/>
+      <c r="B50" s="75"/>
+      <c r="C50" s="75"/>
       <c r="D50" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="68"/>
-      <c r="F50" s="68"/>
+      <c r="E50" s="75"/>
+      <c r="F50" s="75"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
@@ -13942,10 +13900,9 @@
       <c r="AQ50" s="8"/>
       <c r="AR50" s="8"/>
       <c r="AS50" s="58"/>
-      <c r="AT50" s="84"/>
+      <c r="AT50" s="68"/>
       <c r="AU50" s="10"/>
-      <c r="AV50" s="11"/>
-      <c r="AX50" s="8"/>
+      <c r="AV50" s="47"/>
       <c r="AY50" s="8"/>
       <c r="AZ50" s="8"/>
       <c r="BA50" s="9"/>
@@ -14124,22 +14081,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="69" t="s">
+      <c r="A51" s="85" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="74" t="s">
+      <c r="B51" s="76" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="70" t="s">
+      <c r="C51" s="78" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="73" t="s">
+      <c r="E51" s="77" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="75" t="s">
+      <c r="F51" s="79" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14180,10 +14137,9 @@
       <c r="AQ51" s="8"/>
       <c r="AR51" s="8"/>
       <c r="AS51" s="58"/>
-      <c r="AT51" s="84"/>
+      <c r="AT51" s="68"/>
       <c r="AU51" s="10"/>
-      <c r="AV51" s="11"/>
-      <c r="AX51" s="8"/>
+      <c r="AV51" s="47"/>
       <c r="AY51" s="8"/>
       <c r="AZ51" s="8"/>
       <c r="BA51" s="9"/>
@@ -14362,14 +14318,14 @@
       <c r="HR51" s="8"/>
     </row>
     <row r="52" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="68"/>
-      <c r="B52" s="68"/>
-      <c r="C52" s="68"/>
+      <c r="A52" s="75"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
       <c r="D52" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="68"/>
-      <c r="F52" s="68"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="8"/>
@@ -14408,10 +14364,9 @@
       <c r="AQ52" s="8"/>
       <c r="AR52" s="8"/>
       <c r="AS52" s="58"/>
-      <c r="AT52" s="84"/>
+      <c r="AT52" s="68"/>
       <c r="AU52" s="10"/>
-      <c r="AV52" s="11"/>
-      <c r="AX52" s="8"/>
+      <c r="AV52" s="47"/>
       <c r="AY52" s="8"/>
       <c r="AZ52" s="8"/>
       <c r="BA52" s="9"/>
@@ -14590,20 +14545,20 @@
       <c r="HR52" s="8"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="68"/>
-      <c r="B53" s="74" t="s">
+      <c r="A53" s="75"/>
+      <c r="B53" s="76" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="70" t="s">
+      <c r="C53" s="78" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="77" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="75" t="s">
+      <c r="F53" s="79" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14644,10 +14599,9 @@
       <c r="AQ53" s="8"/>
       <c r="AR53" s="8"/>
       <c r="AS53" s="58"/>
-      <c r="AT53" s="84"/>
+      <c r="AT53" s="68"/>
       <c r="AU53" s="10"/>
-      <c r="AV53" s="11"/>
-      <c r="AX53" s="8"/>
+      <c r="AV53" s="47"/>
       <c r="AY53" s="8"/>
       <c r="AZ53" s="8"/>
       <c r="BA53" s="9"/>
@@ -14826,14 +14780,14 @@
       <c r="HR53" s="8"/>
     </row>
     <row r="54" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="68"/>
-      <c r="B54" s="68"/>
-      <c r="C54" s="68"/>
+      <c r="A54" s="75"/>
+      <c r="B54" s="75"/>
+      <c r="C54" s="75"/>
       <c r="D54" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="68"/>
-      <c r="F54" s="68"/>
+      <c r="E54" s="75"/>
+      <c r="F54" s="75"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
@@ -14872,10 +14826,9 @@
       <c r="AQ54" s="8"/>
       <c r="AR54" s="8"/>
       <c r="AS54" s="58"/>
-      <c r="AT54" s="84"/>
+      <c r="AT54" s="68"/>
       <c r="AU54" s="10"/>
-      <c r="AV54" s="11"/>
-      <c r="AX54" s="8"/>
+      <c r="AV54" s="47"/>
       <c r="AY54" s="8"/>
       <c r="AZ54" s="8"/>
       <c r="BA54" s="9"/>
@@ -15054,22 +15007,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="69" t="s">
+      <c r="A55" s="85" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="74" t="s">
+      <c r="B55" s="76" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="70" t="s">
+      <c r="C55" s="78" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="73" t="s">
+      <c r="E55" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="75" t="s">
+      <c r="F55" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -15110,10 +15063,9 @@
       <c r="AQ55" s="8"/>
       <c r="AR55" s="8"/>
       <c r="AS55" s="58"/>
-      <c r="AT55" s="84"/>
+      <c r="AT55" s="68"/>
       <c r="AU55" s="10"/>
-      <c r="AV55" s="11"/>
-      <c r="AX55" s="8"/>
+      <c r="AV55" s="47"/>
       <c r="AY55" s="8"/>
       <c r="AZ55" s="8"/>
       <c r="BA55" s="9"/>
@@ -15292,14 +15244,14 @@
       <c r="HR55" s="8"/>
     </row>
     <row r="56" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="68"/>
-      <c r="B56" s="68"/>
-      <c r="C56" s="68"/>
+      <c r="A56" s="75"/>
+      <c r="B56" s="75"/>
+      <c r="C56" s="75"/>
       <c r="D56" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="68"/>
-      <c r="F56" s="68"/>
+      <c r="E56" s="75"/>
+      <c r="F56" s="75"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
@@ -15338,10 +15290,9 @@
       <c r="AQ56" s="8"/>
       <c r="AR56" s="8"/>
       <c r="AS56" s="58"/>
-      <c r="AT56" s="84"/>
+      <c r="AT56" s="68"/>
       <c r="AU56" s="10"/>
-      <c r="AV56" s="11"/>
-      <c r="AX56" s="8"/>
+      <c r="AV56" s="47"/>
       <c r="AY56" s="8"/>
       <c r="AZ56" s="8"/>
       <c r="BA56" s="9"/>
@@ -15520,20 +15471,20 @@
       <c r="HR56" s="8"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="68"/>
-      <c r="B57" s="74" t="s">
+      <c r="A57" s="75"/>
+      <c r="B57" s="76" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="70" t="s">
+      <c r="C57" s="78" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="73" t="s">
+      <c r="E57" s="77" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="75" t="s">
+      <c r="F57" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15574,10 +15525,9 @@
       <c r="AQ57" s="8"/>
       <c r="AR57" s="8"/>
       <c r="AS57" s="58"/>
-      <c r="AT57" s="84"/>
+      <c r="AT57" s="68"/>
       <c r="AU57" s="10"/>
-      <c r="AV57" s="11"/>
-      <c r="AX57" s="8"/>
+      <c r="AV57" s="47"/>
       <c r="AY57" s="8"/>
       <c r="AZ57" s="8"/>
       <c r="BA57" s="9"/>
@@ -15756,14 +15706,14 @@
       <c r="HR57" s="8"/>
     </row>
     <row r="58" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="68"/>
-      <c r="B58" s="68"/>
-      <c r="C58" s="68"/>
+      <c r="A58" s="75"/>
+      <c r="B58" s="75"/>
+      <c r="C58" s="75"/>
       <c r="D58" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="68"/>
-      <c r="F58" s="68"/>
+      <c r="E58" s="75"/>
+      <c r="F58" s="75"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
@@ -15802,10 +15752,9 @@
       <c r="AQ58" s="8"/>
       <c r="AR58" s="8"/>
       <c r="AS58" s="58"/>
-      <c r="AT58" s="84"/>
+      <c r="AT58" s="68"/>
       <c r="AU58" s="10"/>
-      <c r="AV58" s="11"/>
-      <c r="AX58" s="8"/>
+      <c r="AV58" s="47"/>
       <c r="AY58" s="8"/>
       <c r="AZ58" s="8"/>
       <c r="BA58" s="9"/>
@@ -15984,20 +15933,20 @@
       <c r="HR58" s="8"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="68"/>
-      <c r="B59" s="74" t="s">
+      <c r="A59" s="75"/>
+      <c r="B59" s="76" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="70" t="s">
+      <c r="C59" s="78" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="73" t="s">
+      <c r="E59" s="77" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="75" t="s">
+      <c r="F59" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -16038,10 +15987,9 @@
       <c r="AQ59" s="8"/>
       <c r="AR59" s="8"/>
       <c r="AS59" s="58"/>
-      <c r="AT59" s="84"/>
+      <c r="AT59" s="68"/>
       <c r="AU59" s="10"/>
-      <c r="AV59" s="11"/>
-      <c r="AX59" s="8"/>
+      <c r="AV59" s="47"/>
       <c r="AY59" s="8"/>
       <c r="AZ59" s="8"/>
       <c r="BA59" s="9"/>
@@ -16220,14 +16168,14 @@
       <c r="HR59" s="8"/>
     </row>
     <row r="60" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="68"/>
-      <c r="B60" s="68"/>
-      <c r="C60" s="68"/>
+      <c r="A60" s="75"/>
+      <c r="B60" s="75"/>
+      <c r="C60" s="75"/>
       <c r="D60" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="68"/>
-      <c r="F60" s="68"/>
+      <c r="E60" s="75"/>
+      <c r="F60" s="75"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
@@ -16266,10 +16214,9 @@
       <c r="AQ60" s="8"/>
       <c r="AR60" s="8"/>
       <c r="AS60" s="58"/>
-      <c r="AT60" s="84"/>
+      <c r="AT60" s="68"/>
       <c r="AU60" s="10"/>
-      <c r="AV60" s="11"/>
-      <c r="AX60" s="8"/>
+      <c r="AV60" s="47"/>
       <c r="AY60" s="8"/>
       <c r="AZ60" s="8"/>
       <c r="BA60" s="9"/>
@@ -16448,20 +16395,20 @@
       <c r="HR60" s="8"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="68"/>
-      <c r="B61" s="74" t="s">
+      <c r="A61" s="75"/>
+      <c r="B61" s="76" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="70" t="s">
+      <c r="C61" s="78" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="73" t="s">
+      <c r="E61" s="77" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="75" t="s">
+      <c r="F61" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16502,10 +16449,9 @@
       <c r="AQ61" s="8"/>
       <c r="AR61" s="8"/>
       <c r="AS61" s="58"/>
-      <c r="AT61" s="84"/>
+      <c r="AT61" s="68"/>
       <c r="AU61" s="10"/>
-      <c r="AV61" s="11"/>
-      <c r="AX61" s="8"/>
+      <c r="AV61" s="47"/>
       <c r="AY61" s="8"/>
       <c r="AZ61" s="8"/>
       <c r="BA61" s="9"/>
@@ -16684,14 +16630,14 @@
       <c r="HR61" s="8"/>
     </row>
     <row r="62" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="68"/>
-      <c r="B62" s="68"/>
-      <c r="C62" s="68"/>
+      <c r="A62" s="75"/>
+      <c r="B62" s="75"/>
+      <c r="C62" s="75"/>
       <c r="D62" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="68"/>
-      <c r="F62" s="68"/>
+      <c r="E62" s="75"/>
+      <c r="F62" s="75"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
       <c r="I62" s="8"/>
@@ -16730,10 +16676,9 @@
       <c r="AQ62" s="8"/>
       <c r="AR62" s="8"/>
       <c r="AS62" s="58"/>
-      <c r="AT62" s="84"/>
+      <c r="AT62" s="68"/>
       <c r="AU62" s="10"/>
-      <c r="AV62" s="11"/>
-      <c r="AX62" s="8"/>
+      <c r="AV62" s="47"/>
       <c r="AY62" s="8"/>
       <c r="AZ62" s="8"/>
       <c r="BA62" s="9"/>
@@ -16912,20 +16857,20 @@
       <c r="HR62" s="8"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="68"/>
-      <c r="B63" s="74" t="s">
+      <c r="A63" s="75"/>
+      <c r="B63" s="76" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="70" t="s">
+      <c r="C63" s="78" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="73" t="s">
+      <c r="E63" s="77" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="75" t="s">
+      <c r="F63" s="79" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -16966,10 +16911,9 @@
       <c r="AQ63" s="8"/>
       <c r="AR63" s="8"/>
       <c r="AS63" s="58"/>
-      <c r="AT63" s="84"/>
+      <c r="AT63" s="68"/>
       <c r="AU63" s="10"/>
-      <c r="AV63" s="11"/>
-      <c r="AX63" s="8"/>
+      <c r="AV63" s="47"/>
       <c r="AY63" s="8"/>
       <c r="AZ63" s="8"/>
       <c r="BA63" s="9"/>
@@ -17148,14 +17092,14 @@
       <c r="HR63" s="8"/>
     </row>
     <row r="64" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="68"/>
-      <c r="B64" s="68"/>
-      <c r="C64" s="68"/>
+      <c r="A64" s="75"/>
+      <c r="B64" s="75"/>
+      <c r="C64" s="75"/>
       <c r="D64" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="68"/>
-      <c r="F64" s="68"/>
+      <c r="E64" s="75"/>
+      <c r="F64" s="75"/>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
@@ -17194,10 +17138,9 @@
       <c r="AQ64" s="8"/>
       <c r="AR64" s="8"/>
       <c r="AS64" s="58"/>
-      <c r="AT64" s="84"/>
+      <c r="AT64" s="68"/>
       <c r="AU64" s="10"/>
-      <c r="AV64" s="11"/>
-      <c r="AX64" s="8"/>
+      <c r="AV64" s="47"/>
       <c r="AY64" s="8"/>
       <c r="AZ64" s="8"/>
       <c r="BA64" s="9"/>
@@ -17376,20 +17319,20 @@
       <c r="HR64" s="8"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="68"/>
-      <c r="B65" s="74" t="s">
+      <c r="A65" s="75"/>
+      <c r="B65" s="76" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="70" t="s">
+      <c r="C65" s="78" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="73" t="s">
+      <c r="E65" s="77" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="75" t="s">
+      <c r="F65" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17430,10 +17373,9 @@
       <c r="AQ65" s="8"/>
       <c r="AR65" s="8"/>
       <c r="AS65" s="58"/>
-      <c r="AT65" s="84"/>
+      <c r="AT65" s="68"/>
       <c r="AU65" s="10"/>
-      <c r="AV65" s="11"/>
-      <c r="AX65" s="8"/>
+      <c r="AV65" s="47"/>
       <c r="AY65" s="8"/>
       <c r="AZ65" s="8"/>
       <c r="BA65" s="9"/>
@@ -17612,14 +17554,14 @@
       <c r="HR65" s="8"/>
     </row>
     <row r="66" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="68"/>
-      <c r="B66" s="68"/>
-      <c r="C66" s="68"/>
+      <c r="A66" s="75"/>
+      <c r="B66" s="75"/>
+      <c r="C66" s="75"/>
       <c r="D66" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="68"/>
-      <c r="F66" s="68"/>
+      <c r="E66" s="75"/>
+      <c r="F66" s="75"/>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
@@ -17658,10 +17600,9 @@
       <c r="AQ66" s="8"/>
       <c r="AR66" s="8"/>
       <c r="AS66" s="58"/>
-      <c r="AT66" s="84"/>
+      <c r="AT66" s="68"/>
       <c r="AU66" s="10"/>
-      <c r="AV66" s="11"/>
-      <c r="AX66" s="8"/>
+      <c r="AV66" s="47"/>
       <c r="AY66" s="8"/>
       <c r="AZ66" s="8"/>
       <c r="BA66" s="9"/>
@@ -17840,22 +17781,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="69" t="s">
+      <c r="A67" s="85" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="74" t="s">
+      <c r="B67" s="76" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="70" t="s">
+      <c r="C67" s="78" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="73" t="s">
+      <c r="E67" s="77" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="75" t="s">
+      <c r="F67" s="79" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -17896,10 +17837,9 @@
       <c r="AQ67" s="8"/>
       <c r="AR67" s="7"/>
       <c r="AS67" s="58"/>
-      <c r="AT67" s="84"/>
+      <c r="AT67" s="68"/>
       <c r="AU67" s="10"/>
-      <c r="AV67" s="11"/>
-      <c r="AX67" s="8"/>
+      <c r="AV67" s="47"/>
       <c r="AY67" s="8"/>
       <c r="AZ67" s="8"/>
       <c r="BA67" s="9"/>
@@ -18078,14 +18018,14 @@
       <c r="HR67" s="8"/>
     </row>
     <row r="68" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="68"/>
-      <c r="B68" s="68"/>
-      <c r="C68" s="68"/>
+      <c r="A68" s="75"/>
+      <c r="B68" s="75"/>
+      <c r="C68" s="75"/>
       <c r="D68" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="68"/>
-      <c r="F68" s="68"/>
+      <c r="E68" s="75"/>
+      <c r="F68" s="75"/>
       <c r="G68" s="8"/>
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
@@ -18124,11 +18064,10 @@
       <c r="AQ68" s="8"/>
       <c r="AR68" s="8"/>
       <c r="AS68" s="58"/>
-      <c r="AT68" s="84"/>
+      <c r="AT68" s="68"/>
       <c r="AU68" s="10"/>
-      <c r="AV68" s="11"/>
-      <c r="AW68" s="89"/>
-      <c r="AX68" s="8"/>
+      <c r="AV68" s="47"/>
+      <c r="AW68" s="61"/>
       <c r="AY68" s="8"/>
       <c r="AZ68" s="8"/>
       <c r="BA68" s="9"/>
@@ -18307,20 +18246,20 @@
       <c r="HR68" s="8"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="68"/>
-      <c r="B69" s="74" t="s">
+      <c r="A69" s="75"/>
+      <c r="B69" s="76" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="70" t="s">
+      <c r="C69" s="78" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="73" t="s">
+      <c r="E69" s="77" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="75" t="s">
+      <c r="F69" s="79" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18362,11 +18301,11 @@
       <c r="AQ69" s="16"/>
       <c r="AR69" s="16"/>
       <c r="AS69" s="54"/>
-      <c r="AT69" s="84"/>
+      <c r="AT69" s="68"/>
       <c r="AU69" s="10"/>
-      <c r="AV69" s="11"/>
-      <c r="AW69" s="86"/>
-      <c r="AX69" s="16"/>
+      <c r="AV69" s="47"/>
+      <c r="AW69" s="54"/>
+      <c r="AX69" s="70"/>
       <c r="AY69" s="16"/>
       <c r="AZ69" s="16"/>
       <c r="BA69" s="9"/>
@@ -18545,14 +18484,14 @@
       <c r="HR69" s="8"/>
     </row>
     <row r="70" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="68"/>
-      <c r="B70" s="68"/>
-      <c r="C70" s="68"/>
+      <c r="A70" s="75"/>
+      <c r="B70" s="75"/>
+      <c r="C70" s="75"/>
       <c r="D70" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="68"/>
-      <c r="F70" s="68"/>
+      <c r="E70" s="75"/>
+      <c r="F70" s="75"/>
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
       <c r="I70" s="8"/>
@@ -18591,10 +18530,11 @@
       <c r="AQ70" s="8"/>
       <c r="AR70" s="8"/>
       <c r="AS70" s="58"/>
-      <c r="AT70" s="84"/>
+      <c r="AT70" s="68"/>
       <c r="AU70" s="10"/>
-      <c r="AV70" s="11"/>
-      <c r="AX70" s="8"/>
+      <c r="AV70" s="47"/>
+      <c r="AW70" s="56"/>
+      <c r="AX70" s="72"/>
       <c r="AY70" s="8"/>
       <c r="AZ70" s="8"/>
       <c r="BA70" s="9"/>
@@ -18773,20 +18713,20 @@
       <c r="HR70" s="8"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="68"/>
-      <c r="B71" s="74" t="s">
+      <c r="A71" s="75"/>
+      <c r="B71" s="76" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="70" t="s">
+      <c r="C71" s="78" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="73" t="s">
+      <c r="E71" s="77" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="75" t="s">
+      <c r="F71" s="79" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -18827,10 +18767,9 @@
       <c r="AQ71" s="8"/>
       <c r="AR71" s="8"/>
       <c r="AS71" s="58"/>
-      <c r="AT71" s="84"/>
+      <c r="AT71" s="68"/>
       <c r="AU71" s="10"/>
-      <c r="AV71" s="11"/>
-      <c r="AX71" s="8"/>
+      <c r="AV71" s="47"/>
       <c r="AY71" s="8"/>
       <c r="AZ71" s="8"/>
       <c r="BA71" s="9"/>
@@ -19009,14 +18948,14 @@
       <c r="HR71" s="8"/>
     </row>
     <row r="72" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="68"/>
-      <c r="B72" s="68"/>
-      <c r="C72" s="68"/>
+      <c r="A72" s="75"/>
+      <c r="B72" s="75"/>
+      <c r="C72" s="75"/>
       <c r="D72" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="68"/>
-      <c r="F72" s="68"/>
+      <c r="E72" s="75"/>
+      <c r="F72" s="75"/>
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
@@ -19055,10 +18994,9 @@
       <c r="AQ72" s="8"/>
       <c r="AR72" s="8"/>
       <c r="AS72" s="58"/>
-      <c r="AT72" s="84"/>
+      <c r="AT72" s="68"/>
       <c r="AU72" s="10"/>
-      <c r="AV72" s="11"/>
-      <c r="AX72" s="8"/>
+      <c r="AV72" s="47"/>
       <c r="AY72" s="8"/>
       <c r="AZ72" s="8"/>
       <c r="BA72" s="9"/>
@@ -19237,20 +19175,20 @@
       <c r="HR72" s="8"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="68"/>
-      <c r="B73" s="74" t="s">
+      <c r="A73" s="75"/>
+      <c r="B73" s="76" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="70" t="s">
+      <c r="C73" s="78" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="73" t="s">
+      <c r="E73" s="77" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="75" t="s">
+      <c r="F73" s="79" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19291,10 +19229,9 @@
       <c r="AQ73" s="8"/>
       <c r="AR73" s="8"/>
       <c r="AS73" s="58"/>
-      <c r="AT73" s="84"/>
+      <c r="AT73" s="68"/>
       <c r="AU73" s="10"/>
-      <c r="AV73" s="11"/>
-      <c r="AX73" s="8"/>
+      <c r="AV73" s="47"/>
       <c r="AY73" s="8"/>
       <c r="AZ73" s="8"/>
       <c r="BA73" s="9"/>
@@ -19473,14 +19410,14 @@
       <c r="HR73" s="8"/>
     </row>
     <row r="74" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="68"/>
-      <c r="B74" s="68"/>
-      <c r="C74" s="68"/>
+      <c r="A74" s="75"/>
+      <c r="B74" s="75"/>
+      <c r="C74" s="75"/>
       <c r="D74" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="68"/>
-      <c r="F74" s="68"/>
+      <c r="E74" s="75"/>
+      <c r="F74" s="75"/>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>
@@ -19519,10 +19456,9 @@
       <c r="AQ74" s="8"/>
       <c r="AR74" s="8"/>
       <c r="AS74" s="58"/>
-      <c r="AT74" s="84"/>
+      <c r="AT74" s="68"/>
       <c r="AU74" s="10"/>
-      <c r="AV74" s="11"/>
-      <c r="AX74" s="8"/>
+      <c r="AV74" s="47"/>
       <c r="AY74" s="8"/>
       <c r="AZ74" s="8"/>
       <c r="BA74" s="9"/>
@@ -19701,20 +19637,20 @@
       <c r="HR74" s="8"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="68"/>
-      <c r="B75" s="74" t="s">
+      <c r="A75" s="75"/>
+      <c r="B75" s="76" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="70" t="s">
+      <c r="C75" s="78" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="73" t="s">
+      <c r="E75" s="77" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="75" t="s">
+      <c r="F75" s="79" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19755,10 +19691,9 @@
       <c r="AQ75" s="8"/>
       <c r="AR75" s="8"/>
       <c r="AS75" s="58"/>
-      <c r="AT75" s="84"/>
+      <c r="AT75" s="68"/>
       <c r="AU75" s="10"/>
-      <c r="AV75" s="11"/>
-      <c r="AX75" s="8"/>
+      <c r="AV75" s="47"/>
       <c r="AY75" s="8"/>
       <c r="AZ75" s="8"/>
       <c r="BA75" s="9"/>
@@ -19937,14 +19872,14 @@
       <c r="HR75" s="8"/>
     </row>
     <row r="76" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="68"/>
-      <c r="B76" s="68"/>
-      <c r="C76" s="68"/>
+      <c r="A76" s="75"/>
+      <c r="B76" s="75"/>
+      <c r="C76" s="75"/>
       <c r="D76" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="68"/>
-      <c r="F76" s="68"/>
+      <c r="E76" s="75"/>
+      <c r="F76" s="75"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
       <c r="I76" s="8"/>
@@ -19983,10 +19918,9 @@
       <c r="AQ76" s="8"/>
       <c r="AR76" s="8"/>
       <c r="AS76" s="58"/>
-      <c r="AT76" s="84"/>
+      <c r="AT76" s="68"/>
       <c r="AU76" s="10"/>
-      <c r="AV76" s="11"/>
-      <c r="AX76" s="8"/>
+      <c r="AV76" s="47"/>
       <c r="AY76" s="8"/>
       <c r="AZ76" s="8"/>
       <c r="BA76" s="9"/>
@@ -20165,20 +20099,20 @@
       <c r="HR76" s="8"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="68"/>
-      <c r="B77" s="74" t="s">
+      <c r="A77" s="75"/>
+      <c r="B77" s="76" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="70" t="s">
+      <c r="C77" s="78" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="73" t="s">
+      <c r="E77" s="77" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="75" t="s">
+      <c r="F77" s="79" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20219,10 +20153,9 @@
       <c r="AQ77" s="8"/>
       <c r="AR77" s="8"/>
       <c r="AS77" s="58"/>
-      <c r="AT77" s="84"/>
+      <c r="AT77" s="68"/>
       <c r="AU77" s="10"/>
-      <c r="AV77" s="11"/>
-      <c r="AX77" s="8"/>
+      <c r="AV77" s="47"/>
       <c r="AY77" s="8"/>
       <c r="AZ77" s="8"/>
       <c r="BA77" s="9"/>
@@ -20401,14 +20334,14 @@
       <c r="HR77" s="8"/>
     </row>
     <row r="78" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="68"/>
-      <c r="B78" s="68"/>
-      <c r="C78" s="68"/>
+      <c r="A78" s="75"/>
+      <c r="B78" s="75"/>
+      <c r="C78" s="75"/>
       <c r="D78" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="68"/>
-      <c r="F78" s="68"/>
+      <c r="E78" s="75"/>
+      <c r="F78" s="75"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
       <c r="I78" s="8"/>
@@ -20447,10 +20380,9 @@
       <c r="AQ78" s="8"/>
       <c r="AR78" s="8"/>
       <c r="AS78" s="58"/>
-      <c r="AT78" s="84"/>
+      <c r="AT78" s="68"/>
       <c r="AU78" s="10"/>
-      <c r="AV78" s="11"/>
-      <c r="AX78" s="8"/>
+      <c r="AV78" s="47"/>
       <c r="AY78" s="8"/>
       <c r="AZ78" s="8"/>
       <c r="BA78" s="9"/>
@@ -20629,22 +20561,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="69" t="s">
+      <c r="A79" s="85" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="74" t="s">
+      <c r="B79" s="76" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="77" t="s">
+      <c r="C79" s="74" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="73" t="s">
+      <c r="E79" s="77" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="75" t="s">
+      <c r="F79" s="79" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20685,10 +20617,9 @@
       <c r="AQ79" s="8"/>
       <c r="AR79" s="8"/>
       <c r="AS79" s="58"/>
-      <c r="AT79" s="84"/>
+      <c r="AT79" s="68"/>
       <c r="AU79" s="10"/>
-      <c r="AV79" s="11"/>
-      <c r="AX79" s="8"/>
+      <c r="AV79" s="47"/>
       <c r="AY79" s="8"/>
       <c r="AZ79" s="8"/>
       <c r="BA79" s="9"/>
@@ -20867,14 +20798,14 @@
       <c r="HR79" s="8"/>
     </row>
     <row r="80" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="68"/>
-      <c r="B80" s="68"/>
-      <c r="C80" s="68"/>
+      <c r="A80" s="75"/>
+      <c r="B80" s="75"/>
+      <c r="C80" s="75"/>
       <c r="D80" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="68"/>
-      <c r="F80" s="68"/>
+      <c r="E80" s="75"/>
+      <c r="F80" s="75"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
       <c r="I80" s="8"/>
@@ -20913,10 +20844,9 @@
       <c r="AQ80" s="8"/>
       <c r="AR80" s="8"/>
       <c r="AS80" s="58"/>
-      <c r="AT80" s="84"/>
+      <c r="AT80" s="68"/>
       <c r="AU80" s="10"/>
-      <c r="AV80" s="11"/>
-      <c r="AX80" s="8"/>
+      <c r="AV80" s="47"/>
       <c r="AY80" s="8"/>
       <c r="AZ80" s="8"/>
       <c r="BA80" s="9"/>
@@ -21095,20 +21025,20 @@
       <c r="HR80" s="8"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="68"/>
-      <c r="B81" s="74" t="s">
+      <c r="A81" s="75"/>
+      <c r="B81" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="77" t="s">
+      <c r="C81" s="74" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="73" t="s">
+      <c r="E81" s="77" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="75" t="s">
+      <c r="F81" s="79" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -21149,10 +21079,9 @@
       <c r="AQ81" s="8"/>
       <c r="AR81" s="8"/>
       <c r="AS81" s="58"/>
-      <c r="AT81" s="84"/>
+      <c r="AT81" s="68"/>
       <c r="AU81" s="10"/>
-      <c r="AV81" s="11"/>
-      <c r="AX81" s="8"/>
+      <c r="AV81" s="47"/>
       <c r="AY81" s="8"/>
       <c r="AZ81" s="8"/>
       <c r="BA81" s="9"/>
@@ -21331,14 +21260,14 @@
       <c r="HR81" s="8"/>
     </row>
     <row r="82" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="68"/>
-      <c r="B82" s="68"/>
-      <c r="C82" s="68"/>
+      <c r="A82" s="75"/>
+      <c r="B82" s="75"/>
+      <c r="C82" s="75"/>
       <c r="D82" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="68"/>
-      <c r="F82" s="68"/>
+      <c r="E82" s="75"/>
+      <c r="F82" s="75"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
       <c r="I82" s="8"/>
@@ -21377,10 +21306,9 @@
       <c r="AQ82" s="8"/>
       <c r="AR82" s="8"/>
       <c r="AS82" s="58"/>
-      <c r="AT82" s="84"/>
+      <c r="AT82" s="68"/>
       <c r="AU82" s="10"/>
-      <c r="AV82" s="11"/>
-      <c r="AX82" s="8"/>
+      <c r="AV82" s="47"/>
       <c r="AY82" s="8"/>
       <c r="AZ82" s="8"/>
       <c r="BA82" s="9"/>
@@ -21559,20 +21487,20 @@
       <c r="HR82" s="8"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="68"/>
-      <c r="B83" s="74" t="s">
+      <c r="A83" s="75"/>
+      <c r="B83" s="76" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="70" t="s">
+      <c r="C83" s="78" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="73" t="s">
+      <c r="E83" s="77" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="75" t="s">
+      <c r="F83" s="79" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21613,10 +21541,9 @@
       <c r="AQ83" s="8"/>
       <c r="AR83" s="8"/>
       <c r="AS83" s="58"/>
-      <c r="AT83" s="84"/>
+      <c r="AT83" s="68"/>
       <c r="AU83" s="10"/>
-      <c r="AV83" s="11"/>
-      <c r="AX83" s="8"/>
+      <c r="AV83" s="47"/>
       <c r="AY83" s="8"/>
       <c r="AZ83" s="8"/>
       <c r="BA83" s="9"/>
@@ -21795,14 +21722,14 @@
       <c r="HR83" s="8"/>
     </row>
     <row r="84" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="68"/>
-      <c r="B84" s="68"/>
-      <c r="C84" s="68"/>
+      <c r="A84" s="75"/>
+      <c r="B84" s="75"/>
+      <c r="C84" s="75"/>
       <c r="D84" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="68"/>
-      <c r="F84" s="68"/>
+      <c r="E84" s="75"/>
+      <c r="F84" s="75"/>
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
@@ -21841,10 +21768,9 @@
       <c r="AQ84" s="8"/>
       <c r="AR84" s="8"/>
       <c r="AS84" s="58"/>
-      <c r="AT84" s="84"/>
+      <c r="AT84" s="68"/>
       <c r="AU84" s="10"/>
-      <c r="AV84" s="11"/>
-      <c r="AX84" s="8"/>
+      <c r="AV84" s="47"/>
       <c r="AY84" s="8"/>
       <c r="AZ84" s="8"/>
       <c r="BA84" s="9"/>
@@ -22023,20 +21949,20 @@
       <c r="HR84" s="8"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="68"/>
-      <c r="B85" s="74" t="s">
+      <c r="A85" s="75"/>
+      <c r="B85" s="76" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="81" t="s">
+      <c r="C85" s="87" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="73" t="s">
+      <c r="E85" s="77" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="75"/>
+      <c r="F85" s="79"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -22075,10 +22001,9 @@
       <c r="AQ85" s="8"/>
       <c r="AR85" s="8"/>
       <c r="AS85" s="58"/>
-      <c r="AT85" s="84"/>
+      <c r="AT85" s="68"/>
       <c r="AU85" s="10"/>
-      <c r="AV85" s="11"/>
-      <c r="AX85" s="8"/>
+      <c r="AV85" s="47"/>
       <c r="AY85" s="8"/>
       <c r="AZ85" s="8"/>
       <c r="BA85" s="9"/>
@@ -22257,14 +22182,14 @@
       <c r="HR85" s="17"/>
     </row>
     <row r="86" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="68"/>
-      <c r="B86" s="68"/>
-      <c r="C86" s="68"/>
+      <c r="A86" s="75"/>
+      <c r="B86" s="75"/>
+      <c r="C86" s="75"/>
       <c r="D86" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="68"/>
-      <c r="F86" s="68"/>
+      <c r="E86" s="75"/>
+      <c r="F86" s="75"/>
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
@@ -22303,10 +22228,9 @@
       <c r="AQ86" s="8"/>
       <c r="AR86" s="8"/>
       <c r="AS86" s="58"/>
-      <c r="AT86" s="84"/>
+      <c r="AT86" s="68"/>
       <c r="AU86" s="10"/>
-      <c r="AV86" s="11"/>
-      <c r="AX86" s="8"/>
+      <c r="AV86" s="47"/>
       <c r="AY86" s="8"/>
       <c r="AZ86" s="8"/>
       <c r="BA86" s="9"/>
@@ -22486,6 +22410,187 @@
     </row>
   </sheetData>
   <mergeCells count="205">
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
     <mergeCell ref="C79:C80"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="E79:E80"/>
@@ -22510,187 +22615,6 @@
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="AP1:AV1"/>
     <mergeCell ref="E59:E60"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
neuralop fno training mit darcy flow erfolgreich getestet
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{555DB17D-D7C6-4413-8180-244C296AC2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13367A7E-B423-40C5-A7D7-365D025C4719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1147,7 +1147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1261,52 +1261,54 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1624,15 +1626,17 @@
     <col min="46" max="46" width="2.140625" style="58" customWidth="1"/>
     <col min="47" max="48" width="2.140625" customWidth="1"/>
     <col min="49" max="49" width="2.140625" style="67" customWidth="1"/>
-    <col min="50" max="50" width="2.140625" style="66" customWidth="1"/>
-    <col min="51" max="226" width="2.140625" customWidth="1"/>
+    <col min="50" max="50" width="2.140625" style="73" customWidth="1"/>
+    <col min="51" max="51" width="2.140625" customWidth="1"/>
+    <col min="52" max="52" width="2.140625" style="66" customWidth="1"/>
+    <col min="53" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="80" t="s">
+      <c r="G1" s="74" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="75"/>
@@ -1641,7 +1645,7 @@
       <c r="K1" s="75"/>
       <c r="L1" s="75"/>
       <c r="M1" s="75"/>
-      <c r="N1" s="80" t="s">
+      <c r="N1" s="74" t="s">
         <v>2</v>
       </c>
       <c r="O1" s="75"/>
@@ -1650,7 +1654,7 @@
       <c r="R1" s="75"/>
       <c r="S1" s="75"/>
       <c r="T1" s="75"/>
-      <c r="U1" s="80" t="s">
+      <c r="U1" s="74" t="s">
         <v>3</v>
       </c>
       <c r="V1" s="75"/>
@@ -1659,7 +1663,7 @@
       <c r="Y1" s="75"/>
       <c r="Z1" s="75"/>
       <c r="AA1" s="75"/>
-      <c r="AB1" s="81" t="s">
+      <c r="AB1" s="90" t="s">
         <v>4</v>
       </c>
       <c r="AC1" s="75"/>
@@ -1668,7 +1672,7 @@
       <c r="AF1" s="75"/>
       <c r="AG1" s="75"/>
       <c r="AH1" s="75"/>
-      <c r="AI1" s="80" t="s">
+      <c r="AI1" s="74" t="s">
         <v>5</v>
       </c>
       <c r="AJ1" s="75"/>
@@ -1677,7 +1681,7 @@
       <c r="AM1" s="75"/>
       <c r="AN1" s="75"/>
       <c r="AO1" s="75"/>
-      <c r="AP1" s="80" t="s">
+      <c r="AP1" s="74" t="s">
         <v>6</v>
       </c>
       <c r="AQ1" s="75"/>
@@ -1686,7 +1690,7 @@
       <c r="AT1" s="75"/>
       <c r="AU1" s="75"/>
       <c r="AV1" s="75"/>
-      <c r="AW1" s="80" t="s">
+      <c r="AW1" s="74" t="s">
         <v>7</v>
       </c>
       <c r="AX1" s="75"/>
@@ -1695,7 +1699,7 @@
       <c r="BA1" s="75"/>
       <c r="BB1" s="75"/>
       <c r="BC1" s="75"/>
-      <c r="BD1" s="80" t="s">
+      <c r="BD1" s="74" t="s">
         <v>8</v>
       </c>
       <c r="BE1" s="75"/>
@@ -1704,7 +1708,7 @@
       <c r="BH1" s="75"/>
       <c r="BI1" s="75"/>
       <c r="BJ1" s="75"/>
-      <c r="BK1" s="80" t="s">
+      <c r="BK1" s="74" t="s">
         <v>9</v>
       </c>
       <c r="BL1" s="75"/>
@@ -1713,7 +1717,7 @@
       <c r="BO1" s="75"/>
       <c r="BP1" s="75"/>
       <c r="BQ1" s="75"/>
-      <c r="BR1" s="80" t="s">
+      <c r="BR1" s="74" t="s">
         <v>10</v>
       </c>
       <c r="BS1" s="75"/>
@@ -1722,7 +1726,7 @@
       <c r="BV1" s="75"/>
       <c r="BW1" s="75"/>
       <c r="BX1" s="75"/>
-      <c r="BY1" s="80" t="s">
+      <c r="BY1" s="74" t="s">
         <v>11</v>
       </c>
       <c r="BZ1" s="75"/>
@@ -1731,7 +1735,7 @@
       <c r="CC1" s="75"/>
       <c r="CD1" s="75"/>
       <c r="CE1" s="75"/>
-      <c r="CF1" s="80" t="s">
+      <c r="CF1" s="74" t="s">
         <v>12</v>
       </c>
       <c r="CG1" s="75"/>
@@ -1740,7 +1744,7 @@
       <c r="CJ1" s="75"/>
       <c r="CK1" s="75"/>
       <c r="CL1" s="75"/>
-      <c r="CM1" s="80" t="s">
+      <c r="CM1" s="74" t="s">
         <v>13</v>
       </c>
       <c r="CN1" s="75"/>
@@ -1749,7 +1753,7 @@
       <c r="CQ1" s="75"/>
       <c r="CR1" s="75"/>
       <c r="CS1" s="75"/>
-      <c r="CT1" s="80" t="s">
+      <c r="CT1" s="74" t="s">
         <v>14</v>
       </c>
       <c r="CU1" s="75"/>
@@ -1758,7 +1762,7 @@
       <c r="CX1" s="75"/>
       <c r="CY1" s="75"/>
       <c r="CZ1" s="75"/>
-      <c r="DA1" s="80" t="s">
+      <c r="DA1" s="74" t="s">
         <v>15</v>
       </c>
       <c r="DB1" s="75"/>
@@ -1767,7 +1771,7 @@
       <c r="DE1" s="75"/>
       <c r="DF1" s="75"/>
       <c r="DG1" s="75"/>
-      <c r="DH1" s="80" t="s">
+      <c r="DH1" s="74" t="s">
         <v>16</v>
       </c>
       <c r="DI1" s="75"/>
@@ -1776,7 +1780,7 @@
       <c r="DL1" s="75"/>
       <c r="DM1" s="75"/>
       <c r="DN1" s="75"/>
-      <c r="DO1" s="80" t="s">
+      <c r="DO1" s="74" t="s">
         <v>17</v>
       </c>
       <c r="DP1" s="75"/>
@@ -1785,7 +1789,7 @@
       <c r="DS1" s="75"/>
       <c r="DT1" s="75"/>
       <c r="DU1" s="75"/>
-      <c r="DV1" s="80" t="s">
+      <c r="DV1" s="74" t="s">
         <v>18</v>
       </c>
       <c r="DW1" s="75"/>
@@ -1794,7 +1798,7 @@
       <c r="DZ1" s="75"/>
       <c r="EA1" s="75"/>
       <c r="EB1" s="75"/>
-      <c r="EC1" s="80" t="s">
+      <c r="EC1" s="74" t="s">
         <v>19</v>
       </c>
       <c r="ED1" s="75"/>
@@ -1803,7 +1807,7 @@
       <c r="EG1" s="75"/>
       <c r="EH1" s="75"/>
       <c r="EI1" s="75"/>
-      <c r="EJ1" s="80" t="s">
+      <c r="EJ1" s="74" t="s">
         <v>20</v>
       </c>
       <c r="EK1" s="75"/>
@@ -1812,7 +1816,7 @@
       <c r="EN1" s="75"/>
       <c r="EO1" s="75"/>
       <c r="EP1" s="75"/>
-      <c r="EQ1" s="80" t="s">
+      <c r="EQ1" s="74" t="s">
         <v>21</v>
       </c>
       <c r="ER1" s="75"/>
@@ -1821,7 +1825,7 @@
       <c r="EU1" s="75"/>
       <c r="EV1" s="75"/>
       <c r="EW1" s="75"/>
-      <c r="EX1" s="80" t="s">
+      <c r="EX1" s="74" t="s">
         <v>22</v>
       </c>
       <c r="EY1" s="75"/>
@@ -1830,7 +1834,7 @@
       <c r="FB1" s="75"/>
       <c r="FC1" s="75"/>
       <c r="FD1" s="75"/>
-      <c r="FE1" s="80" t="s">
+      <c r="FE1" s="74" t="s">
         <v>23</v>
       </c>
       <c r="FF1" s="75"/>
@@ -1839,7 +1843,7 @@
       <c r="FI1" s="75"/>
       <c r="FJ1" s="75"/>
       <c r="FK1" s="75"/>
-      <c r="FL1" s="80" t="s">
+      <c r="FL1" s="74" t="s">
         <v>24</v>
       </c>
       <c r="FM1" s="75"/>
@@ -1848,7 +1852,7 @@
       <c r="FP1" s="75"/>
       <c r="FQ1" s="75"/>
       <c r="FR1" s="75"/>
-      <c r="FS1" s="80" t="s">
+      <c r="FS1" s="74" t="s">
         <v>25</v>
       </c>
       <c r="FT1" s="75"/>
@@ -1857,7 +1861,7 @@
       <c r="FW1" s="75"/>
       <c r="FX1" s="75"/>
       <c r="FY1" s="75"/>
-      <c r="FZ1" s="80" t="s">
+      <c r="FZ1" s="74" t="s">
         <v>26</v>
       </c>
       <c r="GA1" s="75"/>
@@ -1866,7 +1870,7 @@
       <c r="GD1" s="75"/>
       <c r="GE1" s="75"/>
       <c r="GF1" s="75"/>
-      <c r="GG1" s="80" t="s">
+      <c r="GG1" s="74" t="s">
         <v>27</v>
       </c>
       <c r="GH1" s="75"/>
@@ -1875,7 +1879,7 @@
       <c r="GK1" s="75"/>
       <c r="GL1" s="75"/>
       <c r="GM1" s="75"/>
-      <c r="GN1" s="80" t="s">
+      <c r="GN1" s="74" t="s">
         <v>28</v>
       </c>
       <c r="GO1" s="75"/>
@@ -1884,7 +1888,7 @@
       <c r="GR1" s="75"/>
       <c r="GS1" s="75"/>
       <c r="GT1" s="75"/>
-      <c r="GU1" s="80" t="s">
+      <c r="GU1" s="74" t="s">
         <v>29</v>
       </c>
       <c r="GV1" s="75"/>
@@ -1893,7 +1897,7 @@
       <c r="GY1" s="75"/>
       <c r="GZ1" s="75"/>
       <c r="HA1" s="75"/>
-      <c r="HB1" s="80" t="s">
+      <c r="HB1" s="74" t="s">
         <v>30</v>
       </c>
       <c r="HC1" s="75"/>
@@ -1902,7 +1906,7 @@
       <c r="HF1" s="75"/>
       <c r="HG1" s="75"/>
       <c r="HH1" s="75"/>
-      <c r="HI1" s="80" t="s">
+      <c r="HI1" s="74" t="s">
         <v>31</v>
       </c>
       <c r="HJ1" s="75"/>
@@ -1911,7 +1915,7 @@
       <c r="HM1" s="75"/>
       <c r="HN1" s="75"/>
       <c r="HO1" s="75"/>
-      <c r="HP1" s="80" t="s">
+      <c r="HP1" s="74" t="s">
         <v>32</v>
       </c>
       <c r="HQ1" s="75"/>
@@ -2050,13 +2054,13 @@
       <c r="AW2" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="AX2" s="63" t="s">
+      <c r="AX2" s="62" t="s">
         <v>35</v>
       </c>
       <c r="AY2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AZ2" s="2" t="s">
+      <c r="AZ2" s="63" t="s">
         <v>35</v>
       </c>
       <c r="BA2" s="2" t="s">
@@ -2715,13 +2719,13 @@
       <c r="AW3" s="50">
         <v>46293</v>
       </c>
-      <c r="AX3" s="64">
+      <c r="AX3" s="50">
         <v>46294</v>
       </c>
       <c r="AY3" s="3">
         <v>46295</v>
       </c>
-      <c r="AZ3" s="3">
+      <c r="AZ3" s="64">
         <v>46296</v>
       </c>
       <c r="BA3" s="3">
@@ -3307,9 +3311,9 @@
       <c r="AU4" s="5"/>
       <c r="AV4" s="5"/>
       <c r="AW4" s="51"/>
-      <c r="AX4" s="65"/>
+      <c r="AX4" s="51"/>
       <c r="AY4" s="5"/>
-      <c r="AZ4" s="5"/>
+      <c r="AZ4" s="65"/>
       <c r="BA4" s="5"/>
       <c r="BB4" s="5"/>
       <c r="BC4" s="5"/>
@@ -3486,20 +3490,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="86"/>
-      <c r="C5" s="84" t="s">
+      <c r="B5" s="85"/>
+      <c r="C5" s="78" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="88" t="s">
+      <c r="E5" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="82"/>
+      <c r="F5" s="87"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3542,7 +3546,6 @@
       <c r="AU5" s="10"/>
       <c r="AV5" s="47"/>
       <c r="AY5" s="8"/>
-      <c r="AZ5" s="8"/>
       <c r="BA5" s="9"/>
       <c r="BB5" s="10"/>
       <c r="BC5" s="11"/>
@@ -3719,14 +3722,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83"/>
-      <c r="B6" s="83"/>
-      <c r="C6" s="83"/>
+      <c r="A6" s="79"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3769,7 +3772,6 @@
       <c r="AU6" s="10"/>
       <c r="AV6" s="47"/>
       <c r="AY6" s="8"/>
-      <c r="AZ6" s="8"/>
       <c r="BA6" s="9"/>
       <c r="BB6" s="10"/>
       <c r="BC6" s="11"/>
@@ -3946,18 +3948,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="83"/>
-      <c r="B7" s="86"/>
-      <c r="C7" s="84" t="s">
+      <c r="A7" s="79"/>
+      <c r="B7" s="85"/>
+      <c r="C7" s="78" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="88" t="s">
+      <c r="E7" s="83" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="82"/>
+      <c r="F7" s="87"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -4000,7 +4002,6 @@
       <c r="AU7" s="10"/>
       <c r="AV7" s="47"/>
       <c r="AY7" s="8"/>
-      <c r="AZ7" s="8"/>
       <c r="BA7" s="9"/>
       <c r="BB7" s="10"/>
       <c r="BC7" s="11"/>
@@ -4177,14 +4178,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="83"/>
-      <c r="B8" s="83"/>
-      <c r="C8" s="83"/>
+      <c r="A8" s="79"/>
+      <c r="B8" s="79"/>
+      <c r="C8" s="79"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="83"/>
-      <c r="F8" s="83"/>
+      <c r="E8" s="79"/>
+      <c r="F8" s="79"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4227,7 +4228,6 @@
       <c r="AU8" s="10"/>
       <c r="AV8" s="47"/>
       <c r="AY8" s="8"/>
-      <c r="AZ8" s="8"/>
       <c r="BA8" s="9"/>
       <c r="BB8" s="10"/>
       <c r="BC8" s="11"/>
@@ -4404,18 +4404,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="83"/>
-      <c r="B9" s="86"/>
-      <c r="C9" s="84" t="s">
+      <c r="A9" s="79"/>
+      <c r="B9" s="85"/>
+      <c r="C9" s="78" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="88" t="s">
+      <c r="E9" s="83" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="82"/>
+      <c r="F9" s="87"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4458,7 +4458,6 @@
       <c r="AU9" s="10"/>
       <c r="AV9" s="47"/>
       <c r="AY9" s="8"/>
-      <c r="AZ9" s="8"/>
       <c r="BA9" s="9"/>
       <c r="BB9" s="10"/>
       <c r="BC9" s="11"/>
@@ -4635,14 +4634,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="83"/>
-      <c r="B10" s="83"/>
-      <c r="C10" s="83"/>
+      <c r="A10" s="79"/>
+      <c r="B10" s="79"/>
+      <c r="C10" s="79"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="83"/>
-      <c r="F10" s="83"/>
+      <c r="E10" s="79"/>
+      <c r="F10" s="79"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4685,7 +4684,6 @@
       <c r="AU10" s="10"/>
       <c r="AV10" s="47"/>
       <c r="AY10" s="8"/>
-      <c r="AZ10" s="8"/>
       <c r="BA10" s="9"/>
       <c r="BB10" s="10"/>
       <c r="BC10" s="11"/>
@@ -4862,18 +4860,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="83"/>
-      <c r="B11" s="86"/>
-      <c r="C11" s="84" t="s">
+      <c r="A11" s="79"/>
+      <c r="B11" s="85"/>
+      <c r="C11" s="78" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="88" t="s">
+      <c r="E11" s="83" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="82"/>
+      <c r="F11" s="87"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -4916,7 +4914,6 @@
       <c r="AU11" s="10"/>
       <c r="AV11" s="47"/>
       <c r="AY11" s="8"/>
-      <c r="AZ11" s="8"/>
       <c r="BA11" s="9"/>
       <c r="BB11" s="10"/>
       <c r="BC11" s="11"/>
@@ -5093,14 +5090,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="83"/>
-      <c r="B12" s="83"/>
-      <c r="C12" s="83"/>
+      <c r="A12" s="79"/>
+      <c r="B12" s="79"/>
+      <c r="C12" s="79"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="83"/>
-      <c r="F12" s="83"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="79"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5143,7 +5140,6 @@
       <c r="AU12" s="10"/>
       <c r="AV12" s="47"/>
       <c r="AY12" s="8"/>
-      <c r="AZ12" s="8"/>
       <c r="BA12" s="9"/>
       <c r="BB12" s="10"/>
       <c r="BC12" s="11"/>
@@ -5320,18 +5316,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="83"/>
-      <c r="B13" s="86"/>
-      <c r="C13" s="84" t="s">
+      <c r="A13" s="79"/>
+      <c r="B13" s="85"/>
+      <c r="C13" s="78" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="88" t="s">
+      <c r="E13" s="83" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="82"/>
+      <c r="F13" s="87"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5374,7 +5370,6 @@
       <c r="AU13" s="10"/>
       <c r="AV13" s="47"/>
       <c r="AY13" s="8"/>
-      <c r="AZ13" s="8"/>
       <c r="BA13" s="9"/>
       <c r="BB13" s="10"/>
       <c r="BC13" s="11"/>
@@ -5551,14 +5546,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="83"/>
-      <c r="B14" s="83"/>
-      <c r="C14" s="83"/>
+      <c r="A14" s="79"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="79"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="83"/>
-      <c r="F14" s="83"/>
+      <c r="E14" s="79"/>
+      <c r="F14" s="79"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5601,7 +5596,6 @@
       <c r="AU14" s="10"/>
       <c r="AV14" s="47"/>
       <c r="AY14" s="8"/>
-      <c r="AZ14" s="8"/>
       <c r="BA14" s="9"/>
       <c r="BB14" s="10"/>
       <c r="BC14" s="11"/>
@@ -5778,18 +5772,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="83"/>
-      <c r="B15" s="86"/>
-      <c r="C15" s="84" t="s">
+      <c r="A15" s="79"/>
+      <c r="B15" s="85"/>
+      <c r="C15" s="78" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="88" t="s">
+      <c r="E15" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="82"/>
+      <c r="F15" s="87"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -5832,7 +5826,6 @@
       <c r="AU15" s="10"/>
       <c r="AV15" s="47"/>
       <c r="AY15" s="8"/>
-      <c r="AZ15" s="8"/>
       <c r="BA15" s="9"/>
       <c r="BB15" s="10"/>
       <c r="BC15" s="11"/>
@@ -6009,14 +6002,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="83"/>
-      <c r="B16" s="83"/>
-      <c r="C16" s="83"/>
+      <c r="A16" s="79"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="79"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="83"/>
-      <c r="F16" s="83"/>
+      <c r="E16" s="79"/>
+      <c r="F16" s="79"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6059,7 +6052,6 @@
       <c r="AU16" s="10"/>
       <c r="AV16" s="47"/>
       <c r="AY16" s="8"/>
-      <c r="AZ16" s="8"/>
       <c r="BA16" s="9"/>
       <c r="BB16" s="10"/>
       <c r="BC16" s="11"/>
@@ -6236,18 +6228,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="83"/>
-      <c r="B17" s="86"/>
-      <c r="C17" s="84" t="s">
+      <c r="A17" s="79"/>
+      <c r="B17" s="85"/>
+      <c r="C17" s="78" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="88" t="s">
+      <c r="E17" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="82"/>
+      <c r="F17" s="87"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6290,7 +6282,6 @@
       <c r="AU17" s="10"/>
       <c r="AV17" s="47"/>
       <c r="AY17" s="8"/>
-      <c r="AZ17" s="8"/>
       <c r="BA17" s="9"/>
       <c r="BB17" s="10"/>
       <c r="BC17" s="11"/>
@@ -6467,14 +6458,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="83"/>
-      <c r="B18" s="83"/>
-      <c r="C18" s="83"/>
+      <c r="A18" s="79"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="83"/>
-      <c r="F18" s="83"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="79"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6517,7 +6508,6 @@
       <c r="AU18" s="10"/>
       <c r="AV18" s="47"/>
       <c r="AY18" s="8"/>
-      <c r="AZ18" s="8"/>
       <c r="BA18" s="9"/>
       <c r="BB18" s="10"/>
       <c r="BC18" s="11"/>
@@ -6694,18 +6684,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="83"/>
-      <c r="B19" s="86"/>
-      <c r="C19" s="84" t="s">
+      <c r="A19" s="79"/>
+      <c r="B19" s="85"/>
+      <c r="C19" s="78" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="88" t="s">
+      <c r="E19" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="82"/>
+      <c r="F19" s="87"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6748,7 +6738,6 @@
       <c r="AU19" s="10"/>
       <c r="AV19" s="47"/>
       <c r="AY19" s="8"/>
-      <c r="AZ19" s="8"/>
       <c r="BA19" s="9"/>
       <c r="BB19" s="10"/>
       <c r="BC19" s="11"/>
@@ -6925,14 +6914,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="83"/>
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
+      <c r="A20" s="79"/>
+      <c r="B20" s="79"/>
+      <c r="C20" s="79"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="83"/>
-      <c r="F20" s="83"/>
+      <c r="E20" s="79"/>
+      <c r="F20" s="79"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -6975,7 +6964,6 @@
       <c r="AU20" s="10"/>
       <c r="AV20" s="47"/>
       <c r="AY20" s="8"/>
-      <c r="AZ20" s="8"/>
       <c r="BA20" s="9"/>
       <c r="BB20" s="10"/>
       <c r="BC20" s="11"/>
@@ -7152,18 +7140,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="83"/>
-      <c r="B21" s="86"/>
-      <c r="C21" s="84" t="s">
+      <c r="A21" s="79"/>
+      <c r="B21" s="85"/>
+      <c r="C21" s="78" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="88" t="s">
+      <c r="E21" s="83" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="82"/>
+      <c r="F21" s="87"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7206,7 +7194,6 @@
       <c r="AU21" s="10"/>
       <c r="AV21" s="47"/>
       <c r="AY21" s="8"/>
-      <c r="AZ21" s="8"/>
       <c r="BA21" s="9"/>
       <c r="BB21" s="10"/>
       <c r="BC21" s="11"/>
@@ -7383,14 +7370,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="89"/>
-      <c r="B22" s="89"/>
-      <c r="C22" s="89"/>
+      <c r="A22" s="86"/>
+      <c r="B22" s="86"/>
+      <c r="C22" s="86"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="89"/>
-      <c r="F22" s="89"/>
+      <c r="E22" s="86"/>
+      <c r="F22" s="86"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7432,9 +7419,8 @@
       <c r="AT22" s="68"/>
       <c r="AU22" s="40"/>
       <c r="AV22" s="48"/>
-      <c r="AX22" s="69"/>
       <c r="AY22" s="38"/>
-      <c r="AZ22" s="38"/>
+      <c r="AZ22" s="69"/>
       <c r="BA22" s="39"/>
       <c r="BB22" s="40"/>
       <c r="BC22" s="41"/>
@@ -7611,22 +7597,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="85" t="s">
+      <c r="A23" s="76" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="76" t="s">
+      <c r="B23" s="81" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="78" t="s">
+      <c r="C23" s="77" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="77" t="s">
+      <c r="E23" s="80" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="79" t="s">
+      <c r="F23" s="82" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7673,7 +7659,6 @@
       <c r="AV23" s="47"/>
       <c r="AW23" s="54"/>
       <c r="AY23" s="8"/>
-      <c r="AZ23" s="8"/>
       <c r="BA23" s="9"/>
       <c r="BB23" s="10"/>
       <c r="BC23" s="11"/>
@@ -7902,7 +7887,6 @@
       <c r="AV24" s="47"/>
       <c r="AW24" s="56"/>
       <c r="AY24" s="8"/>
-      <c r="AZ24" s="8"/>
       <c r="BA24" s="9"/>
       <c r="BB24" s="10"/>
       <c r="BC24" s="11"/>
@@ -8080,19 +8064,19 @@
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="75"/>
-      <c r="B25" s="76" t="s">
+      <c r="B25" s="81" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="78" t="s">
+      <c r="C25" s="77" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="77" t="s">
+      <c r="E25" s="80" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="79" t="s">
+      <c r="F25" s="82" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8356,7 +8340,6 @@
       <c r="AU26" s="10"/>
       <c r="AV26" s="47"/>
       <c r="AY26" s="8"/>
-      <c r="AZ26" s="8"/>
       <c r="BA26" s="9"/>
       <c r="BB26" s="10"/>
       <c r="BC26" s="11"/>
@@ -8534,19 +8517,19 @@
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="75"/>
-      <c r="B27" s="76" t="s">
+      <c r="B27" s="81" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="87" t="s">
+      <c r="C27" s="88" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="77" t="s">
+      <c r="E27" s="80" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="79"/>
+      <c r="F27" s="82"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8588,7 +8571,7 @@
       <c r="AU27" s="10"/>
       <c r="AV27" s="47"/>
       <c r="AY27" s="8"/>
-      <c r="AZ27" s="17"/>
+      <c r="AZ27" s="91"/>
       <c r="BA27" s="9"/>
       <c r="BB27" s="10"/>
       <c r="BC27" s="11"/>
@@ -8814,7 +8797,7 @@
       <c r="AU28" s="10"/>
       <c r="AV28" s="47"/>
       <c r="AY28" s="8"/>
-      <c r="AZ28" s="43"/>
+      <c r="AZ28" s="72"/>
       <c r="BA28" s="9"/>
       <c r="BB28" s="10"/>
       <c r="BC28" s="11"/>
@@ -8991,22 +8974,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="85" t="s">
+      <c r="A29" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="76" t="s">
+      <c r="B29" s="81" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="78" t="s">
+      <c r="C29" s="77" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="77" t="s">
+      <c r="E29" s="80" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="79" t="s">
+      <c r="F29" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9050,7 +9033,6 @@
       <c r="AU29" s="10"/>
       <c r="AV29" s="47"/>
       <c r="AY29" s="8"/>
-      <c r="AZ29" s="8"/>
       <c r="BA29" s="9"/>
       <c r="BB29" s="10"/>
       <c r="BC29" s="11"/>
@@ -9277,7 +9259,6 @@
       <c r="AU30" s="10"/>
       <c r="AV30" s="47"/>
       <c r="AY30" s="8"/>
-      <c r="AZ30" s="8"/>
       <c r="BA30" s="9"/>
       <c r="BB30" s="10"/>
       <c r="BC30" s="11"/>
@@ -9455,19 +9436,19 @@
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="75"/>
-      <c r="B31" s="76" t="s">
+      <c r="B31" s="81" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="78" t="s">
+      <c r="C31" s="77" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="77" t="s">
+      <c r="E31" s="80" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="79" t="s">
+      <c r="F31" s="82" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9512,7 +9493,6 @@
       <c r="AU31" s="10"/>
       <c r="AV31" s="47"/>
       <c r="AY31" s="8"/>
-      <c r="AZ31" s="8"/>
       <c r="BA31" s="9"/>
       <c r="BB31" s="10"/>
       <c r="BC31" s="11"/>
@@ -9739,7 +9719,6 @@
       <c r="AU32" s="10"/>
       <c r="AV32" s="47"/>
       <c r="AY32" s="8"/>
-      <c r="AZ32" s="8"/>
       <c r="BA32" s="9"/>
       <c r="BB32" s="10"/>
       <c r="BC32" s="11"/>
@@ -9917,19 +9896,19 @@
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="75"/>
-      <c r="B33" s="76" t="s">
+      <c r="B33" s="81" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="78" t="s">
+      <c r="C33" s="77" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="77" t="s">
+      <c r="E33" s="80" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="79" t="s">
+      <c r="F33" s="82" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -9974,7 +9953,6 @@
       <c r="AU33" s="10"/>
       <c r="AV33" s="47"/>
       <c r="AY33" s="16"/>
-      <c r="AZ33" s="8"/>
       <c r="BA33" s="9"/>
       <c r="BB33" s="10"/>
       <c r="BC33" s="11"/>
@@ -10201,7 +10179,6 @@
       <c r="AU34" s="10"/>
       <c r="AV34" s="60"/>
       <c r="AY34" s="8"/>
-      <c r="AZ34" s="8"/>
       <c r="BA34" s="9"/>
       <c r="BB34" s="10"/>
       <c r="BC34" s="11"/>
@@ -10379,19 +10356,19 @@
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="75"/>
-      <c r="B35" s="76" t="s">
+      <c r="B35" s="81" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="78" t="s">
+      <c r="C35" s="77" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="77" t="s">
+      <c r="E35" s="80" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="79" t="s">
+      <c r="F35" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10436,7 +10413,6 @@
       <c r="AU35" s="10"/>
       <c r="AV35" s="47"/>
       <c r="AY35" s="8"/>
-      <c r="AZ35" s="8"/>
       <c r="BA35" s="9"/>
       <c r="BB35" s="10"/>
       <c r="BC35" s="11"/>
@@ -10663,7 +10639,6 @@
       <c r="AU36" s="10"/>
       <c r="AV36" s="47"/>
       <c r="AY36" s="8"/>
-      <c r="AZ36" s="8"/>
       <c r="BA36" s="9"/>
       <c r="BB36" s="10"/>
       <c r="BC36" s="11"/>
@@ -10841,19 +10816,19 @@
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="75"/>
-      <c r="B37" s="76" t="s">
+      <c r="B37" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="78" t="s">
+      <c r="C37" s="77" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="77" t="s">
+      <c r="E37" s="80" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="79" t="s">
+      <c r="F37" s="82" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -10898,7 +10873,6 @@
       <c r="AU37" s="10"/>
       <c r="AV37" s="47"/>
       <c r="AY37" s="8"/>
-      <c r="AZ37" s="8"/>
       <c r="BA37" s="9"/>
       <c r="BB37" s="10"/>
       <c r="BC37" s="11"/>
@@ -11125,7 +11099,6 @@
       <c r="AU38" s="10"/>
       <c r="AV38" s="47"/>
       <c r="AY38" s="8"/>
-      <c r="AZ38" s="8"/>
       <c r="BA38" s="9"/>
       <c r="BB38" s="10"/>
       <c r="BC38" s="11"/>
@@ -11303,19 +11276,19 @@
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="75"/>
-      <c r="B39" s="76" t="s">
+      <c r="B39" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="78" t="s">
+      <c r="C39" s="77" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="77" t="s">
+      <c r="E39" s="80" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="79" t="s">
+      <c r="F39" s="82" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11360,7 +11333,6 @@
       <c r="AU39" s="10"/>
       <c r="AV39" s="47"/>
       <c r="AY39" s="8"/>
-      <c r="AZ39" s="8"/>
       <c r="BA39" s="9"/>
       <c r="BB39" s="10"/>
       <c r="BC39" s="11"/>
@@ -11587,7 +11559,7 @@
       <c r="AU40" s="10"/>
       <c r="AV40" s="47"/>
       <c r="AY40" s="8"/>
-      <c r="AZ40" s="8"/>
+      <c r="AZ40" s="92"/>
       <c r="BA40" s="9"/>
       <c r="BB40" s="10"/>
       <c r="BC40" s="11"/>
@@ -11764,22 +11736,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="85" t="s">
+      <c r="A41" s="76" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="76" t="s">
+      <c r="B41" s="81" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="78" t="s">
+      <c r="C41" s="77" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="77" t="s">
+      <c r="E41" s="80" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="79" t="s">
+      <c r="F41" s="82" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -11824,7 +11796,6 @@
       <c r="AU41" s="10"/>
       <c r="AV41" s="47"/>
       <c r="AY41" s="8"/>
-      <c r="AZ41" s="8"/>
       <c r="BA41" s="9"/>
       <c r="BB41" s="10"/>
       <c r="BC41" s="11"/>
@@ -12051,7 +12022,6 @@
       <c r="AU42" s="10"/>
       <c r="AV42" s="47"/>
       <c r="AY42" s="8"/>
-      <c r="AZ42" s="8"/>
       <c r="BA42" s="9"/>
       <c r="BB42" s="10"/>
       <c r="BC42" s="11"/>
@@ -12229,19 +12199,19 @@
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="75"/>
-      <c r="B43" s="76" t="s">
+      <c r="B43" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="78" t="s">
+      <c r="C43" s="77" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="77" t="s">
+      <c r="E43" s="80" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="79" t="s">
+      <c r="F43" s="82" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12285,7 +12255,6 @@
       <c r="AU43" s="10"/>
       <c r="AV43" s="47"/>
       <c r="AY43" s="8"/>
-      <c r="AZ43" s="8"/>
       <c r="BA43" s="9"/>
       <c r="BB43" s="10"/>
       <c r="BC43" s="11"/>
@@ -12512,9 +12481,8 @@
       <c r="AT44" s="68"/>
       <c r="AU44" s="10"/>
       <c r="AV44" s="47"/>
-      <c r="AX44" s="73"/>
+      <c r="AX44" s="61"/>
       <c r="AY44" s="8"/>
-      <c r="AZ44" s="8"/>
       <c r="BA44" s="9"/>
       <c r="BB44" s="10"/>
       <c r="BC44" s="11"/>
@@ -12692,19 +12660,19 @@
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="75"/>
-      <c r="B45" s="76" t="s">
+      <c r="B45" s="81" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="78" t="s">
+      <c r="C45" s="77" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="77" t="s">
+      <c r="E45" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="79" t="s">
+      <c r="F45" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12749,7 +12717,6 @@
       <c r="AV45" s="47"/>
       <c r="AW45" s="52"/>
       <c r="AY45" s="8"/>
-      <c r="AZ45" s="8"/>
       <c r="BA45" s="9"/>
       <c r="BB45" s="10"/>
       <c r="BC45" s="11"/>
@@ -12977,7 +12944,6 @@
       <c r="AV46" s="47"/>
       <c r="AW46" s="56"/>
       <c r="AY46" s="8"/>
-      <c r="AZ46" s="8"/>
       <c r="BA46" s="9"/>
       <c r="BB46" s="10"/>
       <c r="BC46" s="11"/>
@@ -13154,22 +13120,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="85" t="s">
+      <c r="A47" s="76" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="76" t="s">
+      <c r="B47" s="81" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="78" t="s">
+      <c r="C47" s="77" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="77" t="s">
+      <c r="E47" s="80" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="79" t="s">
+      <c r="F47" s="82" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13213,9 +13179,9 @@
       <c r="AT47" s="68"/>
       <c r="AU47" s="10"/>
       <c r="AV47" s="47"/>
-      <c r="AX47" s="71"/>
+      <c r="AX47" s="52"/>
       <c r="AY47" s="7"/>
-      <c r="AZ47" s="7"/>
+      <c r="AZ47" s="71"/>
       <c r="BA47" s="9"/>
       <c r="BB47" s="10"/>
       <c r="BC47" s="11"/>
@@ -13442,7 +13408,7 @@
       <c r="AU48" s="10"/>
       <c r="AV48" s="47"/>
       <c r="AY48" s="8"/>
-      <c r="AZ48" s="8"/>
+      <c r="AZ48" s="72"/>
       <c r="BA48" s="9"/>
       <c r="BB48" s="10"/>
       <c r="BC48" s="11"/>
@@ -13620,19 +13586,19 @@
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="75"/>
-      <c r="B49" s="76" t="s">
+      <c r="B49" s="81" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="78" t="s">
+      <c r="C49" s="77" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="77" t="s">
+      <c r="E49" s="80" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="79" t="s">
+      <c r="F49" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13677,7 +13643,6 @@
       <c r="AU49" s="10"/>
       <c r="AV49" s="47"/>
       <c r="AY49" s="8"/>
-      <c r="AZ49" s="8"/>
       <c r="BA49" s="9"/>
       <c r="BB49" s="10"/>
       <c r="BC49" s="11"/>
@@ -13904,7 +13869,6 @@
       <c r="AU50" s="10"/>
       <c r="AV50" s="47"/>
       <c r="AY50" s="8"/>
-      <c r="AZ50" s="8"/>
       <c r="BA50" s="9"/>
       <c r="BB50" s="10"/>
       <c r="BC50" s="11"/>
@@ -14081,22 +14045,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="85" t="s">
+      <c r="A51" s="76" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="76" t="s">
+      <c r="B51" s="81" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="78" t="s">
+      <c r="C51" s="77" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="77" t="s">
+      <c r="E51" s="80" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="79" t="s">
+      <c r="F51" s="82" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14141,7 +14105,6 @@
       <c r="AU51" s="10"/>
       <c r="AV51" s="47"/>
       <c r="AY51" s="8"/>
-      <c r="AZ51" s="8"/>
       <c r="BA51" s="9"/>
       <c r="BB51" s="10"/>
       <c r="BC51" s="11"/>
@@ -14368,7 +14331,6 @@
       <c r="AU52" s="10"/>
       <c r="AV52" s="47"/>
       <c r="AY52" s="8"/>
-      <c r="AZ52" s="8"/>
       <c r="BA52" s="9"/>
       <c r="BB52" s="10"/>
       <c r="BC52" s="11"/>
@@ -14546,19 +14508,19 @@
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="75"/>
-      <c r="B53" s="76" t="s">
+      <c r="B53" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="78" t="s">
+      <c r="C53" s="77" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="77" t="s">
+      <c r="E53" s="80" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="79" t="s">
+      <c r="F53" s="82" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14603,7 +14565,6 @@
       <c r="AU53" s="10"/>
       <c r="AV53" s="47"/>
       <c r="AY53" s="8"/>
-      <c r="AZ53" s="8"/>
       <c r="BA53" s="9"/>
       <c r="BB53" s="10"/>
       <c r="BC53" s="11"/>
@@ -14830,7 +14791,6 @@
       <c r="AU54" s="10"/>
       <c r="AV54" s="47"/>
       <c r="AY54" s="8"/>
-      <c r="AZ54" s="8"/>
       <c r="BA54" s="9"/>
       <c r="BB54" s="10"/>
       <c r="BC54" s="11"/>
@@ -15007,22 +14967,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="85" t="s">
+      <c r="A55" s="76" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="76" t="s">
+      <c r="B55" s="81" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="78" t="s">
+      <c r="C55" s="77" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="77" t="s">
+      <c r="E55" s="80" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="79" t="s">
+      <c r="F55" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -15067,7 +15027,6 @@
       <c r="AU55" s="10"/>
       <c r="AV55" s="47"/>
       <c r="AY55" s="8"/>
-      <c r="AZ55" s="8"/>
       <c r="BA55" s="9"/>
       <c r="BB55" s="10"/>
       <c r="BC55" s="11"/>
@@ -15294,7 +15253,6 @@
       <c r="AU56" s="10"/>
       <c r="AV56" s="47"/>
       <c r="AY56" s="8"/>
-      <c r="AZ56" s="8"/>
       <c r="BA56" s="9"/>
       <c r="BB56" s="10"/>
       <c r="BC56" s="11"/>
@@ -15472,19 +15430,19 @@
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="75"/>
-      <c r="B57" s="76" t="s">
+      <c r="B57" s="81" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="78" t="s">
+      <c r="C57" s="77" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="77" t="s">
+      <c r="E57" s="80" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="79" t="s">
+      <c r="F57" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15529,7 +15487,6 @@
       <c r="AU57" s="10"/>
       <c r="AV57" s="47"/>
       <c r="AY57" s="8"/>
-      <c r="AZ57" s="8"/>
       <c r="BA57" s="9"/>
       <c r="BB57" s="10"/>
       <c r="BC57" s="11"/>
@@ -15756,7 +15713,6 @@
       <c r="AU58" s="10"/>
       <c r="AV58" s="47"/>
       <c r="AY58" s="8"/>
-      <c r="AZ58" s="8"/>
       <c r="BA58" s="9"/>
       <c r="BB58" s="10"/>
       <c r="BC58" s="11"/>
@@ -15934,19 +15890,19 @@
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="75"/>
-      <c r="B59" s="76" t="s">
+      <c r="B59" s="81" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="78" t="s">
+      <c r="C59" s="77" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="77" t="s">
+      <c r="E59" s="80" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="79" t="s">
+      <c r="F59" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -15991,7 +15947,6 @@
       <c r="AU59" s="10"/>
       <c r="AV59" s="47"/>
       <c r="AY59" s="8"/>
-      <c r="AZ59" s="8"/>
       <c r="BA59" s="9"/>
       <c r="BB59" s="10"/>
       <c r="BC59" s="11"/>
@@ -16218,7 +16173,6 @@
       <c r="AU60" s="10"/>
       <c r="AV60" s="47"/>
       <c r="AY60" s="8"/>
-      <c r="AZ60" s="8"/>
       <c r="BA60" s="9"/>
       <c r="BB60" s="10"/>
       <c r="BC60" s="11"/>
@@ -16396,19 +16350,19 @@
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="75"/>
-      <c r="B61" s="76" t="s">
+      <c r="B61" s="81" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="78" t="s">
+      <c r="C61" s="77" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="77" t="s">
+      <c r="E61" s="80" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="79" t="s">
+      <c r="F61" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16453,7 +16407,6 @@
       <c r="AU61" s="10"/>
       <c r="AV61" s="47"/>
       <c r="AY61" s="8"/>
-      <c r="AZ61" s="8"/>
       <c r="BA61" s="9"/>
       <c r="BB61" s="10"/>
       <c r="BC61" s="11"/>
@@ -16680,7 +16633,6 @@
       <c r="AU62" s="10"/>
       <c r="AV62" s="47"/>
       <c r="AY62" s="8"/>
-      <c r="AZ62" s="8"/>
       <c r="BA62" s="9"/>
       <c r="BB62" s="10"/>
       <c r="BC62" s="11"/>
@@ -16858,19 +16810,19 @@
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="75"/>
-      <c r="B63" s="76" t="s">
+      <c r="B63" s="81" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="78" t="s">
+      <c r="C63" s="77" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="77" t="s">
+      <c r="E63" s="80" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="79" t="s">
+      <c r="F63" s="82" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -16915,7 +16867,6 @@
       <c r="AU63" s="10"/>
       <c r="AV63" s="47"/>
       <c r="AY63" s="8"/>
-      <c r="AZ63" s="8"/>
       <c r="BA63" s="9"/>
       <c r="BB63" s="10"/>
       <c r="BC63" s="11"/>
@@ -17142,7 +17093,6 @@
       <c r="AU64" s="10"/>
       <c r="AV64" s="47"/>
       <c r="AY64" s="8"/>
-      <c r="AZ64" s="8"/>
       <c r="BA64" s="9"/>
       <c r="BB64" s="10"/>
       <c r="BC64" s="11"/>
@@ -17320,19 +17270,19 @@
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="75"/>
-      <c r="B65" s="76" t="s">
+      <c r="B65" s="81" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="78" t="s">
+      <c r="C65" s="77" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="77" t="s">
+      <c r="E65" s="80" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="79" t="s">
+      <c r="F65" s="82" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17377,7 +17327,6 @@
       <c r="AU65" s="10"/>
       <c r="AV65" s="47"/>
       <c r="AY65" s="8"/>
-      <c r="AZ65" s="8"/>
       <c r="BA65" s="9"/>
       <c r="BB65" s="10"/>
       <c r="BC65" s="11"/>
@@ -17604,7 +17553,6 @@
       <c r="AU66" s="10"/>
       <c r="AV66" s="47"/>
       <c r="AY66" s="8"/>
-      <c r="AZ66" s="8"/>
       <c r="BA66" s="9"/>
       <c r="BB66" s="10"/>
       <c r="BC66" s="11"/>
@@ -17781,22 +17729,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="85" t="s">
+      <c r="A67" s="76" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="76" t="s">
+      <c r="B67" s="81" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="78" t="s">
+      <c r="C67" s="77" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="77" t="s">
+      <c r="E67" s="80" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="79" t="s">
+      <c r="F67" s="82" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -17841,7 +17789,6 @@
       <c r="AU67" s="10"/>
       <c r="AV67" s="47"/>
       <c r="AY67" s="8"/>
-      <c r="AZ67" s="8"/>
       <c r="BA67" s="9"/>
       <c r="BB67" s="10"/>
       <c r="BC67" s="11"/>
@@ -18069,7 +18016,6 @@
       <c r="AV68" s="47"/>
       <c r="AW68" s="61"/>
       <c r="AY68" s="8"/>
-      <c r="AZ68" s="8"/>
       <c r="BA68" s="9"/>
       <c r="BB68" s="10"/>
       <c r="BC68" s="11"/>
@@ -18247,19 +18193,19 @@
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="75"/>
-      <c r="B69" s="76" t="s">
+      <c r="B69" s="81" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="78" t="s">
+      <c r="C69" s="77" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="77" t="s">
+      <c r="E69" s="80" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="79" t="s">
+      <c r="F69" s="82" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18305,9 +18251,9 @@
       <c r="AU69" s="10"/>
       <c r="AV69" s="47"/>
       <c r="AW69" s="54"/>
-      <c r="AX69" s="70"/>
+      <c r="AX69" s="54"/>
       <c r="AY69" s="16"/>
-      <c r="AZ69" s="16"/>
+      <c r="AZ69" s="70"/>
       <c r="BA69" s="9"/>
       <c r="BB69" s="10"/>
       <c r="BC69" s="11"/>
@@ -18534,9 +18480,8 @@
       <c r="AU70" s="10"/>
       <c r="AV70" s="47"/>
       <c r="AW70" s="56"/>
-      <c r="AX70" s="72"/>
+      <c r="AX70" s="56"/>
       <c r="AY70" s="8"/>
-      <c r="AZ70" s="8"/>
       <c r="BA70" s="9"/>
       <c r="BB70" s="10"/>
       <c r="BC70" s="11"/>
@@ -18714,19 +18659,19 @@
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="75"/>
-      <c r="B71" s="76" t="s">
+      <c r="B71" s="81" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="78" t="s">
+      <c r="C71" s="77" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="77" t="s">
+      <c r="E71" s="80" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="79" t="s">
+      <c r="F71" s="82" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -18771,7 +18716,6 @@
       <c r="AU71" s="10"/>
       <c r="AV71" s="47"/>
       <c r="AY71" s="8"/>
-      <c r="AZ71" s="8"/>
       <c r="BA71" s="9"/>
       <c r="BB71" s="10"/>
       <c r="BC71" s="11"/>
@@ -18998,7 +18942,6 @@
       <c r="AU72" s="10"/>
       <c r="AV72" s="47"/>
       <c r="AY72" s="8"/>
-      <c r="AZ72" s="8"/>
       <c r="BA72" s="9"/>
       <c r="BB72" s="10"/>
       <c r="BC72" s="11"/>
@@ -19176,19 +19119,19 @@
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="75"/>
-      <c r="B73" s="76" t="s">
+      <c r="B73" s="81" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="78" t="s">
+      <c r="C73" s="77" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="77" t="s">
+      <c r="E73" s="80" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="79" t="s">
+      <c r="F73" s="82" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19233,7 +19176,6 @@
       <c r="AU73" s="10"/>
       <c r="AV73" s="47"/>
       <c r="AY73" s="8"/>
-      <c r="AZ73" s="8"/>
       <c r="BA73" s="9"/>
       <c r="BB73" s="10"/>
       <c r="BC73" s="11"/>
@@ -19460,7 +19402,6 @@
       <c r="AU74" s="10"/>
       <c r="AV74" s="47"/>
       <c r="AY74" s="8"/>
-      <c r="AZ74" s="8"/>
       <c r="BA74" s="9"/>
       <c r="BB74" s="10"/>
       <c r="BC74" s="11"/>
@@ -19638,19 +19579,19 @@
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="75"/>
-      <c r="B75" s="76" t="s">
+      <c r="B75" s="81" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="78" t="s">
+      <c r="C75" s="77" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="77" t="s">
+      <c r="E75" s="80" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="79" t="s">
+      <c r="F75" s="82" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19695,7 +19636,6 @@
       <c r="AU75" s="10"/>
       <c r="AV75" s="47"/>
       <c r="AY75" s="8"/>
-      <c r="AZ75" s="8"/>
       <c r="BA75" s="9"/>
       <c r="BB75" s="10"/>
       <c r="BC75" s="11"/>
@@ -19922,7 +19862,6 @@
       <c r="AU76" s="10"/>
       <c r="AV76" s="47"/>
       <c r="AY76" s="8"/>
-      <c r="AZ76" s="8"/>
       <c r="BA76" s="9"/>
       <c r="BB76" s="10"/>
       <c r="BC76" s="11"/>
@@ -20100,19 +20039,19 @@
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="75"/>
-      <c r="B77" s="76" t="s">
+      <c r="B77" s="81" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="78" t="s">
+      <c r="C77" s="77" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="77" t="s">
+      <c r="E77" s="80" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="79" t="s">
+      <c r="F77" s="82" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20157,7 +20096,6 @@
       <c r="AU77" s="10"/>
       <c r="AV77" s="47"/>
       <c r="AY77" s="8"/>
-      <c r="AZ77" s="8"/>
       <c r="BA77" s="9"/>
       <c r="BB77" s="10"/>
       <c r="BC77" s="11"/>
@@ -20384,7 +20322,6 @@
       <c r="AU78" s="10"/>
       <c r="AV78" s="47"/>
       <c r="AY78" s="8"/>
-      <c r="AZ78" s="8"/>
       <c r="BA78" s="9"/>
       <c r="BB78" s="10"/>
       <c r="BC78" s="11"/>
@@ -20561,22 +20498,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="85" t="s">
+      <c r="A79" s="76" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="76" t="s">
+      <c r="B79" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="74" t="s">
+      <c r="C79" s="84" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="77" t="s">
+      <c r="E79" s="80" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="79" t="s">
+      <c r="F79" s="82" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20621,7 +20558,6 @@
       <c r="AU79" s="10"/>
       <c r="AV79" s="47"/>
       <c r="AY79" s="8"/>
-      <c r="AZ79" s="8"/>
       <c r="BA79" s="9"/>
       <c r="BB79" s="10"/>
       <c r="BC79" s="11"/>
@@ -20848,7 +20784,6 @@
       <c r="AU80" s="10"/>
       <c r="AV80" s="47"/>
       <c r="AY80" s="8"/>
-      <c r="AZ80" s="8"/>
       <c r="BA80" s="9"/>
       <c r="BB80" s="10"/>
       <c r="BC80" s="11"/>
@@ -21026,19 +20961,19 @@
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="75"/>
-      <c r="B81" s="76" t="s">
+      <c r="B81" s="81" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="74" t="s">
+      <c r="C81" s="84" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="77" t="s">
+      <c r="E81" s="80" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="79" t="s">
+      <c r="F81" s="82" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -21083,7 +21018,6 @@
       <c r="AU81" s="10"/>
       <c r="AV81" s="47"/>
       <c r="AY81" s="8"/>
-      <c r="AZ81" s="8"/>
       <c r="BA81" s="9"/>
       <c r="BB81" s="10"/>
       <c r="BC81" s="11"/>
@@ -21310,7 +21244,6 @@
       <c r="AU82" s="10"/>
       <c r="AV82" s="47"/>
       <c r="AY82" s="8"/>
-      <c r="AZ82" s="8"/>
       <c r="BA82" s="9"/>
       <c r="BB82" s="10"/>
       <c r="BC82" s="11"/>
@@ -21488,19 +21421,19 @@
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="75"/>
-      <c r="B83" s="76" t="s">
+      <c r="B83" s="81" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="78" t="s">
+      <c r="C83" s="77" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="77" t="s">
+      <c r="E83" s="80" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="79" t="s">
+      <c r="F83" s="82" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21545,7 +21478,6 @@
       <c r="AU83" s="10"/>
       <c r="AV83" s="47"/>
       <c r="AY83" s="8"/>
-      <c r="AZ83" s="8"/>
       <c r="BA83" s="9"/>
       <c r="BB83" s="10"/>
       <c r="BC83" s="11"/>
@@ -21772,7 +21704,6 @@
       <c r="AU84" s="10"/>
       <c r="AV84" s="47"/>
       <c r="AY84" s="8"/>
-      <c r="AZ84" s="8"/>
       <c r="BA84" s="9"/>
       <c r="BB84" s="10"/>
       <c r="BC84" s="11"/>
@@ -21950,19 +21881,19 @@
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="75"/>
-      <c r="B85" s="76" t="s">
+      <c r="B85" s="81" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="87" t="s">
+      <c r="C85" s="88" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="77" t="s">
+      <c r="E85" s="80" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="79"/>
+      <c r="F85" s="82"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -22005,7 +21936,6 @@
       <c r="AU85" s="10"/>
       <c r="AV85" s="47"/>
       <c r="AY85" s="8"/>
-      <c r="AZ85" s="8"/>
       <c r="BA85" s="9"/>
       <c r="BB85" s="10"/>
       <c r="BC85" s="11"/>
@@ -22232,7 +22162,6 @@
       <c r="AU86" s="10"/>
       <c r="AV86" s="47"/>
       <c r="AY86" s="8"/>
-      <c r="AZ86" s="8"/>
       <c r="BA86" s="9"/>
       <c r="BB86" s="10"/>
       <c r="BC86" s="11"/>
@@ -22410,20 +22339,173 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="GU1:HA1"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
     <mergeCell ref="E85:E86"/>
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="B85:B86"/>
@@ -22448,173 +22530,20 @@
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="GU1:HA1"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
NO Konzeption sortiert. Datengenerierungspipeline gestartet
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13367A7E-B423-40C5-A7D7-365D025C4719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752CAFCF-9827-4CC8-BC47-8E2F67B42E6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
@@ -1147,7 +1147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1262,53 +1262,54 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1628,298 +1629,300 @@
     <col min="49" max="49" width="2.140625" style="67" customWidth="1"/>
     <col min="50" max="50" width="2.140625" style="73" customWidth="1"/>
     <col min="51" max="51" width="2.140625" customWidth="1"/>
-    <col min="52" max="52" width="2.140625" style="66" customWidth="1"/>
-    <col min="53" max="226" width="2.140625" customWidth="1"/>
+    <col min="52" max="52" width="2.140625" style="74" customWidth="1"/>
+    <col min="53" max="55" width="2.140625" customWidth="1"/>
+    <col min="56" max="56" width="2.140625" style="66" customWidth="1"/>
+    <col min="57" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="74" t="s">
+      <c r="G1" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="74" t="s">
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="74" t="s">
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="75"/>
-      <c r="W1" s="75"/>
-      <c r="X1" s="75"/>
-      <c r="Y1" s="75"/>
-      <c r="Z1" s="75"/>
-      <c r="AA1" s="75"/>
-      <c r="AB1" s="90" t="s">
+      <c r="V1" s="77"/>
+      <c r="W1" s="77"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="77"/>
+      <c r="Z1" s="77"/>
+      <c r="AA1" s="77"/>
+      <c r="AB1" s="83" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="75"/>
-      <c r="AD1" s="75"/>
-      <c r="AE1" s="75"/>
-      <c r="AF1" s="75"/>
-      <c r="AG1" s="75"/>
-      <c r="AH1" s="75"/>
-      <c r="AI1" s="74" t="s">
+      <c r="AC1" s="77"/>
+      <c r="AD1" s="77"/>
+      <c r="AE1" s="77"/>
+      <c r="AF1" s="77"/>
+      <c r="AG1" s="77"/>
+      <c r="AH1" s="77"/>
+      <c r="AI1" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="75"/>
-      <c r="AK1" s="75"/>
-      <c r="AL1" s="75"/>
-      <c r="AM1" s="75"/>
-      <c r="AN1" s="75"/>
-      <c r="AO1" s="75"/>
-      <c r="AP1" s="74" t="s">
+      <c r="AJ1" s="77"/>
+      <c r="AK1" s="77"/>
+      <c r="AL1" s="77"/>
+      <c r="AM1" s="77"/>
+      <c r="AN1" s="77"/>
+      <c r="AO1" s="77"/>
+      <c r="AP1" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="75"/>
-      <c r="AR1" s="75"/>
-      <c r="AS1" s="75"/>
-      <c r="AT1" s="75"/>
-      <c r="AU1" s="75"/>
-      <c r="AV1" s="75"/>
-      <c r="AW1" s="74" t="s">
+      <c r="AQ1" s="77"/>
+      <c r="AR1" s="77"/>
+      <c r="AS1" s="77"/>
+      <c r="AT1" s="77"/>
+      <c r="AU1" s="77"/>
+      <c r="AV1" s="77"/>
+      <c r="AW1" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="75"/>
-      <c r="AY1" s="75"/>
-      <c r="AZ1" s="75"/>
-      <c r="BA1" s="75"/>
-      <c r="BB1" s="75"/>
-      <c r="BC1" s="75"/>
-      <c r="BD1" s="74" t="s">
+      <c r="AX1" s="77"/>
+      <c r="AY1" s="77"/>
+      <c r="AZ1" s="77"/>
+      <c r="BA1" s="77"/>
+      <c r="BB1" s="77"/>
+      <c r="BC1" s="77"/>
+      <c r="BD1" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="75"/>
-      <c r="BF1" s="75"/>
-      <c r="BG1" s="75"/>
-      <c r="BH1" s="75"/>
-      <c r="BI1" s="75"/>
-      <c r="BJ1" s="75"/>
-      <c r="BK1" s="74" t="s">
+      <c r="BE1" s="77"/>
+      <c r="BF1" s="77"/>
+      <c r="BG1" s="77"/>
+      <c r="BH1" s="77"/>
+      <c r="BI1" s="77"/>
+      <c r="BJ1" s="77"/>
+      <c r="BK1" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="75"/>
-      <c r="BM1" s="75"/>
-      <c r="BN1" s="75"/>
-      <c r="BO1" s="75"/>
-      <c r="BP1" s="75"/>
-      <c r="BQ1" s="75"/>
-      <c r="BR1" s="74" t="s">
+      <c r="BL1" s="77"/>
+      <c r="BM1" s="77"/>
+      <c r="BN1" s="77"/>
+      <c r="BO1" s="77"/>
+      <c r="BP1" s="77"/>
+      <c r="BQ1" s="77"/>
+      <c r="BR1" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="75"/>
-      <c r="BT1" s="75"/>
-      <c r="BU1" s="75"/>
-      <c r="BV1" s="75"/>
-      <c r="BW1" s="75"/>
-      <c r="BX1" s="75"/>
-      <c r="BY1" s="74" t="s">
+      <c r="BS1" s="77"/>
+      <c r="BT1" s="77"/>
+      <c r="BU1" s="77"/>
+      <c r="BV1" s="77"/>
+      <c r="BW1" s="77"/>
+      <c r="BX1" s="77"/>
+      <c r="BY1" s="82" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="75"/>
-      <c r="CA1" s="75"/>
-      <c r="CB1" s="75"/>
-      <c r="CC1" s="75"/>
-      <c r="CD1" s="75"/>
-      <c r="CE1" s="75"/>
-      <c r="CF1" s="74" t="s">
+      <c r="BZ1" s="77"/>
+      <c r="CA1" s="77"/>
+      <c r="CB1" s="77"/>
+      <c r="CC1" s="77"/>
+      <c r="CD1" s="77"/>
+      <c r="CE1" s="77"/>
+      <c r="CF1" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="75"/>
-      <c r="CH1" s="75"/>
-      <c r="CI1" s="75"/>
-      <c r="CJ1" s="75"/>
-      <c r="CK1" s="75"/>
-      <c r="CL1" s="75"/>
-      <c r="CM1" s="74" t="s">
+      <c r="CG1" s="77"/>
+      <c r="CH1" s="77"/>
+      <c r="CI1" s="77"/>
+      <c r="CJ1" s="77"/>
+      <c r="CK1" s="77"/>
+      <c r="CL1" s="77"/>
+      <c r="CM1" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="75"/>
-      <c r="CO1" s="75"/>
-      <c r="CP1" s="75"/>
-      <c r="CQ1" s="75"/>
-      <c r="CR1" s="75"/>
-      <c r="CS1" s="75"/>
-      <c r="CT1" s="74" t="s">
+      <c r="CN1" s="77"/>
+      <c r="CO1" s="77"/>
+      <c r="CP1" s="77"/>
+      <c r="CQ1" s="77"/>
+      <c r="CR1" s="77"/>
+      <c r="CS1" s="77"/>
+      <c r="CT1" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="75"/>
-      <c r="CV1" s="75"/>
-      <c r="CW1" s="75"/>
-      <c r="CX1" s="75"/>
-      <c r="CY1" s="75"/>
-      <c r="CZ1" s="75"/>
-      <c r="DA1" s="74" t="s">
+      <c r="CU1" s="77"/>
+      <c r="CV1" s="77"/>
+      <c r="CW1" s="77"/>
+      <c r="CX1" s="77"/>
+      <c r="CY1" s="77"/>
+      <c r="CZ1" s="77"/>
+      <c r="DA1" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="75"/>
-      <c r="DC1" s="75"/>
-      <c r="DD1" s="75"/>
-      <c r="DE1" s="75"/>
-      <c r="DF1" s="75"/>
-      <c r="DG1" s="75"/>
-      <c r="DH1" s="74" t="s">
+      <c r="DB1" s="77"/>
+      <c r="DC1" s="77"/>
+      <c r="DD1" s="77"/>
+      <c r="DE1" s="77"/>
+      <c r="DF1" s="77"/>
+      <c r="DG1" s="77"/>
+      <c r="DH1" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="75"/>
-      <c r="DJ1" s="75"/>
-      <c r="DK1" s="75"/>
-      <c r="DL1" s="75"/>
-      <c r="DM1" s="75"/>
-      <c r="DN1" s="75"/>
-      <c r="DO1" s="74" t="s">
+      <c r="DI1" s="77"/>
+      <c r="DJ1" s="77"/>
+      <c r="DK1" s="77"/>
+      <c r="DL1" s="77"/>
+      <c r="DM1" s="77"/>
+      <c r="DN1" s="77"/>
+      <c r="DO1" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="75"/>
-      <c r="DQ1" s="75"/>
-      <c r="DR1" s="75"/>
-      <c r="DS1" s="75"/>
-      <c r="DT1" s="75"/>
-      <c r="DU1" s="75"/>
-      <c r="DV1" s="74" t="s">
+      <c r="DP1" s="77"/>
+      <c r="DQ1" s="77"/>
+      <c r="DR1" s="77"/>
+      <c r="DS1" s="77"/>
+      <c r="DT1" s="77"/>
+      <c r="DU1" s="77"/>
+      <c r="DV1" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="75"/>
-      <c r="DX1" s="75"/>
-      <c r="DY1" s="75"/>
-      <c r="DZ1" s="75"/>
-      <c r="EA1" s="75"/>
-      <c r="EB1" s="75"/>
-      <c r="EC1" s="74" t="s">
+      <c r="DW1" s="77"/>
+      <c r="DX1" s="77"/>
+      <c r="DY1" s="77"/>
+      <c r="DZ1" s="77"/>
+      <c r="EA1" s="77"/>
+      <c r="EB1" s="77"/>
+      <c r="EC1" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="75"/>
-      <c r="EE1" s="75"/>
-      <c r="EF1" s="75"/>
-      <c r="EG1" s="75"/>
-      <c r="EH1" s="75"/>
-      <c r="EI1" s="75"/>
-      <c r="EJ1" s="74" t="s">
+      <c r="ED1" s="77"/>
+      <c r="EE1" s="77"/>
+      <c r="EF1" s="77"/>
+      <c r="EG1" s="77"/>
+      <c r="EH1" s="77"/>
+      <c r="EI1" s="77"/>
+      <c r="EJ1" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="75"/>
-      <c r="EL1" s="75"/>
-      <c r="EM1" s="75"/>
-      <c r="EN1" s="75"/>
-      <c r="EO1" s="75"/>
-      <c r="EP1" s="75"/>
-      <c r="EQ1" s="74" t="s">
+      <c r="EK1" s="77"/>
+      <c r="EL1" s="77"/>
+      <c r="EM1" s="77"/>
+      <c r="EN1" s="77"/>
+      <c r="EO1" s="77"/>
+      <c r="EP1" s="77"/>
+      <c r="EQ1" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="75"/>
-      <c r="ES1" s="75"/>
-      <c r="ET1" s="75"/>
-      <c r="EU1" s="75"/>
-      <c r="EV1" s="75"/>
-      <c r="EW1" s="75"/>
-      <c r="EX1" s="74" t="s">
+      <c r="ER1" s="77"/>
+      <c r="ES1" s="77"/>
+      <c r="ET1" s="77"/>
+      <c r="EU1" s="77"/>
+      <c r="EV1" s="77"/>
+      <c r="EW1" s="77"/>
+      <c r="EX1" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="75"/>
-      <c r="EZ1" s="75"/>
-      <c r="FA1" s="75"/>
-      <c r="FB1" s="75"/>
-      <c r="FC1" s="75"/>
-      <c r="FD1" s="75"/>
-      <c r="FE1" s="74" t="s">
+      <c r="EY1" s="77"/>
+      <c r="EZ1" s="77"/>
+      <c r="FA1" s="77"/>
+      <c r="FB1" s="77"/>
+      <c r="FC1" s="77"/>
+      <c r="FD1" s="77"/>
+      <c r="FE1" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="75"/>
-      <c r="FG1" s="75"/>
-      <c r="FH1" s="75"/>
-      <c r="FI1" s="75"/>
-      <c r="FJ1" s="75"/>
-      <c r="FK1" s="75"/>
-      <c r="FL1" s="74" t="s">
+      <c r="FF1" s="77"/>
+      <c r="FG1" s="77"/>
+      <c r="FH1" s="77"/>
+      <c r="FI1" s="77"/>
+      <c r="FJ1" s="77"/>
+      <c r="FK1" s="77"/>
+      <c r="FL1" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="75"/>
-      <c r="FN1" s="75"/>
-      <c r="FO1" s="75"/>
-      <c r="FP1" s="75"/>
-      <c r="FQ1" s="75"/>
-      <c r="FR1" s="75"/>
-      <c r="FS1" s="74" t="s">
+      <c r="FM1" s="77"/>
+      <c r="FN1" s="77"/>
+      <c r="FO1" s="77"/>
+      <c r="FP1" s="77"/>
+      <c r="FQ1" s="77"/>
+      <c r="FR1" s="77"/>
+      <c r="FS1" s="82" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="75"/>
-      <c r="FU1" s="75"/>
-      <c r="FV1" s="75"/>
-      <c r="FW1" s="75"/>
-      <c r="FX1" s="75"/>
-      <c r="FY1" s="75"/>
-      <c r="FZ1" s="74" t="s">
+      <c r="FT1" s="77"/>
+      <c r="FU1" s="77"/>
+      <c r="FV1" s="77"/>
+      <c r="FW1" s="77"/>
+      <c r="FX1" s="77"/>
+      <c r="FY1" s="77"/>
+      <c r="FZ1" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="75"/>
-      <c r="GB1" s="75"/>
-      <c r="GC1" s="75"/>
-      <c r="GD1" s="75"/>
-      <c r="GE1" s="75"/>
-      <c r="GF1" s="75"/>
-      <c r="GG1" s="74" t="s">
+      <c r="GA1" s="77"/>
+      <c r="GB1" s="77"/>
+      <c r="GC1" s="77"/>
+      <c r="GD1" s="77"/>
+      <c r="GE1" s="77"/>
+      <c r="GF1" s="77"/>
+      <c r="GG1" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="75"/>
-      <c r="GI1" s="75"/>
-      <c r="GJ1" s="75"/>
-      <c r="GK1" s="75"/>
-      <c r="GL1" s="75"/>
-      <c r="GM1" s="75"/>
-      <c r="GN1" s="74" t="s">
+      <c r="GH1" s="77"/>
+      <c r="GI1" s="77"/>
+      <c r="GJ1" s="77"/>
+      <c r="GK1" s="77"/>
+      <c r="GL1" s="77"/>
+      <c r="GM1" s="77"/>
+      <c r="GN1" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="75"/>
-      <c r="GP1" s="75"/>
-      <c r="GQ1" s="75"/>
-      <c r="GR1" s="75"/>
-      <c r="GS1" s="75"/>
-      <c r="GT1" s="75"/>
-      <c r="GU1" s="74" t="s">
+      <c r="GO1" s="77"/>
+      <c r="GP1" s="77"/>
+      <c r="GQ1" s="77"/>
+      <c r="GR1" s="77"/>
+      <c r="GS1" s="77"/>
+      <c r="GT1" s="77"/>
+      <c r="GU1" s="82" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="75"/>
-      <c r="GW1" s="75"/>
-      <c r="GX1" s="75"/>
-      <c r="GY1" s="75"/>
-      <c r="GZ1" s="75"/>
-      <c r="HA1" s="75"/>
-      <c r="HB1" s="74" t="s">
+      <c r="GV1" s="77"/>
+      <c r="GW1" s="77"/>
+      <c r="GX1" s="77"/>
+      <c r="GY1" s="77"/>
+      <c r="GZ1" s="77"/>
+      <c r="HA1" s="77"/>
+      <c r="HB1" s="82" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="75"/>
-      <c r="HD1" s="75"/>
-      <c r="HE1" s="75"/>
-      <c r="HF1" s="75"/>
-      <c r="HG1" s="75"/>
-      <c r="HH1" s="75"/>
-      <c r="HI1" s="74" t="s">
+      <c r="HC1" s="77"/>
+      <c r="HD1" s="77"/>
+      <c r="HE1" s="77"/>
+      <c r="HF1" s="77"/>
+      <c r="HG1" s="77"/>
+      <c r="HH1" s="77"/>
+      <c r="HI1" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="75"/>
-      <c r="HK1" s="75"/>
-      <c r="HL1" s="75"/>
-      <c r="HM1" s="75"/>
-      <c r="HN1" s="75"/>
-      <c r="HO1" s="75"/>
-      <c r="HP1" s="74" t="s">
+      <c r="HJ1" s="77"/>
+      <c r="HK1" s="77"/>
+      <c r="HL1" s="77"/>
+      <c r="HM1" s="77"/>
+      <c r="HN1" s="77"/>
+      <c r="HO1" s="77"/>
+      <c r="HP1" s="82" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="75"/>
-      <c r="HR1" s="75"/>
+      <c r="HQ1" s="77"/>
+      <c r="HR1" s="77"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="1" t="s">
@@ -2060,7 +2063,7 @@
       <c r="AY2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AZ2" s="63" t="s">
+      <c r="AZ2" s="62" t="s">
         <v>35</v>
       </c>
       <c r="BA2" s="2" t="s">
@@ -2072,7 +2075,7 @@
       <c r="BC2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="BD2" s="2" t="s">
+      <c r="BD2" s="63" t="s">
         <v>34</v>
       </c>
       <c r="BE2" s="2" t="s">
@@ -2725,7 +2728,7 @@
       <c r="AY3" s="3">
         <v>46295</v>
       </c>
-      <c r="AZ3" s="64">
+      <c r="AZ3" s="50">
         <v>46296</v>
       </c>
       <c r="BA3" s="3">
@@ -2737,7 +2740,7 @@
       <c r="BC3" s="3">
         <v>46299</v>
       </c>
-      <c r="BD3" s="3">
+      <c r="BD3" s="64">
         <v>46300</v>
       </c>
       <c r="BE3" s="3">
@@ -3313,11 +3316,11 @@
       <c r="AW4" s="51"/>
       <c r="AX4" s="51"/>
       <c r="AY4" s="5"/>
-      <c r="AZ4" s="65"/>
+      <c r="AZ4" s="51"/>
       <c r="BA4" s="5"/>
       <c r="BB4" s="5"/>
       <c r="BC4" s="5"/>
-      <c r="BD4" s="5"/>
+      <c r="BD4" s="65"/>
       <c r="BE4" s="5"/>
       <c r="BF4" s="5"/>
       <c r="BG4" s="5"/>
@@ -3490,20 +3493,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="85"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="88"/>
+      <c r="C5" s="86" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="83" t="s">
+      <c r="E5" s="90" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="87"/>
+      <c r="F5" s="84"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3545,11 +3548,10 @@
       <c r="AT5" s="68"/>
       <c r="AU5" s="10"/>
       <c r="AV5" s="47"/>
-      <c r="AY5" s="8"/>
+      <c r="AY5" s="74"/>
       <c r="BA5" s="9"/>
       <c r="BB5" s="10"/>
       <c r="BC5" s="11"/>
-      <c r="BD5" s="8"/>
       <c r="BE5" s="8"/>
       <c r="BF5" s="8"/>
       <c r="BG5" s="8"/>
@@ -3722,14 +3724,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="79"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="79"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="85"/>
+      <c r="C6" s="85"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3771,11 +3773,10 @@
       <c r="AT6" s="68"/>
       <c r="AU6" s="10"/>
       <c r="AV6" s="47"/>
-      <c r="AY6" s="8"/>
+      <c r="AY6" s="74"/>
       <c r="BA6" s="9"/>
       <c r="BB6" s="10"/>
       <c r="BC6" s="11"/>
-      <c r="BD6" s="8"/>
       <c r="BE6" s="8"/>
       <c r="BF6" s="8"/>
       <c r="BG6" s="8"/>
@@ -3948,18 +3949,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="79"/>
-      <c r="B7" s="85"/>
-      <c r="C7" s="78" t="s">
+      <c r="A7" s="85"/>
+      <c r="B7" s="88"/>
+      <c r="C7" s="86" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="83" t="s">
+      <c r="E7" s="90" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="87"/>
+      <c r="F7" s="84"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -4001,11 +4002,10 @@
       <c r="AT7" s="68"/>
       <c r="AU7" s="10"/>
       <c r="AV7" s="47"/>
-      <c r="AY7" s="8"/>
+      <c r="AY7" s="74"/>
       <c r="BA7" s="9"/>
       <c r="BB7" s="10"/>
       <c r="BC7" s="11"/>
-      <c r="BD7" s="8"/>
       <c r="BE7" s="8"/>
       <c r="BF7" s="8"/>
       <c r="BG7" s="8"/>
@@ -4178,14 +4178,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
+      <c r="A8" s="85"/>
+      <c r="B8" s="85"/>
+      <c r="C8" s="85"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="79"/>
-      <c r="F8" s="79"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="85"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4227,11 +4227,10 @@
       <c r="AT8" s="68"/>
       <c r="AU8" s="10"/>
       <c r="AV8" s="47"/>
-      <c r="AY8" s="8"/>
+      <c r="AY8" s="74"/>
       <c r="BA8" s="9"/>
       <c r="BB8" s="10"/>
       <c r="BC8" s="11"/>
-      <c r="BD8" s="8"/>
       <c r="BE8" s="8"/>
       <c r="BF8" s="8"/>
       <c r="BG8" s="8"/>
@@ -4404,18 +4403,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="79"/>
-      <c r="B9" s="85"/>
-      <c r="C9" s="78" t="s">
+      <c r="A9" s="85"/>
+      <c r="B9" s="88"/>
+      <c r="C9" s="86" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="83" t="s">
+      <c r="E9" s="90" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="87"/>
+      <c r="F9" s="84"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4457,11 +4456,10 @@
       <c r="AT9" s="68"/>
       <c r="AU9" s="10"/>
       <c r="AV9" s="47"/>
-      <c r="AY9" s="8"/>
+      <c r="AY9" s="74"/>
       <c r="BA9" s="9"/>
       <c r="BB9" s="10"/>
       <c r="BC9" s="11"/>
-      <c r="BD9" s="8"/>
       <c r="BE9" s="8"/>
       <c r="BF9" s="8"/>
       <c r="BG9" s="8"/>
@@ -4634,14 +4632,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="79"/>
-      <c r="B10" s="79"/>
-      <c r="C10" s="79"/>
+      <c r="A10" s="85"/>
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="79"/>
-      <c r="F10" s="79"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4683,11 +4681,10 @@
       <c r="AT10" s="68"/>
       <c r="AU10" s="10"/>
       <c r="AV10" s="47"/>
-      <c r="AY10" s="8"/>
+      <c r="AY10" s="74"/>
       <c r="BA10" s="9"/>
       <c r="BB10" s="10"/>
       <c r="BC10" s="11"/>
-      <c r="BD10" s="8"/>
       <c r="BE10" s="8"/>
       <c r="BF10" s="8"/>
       <c r="BG10" s="8"/>
@@ -4860,18 +4857,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="79"/>
-      <c r="B11" s="85"/>
-      <c r="C11" s="78" t="s">
+      <c r="A11" s="85"/>
+      <c r="B11" s="88"/>
+      <c r="C11" s="86" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="83" t="s">
+      <c r="E11" s="90" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="87"/>
+      <c r="F11" s="84"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -4913,11 +4910,10 @@
       <c r="AT11" s="68"/>
       <c r="AU11" s="10"/>
       <c r="AV11" s="47"/>
-      <c r="AY11" s="8"/>
+      <c r="AY11" s="74"/>
       <c r="BA11" s="9"/>
       <c r="BB11" s="10"/>
       <c r="BC11" s="11"/>
-      <c r="BD11" s="8"/>
       <c r="BE11" s="8"/>
       <c r="BF11" s="8"/>
       <c r="BG11" s="8"/>
@@ -5090,14 +5086,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="79"/>
-      <c r="B12" s="79"/>
-      <c r="C12" s="79"/>
+      <c r="A12" s="85"/>
+      <c r="B12" s="85"/>
+      <c r="C12" s="85"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="79"/>
-      <c r="F12" s="79"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="85"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5139,11 +5135,10 @@
       <c r="AT12" s="68"/>
       <c r="AU12" s="10"/>
       <c r="AV12" s="47"/>
-      <c r="AY12" s="8"/>
+      <c r="AY12" s="74"/>
       <c r="BA12" s="9"/>
       <c r="BB12" s="10"/>
       <c r="BC12" s="11"/>
-      <c r="BD12" s="8"/>
       <c r="BE12" s="8"/>
       <c r="BF12" s="8"/>
       <c r="BG12" s="8"/>
@@ -5316,18 +5311,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="79"/>
-      <c r="B13" s="85"/>
-      <c r="C13" s="78" t="s">
+      <c r="A13" s="85"/>
+      <c r="B13" s="88"/>
+      <c r="C13" s="86" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="83" t="s">
+      <c r="E13" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="87"/>
+      <c r="F13" s="84"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5369,11 +5364,10 @@
       <c r="AT13" s="68"/>
       <c r="AU13" s="10"/>
       <c r="AV13" s="47"/>
-      <c r="AY13" s="8"/>
+      <c r="AY13" s="74"/>
       <c r="BA13" s="9"/>
       <c r="BB13" s="10"/>
       <c r="BC13" s="11"/>
-      <c r="BD13" s="8"/>
       <c r="BE13" s="8"/>
       <c r="BF13" s="8"/>
       <c r="BG13" s="8"/>
@@ -5546,14 +5540,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="79"/>
-      <c r="B14" s="79"/>
-      <c r="C14" s="79"/>
+      <c r="A14" s="85"/>
+      <c r="B14" s="85"/>
+      <c r="C14" s="85"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="79"/>
-      <c r="F14" s="79"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="85"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5595,11 +5589,10 @@
       <c r="AT14" s="68"/>
       <c r="AU14" s="10"/>
       <c r="AV14" s="47"/>
-      <c r="AY14" s="8"/>
+      <c r="AY14" s="74"/>
       <c r="BA14" s="9"/>
       <c r="BB14" s="10"/>
       <c r="BC14" s="11"/>
-      <c r="BD14" s="8"/>
       <c r="BE14" s="8"/>
       <c r="BF14" s="8"/>
       <c r="BG14" s="8"/>
@@ -5772,18 +5765,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="79"/>
-      <c r="B15" s="85"/>
-      <c r="C15" s="78" t="s">
+      <c r="A15" s="85"/>
+      <c r="B15" s="88"/>
+      <c r="C15" s="86" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="83" t="s">
+      <c r="E15" s="90" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="87"/>
+      <c r="F15" s="84"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -5825,11 +5818,10 @@
       <c r="AT15" s="68"/>
       <c r="AU15" s="10"/>
       <c r="AV15" s="47"/>
-      <c r="AY15" s="8"/>
+      <c r="AY15" s="74"/>
       <c r="BA15" s="9"/>
       <c r="BB15" s="10"/>
       <c r="BC15" s="11"/>
-      <c r="BD15" s="8"/>
       <c r="BE15" s="8"/>
       <c r="BF15" s="8"/>
       <c r="BG15" s="8"/>
@@ -6002,14 +5994,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="79"/>
-      <c r="B16" s="79"/>
-      <c r="C16" s="79"/>
+      <c r="A16" s="85"/>
+      <c r="B16" s="85"/>
+      <c r="C16" s="85"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="79"/>
-      <c r="F16" s="79"/>
+      <c r="E16" s="85"/>
+      <c r="F16" s="85"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6051,11 +6043,10 @@
       <c r="AT16" s="68"/>
       <c r="AU16" s="10"/>
       <c r="AV16" s="47"/>
-      <c r="AY16" s="8"/>
+      <c r="AY16" s="74"/>
       <c r="BA16" s="9"/>
       <c r="BB16" s="10"/>
       <c r="BC16" s="11"/>
-      <c r="BD16" s="8"/>
       <c r="BE16" s="8"/>
       <c r="BF16" s="8"/>
       <c r="BG16" s="8"/>
@@ -6228,18 +6219,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="79"/>
-      <c r="B17" s="85"/>
-      <c r="C17" s="78" t="s">
+      <c r="A17" s="85"/>
+      <c r="B17" s="88"/>
+      <c r="C17" s="86" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="83" t="s">
+      <c r="E17" s="90" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="87"/>
+      <c r="F17" s="84"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6281,11 +6272,10 @@
       <c r="AT17" s="68"/>
       <c r="AU17" s="10"/>
       <c r="AV17" s="47"/>
-      <c r="AY17" s="8"/>
+      <c r="AY17" s="74"/>
       <c r="BA17" s="9"/>
       <c r="BB17" s="10"/>
       <c r="BC17" s="11"/>
-      <c r="BD17" s="8"/>
       <c r="BE17" s="8"/>
       <c r="BF17" s="8"/>
       <c r="BG17" s="8"/>
@@ -6458,14 +6448,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="79"/>
-      <c r="B18" s="79"/>
-      <c r="C18" s="79"/>
+      <c r="A18" s="85"/>
+      <c r="B18" s="85"/>
+      <c r="C18" s="85"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="79"/>
-      <c r="F18" s="79"/>
+      <c r="E18" s="85"/>
+      <c r="F18" s="85"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6507,11 +6497,10 @@
       <c r="AT18" s="68"/>
       <c r="AU18" s="10"/>
       <c r="AV18" s="47"/>
-      <c r="AY18" s="8"/>
+      <c r="AY18" s="74"/>
       <c r="BA18" s="9"/>
       <c r="BB18" s="10"/>
       <c r="BC18" s="11"/>
-      <c r="BD18" s="8"/>
       <c r="BE18" s="8"/>
       <c r="BF18" s="8"/>
       <c r="BG18" s="8"/>
@@ -6684,18 +6673,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="79"/>
-      <c r="B19" s="85"/>
-      <c r="C19" s="78" t="s">
+      <c r="A19" s="85"/>
+      <c r="B19" s="88"/>
+      <c r="C19" s="86" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="83" t="s">
+      <c r="E19" s="90" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="87"/>
+      <c r="F19" s="84"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6737,11 +6726,10 @@
       <c r="AT19" s="68"/>
       <c r="AU19" s="10"/>
       <c r="AV19" s="47"/>
-      <c r="AY19" s="8"/>
+      <c r="AY19" s="74"/>
       <c r="BA19" s="9"/>
       <c r="BB19" s="10"/>
       <c r="BC19" s="11"/>
-      <c r="BD19" s="8"/>
       <c r="BE19" s="8"/>
       <c r="BF19" s="8"/>
       <c r="BG19" s="8"/>
@@ -6914,14 +6902,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="79"/>
-      <c r="B20" s="79"/>
-      <c r="C20" s="79"/>
+      <c r="A20" s="85"/>
+      <c r="B20" s="85"/>
+      <c r="C20" s="85"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="79"/>
-      <c r="F20" s="79"/>
+      <c r="E20" s="85"/>
+      <c r="F20" s="85"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -6963,11 +6951,10 @@
       <c r="AT20" s="68"/>
       <c r="AU20" s="10"/>
       <c r="AV20" s="47"/>
-      <c r="AY20" s="8"/>
+      <c r="AY20" s="74"/>
       <c r="BA20" s="9"/>
       <c r="BB20" s="10"/>
       <c r="BC20" s="11"/>
-      <c r="BD20" s="8"/>
       <c r="BE20" s="8"/>
       <c r="BF20" s="8"/>
       <c r="BG20" s="8"/>
@@ -7140,18 +7127,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="79"/>
-      <c r="B21" s="85"/>
-      <c r="C21" s="78" t="s">
+      <c r="A21" s="85"/>
+      <c r="B21" s="88"/>
+      <c r="C21" s="86" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="83" t="s">
+      <c r="E21" s="90" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="87"/>
+      <c r="F21" s="84"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7193,11 +7180,10 @@
       <c r="AT21" s="68"/>
       <c r="AU21" s="10"/>
       <c r="AV21" s="47"/>
-      <c r="AY21" s="8"/>
+      <c r="AY21" s="74"/>
       <c r="BA21" s="9"/>
       <c r="BB21" s="10"/>
       <c r="BC21" s="11"/>
-      <c r="BD21" s="8"/>
       <c r="BE21" s="8"/>
       <c r="BF21" s="8"/>
       <c r="BG21" s="8"/>
@@ -7370,14 +7356,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="86"/>
-      <c r="B22" s="86"/>
-      <c r="C22" s="86"/>
+      <c r="A22" s="91"/>
+      <c r="B22" s="91"/>
+      <c r="C22" s="91"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="86"/>
-      <c r="F22" s="86"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="91"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7419,12 +7405,11 @@
       <c r="AT22" s="68"/>
       <c r="AU22" s="40"/>
       <c r="AV22" s="48"/>
-      <c r="AY22" s="38"/>
-      <c r="AZ22" s="69"/>
+      <c r="AY22" s="75"/>
       <c r="BA22" s="39"/>
       <c r="BB22" s="40"/>
       <c r="BC22" s="41"/>
-      <c r="BD22" s="38"/>
+      <c r="BD22" s="69"/>
       <c r="BE22" s="38"/>
       <c r="BF22" s="38"/>
       <c r="BG22" s="38"/>
@@ -7597,22 +7582,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="76" t="s">
+      <c r="A23" s="87" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="77" t="s">
+      <c r="C23" s="80" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="80" t="s">
+      <c r="E23" s="79" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="82" t="s">
+      <c r="F23" s="81" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7658,11 +7643,11 @@
       <c r="AU23" s="10"/>
       <c r="AV23" s="47"/>
       <c r="AW23" s="54"/>
-      <c r="AY23" s="8"/>
+      <c r="AY23" s="74"/>
       <c r="BA23" s="9"/>
       <c r="BB23" s="10"/>
       <c r="BC23" s="11"/>
-      <c r="BD23" s="16"/>
+      <c r="BD23" s="70"/>
       <c r="BE23" s="8"/>
       <c r="BF23" s="8"/>
       <c r="BG23" s="8"/>
@@ -7835,14 +7820,14 @@
       <c r="HR23" s="8"/>
     </row>
     <row r="24" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="75"/>
-      <c r="B24" s="75"/>
-      <c r="C24" s="75"/>
+      <c r="A24" s="77"/>
+      <c r="B24" s="77"/>
+      <c r="C24" s="77"/>
       <c r="D24" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="75"/>
-      <c r="F24" s="75"/>
+      <c r="E24" s="77"/>
+      <c r="F24" s="77"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
@@ -7886,11 +7871,11 @@
       <c r="AU24" s="10"/>
       <c r="AV24" s="47"/>
       <c r="AW24" s="56"/>
-      <c r="AY24" s="8"/>
+      <c r="AY24" s="74"/>
       <c r="BA24" s="9"/>
       <c r="BB24" s="10"/>
       <c r="BC24" s="11"/>
-      <c r="BD24" s="8"/>
+      <c r="BD24" s="72"/>
       <c r="BE24" s="8"/>
       <c r="BF24" s="8"/>
       <c r="BG24" s="8"/>
@@ -8063,20 +8048,20 @@
       <c r="HR24" s="8"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="75"/>
-      <c r="B25" s="81" t="s">
+      <c r="A25" s="77"/>
+      <c r="B25" s="78" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="77" t="s">
+      <c r="C25" s="80" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="80" t="s">
+      <c r="E25" s="79" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="82" t="s">
+      <c r="F25" s="81" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8117,7 +8102,7 @@
       <c r="AT25" s="68"/>
       <c r="AU25" s="10"/>
       <c r="AV25" s="47"/>
-      <c r="AY25" s="8"/>
+      <c r="AY25" s="74"/>
       <c r="BA25" s="9"/>
       <c r="BB25" s="10"/>
       <c r="BC25" s="11"/>
@@ -8290,14 +8275,14 @@
       <c r="HS25" s="8"/>
     </row>
     <row r="26" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="75"/>
-      <c r="B26" s="75"/>
-      <c r="C26" s="75"/>
+      <c r="A26" s="77"/>
+      <c r="B26" s="77"/>
+      <c r="C26" s="77"/>
       <c r="D26" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="75"/>
-      <c r="F26" s="75"/>
+      <c r="E26" s="77"/>
+      <c r="F26" s="77"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
@@ -8339,11 +8324,10 @@
       <c r="AT26" s="68"/>
       <c r="AU26" s="10"/>
       <c r="AV26" s="47"/>
-      <c r="AY26" s="8"/>
+      <c r="AY26" s="74"/>
       <c r="BA26" s="9"/>
       <c r="BB26" s="10"/>
       <c r="BC26" s="11"/>
-      <c r="BD26" s="8"/>
       <c r="BE26" s="8"/>
       <c r="BF26" s="8"/>
       <c r="BG26" s="8"/>
@@ -8516,20 +8500,20 @@
       <c r="HR26" s="8"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="75"/>
-      <c r="B27" s="81" t="s">
+      <c r="A27" s="77"/>
+      <c r="B27" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="88" t="s">
+      <c r="C27" s="89" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="80" t="s">
+      <c r="E27" s="79" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="82"/>
+      <c r="F27" s="81"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8570,12 +8554,11 @@
       <c r="AT27" s="68"/>
       <c r="AU27" s="10"/>
       <c r="AV27" s="47"/>
-      <c r="AY27" s="8"/>
-      <c r="AZ27" s="91"/>
+      <c r="AY27" s="74"/>
+      <c r="AZ27" s="93"/>
       <c r="BA27" s="9"/>
       <c r="BB27" s="10"/>
       <c r="BC27" s="11"/>
-      <c r="BD27" s="8"/>
       <c r="BE27" s="8"/>
       <c r="BF27" s="8"/>
       <c r="BG27" s="8"/>
@@ -8748,14 +8731,14 @@
       <c r="HR27" s="8"/>
     </row>
     <row r="28" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="75"/>
-      <c r="B28" s="75"/>
-      <c r="C28" s="75"/>
+      <c r="A28" s="77"/>
+      <c r="B28" s="77"/>
+      <c r="C28" s="77"/>
       <c r="D28" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="75"/>
-      <c r="F28" s="75"/>
+      <c r="E28" s="77"/>
+      <c r="F28" s="77"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
@@ -8796,12 +8779,11 @@
       <c r="AT28" s="68"/>
       <c r="AU28" s="10"/>
       <c r="AV28" s="47"/>
-      <c r="AY28" s="8"/>
-      <c r="AZ28" s="72"/>
+      <c r="AY28" s="74"/>
+      <c r="AZ28" s="56"/>
       <c r="BA28" s="9"/>
       <c r="BB28" s="10"/>
       <c r="BC28" s="11"/>
-      <c r="BD28" s="8"/>
       <c r="BE28" s="8"/>
       <c r="BF28" s="8"/>
       <c r="BG28" s="8"/>
@@ -8974,22 +8956,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="76" t="s">
+      <c r="A29" s="87" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="78" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="77" t="s">
+      <c r="C29" s="80" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="80" t="s">
+      <c r="E29" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="82" t="s">
+      <c r="F29" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9032,11 +9014,10 @@
       <c r="AT29" s="68"/>
       <c r="AU29" s="10"/>
       <c r="AV29" s="47"/>
-      <c r="AY29" s="8"/>
+      <c r="AY29" s="74"/>
       <c r="BA29" s="9"/>
       <c r="BB29" s="10"/>
       <c r="BC29" s="11"/>
-      <c r="BD29" s="8"/>
       <c r="BE29" s="8"/>
       <c r="BF29" s="8"/>
       <c r="BG29" s="8"/>
@@ -9209,14 +9190,14 @@
       <c r="HR29" s="8"/>
     </row>
     <row r="30" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="75"/>
-      <c r="B30" s="75"/>
-      <c r="C30" s="75"/>
+      <c r="A30" s="77"/>
+      <c r="B30" s="77"/>
+      <c r="C30" s="77"/>
       <c r="D30" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="75"/>
-      <c r="F30" s="75"/>
+      <c r="E30" s="77"/>
+      <c r="F30" s="77"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
@@ -9258,11 +9239,10 @@
       <c r="AT30" s="68"/>
       <c r="AU30" s="10"/>
       <c r="AV30" s="47"/>
-      <c r="AY30" s="8"/>
+      <c r="AY30" s="74"/>
       <c r="BA30" s="9"/>
       <c r="BB30" s="10"/>
       <c r="BC30" s="11"/>
-      <c r="BD30" s="8"/>
       <c r="BE30" s="8"/>
       <c r="BF30" s="8"/>
       <c r="BG30" s="8"/>
@@ -9435,20 +9415,20 @@
       <c r="HR30" s="8"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="75"/>
-      <c r="B31" s="81" t="s">
+      <c r="A31" s="77"/>
+      <c r="B31" s="78" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="77" t="s">
+      <c r="C31" s="80" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="80" t="s">
+      <c r="E31" s="79" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="82" t="s">
+      <c r="F31" s="81" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9492,11 +9472,10 @@
       <c r="AT31" s="68"/>
       <c r="AU31" s="10"/>
       <c r="AV31" s="47"/>
-      <c r="AY31" s="8"/>
+      <c r="AY31" s="74"/>
       <c r="BA31" s="9"/>
       <c r="BB31" s="10"/>
       <c r="BC31" s="11"/>
-      <c r="BD31" s="8"/>
       <c r="BE31" s="8"/>
       <c r="BF31" s="8"/>
       <c r="BG31" s="8"/>
@@ -9669,14 +9648,14 @@
       <c r="HR31" s="8"/>
     </row>
     <row r="32" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="75"/>
-      <c r="B32" s="75"/>
-      <c r="C32" s="75"/>
+      <c r="A32" s="77"/>
+      <c r="B32" s="77"/>
+      <c r="C32" s="77"/>
       <c r="D32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
+      <c r="E32" s="77"/>
+      <c r="F32" s="77"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="8"/>
@@ -9718,11 +9697,10 @@
       <c r="AT32" s="68"/>
       <c r="AU32" s="10"/>
       <c r="AV32" s="47"/>
-      <c r="AY32" s="8"/>
+      <c r="AY32" s="74"/>
       <c r="BA32" s="9"/>
       <c r="BB32" s="10"/>
       <c r="BC32" s="11"/>
-      <c r="BD32" s="8"/>
       <c r="BE32" s="8"/>
       <c r="BF32" s="8"/>
       <c r="BG32" s="8"/>
@@ -9895,20 +9873,20 @@
       <c r="HR32" s="8"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="75"/>
-      <c r="B33" s="81" t="s">
+      <c r="A33" s="77"/>
+      <c r="B33" s="78" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="80" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="80" t="s">
+      <c r="E33" s="79" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="82" t="s">
+      <c r="F33" s="81" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -9952,11 +9930,10 @@
       <c r="AT33" s="68"/>
       <c r="AU33" s="10"/>
       <c r="AV33" s="47"/>
-      <c r="AY33" s="16"/>
+      <c r="AY33" s="54"/>
       <c r="BA33" s="9"/>
       <c r="BB33" s="10"/>
       <c r="BC33" s="11"/>
-      <c r="BD33" s="8"/>
       <c r="BE33" s="8"/>
       <c r="BF33" s="8"/>
       <c r="BG33" s="8"/>
@@ -10129,14 +10106,14 @@
       <c r="HR33" s="8"/>
     </row>
     <row r="34" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="75"/>
-      <c r="B34" s="75"/>
-      <c r="C34" s="75"/>
+      <c r="A34" s="77"/>
+      <c r="B34" s="77"/>
+      <c r="C34" s="77"/>
       <c r="D34" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="75"/>
-      <c r="F34" s="75"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
@@ -10178,11 +10155,10 @@
       <c r="AT34" s="68"/>
       <c r="AU34" s="10"/>
       <c r="AV34" s="60"/>
-      <c r="AY34" s="8"/>
+      <c r="AY34" s="74"/>
       <c r="BA34" s="9"/>
       <c r="BB34" s="10"/>
       <c r="BC34" s="11"/>
-      <c r="BD34" s="8"/>
       <c r="BE34" s="8"/>
       <c r="BF34" s="8"/>
       <c r="BG34" s="8"/>
@@ -10355,20 +10331,20 @@
       <c r="HR34" s="8"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="75"/>
-      <c r="B35" s="81" t="s">
+      <c r="A35" s="77"/>
+      <c r="B35" s="78" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="80" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="80" t="s">
+      <c r="E35" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="82" t="s">
+      <c r="F35" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10412,11 +10388,10 @@
       <c r="AT35" s="68"/>
       <c r="AU35" s="10"/>
       <c r="AV35" s="47"/>
-      <c r="AY35" s="8"/>
+      <c r="AY35" s="74"/>
       <c r="BA35" s="9"/>
       <c r="BB35" s="10"/>
       <c r="BC35" s="11"/>
-      <c r="BD35" s="8"/>
       <c r="BE35" s="8"/>
       <c r="BF35" s="16"/>
       <c r="BG35" s="16"/>
@@ -10589,14 +10564,14 @@
       <c r="HR35" s="8"/>
     </row>
     <row r="36" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="75"/>
-      <c r="B36" s="75"/>
-      <c r="C36" s="75"/>
+      <c r="A36" s="77"/>
+      <c r="B36" s="77"/>
+      <c r="C36" s="77"/>
       <c r="D36" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="75"/>
-      <c r="F36" s="75"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
@@ -10638,11 +10613,10 @@
       <c r="AT36" s="68"/>
       <c r="AU36" s="10"/>
       <c r="AV36" s="47"/>
-      <c r="AY36" s="8"/>
+      <c r="AY36" s="74"/>
       <c r="BA36" s="9"/>
       <c r="BB36" s="10"/>
       <c r="BC36" s="11"/>
-      <c r="BD36" s="8"/>
       <c r="BE36" s="8"/>
       <c r="BF36" s="8"/>
       <c r="BG36" s="8"/>
@@ -10815,20 +10789,20 @@
       <c r="HR36" s="8"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="75"/>
-      <c r="B37" s="81" t="s">
+      <c r="A37" s="77"/>
+      <c r="B37" s="78" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="80" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="80" t="s">
+      <c r="E37" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="82" t="s">
+      <c r="F37" s="81" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -10872,11 +10846,10 @@
       <c r="AT37" s="68"/>
       <c r="AU37" s="10"/>
       <c r="AV37" s="47"/>
-      <c r="AY37" s="8"/>
+      <c r="AY37" s="74"/>
       <c r="BA37" s="9"/>
       <c r="BB37" s="10"/>
       <c r="BC37" s="11"/>
-      <c r="BD37" s="8"/>
       <c r="BE37" s="8"/>
       <c r="BF37" s="8"/>
       <c r="BG37" s="8"/>
@@ -11049,14 +11022,14 @@
       <c r="HR37" s="8"/>
     </row>
     <row r="38" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="75"/>
-      <c r="B38" s="75"/>
-      <c r="C38" s="75"/>
+      <c r="A38" s="77"/>
+      <c r="B38" s="77"/>
+      <c r="C38" s="77"/>
       <c r="D38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
@@ -11098,11 +11071,10 @@
       <c r="AT38" s="68"/>
       <c r="AU38" s="10"/>
       <c r="AV38" s="47"/>
-      <c r="AY38" s="8"/>
+      <c r="AY38" s="74"/>
       <c r="BA38" s="9"/>
       <c r="BB38" s="10"/>
       <c r="BC38" s="11"/>
-      <c r="BD38" s="8"/>
       <c r="BE38" s="8"/>
       <c r="BF38" s="8"/>
       <c r="BG38" s="8"/>
@@ -11275,20 +11247,20 @@
       <c r="HR38" s="8"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="75"/>
-      <c r="B39" s="81" t="s">
+      <c r="A39" s="77"/>
+      <c r="B39" s="78" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="80" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="80" t="s">
+      <c r="E39" s="79" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="82" t="s">
+      <c r="F39" s="81" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11332,11 +11304,10 @@
       <c r="AT39" s="68"/>
       <c r="AU39" s="10"/>
       <c r="AV39" s="47"/>
-      <c r="AY39" s="8"/>
+      <c r="AY39" s="74"/>
       <c r="BA39" s="9"/>
       <c r="BB39" s="10"/>
       <c r="BC39" s="11"/>
-      <c r="BD39" s="8"/>
       <c r="BE39" s="8"/>
       <c r="BF39" s="8"/>
       <c r="BG39" s="8"/>
@@ -11509,14 +11480,14 @@
       <c r="HR39" s="8"/>
     </row>
     <row r="40" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="75"/>
-      <c r="B40" s="75"/>
-      <c r="C40" s="75"/>
+      <c r="A40" s="77"/>
+      <c r="B40" s="77"/>
+      <c r="C40" s="77"/>
       <c r="D40" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="75"/>
-      <c r="F40" s="75"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
@@ -11558,12 +11529,11 @@
       <c r="AT40" s="68"/>
       <c r="AU40" s="10"/>
       <c r="AV40" s="47"/>
-      <c r="AY40" s="8"/>
-      <c r="AZ40" s="92"/>
+      <c r="AY40" s="74"/>
+      <c r="AZ40" s="60"/>
       <c r="BA40" s="9"/>
       <c r="BB40" s="10"/>
       <c r="BC40" s="11"/>
-      <c r="BD40" s="8"/>
       <c r="BE40" s="8"/>
       <c r="BF40" s="8"/>
       <c r="BG40" s="8"/>
@@ -11736,22 +11706,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="76" t="s">
+      <c r="A41" s="87" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="81" t="s">
+      <c r="B41" s="78" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="80" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="80" t="s">
+      <c r="E41" s="79" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="82" t="s">
+      <c r="F41" s="81" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -11795,11 +11765,10 @@
       <c r="AT41" s="68"/>
       <c r="AU41" s="10"/>
       <c r="AV41" s="47"/>
-      <c r="AY41" s="8"/>
+      <c r="AY41" s="74"/>
       <c r="BA41" s="9"/>
       <c r="BB41" s="10"/>
       <c r="BC41" s="11"/>
-      <c r="BD41" s="8"/>
       <c r="BE41" s="8"/>
       <c r="BF41" s="8"/>
       <c r="BG41" s="8"/>
@@ -11972,14 +11941,14 @@
       <c r="HR41" s="8"/>
     </row>
     <row r="42" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="75"/>
-      <c r="B42" s="75"/>
-      <c r="C42" s="75"/>
+      <c r="A42" s="77"/>
+      <c r="B42" s="77"/>
+      <c r="C42" s="77"/>
       <c r="D42" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="75"/>
-      <c r="F42" s="75"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="8"/>
@@ -12021,11 +11990,10 @@
       <c r="AT42" s="68"/>
       <c r="AU42" s="10"/>
       <c r="AV42" s="47"/>
-      <c r="AY42" s="8"/>
+      <c r="AY42" s="74"/>
       <c r="BA42" s="9"/>
       <c r="BB42" s="10"/>
       <c r="BC42" s="11"/>
-      <c r="BD42" s="8"/>
       <c r="BE42" s="8"/>
       <c r="BF42" s="8"/>
       <c r="BG42" s="8"/>
@@ -12198,20 +12166,20 @@
       <c r="HR42" s="8"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="75"/>
-      <c r="B43" s="81" t="s">
+      <c r="A43" s="77"/>
+      <c r="B43" s="78" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="80" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="80" t="s">
+      <c r="E43" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="82" t="s">
+      <c r="F43" s="81" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12254,11 +12222,10 @@
       <c r="AT43" s="68"/>
       <c r="AU43" s="10"/>
       <c r="AV43" s="47"/>
-      <c r="AY43" s="8"/>
+      <c r="AY43" s="74"/>
       <c r="BA43" s="9"/>
       <c r="BB43" s="10"/>
       <c r="BC43" s="11"/>
-      <c r="BD43" s="8"/>
       <c r="BE43" s="8"/>
       <c r="BF43" s="8"/>
       <c r="BG43" s="8"/>
@@ -12431,14 +12398,14 @@
       <c r="HR43" s="8"/>
     </row>
     <row r="44" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="75"/>
-      <c r="B44" s="75"/>
-      <c r="C44" s="75"/>
+      <c r="A44" s="77"/>
+      <c r="B44" s="77"/>
+      <c r="C44" s="77"/>
       <c r="D44" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="75"/>
-      <c r="F44" s="75"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="8"/>
@@ -12482,11 +12449,10 @@
       <c r="AU44" s="10"/>
       <c r="AV44" s="47"/>
       <c r="AX44" s="61"/>
-      <c r="AY44" s="8"/>
+      <c r="AY44" s="74"/>
       <c r="BA44" s="9"/>
       <c r="BB44" s="10"/>
       <c r="BC44" s="11"/>
-      <c r="BD44" s="8"/>
       <c r="BE44" s="8"/>
       <c r="BF44" s="8"/>
       <c r="BG44" s="8"/>
@@ -12659,20 +12625,20 @@
       <c r="HR44" s="8"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="75"/>
-      <c r="B45" s="81" t="s">
+      <c r="A45" s="77"/>
+      <c r="B45" s="78" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="77" t="s">
+      <c r="C45" s="80" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="80" t="s">
+      <c r="E45" s="79" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="82" t="s">
+      <c r="F45" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12716,11 +12682,10 @@
       <c r="AU45" s="10"/>
       <c r="AV45" s="47"/>
       <c r="AW45" s="52"/>
-      <c r="AY45" s="8"/>
+      <c r="AY45" s="74"/>
       <c r="BA45" s="9"/>
       <c r="BB45" s="10"/>
       <c r="BC45" s="11"/>
-      <c r="BD45" s="8"/>
       <c r="BE45" s="8"/>
       <c r="BF45" s="8"/>
       <c r="BG45" s="8"/>
@@ -12893,14 +12858,14 @@
       <c r="HR45" s="8"/>
     </row>
     <row r="46" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="75"/>
-      <c r="B46" s="75"/>
-      <c r="C46" s="75"/>
+      <c r="A46" s="77"/>
+      <c r="B46" s="77"/>
+      <c r="C46" s="77"/>
       <c r="D46" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="75"/>
-      <c r="F46" s="75"/>
+      <c r="E46" s="77"/>
+      <c r="F46" s="77"/>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="8"/>
@@ -12943,11 +12908,10 @@
       <c r="AU46" s="10"/>
       <c r="AV46" s="47"/>
       <c r="AW46" s="56"/>
-      <c r="AY46" s="8"/>
+      <c r="AY46" s="74"/>
       <c r="BA46" s="9"/>
       <c r="BB46" s="10"/>
       <c r="BC46" s="11"/>
-      <c r="BD46" s="8"/>
       <c r="BE46" s="8"/>
       <c r="BF46" s="8"/>
       <c r="BG46" s="8"/>
@@ -13120,22 +13084,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="76" t="s">
+      <c r="A47" s="87" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="81" t="s">
+      <c r="B47" s="78" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="77" t="s">
+      <c r="C47" s="80" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="80" t="s">
+      <c r="E47" s="79" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="82" t="s">
+      <c r="F47" s="81" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13180,12 +13144,12 @@
       <c r="AU47" s="10"/>
       <c r="AV47" s="47"/>
       <c r="AX47" s="52"/>
-      <c r="AY47" s="7"/>
-      <c r="AZ47" s="71"/>
+      <c r="AY47" s="52"/>
+      <c r="AZ47" s="52"/>
       <c r="BA47" s="9"/>
       <c r="BB47" s="10"/>
       <c r="BC47" s="11"/>
-      <c r="BD47" s="7"/>
+      <c r="BD47" s="71"/>
       <c r="BE47" s="7"/>
       <c r="BF47" s="8"/>
       <c r="BG47" s="8"/>
@@ -13358,14 +13322,14 @@
       <c r="HR47" s="8"/>
     </row>
     <row r="48" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="75"/>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
+      <c r="A48" s="77"/>
+      <c r="B48" s="77"/>
+      <c r="C48" s="77"/>
       <c r="D48" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="75"/>
-      <c r="F48" s="75"/>
+      <c r="E48" s="77"/>
+      <c r="F48" s="77"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
@@ -13407,12 +13371,12 @@
       <c r="AT48" s="68"/>
       <c r="AU48" s="10"/>
       <c r="AV48" s="47"/>
-      <c r="AY48" s="8"/>
-      <c r="AZ48" s="72"/>
+      <c r="AY48" s="74"/>
+      <c r="AZ48" s="56"/>
       <c r="BA48" s="9"/>
       <c r="BB48" s="10"/>
       <c r="BC48" s="11"/>
-      <c r="BD48" s="8"/>
+      <c r="BD48" s="72"/>
       <c r="BE48" s="8"/>
       <c r="BF48" s="8"/>
       <c r="BG48" s="8"/>
@@ -13585,20 +13549,20 @@
       <c r="HR48" s="8"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="75"/>
-      <c r="B49" s="81" t="s">
+      <c r="A49" s="77"/>
+      <c r="B49" s="78" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="77" t="s">
+      <c r="C49" s="80" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="80" t="s">
+      <c r="E49" s="79" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="82" t="s">
+      <c r="F49" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13642,11 +13606,10 @@
       <c r="AT49" s="68"/>
       <c r="AU49" s="10"/>
       <c r="AV49" s="47"/>
-      <c r="AY49" s="8"/>
+      <c r="AY49" s="74"/>
       <c r="BA49" s="9"/>
       <c r="BB49" s="10"/>
       <c r="BC49" s="11"/>
-      <c r="BD49" s="8"/>
       <c r="BE49" s="8"/>
       <c r="BF49" s="8"/>
       <c r="BG49" s="8"/>
@@ -13819,14 +13782,14 @@
       <c r="HR49" s="8"/>
     </row>
     <row r="50" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="75"/>
-      <c r="B50" s="75"/>
-      <c r="C50" s="75"/>
+      <c r="A50" s="77"/>
+      <c r="B50" s="77"/>
+      <c r="C50" s="77"/>
       <c r="D50" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="75"/>
-      <c r="F50" s="75"/>
+      <c r="E50" s="77"/>
+      <c r="F50" s="77"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
@@ -13868,11 +13831,10 @@
       <c r="AT50" s="68"/>
       <c r="AU50" s="10"/>
       <c r="AV50" s="47"/>
-      <c r="AY50" s="8"/>
+      <c r="AY50" s="74"/>
       <c r="BA50" s="9"/>
       <c r="BB50" s="10"/>
       <c r="BC50" s="11"/>
-      <c r="BD50" s="8"/>
       <c r="BE50" s="8"/>
       <c r="BF50" s="8"/>
       <c r="BG50" s="8"/>
@@ -14045,22 +14007,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="76" t="s">
+      <c r="A51" s="87" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="81" t="s">
+      <c r="B51" s="78" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="77" t="s">
+      <c r="C51" s="80" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="80" t="s">
+      <c r="E51" s="79" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="82" t="s">
+      <c r="F51" s="81" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14104,11 +14066,10 @@
       <c r="AT51" s="68"/>
       <c r="AU51" s="10"/>
       <c r="AV51" s="47"/>
-      <c r="AY51" s="8"/>
+      <c r="AY51" s="74"/>
       <c r="BA51" s="9"/>
       <c r="BB51" s="10"/>
       <c r="BC51" s="11"/>
-      <c r="BD51" s="8"/>
       <c r="BE51" s="8"/>
       <c r="BF51" s="8"/>
       <c r="BG51" s="8"/>
@@ -14281,14 +14242,14 @@
       <c r="HR51" s="8"/>
     </row>
     <row r="52" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="75"/>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
+      <c r="A52" s="77"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="77"/>
       <c r="D52" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="75"/>
-      <c r="F52" s="75"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="77"/>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="8"/>
@@ -14330,11 +14291,10 @@
       <c r="AT52" s="68"/>
       <c r="AU52" s="10"/>
       <c r="AV52" s="47"/>
-      <c r="AY52" s="8"/>
+      <c r="AY52" s="74"/>
       <c r="BA52" s="9"/>
       <c r="BB52" s="10"/>
       <c r="BC52" s="11"/>
-      <c r="BD52" s="8"/>
       <c r="BE52" s="8"/>
       <c r="BF52" s="8"/>
       <c r="BG52" s="8"/>
@@ -14507,20 +14467,20 @@
       <c r="HR52" s="8"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="75"/>
-      <c r="B53" s="81" t="s">
+      <c r="A53" s="77"/>
+      <c r="B53" s="78" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="77" t="s">
+      <c r="C53" s="80" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="80" t="s">
+      <c r="E53" s="79" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="82" t="s">
+      <c r="F53" s="81" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14564,11 +14524,10 @@
       <c r="AT53" s="68"/>
       <c r="AU53" s="10"/>
       <c r="AV53" s="47"/>
-      <c r="AY53" s="8"/>
+      <c r="AY53" s="74"/>
       <c r="BA53" s="9"/>
       <c r="BB53" s="10"/>
       <c r="BC53" s="11"/>
-      <c r="BD53" s="8"/>
       <c r="BE53" s="8"/>
       <c r="BF53" s="8"/>
       <c r="BG53" s="8"/>
@@ -14741,14 +14700,14 @@
       <c r="HR53" s="8"/>
     </row>
     <row r="54" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="75"/>
-      <c r="B54" s="75"/>
-      <c r="C54" s="75"/>
+      <c r="A54" s="77"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="77"/>
       <c r="D54" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="75"/>
-      <c r="F54" s="75"/>
+      <c r="E54" s="77"/>
+      <c r="F54" s="77"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
@@ -14790,11 +14749,10 @@
       <c r="AT54" s="68"/>
       <c r="AU54" s="10"/>
       <c r="AV54" s="47"/>
-      <c r="AY54" s="8"/>
+      <c r="AY54" s="74"/>
       <c r="BA54" s="9"/>
       <c r="BB54" s="10"/>
       <c r="BC54" s="11"/>
-      <c r="BD54" s="8"/>
       <c r="BE54" s="8"/>
       <c r="BF54" s="8"/>
       <c r="BG54" s="8"/>
@@ -14967,22 +14925,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="76" t="s">
+      <c r="A55" s="87" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="81" t="s">
+      <c r="B55" s="78" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="77" t="s">
+      <c r="C55" s="80" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="80" t="s">
+      <c r="E55" s="79" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="82" t="s">
+      <c r="F55" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -15026,11 +14984,10 @@
       <c r="AT55" s="68"/>
       <c r="AU55" s="10"/>
       <c r="AV55" s="47"/>
-      <c r="AY55" s="8"/>
+      <c r="AY55" s="74"/>
       <c r="BA55" s="9"/>
       <c r="BB55" s="10"/>
       <c r="BC55" s="11"/>
-      <c r="BD55" s="8"/>
       <c r="BE55" s="8"/>
       <c r="BF55" s="8"/>
       <c r="BG55" s="8"/>
@@ -15203,14 +15160,14 @@
       <c r="HR55" s="8"/>
     </row>
     <row r="56" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="75"/>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
+      <c r="A56" s="77"/>
+      <c r="B56" s="77"/>
+      <c r="C56" s="77"/>
       <c r="D56" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="75"/>
-      <c r="F56" s="75"/>
+      <c r="E56" s="77"/>
+      <c r="F56" s="77"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
@@ -15252,11 +15209,10 @@
       <c r="AT56" s="68"/>
       <c r="AU56" s="10"/>
       <c r="AV56" s="47"/>
-      <c r="AY56" s="8"/>
+      <c r="AY56" s="74"/>
       <c r="BA56" s="9"/>
       <c r="BB56" s="10"/>
       <c r="BC56" s="11"/>
-      <c r="BD56" s="8"/>
       <c r="BE56" s="8"/>
       <c r="BF56" s="8"/>
       <c r="BG56" s="8"/>
@@ -15429,20 +15385,20 @@
       <c r="HR56" s="8"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="75"/>
-      <c r="B57" s="81" t="s">
+      <c r="A57" s="77"/>
+      <c r="B57" s="78" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="77" t="s">
+      <c r="C57" s="80" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="80" t="s">
+      <c r="E57" s="79" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="82" t="s">
+      <c r="F57" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15486,11 +15442,10 @@
       <c r="AT57" s="68"/>
       <c r="AU57" s="10"/>
       <c r="AV57" s="47"/>
-      <c r="AY57" s="8"/>
+      <c r="AY57" s="74"/>
       <c r="BA57" s="9"/>
       <c r="BB57" s="10"/>
       <c r="BC57" s="11"/>
-      <c r="BD57" s="8"/>
       <c r="BE57" s="8"/>
       <c r="BF57" s="8"/>
       <c r="BG57" s="8"/>
@@ -15663,14 +15618,14 @@
       <c r="HR57" s="8"/>
     </row>
     <row r="58" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="75"/>
-      <c r="B58" s="75"/>
-      <c r="C58" s="75"/>
+      <c r="A58" s="77"/>
+      <c r="B58" s="77"/>
+      <c r="C58" s="77"/>
       <c r="D58" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="75"/>
-      <c r="F58" s="75"/>
+      <c r="E58" s="77"/>
+      <c r="F58" s="77"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
@@ -15712,11 +15667,10 @@
       <c r="AT58" s="68"/>
       <c r="AU58" s="10"/>
       <c r="AV58" s="47"/>
-      <c r="AY58" s="8"/>
+      <c r="AY58" s="74"/>
       <c r="BA58" s="9"/>
       <c r="BB58" s="10"/>
       <c r="BC58" s="11"/>
-      <c r="BD58" s="8"/>
       <c r="BE58" s="8"/>
       <c r="BF58" s="8"/>
       <c r="BG58" s="8"/>
@@ -15889,20 +15843,20 @@
       <c r="HR58" s="8"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="75"/>
-      <c r="B59" s="81" t="s">
+      <c r="A59" s="77"/>
+      <c r="B59" s="78" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="77" t="s">
+      <c r="C59" s="80" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="80" t="s">
+      <c r="E59" s="79" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="82" t="s">
+      <c r="F59" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -15946,11 +15900,10 @@
       <c r="AT59" s="68"/>
       <c r="AU59" s="10"/>
       <c r="AV59" s="47"/>
-      <c r="AY59" s="8"/>
+      <c r="AY59" s="74"/>
       <c r="BA59" s="9"/>
       <c r="BB59" s="10"/>
       <c r="BC59" s="11"/>
-      <c r="BD59" s="8"/>
       <c r="BE59" s="8"/>
       <c r="BF59" s="8"/>
       <c r="BG59" s="8"/>
@@ -16123,14 +16076,14 @@
       <c r="HR59" s="8"/>
     </row>
     <row r="60" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="75"/>
-      <c r="B60" s="75"/>
-      <c r="C60" s="75"/>
+      <c r="A60" s="77"/>
+      <c r="B60" s="77"/>
+      <c r="C60" s="77"/>
       <c r="D60" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="75"/>
-      <c r="F60" s="75"/>
+      <c r="E60" s="77"/>
+      <c r="F60" s="77"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
@@ -16172,11 +16125,10 @@
       <c r="AT60" s="68"/>
       <c r="AU60" s="10"/>
       <c r="AV60" s="47"/>
-      <c r="AY60" s="8"/>
+      <c r="AY60" s="74"/>
       <c r="BA60" s="9"/>
       <c r="BB60" s="10"/>
       <c r="BC60" s="11"/>
-      <c r="BD60" s="8"/>
       <c r="BE60" s="8"/>
       <c r="BF60" s="8"/>
       <c r="BG60" s="8"/>
@@ -16349,20 +16301,20 @@
       <c r="HR60" s="8"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="75"/>
-      <c r="B61" s="81" t="s">
+      <c r="A61" s="77"/>
+      <c r="B61" s="78" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="77" t="s">
+      <c r="C61" s="80" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="80" t="s">
+      <c r="E61" s="79" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="82" t="s">
+      <c r="F61" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16406,11 +16358,10 @@
       <c r="AT61" s="68"/>
       <c r="AU61" s="10"/>
       <c r="AV61" s="47"/>
-      <c r="AY61" s="8"/>
+      <c r="AY61" s="74"/>
       <c r="BA61" s="9"/>
       <c r="BB61" s="10"/>
       <c r="BC61" s="11"/>
-      <c r="BD61" s="8"/>
       <c r="BE61" s="8"/>
       <c r="BF61" s="8"/>
       <c r="BG61" s="8"/>
@@ -16583,14 +16534,14 @@
       <c r="HR61" s="8"/>
     </row>
     <row r="62" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="75"/>
-      <c r="B62" s="75"/>
-      <c r="C62" s="75"/>
+      <c r="A62" s="77"/>
+      <c r="B62" s="77"/>
+      <c r="C62" s="77"/>
       <c r="D62" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="75"/>
-      <c r="F62" s="75"/>
+      <c r="E62" s="77"/>
+      <c r="F62" s="77"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
       <c r="I62" s="8"/>
@@ -16632,11 +16583,10 @@
       <c r="AT62" s="68"/>
       <c r="AU62" s="10"/>
       <c r="AV62" s="47"/>
-      <c r="AY62" s="8"/>
+      <c r="AY62" s="74"/>
       <c r="BA62" s="9"/>
       <c r="BB62" s="10"/>
       <c r="BC62" s="11"/>
-      <c r="BD62" s="8"/>
       <c r="BE62" s="8"/>
       <c r="BF62" s="8"/>
       <c r="BG62" s="8"/>
@@ -16809,20 +16759,20 @@
       <c r="HR62" s="8"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="75"/>
-      <c r="B63" s="81" t="s">
+      <c r="A63" s="77"/>
+      <c r="B63" s="78" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="77" t="s">
+      <c r="C63" s="80" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="80" t="s">
+      <c r="E63" s="79" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="82" t="s">
+      <c r="F63" s="81" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -16866,11 +16816,10 @@
       <c r="AT63" s="68"/>
       <c r="AU63" s="10"/>
       <c r="AV63" s="47"/>
-      <c r="AY63" s="8"/>
+      <c r="AY63" s="74"/>
       <c r="BA63" s="9"/>
       <c r="BB63" s="10"/>
       <c r="BC63" s="11"/>
-      <c r="BD63" s="8"/>
       <c r="BE63" s="8"/>
       <c r="BF63" s="8"/>
       <c r="BG63" s="8"/>
@@ -17043,14 +16992,14 @@
       <c r="HR63" s="8"/>
     </row>
     <row r="64" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="75"/>
-      <c r="B64" s="75"/>
-      <c r="C64" s="75"/>
+      <c r="A64" s="77"/>
+      <c r="B64" s="77"/>
+      <c r="C64" s="77"/>
       <c r="D64" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="75"/>
-      <c r="F64" s="75"/>
+      <c r="E64" s="77"/>
+      <c r="F64" s="77"/>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
@@ -17092,11 +17041,10 @@
       <c r="AT64" s="68"/>
       <c r="AU64" s="10"/>
       <c r="AV64" s="47"/>
-      <c r="AY64" s="8"/>
+      <c r="AY64" s="74"/>
       <c r="BA64" s="9"/>
       <c r="BB64" s="10"/>
       <c r="BC64" s="11"/>
-      <c r="BD64" s="8"/>
       <c r="BE64" s="8"/>
       <c r="BF64" s="8"/>
       <c r="BG64" s="8"/>
@@ -17269,20 +17217,20 @@
       <c r="HR64" s="8"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="75"/>
-      <c r="B65" s="81" t="s">
+      <c r="A65" s="77"/>
+      <c r="B65" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="77" t="s">
+      <c r="C65" s="80" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="80" t="s">
+      <c r="E65" s="79" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="82" t="s">
+      <c r="F65" s="81" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17326,11 +17274,10 @@
       <c r="AT65" s="68"/>
       <c r="AU65" s="10"/>
       <c r="AV65" s="47"/>
-      <c r="AY65" s="8"/>
+      <c r="AY65" s="74"/>
       <c r="BA65" s="9"/>
       <c r="BB65" s="10"/>
       <c r="BC65" s="11"/>
-      <c r="BD65" s="8"/>
       <c r="BE65" s="8"/>
       <c r="BF65" s="8"/>
       <c r="BG65" s="8"/>
@@ -17503,14 +17450,14 @@
       <c r="HR65" s="8"/>
     </row>
     <row r="66" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="75"/>
-      <c r="B66" s="75"/>
-      <c r="C66" s="75"/>
+      <c r="A66" s="77"/>
+      <c r="B66" s="77"/>
+      <c r="C66" s="77"/>
       <c r="D66" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="75"/>
-      <c r="F66" s="75"/>
+      <c r="E66" s="77"/>
+      <c r="F66" s="77"/>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
@@ -17552,11 +17499,10 @@
       <c r="AT66" s="68"/>
       <c r="AU66" s="10"/>
       <c r="AV66" s="47"/>
-      <c r="AY66" s="8"/>
+      <c r="AY66" s="74"/>
       <c r="BA66" s="9"/>
       <c r="BB66" s="10"/>
       <c r="BC66" s="11"/>
-      <c r="BD66" s="8"/>
       <c r="BE66" s="8"/>
       <c r="BF66" s="8"/>
       <c r="BG66" s="8"/>
@@ -17729,22 +17675,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="76" t="s">
+      <c r="A67" s="87" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="81" t="s">
+      <c r="B67" s="78" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="77" t="s">
+      <c r="C67" s="80" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="80" t="s">
+      <c r="E67" s="79" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="82" t="s">
+      <c r="F67" s="81" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -17788,11 +17734,10 @@
       <c r="AT67" s="68"/>
       <c r="AU67" s="10"/>
       <c r="AV67" s="47"/>
-      <c r="AY67" s="8"/>
+      <c r="AY67" s="74"/>
       <c r="BA67" s="9"/>
       <c r="BB67" s="10"/>
       <c r="BC67" s="11"/>
-      <c r="BD67" s="8"/>
       <c r="BE67" s="8"/>
       <c r="BF67" s="8"/>
       <c r="BG67" s="8"/>
@@ -17965,14 +17910,14 @@
       <c r="HR67" s="8"/>
     </row>
     <row r="68" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="75"/>
-      <c r="B68" s="75"/>
-      <c r="C68" s="75"/>
+      <c r="A68" s="77"/>
+      <c r="B68" s="77"/>
+      <c r="C68" s="77"/>
       <c r="D68" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="75"/>
-      <c r="F68" s="75"/>
+      <c r="E68" s="77"/>
+      <c r="F68" s="77"/>
       <c r="G68" s="8"/>
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
@@ -18015,11 +17960,10 @@
       <c r="AU68" s="10"/>
       <c r="AV68" s="47"/>
       <c r="AW68" s="61"/>
-      <c r="AY68" s="8"/>
+      <c r="AY68" s="74"/>
       <c r="BA68" s="9"/>
       <c r="BB68" s="10"/>
       <c r="BC68" s="11"/>
-      <c r="BD68" s="8"/>
       <c r="BE68" s="8"/>
       <c r="BF68" s="8"/>
       <c r="BG68" s="8"/>
@@ -18192,20 +18136,20 @@
       <c r="HR68" s="8"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="75"/>
-      <c r="B69" s="81" t="s">
+      <c r="A69" s="77"/>
+      <c r="B69" s="78" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="77" t="s">
+      <c r="C69" s="80" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="80" t="s">
+      <c r="E69" s="79" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="82" t="s">
+      <c r="F69" s="81" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18252,12 +18196,12 @@
       <c r="AV69" s="47"/>
       <c r="AW69" s="54"/>
       <c r="AX69" s="54"/>
-      <c r="AY69" s="16"/>
-      <c r="AZ69" s="70"/>
+      <c r="AY69" s="54"/>
+      <c r="AZ69" s="54"/>
       <c r="BA69" s="9"/>
       <c r="BB69" s="10"/>
       <c r="BC69" s="11"/>
-      <c r="BD69" s="16"/>
+      <c r="BD69" s="70"/>
       <c r="BE69" s="16"/>
       <c r="BF69" s="16"/>
       <c r="BG69" s="16"/>
@@ -18430,14 +18374,14 @@
       <c r="HR69" s="8"/>
     </row>
     <row r="70" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="75"/>
-      <c r="B70" s="75"/>
-      <c r="C70" s="75"/>
+      <c r="A70" s="77"/>
+      <c r="B70" s="77"/>
+      <c r="C70" s="77"/>
       <c r="D70" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="75"/>
-      <c r="F70" s="75"/>
+      <c r="E70" s="77"/>
+      <c r="F70" s="77"/>
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
       <c r="I70" s="8"/>
@@ -18481,11 +18425,11 @@
       <c r="AV70" s="47"/>
       <c r="AW70" s="56"/>
       <c r="AX70" s="56"/>
-      <c r="AY70" s="8"/>
+      <c r="AY70" s="74"/>
       <c r="BA70" s="9"/>
       <c r="BB70" s="10"/>
       <c r="BC70" s="11"/>
-      <c r="BD70" s="8"/>
+      <c r="BD70" s="72"/>
       <c r="BE70" s="8"/>
       <c r="BF70" s="8"/>
       <c r="BG70" s="8"/>
@@ -18658,20 +18602,20 @@
       <c r="HR70" s="8"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="75"/>
-      <c r="B71" s="81" t="s">
+      <c r="A71" s="77"/>
+      <c r="B71" s="78" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="77" t="s">
+      <c r="C71" s="80" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="80" t="s">
+      <c r="E71" s="79" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="82" t="s">
+      <c r="F71" s="81" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -18715,11 +18659,10 @@
       <c r="AT71" s="68"/>
       <c r="AU71" s="10"/>
       <c r="AV71" s="47"/>
-      <c r="AY71" s="8"/>
+      <c r="AY71" s="74"/>
       <c r="BA71" s="9"/>
       <c r="BB71" s="10"/>
       <c r="BC71" s="11"/>
-      <c r="BD71" s="8"/>
       <c r="BE71" s="8"/>
       <c r="BF71" s="8"/>
       <c r="BG71" s="8"/>
@@ -18892,14 +18835,14 @@
       <c r="HR71" s="8"/>
     </row>
     <row r="72" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="75"/>
-      <c r="B72" s="75"/>
-      <c r="C72" s="75"/>
+      <c r="A72" s="77"/>
+      <c r="B72" s="77"/>
+      <c r="C72" s="77"/>
       <c r="D72" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="75"/>
-      <c r="F72" s="75"/>
+      <c r="E72" s="77"/>
+      <c r="F72" s="77"/>
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
@@ -18941,11 +18884,10 @@
       <c r="AT72" s="68"/>
       <c r="AU72" s="10"/>
       <c r="AV72" s="47"/>
-      <c r="AY72" s="8"/>
+      <c r="AY72" s="74"/>
       <c r="BA72" s="9"/>
       <c r="BB72" s="10"/>
       <c r="BC72" s="11"/>
-      <c r="BD72" s="8"/>
       <c r="BE72" s="8"/>
       <c r="BF72" s="8"/>
       <c r="BG72" s="8"/>
@@ -19118,20 +19060,20 @@
       <c r="HR72" s="8"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="75"/>
-      <c r="B73" s="81" t="s">
+      <c r="A73" s="77"/>
+      <c r="B73" s="78" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="77" t="s">
+      <c r="C73" s="80" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="80" t="s">
+      <c r="E73" s="79" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="82" t="s">
+      <c r="F73" s="81" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19175,11 +19117,10 @@
       <c r="AT73" s="68"/>
       <c r="AU73" s="10"/>
       <c r="AV73" s="47"/>
-      <c r="AY73" s="8"/>
+      <c r="AY73" s="74"/>
       <c r="BA73" s="9"/>
       <c r="BB73" s="10"/>
       <c r="BC73" s="11"/>
-      <c r="BD73" s="8"/>
       <c r="BE73" s="8"/>
       <c r="BF73" s="8"/>
       <c r="BG73" s="8"/>
@@ -19352,14 +19293,14 @@
       <c r="HR73" s="8"/>
     </row>
     <row r="74" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="75"/>
-      <c r="B74" s="75"/>
-      <c r="C74" s="75"/>
+      <c r="A74" s="77"/>
+      <c r="B74" s="77"/>
+      <c r="C74" s="77"/>
       <c r="D74" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="75"/>
-      <c r="F74" s="75"/>
+      <c r="E74" s="77"/>
+      <c r="F74" s="77"/>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>
@@ -19401,11 +19342,10 @@
       <c r="AT74" s="68"/>
       <c r="AU74" s="10"/>
       <c r="AV74" s="47"/>
-      <c r="AY74" s="8"/>
+      <c r="AY74" s="74"/>
       <c r="BA74" s="9"/>
       <c r="BB74" s="10"/>
       <c r="BC74" s="11"/>
-      <c r="BD74" s="8"/>
       <c r="BE74" s="8"/>
       <c r="BF74" s="8"/>
       <c r="BG74" s="8"/>
@@ -19578,20 +19518,20 @@
       <c r="HR74" s="8"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="75"/>
-      <c r="B75" s="81" t="s">
+      <c r="A75" s="77"/>
+      <c r="B75" s="78" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="77" t="s">
+      <c r="C75" s="80" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="80" t="s">
+      <c r="E75" s="79" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="82" t="s">
+      <c r="F75" s="81" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19635,11 +19575,10 @@
       <c r="AT75" s="68"/>
       <c r="AU75" s="10"/>
       <c r="AV75" s="47"/>
-      <c r="AY75" s="8"/>
+      <c r="AY75" s="74"/>
       <c r="BA75" s="9"/>
       <c r="BB75" s="10"/>
       <c r="BC75" s="11"/>
-      <c r="BD75" s="8"/>
       <c r="BE75" s="8"/>
       <c r="BF75" s="8"/>
       <c r="BG75" s="8"/>
@@ -19812,14 +19751,14 @@
       <c r="HR75" s="8"/>
     </row>
     <row r="76" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="75"/>
-      <c r="B76" s="75"/>
-      <c r="C76" s="75"/>
+      <c r="A76" s="77"/>
+      <c r="B76" s="77"/>
+      <c r="C76" s="77"/>
       <c r="D76" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="75"/>
-      <c r="F76" s="75"/>
+      <c r="E76" s="77"/>
+      <c r="F76" s="77"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
       <c r="I76" s="8"/>
@@ -19861,11 +19800,10 @@
       <c r="AT76" s="68"/>
       <c r="AU76" s="10"/>
       <c r="AV76" s="47"/>
-      <c r="AY76" s="8"/>
+      <c r="AY76" s="74"/>
       <c r="BA76" s="9"/>
       <c r="BB76" s="10"/>
       <c r="BC76" s="11"/>
-      <c r="BD76" s="8"/>
       <c r="BE76" s="8"/>
       <c r="BF76" s="8"/>
       <c r="BG76" s="8"/>
@@ -20038,20 +19976,20 @@
       <c r="HR76" s="8"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="75"/>
-      <c r="B77" s="81" t="s">
+      <c r="A77" s="77"/>
+      <c r="B77" s="78" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="77" t="s">
+      <c r="C77" s="80" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="80" t="s">
+      <c r="E77" s="79" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="82" t="s">
+      <c r="F77" s="81" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20095,11 +20033,10 @@
       <c r="AT77" s="68"/>
       <c r="AU77" s="10"/>
       <c r="AV77" s="47"/>
-      <c r="AY77" s="8"/>
+      <c r="AY77" s="74"/>
       <c r="BA77" s="9"/>
       <c r="BB77" s="10"/>
       <c r="BC77" s="11"/>
-      <c r="BD77" s="8"/>
       <c r="BE77" s="8"/>
       <c r="BF77" s="8"/>
       <c r="BG77" s="8"/>
@@ -20272,14 +20209,14 @@
       <c r="HR77" s="8"/>
     </row>
     <row r="78" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="75"/>
-      <c r="B78" s="75"/>
-      <c r="C78" s="75"/>
+      <c r="A78" s="77"/>
+      <c r="B78" s="77"/>
+      <c r="C78" s="77"/>
       <c r="D78" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="75"/>
-      <c r="F78" s="75"/>
+      <c r="E78" s="77"/>
+      <c r="F78" s="77"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
       <c r="I78" s="8"/>
@@ -20321,11 +20258,10 @@
       <c r="AT78" s="68"/>
       <c r="AU78" s="10"/>
       <c r="AV78" s="47"/>
-      <c r="AY78" s="8"/>
+      <c r="AY78" s="74"/>
       <c r="BA78" s="9"/>
       <c r="BB78" s="10"/>
       <c r="BC78" s="11"/>
-      <c r="BD78" s="8"/>
       <c r="BE78" s="8"/>
       <c r="BF78" s="8"/>
       <c r="BG78" s="8"/>
@@ -20498,22 +20434,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="76" t="s">
+      <c r="A79" s="87" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="81" t="s">
+      <c r="B79" s="78" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="84" t="s">
+      <c r="C79" s="76" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="80" t="s">
+      <c r="E79" s="79" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="82" t="s">
+      <c r="F79" s="81" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20557,11 +20493,10 @@
       <c r="AT79" s="68"/>
       <c r="AU79" s="10"/>
       <c r="AV79" s="47"/>
-      <c r="AY79" s="8"/>
+      <c r="AY79" s="74"/>
       <c r="BA79" s="9"/>
       <c r="BB79" s="10"/>
       <c r="BC79" s="11"/>
-      <c r="BD79" s="8"/>
       <c r="BE79" s="8"/>
       <c r="BF79" s="8"/>
       <c r="BG79" s="8"/>
@@ -20734,14 +20669,14 @@
       <c r="HR79" s="8"/>
     </row>
     <row r="80" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="75"/>
-      <c r="B80" s="75"/>
-      <c r="C80" s="75"/>
+      <c r="A80" s="77"/>
+      <c r="B80" s="77"/>
+      <c r="C80" s="77"/>
       <c r="D80" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="75"/>
-      <c r="F80" s="75"/>
+      <c r="E80" s="77"/>
+      <c r="F80" s="77"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
       <c r="I80" s="8"/>
@@ -20783,11 +20718,10 @@
       <c r="AT80" s="68"/>
       <c r="AU80" s="10"/>
       <c r="AV80" s="47"/>
-      <c r="AY80" s="8"/>
+      <c r="AY80" s="74"/>
       <c r="BA80" s="9"/>
       <c r="BB80" s="10"/>
       <c r="BC80" s="11"/>
-      <c r="BD80" s="8"/>
       <c r="BE80" s="8"/>
       <c r="BF80" s="8"/>
       <c r="BG80" s="8"/>
@@ -20960,20 +20894,20 @@
       <c r="HR80" s="8"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="75"/>
-      <c r="B81" s="81" t="s">
+      <c r="A81" s="77"/>
+      <c r="B81" s="78" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="84" t="s">
+      <c r="C81" s="76" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="80" t="s">
+      <c r="E81" s="79" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="82" t="s">
+      <c r="F81" s="81" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -21017,11 +20951,10 @@
       <c r="AT81" s="68"/>
       <c r="AU81" s="10"/>
       <c r="AV81" s="47"/>
-      <c r="AY81" s="8"/>
+      <c r="AY81" s="74"/>
       <c r="BA81" s="9"/>
       <c r="BB81" s="10"/>
       <c r="BC81" s="11"/>
-      <c r="BD81" s="8"/>
       <c r="BE81" s="8"/>
       <c r="BF81" s="8"/>
       <c r="BG81" s="8"/>
@@ -21194,14 +21127,14 @@
       <c r="HR81" s="8"/>
     </row>
     <row r="82" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="75"/>
-      <c r="B82" s="75"/>
-      <c r="C82" s="75"/>
+      <c r="A82" s="77"/>
+      <c r="B82" s="77"/>
+      <c r="C82" s="77"/>
       <c r="D82" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="75"/>
-      <c r="F82" s="75"/>
+      <c r="E82" s="77"/>
+      <c r="F82" s="77"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
       <c r="I82" s="8"/>
@@ -21243,11 +21176,10 @@
       <c r="AT82" s="68"/>
       <c r="AU82" s="10"/>
       <c r="AV82" s="47"/>
-      <c r="AY82" s="8"/>
+      <c r="AY82" s="74"/>
       <c r="BA82" s="9"/>
       <c r="BB82" s="10"/>
       <c r="BC82" s="11"/>
-      <c r="BD82" s="8"/>
       <c r="BE82" s="8"/>
       <c r="BF82" s="8"/>
       <c r="BG82" s="8"/>
@@ -21420,20 +21352,20 @@
       <c r="HR82" s="8"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="75"/>
-      <c r="B83" s="81" t="s">
+      <c r="A83" s="77"/>
+      <c r="B83" s="78" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="77" t="s">
+      <c r="C83" s="80" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="80" t="s">
+      <c r="E83" s="79" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="82" t="s">
+      <c r="F83" s="81" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21477,11 +21409,10 @@
       <c r="AT83" s="68"/>
       <c r="AU83" s="10"/>
       <c r="AV83" s="47"/>
-      <c r="AY83" s="8"/>
+      <c r="AY83" s="74"/>
       <c r="BA83" s="9"/>
       <c r="BB83" s="10"/>
       <c r="BC83" s="11"/>
-      <c r="BD83" s="8"/>
       <c r="BE83" s="8"/>
       <c r="BF83" s="8"/>
       <c r="BG83" s="8"/>
@@ -21654,14 +21585,14 @@
       <c r="HR83" s="8"/>
     </row>
     <row r="84" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="75"/>
-      <c r="B84" s="75"/>
-      <c r="C84" s="75"/>
+      <c r="A84" s="77"/>
+      <c r="B84" s="77"/>
+      <c r="C84" s="77"/>
       <c r="D84" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="75"/>
-      <c r="F84" s="75"/>
+      <c r="E84" s="77"/>
+      <c r="F84" s="77"/>
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
@@ -21703,11 +21634,10 @@
       <c r="AT84" s="68"/>
       <c r="AU84" s="10"/>
       <c r="AV84" s="47"/>
-      <c r="AY84" s="8"/>
+      <c r="AY84" s="74"/>
       <c r="BA84" s="9"/>
       <c r="BB84" s="10"/>
       <c r="BC84" s="11"/>
-      <c r="BD84" s="8"/>
       <c r="BE84" s="8"/>
       <c r="BF84" s="8"/>
       <c r="BG84" s="8"/>
@@ -21880,20 +21810,20 @@
       <c r="HR84" s="8"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="75"/>
-      <c r="B85" s="81" t="s">
+      <c r="A85" s="77"/>
+      <c r="B85" s="78" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="88" t="s">
+      <c r="C85" s="89" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="80" t="s">
+      <c r="E85" s="79" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="82"/>
+      <c r="F85" s="81"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -21935,11 +21865,10 @@
       <c r="AT85" s="68"/>
       <c r="AU85" s="10"/>
       <c r="AV85" s="47"/>
-      <c r="AY85" s="8"/>
+      <c r="AY85" s="74"/>
       <c r="BA85" s="9"/>
       <c r="BB85" s="10"/>
       <c r="BC85" s="11"/>
-      <c r="BD85" s="8"/>
       <c r="BE85" s="8"/>
       <c r="BF85" s="8"/>
       <c r="BG85" s="8"/>
@@ -22112,14 +22041,14 @@
       <c r="HR85" s="17"/>
     </row>
     <row r="86" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="75"/>
-      <c r="B86" s="75"/>
-      <c r="C86" s="75"/>
+      <c r="A86" s="77"/>
+      <c r="B86" s="77"/>
+      <c r="C86" s="77"/>
       <c r="D86" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="75"/>
-      <c r="F86" s="75"/>
+      <c r="E86" s="77"/>
+      <c r="F86" s="77"/>
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
       <c r="I86" s="8"/>
@@ -22161,11 +22090,10 @@
       <c r="AT86" s="68"/>
       <c r="AU86" s="10"/>
       <c r="AV86" s="47"/>
-      <c r="AY86" s="8"/>
+      <c r="AY86" s="74"/>
       <c r="BA86" s="9"/>
       <c r="BB86" s="10"/>
       <c r="BC86" s="11"/>
-      <c r="BD86" s="8"/>
       <c r="BE86" s="8"/>
       <c r="BF86" s="8"/>
       <c r="BG86" s="8"/>
@@ -22339,6 +22267,187 @@
     </row>
   </sheetData>
   <mergeCells count="205">
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
     <mergeCell ref="C79:C80"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="E79:E80"/>
@@ -22363,187 +22472,6 @@
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="AP1:AV1"/>
     <mergeCell ref="E59:E60"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
datengenerator smoke_train getestet. funtkioniert. Nur FNO lernt fälschlicherweise rho exakt auf phi in jede raumrichtung abzubilden.
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752CAFCF-9827-4CC8-BC47-8E2F67B42E6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D48EBAF-6A00-4D1A-9EF1-CD2984DB2244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
@@ -1147,7 +1147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1259,57 +1259,56 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1627,19 +1626,21 @@
     <col min="46" max="46" width="2.140625" style="58" customWidth="1"/>
     <col min="47" max="48" width="2.140625" customWidth="1"/>
     <col min="49" max="49" width="2.140625" style="67" customWidth="1"/>
-    <col min="50" max="50" width="2.140625" style="73" customWidth="1"/>
+    <col min="50" max="50" width="2.140625" style="71" customWidth="1"/>
     <col min="51" max="51" width="2.140625" customWidth="1"/>
-    <col min="52" max="52" width="2.140625" style="74" customWidth="1"/>
+    <col min="52" max="52" width="2.140625" style="72" customWidth="1"/>
     <col min="53" max="55" width="2.140625" customWidth="1"/>
-    <col min="56" max="56" width="2.140625" style="66" customWidth="1"/>
-    <col min="57" max="226" width="2.140625" customWidth="1"/>
+    <col min="56" max="56" width="2.140625" style="74" customWidth="1"/>
+    <col min="57" max="57" width="2.140625" customWidth="1"/>
+    <col min="58" max="58" width="2.140625" style="66" customWidth="1"/>
+    <col min="59" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="82" t="s">
+      <c r="G1" s="76" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="77"/>
@@ -1648,7 +1649,7 @@
       <c r="K1" s="77"/>
       <c r="L1" s="77"/>
       <c r="M1" s="77"/>
-      <c r="N1" s="82" t="s">
+      <c r="N1" s="76" t="s">
         <v>2</v>
       </c>
       <c r="O1" s="77"/>
@@ -1657,7 +1658,7 @@
       <c r="R1" s="77"/>
       <c r="S1" s="77"/>
       <c r="T1" s="77"/>
-      <c r="U1" s="82" t="s">
+      <c r="U1" s="76" t="s">
         <v>3</v>
       </c>
       <c r="V1" s="77"/>
@@ -1666,7 +1667,7 @@
       <c r="Y1" s="77"/>
       <c r="Z1" s="77"/>
       <c r="AA1" s="77"/>
-      <c r="AB1" s="83" t="s">
+      <c r="AB1" s="92" t="s">
         <v>4</v>
       </c>
       <c r="AC1" s="77"/>
@@ -1675,7 +1676,7 @@
       <c r="AF1" s="77"/>
       <c r="AG1" s="77"/>
       <c r="AH1" s="77"/>
-      <c r="AI1" s="82" t="s">
+      <c r="AI1" s="76" t="s">
         <v>5</v>
       </c>
       <c r="AJ1" s="77"/>
@@ -1684,7 +1685,7 @@
       <c r="AM1" s="77"/>
       <c r="AN1" s="77"/>
       <c r="AO1" s="77"/>
-      <c r="AP1" s="82" t="s">
+      <c r="AP1" s="76" t="s">
         <v>6</v>
       </c>
       <c r="AQ1" s="77"/>
@@ -1693,7 +1694,7 @@
       <c r="AT1" s="77"/>
       <c r="AU1" s="77"/>
       <c r="AV1" s="77"/>
-      <c r="AW1" s="82" t="s">
+      <c r="AW1" s="76" t="s">
         <v>7</v>
       </c>
       <c r="AX1" s="77"/>
@@ -1702,7 +1703,7 @@
       <c r="BA1" s="77"/>
       <c r="BB1" s="77"/>
       <c r="BC1" s="77"/>
-      <c r="BD1" s="82" t="s">
+      <c r="BD1" s="76" t="s">
         <v>8</v>
       </c>
       <c r="BE1" s="77"/>
@@ -1711,7 +1712,7 @@
       <c r="BH1" s="77"/>
       <c r="BI1" s="77"/>
       <c r="BJ1" s="77"/>
-      <c r="BK1" s="82" t="s">
+      <c r="BK1" s="76" t="s">
         <v>9</v>
       </c>
       <c r="BL1" s="77"/>
@@ -1720,7 +1721,7 @@
       <c r="BO1" s="77"/>
       <c r="BP1" s="77"/>
       <c r="BQ1" s="77"/>
-      <c r="BR1" s="82" t="s">
+      <c r="BR1" s="76" t="s">
         <v>10</v>
       </c>
       <c r="BS1" s="77"/>
@@ -1729,7 +1730,7 @@
       <c r="BV1" s="77"/>
       <c r="BW1" s="77"/>
       <c r="BX1" s="77"/>
-      <c r="BY1" s="82" t="s">
+      <c r="BY1" s="76" t="s">
         <v>11</v>
       </c>
       <c r="BZ1" s="77"/>
@@ -1738,7 +1739,7 @@
       <c r="CC1" s="77"/>
       <c r="CD1" s="77"/>
       <c r="CE1" s="77"/>
-      <c r="CF1" s="82" t="s">
+      <c r="CF1" s="76" t="s">
         <v>12</v>
       </c>
       <c r="CG1" s="77"/>
@@ -1747,7 +1748,7 @@
       <c r="CJ1" s="77"/>
       <c r="CK1" s="77"/>
       <c r="CL1" s="77"/>
-      <c r="CM1" s="82" t="s">
+      <c r="CM1" s="76" t="s">
         <v>13</v>
       </c>
       <c r="CN1" s="77"/>
@@ -1756,7 +1757,7 @@
       <c r="CQ1" s="77"/>
       <c r="CR1" s="77"/>
       <c r="CS1" s="77"/>
-      <c r="CT1" s="82" t="s">
+      <c r="CT1" s="76" t="s">
         <v>14</v>
       </c>
       <c r="CU1" s="77"/>
@@ -1765,7 +1766,7 @@
       <c r="CX1" s="77"/>
       <c r="CY1" s="77"/>
       <c r="CZ1" s="77"/>
-      <c r="DA1" s="82" t="s">
+      <c r="DA1" s="76" t="s">
         <v>15</v>
       </c>
       <c r="DB1" s="77"/>
@@ -1774,7 +1775,7 @@
       <c r="DE1" s="77"/>
       <c r="DF1" s="77"/>
       <c r="DG1" s="77"/>
-      <c r="DH1" s="82" t="s">
+      <c r="DH1" s="76" t="s">
         <v>16</v>
       </c>
       <c r="DI1" s="77"/>
@@ -1783,7 +1784,7 @@
       <c r="DL1" s="77"/>
       <c r="DM1" s="77"/>
       <c r="DN1" s="77"/>
-      <c r="DO1" s="82" t="s">
+      <c r="DO1" s="76" t="s">
         <v>17</v>
       </c>
       <c r="DP1" s="77"/>
@@ -1792,7 +1793,7 @@
       <c r="DS1" s="77"/>
       <c r="DT1" s="77"/>
       <c r="DU1" s="77"/>
-      <c r="DV1" s="82" t="s">
+      <c r="DV1" s="76" t="s">
         <v>18</v>
       </c>
       <c r="DW1" s="77"/>
@@ -1801,7 +1802,7 @@
       <c r="DZ1" s="77"/>
       <c r="EA1" s="77"/>
       <c r="EB1" s="77"/>
-      <c r="EC1" s="82" t="s">
+      <c r="EC1" s="76" t="s">
         <v>19</v>
       </c>
       <c r="ED1" s="77"/>
@@ -1810,7 +1811,7 @@
       <c r="EG1" s="77"/>
       <c r="EH1" s="77"/>
       <c r="EI1" s="77"/>
-      <c r="EJ1" s="82" t="s">
+      <c r="EJ1" s="76" t="s">
         <v>20</v>
       </c>
       <c r="EK1" s="77"/>
@@ -1819,7 +1820,7 @@
       <c r="EN1" s="77"/>
       <c r="EO1" s="77"/>
       <c r="EP1" s="77"/>
-      <c r="EQ1" s="82" t="s">
+      <c r="EQ1" s="76" t="s">
         <v>21</v>
       </c>
       <c r="ER1" s="77"/>
@@ -1828,7 +1829,7 @@
       <c r="EU1" s="77"/>
       <c r="EV1" s="77"/>
       <c r="EW1" s="77"/>
-      <c r="EX1" s="82" t="s">
+      <c r="EX1" s="76" t="s">
         <v>22</v>
       </c>
       <c r="EY1" s="77"/>
@@ -1837,7 +1838,7 @@
       <c r="FB1" s="77"/>
       <c r="FC1" s="77"/>
       <c r="FD1" s="77"/>
-      <c r="FE1" s="82" t="s">
+      <c r="FE1" s="76" t="s">
         <v>23</v>
       </c>
       <c r="FF1" s="77"/>
@@ -1846,7 +1847,7 @@
       <c r="FI1" s="77"/>
       <c r="FJ1" s="77"/>
       <c r="FK1" s="77"/>
-      <c r="FL1" s="82" t="s">
+      <c r="FL1" s="76" t="s">
         <v>24</v>
       </c>
       <c r="FM1" s="77"/>
@@ -1855,7 +1856,7 @@
       <c r="FP1" s="77"/>
       <c r="FQ1" s="77"/>
       <c r="FR1" s="77"/>
-      <c r="FS1" s="82" t="s">
+      <c r="FS1" s="76" t="s">
         <v>25</v>
       </c>
       <c r="FT1" s="77"/>
@@ -1864,7 +1865,7 @@
       <c r="FW1" s="77"/>
       <c r="FX1" s="77"/>
       <c r="FY1" s="77"/>
-      <c r="FZ1" s="82" t="s">
+      <c r="FZ1" s="76" t="s">
         <v>26</v>
       </c>
       <c r="GA1" s="77"/>
@@ -1873,7 +1874,7 @@
       <c r="GD1" s="77"/>
       <c r="GE1" s="77"/>
       <c r="GF1" s="77"/>
-      <c r="GG1" s="82" t="s">
+      <c r="GG1" s="76" t="s">
         <v>27</v>
       </c>
       <c r="GH1" s="77"/>
@@ -1882,7 +1883,7 @@
       <c r="GK1" s="77"/>
       <c r="GL1" s="77"/>
       <c r="GM1" s="77"/>
-      <c r="GN1" s="82" t="s">
+      <c r="GN1" s="76" t="s">
         <v>28</v>
       </c>
       <c r="GO1" s="77"/>
@@ -1891,7 +1892,7 @@
       <c r="GR1" s="77"/>
       <c r="GS1" s="77"/>
       <c r="GT1" s="77"/>
-      <c r="GU1" s="82" t="s">
+      <c r="GU1" s="76" t="s">
         <v>29</v>
       </c>
       <c r="GV1" s="77"/>
@@ -1900,7 +1901,7 @@
       <c r="GY1" s="77"/>
       <c r="GZ1" s="77"/>
       <c r="HA1" s="77"/>
-      <c r="HB1" s="82" t="s">
+      <c r="HB1" s="76" t="s">
         <v>30</v>
       </c>
       <c r="HC1" s="77"/>
@@ -1909,7 +1910,7 @@
       <c r="HF1" s="77"/>
       <c r="HG1" s="77"/>
       <c r="HH1" s="77"/>
-      <c r="HI1" s="82" t="s">
+      <c r="HI1" s="76" t="s">
         <v>31</v>
       </c>
       <c r="HJ1" s="77"/>
@@ -1918,7 +1919,7 @@
       <c r="HM1" s="77"/>
       <c r="HN1" s="77"/>
       <c r="HO1" s="77"/>
-      <c r="HP1" s="82" t="s">
+      <c r="HP1" s="76" t="s">
         <v>32</v>
       </c>
       <c r="HQ1" s="77"/>
@@ -2075,13 +2076,13 @@
       <c r="BC2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="BD2" s="63" t="s">
+      <c r="BD2" s="62" t="s">
         <v>34</v>
       </c>
       <c r="BE2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="BF2" s="2" t="s">
+      <c r="BF2" s="63" t="s">
         <v>34</v>
       </c>
       <c r="BG2" s="2" t="s">
@@ -2740,13 +2741,13 @@
       <c r="BC3" s="3">
         <v>46299</v>
       </c>
-      <c r="BD3" s="64">
+      <c r="BD3" s="50">
         <v>46300</v>
       </c>
       <c r="BE3" s="3">
         <v>46301</v>
       </c>
-      <c r="BF3" s="3">
+      <c r="BF3" s="64">
         <v>46302</v>
       </c>
       <c r="BG3" s="3">
@@ -3320,9 +3321,9 @@
       <c r="BA4" s="5"/>
       <c r="BB4" s="5"/>
       <c r="BC4" s="5"/>
-      <c r="BD4" s="65"/>
+      <c r="BD4" s="51"/>
       <c r="BE4" s="5"/>
-      <c r="BF4" s="5"/>
+      <c r="BF4" s="65"/>
       <c r="BG4" s="5"/>
       <c r="BH4" s="5"/>
       <c r="BI4" s="5"/>
@@ -3493,20 +3494,20 @@
       <c r="HR4" s="5"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92" t="s">
+      <c r="A5" s="91" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="88"/>
-      <c r="C5" s="86" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="80" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="90" t="s">
+      <c r="E5" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="84"/>
+      <c r="F5" s="89"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
@@ -3548,12 +3549,11 @@
       <c r="AT5" s="68"/>
       <c r="AU5" s="10"/>
       <c r="AV5" s="47"/>
-      <c r="AY5" s="74"/>
+      <c r="AY5" s="72"/>
       <c r="BA5" s="9"/>
       <c r="BB5" s="10"/>
-      <c r="BC5" s="11"/>
+      <c r="BC5" s="47"/>
       <c r="BE5" s="8"/>
-      <c r="BF5" s="8"/>
       <c r="BG5" s="8"/>
       <c r="BH5" s="9"/>
       <c r="BI5" s="10"/>
@@ -3724,14 +3724,14 @@
       <c r="HR5" s="8"/>
     </row>
     <row r="6" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="85"/>
-      <c r="B6" s="85"/>
-      <c r="C6" s="85"/>
+      <c r="A6" s="81"/>
+      <c r="B6" s="81"/>
+      <c r="C6" s="81"/>
       <c r="D6" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="85"/>
-      <c r="F6" s="85"/>
+      <c r="E6" s="81"/>
+      <c r="F6" s="81"/>
       <c r="G6" s="8"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
@@ -3773,12 +3773,11 @@
       <c r="AT6" s="68"/>
       <c r="AU6" s="10"/>
       <c r="AV6" s="47"/>
-      <c r="AY6" s="74"/>
+      <c r="AY6" s="72"/>
       <c r="BA6" s="9"/>
       <c r="BB6" s="10"/>
-      <c r="BC6" s="11"/>
+      <c r="BC6" s="47"/>
       <c r="BE6" s="8"/>
-      <c r="BF6" s="8"/>
       <c r="BG6" s="8"/>
       <c r="BH6" s="9"/>
       <c r="BI6" s="10"/>
@@ -3949,18 +3948,18 @@
       <c r="HR6" s="8"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="85"/>
-      <c r="B7" s="88"/>
-      <c r="C7" s="86" t="s">
+      <c r="A7" s="81"/>
+      <c r="B7" s="87"/>
+      <c r="C7" s="80" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="90" t="s">
+      <c r="E7" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="84"/>
+      <c r="F7" s="89"/>
       <c r="G7" s="8"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -4002,12 +4001,11 @@
       <c r="AT7" s="68"/>
       <c r="AU7" s="10"/>
       <c r="AV7" s="47"/>
-      <c r="AY7" s="74"/>
+      <c r="AY7" s="72"/>
       <c r="BA7" s="9"/>
       <c r="BB7" s="10"/>
-      <c r="BC7" s="11"/>
+      <c r="BC7" s="47"/>
       <c r="BE7" s="8"/>
-      <c r="BF7" s="8"/>
       <c r="BG7" s="8"/>
       <c r="BH7" s="9"/>
       <c r="BI7" s="10"/>
@@ -4178,14 +4176,14 @@
       <c r="HR7" s="8"/>
     </row>
     <row r="8" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="85"/>
-      <c r="B8" s="85"/>
-      <c r="C8" s="85"/>
+      <c r="A8" s="81"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="81"/>
       <c r="D8" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="85"/>
-      <c r="F8" s="85"/>
+      <c r="E8" s="81"/>
+      <c r="F8" s="81"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4227,12 +4225,11 @@
       <c r="AT8" s="68"/>
       <c r="AU8" s="10"/>
       <c r="AV8" s="47"/>
-      <c r="AY8" s="74"/>
+      <c r="AY8" s="72"/>
       <c r="BA8" s="9"/>
       <c r="BB8" s="10"/>
-      <c r="BC8" s="11"/>
+      <c r="BC8" s="47"/>
       <c r="BE8" s="8"/>
-      <c r="BF8" s="8"/>
       <c r="BG8" s="8"/>
       <c r="BH8" s="9"/>
       <c r="BI8" s="10"/>
@@ -4403,18 +4400,18 @@
       <c r="HR8" s="8"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="85"/>
-      <c r="B9" s="88"/>
-      <c r="C9" s="86" t="s">
+      <c r="A9" s="81"/>
+      <c r="B9" s="87"/>
+      <c r="C9" s="80" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="90" t="s">
+      <c r="E9" s="85" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="84"/>
+      <c r="F9" s="89"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -4456,12 +4453,11 @@
       <c r="AT9" s="68"/>
       <c r="AU9" s="10"/>
       <c r="AV9" s="47"/>
-      <c r="AY9" s="74"/>
+      <c r="AY9" s="72"/>
       <c r="BA9" s="9"/>
       <c r="BB9" s="10"/>
-      <c r="BC9" s="11"/>
+      <c r="BC9" s="47"/>
       <c r="BE9" s="8"/>
-      <c r="BF9" s="8"/>
       <c r="BG9" s="8"/>
       <c r="BH9" s="9"/>
       <c r="BI9" s="10"/>
@@ -4632,14 +4628,14 @@
       <c r="HR9" s="8"/>
     </row>
     <row r="10" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="85"/>
-      <c r="B10" s="85"/>
-      <c r="C10" s="85"/>
+      <c r="A10" s="81"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="81"/>
       <c r="D10" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="85"/>
-      <c r="F10" s="85"/>
+      <c r="E10" s="81"/>
+      <c r="F10" s="81"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -4681,12 +4677,11 @@
       <c r="AT10" s="68"/>
       <c r="AU10" s="10"/>
       <c r="AV10" s="47"/>
-      <c r="AY10" s="74"/>
+      <c r="AY10" s="72"/>
       <c r="BA10" s="9"/>
       <c r="BB10" s="10"/>
-      <c r="BC10" s="11"/>
+      <c r="BC10" s="47"/>
       <c r="BE10" s="8"/>
-      <c r="BF10" s="8"/>
       <c r="BG10" s="8"/>
       <c r="BH10" s="9"/>
       <c r="BI10" s="10"/>
@@ -4857,18 +4852,18 @@
       <c r="HR10" s="8"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="85"/>
-      <c r="B11" s="88"/>
-      <c r="C11" s="86" t="s">
+      <c r="A11" s="81"/>
+      <c r="B11" s="87"/>
+      <c r="C11" s="80" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="90" t="s">
+      <c r="E11" s="85" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="84"/>
+      <c r="F11" s="89"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -4910,12 +4905,11 @@
       <c r="AT11" s="68"/>
       <c r="AU11" s="10"/>
       <c r="AV11" s="47"/>
-      <c r="AY11" s="74"/>
+      <c r="AY11" s="72"/>
       <c r="BA11" s="9"/>
       <c r="BB11" s="10"/>
-      <c r="BC11" s="11"/>
+      <c r="BC11" s="47"/>
       <c r="BE11" s="8"/>
-      <c r="BF11" s="8"/>
       <c r="BG11" s="8"/>
       <c r="BH11" s="9"/>
       <c r="BI11" s="10"/>
@@ -5086,14 +5080,14 @@
       <c r="HR11" s="8"/>
     </row>
     <row r="12" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="85"/>
-      <c r="B12" s="85"/>
-      <c r="C12" s="85"/>
+      <c r="A12" s="81"/>
+      <c r="B12" s="81"/>
+      <c r="C12" s="81"/>
       <c r="D12" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="85"/>
-      <c r="F12" s="85"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="81"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -5135,12 +5129,11 @@
       <c r="AT12" s="68"/>
       <c r="AU12" s="10"/>
       <c r="AV12" s="47"/>
-      <c r="AY12" s="74"/>
+      <c r="AY12" s="72"/>
       <c r="BA12" s="9"/>
       <c r="BB12" s="10"/>
-      <c r="BC12" s="11"/>
+      <c r="BC12" s="47"/>
       <c r="BE12" s="8"/>
-      <c r="BF12" s="8"/>
       <c r="BG12" s="8"/>
       <c r="BH12" s="9"/>
       <c r="BI12" s="10"/>
@@ -5311,18 +5304,18 @@
       <c r="HR12" s="8"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="85"/>
-      <c r="B13" s="88"/>
-      <c r="C13" s="86" t="s">
+      <c r="A13" s="81"/>
+      <c r="B13" s="87"/>
+      <c r="C13" s="80" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="90" t="s">
+      <c r="E13" s="85" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="84"/>
+      <c r="F13" s="89"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -5364,12 +5357,11 @@
       <c r="AT13" s="68"/>
       <c r="AU13" s="10"/>
       <c r="AV13" s="47"/>
-      <c r="AY13" s="74"/>
+      <c r="AY13" s="72"/>
       <c r="BA13" s="9"/>
       <c r="BB13" s="10"/>
-      <c r="BC13" s="11"/>
+      <c r="BC13" s="47"/>
       <c r="BE13" s="8"/>
-      <c r="BF13" s="8"/>
       <c r="BG13" s="8"/>
       <c r="BH13" s="9"/>
       <c r="BI13" s="10"/>
@@ -5540,14 +5532,14 @@
       <c r="HR13" s="8"/>
     </row>
     <row r="14" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="85"/>
-      <c r="B14" s="85"/>
-      <c r="C14" s="85"/>
+      <c r="A14" s="81"/>
+      <c r="B14" s="81"/>
+      <c r="C14" s="81"/>
       <c r="D14" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="85"/>
-      <c r="F14" s="85"/>
+      <c r="E14" s="81"/>
+      <c r="F14" s="81"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5589,12 +5581,11 @@
       <c r="AT14" s="68"/>
       <c r="AU14" s="10"/>
       <c r="AV14" s="47"/>
-      <c r="AY14" s="74"/>
+      <c r="AY14" s="72"/>
       <c r="BA14" s="9"/>
       <c r="BB14" s="10"/>
-      <c r="BC14" s="11"/>
+      <c r="BC14" s="47"/>
       <c r="BE14" s="8"/>
-      <c r="BF14" s="8"/>
       <c r="BG14" s="8"/>
       <c r="BH14" s="9"/>
       <c r="BI14" s="10"/>
@@ -5765,18 +5756,18 @@
       <c r="HR14" s="8"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="85"/>
-      <c r="B15" s="88"/>
-      <c r="C15" s="86" t="s">
+      <c r="A15" s="81"/>
+      <c r="B15" s="87"/>
+      <c r="C15" s="80" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="90" t="s">
+      <c r="E15" s="85" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="84"/>
+      <c r="F15" s="89"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
@@ -5818,12 +5809,11 @@
       <c r="AT15" s="68"/>
       <c r="AU15" s="10"/>
       <c r="AV15" s="47"/>
-      <c r="AY15" s="74"/>
+      <c r="AY15" s="72"/>
       <c r="BA15" s="9"/>
       <c r="BB15" s="10"/>
-      <c r="BC15" s="11"/>
+      <c r="BC15" s="47"/>
       <c r="BE15" s="8"/>
-      <c r="BF15" s="8"/>
       <c r="BG15" s="8"/>
       <c r="BH15" s="9"/>
       <c r="BI15" s="10"/>
@@ -5994,14 +5984,14 @@
       <c r="HR15" s="8"/>
     </row>
     <row r="16" spans="1:226" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="85"/>
-      <c r="B16" s="85"/>
-      <c r="C16" s="85"/>
+      <c r="A16" s="81"/>
+      <c r="B16" s="81"/>
+      <c r="C16" s="81"/>
       <c r="D16" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="85"/>
-      <c r="F16" s="85"/>
+      <c r="E16" s="81"/>
+      <c r="F16" s="81"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -6043,12 +6033,11 @@
       <c r="AT16" s="68"/>
       <c r="AU16" s="10"/>
       <c r="AV16" s="47"/>
-      <c r="AY16" s="74"/>
+      <c r="AY16" s="72"/>
       <c r="BA16" s="9"/>
       <c r="BB16" s="10"/>
-      <c r="BC16" s="11"/>
+      <c r="BC16" s="47"/>
       <c r="BE16" s="8"/>
-      <c r="BF16" s="8"/>
       <c r="BG16" s="8"/>
       <c r="BH16" s="9"/>
       <c r="BI16" s="10"/>
@@ -6219,18 +6208,18 @@
       <c r="HR16" s="8"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="85"/>
-      <c r="B17" s="88"/>
-      <c r="C17" s="86" t="s">
+      <c r="A17" s="81"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="80" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="90" t="s">
+      <c r="E17" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="84"/>
+      <c r="F17" s="89"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -6272,12 +6261,11 @@
       <c r="AT17" s="68"/>
       <c r="AU17" s="10"/>
       <c r="AV17" s="47"/>
-      <c r="AY17" s="74"/>
+      <c r="AY17" s="72"/>
       <c r="BA17" s="9"/>
       <c r="BB17" s="10"/>
-      <c r="BC17" s="11"/>
+      <c r="BC17" s="47"/>
       <c r="BE17" s="8"/>
-      <c r="BF17" s="8"/>
       <c r="BG17" s="8"/>
       <c r="BH17" s="9"/>
       <c r="BI17" s="10"/>
@@ -6448,14 +6436,14 @@
       <c r="HR17" s="8"/>
     </row>
     <row r="18" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="85"/>
-      <c r="B18" s="85"/>
-      <c r="C18" s="85"/>
+      <c r="A18" s="81"/>
+      <c r="B18" s="81"/>
+      <c r="C18" s="81"/>
       <c r="D18" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="85"/>
-      <c r="F18" s="85"/>
+      <c r="E18" s="81"/>
+      <c r="F18" s="81"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
@@ -6497,12 +6485,11 @@
       <c r="AT18" s="68"/>
       <c r="AU18" s="10"/>
       <c r="AV18" s="47"/>
-      <c r="AY18" s="74"/>
+      <c r="AY18" s="72"/>
       <c r="BA18" s="9"/>
       <c r="BB18" s="10"/>
-      <c r="BC18" s="11"/>
+      <c r="BC18" s="47"/>
       <c r="BE18" s="8"/>
-      <c r="BF18" s="8"/>
       <c r="BG18" s="8"/>
       <c r="BH18" s="9"/>
       <c r="BI18" s="10"/>
@@ -6673,18 +6660,18 @@
       <c r="HR18" s="8"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="85"/>
-      <c r="B19" s="88"/>
-      <c r="C19" s="86" t="s">
+      <c r="A19" s="81"/>
+      <c r="B19" s="87"/>
+      <c r="C19" s="80" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="90" t="s">
+      <c r="E19" s="85" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="84"/>
+      <c r="F19" s="89"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -6726,12 +6713,11 @@
       <c r="AT19" s="68"/>
       <c r="AU19" s="10"/>
       <c r="AV19" s="47"/>
-      <c r="AY19" s="74"/>
+      <c r="AY19" s="72"/>
       <c r="BA19" s="9"/>
       <c r="BB19" s="10"/>
-      <c r="BC19" s="11"/>
+      <c r="BC19" s="47"/>
       <c r="BE19" s="8"/>
-      <c r="BF19" s="8"/>
       <c r="BG19" s="8"/>
       <c r="BH19" s="9"/>
       <c r="BI19" s="10"/>
@@ -6902,14 +6888,14 @@
       <c r="HR19" s="8"/>
     </row>
     <row r="20" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="85"/>
-      <c r="B20" s="85"/>
-      <c r="C20" s="85"/>
+      <c r="A20" s="81"/>
+      <c r="B20" s="81"/>
+      <c r="C20" s="81"/>
       <c r="D20" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="85"/>
-      <c r="F20" s="85"/>
+      <c r="E20" s="81"/>
+      <c r="F20" s="81"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -6951,12 +6937,11 @@
       <c r="AT20" s="68"/>
       <c r="AU20" s="10"/>
       <c r="AV20" s="47"/>
-      <c r="AY20" s="74"/>
+      <c r="AY20" s="72"/>
       <c r="BA20" s="9"/>
       <c r="BB20" s="10"/>
-      <c r="BC20" s="11"/>
+      <c r="BC20" s="47"/>
       <c r="BE20" s="8"/>
-      <c r="BF20" s="8"/>
       <c r="BG20" s="8"/>
       <c r="BH20" s="9"/>
       <c r="BI20" s="10"/>
@@ -7127,18 +7112,18 @@
       <c r="HR20" s="8"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="85"/>
-      <c r="B21" s="88"/>
-      <c r="C21" s="86" t="s">
+      <c r="A21" s="81"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="80" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="90" t="s">
+      <c r="E21" s="85" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="84"/>
+      <c r="F21" s="89"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
@@ -7180,12 +7165,11 @@
       <c r="AT21" s="68"/>
       <c r="AU21" s="10"/>
       <c r="AV21" s="47"/>
-      <c r="AY21" s="74"/>
+      <c r="AY21" s="72"/>
       <c r="BA21" s="9"/>
       <c r="BB21" s="10"/>
-      <c r="BC21" s="11"/>
+      <c r="BC21" s="47"/>
       <c r="BE21" s="8"/>
-      <c r="BF21" s="8"/>
       <c r="BG21" s="8"/>
       <c r="BH21" s="9"/>
       <c r="BI21" s="10"/>
@@ -7356,14 +7340,14 @@
       <c r="HR21" s="8"/>
     </row>
     <row r="22" spans="1:227" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="91"/>
-      <c r="B22" s="91"/>
-      <c r="C22" s="91"/>
+      <c r="A22" s="88"/>
+      <c r="B22" s="88"/>
+      <c r="C22" s="88"/>
       <c r="D22" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="91"/>
-      <c r="F22" s="91"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
@@ -7405,13 +7389,12 @@
       <c r="AT22" s="68"/>
       <c r="AU22" s="40"/>
       <c r="AV22" s="48"/>
-      <c r="AY22" s="75"/>
+      <c r="AY22" s="73"/>
       <c r="BA22" s="39"/>
       <c r="BB22" s="40"/>
-      <c r="BC22" s="41"/>
-      <c r="BD22" s="69"/>
+      <c r="BC22" s="48"/>
       <c r="BE22" s="38"/>
-      <c r="BF22" s="38"/>
+      <c r="BF22" s="69"/>
       <c r="BG22" s="38"/>
       <c r="BH22" s="39"/>
       <c r="BI22" s="40"/>
@@ -7582,22 +7565,22 @@
       <c r="HR22" s="38"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="87" t="s">
+      <c r="A23" s="78" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="78" t="s">
+      <c r="B23" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="80" t="s">
+      <c r="C23" s="79" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="79" t="s">
+      <c r="E23" s="82" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="81" t="s">
+      <c r="F23" s="84" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="8"/>
@@ -7643,13 +7626,12 @@
       <c r="AU23" s="10"/>
       <c r="AV23" s="47"/>
       <c r="AW23" s="54"/>
-      <c r="AY23" s="74"/>
+      <c r="AY23" s="72"/>
       <c r="BA23" s="9"/>
       <c r="BB23" s="10"/>
-      <c r="BC23" s="11"/>
-      <c r="BD23" s="70"/>
+      <c r="BC23" s="47"/>
+      <c r="BD23" s="54"/>
       <c r="BE23" s="8"/>
-      <c r="BF23" s="8"/>
       <c r="BG23" s="8"/>
       <c r="BH23" s="9"/>
       <c r="BI23" s="10"/>
@@ -7871,13 +7853,12 @@
       <c r="AU24" s="10"/>
       <c r="AV24" s="47"/>
       <c r="AW24" s="56"/>
-      <c r="AY24" s="74"/>
+      <c r="AY24" s="72"/>
       <c r="BA24" s="9"/>
       <c r="BB24" s="10"/>
-      <c r="BC24" s="11"/>
-      <c r="BD24" s="72"/>
+      <c r="BC24" s="47"/>
+      <c r="BD24" s="56"/>
       <c r="BE24" s="8"/>
-      <c r="BF24" s="8"/>
       <c r="BG24" s="8"/>
       <c r="BH24" s="9"/>
       <c r="BI24" s="10"/>
@@ -8049,19 +8030,19 @@
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="77"/>
-      <c r="B25" s="78" t="s">
+      <c r="B25" s="83" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="80" t="s">
+      <c r="C25" s="79" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="79" t="s">
+      <c r="E25" s="82" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="81" t="s">
+      <c r="F25" s="84" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="8"/>
@@ -8102,10 +8083,10 @@
       <c r="AT25" s="68"/>
       <c r="AU25" s="10"/>
       <c r="AV25" s="47"/>
-      <c r="AY25" s="74"/>
+      <c r="AY25" s="72"/>
       <c r="BA25" s="9"/>
       <c r="BB25" s="10"/>
-      <c r="BC25" s="11"/>
+      <c r="BC25" s="47"/>
       <c r="BG25" s="16"/>
       <c r="BH25" s="9"/>
       <c r="BI25" s="10"/>
@@ -8324,12 +8305,11 @@
       <c r="AT26" s="68"/>
       <c r="AU26" s="10"/>
       <c r="AV26" s="47"/>
-      <c r="AY26" s="74"/>
+      <c r="AY26" s="72"/>
       <c r="BA26" s="9"/>
       <c r="BB26" s="10"/>
-      <c r="BC26" s="11"/>
+      <c r="BC26" s="47"/>
       <c r="BE26" s="8"/>
-      <c r="BF26" s="8"/>
       <c r="BG26" s="8"/>
       <c r="BH26" s="9"/>
       <c r="BI26" s="10"/>
@@ -8501,19 +8481,19 @@
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="77"/>
-      <c r="B27" s="78" t="s">
+      <c r="B27" s="83" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="89" t="s">
+      <c r="C27" s="90" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="79" t="s">
+      <c r="E27" s="82" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="81"/>
+      <c r="F27" s="84"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -8554,13 +8534,12 @@
       <c r="AT27" s="68"/>
       <c r="AU27" s="10"/>
       <c r="AV27" s="47"/>
-      <c r="AY27" s="74"/>
-      <c r="AZ27" s="93"/>
+      <c r="AY27" s="72"/>
+      <c r="AZ27" s="75"/>
       <c r="BA27" s="9"/>
       <c r="BB27" s="10"/>
-      <c r="BC27" s="11"/>
+      <c r="BC27" s="47"/>
       <c r="BE27" s="8"/>
-      <c r="BF27" s="8"/>
       <c r="BG27" s="8"/>
       <c r="BH27" s="9"/>
       <c r="BI27" s="10"/>
@@ -8779,13 +8758,12 @@
       <c r="AT28" s="68"/>
       <c r="AU28" s="10"/>
       <c r="AV28" s="47"/>
-      <c r="AY28" s="74"/>
+      <c r="AY28" s="72"/>
       <c r="AZ28" s="56"/>
       <c r="BA28" s="9"/>
       <c r="BB28" s="10"/>
-      <c r="BC28" s="11"/>
+      <c r="BC28" s="47"/>
       <c r="BE28" s="8"/>
-      <c r="BF28" s="8"/>
       <c r="BG28" s="8"/>
       <c r="BH28" s="9"/>
       <c r="BI28" s="10"/>
@@ -8956,22 +8934,22 @@
       <c r="HR28" s="8"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="87" t="s">
+      <c r="A29" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="78" t="s">
+      <c r="B29" s="83" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="80" t="s">
+      <c r="C29" s="79" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="79" t="s">
+      <c r="E29" s="82" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="81" t="s">
+      <c r="F29" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="8"/>
@@ -9014,12 +8992,11 @@
       <c r="AT29" s="68"/>
       <c r="AU29" s="10"/>
       <c r="AV29" s="47"/>
-      <c r="AY29" s="74"/>
+      <c r="AY29" s="72"/>
       <c r="BA29" s="9"/>
       <c r="BB29" s="10"/>
-      <c r="BC29" s="11"/>
+      <c r="BC29" s="47"/>
       <c r="BE29" s="8"/>
-      <c r="BF29" s="8"/>
       <c r="BG29" s="8"/>
       <c r="BH29" s="9"/>
       <c r="BI29" s="10"/>
@@ -9239,12 +9216,11 @@
       <c r="AT30" s="68"/>
       <c r="AU30" s="10"/>
       <c r="AV30" s="47"/>
-      <c r="AY30" s="74"/>
+      <c r="AY30" s="72"/>
       <c r="BA30" s="9"/>
       <c r="BB30" s="10"/>
-      <c r="BC30" s="11"/>
+      <c r="BC30" s="47"/>
       <c r="BE30" s="8"/>
-      <c r="BF30" s="8"/>
       <c r="BG30" s="8"/>
       <c r="BH30" s="9"/>
       <c r="BI30" s="10"/>
@@ -9416,19 +9392,19 @@
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="77"/>
-      <c r="B31" s="78" t="s">
+      <c r="B31" s="83" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="80" t="s">
+      <c r="C31" s="79" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="79" t="s">
+      <c r="E31" s="82" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="81" t="s">
+      <c r="F31" s="84" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="8"/>
@@ -9472,12 +9448,11 @@
       <c r="AT31" s="68"/>
       <c r="AU31" s="10"/>
       <c r="AV31" s="47"/>
-      <c r="AY31" s="74"/>
+      <c r="AY31" s="72"/>
       <c r="BA31" s="9"/>
       <c r="BB31" s="10"/>
-      <c r="BC31" s="11"/>
+      <c r="BC31" s="47"/>
       <c r="BE31" s="8"/>
-      <c r="BF31" s="8"/>
       <c r="BG31" s="8"/>
       <c r="BH31" s="9"/>
       <c r="BI31" s="10"/>
@@ -9697,12 +9672,11 @@
       <c r="AT32" s="68"/>
       <c r="AU32" s="10"/>
       <c r="AV32" s="47"/>
-      <c r="AY32" s="74"/>
+      <c r="AY32" s="72"/>
       <c r="BA32" s="9"/>
       <c r="BB32" s="10"/>
-      <c r="BC32" s="11"/>
+      <c r="BC32" s="47"/>
       <c r="BE32" s="8"/>
-      <c r="BF32" s="8"/>
       <c r="BG32" s="8"/>
       <c r="BH32" s="9"/>
       <c r="BI32" s="10"/>
@@ -9874,19 +9848,19 @@
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="77"/>
-      <c r="B33" s="78" t="s">
+      <c r="B33" s="83" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="80" t="s">
+      <c r="C33" s="79" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="79" t="s">
+      <c r="E33" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="81" t="s">
+      <c r="F33" s="84" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="8"/>
@@ -9933,9 +9907,8 @@
       <c r="AY33" s="54"/>
       <c r="BA33" s="9"/>
       <c r="BB33" s="10"/>
-      <c r="BC33" s="11"/>
+      <c r="BC33" s="47"/>
       <c r="BE33" s="8"/>
-      <c r="BF33" s="8"/>
       <c r="BG33" s="8"/>
       <c r="BH33" s="9"/>
       <c r="BI33" s="10"/>
@@ -10155,12 +10128,11 @@
       <c r="AT34" s="68"/>
       <c r="AU34" s="10"/>
       <c r="AV34" s="60"/>
-      <c r="AY34" s="74"/>
+      <c r="AY34" s="72"/>
       <c r="BA34" s="9"/>
       <c r="BB34" s="10"/>
-      <c r="BC34" s="11"/>
+      <c r="BC34" s="47"/>
       <c r="BE34" s="8"/>
-      <c r="BF34" s="8"/>
       <c r="BG34" s="8"/>
       <c r="BH34" s="9"/>
       <c r="BI34" s="10"/>
@@ -10332,19 +10304,19 @@
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="77"/>
-      <c r="B35" s="78" t="s">
+      <c r="B35" s="83" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="80" t="s">
+      <c r="C35" s="79" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="79" t="s">
+      <c r="E35" s="82" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="81" t="s">
+      <c r="F35" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="8"/>
@@ -10388,12 +10360,12 @@
       <c r="AT35" s="68"/>
       <c r="AU35" s="10"/>
       <c r="AV35" s="47"/>
-      <c r="AY35" s="74"/>
+      <c r="AY35" s="72"/>
       <c r="BA35" s="9"/>
       <c r="BB35" s="10"/>
-      <c r="BC35" s="11"/>
+      <c r="BC35" s="47"/>
       <c r="BE35" s="8"/>
-      <c r="BF35" s="16"/>
+      <c r="BF35" s="70"/>
       <c r="BG35" s="16"/>
       <c r="BH35" s="9"/>
       <c r="BI35" s="10"/>
@@ -10613,12 +10585,11 @@
       <c r="AT36" s="68"/>
       <c r="AU36" s="10"/>
       <c r="AV36" s="47"/>
-      <c r="AY36" s="74"/>
+      <c r="AY36" s="72"/>
       <c r="BA36" s="9"/>
       <c r="BB36" s="10"/>
-      <c r="BC36" s="11"/>
+      <c r="BC36" s="47"/>
       <c r="BE36" s="8"/>
-      <c r="BF36" s="8"/>
       <c r="BG36" s="8"/>
       <c r="BH36" s="9"/>
       <c r="BI36" s="10"/>
@@ -10790,19 +10761,19 @@
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="77"/>
-      <c r="B37" s="78" t="s">
+      <c r="B37" s="83" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="80" t="s">
+      <c r="C37" s="79" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="79" t="s">
+      <c r="E37" s="82" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="81" t="s">
+      <c r="F37" s="84" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="8"/>
@@ -10846,12 +10817,11 @@
       <c r="AT37" s="68"/>
       <c r="AU37" s="10"/>
       <c r="AV37" s="47"/>
-      <c r="AY37" s="74"/>
+      <c r="AY37" s="72"/>
       <c r="BA37" s="9"/>
       <c r="BB37" s="10"/>
-      <c r="BC37" s="11"/>
+      <c r="BC37" s="47"/>
       <c r="BE37" s="8"/>
-      <c r="BF37" s="8"/>
       <c r="BG37" s="8"/>
       <c r="BH37" s="9"/>
       <c r="BI37" s="10"/>
@@ -11071,12 +11041,11 @@
       <c r="AT38" s="68"/>
       <c r="AU38" s="10"/>
       <c r="AV38" s="47"/>
-      <c r="AY38" s="74"/>
+      <c r="AY38" s="72"/>
       <c r="BA38" s="9"/>
       <c r="BB38" s="10"/>
-      <c r="BC38" s="11"/>
+      <c r="BC38" s="47"/>
       <c r="BE38" s="8"/>
-      <c r="BF38" s="8"/>
       <c r="BG38" s="8"/>
       <c r="BH38" s="9"/>
       <c r="BI38" s="10"/>
@@ -11248,19 +11217,19 @@
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="77"/>
-      <c r="B39" s="78" t="s">
+      <c r="B39" s="83" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="80" t="s">
+      <c r="C39" s="79" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="79" t="s">
+      <c r="E39" s="82" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="81" t="s">
+      <c r="F39" s="84" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="8"/>
@@ -11304,12 +11273,11 @@
       <c r="AT39" s="68"/>
       <c r="AU39" s="10"/>
       <c r="AV39" s="47"/>
-      <c r="AY39" s="74"/>
+      <c r="AY39" s="72"/>
       <c r="BA39" s="9"/>
       <c r="BB39" s="10"/>
-      <c r="BC39" s="11"/>
+      <c r="BC39" s="47"/>
       <c r="BE39" s="8"/>
-      <c r="BF39" s="8"/>
       <c r="BG39" s="8"/>
       <c r="BH39" s="9"/>
       <c r="BI39" s="10"/>
@@ -11529,13 +11497,12 @@
       <c r="AT40" s="68"/>
       <c r="AU40" s="10"/>
       <c r="AV40" s="47"/>
-      <c r="AY40" s="74"/>
+      <c r="AY40" s="72"/>
       <c r="AZ40" s="60"/>
       <c r="BA40" s="9"/>
       <c r="BB40" s="10"/>
-      <c r="BC40" s="11"/>
+      <c r="BC40" s="47"/>
       <c r="BE40" s="8"/>
-      <c r="BF40" s="8"/>
       <c r="BG40" s="8"/>
       <c r="BH40" s="9"/>
       <c r="BI40" s="10"/>
@@ -11706,22 +11673,22 @@
       <c r="HR40" s="8"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="87" t="s">
+      <c r="A41" s="78" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="78" t="s">
+      <c r="B41" s="83" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="80" t="s">
+      <c r="C41" s="79" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="79" t="s">
+      <c r="E41" s="82" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="81" t="s">
+      <c r="F41" s="84" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="8"/>
@@ -11765,12 +11732,11 @@
       <c r="AT41" s="68"/>
       <c r="AU41" s="10"/>
       <c r="AV41" s="47"/>
-      <c r="AY41" s="74"/>
+      <c r="AY41" s="72"/>
       <c r="BA41" s="9"/>
       <c r="BB41" s="10"/>
-      <c r="BC41" s="11"/>
+      <c r="BC41" s="47"/>
       <c r="BE41" s="8"/>
-      <c r="BF41" s="8"/>
       <c r="BG41" s="8"/>
       <c r="BH41" s="9"/>
       <c r="BI41" s="10"/>
@@ -11990,12 +11956,11 @@
       <c r="AT42" s="68"/>
       <c r="AU42" s="10"/>
       <c r="AV42" s="47"/>
-      <c r="AY42" s="74"/>
+      <c r="AY42" s="72"/>
       <c r="BA42" s="9"/>
       <c r="BB42" s="10"/>
-      <c r="BC42" s="11"/>
+      <c r="BC42" s="47"/>
       <c r="BE42" s="8"/>
-      <c r="BF42" s="8"/>
       <c r="BG42" s="8"/>
       <c r="BH42" s="9"/>
       <c r="BI42" s="10"/>
@@ -12167,19 +12132,19 @@
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="77"/>
-      <c r="B43" s="78" t="s">
+      <c r="B43" s="83" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="80" t="s">
+      <c r="C43" s="79" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="79" t="s">
+      <c r="E43" s="82" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="81" t="s">
+      <c r="F43" s="84" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="8"/>
@@ -12222,12 +12187,11 @@
       <c r="AT43" s="68"/>
       <c r="AU43" s="10"/>
       <c r="AV43" s="47"/>
-      <c r="AY43" s="74"/>
+      <c r="AY43" s="72"/>
       <c r="BA43" s="9"/>
       <c r="BB43" s="10"/>
-      <c r="BC43" s="11"/>
+      <c r="BC43" s="47"/>
       <c r="BE43" s="8"/>
-      <c r="BF43" s="8"/>
       <c r="BG43" s="8"/>
       <c r="BH43" s="9"/>
       <c r="BI43" s="10"/>
@@ -12449,12 +12413,11 @@
       <c r="AU44" s="10"/>
       <c r="AV44" s="47"/>
       <c r="AX44" s="61"/>
-      <c r="AY44" s="74"/>
+      <c r="AY44" s="72"/>
       <c r="BA44" s="9"/>
       <c r="BB44" s="10"/>
-      <c r="BC44" s="11"/>
+      <c r="BC44" s="47"/>
       <c r="BE44" s="8"/>
-      <c r="BF44" s="8"/>
       <c r="BG44" s="8"/>
       <c r="BH44" s="9"/>
       <c r="BI44" s="10"/>
@@ -12626,19 +12589,19 @@
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="77"/>
-      <c r="B45" s="78" t="s">
+      <c r="B45" s="83" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="80" t="s">
+      <c r="C45" s="79" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="79" t="s">
+      <c r="E45" s="82" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="81" t="s">
+      <c r="F45" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="8"/>
@@ -12682,12 +12645,11 @@
       <c r="AU45" s="10"/>
       <c r="AV45" s="47"/>
       <c r="AW45" s="52"/>
-      <c r="AY45" s="74"/>
+      <c r="AY45" s="72"/>
       <c r="BA45" s="9"/>
       <c r="BB45" s="10"/>
-      <c r="BC45" s="11"/>
+      <c r="BC45" s="47"/>
       <c r="BE45" s="8"/>
-      <c r="BF45" s="8"/>
       <c r="BG45" s="8"/>
       <c r="BH45" s="9"/>
       <c r="BI45" s="10"/>
@@ -12908,12 +12870,11 @@
       <c r="AU46" s="10"/>
       <c r="AV46" s="47"/>
       <c r="AW46" s="56"/>
-      <c r="AY46" s="74"/>
+      <c r="AY46" s="72"/>
       <c r="BA46" s="9"/>
       <c r="BB46" s="10"/>
-      <c r="BC46" s="11"/>
+      <c r="BC46" s="47"/>
       <c r="BE46" s="8"/>
-      <c r="BF46" s="8"/>
       <c r="BG46" s="8"/>
       <c r="BH46" s="9"/>
       <c r="BI46" s="10"/>
@@ -13084,22 +13045,22 @@
       <c r="HR46" s="8"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="87" t="s">
+      <c r="A47" s="78" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="78" t="s">
+      <c r="B47" s="83" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="80" t="s">
+      <c r="C47" s="79" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="79" t="s">
+      <c r="E47" s="82" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="81" t="s">
+      <c r="F47" s="84" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="8"/>
@@ -13148,10 +13109,9 @@
       <c r="AZ47" s="52"/>
       <c r="BA47" s="9"/>
       <c r="BB47" s="10"/>
-      <c r="BC47" s="11"/>
-      <c r="BD47" s="71"/>
+      <c r="BC47" s="47"/>
+      <c r="BD47" s="52"/>
       <c r="BE47" s="7"/>
-      <c r="BF47" s="8"/>
       <c r="BG47" s="8"/>
       <c r="BH47" s="9"/>
       <c r="BI47" s="10"/>
@@ -13371,14 +13331,13 @@
       <c r="AT48" s="68"/>
       <c r="AU48" s="10"/>
       <c r="AV48" s="47"/>
-      <c r="AY48" s="74"/>
+      <c r="AY48" s="72"/>
       <c r="AZ48" s="56"/>
       <c r="BA48" s="9"/>
       <c r="BB48" s="10"/>
-      <c r="BC48" s="11"/>
-      <c r="BD48" s="72"/>
-      <c r="BE48" s="8"/>
-      <c r="BF48" s="8"/>
+      <c r="BC48" s="47"/>
+      <c r="BD48" s="56"/>
+      <c r="BE48" s="43"/>
       <c r="BG48" s="8"/>
       <c r="BH48" s="9"/>
       <c r="BI48" s="10"/>
@@ -13550,19 +13509,19 @@
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="77"/>
-      <c r="B49" s="78" t="s">
+      <c r="B49" s="83" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="80" t="s">
+      <c r="C49" s="79" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="79" t="s">
+      <c r="E49" s="82" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="81" t="s">
+      <c r="F49" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="8"/>
@@ -13606,12 +13565,11 @@
       <c r="AT49" s="68"/>
       <c r="AU49" s="10"/>
       <c r="AV49" s="47"/>
-      <c r="AY49" s="74"/>
+      <c r="AY49" s="72"/>
       <c r="BA49" s="9"/>
       <c r="BB49" s="10"/>
-      <c r="BC49" s="11"/>
+      <c r="BC49" s="47"/>
       <c r="BE49" s="8"/>
-      <c r="BF49" s="8"/>
       <c r="BG49" s="8"/>
       <c r="BH49" s="9"/>
       <c r="BI49" s="10"/>
@@ -13831,12 +13789,11 @@
       <c r="AT50" s="68"/>
       <c r="AU50" s="10"/>
       <c r="AV50" s="47"/>
-      <c r="AY50" s="74"/>
+      <c r="AY50" s="72"/>
       <c r="BA50" s="9"/>
       <c r="BB50" s="10"/>
-      <c r="BC50" s="11"/>
+      <c r="BC50" s="47"/>
       <c r="BE50" s="8"/>
-      <c r="BF50" s="8"/>
       <c r="BG50" s="8"/>
       <c r="BH50" s="9"/>
       <c r="BI50" s="10"/>
@@ -14007,22 +13964,22 @@
       <c r="HR50" s="8"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="87" t="s">
+      <c r="A51" s="78" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="78" t="s">
+      <c r="B51" s="83" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="80" t="s">
+      <c r="C51" s="79" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="79" t="s">
+      <c r="E51" s="82" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="81" t="s">
+      <c r="F51" s="84" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="8"/>
@@ -14066,12 +14023,11 @@
       <c r="AT51" s="68"/>
       <c r="AU51" s="10"/>
       <c r="AV51" s="47"/>
-      <c r="AY51" s="74"/>
+      <c r="AY51" s="72"/>
       <c r="BA51" s="9"/>
       <c r="BB51" s="10"/>
-      <c r="BC51" s="11"/>
+      <c r="BC51" s="47"/>
       <c r="BE51" s="8"/>
-      <c r="BF51" s="8"/>
       <c r="BG51" s="8"/>
       <c r="BH51" s="9"/>
       <c r="BI51" s="10"/>
@@ -14291,12 +14247,11 @@
       <c r="AT52" s="68"/>
       <c r="AU52" s="10"/>
       <c r="AV52" s="47"/>
-      <c r="AY52" s="74"/>
+      <c r="AY52" s="72"/>
       <c r="BA52" s="9"/>
       <c r="BB52" s="10"/>
-      <c r="BC52" s="11"/>
+      <c r="BC52" s="47"/>
       <c r="BE52" s="8"/>
-      <c r="BF52" s="8"/>
       <c r="BG52" s="8"/>
       <c r="BH52" s="9"/>
       <c r="BI52" s="10"/>
@@ -14468,19 +14423,19 @@
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="77"/>
-      <c r="B53" s="78" t="s">
+      <c r="B53" s="83" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="80" t="s">
+      <c r="C53" s="79" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="79" t="s">
+      <c r="E53" s="82" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="81" t="s">
+      <c r="F53" s="84" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="8"/>
@@ -14524,12 +14479,11 @@
       <c r="AT53" s="68"/>
       <c r="AU53" s="10"/>
       <c r="AV53" s="47"/>
-      <c r="AY53" s="74"/>
+      <c r="AY53" s="72"/>
       <c r="BA53" s="9"/>
       <c r="BB53" s="10"/>
-      <c r="BC53" s="11"/>
+      <c r="BC53" s="47"/>
       <c r="BE53" s="8"/>
-      <c r="BF53" s="8"/>
       <c r="BG53" s="8"/>
       <c r="BH53" s="9"/>
       <c r="BI53" s="10"/>
@@ -14749,12 +14703,11 @@
       <c r="AT54" s="68"/>
       <c r="AU54" s="10"/>
       <c r="AV54" s="47"/>
-      <c r="AY54" s="74"/>
+      <c r="AY54" s="72"/>
       <c r="BA54" s="9"/>
       <c r="BB54" s="10"/>
-      <c r="BC54" s="11"/>
+      <c r="BC54" s="47"/>
       <c r="BE54" s="8"/>
-      <c r="BF54" s="8"/>
       <c r="BG54" s="8"/>
       <c r="BH54" s="9"/>
       <c r="BI54" s="10"/>
@@ -14925,22 +14878,22 @@
       <c r="HR54" s="8"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="87" t="s">
+      <c r="A55" s="78" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="78" t="s">
+      <c r="B55" s="83" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="80" t="s">
+      <c r="C55" s="79" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="79" t="s">
+      <c r="E55" s="82" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="81" t="s">
+      <c r="F55" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="8"/>
@@ -14984,12 +14937,11 @@
       <c r="AT55" s="68"/>
       <c r="AU55" s="10"/>
       <c r="AV55" s="47"/>
-      <c r="AY55" s="74"/>
+      <c r="AY55" s="72"/>
       <c r="BA55" s="9"/>
       <c r="BB55" s="10"/>
-      <c r="BC55" s="11"/>
+      <c r="BC55" s="47"/>
       <c r="BE55" s="8"/>
-      <c r="BF55" s="8"/>
       <c r="BG55" s="8"/>
       <c r="BH55" s="9"/>
       <c r="BI55" s="10"/>
@@ -15209,12 +15161,11 @@
       <c r="AT56" s="68"/>
       <c r="AU56" s="10"/>
       <c r="AV56" s="47"/>
-      <c r="AY56" s="74"/>
+      <c r="AY56" s="72"/>
       <c r="BA56" s="9"/>
       <c r="BB56" s="10"/>
-      <c r="BC56" s="11"/>
+      <c r="BC56" s="47"/>
       <c r="BE56" s="8"/>
-      <c r="BF56" s="8"/>
       <c r="BG56" s="8"/>
       <c r="BH56" s="9"/>
       <c r="BI56" s="10"/>
@@ -15386,19 +15337,19 @@
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="77"/>
-      <c r="B57" s="78" t="s">
+      <c r="B57" s="83" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="80" t="s">
+      <c r="C57" s="79" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="79" t="s">
+      <c r="E57" s="82" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="81" t="s">
+      <c r="F57" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="8"/>
@@ -15442,12 +15393,11 @@
       <c r="AT57" s="68"/>
       <c r="AU57" s="10"/>
       <c r="AV57" s="47"/>
-      <c r="AY57" s="74"/>
+      <c r="AY57" s="72"/>
       <c r="BA57" s="9"/>
       <c r="BB57" s="10"/>
-      <c r="BC57" s="11"/>
+      <c r="BC57" s="47"/>
       <c r="BE57" s="8"/>
-      <c r="BF57" s="8"/>
       <c r="BG57" s="8"/>
       <c r="BH57" s="9"/>
       <c r="BI57" s="10"/>
@@ -15667,12 +15617,11 @@
       <c r="AT58" s="68"/>
       <c r="AU58" s="10"/>
       <c r="AV58" s="47"/>
-      <c r="AY58" s="74"/>
+      <c r="AY58" s="72"/>
       <c r="BA58" s="9"/>
       <c r="BB58" s="10"/>
-      <c r="BC58" s="11"/>
+      <c r="BC58" s="47"/>
       <c r="BE58" s="8"/>
-      <c r="BF58" s="8"/>
       <c r="BG58" s="8"/>
       <c r="BH58" s="9"/>
       <c r="BI58" s="10"/>
@@ -15844,19 +15793,19 @@
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="77"/>
-      <c r="B59" s="78" t="s">
+      <c r="B59" s="83" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="80" t="s">
+      <c r="C59" s="79" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="79" t="s">
+      <c r="E59" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="81" t="s">
+      <c r="F59" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="8"/>
@@ -15900,12 +15849,11 @@
       <c r="AT59" s="68"/>
       <c r="AU59" s="10"/>
       <c r="AV59" s="47"/>
-      <c r="AY59" s="74"/>
+      <c r="AY59" s="72"/>
       <c r="BA59" s="9"/>
       <c r="BB59" s="10"/>
-      <c r="BC59" s="11"/>
+      <c r="BC59" s="47"/>
       <c r="BE59" s="8"/>
-      <c r="BF59" s="8"/>
       <c r="BG59" s="8"/>
       <c r="BH59" s="9"/>
       <c r="BI59" s="10"/>
@@ -16125,12 +16073,11 @@
       <c r="AT60" s="68"/>
       <c r="AU60" s="10"/>
       <c r="AV60" s="47"/>
-      <c r="AY60" s="74"/>
+      <c r="AY60" s="72"/>
       <c r="BA60" s="9"/>
       <c r="BB60" s="10"/>
-      <c r="BC60" s="11"/>
+      <c r="BC60" s="47"/>
       <c r="BE60" s="8"/>
-      <c r="BF60" s="8"/>
       <c r="BG60" s="8"/>
       <c r="BH60" s="9"/>
       <c r="BI60" s="10"/>
@@ -16302,19 +16249,19 @@
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="77"/>
-      <c r="B61" s="78" t="s">
+      <c r="B61" s="83" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="80" t="s">
+      <c r="C61" s="79" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="79" t="s">
+      <c r="E61" s="82" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="81" t="s">
+      <c r="F61" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="8"/>
@@ -16358,12 +16305,11 @@
       <c r="AT61" s="68"/>
       <c r="AU61" s="10"/>
       <c r="AV61" s="47"/>
-      <c r="AY61" s="74"/>
+      <c r="AY61" s="72"/>
       <c r="BA61" s="9"/>
       <c r="BB61" s="10"/>
-      <c r="BC61" s="11"/>
+      <c r="BC61" s="47"/>
       <c r="BE61" s="8"/>
-      <c r="BF61" s="8"/>
       <c r="BG61" s="8"/>
       <c r="BH61" s="9"/>
       <c r="BI61" s="10"/>
@@ -16583,12 +16529,11 @@
       <c r="AT62" s="68"/>
       <c r="AU62" s="10"/>
       <c r="AV62" s="47"/>
-      <c r="AY62" s="74"/>
+      <c r="AY62" s="72"/>
       <c r="BA62" s="9"/>
       <c r="BB62" s="10"/>
-      <c r="BC62" s="11"/>
+      <c r="BC62" s="47"/>
       <c r="BE62" s="8"/>
-      <c r="BF62" s="8"/>
       <c r="BG62" s="8"/>
       <c r="BH62" s="9"/>
       <c r="BI62" s="10"/>
@@ -16760,19 +16705,19 @@
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="77"/>
-      <c r="B63" s="78" t="s">
+      <c r="B63" s="83" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="80" t="s">
+      <c r="C63" s="79" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="79" t="s">
+      <c r="E63" s="82" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="81" t="s">
+      <c r="F63" s="84" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="8"/>
@@ -16816,12 +16761,11 @@
       <c r="AT63" s="68"/>
       <c r="AU63" s="10"/>
       <c r="AV63" s="47"/>
-      <c r="AY63" s="74"/>
+      <c r="AY63" s="72"/>
       <c r="BA63" s="9"/>
       <c r="BB63" s="10"/>
-      <c r="BC63" s="11"/>
+      <c r="BC63" s="47"/>
       <c r="BE63" s="8"/>
-      <c r="BF63" s="8"/>
       <c r="BG63" s="8"/>
       <c r="BH63" s="9"/>
       <c r="BI63" s="10"/>
@@ -17041,12 +16985,11 @@
       <c r="AT64" s="68"/>
       <c r="AU64" s="10"/>
       <c r="AV64" s="47"/>
-      <c r="AY64" s="74"/>
+      <c r="AY64" s="72"/>
       <c r="BA64" s="9"/>
       <c r="BB64" s="10"/>
-      <c r="BC64" s="11"/>
+      <c r="BC64" s="47"/>
       <c r="BE64" s="8"/>
-      <c r="BF64" s="8"/>
       <c r="BG64" s="8"/>
       <c r="BH64" s="9"/>
       <c r="BI64" s="10"/>
@@ -17218,19 +17161,19 @@
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="77"/>
-      <c r="B65" s="78" t="s">
+      <c r="B65" s="83" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="80" t="s">
+      <c r="C65" s="79" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="79" t="s">
+      <c r="E65" s="82" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="81" t="s">
+      <c r="F65" s="84" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="8"/>
@@ -17274,12 +17217,11 @@
       <c r="AT65" s="68"/>
       <c r="AU65" s="10"/>
       <c r="AV65" s="47"/>
-      <c r="AY65" s="74"/>
+      <c r="AY65" s="72"/>
       <c r="BA65" s="9"/>
       <c r="BB65" s="10"/>
-      <c r="BC65" s="11"/>
+      <c r="BC65" s="47"/>
       <c r="BE65" s="8"/>
-      <c r="BF65" s="8"/>
       <c r="BG65" s="8"/>
       <c r="BH65" s="9"/>
       <c r="BI65" s="10"/>
@@ -17499,12 +17441,11 @@
       <c r="AT66" s="68"/>
       <c r="AU66" s="10"/>
       <c r="AV66" s="47"/>
-      <c r="AY66" s="74"/>
+      <c r="AY66" s="72"/>
       <c r="BA66" s="9"/>
       <c r="BB66" s="10"/>
-      <c r="BC66" s="11"/>
+      <c r="BC66" s="47"/>
       <c r="BE66" s="8"/>
-      <c r="BF66" s="8"/>
       <c r="BG66" s="8"/>
       <c r="BH66" s="9"/>
       <c r="BI66" s="10"/>
@@ -17675,22 +17616,22 @@
       <c r="HR66" s="8"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="87" t="s">
+      <c r="A67" s="78" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="78" t="s">
+      <c r="B67" s="83" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="80" t="s">
+      <c r="C67" s="79" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="79" t="s">
+      <c r="E67" s="82" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="81" t="s">
+      <c r="F67" s="84" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="8"/>
@@ -17734,12 +17675,11 @@
       <c r="AT67" s="68"/>
       <c r="AU67" s="10"/>
       <c r="AV67" s="47"/>
-      <c r="AY67" s="74"/>
+      <c r="AY67" s="72"/>
       <c r="BA67" s="9"/>
       <c r="BB67" s="10"/>
-      <c r="BC67" s="11"/>
+      <c r="BC67" s="47"/>
       <c r="BE67" s="8"/>
-      <c r="BF67" s="8"/>
       <c r="BG67" s="8"/>
       <c r="BH67" s="9"/>
       <c r="BI67" s="10"/>
@@ -17960,12 +17900,11 @@
       <c r="AU68" s="10"/>
       <c r="AV68" s="47"/>
       <c r="AW68" s="61"/>
-      <c r="AY68" s="74"/>
+      <c r="AY68" s="72"/>
       <c r="BA68" s="9"/>
       <c r="BB68" s="10"/>
-      <c r="BC68" s="11"/>
+      <c r="BC68" s="47"/>
       <c r="BE68" s="8"/>
-      <c r="BF68" s="8"/>
       <c r="BG68" s="8"/>
       <c r="BH68" s="9"/>
       <c r="BI68" s="10"/>
@@ -18137,19 +18076,19 @@
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="77"/>
-      <c r="B69" s="78" t="s">
+      <c r="B69" s="83" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="80" t="s">
+      <c r="C69" s="79" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="79" t="s">
+      <c r="E69" s="82" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="81" t="s">
+      <c r="F69" s="84" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="8"/>
@@ -18200,10 +18139,10 @@
       <c r="AZ69" s="54"/>
       <c r="BA69" s="9"/>
       <c r="BB69" s="10"/>
-      <c r="BC69" s="11"/>
-      <c r="BD69" s="70"/>
+      <c r="BC69" s="47"/>
+      <c r="BD69" s="54"/>
       <c r="BE69" s="16"/>
-      <c r="BF69" s="16"/>
+      <c r="BF69" s="70"/>
       <c r="BG69" s="16"/>
       <c r="BH69" s="9"/>
       <c r="BI69" s="10"/>
@@ -18425,13 +18364,12 @@
       <c r="AV70" s="47"/>
       <c r="AW70" s="56"/>
       <c r="AX70" s="56"/>
-      <c r="AY70" s="74"/>
+      <c r="AY70" s="72"/>
       <c r="BA70" s="9"/>
       <c r="BB70" s="10"/>
-      <c r="BC70" s="11"/>
-      <c r="BD70" s="72"/>
+      <c r="BC70" s="47"/>
+      <c r="BD70" s="56"/>
       <c r="BE70" s="8"/>
-      <c r="BF70" s="8"/>
       <c r="BG70" s="8"/>
       <c r="BH70" s="9"/>
       <c r="BI70" s="10"/>
@@ -18603,19 +18541,19 @@
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="77"/>
-      <c r="B71" s="78" t="s">
+      <c r="B71" s="83" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="80" t="s">
+      <c r="C71" s="79" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="79" t="s">
+      <c r="E71" s="82" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="81" t="s">
+      <c r="F71" s="84" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="8"/>
@@ -18659,12 +18597,11 @@
       <c r="AT71" s="68"/>
       <c r="AU71" s="10"/>
       <c r="AV71" s="47"/>
-      <c r="AY71" s="74"/>
+      <c r="AY71" s="72"/>
       <c r="BA71" s="9"/>
       <c r="BB71" s="10"/>
-      <c r="BC71" s="11"/>
+      <c r="BC71" s="47"/>
       <c r="BE71" s="8"/>
-      <c r="BF71" s="8"/>
       <c r="BG71" s="8"/>
       <c r="BH71" s="9"/>
       <c r="BI71" s="10"/>
@@ -18884,12 +18821,11 @@
       <c r="AT72" s="68"/>
       <c r="AU72" s="10"/>
       <c r="AV72" s="47"/>
-      <c r="AY72" s="74"/>
+      <c r="AY72" s="72"/>
       <c r="BA72" s="9"/>
       <c r="BB72" s="10"/>
-      <c r="BC72" s="11"/>
+      <c r="BC72" s="47"/>
       <c r="BE72" s="8"/>
-      <c r="BF72" s="8"/>
       <c r="BG72" s="8"/>
       <c r="BH72" s="9"/>
       <c r="BI72" s="10"/>
@@ -19061,19 +18997,19 @@
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="77"/>
-      <c r="B73" s="78" t="s">
+      <c r="B73" s="83" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="80" t="s">
+      <c r="C73" s="79" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="79" t="s">
+      <c r="E73" s="82" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="81" t="s">
+      <c r="F73" s="84" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="8"/>
@@ -19117,12 +19053,11 @@
       <c r="AT73" s="68"/>
       <c r="AU73" s="10"/>
       <c r="AV73" s="47"/>
-      <c r="AY73" s="74"/>
+      <c r="AY73" s="72"/>
       <c r="BA73" s="9"/>
       <c r="BB73" s="10"/>
-      <c r="BC73" s="11"/>
+      <c r="BC73" s="47"/>
       <c r="BE73" s="8"/>
-      <c r="BF73" s="8"/>
       <c r="BG73" s="8"/>
       <c r="BH73" s="9"/>
       <c r="BI73" s="10"/>
@@ -19342,12 +19277,11 @@
       <c r="AT74" s="68"/>
       <c r="AU74" s="10"/>
       <c r="AV74" s="47"/>
-      <c r="AY74" s="74"/>
+      <c r="AY74" s="72"/>
       <c r="BA74" s="9"/>
       <c r="BB74" s="10"/>
-      <c r="BC74" s="11"/>
+      <c r="BC74" s="47"/>
       <c r="BE74" s="8"/>
-      <c r="BF74" s="8"/>
       <c r="BG74" s="8"/>
       <c r="BH74" s="9"/>
       <c r="BI74" s="10"/>
@@ -19519,19 +19453,19 @@
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="77"/>
-      <c r="B75" s="78" t="s">
+      <c r="B75" s="83" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="80" t="s">
+      <c r="C75" s="79" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="79" t="s">
+      <c r="E75" s="82" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="81" t="s">
+      <c r="F75" s="84" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="8"/>
@@ -19575,12 +19509,11 @@
       <c r="AT75" s="68"/>
       <c r="AU75" s="10"/>
       <c r="AV75" s="47"/>
-      <c r="AY75" s="74"/>
+      <c r="AY75" s="72"/>
       <c r="BA75" s="9"/>
       <c r="BB75" s="10"/>
-      <c r="BC75" s="11"/>
+      <c r="BC75" s="47"/>
       <c r="BE75" s="8"/>
-      <c r="BF75" s="8"/>
       <c r="BG75" s="8"/>
       <c r="BH75" s="9"/>
       <c r="BI75" s="10"/>
@@ -19800,12 +19733,11 @@
       <c r="AT76" s="68"/>
       <c r="AU76" s="10"/>
       <c r="AV76" s="47"/>
-      <c r="AY76" s="74"/>
+      <c r="AY76" s="72"/>
       <c r="BA76" s="9"/>
       <c r="BB76" s="10"/>
-      <c r="BC76" s="11"/>
+      <c r="BC76" s="47"/>
       <c r="BE76" s="8"/>
-      <c r="BF76" s="8"/>
       <c r="BG76" s="8"/>
       <c r="BH76" s="9"/>
       <c r="BI76" s="10"/>
@@ -19977,19 +19909,19 @@
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="77"/>
-      <c r="B77" s="78" t="s">
+      <c r="B77" s="83" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="80" t="s">
+      <c r="C77" s="79" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="79" t="s">
+      <c r="E77" s="82" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="81" t="s">
+      <c r="F77" s="84" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="8"/>
@@ -20033,12 +19965,11 @@
       <c r="AT77" s="68"/>
       <c r="AU77" s="10"/>
       <c r="AV77" s="47"/>
-      <c r="AY77" s="74"/>
+      <c r="AY77" s="72"/>
       <c r="BA77" s="9"/>
       <c r="BB77" s="10"/>
-      <c r="BC77" s="11"/>
+      <c r="BC77" s="47"/>
       <c r="BE77" s="8"/>
-      <c r="BF77" s="8"/>
       <c r="BG77" s="8"/>
       <c r="BH77" s="9"/>
       <c r="BI77" s="10"/>
@@ -20258,12 +20189,11 @@
       <c r="AT78" s="68"/>
       <c r="AU78" s="10"/>
       <c r="AV78" s="47"/>
-      <c r="AY78" s="74"/>
+      <c r="AY78" s="72"/>
       <c r="BA78" s="9"/>
       <c r="BB78" s="10"/>
-      <c r="BC78" s="11"/>
+      <c r="BC78" s="47"/>
       <c r="BE78" s="8"/>
-      <c r="BF78" s="8"/>
       <c r="BG78" s="8"/>
       <c r="BH78" s="9"/>
       <c r="BI78" s="10"/>
@@ -20434,22 +20364,22 @@
       <c r="HR78" s="8"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="87" t="s">
+      <c r="A79" s="78" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="78" t="s">
+      <c r="B79" s="83" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="76" t="s">
+      <c r="C79" s="86" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="79" t="s">
+      <c r="E79" s="82" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="81" t="s">
+      <c r="F79" s="84" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="8"/>
@@ -20493,12 +20423,11 @@
       <c r="AT79" s="68"/>
       <c r="AU79" s="10"/>
       <c r="AV79" s="47"/>
-      <c r="AY79" s="74"/>
+      <c r="AY79" s="72"/>
       <c r="BA79" s="9"/>
       <c r="BB79" s="10"/>
-      <c r="BC79" s="11"/>
+      <c r="BC79" s="47"/>
       <c r="BE79" s="8"/>
-      <c r="BF79" s="8"/>
       <c r="BG79" s="8"/>
       <c r="BH79" s="9"/>
       <c r="BI79" s="10"/>
@@ -20718,12 +20647,11 @@
       <c r="AT80" s="68"/>
       <c r="AU80" s="10"/>
       <c r="AV80" s="47"/>
-      <c r="AY80" s="74"/>
+      <c r="AY80" s="72"/>
       <c r="BA80" s="9"/>
       <c r="BB80" s="10"/>
-      <c r="BC80" s="11"/>
+      <c r="BC80" s="47"/>
       <c r="BE80" s="8"/>
-      <c r="BF80" s="8"/>
       <c r="BG80" s="8"/>
       <c r="BH80" s="9"/>
       <c r="BI80" s="10"/>
@@ -20895,19 +20823,19 @@
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="77"/>
-      <c r="B81" s="78" t="s">
+      <c r="B81" s="83" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="76" t="s">
+      <c r="C81" s="86" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="79" t="s">
+      <c r="E81" s="82" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="81" t="s">
+      <c r="F81" s="84" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="8"/>
@@ -20951,12 +20879,11 @@
       <c r="AT81" s="68"/>
       <c r="AU81" s="10"/>
       <c r="AV81" s="47"/>
-      <c r="AY81" s="74"/>
+      <c r="AY81" s="72"/>
       <c r="BA81" s="9"/>
       <c r="BB81" s="10"/>
-      <c r="BC81" s="11"/>
+      <c r="BC81" s="47"/>
       <c r="BE81" s="8"/>
-      <c r="BF81" s="8"/>
       <c r="BG81" s="8"/>
       <c r="BH81" s="9"/>
       <c r="BI81" s="10"/>
@@ -21176,12 +21103,11 @@
       <c r="AT82" s="68"/>
       <c r="AU82" s="10"/>
       <c r="AV82" s="47"/>
-      <c r="AY82" s="74"/>
+      <c r="AY82" s="72"/>
       <c r="BA82" s="9"/>
       <c r="BB82" s="10"/>
-      <c r="BC82" s="11"/>
+      <c r="BC82" s="47"/>
       <c r="BE82" s="8"/>
-      <c r="BF82" s="8"/>
       <c r="BG82" s="8"/>
       <c r="BH82" s="9"/>
       <c r="BI82" s="10"/>
@@ -21353,19 +21279,19 @@
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="77"/>
-      <c r="B83" s="78" t="s">
+      <c r="B83" s="83" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="80" t="s">
+      <c r="C83" s="79" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="79" t="s">
+      <c r="E83" s="82" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="81" t="s">
+      <c r="F83" s="84" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="8"/>
@@ -21409,12 +21335,11 @@
       <c r="AT83" s="68"/>
       <c r="AU83" s="10"/>
       <c r="AV83" s="47"/>
-      <c r="AY83" s="74"/>
+      <c r="AY83" s="72"/>
       <c r="BA83" s="9"/>
       <c r="BB83" s="10"/>
-      <c r="BC83" s="11"/>
+      <c r="BC83" s="47"/>
       <c r="BE83" s="8"/>
-      <c r="BF83" s="8"/>
       <c r="BG83" s="8"/>
       <c r="BH83" s="9"/>
       <c r="BI83" s="10"/>
@@ -21634,12 +21559,11 @@
       <c r="AT84" s="68"/>
       <c r="AU84" s="10"/>
       <c r="AV84" s="47"/>
-      <c r="AY84" s="74"/>
+      <c r="AY84" s="72"/>
       <c r="BA84" s="9"/>
       <c r="BB84" s="10"/>
-      <c r="BC84" s="11"/>
+      <c r="BC84" s="47"/>
       <c r="BE84" s="8"/>
-      <c r="BF84" s="8"/>
       <c r="BG84" s="8"/>
       <c r="BH84" s="9"/>
       <c r="BI84" s="10"/>
@@ -21811,19 +21735,19 @@
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="77"/>
-      <c r="B85" s="78" t="s">
+      <c r="B85" s="83" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="89" t="s">
+      <c r="C85" s="90" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="79" t="s">
+      <c r="E85" s="82" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="81"/>
+      <c r="F85" s="84"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
@@ -21865,12 +21789,11 @@
       <c r="AT85" s="68"/>
       <c r="AU85" s="10"/>
       <c r="AV85" s="47"/>
-      <c r="AY85" s="74"/>
+      <c r="AY85" s="72"/>
       <c r="BA85" s="9"/>
       <c r="BB85" s="10"/>
-      <c r="BC85" s="11"/>
+      <c r="BC85" s="47"/>
       <c r="BE85" s="8"/>
-      <c r="BF85" s="8"/>
       <c r="BG85" s="8"/>
       <c r="BH85" s="9"/>
       <c r="BI85" s="10"/>
@@ -22090,12 +22013,11 @@
       <c r="AT86" s="68"/>
       <c r="AU86" s="10"/>
       <c r="AV86" s="47"/>
-      <c r="AY86" s="74"/>
+      <c r="AY86" s="72"/>
       <c r="BA86" s="9"/>
       <c r="BB86" s="10"/>
-      <c r="BC86" s="11"/>
+      <c r="BC86" s="47"/>
       <c r="BE86" s="8"/>
-      <c r="BF86" s="8"/>
       <c r="BG86" s="8"/>
       <c r="BH86" s="9"/>
       <c r="BI86" s="10"/>
@@ -22267,20 +22189,173 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="GU1:HA1"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E75:E76"/>
     <mergeCell ref="E85:E86"/>
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="B85:B86"/>
@@ -22305,173 +22380,20 @@
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="F85:F86"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="GU1:HA1"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E39:E40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Narmalisierung und Ranges auf Konsultationsfeedback angepasst und Restrukturierungen
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31278AB-ACFE-404E-8C56-E18CBB9949AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36225C68-02FE-4663-B6A4-01E8D1768D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -980,7 +980,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1063,6 +1063,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFD966"/>
         <bgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1162,7 +1174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1272,7 +1284,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1282,20 +1305,8 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1309,9 +1320,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1600,298 +1613,300 @@
     <col min="59" max="60" width="2.140625" customWidth="1"/>
     <col min="61" max="61" width="2.140625" style="1" customWidth="1"/>
     <col min="62" max="62" width="2.140625" customWidth="1"/>
-    <col min="63" max="63" width="2.140625" style="2" customWidth="1"/>
-    <col min="64" max="226" width="2.140625" customWidth="1"/>
+    <col min="63" max="63" width="2.140625" style="1" customWidth="1"/>
+    <col min="64" max="65" width="2.140625" customWidth="1"/>
+    <col min="66" max="66" width="2.140625" style="2" customWidth="1"/>
+    <col min="67" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="82" t="s">
+      <c r="G1" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82" t="s">
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="82"/>
-      <c r="R1" s="82"/>
-      <c r="S1" s="82"/>
-      <c r="T1" s="82"/>
-      <c r="U1" s="82" t="s">
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="82"/>
-      <c r="W1" s="82"/>
-      <c r="X1" s="82"/>
-      <c r="Y1" s="82"/>
-      <c r="Z1" s="82"/>
-      <c r="AA1" s="82"/>
-      <c r="AB1" s="82" t="s">
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="82"/>
-      <c r="AD1" s="82"/>
-      <c r="AE1" s="82"/>
-      <c r="AF1" s="82"/>
-      <c r="AG1" s="82"/>
-      <c r="AH1" s="82"/>
-      <c r="AI1" s="82" t="s">
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="82"/>
-      <c r="AK1" s="82"/>
-      <c r="AL1" s="82"/>
-      <c r="AM1" s="82"/>
-      <c r="AN1" s="82"/>
-      <c r="AO1" s="82"/>
-      <c r="AP1" s="82" t="s">
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="69"/>
+      <c r="AM1" s="69"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="82"/>
-      <c r="AR1" s="82"/>
-      <c r="AS1" s="82"/>
-      <c r="AT1" s="82"/>
-      <c r="AU1" s="82"/>
-      <c r="AV1" s="82"/>
-      <c r="AW1" s="82" t="s">
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="69"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="82"/>
-      <c r="AY1" s="82"/>
-      <c r="AZ1" s="82"/>
-      <c r="BA1" s="82"/>
-      <c r="BB1" s="82"/>
-      <c r="BC1" s="82"/>
-      <c r="BD1" s="82" t="s">
+      <c r="AX1" s="69"/>
+      <c r="AY1" s="69"/>
+      <c r="AZ1" s="69"/>
+      <c r="BA1" s="69"/>
+      <c r="BB1" s="69"/>
+      <c r="BC1" s="69"/>
+      <c r="BD1" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="82"/>
-      <c r="BF1" s="82"/>
-      <c r="BG1" s="82"/>
-      <c r="BH1" s="82"/>
-      <c r="BI1" s="82"/>
-      <c r="BJ1" s="82"/>
-      <c r="BK1" s="82" t="s">
+      <c r="BE1" s="69"/>
+      <c r="BF1" s="69"/>
+      <c r="BG1" s="69"/>
+      <c r="BH1" s="69"/>
+      <c r="BI1" s="69"/>
+      <c r="BJ1" s="69"/>
+      <c r="BK1" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="82"/>
-      <c r="BM1" s="82"/>
-      <c r="BN1" s="82"/>
-      <c r="BO1" s="82"/>
-      <c r="BP1" s="82"/>
-      <c r="BQ1" s="82"/>
-      <c r="BR1" s="82" t="s">
+      <c r="BL1" s="69"/>
+      <c r="BM1" s="69"/>
+      <c r="BN1" s="69"/>
+      <c r="BO1" s="69"/>
+      <c r="BP1" s="69"/>
+      <c r="BQ1" s="69"/>
+      <c r="BR1" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="82"/>
-      <c r="BT1" s="82"/>
-      <c r="BU1" s="82"/>
-      <c r="BV1" s="82"/>
-      <c r="BW1" s="82"/>
-      <c r="BX1" s="82"/>
-      <c r="BY1" s="82" t="s">
+      <c r="BS1" s="69"/>
+      <c r="BT1" s="69"/>
+      <c r="BU1" s="69"/>
+      <c r="BV1" s="69"/>
+      <c r="BW1" s="69"/>
+      <c r="BX1" s="69"/>
+      <c r="BY1" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="82"/>
-      <c r="CA1" s="82"/>
-      <c r="CB1" s="82"/>
-      <c r="CC1" s="82"/>
-      <c r="CD1" s="82"/>
-      <c r="CE1" s="82"/>
-      <c r="CF1" s="82" t="s">
+      <c r="BZ1" s="69"/>
+      <c r="CA1" s="69"/>
+      <c r="CB1" s="69"/>
+      <c r="CC1" s="69"/>
+      <c r="CD1" s="69"/>
+      <c r="CE1" s="69"/>
+      <c r="CF1" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="82"/>
-      <c r="CH1" s="82"/>
-      <c r="CI1" s="82"/>
-      <c r="CJ1" s="82"/>
-      <c r="CK1" s="82"/>
-      <c r="CL1" s="82"/>
-      <c r="CM1" s="82" t="s">
+      <c r="CG1" s="69"/>
+      <c r="CH1" s="69"/>
+      <c r="CI1" s="69"/>
+      <c r="CJ1" s="69"/>
+      <c r="CK1" s="69"/>
+      <c r="CL1" s="69"/>
+      <c r="CM1" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="82"/>
-      <c r="CO1" s="82"/>
-      <c r="CP1" s="82"/>
-      <c r="CQ1" s="82"/>
-      <c r="CR1" s="82"/>
-      <c r="CS1" s="82"/>
-      <c r="CT1" s="82" t="s">
+      <c r="CN1" s="69"/>
+      <c r="CO1" s="69"/>
+      <c r="CP1" s="69"/>
+      <c r="CQ1" s="69"/>
+      <c r="CR1" s="69"/>
+      <c r="CS1" s="69"/>
+      <c r="CT1" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="82"/>
-      <c r="CV1" s="82"/>
-      <c r="CW1" s="82"/>
-      <c r="CX1" s="82"/>
-      <c r="CY1" s="82"/>
-      <c r="CZ1" s="82"/>
-      <c r="DA1" s="82" t="s">
+      <c r="CU1" s="69"/>
+      <c r="CV1" s="69"/>
+      <c r="CW1" s="69"/>
+      <c r="CX1" s="69"/>
+      <c r="CY1" s="69"/>
+      <c r="CZ1" s="69"/>
+      <c r="DA1" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="82"/>
-      <c r="DC1" s="82"/>
-      <c r="DD1" s="82"/>
-      <c r="DE1" s="82"/>
-      <c r="DF1" s="82"/>
-      <c r="DG1" s="82"/>
-      <c r="DH1" s="82" t="s">
+      <c r="DB1" s="69"/>
+      <c r="DC1" s="69"/>
+      <c r="DD1" s="69"/>
+      <c r="DE1" s="69"/>
+      <c r="DF1" s="69"/>
+      <c r="DG1" s="69"/>
+      <c r="DH1" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="82"/>
-      <c r="DJ1" s="82"/>
-      <c r="DK1" s="82"/>
-      <c r="DL1" s="82"/>
-      <c r="DM1" s="82"/>
-      <c r="DN1" s="82"/>
-      <c r="DO1" s="82" t="s">
+      <c r="DI1" s="69"/>
+      <c r="DJ1" s="69"/>
+      <c r="DK1" s="69"/>
+      <c r="DL1" s="69"/>
+      <c r="DM1" s="69"/>
+      <c r="DN1" s="69"/>
+      <c r="DO1" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="82"/>
-      <c r="DQ1" s="82"/>
-      <c r="DR1" s="82"/>
-      <c r="DS1" s="82"/>
-      <c r="DT1" s="82"/>
-      <c r="DU1" s="82"/>
-      <c r="DV1" s="82" t="s">
+      <c r="DP1" s="69"/>
+      <c r="DQ1" s="69"/>
+      <c r="DR1" s="69"/>
+      <c r="DS1" s="69"/>
+      <c r="DT1" s="69"/>
+      <c r="DU1" s="69"/>
+      <c r="DV1" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="82"/>
-      <c r="DX1" s="82"/>
-      <c r="DY1" s="82"/>
-      <c r="DZ1" s="82"/>
-      <c r="EA1" s="82"/>
-      <c r="EB1" s="82"/>
-      <c r="EC1" s="82" t="s">
+      <c r="DW1" s="69"/>
+      <c r="DX1" s="69"/>
+      <c r="DY1" s="69"/>
+      <c r="DZ1" s="69"/>
+      <c r="EA1" s="69"/>
+      <c r="EB1" s="69"/>
+      <c r="EC1" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="82"/>
-      <c r="EE1" s="82"/>
-      <c r="EF1" s="82"/>
-      <c r="EG1" s="82"/>
-      <c r="EH1" s="82"/>
-      <c r="EI1" s="82"/>
-      <c r="EJ1" s="82" t="s">
+      <c r="ED1" s="69"/>
+      <c r="EE1" s="69"/>
+      <c r="EF1" s="69"/>
+      <c r="EG1" s="69"/>
+      <c r="EH1" s="69"/>
+      <c r="EI1" s="69"/>
+      <c r="EJ1" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="82"/>
-      <c r="EL1" s="82"/>
-      <c r="EM1" s="82"/>
-      <c r="EN1" s="82"/>
-      <c r="EO1" s="82"/>
-      <c r="EP1" s="82"/>
-      <c r="EQ1" s="82" t="s">
+      <c r="EK1" s="69"/>
+      <c r="EL1" s="69"/>
+      <c r="EM1" s="69"/>
+      <c r="EN1" s="69"/>
+      <c r="EO1" s="69"/>
+      <c r="EP1" s="69"/>
+      <c r="EQ1" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="82"/>
-      <c r="ES1" s="82"/>
-      <c r="ET1" s="82"/>
-      <c r="EU1" s="82"/>
-      <c r="EV1" s="82"/>
-      <c r="EW1" s="82"/>
-      <c r="EX1" s="82" t="s">
+      <c r="ER1" s="69"/>
+      <c r="ES1" s="69"/>
+      <c r="ET1" s="69"/>
+      <c r="EU1" s="69"/>
+      <c r="EV1" s="69"/>
+      <c r="EW1" s="69"/>
+      <c r="EX1" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="82"/>
-      <c r="EZ1" s="82"/>
-      <c r="FA1" s="82"/>
-      <c r="FB1" s="82"/>
-      <c r="FC1" s="82"/>
-      <c r="FD1" s="82"/>
-      <c r="FE1" s="82" t="s">
+      <c r="EY1" s="69"/>
+      <c r="EZ1" s="69"/>
+      <c r="FA1" s="69"/>
+      <c r="FB1" s="69"/>
+      <c r="FC1" s="69"/>
+      <c r="FD1" s="69"/>
+      <c r="FE1" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="82"/>
-      <c r="FG1" s="82"/>
-      <c r="FH1" s="82"/>
-      <c r="FI1" s="82"/>
-      <c r="FJ1" s="82"/>
-      <c r="FK1" s="82"/>
-      <c r="FL1" s="82" t="s">
+      <c r="FF1" s="69"/>
+      <c r="FG1" s="69"/>
+      <c r="FH1" s="69"/>
+      <c r="FI1" s="69"/>
+      <c r="FJ1" s="69"/>
+      <c r="FK1" s="69"/>
+      <c r="FL1" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="82"/>
-      <c r="FN1" s="82"/>
-      <c r="FO1" s="82"/>
-      <c r="FP1" s="82"/>
-      <c r="FQ1" s="82"/>
-      <c r="FR1" s="82"/>
-      <c r="FS1" s="82" t="s">
+      <c r="FM1" s="69"/>
+      <c r="FN1" s="69"/>
+      <c r="FO1" s="69"/>
+      <c r="FP1" s="69"/>
+      <c r="FQ1" s="69"/>
+      <c r="FR1" s="69"/>
+      <c r="FS1" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="82"/>
-      <c r="FU1" s="82"/>
-      <c r="FV1" s="82"/>
-      <c r="FW1" s="82"/>
-      <c r="FX1" s="82"/>
-      <c r="FY1" s="82"/>
-      <c r="FZ1" s="82" t="s">
+      <c r="FT1" s="69"/>
+      <c r="FU1" s="69"/>
+      <c r="FV1" s="69"/>
+      <c r="FW1" s="69"/>
+      <c r="FX1" s="69"/>
+      <c r="FY1" s="69"/>
+      <c r="FZ1" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="82"/>
-      <c r="GB1" s="82"/>
-      <c r="GC1" s="82"/>
-      <c r="GD1" s="82"/>
-      <c r="GE1" s="82"/>
-      <c r="GF1" s="82"/>
-      <c r="GG1" s="82" t="s">
+      <c r="GA1" s="69"/>
+      <c r="GB1" s="69"/>
+      <c r="GC1" s="69"/>
+      <c r="GD1" s="69"/>
+      <c r="GE1" s="69"/>
+      <c r="GF1" s="69"/>
+      <c r="GG1" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="82"/>
-      <c r="GI1" s="82"/>
-      <c r="GJ1" s="82"/>
-      <c r="GK1" s="82"/>
-      <c r="GL1" s="82"/>
-      <c r="GM1" s="82"/>
-      <c r="GN1" s="82" t="s">
+      <c r="GH1" s="69"/>
+      <c r="GI1" s="69"/>
+      <c r="GJ1" s="69"/>
+      <c r="GK1" s="69"/>
+      <c r="GL1" s="69"/>
+      <c r="GM1" s="69"/>
+      <c r="GN1" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="82"/>
-      <c r="GP1" s="82"/>
-      <c r="GQ1" s="82"/>
-      <c r="GR1" s="82"/>
-      <c r="GS1" s="82"/>
-      <c r="GT1" s="82"/>
-      <c r="GU1" s="82" t="s">
+      <c r="GO1" s="69"/>
+      <c r="GP1" s="69"/>
+      <c r="GQ1" s="69"/>
+      <c r="GR1" s="69"/>
+      <c r="GS1" s="69"/>
+      <c r="GT1" s="69"/>
+      <c r="GU1" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="82"/>
-      <c r="GW1" s="82"/>
-      <c r="GX1" s="82"/>
-      <c r="GY1" s="82"/>
-      <c r="GZ1" s="82"/>
-      <c r="HA1" s="82"/>
-      <c r="HB1" s="82" t="s">
+      <c r="GV1" s="69"/>
+      <c r="GW1" s="69"/>
+      <c r="GX1" s="69"/>
+      <c r="GY1" s="69"/>
+      <c r="GZ1" s="69"/>
+      <c r="HA1" s="69"/>
+      <c r="HB1" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="82"/>
-      <c r="HD1" s="82"/>
-      <c r="HE1" s="82"/>
-      <c r="HF1" s="82"/>
-      <c r="HG1" s="82"/>
-      <c r="HH1" s="82"/>
-      <c r="HI1" s="82" t="s">
+      <c r="HC1" s="69"/>
+      <c r="HD1" s="69"/>
+      <c r="HE1" s="69"/>
+      <c r="HF1" s="69"/>
+      <c r="HG1" s="69"/>
+      <c r="HH1" s="69"/>
+      <c r="HI1" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="82"/>
-      <c r="HK1" s="82"/>
-      <c r="HL1" s="82"/>
-      <c r="HM1" s="82"/>
-      <c r="HN1" s="82"/>
-      <c r="HO1" s="82"/>
-      <c r="HP1" s="82" t="s">
+      <c r="HJ1" s="69"/>
+      <c r="HK1" s="69"/>
+      <c r="HL1" s="69"/>
+      <c r="HM1" s="69"/>
+      <c r="HN1" s="69"/>
+      <c r="HO1" s="69"/>
+      <c r="HP1" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="82"/>
-      <c r="HR1" s="82"/>
+      <c r="HQ1" s="69"/>
+      <c r="HR1" s="69"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3" t="s">
@@ -2065,7 +2080,7 @@
       <c r="BJ2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="BK2" s="7" t="s">
+      <c r="BK2" s="6" t="s">
         <v>34</v>
       </c>
       <c r="BL2" s="4" t="s">
@@ -2074,7 +2089,7 @@
       <c r="BM2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BN2" s="7" t="s">
         <v>35</v>
       </c>
       <c r="BO2" s="4" t="s">
@@ -2730,7 +2745,7 @@
       <c r="BJ3" s="8">
         <v>46306</v>
       </c>
-      <c r="BK3" s="10">
+      <c r="BK3" s="9">
         <v>46307</v>
       </c>
       <c r="BL3" s="8">
@@ -2739,7 +2754,7 @@
       <c r="BM3" s="8">
         <v>46309</v>
       </c>
-      <c r="BN3" s="8">
+      <c r="BN3" s="10">
         <v>46310</v>
       </c>
       <c r="BO3" s="8">
@@ -3296,10 +3311,10 @@
       <c r="BH4" s="12"/>
       <c r="BI4" s="13"/>
       <c r="BJ4" s="12"/>
-      <c r="BK4" s="14"/>
+      <c r="BK4" s="13"/>
       <c r="BL4" s="12"/>
       <c r="BM4" s="12"/>
-      <c r="BN4" s="12"/>
+      <c r="BN4" s="14"/>
       <c r="BO4" s="12"/>
       <c r="BP4" s="12"/>
       <c r="BQ4" s="12"/>
@@ -3462,20 +3477,20 @@
       <c r="HR4" s="12"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="75" t="s">
+      <c r="B5" s="71"/>
+      <c r="C5" s="72" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="70" t="s">
+      <c r="E5" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="71"/>
+      <c r="F5" s="74"/>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
       <c r="I5" s="17"/>
@@ -3525,10 +3540,9 @@
       <c r="BG5" s="17"/>
       <c r="BH5" s="22"/>
       <c r="BI5" s="21"/>
-      <c r="BJ5" s="20"/>
+      <c r="BJ5" s="21"/>
       <c r="BL5" s="17"/>
       <c r="BM5" s="17"/>
-      <c r="BN5" s="17"/>
       <c r="BO5" s="18"/>
       <c r="BP5" s="19"/>
       <c r="BQ5" s="20"/>
@@ -3691,14 +3705,14 @@
       <c r="HR5" s="17"/>
     </row>
     <row r="6" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="77"/>
-      <c r="B6" s="77"/>
-      <c r="C6" s="77"/>
+      <c r="A6" s="70"/>
+      <c r="B6" s="70"/>
+      <c r="C6" s="70"/>
       <c r="D6" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
       <c r="G6" s="17"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
@@ -3748,10 +3762,9 @@
       <c r="BG6" s="17"/>
       <c r="BH6" s="22"/>
       <c r="BI6" s="21"/>
-      <c r="BJ6" s="20"/>
+      <c r="BJ6" s="21"/>
       <c r="BL6" s="17"/>
       <c r="BM6" s="17"/>
-      <c r="BN6" s="17"/>
       <c r="BO6" s="18"/>
       <c r="BP6" s="19"/>
       <c r="BQ6" s="20"/>
@@ -3914,18 +3927,18 @@
       <c r="HR6" s="17"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="77"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="75" t="s">
+      <c r="A7" s="70"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="72" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="70" t="s">
+      <c r="E7" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="71"/>
+      <c r="F7" s="74"/>
       <c r="G7" s="17"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -3975,10 +3988,9 @@
       <c r="BG7" s="17"/>
       <c r="BH7" s="22"/>
       <c r="BI7" s="21"/>
-      <c r="BJ7" s="20"/>
+      <c r="BJ7" s="21"/>
       <c r="BL7" s="17"/>
       <c r="BM7" s="17"/>
-      <c r="BN7" s="17"/>
       <c r="BO7" s="18"/>
       <c r="BP7" s="19"/>
       <c r="BQ7" s="20"/>
@@ -4141,14 +4153,14 @@
       <c r="HR7" s="17"/>
     </row>
     <row r="8" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="77"/>
-      <c r="B8" s="77"/>
-      <c r="C8" s="77"/>
+      <c r="A8" s="70"/>
+      <c r="B8" s="70"/>
+      <c r="C8" s="70"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="70"/>
-      <c r="F8" s="70"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="73"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
@@ -4198,10 +4210,9 @@
       <c r="BG8" s="17"/>
       <c r="BH8" s="22"/>
       <c r="BI8" s="21"/>
-      <c r="BJ8" s="20"/>
+      <c r="BJ8" s="21"/>
       <c r="BL8" s="17"/>
       <c r="BM8" s="17"/>
-      <c r="BN8" s="17"/>
       <c r="BO8" s="18"/>
       <c r="BP8" s="19"/>
       <c r="BQ8" s="20"/>
@@ -4364,18 +4375,18 @@
       <c r="HR8" s="17"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="77"/>
-      <c r="B9" s="73"/>
-      <c r="C9" s="75" t="s">
+      <c r="A9" s="70"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="72" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="70" t="s">
+      <c r="E9" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="71"/>
+      <c r="F9" s="74"/>
       <c r="G9" s="17"/>
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
@@ -4425,10 +4436,9 @@
       <c r="BG9" s="17"/>
       <c r="BH9" s="22"/>
       <c r="BI9" s="21"/>
-      <c r="BJ9" s="20"/>
+      <c r="BJ9" s="21"/>
       <c r="BL9" s="17"/>
       <c r="BM9" s="17"/>
-      <c r="BN9" s="17"/>
       <c r="BO9" s="18"/>
       <c r="BP9" s="19"/>
       <c r="BQ9" s="20"/>
@@ -4591,14 +4601,14 @@
       <c r="HR9" s="17"/>
     </row>
     <row r="10" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="77"/>
-      <c r="B10" s="77"/>
-      <c r="C10" s="77"/>
+      <c r="A10" s="70"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
       <c r="D10" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="70"/>
-      <c r="F10" s="70"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -4648,10 +4658,9 @@
       <c r="BG10" s="17"/>
       <c r="BH10" s="22"/>
       <c r="BI10" s="21"/>
-      <c r="BJ10" s="20"/>
+      <c r="BJ10" s="21"/>
       <c r="BL10" s="17"/>
       <c r="BM10" s="17"/>
-      <c r="BN10" s="17"/>
       <c r="BO10" s="18"/>
       <c r="BP10" s="19"/>
       <c r="BQ10" s="20"/>
@@ -4814,18 +4823,18 @@
       <c r="HR10" s="17"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="77"/>
-      <c r="B11" s="73"/>
-      <c r="C11" s="75" t="s">
+      <c r="A11" s="70"/>
+      <c r="B11" s="71"/>
+      <c r="C11" s="72" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="70" t="s">
+      <c r="E11" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="71"/>
+      <c r="F11" s="74"/>
       <c r="G11" s="17"/>
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
@@ -4875,10 +4884,9 @@
       <c r="BG11" s="17"/>
       <c r="BH11" s="22"/>
       <c r="BI11" s="21"/>
-      <c r="BJ11" s="20"/>
+      <c r="BJ11" s="21"/>
       <c r="BL11" s="17"/>
       <c r="BM11" s="17"/>
-      <c r="BN11" s="17"/>
       <c r="BO11" s="18"/>
       <c r="BP11" s="19"/>
       <c r="BQ11" s="20"/>
@@ -5041,14 +5049,14 @@
       <c r="HR11" s="17"/>
     </row>
     <row r="12" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="77"/>
-      <c r="B12" s="77"/>
-      <c r="C12" s="77"/>
+      <c r="A12" s="70"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
       <c r="D12" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="70"/>
-      <c r="F12" s="70"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -5098,10 +5106,9 @@
       <c r="BG12" s="17"/>
       <c r="BH12" s="22"/>
       <c r="BI12" s="21"/>
-      <c r="BJ12" s="20"/>
+      <c r="BJ12" s="21"/>
       <c r="BL12" s="17"/>
       <c r="BM12" s="17"/>
-      <c r="BN12" s="17"/>
       <c r="BO12" s="18"/>
       <c r="BP12" s="19"/>
       <c r="BQ12" s="20"/>
@@ -5264,18 +5271,18 @@
       <c r="HR12" s="17"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="77"/>
-      <c r="B13" s="73"/>
-      <c r="C13" s="75" t="s">
+      <c r="A13" s="70"/>
+      <c r="B13" s="71"/>
+      <c r="C13" s="72" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="70" t="s">
+      <c r="E13" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="71"/>
+      <c r="F13" s="74"/>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
       <c r="I13" s="17"/>
@@ -5325,10 +5332,9 @@
       <c r="BG13" s="17"/>
       <c r="BH13" s="22"/>
       <c r="BI13" s="21"/>
-      <c r="BJ13" s="20"/>
+      <c r="BJ13" s="21"/>
       <c r="BL13" s="17"/>
       <c r="BM13" s="17"/>
-      <c r="BN13" s="17"/>
       <c r="BO13" s="18"/>
       <c r="BP13" s="19"/>
       <c r="BQ13" s="20"/>
@@ -5491,14 +5497,14 @@
       <c r="HR13" s="17"/>
     </row>
     <row r="14" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="77"/>
-      <c r="B14" s="77"/>
-      <c r="C14" s="77"/>
+      <c r="A14" s="70"/>
+      <c r="B14" s="70"/>
+      <c r="C14" s="70"/>
       <c r="D14" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -5548,10 +5554,9 @@
       <c r="BG14" s="17"/>
       <c r="BH14" s="22"/>
       <c r="BI14" s="21"/>
-      <c r="BJ14" s="20"/>
+      <c r="BJ14" s="21"/>
       <c r="BL14" s="17"/>
       <c r="BM14" s="17"/>
-      <c r="BN14" s="17"/>
       <c r="BO14" s="18"/>
       <c r="BP14" s="19"/>
       <c r="BQ14" s="20"/>
@@ -5714,18 +5719,18 @@
       <c r="HR14" s="17"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="77"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="75" t="s">
+      <c r="A15" s="70"/>
+      <c r="B15" s="71"/>
+      <c r="C15" s="72" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="70" t="s">
+      <c r="E15" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="71"/>
+      <c r="F15" s="74"/>
       <c r="G15" s="17"/>
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
@@ -5775,10 +5780,9 @@
       <c r="BG15" s="17"/>
       <c r="BH15" s="22"/>
       <c r="BI15" s="21"/>
-      <c r="BJ15" s="20"/>
+      <c r="BJ15" s="21"/>
       <c r="BL15" s="17"/>
       <c r="BM15" s="17"/>
-      <c r="BN15" s="17"/>
       <c r="BO15" s="18"/>
       <c r="BP15" s="19"/>
       <c r="BQ15" s="20"/>
@@ -5941,14 +5945,14 @@
       <c r="HR15" s="17"/>
     </row>
     <row r="16" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="77"/>
-      <c r="B16" s="77"/>
-      <c r="C16" s="77"/>
+      <c r="A16" s="70"/>
+      <c r="B16" s="70"/>
+      <c r="C16" s="70"/>
       <c r="D16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
+      <c r="E16" s="73"/>
+      <c r="F16" s="73"/>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -5998,10 +6002,9 @@
       <c r="BG16" s="17"/>
       <c r="BH16" s="22"/>
       <c r="BI16" s="21"/>
-      <c r="BJ16" s="20"/>
+      <c r="BJ16" s="21"/>
       <c r="BL16" s="17"/>
       <c r="BM16" s="17"/>
-      <c r="BN16" s="17"/>
       <c r="BO16" s="18"/>
       <c r="BP16" s="19"/>
       <c r="BQ16" s="20"/>
@@ -6164,18 +6167,18 @@
       <c r="HR16" s="17"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="77"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="75" t="s">
+      <c r="A17" s="70"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="72" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="70" t="s">
+      <c r="E17" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="71"/>
+      <c r="F17" s="74"/>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
@@ -6225,10 +6228,9 @@
       <c r="BG17" s="17"/>
       <c r="BH17" s="22"/>
       <c r="BI17" s="21"/>
-      <c r="BJ17" s="20"/>
+      <c r="BJ17" s="21"/>
       <c r="BL17" s="17"/>
       <c r="BM17" s="17"/>
-      <c r="BN17" s="17"/>
       <c r="BO17" s="18"/>
       <c r="BP17" s="19"/>
       <c r="BQ17" s="20"/>
@@ -6391,14 +6393,14 @@
       <c r="HR17" s="17"/>
     </row>
     <row r="18" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="77"/>
-      <c r="B18" s="77"/>
-      <c r="C18" s="77"/>
+      <c r="A18" s="70"/>
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
       <c r="D18" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="70"/>
-      <c r="F18" s="70"/>
+      <c r="E18" s="73"/>
+      <c r="F18" s="73"/>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -6448,10 +6450,9 @@
       <c r="BG18" s="17"/>
       <c r="BH18" s="22"/>
       <c r="BI18" s="21"/>
-      <c r="BJ18" s="20"/>
+      <c r="BJ18" s="21"/>
       <c r="BL18" s="17"/>
       <c r="BM18" s="17"/>
-      <c r="BN18" s="17"/>
       <c r="BO18" s="18"/>
       <c r="BP18" s="19"/>
       <c r="BQ18" s="20"/>
@@ -6614,18 +6615,18 @@
       <c r="HR18" s="17"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="77"/>
-      <c r="B19" s="73"/>
-      <c r="C19" s="75" t="s">
+      <c r="A19" s="70"/>
+      <c r="B19" s="71"/>
+      <c r="C19" s="72" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="70" t="s">
+      <c r="E19" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="71"/>
+      <c r="F19" s="74"/>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
@@ -6675,10 +6676,9 @@
       <c r="BG19" s="17"/>
       <c r="BH19" s="22"/>
       <c r="BI19" s="21"/>
-      <c r="BJ19" s="20"/>
+      <c r="BJ19" s="21"/>
       <c r="BL19" s="17"/>
       <c r="BM19" s="17"/>
-      <c r="BN19" s="17"/>
       <c r="BO19" s="18"/>
       <c r="BP19" s="19"/>
       <c r="BQ19" s="20"/>
@@ -6841,14 +6841,14 @@
       <c r="HR19" s="17"/>
     </row>
     <row r="20" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="77"/>
-      <c r="B20" s="77"/>
-      <c r="C20" s="77"/>
+      <c r="A20" s="70"/>
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
       <c r="D20" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="73"/>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
@@ -6898,10 +6898,9 @@
       <c r="BG20" s="17"/>
       <c r="BH20" s="22"/>
       <c r="BI20" s="21"/>
-      <c r="BJ20" s="20"/>
+      <c r="BJ20" s="21"/>
       <c r="BL20" s="17"/>
       <c r="BM20" s="17"/>
-      <c r="BN20" s="17"/>
       <c r="BO20" s="18"/>
       <c r="BP20" s="19"/>
       <c r="BQ20" s="20"/>
@@ -7064,18 +7063,18 @@
       <c r="HR20" s="17"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="77"/>
-      <c r="B21" s="78"/>
-      <c r="C21" s="79" t="s">
+      <c r="A21" s="70"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="78" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="80" t="s">
+      <c r="E21" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="81"/>
+      <c r="F21" s="80"/>
       <c r="G21" s="17"/>
       <c r="H21" s="17"/>
       <c r="I21" s="17"/>
@@ -7125,10 +7124,9 @@
       <c r="BG21" s="17"/>
       <c r="BH21" s="22"/>
       <c r="BI21" s="21"/>
-      <c r="BJ21" s="20"/>
+      <c r="BJ21" s="21"/>
       <c r="BL21" s="17"/>
       <c r="BM21" s="17"/>
-      <c r="BN21" s="17"/>
       <c r="BO21" s="18"/>
       <c r="BP21" s="19"/>
       <c r="BQ21" s="20"/>
@@ -7291,14 +7289,14 @@
       <c r="HR21" s="17"/>
     </row>
     <row r="22" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="77"/>
-      <c r="B22" s="77"/>
-      <c r="C22" s="77"/>
+      <c r="A22" s="70"/>
+      <c r="B22" s="70"/>
+      <c r="C22" s="70"/>
       <c r="D22" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="80"/>
-      <c r="F22" s="80"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
       <c r="G22" s="30"/>
       <c r="H22" s="30"/>
       <c r="I22" s="30"/>
@@ -7348,11 +7346,10 @@
       <c r="BG22" s="30"/>
       <c r="BH22" s="66"/>
       <c r="BI22" s="21"/>
-      <c r="BJ22" s="33"/>
-      <c r="BK22" s="67"/>
+      <c r="BJ22" s="35"/>
       <c r="BL22" s="30"/>
       <c r="BM22" s="30"/>
-      <c r="BN22" s="30"/>
+      <c r="BN22" s="67"/>
       <c r="BO22" s="31"/>
       <c r="BP22" s="32"/>
       <c r="BQ22" s="33"/>
@@ -7515,22 +7512,22 @@
       <c r="HR22" s="30"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="72" t="s">
+      <c r="A23" s="75" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="73" t="s">
+      <c r="B23" s="71" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="75" t="s">
+      <c r="C23" s="72" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="70" t="s">
+      <c r="E23" s="73" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="71" t="s">
+      <c r="F23" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="17"/>
@@ -7585,11 +7582,10 @@
       <c r="BG23" s="17"/>
       <c r="BH23" s="22"/>
       <c r="BI23" s="21"/>
-      <c r="BJ23" s="20"/>
-      <c r="BK23" s="68"/>
+      <c r="BJ23" s="21"/>
+      <c r="BK23" s="38"/>
       <c r="BL23" s="17"/>
       <c r="BM23" s="17"/>
-      <c r="BN23" s="17"/>
       <c r="BO23" s="18"/>
       <c r="BP23" s="19"/>
       <c r="BQ23" s="20"/>
@@ -7752,14 +7748,14 @@
       <c r="HR23" s="17"/>
     </row>
     <row r="24" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="72"/>
-      <c r="B24" s="72"/>
-      <c r="C24" s="72"/>
+      <c r="A24" s="75"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="75"/>
       <c r="D24" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
+      <c r="E24" s="73"/>
+      <c r="F24" s="73"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
@@ -7812,11 +7808,10 @@
       <c r="BG24" s="17"/>
       <c r="BH24" s="22"/>
       <c r="BI24" s="21"/>
-      <c r="BJ24" s="20"/>
+      <c r="BJ24" s="21"/>
       <c r="BK24" s="42"/>
       <c r="BL24" s="17"/>
       <c r="BM24" s="17"/>
-      <c r="BN24" s="17"/>
       <c r="BO24" s="18"/>
       <c r="BP24" s="19"/>
       <c r="BQ24" s="20"/>
@@ -7979,20 +7974,20 @@
       <c r="HR24" s="17"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="72"/>
-      <c r="B25" s="73" t="s">
+      <c r="A25" s="75"/>
+      <c r="B25" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="75" t="s">
+      <c r="C25" s="72" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="70" t="s">
+      <c r="E25" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="71" t="s">
+      <c r="F25" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="17"/>
@@ -8039,10 +8034,9 @@
       <c r="BC25" s="21"/>
       <c r="BH25" s="22"/>
       <c r="BI25" s="21"/>
-      <c r="BJ25" s="20"/>
+      <c r="BJ25" s="21"/>
       <c r="BL25" s="17"/>
       <c r="BM25" s="68"/>
-      <c r="BN25" s="17"/>
       <c r="BO25" s="18"/>
       <c r="BP25" s="19"/>
       <c r="BQ25" s="20"/>
@@ -8203,14 +8197,14 @@
       <c r="HS25" s="17"/>
     </row>
     <row r="26" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="72"/>
-      <c r="B26" s="72"/>
-      <c r="C26" s="72"/>
+      <c r="A26" s="75"/>
+      <c r="B26" s="75"/>
+      <c r="C26" s="75"/>
       <c r="D26" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="70"/>
-      <c r="F26" s="70"/>
+      <c r="E26" s="73"/>
+      <c r="F26" s="73"/>
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -8260,10 +8254,9 @@
       <c r="BG26" s="17"/>
       <c r="BH26" s="22"/>
       <c r="BI26" s="21"/>
-      <c r="BJ26" s="20"/>
+      <c r="BJ26" s="21"/>
       <c r="BL26" s="17"/>
-      <c r="BM26" s="17"/>
-      <c r="BN26" s="17"/>
+      <c r="BM26" s="42"/>
       <c r="BO26" s="18"/>
       <c r="BP26" s="19"/>
       <c r="BQ26" s="20"/>
@@ -8426,8 +8419,8 @@
       <c r="HR26" s="17"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="72"/>
-      <c r="B27" s="73" t="s">
+      <c r="A27" s="75"/>
+      <c r="B27" s="71" t="s">
         <v>73</v>
       </c>
       <c r="C27" s="76" t="s">
@@ -8436,10 +8429,10 @@
       <c r="D27" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="70" t="s">
+      <c r="E27" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="71"/>
+      <c r="F27" s="74"/>
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -8489,10 +8482,9 @@
       <c r="BG27" s="17"/>
       <c r="BH27" s="22"/>
       <c r="BI27" s="21"/>
-      <c r="BJ27" s="20"/>
+      <c r="BJ27" s="21"/>
       <c r="BL27" s="17"/>
       <c r="BM27" s="17"/>
-      <c r="BN27" s="17"/>
       <c r="BO27" s="18"/>
       <c r="BP27" s="19"/>
       <c r="BQ27" s="20"/>
@@ -8655,14 +8647,14 @@
       <c r="HR27" s="17"/>
     </row>
     <row r="28" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="72"/>
-      <c r="B28" s="72"/>
-      <c r="C28" s="72"/>
+      <c r="A28" s="75"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
       <c r="D28" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
+      <c r="E28" s="73"/>
+      <c r="F28" s="73"/>
       <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -8712,10 +8704,9 @@
       <c r="BG28" s="17"/>
       <c r="BH28" s="22"/>
       <c r="BI28" s="21"/>
-      <c r="BJ28" s="20"/>
+      <c r="BJ28" s="21"/>
       <c r="BL28" s="17"/>
       <c r="BM28" s="17"/>
-      <c r="BN28" s="17"/>
       <c r="BO28" s="18"/>
       <c r="BP28" s="19"/>
       <c r="BQ28" s="20"/>
@@ -8878,22 +8869,22 @@
       <c r="HR28" s="17"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="72" t="s">
+      <c r="A29" s="75" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="73" t="s">
+      <c r="B29" s="71" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="75" t="s">
+      <c r="C29" s="72" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="70" t="s">
+      <c r="E29" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="71" t="s">
+      <c r="F29" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="17"/>
@@ -8944,10 +8935,9 @@
       <c r="BG29" s="17"/>
       <c r="BH29" s="22"/>
       <c r="BI29" s="21"/>
-      <c r="BJ29" s="20"/>
+      <c r="BJ29" s="21"/>
       <c r="BL29" s="17"/>
       <c r="BM29" s="17"/>
-      <c r="BN29" s="17"/>
       <c r="BO29" s="18"/>
       <c r="BP29" s="19"/>
       <c r="BQ29" s="20"/>
@@ -9110,14 +9100,14 @@
       <c r="HR29" s="17"/>
     </row>
     <row r="30" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="72"/>
-      <c r="B30" s="72"/>
-      <c r="C30" s="72"/>
+      <c r="A30" s="75"/>
+      <c r="B30" s="75"/>
+      <c r="C30" s="75"/>
       <c r="D30" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
+      <c r="E30" s="73"/>
+      <c r="F30" s="73"/>
       <c r="G30" s="17"/>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -9167,10 +9157,9 @@
       <c r="BG30" s="17"/>
       <c r="BH30" s="22"/>
       <c r="BI30" s="21"/>
-      <c r="BJ30" s="20"/>
+      <c r="BJ30" s="21"/>
       <c r="BL30" s="17"/>
       <c r="BM30" s="17"/>
-      <c r="BN30" s="17"/>
       <c r="BO30" s="18"/>
       <c r="BP30" s="19"/>
       <c r="BQ30" s="20"/>
@@ -9333,20 +9322,20 @@
       <c r="HR30" s="17"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="72"/>
-      <c r="B31" s="73" t="s">
+      <c r="A31" s="75"/>
+      <c r="B31" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="75" t="s">
+      <c r="C31" s="72" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="70" t="s">
+      <c r="E31" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="71" t="s">
+      <c r="F31" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="17"/>
@@ -9398,10 +9387,9 @@
       <c r="BG31" s="17"/>
       <c r="BH31" s="22"/>
       <c r="BI31" s="21"/>
-      <c r="BJ31" s="20"/>
+      <c r="BJ31" s="21"/>
       <c r="BL31" s="17"/>
       <c r="BM31" s="17"/>
-      <c r="BN31" s="17"/>
       <c r="BO31" s="18"/>
       <c r="BP31" s="19"/>
       <c r="BQ31" s="20"/>
@@ -9564,14 +9552,14 @@
       <c r="HR31" s="17"/>
     </row>
     <row r="32" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="72"/>
-      <c r="B32" s="72"/>
-      <c r="C32" s="72"/>
+      <c r="A32" s="75"/>
+      <c r="B32" s="75"/>
+      <c r="C32" s="75"/>
       <c r="D32" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
+      <c r="E32" s="73"/>
+      <c r="F32" s="73"/>
       <c r="G32" s="17"/>
       <c r="H32" s="17"/>
       <c r="I32" s="17"/>
@@ -9621,10 +9609,9 @@
       <c r="BG32" s="17"/>
       <c r="BH32" s="22"/>
       <c r="BI32" s="21"/>
-      <c r="BJ32" s="20"/>
+      <c r="BJ32" s="21"/>
       <c r="BL32" s="17"/>
       <c r="BM32" s="17"/>
-      <c r="BN32" s="17"/>
       <c r="BO32" s="18"/>
       <c r="BP32" s="19"/>
       <c r="BQ32" s="20"/>
@@ -9787,20 +9774,20 @@
       <c r="HR32" s="17"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="72"/>
-      <c r="B33" s="73" t="s">
+      <c r="A33" s="75"/>
+      <c r="B33" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="75" t="s">
+      <c r="C33" s="72" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="70" t="s">
+      <c r="E33" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="71" t="s">
+      <c r="F33" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="17"/>
@@ -9852,10 +9839,9 @@
       <c r="BG33" s="17"/>
       <c r="BH33" s="22"/>
       <c r="BI33" s="21"/>
-      <c r="BJ33" s="20"/>
+      <c r="BJ33" s="21"/>
       <c r="BL33" s="17"/>
       <c r="BM33" s="17"/>
-      <c r="BN33" s="17"/>
       <c r="BO33" s="18"/>
       <c r="BP33" s="19"/>
       <c r="BQ33" s="20"/>
@@ -10018,14 +10004,14 @@
       <c r="HR33" s="17"/>
     </row>
     <row r="34" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="72"/>
-      <c r="B34" s="72"/>
-      <c r="C34" s="72"/>
+      <c r="A34" s="75"/>
+      <c r="B34" s="75"/>
+      <c r="C34" s="75"/>
       <c r="D34" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="70"/>
-      <c r="F34" s="70"/>
+      <c r="E34" s="73"/>
+      <c r="F34" s="73"/>
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
@@ -10075,10 +10061,9 @@
       <c r="BG34" s="17"/>
       <c r="BH34" s="22"/>
       <c r="BI34" s="21"/>
-      <c r="BJ34" s="20"/>
+      <c r="BJ34" s="21"/>
       <c r="BL34" s="17"/>
       <c r="BM34" s="17"/>
-      <c r="BN34" s="17"/>
       <c r="BO34" s="18"/>
       <c r="BP34" s="19"/>
       <c r="BQ34" s="20"/>
@@ -10241,20 +10226,20 @@
       <c r="HR34" s="17"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="72"/>
-      <c r="B35" s="73" t="s">
+      <c r="A35" s="75"/>
+      <c r="B35" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="75" t="s">
+      <c r="C35" s="72" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="70" t="s">
+      <c r="E35" s="73" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="71" t="s">
+      <c r="F35" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="17"/>
@@ -10307,10 +10292,9 @@
       <c r="BG35" s="39"/>
       <c r="BH35" s="22"/>
       <c r="BI35" s="21"/>
-      <c r="BJ35" s="20"/>
+      <c r="BJ35" s="21"/>
       <c r="BL35" s="17"/>
       <c r="BM35" s="17"/>
-      <c r="BN35" s="17"/>
       <c r="BO35" s="18"/>
       <c r="BP35" s="19"/>
       <c r="BQ35" s="20"/>
@@ -10473,14 +10457,14 @@
       <c r="HR35" s="17"/>
     </row>
     <row r="36" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="72"/>
-      <c r="B36" s="72"/>
-      <c r="C36" s="72"/>
+      <c r="A36" s="75"/>
+      <c r="B36" s="75"/>
+      <c r="C36" s="75"/>
       <c r="D36" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="70"/>
-      <c r="F36" s="70"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
       <c r="G36" s="17"/>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
@@ -10531,10 +10515,9 @@
       <c r="BG36" s="17"/>
       <c r="BH36" s="22"/>
       <c r="BI36" s="42"/>
-      <c r="BJ36" s="20"/>
+      <c r="BJ36" s="21"/>
       <c r="BL36" s="17"/>
       <c r="BM36" s="17"/>
-      <c r="BN36" s="17"/>
       <c r="BO36" s="18"/>
       <c r="BP36" s="19"/>
       <c r="BQ36" s="20"/>
@@ -10697,20 +10680,20 @@
       <c r="HR36" s="17"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="72"/>
-      <c r="B37" s="73" t="s">
+      <c r="A37" s="75"/>
+      <c r="B37" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="75" t="s">
+      <c r="C37" s="72" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="70" t="s">
+      <c r="E37" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="71" t="s">
+      <c r="F37" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="17"/>
@@ -10762,10 +10745,9 @@
       <c r="BG37" s="17"/>
       <c r="BH37" s="22"/>
       <c r="BI37" s="21"/>
-      <c r="BJ37" s="20"/>
+      <c r="BJ37" s="21"/>
       <c r="BL37" s="17"/>
       <c r="BM37" s="17"/>
-      <c r="BN37" s="17"/>
       <c r="BO37" s="18"/>
       <c r="BP37" s="19"/>
       <c r="BQ37" s="20"/>
@@ -10928,14 +10910,14 @@
       <c r="HR37" s="17"/>
     </row>
     <row r="38" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="72"/>
-      <c r="B38" s="72"/>
-      <c r="C38" s="72"/>
+      <c r="A38" s="75"/>
+      <c r="B38" s="75"/>
+      <c r="C38" s="75"/>
       <c r="D38" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="70"/>
-      <c r="F38" s="70"/>
+      <c r="E38" s="73"/>
+      <c r="F38" s="73"/>
       <c r="G38" s="17"/>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -10985,10 +10967,9 @@
       <c r="BG38" s="17"/>
       <c r="BH38" s="22"/>
       <c r="BI38" s="21"/>
-      <c r="BJ38" s="20"/>
+      <c r="BJ38" s="21"/>
       <c r="BL38" s="17"/>
       <c r="BM38" s="17"/>
-      <c r="BN38" s="17"/>
       <c r="BO38" s="18"/>
       <c r="BP38" s="19"/>
       <c r="BQ38" s="20"/>
@@ -11151,20 +11132,20 @@
       <c r="HR38" s="17"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="72"/>
-      <c r="B39" s="73" t="s">
+      <c r="A39" s="75"/>
+      <c r="B39" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="75" t="s">
+      <c r="C39" s="72" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="70" t="s">
+      <c r="E39" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="71" t="s">
+      <c r="F39" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="17"/>
@@ -11216,10 +11197,10 @@
       <c r="BG39" s="17"/>
       <c r="BH39" s="22"/>
       <c r="BI39" s="21"/>
-      <c r="BJ39" s="20"/>
+      <c r="BJ39" s="21"/>
       <c r="BL39" s="17"/>
       <c r="BM39" s="39"/>
-      <c r="BN39" s="39"/>
+      <c r="BN39" s="68"/>
       <c r="BO39" s="18"/>
       <c r="BP39" s="19"/>
       <c r="BQ39" s="20"/>
@@ -11382,14 +11363,14 @@
       <c r="HR39" s="17"/>
     </row>
     <row r="40" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="72"/>
-      <c r="B40" s="72"/>
-      <c r="C40" s="72"/>
+      <c r="A40" s="75"/>
+      <c r="B40" s="75"/>
+      <c r="C40" s="75"/>
       <c r="D40" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="70"/>
-      <c r="F40" s="70"/>
+      <c r="E40" s="73"/>
+      <c r="F40" s="73"/>
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
@@ -11440,10 +11421,9 @@
       <c r="BG40" s="17"/>
       <c r="BH40" s="22"/>
       <c r="BI40" s="21"/>
-      <c r="BJ40" s="20"/>
+      <c r="BJ40" s="21"/>
       <c r="BL40" s="17"/>
       <c r="BM40" s="17"/>
-      <c r="BN40" s="17"/>
       <c r="BO40" s="18"/>
       <c r="BP40" s="19"/>
       <c r="BQ40" s="20"/>
@@ -11606,22 +11586,22 @@
       <c r="HR40" s="17"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="72" t="s">
+      <c r="A41" s="75" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="73" t="s">
+      <c r="B41" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="75" t="s">
+      <c r="C41" s="72" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="70" t="s">
+      <c r="E41" s="73" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="71" t="s">
+      <c r="F41" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="17"/>
@@ -11673,10 +11653,9 @@
       <c r="BG41" s="17"/>
       <c r="BH41" s="22"/>
       <c r="BI41" s="21"/>
-      <c r="BJ41" s="20"/>
+      <c r="BJ41" s="21"/>
       <c r="BL41" s="17"/>
       <c r="BM41" s="17"/>
-      <c r="BN41" s="17"/>
       <c r="BO41" s="18"/>
       <c r="BP41" s="19"/>
       <c r="BQ41" s="20"/>
@@ -11839,14 +11818,14 @@
       <c r="HR41" s="17"/>
     </row>
     <row r="42" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="72"/>
-      <c r="B42" s="72"/>
-      <c r="C42" s="72"/>
+      <c r="A42" s="75"/>
+      <c r="B42" s="75"/>
+      <c r="C42" s="75"/>
       <c r="D42" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="70"/>
-      <c r="F42" s="70"/>
+      <c r="E42" s="73"/>
+      <c r="F42" s="73"/>
       <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
@@ -11896,10 +11875,9 @@
       <c r="BG42" s="17"/>
       <c r="BH42" s="22"/>
       <c r="BI42" s="21"/>
-      <c r="BJ42" s="20"/>
+      <c r="BJ42" s="21"/>
       <c r="BL42" s="17"/>
       <c r="BM42" s="17"/>
-      <c r="BN42" s="17"/>
       <c r="BO42" s="18"/>
       <c r="BP42" s="19"/>
       <c r="BQ42" s="20"/>
@@ -12062,20 +12040,20 @@
       <c r="HR42" s="17"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="72"/>
-      <c r="B43" s="73" t="s">
+      <c r="A43" s="75"/>
+      <c r="B43" s="71" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="75" t="s">
+      <c r="C43" s="72" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="70" t="s">
+      <c r="E43" s="73" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="71" t="s">
+      <c r="F43" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="17"/>
@@ -12126,10 +12104,9 @@
       <c r="BG43" s="17"/>
       <c r="BH43" s="22"/>
       <c r="BI43" s="21"/>
-      <c r="BJ43" s="20"/>
+      <c r="BJ43" s="21"/>
       <c r="BL43" s="17"/>
       <c r="BM43" s="17"/>
-      <c r="BN43" s="17"/>
       <c r="BO43" s="18"/>
       <c r="BP43" s="19"/>
       <c r="BQ43" s="20"/>
@@ -12292,14 +12269,14 @@
       <c r="HR43" s="17"/>
     </row>
     <row r="44" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="72"/>
-      <c r="B44" s="72"/>
-      <c r="C44" s="72"/>
+      <c r="A44" s="75"/>
+      <c r="B44" s="75"/>
+      <c r="C44" s="75"/>
       <c r="D44" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="70"/>
-      <c r="F44" s="70"/>
+      <c r="E44" s="73"/>
+      <c r="F44" s="73"/>
       <c r="G44" s="17"/>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -12351,10 +12328,9 @@
       <c r="BG44" s="17"/>
       <c r="BH44" s="22"/>
       <c r="BI44" s="21"/>
-      <c r="BJ44" s="20"/>
+      <c r="BJ44" s="21"/>
       <c r="BL44" s="17"/>
       <c r="BM44" s="17"/>
-      <c r="BN44" s="17"/>
       <c r="BO44" s="18"/>
       <c r="BP44" s="19"/>
       <c r="BQ44" s="20"/>
@@ -12517,20 +12493,20 @@
       <c r="HR44" s="17"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="72"/>
-      <c r="B45" s="73" t="s">
+      <c r="A45" s="75"/>
+      <c r="B45" s="71" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="75" t="s">
+      <c r="C45" s="72" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="70" t="s">
+      <c r="E45" s="73" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="71" t="s">
+      <c r="F45" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="17"/>
@@ -12582,10 +12558,9 @@
       <c r="BG45" s="17"/>
       <c r="BH45" s="22"/>
       <c r="BI45" s="21"/>
-      <c r="BJ45" s="20"/>
+      <c r="BJ45" s="21"/>
       <c r="BL45" s="17"/>
       <c r="BM45" s="17"/>
-      <c r="BN45" s="17"/>
       <c r="BO45" s="18"/>
       <c r="BP45" s="19"/>
       <c r="BQ45" s="20"/>
@@ -12748,14 +12723,14 @@
       <c r="HR45" s="17"/>
     </row>
     <row r="46" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="72"/>
-      <c r="B46" s="72"/>
-      <c r="C46" s="72"/>
+      <c r="A46" s="75"/>
+      <c r="B46" s="75"/>
+      <c r="C46" s="75"/>
       <c r="D46" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="70"/>
-      <c r="F46" s="70"/>
+      <c r="E46" s="73"/>
+      <c r="F46" s="73"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
@@ -12806,10 +12781,9 @@
       <c r="BG46" s="17"/>
       <c r="BH46" s="22"/>
       <c r="BI46" s="21"/>
-      <c r="BJ46" s="20"/>
+      <c r="BJ46" s="21"/>
       <c r="BL46" s="17"/>
       <c r="BM46" s="17"/>
-      <c r="BN46" s="17"/>
       <c r="BO46" s="18"/>
       <c r="BP46" s="19"/>
       <c r="BQ46" s="20"/>
@@ -12972,22 +12946,22 @@
       <c r="HR46" s="17"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="72" t="s">
+      <c r="A47" s="75" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="73" t="s">
+      <c r="B47" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="75" t="s">
+      <c r="C47" s="72" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="70" t="s">
+      <c r="E47" s="73" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="71" t="s">
+      <c r="F47" s="74" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="17"/>
@@ -13042,10 +13016,9 @@
       <c r="BG47" s="17"/>
       <c r="BH47" s="22"/>
       <c r="BI47" s="21"/>
-      <c r="BJ47" s="20"/>
+      <c r="BJ47" s="21"/>
       <c r="BL47" s="17"/>
       <c r="BM47" s="17"/>
-      <c r="BN47" s="17"/>
       <c r="BO47" s="18"/>
       <c r="BP47" s="19"/>
       <c r="BQ47" s="20"/>
@@ -13208,14 +13181,14 @@
       <c r="HR47" s="17"/>
     </row>
     <row r="48" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="72"/>
-      <c r="B48" s="72"/>
-      <c r="C48" s="72"/>
+      <c r="A48" s="75"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
       <c r="D48" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="70"/>
-      <c r="F48" s="70"/>
+      <c r="E48" s="73"/>
+      <c r="F48" s="73"/>
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
@@ -13267,10 +13240,9 @@
       <c r="BG48" s="17"/>
       <c r="BH48" s="22"/>
       <c r="BI48" s="21"/>
-      <c r="BJ48" s="20"/>
+      <c r="BJ48" s="21"/>
       <c r="BL48" s="17"/>
       <c r="BM48" s="17"/>
-      <c r="BN48" s="17"/>
       <c r="BO48" s="18"/>
       <c r="BP48" s="19"/>
       <c r="BQ48" s="20"/>
@@ -13433,20 +13405,20 @@
       <c r="HR48" s="17"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="72"/>
-      <c r="B49" s="73" t="s">
+      <c r="A49" s="75"/>
+      <c r="B49" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="75" t="s">
+      <c r="C49" s="72" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="70" t="s">
+      <c r="E49" s="73" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="71" t="s">
+      <c r="F49" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="17"/>
@@ -13498,11 +13470,10 @@
       <c r="BG49" s="17"/>
       <c r="BH49" s="22"/>
       <c r="BI49" s="21"/>
-      <c r="BJ49" s="20"/>
-      <c r="BK49" s="69"/>
+      <c r="BJ49" s="21"/>
+      <c r="BK49" s="27"/>
       <c r="BL49" s="16"/>
       <c r="BM49" s="17"/>
-      <c r="BN49" s="17"/>
       <c r="BO49" s="18"/>
       <c r="BP49" s="19"/>
       <c r="BQ49" s="20"/>
@@ -13665,14 +13636,14 @@
       <c r="HR49" s="17"/>
     </row>
     <row r="50" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="72"/>
-      <c r="B50" s="72"/>
-      <c r="C50" s="72"/>
+      <c r="A50" s="75"/>
+      <c r="B50" s="75"/>
+      <c r="C50" s="75"/>
       <c r="D50" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="70"/>
-      <c r="F50" s="70"/>
+      <c r="E50" s="73"/>
+      <c r="F50" s="73"/>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
@@ -13722,11 +13693,10 @@
       <c r="BG50" s="17"/>
       <c r="BH50" s="22"/>
       <c r="BI50" s="21"/>
-      <c r="BJ50" s="20"/>
+      <c r="BJ50" s="21"/>
       <c r="BK50" s="42"/>
-      <c r="BL50" s="17"/>
+      <c r="BL50" s="42"/>
       <c r="BM50" s="17"/>
-      <c r="BN50" s="17"/>
       <c r="BO50" s="18"/>
       <c r="BP50" s="19"/>
       <c r="BQ50" s="20"/>
@@ -13889,22 +13859,22 @@
       <c r="HR50" s="17"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="72" t="s">
+      <c r="A51" s="75" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="73" t="s">
+      <c r="B51" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="75" t="s">
+      <c r="C51" s="72" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="70" t="s">
+      <c r="E51" s="73" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="71" t="s">
+      <c r="F51" s="74" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="17"/>
@@ -13956,10 +13926,9 @@
       <c r="BG51" s="17"/>
       <c r="BH51" s="22"/>
       <c r="BI51" s="21"/>
-      <c r="BJ51" s="20"/>
+      <c r="BJ51" s="21"/>
       <c r="BL51" s="17"/>
       <c r="BM51" s="17"/>
-      <c r="BN51" s="17"/>
       <c r="BO51" s="18"/>
       <c r="BP51" s="19"/>
       <c r="BQ51" s="20"/>
@@ -14122,14 +14091,14 @@
       <c r="HR51" s="17"/>
     </row>
     <row r="52" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="72"/>
-      <c r="B52" s="72"/>
-      <c r="C52" s="72"/>
+      <c r="A52" s="75"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
       <c r="D52" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="70"/>
-      <c r="F52" s="70"/>
+      <c r="E52" s="73"/>
+      <c r="F52" s="73"/>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
@@ -14179,10 +14148,9 @@
       <c r="BG52" s="17"/>
       <c r="BH52" s="22"/>
       <c r="BI52" s="21"/>
-      <c r="BJ52" s="20"/>
+      <c r="BJ52" s="21"/>
       <c r="BL52" s="17"/>
-      <c r="BM52" s="17"/>
-      <c r="BN52" s="17"/>
+      <c r="BM52" s="82"/>
       <c r="BO52" s="18"/>
       <c r="BP52" s="19"/>
       <c r="BQ52" s="20"/>
@@ -14345,20 +14313,20 @@
       <c r="HR52" s="17"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="72"/>
-      <c r="B53" s="73" t="s">
+      <c r="A53" s="75"/>
+      <c r="B53" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="75" t="s">
+      <c r="C53" s="72" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="70" t="s">
+      <c r="E53" s="73" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="71" t="s">
+      <c r="F53" s="74" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="17"/>
@@ -14410,10 +14378,9 @@
       <c r="BG53" s="17"/>
       <c r="BH53" s="22"/>
       <c r="BI53" s="21"/>
-      <c r="BJ53" s="20"/>
+      <c r="BJ53" s="21"/>
       <c r="BL53" s="17"/>
       <c r="BM53" s="17"/>
-      <c r="BN53" s="17"/>
       <c r="BO53" s="18"/>
       <c r="BP53" s="19"/>
       <c r="BQ53" s="20"/>
@@ -14576,14 +14543,14 @@
       <c r="HR53" s="17"/>
     </row>
     <row r="54" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="72"/>
-      <c r="B54" s="72"/>
-      <c r="C54" s="72"/>
+      <c r="A54" s="75"/>
+      <c r="B54" s="75"/>
+      <c r="C54" s="75"/>
       <c r="D54" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="70"/>
-      <c r="F54" s="70"/>
+      <c r="E54" s="73"/>
+      <c r="F54" s="73"/>
       <c r="G54" s="17"/>
       <c r="H54" s="17"/>
       <c r="I54" s="17"/>
@@ -14633,10 +14600,9 @@
       <c r="BG54" s="17"/>
       <c r="BH54" s="22"/>
       <c r="BI54" s="21"/>
-      <c r="BJ54" s="20"/>
+      <c r="BJ54" s="21"/>
       <c r="BL54" s="17"/>
       <c r="BM54" s="17"/>
-      <c r="BN54" s="17"/>
       <c r="BO54" s="18"/>
       <c r="BP54" s="19"/>
       <c r="BQ54" s="20"/>
@@ -14799,22 +14765,22 @@
       <c r="HR54" s="17"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="72" t="s">
+      <c r="A55" s="75" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="73" t="s">
+      <c r="B55" s="71" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="75" t="s">
+      <c r="C55" s="72" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="70" t="s">
+      <c r="E55" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="71" t="s">
+      <c r="F55" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="17"/>
@@ -14866,10 +14832,9 @@
       <c r="BG55" s="17"/>
       <c r="BH55" s="22"/>
       <c r="BI55" s="21"/>
-      <c r="BJ55" s="20"/>
+      <c r="BJ55" s="21"/>
       <c r="BL55" s="17"/>
       <c r="BM55" s="17"/>
-      <c r="BN55" s="17"/>
       <c r="BO55" s="18"/>
       <c r="BP55" s="19"/>
       <c r="BQ55" s="20"/>
@@ -15032,14 +14997,14 @@
       <c r="HR55" s="17"/>
     </row>
     <row r="56" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="72"/>
-      <c r="B56" s="72"/>
-      <c r="C56" s="72"/>
+      <c r="A56" s="75"/>
+      <c r="B56" s="75"/>
+      <c r="C56" s="75"/>
       <c r="D56" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="70"/>
-      <c r="F56" s="70"/>
+      <c r="E56" s="73"/>
+      <c r="F56" s="73"/>
       <c r="G56" s="17"/>
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
@@ -15089,10 +15054,9 @@
       <c r="BG56" s="17"/>
       <c r="BH56" s="22"/>
       <c r="BI56" s="21"/>
-      <c r="BJ56" s="20"/>
+      <c r="BJ56" s="21"/>
       <c r="BL56" s="17"/>
       <c r="BM56" s="17"/>
-      <c r="BN56" s="17"/>
       <c r="BO56" s="18"/>
       <c r="BP56" s="19"/>
       <c r="BQ56" s="20"/>
@@ -15255,20 +15219,20 @@
       <c r="HR56" s="17"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="72"/>
-      <c r="B57" s="73" t="s">
+      <c r="A57" s="75"/>
+      <c r="B57" s="71" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="75" t="s">
+      <c r="C57" s="72" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="70" t="s">
+      <c r="E57" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="71" t="s">
+      <c r="F57" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="17"/>
@@ -15320,10 +15284,9 @@
       <c r="BG57" s="17"/>
       <c r="BH57" s="22"/>
       <c r="BI57" s="21"/>
-      <c r="BJ57" s="20"/>
+      <c r="BJ57" s="21"/>
       <c r="BL57" s="17"/>
       <c r="BM57" s="17"/>
-      <c r="BN57" s="17"/>
       <c r="BO57" s="18"/>
       <c r="BP57" s="19"/>
       <c r="BQ57" s="20"/>
@@ -15486,14 +15449,14 @@
       <c r="HR57" s="17"/>
     </row>
     <row r="58" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="72"/>
-      <c r="B58" s="72"/>
-      <c r="C58" s="72"/>
+      <c r="A58" s="75"/>
+      <c r="B58" s="75"/>
+      <c r="C58" s="75"/>
       <c r="D58" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="70"/>
-      <c r="F58" s="70"/>
+      <c r="E58" s="73"/>
+      <c r="F58" s="73"/>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
@@ -15543,10 +15506,9 @@
       <c r="BG58" s="17"/>
       <c r="BH58" s="22"/>
       <c r="BI58" s="21"/>
-      <c r="BJ58" s="20"/>
+      <c r="BJ58" s="21"/>
       <c r="BL58" s="17"/>
       <c r="BM58" s="17"/>
-      <c r="BN58" s="17"/>
       <c r="BO58" s="18"/>
       <c r="BP58" s="19"/>
       <c r="BQ58" s="20"/>
@@ -15709,20 +15671,20 @@
       <c r="HR58" s="17"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="72"/>
-      <c r="B59" s="73" t="s">
+      <c r="A59" s="75"/>
+      <c r="B59" s="71" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="75" t="s">
+      <c r="C59" s="72" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="70" t="s">
+      <c r="E59" s="73" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="71" t="s">
+      <c r="F59" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="17"/>
@@ -15774,10 +15736,9 @@
       <c r="BG59" s="17"/>
       <c r="BH59" s="22"/>
       <c r="BI59" s="21"/>
-      <c r="BJ59" s="20"/>
+      <c r="BJ59" s="21"/>
       <c r="BL59" s="17"/>
       <c r="BM59" s="17"/>
-      <c r="BN59" s="17"/>
       <c r="BO59" s="18"/>
       <c r="BP59" s="19"/>
       <c r="BQ59" s="20"/>
@@ -15940,14 +15901,14 @@
       <c r="HR59" s="17"/>
     </row>
     <row r="60" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="72"/>
-      <c r="B60" s="72"/>
-      <c r="C60" s="72"/>
+      <c r="A60" s="75"/>
+      <c r="B60" s="75"/>
+      <c r="C60" s="75"/>
       <c r="D60" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="70"/>
-      <c r="F60" s="70"/>
+      <c r="E60" s="73"/>
+      <c r="F60" s="73"/>
       <c r="G60" s="17"/>
       <c r="H60" s="17"/>
       <c r="I60" s="17"/>
@@ -15997,10 +15958,9 @@
       <c r="BG60" s="17"/>
       <c r="BH60" s="22"/>
       <c r="BI60" s="21"/>
-      <c r="BJ60" s="20"/>
+      <c r="BJ60" s="21"/>
       <c r="BL60" s="17"/>
       <c r="BM60" s="17"/>
-      <c r="BN60" s="17"/>
       <c r="BO60" s="18"/>
       <c r="BP60" s="19"/>
       <c r="BQ60" s="20"/>
@@ -16163,20 +16123,20 @@
       <c r="HR60" s="17"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="72"/>
-      <c r="B61" s="73" t="s">
+      <c r="A61" s="75"/>
+      <c r="B61" s="71" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="75" t="s">
+      <c r="C61" s="72" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="70" t="s">
+      <c r="E61" s="73" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="71" t="s">
+      <c r="F61" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="17"/>
@@ -16228,10 +16188,9 @@
       <c r="BG61" s="17"/>
       <c r="BH61" s="22"/>
       <c r="BI61" s="21"/>
-      <c r="BJ61" s="20"/>
+      <c r="BJ61" s="21"/>
       <c r="BL61" s="17"/>
       <c r="BM61" s="17"/>
-      <c r="BN61" s="17"/>
       <c r="BO61" s="18"/>
       <c r="BP61" s="19"/>
       <c r="BQ61" s="20"/>
@@ -16394,14 +16353,14 @@
       <c r="HR61" s="17"/>
     </row>
     <row r="62" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="72"/>
-      <c r="B62" s="72"/>
-      <c r="C62" s="72"/>
+      <c r="A62" s="75"/>
+      <c r="B62" s="75"/>
+      <c r="C62" s="75"/>
       <c r="D62" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="70"/>
-      <c r="F62" s="70"/>
+      <c r="E62" s="73"/>
+      <c r="F62" s="73"/>
       <c r="G62" s="17"/>
       <c r="H62" s="17"/>
       <c r="I62" s="17"/>
@@ -16451,10 +16410,9 @@
       <c r="BG62" s="17"/>
       <c r="BH62" s="22"/>
       <c r="BI62" s="21"/>
-      <c r="BJ62" s="20"/>
+      <c r="BJ62" s="21"/>
       <c r="BL62" s="17"/>
       <c r="BM62" s="17"/>
-      <c r="BN62" s="17"/>
       <c r="BO62" s="18"/>
       <c r="BP62" s="19"/>
       <c r="BQ62" s="20"/>
@@ -16617,20 +16575,20 @@
       <c r="HR62" s="17"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="72"/>
-      <c r="B63" s="73" t="s">
+      <c r="A63" s="75"/>
+      <c r="B63" s="71" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="75" t="s">
+      <c r="C63" s="72" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="70" t="s">
+      <c r="E63" s="73" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="71" t="s">
+      <c r="F63" s="74" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="17"/>
@@ -16682,10 +16640,9 @@
       <c r="BG63" s="17"/>
       <c r="BH63" s="22"/>
       <c r="BI63" s="21"/>
-      <c r="BJ63" s="20"/>
+      <c r="BJ63" s="21"/>
       <c r="BL63" s="17"/>
       <c r="BM63" s="17"/>
-      <c r="BN63" s="17"/>
       <c r="BO63" s="18"/>
       <c r="BP63" s="19"/>
       <c r="BQ63" s="20"/>
@@ -16848,14 +16805,14 @@
       <c r="HR63" s="17"/>
     </row>
     <row r="64" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="72"/>
-      <c r="B64" s="72"/>
-      <c r="C64" s="72"/>
+      <c r="A64" s="75"/>
+      <c r="B64" s="75"/>
+      <c r="C64" s="75"/>
       <c r="D64" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="70"/>
-      <c r="F64" s="70"/>
+      <c r="E64" s="73"/>
+      <c r="F64" s="73"/>
       <c r="G64" s="17"/>
       <c r="H64" s="17"/>
       <c r="I64" s="17"/>
@@ -16905,10 +16862,9 @@
       <c r="BG64" s="17"/>
       <c r="BH64" s="22"/>
       <c r="BI64" s="21"/>
-      <c r="BJ64" s="20"/>
+      <c r="BJ64" s="21"/>
       <c r="BL64" s="17"/>
       <c r="BM64" s="17"/>
-      <c r="BN64" s="17"/>
       <c r="BO64" s="18"/>
       <c r="BP64" s="19"/>
       <c r="BQ64" s="20"/>
@@ -17071,20 +17027,20 @@
       <c r="HR64" s="17"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="72"/>
-      <c r="B65" s="73" t="s">
+      <c r="A65" s="75"/>
+      <c r="B65" s="71" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="75" t="s">
+      <c r="C65" s="72" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="70" t="s">
+      <c r="E65" s="73" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="71" t="s">
+      <c r="F65" s="74" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="17"/>
@@ -17136,10 +17092,9 @@
       <c r="BG65" s="17"/>
       <c r="BH65" s="22"/>
       <c r="BI65" s="21"/>
-      <c r="BJ65" s="20"/>
+      <c r="BJ65" s="21"/>
       <c r="BL65" s="17"/>
       <c r="BM65" s="17"/>
-      <c r="BN65" s="17"/>
       <c r="BO65" s="18"/>
       <c r="BP65" s="19"/>
       <c r="BQ65" s="20"/>
@@ -17302,14 +17257,14 @@
       <c r="HR65" s="17"/>
     </row>
     <row r="66" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="72"/>
-      <c r="B66" s="72"/>
-      <c r="C66" s="72"/>
+      <c r="A66" s="75"/>
+      <c r="B66" s="75"/>
+      <c r="C66" s="75"/>
       <c r="D66" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="70"/>
-      <c r="F66" s="70"/>
+      <c r="E66" s="73"/>
+      <c r="F66" s="73"/>
       <c r="G66" s="17"/>
       <c r="H66" s="17"/>
       <c r="I66" s="17"/>
@@ -17359,10 +17314,9 @@
       <c r="BG66" s="17"/>
       <c r="BH66" s="22"/>
       <c r="BI66" s="21"/>
-      <c r="BJ66" s="20"/>
+      <c r="BJ66" s="21"/>
       <c r="BL66" s="17"/>
       <c r="BM66" s="17"/>
-      <c r="BN66" s="17"/>
       <c r="BO66" s="18"/>
       <c r="BP66" s="19"/>
       <c r="BQ66" s="20"/>
@@ -17525,22 +17479,22 @@
       <c r="HR66" s="17"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="72" t="s">
+      <c r="A67" s="75" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="73" t="s">
+      <c r="B67" s="71" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="75" t="s">
+      <c r="C67" s="72" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="70" t="s">
+      <c r="E67" s="73" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="71" t="s">
+      <c r="F67" s="74" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="17"/>
@@ -17592,10 +17546,9 @@
       <c r="BG67" s="17"/>
       <c r="BH67" s="22"/>
       <c r="BI67" s="21"/>
-      <c r="BJ67" s="20"/>
+      <c r="BJ67" s="21"/>
       <c r="BL67" s="17"/>
       <c r="BM67" s="17"/>
-      <c r="BN67" s="17"/>
       <c r="BO67" s="18"/>
       <c r="BP67" s="19"/>
       <c r="BQ67" s="20"/>
@@ -17758,14 +17711,14 @@
       <c r="HR67" s="17"/>
     </row>
     <row r="68" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="72"/>
-      <c r="B68" s="72"/>
-      <c r="C68" s="72"/>
+      <c r="A68" s="75"/>
+      <c r="B68" s="75"/>
+      <c r="C68" s="75"/>
       <c r="D68" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="70"/>
-      <c r="F68" s="70"/>
+      <c r="E68" s="73"/>
+      <c r="F68" s="73"/>
       <c r="G68" s="17"/>
       <c r="H68" s="17"/>
       <c r="I68" s="17"/>
@@ -17816,10 +17769,9 @@
       <c r="BG68" s="17"/>
       <c r="BH68" s="22"/>
       <c r="BI68" s="21"/>
-      <c r="BJ68" s="20"/>
+      <c r="BJ68" s="21"/>
       <c r="BL68" s="17"/>
       <c r="BM68" s="17"/>
-      <c r="BN68" s="17"/>
       <c r="BO68" s="18"/>
       <c r="BP68" s="19"/>
       <c r="BQ68" s="20"/>
@@ -17982,20 +17934,20 @@
       <c r="HR68" s="17"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="72"/>
-      <c r="B69" s="73" t="s">
+      <c r="A69" s="75"/>
+      <c r="B69" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="75" t="s">
+      <c r="C69" s="72" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="70" t="s">
+      <c r="E69" s="73" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="71" t="s">
+      <c r="F69" s="74" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="17"/>
@@ -18053,11 +18005,11 @@
       <c r="BG69" s="39"/>
       <c r="BH69" s="22"/>
       <c r="BI69" s="21"/>
-      <c r="BJ69" s="20"/>
-      <c r="BK69" s="68"/>
+      <c r="BJ69" s="21"/>
+      <c r="BK69" s="38"/>
       <c r="BL69" s="39"/>
       <c r="BM69" s="39"/>
-      <c r="BN69" s="39"/>
+      <c r="BN69" s="68"/>
       <c r="BO69" s="18"/>
       <c r="BP69" s="19"/>
       <c r="BQ69" s="20"/>
@@ -18220,14 +18172,14 @@
       <c r="HR69" s="17"/>
     </row>
     <row r="70" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="72"/>
-      <c r="B70" s="72"/>
-      <c r="C70" s="72"/>
+      <c r="A70" s="75"/>
+      <c r="B70" s="75"/>
+      <c r="C70" s="75"/>
       <c r="D70" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="70"/>
-      <c r="F70" s="70"/>
+      <c r="E70" s="73"/>
+      <c r="F70" s="73"/>
       <c r="G70" s="17"/>
       <c r="H70" s="17"/>
       <c r="I70" s="17"/>
@@ -18280,10 +18232,9 @@
       <c r="BG70" s="42"/>
       <c r="BH70" s="22"/>
       <c r="BI70" s="21"/>
-      <c r="BJ70" s="20"/>
+      <c r="BJ70" s="21"/>
       <c r="BL70" s="17"/>
-      <c r="BM70" s="17"/>
-      <c r="BN70" s="17"/>
+      <c r="BM70" s="83"/>
       <c r="BO70" s="18"/>
       <c r="BP70" s="19"/>
       <c r="BQ70" s="20"/>
@@ -18446,20 +18397,20 @@
       <c r="HR70" s="17"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="72"/>
-      <c r="B71" s="73" t="s">
+      <c r="A71" s="75"/>
+      <c r="B71" s="71" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="75" t="s">
+      <c r="C71" s="72" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="70" t="s">
+      <c r="E71" s="73" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="71" t="s">
+      <c r="F71" s="74" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="17"/>
@@ -18511,10 +18462,9 @@
       <c r="BG71" s="17"/>
       <c r="BH71" s="22"/>
       <c r="BI71" s="21"/>
-      <c r="BJ71" s="20"/>
+      <c r="BJ71" s="21"/>
       <c r="BL71" s="17"/>
       <c r="BM71" s="17"/>
-      <c r="BN71" s="17"/>
       <c r="BO71" s="18"/>
       <c r="BP71" s="19"/>
       <c r="BQ71" s="20"/>
@@ -18677,14 +18627,14 @@
       <c r="HR71" s="17"/>
     </row>
     <row r="72" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="72"/>
-      <c r="B72" s="72"/>
-      <c r="C72" s="72"/>
+      <c r="A72" s="75"/>
+      <c r="B72" s="75"/>
+      <c r="C72" s="75"/>
       <c r="D72" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="70"/>
-      <c r="F72" s="70"/>
+      <c r="E72" s="73"/>
+      <c r="F72" s="73"/>
       <c r="G72" s="17"/>
       <c r="H72" s="17"/>
       <c r="I72" s="17"/>
@@ -18734,10 +18684,9 @@
       <c r="BG72" s="17"/>
       <c r="BH72" s="22"/>
       <c r="BI72" s="21"/>
-      <c r="BJ72" s="20"/>
+      <c r="BJ72" s="21"/>
       <c r="BL72" s="17"/>
       <c r="BM72" s="17"/>
-      <c r="BN72" s="17"/>
       <c r="BO72" s="18"/>
       <c r="BP72" s="19"/>
       <c r="BQ72" s="20"/>
@@ -18900,20 +18849,20 @@
       <c r="HR72" s="17"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="72"/>
-      <c r="B73" s="73" t="s">
+      <c r="A73" s="75"/>
+      <c r="B73" s="71" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="75" t="s">
+      <c r="C73" s="72" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="70" t="s">
+      <c r="E73" s="73" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="71" t="s">
+      <c r="F73" s="74" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="17"/>
@@ -18965,10 +18914,9 @@
       <c r="BG73" s="17"/>
       <c r="BH73" s="22"/>
       <c r="BI73" s="21"/>
-      <c r="BJ73" s="20"/>
+      <c r="BJ73" s="21"/>
       <c r="BL73" s="17"/>
       <c r="BM73" s="17"/>
-      <c r="BN73" s="17"/>
       <c r="BO73" s="18"/>
       <c r="BP73" s="19"/>
       <c r="BQ73" s="20"/>
@@ -19131,14 +19079,14 @@
       <c r="HR73" s="17"/>
     </row>
     <row r="74" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="72"/>
-      <c r="B74" s="72"/>
-      <c r="C74" s="72"/>
+      <c r="A74" s="75"/>
+      <c r="B74" s="75"/>
+      <c r="C74" s="75"/>
       <c r="D74" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="70"/>
-      <c r="F74" s="70"/>
+      <c r="E74" s="73"/>
+      <c r="F74" s="73"/>
       <c r="G74" s="17"/>
       <c r="H74" s="17"/>
       <c r="I74" s="17"/>
@@ -19188,10 +19136,9 @@
       <c r="BG74" s="17"/>
       <c r="BH74" s="22"/>
       <c r="BI74" s="21"/>
-      <c r="BJ74" s="20"/>
+      <c r="BJ74" s="21"/>
       <c r="BL74" s="17"/>
       <c r="BM74" s="17"/>
-      <c r="BN74" s="17"/>
       <c r="BO74" s="18"/>
       <c r="BP74" s="19"/>
       <c r="BQ74" s="20"/>
@@ -19354,20 +19301,20 @@
       <c r="HR74" s="17"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="72"/>
-      <c r="B75" s="73" t="s">
+      <c r="A75" s="75"/>
+      <c r="B75" s="71" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="75" t="s">
+      <c r="C75" s="72" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="70" t="s">
+      <c r="E75" s="73" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="71" t="s">
+      <c r="F75" s="74" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="17"/>
@@ -19419,10 +19366,9 @@
       <c r="BG75" s="17"/>
       <c r="BH75" s="22"/>
       <c r="BI75" s="21"/>
-      <c r="BJ75" s="20"/>
+      <c r="BJ75" s="21"/>
       <c r="BL75" s="17"/>
       <c r="BM75" s="17"/>
-      <c r="BN75" s="17"/>
       <c r="BO75" s="18"/>
       <c r="BP75" s="19"/>
       <c r="BQ75" s="20"/>
@@ -19585,14 +19531,14 @@
       <c r="HR75" s="17"/>
     </row>
     <row r="76" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="72"/>
-      <c r="B76" s="72"/>
-      <c r="C76" s="72"/>
+      <c r="A76" s="75"/>
+      <c r="B76" s="75"/>
+      <c r="C76" s="75"/>
       <c r="D76" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="70"/>
-      <c r="F76" s="70"/>
+      <c r="E76" s="73"/>
+      <c r="F76" s="73"/>
       <c r="G76" s="17"/>
       <c r="H76" s="17"/>
       <c r="I76" s="17"/>
@@ -19642,10 +19588,9 @@
       <c r="BG76" s="17"/>
       <c r="BH76" s="22"/>
       <c r="BI76" s="21"/>
-      <c r="BJ76" s="20"/>
+      <c r="BJ76" s="21"/>
       <c r="BL76" s="17"/>
       <c r="BM76" s="17"/>
-      <c r="BN76" s="17"/>
       <c r="BO76" s="18"/>
       <c r="BP76" s="19"/>
       <c r="BQ76" s="20"/>
@@ -19808,20 +19753,20 @@
       <c r="HR76" s="17"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="72"/>
-      <c r="B77" s="73" t="s">
+      <c r="A77" s="75"/>
+      <c r="B77" s="71" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="75" t="s">
+      <c r="C77" s="72" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="70" t="s">
+      <c r="E77" s="73" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="71" t="s">
+      <c r="F77" s="74" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="17"/>
@@ -19873,10 +19818,9 @@
       <c r="BG77" s="17"/>
       <c r="BH77" s="22"/>
       <c r="BI77" s="21"/>
-      <c r="BJ77" s="20"/>
+      <c r="BJ77" s="21"/>
       <c r="BL77" s="17"/>
       <c r="BM77" s="17"/>
-      <c r="BN77" s="17"/>
       <c r="BO77" s="18"/>
       <c r="BP77" s="19"/>
       <c r="BQ77" s="20"/>
@@ -20039,14 +19983,14 @@
       <c r="HR77" s="17"/>
     </row>
     <row r="78" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="72"/>
-      <c r="B78" s="72"/>
-      <c r="C78" s="72"/>
+      <c r="A78" s="75"/>
+      <c r="B78" s="75"/>
+      <c r="C78" s="75"/>
       <c r="D78" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="70"/>
-      <c r="F78" s="70"/>
+      <c r="E78" s="73"/>
+      <c r="F78" s="73"/>
       <c r="G78" s="17"/>
       <c r="H78" s="17"/>
       <c r="I78" s="17"/>
@@ -20096,10 +20040,9 @@
       <c r="BG78" s="17"/>
       <c r="BH78" s="22"/>
       <c r="BI78" s="21"/>
-      <c r="BJ78" s="20"/>
+      <c r="BJ78" s="21"/>
       <c r="BL78" s="17"/>
       <c r="BM78" s="17"/>
-      <c r="BN78" s="17"/>
       <c r="BO78" s="18"/>
       <c r="BP78" s="19"/>
       <c r="BQ78" s="20"/>
@@ -20262,22 +20205,22 @@
       <c r="HR78" s="17"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="72" t="s">
+      <c r="A79" s="75" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="73" t="s">
+      <c r="B79" s="71" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="74" t="s">
+      <c r="C79" s="81" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="70" t="s">
+      <c r="E79" s="73" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="71" t="s">
+      <c r="F79" s="74" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="17"/>
@@ -20329,10 +20272,9 @@
       <c r="BG79" s="17"/>
       <c r="BH79" s="22"/>
       <c r="BI79" s="21"/>
-      <c r="BJ79" s="20"/>
+      <c r="BJ79" s="21"/>
       <c r="BL79" s="17"/>
       <c r="BM79" s="17"/>
-      <c r="BN79" s="17"/>
       <c r="BO79" s="18"/>
       <c r="BP79" s="19"/>
       <c r="BQ79" s="20"/>
@@ -20495,14 +20437,14 @@
       <c r="HR79" s="17"/>
     </row>
     <row r="80" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="72"/>
-      <c r="B80" s="72"/>
-      <c r="C80" s="72"/>
+      <c r="A80" s="75"/>
+      <c r="B80" s="75"/>
+      <c r="C80" s="75"/>
       <c r="D80" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="70"/>
-      <c r="F80" s="70"/>
+      <c r="E80" s="73"/>
+      <c r="F80" s="73"/>
       <c r="G80" s="17"/>
       <c r="H80" s="17"/>
       <c r="I80" s="17"/>
@@ -20552,10 +20494,9 @@
       <c r="BG80" s="17"/>
       <c r="BH80" s="22"/>
       <c r="BI80" s="21"/>
-      <c r="BJ80" s="20"/>
+      <c r="BJ80" s="21"/>
       <c r="BL80" s="17"/>
       <c r="BM80" s="17"/>
-      <c r="BN80" s="17"/>
       <c r="BO80" s="18"/>
       <c r="BP80" s="19"/>
       <c r="BQ80" s="20"/>
@@ -20718,20 +20659,20 @@
       <c r="HR80" s="17"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="72"/>
-      <c r="B81" s="73" t="s">
+      <c r="A81" s="75"/>
+      <c r="B81" s="71" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="74" t="s">
+      <c r="C81" s="81" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="70" t="s">
+      <c r="E81" s="73" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="71" t="s">
+      <c r="F81" s="74" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="17"/>
@@ -20783,10 +20724,9 @@
       <c r="BG81" s="17"/>
       <c r="BH81" s="22"/>
       <c r="BI81" s="21"/>
-      <c r="BJ81" s="20"/>
+      <c r="BJ81" s="21"/>
       <c r="BL81" s="17"/>
       <c r="BM81" s="17"/>
-      <c r="BN81" s="17"/>
       <c r="BO81" s="18"/>
       <c r="BP81" s="19"/>
       <c r="BQ81" s="20"/>
@@ -20949,14 +20889,14 @@
       <c r="HR81" s="17"/>
     </row>
     <row r="82" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="72"/>
-      <c r="B82" s="72"/>
-      <c r="C82" s="72"/>
+      <c r="A82" s="75"/>
+      <c r="B82" s="75"/>
+      <c r="C82" s="75"/>
       <c r="D82" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="70"/>
-      <c r="F82" s="70"/>
+      <c r="E82" s="73"/>
+      <c r="F82" s="73"/>
       <c r="G82" s="17"/>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
@@ -21006,10 +20946,9 @@
       <c r="BG82" s="17"/>
       <c r="BH82" s="22"/>
       <c r="BI82" s="21"/>
-      <c r="BJ82" s="20"/>
+      <c r="BJ82" s="21"/>
       <c r="BL82" s="17"/>
       <c r="BM82" s="17"/>
-      <c r="BN82" s="17"/>
       <c r="BO82" s="18"/>
       <c r="BP82" s="19"/>
       <c r="BQ82" s="20"/>
@@ -21172,20 +21111,20 @@
       <c r="HR82" s="17"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="72"/>
-      <c r="B83" s="73" t="s">
+      <c r="A83" s="75"/>
+      <c r="B83" s="71" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="75" t="s">
+      <c r="C83" s="72" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="70" t="s">
+      <c r="E83" s="73" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="71" t="s">
+      <c r="F83" s="74" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="17"/>
@@ -21237,10 +21176,9 @@
       <c r="BG83" s="17"/>
       <c r="BH83" s="22"/>
       <c r="BI83" s="21"/>
-      <c r="BJ83" s="20"/>
+      <c r="BJ83" s="21"/>
       <c r="BL83" s="17"/>
       <c r="BM83" s="17"/>
-      <c r="BN83" s="17"/>
       <c r="BO83" s="18"/>
       <c r="BP83" s="19"/>
       <c r="BQ83" s="20"/>
@@ -21403,14 +21341,14 @@
       <c r="HR83" s="17"/>
     </row>
     <row r="84" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="72"/>
-      <c r="B84" s="72"/>
-      <c r="C84" s="72"/>
+      <c r="A84" s="75"/>
+      <c r="B84" s="75"/>
+      <c r="C84" s="75"/>
       <c r="D84" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="70"/>
-      <c r="F84" s="70"/>
+      <c r="E84" s="73"/>
+      <c r="F84" s="73"/>
       <c r="G84" s="17"/>
       <c r="H84" s="17"/>
       <c r="I84" s="17"/>
@@ -21460,10 +21398,9 @@
       <c r="BG84" s="17"/>
       <c r="BH84" s="22"/>
       <c r="BI84" s="21"/>
-      <c r="BJ84" s="20"/>
+      <c r="BJ84" s="21"/>
       <c r="BL84" s="17"/>
       <c r="BM84" s="17"/>
-      <c r="BN84" s="17"/>
       <c r="BO84" s="18"/>
       <c r="BP84" s="19"/>
       <c r="BQ84" s="20"/>
@@ -21626,8 +21563,8 @@
       <c r="HR84" s="17"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="72"/>
-      <c r="B85" s="73" t="s">
+      <c r="A85" s="75"/>
+      <c r="B85" s="71" t="s">
         <v>167</v>
       </c>
       <c r="C85" s="76" t="s">
@@ -21636,10 +21573,10 @@
       <c r="D85" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="70" t="s">
+      <c r="E85" s="73" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="71"/>
+      <c r="F85" s="74"/>
       <c r="G85" s="17"/>
       <c r="H85" s="17"/>
       <c r="I85" s="17"/>
@@ -21689,10 +21626,9 @@
       <c r="BG85" s="17"/>
       <c r="BH85" s="22"/>
       <c r="BI85" s="21"/>
-      <c r="BJ85" s="20"/>
+      <c r="BJ85" s="21"/>
       <c r="BL85" s="17"/>
       <c r="BM85" s="17"/>
-      <c r="BN85" s="17"/>
       <c r="BO85" s="18"/>
       <c r="BP85" s="19"/>
       <c r="BQ85" s="20"/>
@@ -21855,14 +21791,14 @@
       <c r="HR85" s="49"/>
     </row>
     <row r="86" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="72"/>
-      <c r="B86" s="72"/>
-      <c r="C86" s="72"/>
+      <c r="A86" s="75"/>
+      <c r="B86" s="75"/>
+      <c r="C86" s="75"/>
       <c r="D86" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="70"/>
-      <c r="F86" s="70"/>
+      <c r="E86" s="73"/>
+      <c r="F86" s="73"/>
       <c r="G86" s="17"/>
       <c r="H86" s="17"/>
       <c r="I86" s="17"/>
@@ -21912,10 +21848,9 @@
       <c r="BG86" s="17"/>
       <c r="BH86" s="22"/>
       <c r="BI86" s="21"/>
-      <c r="BJ86" s="20"/>
+      <c r="BJ86" s="21"/>
       <c r="BL86" s="17"/>
       <c r="BM86" s="17"/>
-      <c r="BN86" s="17"/>
       <c r="BO86" s="18"/>
       <c r="BP86" s="19"/>
       <c r="BQ86" s="20"/>
@@ -22079,33 +22014,160 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
     <mergeCell ref="GN1:GT1"/>
     <mergeCell ref="GU1:HA1"/>
     <mergeCell ref="HB1:HH1"/>
@@ -22130,160 +22192,33 @@
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="C13:C14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="BK1:BQ1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Textentwruf und zugehörige überarbeitet/ hinzugefügt zu FNO-Modell und Space Chargeund mit Anmerkungen
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36225C68-02FE-4663-B6A4-01E8D1768D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DE7FE1-5042-4E74-9B58-DBD54C08F71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1174,7 +1174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1284,18 +1284,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1305,8 +1293,20 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1320,11 +1320,12 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1615,298 +1616,300 @@
     <col min="62" max="62" width="2.140625" customWidth="1"/>
     <col min="63" max="63" width="2.140625" style="1" customWidth="1"/>
     <col min="64" max="65" width="2.140625" customWidth="1"/>
-    <col min="66" max="66" width="2.140625" style="2" customWidth="1"/>
-    <col min="67" max="226" width="2.140625" customWidth="1"/>
+    <col min="66" max="66" width="2.140625" style="1" customWidth="1"/>
+    <col min="67" max="69" width="2.140625" customWidth="1"/>
+    <col min="70" max="70" width="2.140625" style="2" customWidth="1"/>
+    <col min="71" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69" t="s">
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="69" t="s">
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="81"/>
+      <c r="T1" s="81"/>
+      <c r="U1" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="69"/>
-      <c r="W1" s="69"/>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="69"/>
-      <c r="Z1" s="69"/>
-      <c r="AA1" s="69"/>
-      <c r="AB1" s="69" t="s">
+      <c r="V1" s="81"/>
+      <c r="W1" s="81"/>
+      <c r="X1" s="81"/>
+      <c r="Y1" s="81"/>
+      <c r="Z1" s="81"/>
+      <c r="AA1" s="81"/>
+      <c r="AB1" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="69"/>
-      <c r="AD1" s="69"/>
-      <c r="AE1" s="69"/>
-      <c r="AF1" s="69"/>
-      <c r="AG1" s="69"/>
-      <c r="AH1" s="69"/>
-      <c r="AI1" s="69" t="s">
+      <c r="AC1" s="81"/>
+      <c r="AD1" s="81"/>
+      <c r="AE1" s="81"/>
+      <c r="AF1" s="81"/>
+      <c r="AG1" s="81"/>
+      <c r="AH1" s="81"/>
+      <c r="AI1" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="69"/>
-      <c r="AK1" s="69"/>
-      <c r="AL1" s="69"/>
-      <c r="AM1" s="69"/>
-      <c r="AN1" s="69"/>
-      <c r="AO1" s="69"/>
-      <c r="AP1" s="69" t="s">
+      <c r="AJ1" s="81"/>
+      <c r="AK1" s="81"/>
+      <c r="AL1" s="81"/>
+      <c r="AM1" s="81"/>
+      <c r="AN1" s="81"/>
+      <c r="AO1" s="81"/>
+      <c r="AP1" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="69"/>
-      <c r="AR1" s="69"/>
-      <c r="AS1" s="69"/>
-      <c r="AT1" s="69"/>
-      <c r="AU1" s="69"/>
-      <c r="AV1" s="69"/>
-      <c r="AW1" s="69" t="s">
+      <c r="AQ1" s="81"/>
+      <c r="AR1" s="81"/>
+      <c r="AS1" s="81"/>
+      <c r="AT1" s="81"/>
+      <c r="AU1" s="81"/>
+      <c r="AV1" s="81"/>
+      <c r="AW1" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="69"/>
-      <c r="AY1" s="69"/>
-      <c r="AZ1" s="69"/>
-      <c r="BA1" s="69"/>
-      <c r="BB1" s="69"/>
-      <c r="BC1" s="69"/>
-      <c r="BD1" s="69" t="s">
+      <c r="AX1" s="81"/>
+      <c r="AY1" s="81"/>
+      <c r="AZ1" s="81"/>
+      <c r="BA1" s="81"/>
+      <c r="BB1" s="81"/>
+      <c r="BC1" s="81"/>
+      <c r="BD1" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="69"/>
-      <c r="BF1" s="69"/>
-      <c r="BG1" s="69"/>
-      <c r="BH1" s="69"/>
-      <c r="BI1" s="69"/>
-      <c r="BJ1" s="69"/>
-      <c r="BK1" s="69" t="s">
+      <c r="BE1" s="81"/>
+      <c r="BF1" s="81"/>
+      <c r="BG1" s="81"/>
+      <c r="BH1" s="81"/>
+      <c r="BI1" s="81"/>
+      <c r="BJ1" s="81"/>
+      <c r="BK1" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="69"/>
-      <c r="BM1" s="69"/>
-      <c r="BN1" s="69"/>
-      <c r="BO1" s="69"/>
-      <c r="BP1" s="69"/>
-      <c r="BQ1" s="69"/>
-      <c r="BR1" s="69" t="s">
+      <c r="BL1" s="81"/>
+      <c r="BM1" s="81"/>
+      <c r="BN1" s="81"/>
+      <c r="BO1" s="81"/>
+      <c r="BP1" s="81"/>
+      <c r="BQ1" s="81"/>
+      <c r="BR1" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="69"/>
-      <c r="BT1" s="69"/>
-      <c r="BU1" s="69"/>
-      <c r="BV1" s="69"/>
-      <c r="BW1" s="69"/>
-      <c r="BX1" s="69"/>
-      <c r="BY1" s="69" t="s">
+      <c r="BS1" s="81"/>
+      <c r="BT1" s="81"/>
+      <c r="BU1" s="81"/>
+      <c r="BV1" s="81"/>
+      <c r="BW1" s="81"/>
+      <c r="BX1" s="81"/>
+      <c r="BY1" s="81" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="69"/>
-      <c r="CA1" s="69"/>
-      <c r="CB1" s="69"/>
-      <c r="CC1" s="69"/>
-      <c r="CD1" s="69"/>
-      <c r="CE1" s="69"/>
-      <c r="CF1" s="69" t="s">
+      <c r="BZ1" s="81"/>
+      <c r="CA1" s="81"/>
+      <c r="CB1" s="81"/>
+      <c r="CC1" s="81"/>
+      <c r="CD1" s="81"/>
+      <c r="CE1" s="81"/>
+      <c r="CF1" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="69"/>
-      <c r="CH1" s="69"/>
-      <c r="CI1" s="69"/>
-      <c r="CJ1" s="69"/>
-      <c r="CK1" s="69"/>
-      <c r="CL1" s="69"/>
-      <c r="CM1" s="69" t="s">
+      <c r="CG1" s="81"/>
+      <c r="CH1" s="81"/>
+      <c r="CI1" s="81"/>
+      <c r="CJ1" s="81"/>
+      <c r="CK1" s="81"/>
+      <c r="CL1" s="81"/>
+      <c r="CM1" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="69"/>
-      <c r="CO1" s="69"/>
-      <c r="CP1" s="69"/>
-      <c r="CQ1" s="69"/>
-      <c r="CR1" s="69"/>
-      <c r="CS1" s="69"/>
-      <c r="CT1" s="69" t="s">
+      <c r="CN1" s="81"/>
+      <c r="CO1" s="81"/>
+      <c r="CP1" s="81"/>
+      <c r="CQ1" s="81"/>
+      <c r="CR1" s="81"/>
+      <c r="CS1" s="81"/>
+      <c r="CT1" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="69"/>
-      <c r="CV1" s="69"/>
-      <c r="CW1" s="69"/>
-      <c r="CX1" s="69"/>
-      <c r="CY1" s="69"/>
-      <c r="CZ1" s="69"/>
-      <c r="DA1" s="69" t="s">
+      <c r="CU1" s="81"/>
+      <c r="CV1" s="81"/>
+      <c r="CW1" s="81"/>
+      <c r="CX1" s="81"/>
+      <c r="CY1" s="81"/>
+      <c r="CZ1" s="81"/>
+      <c r="DA1" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="69"/>
-      <c r="DC1" s="69"/>
-      <c r="DD1" s="69"/>
-      <c r="DE1" s="69"/>
-      <c r="DF1" s="69"/>
-      <c r="DG1" s="69"/>
-      <c r="DH1" s="69" t="s">
+      <c r="DB1" s="81"/>
+      <c r="DC1" s="81"/>
+      <c r="DD1" s="81"/>
+      <c r="DE1" s="81"/>
+      <c r="DF1" s="81"/>
+      <c r="DG1" s="81"/>
+      <c r="DH1" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="69"/>
-      <c r="DJ1" s="69"/>
-      <c r="DK1" s="69"/>
-      <c r="DL1" s="69"/>
-      <c r="DM1" s="69"/>
-      <c r="DN1" s="69"/>
-      <c r="DO1" s="69" t="s">
+      <c r="DI1" s="81"/>
+      <c r="DJ1" s="81"/>
+      <c r="DK1" s="81"/>
+      <c r="DL1" s="81"/>
+      <c r="DM1" s="81"/>
+      <c r="DN1" s="81"/>
+      <c r="DO1" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="69"/>
-      <c r="DQ1" s="69"/>
-      <c r="DR1" s="69"/>
-      <c r="DS1" s="69"/>
-      <c r="DT1" s="69"/>
-      <c r="DU1" s="69"/>
-      <c r="DV1" s="69" t="s">
+      <c r="DP1" s="81"/>
+      <c r="DQ1" s="81"/>
+      <c r="DR1" s="81"/>
+      <c r="DS1" s="81"/>
+      <c r="DT1" s="81"/>
+      <c r="DU1" s="81"/>
+      <c r="DV1" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="69"/>
-      <c r="DX1" s="69"/>
-      <c r="DY1" s="69"/>
-      <c r="DZ1" s="69"/>
-      <c r="EA1" s="69"/>
-      <c r="EB1" s="69"/>
-      <c r="EC1" s="69" t="s">
+      <c r="DW1" s="81"/>
+      <c r="DX1" s="81"/>
+      <c r="DY1" s="81"/>
+      <c r="DZ1" s="81"/>
+      <c r="EA1" s="81"/>
+      <c r="EB1" s="81"/>
+      <c r="EC1" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="69"/>
-      <c r="EE1" s="69"/>
-      <c r="EF1" s="69"/>
-      <c r="EG1" s="69"/>
-      <c r="EH1" s="69"/>
-      <c r="EI1" s="69"/>
-      <c r="EJ1" s="69" t="s">
+      <c r="ED1" s="81"/>
+      <c r="EE1" s="81"/>
+      <c r="EF1" s="81"/>
+      <c r="EG1" s="81"/>
+      <c r="EH1" s="81"/>
+      <c r="EI1" s="81"/>
+      <c r="EJ1" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="69"/>
-      <c r="EL1" s="69"/>
-      <c r="EM1" s="69"/>
-      <c r="EN1" s="69"/>
-      <c r="EO1" s="69"/>
-      <c r="EP1" s="69"/>
-      <c r="EQ1" s="69" t="s">
+      <c r="EK1" s="81"/>
+      <c r="EL1" s="81"/>
+      <c r="EM1" s="81"/>
+      <c r="EN1" s="81"/>
+      <c r="EO1" s="81"/>
+      <c r="EP1" s="81"/>
+      <c r="EQ1" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="69"/>
-      <c r="ES1" s="69"/>
-      <c r="ET1" s="69"/>
-      <c r="EU1" s="69"/>
-      <c r="EV1" s="69"/>
-      <c r="EW1" s="69"/>
-      <c r="EX1" s="69" t="s">
+      <c r="ER1" s="81"/>
+      <c r="ES1" s="81"/>
+      <c r="ET1" s="81"/>
+      <c r="EU1" s="81"/>
+      <c r="EV1" s="81"/>
+      <c r="EW1" s="81"/>
+      <c r="EX1" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="69"/>
-      <c r="EZ1" s="69"/>
-      <c r="FA1" s="69"/>
-      <c r="FB1" s="69"/>
-      <c r="FC1" s="69"/>
-      <c r="FD1" s="69"/>
-      <c r="FE1" s="69" t="s">
+      <c r="EY1" s="81"/>
+      <c r="EZ1" s="81"/>
+      <c r="FA1" s="81"/>
+      <c r="FB1" s="81"/>
+      <c r="FC1" s="81"/>
+      <c r="FD1" s="81"/>
+      <c r="FE1" s="81" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="69"/>
-      <c r="FG1" s="69"/>
-      <c r="FH1" s="69"/>
-      <c r="FI1" s="69"/>
-      <c r="FJ1" s="69"/>
-      <c r="FK1" s="69"/>
-      <c r="FL1" s="69" t="s">
+      <c r="FF1" s="81"/>
+      <c r="FG1" s="81"/>
+      <c r="FH1" s="81"/>
+      <c r="FI1" s="81"/>
+      <c r="FJ1" s="81"/>
+      <c r="FK1" s="81"/>
+      <c r="FL1" s="81" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="69"/>
-      <c r="FN1" s="69"/>
-      <c r="FO1" s="69"/>
-      <c r="FP1" s="69"/>
-      <c r="FQ1" s="69"/>
-      <c r="FR1" s="69"/>
-      <c r="FS1" s="69" t="s">
+      <c r="FM1" s="81"/>
+      <c r="FN1" s="81"/>
+      <c r="FO1" s="81"/>
+      <c r="FP1" s="81"/>
+      <c r="FQ1" s="81"/>
+      <c r="FR1" s="81"/>
+      <c r="FS1" s="81" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="69"/>
-      <c r="FU1" s="69"/>
-      <c r="FV1" s="69"/>
-      <c r="FW1" s="69"/>
-      <c r="FX1" s="69"/>
-      <c r="FY1" s="69"/>
-      <c r="FZ1" s="69" t="s">
+      <c r="FT1" s="81"/>
+      <c r="FU1" s="81"/>
+      <c r="FV1" s="81"/>
+      <c r="FW1" s="81"/>
+      <c r="FX1" s="81"/>
+      <c r="FY1" s="81"/>
+      <c r="FZ1" s="81" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="69"/>
-      <c r="GB1" s="69"/>
-      <c r="GC1" s="69"/>
-      <c r="GD1" s="69"/>
-      <c r="GE1" s="69"/>
-      <c r="GF1" s="69"/>
-      <c r="GG1" s="69" t="s">
+      <c r="GA1" s="81"/>
+      <c r="GB1" s="81"/>
+      <c r="GC1" s="81"/>
+      <c r="GD1" s="81"/>
+      <c r="GE1" s="81"/>
+      <c r="GF1" s="81"/>
+      <c r="GG1" s="81" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="69"/>
-      <c r="GI1" s="69"/>
-      <c r="GJ1" s="69"/>
-      <c r="GK1" s="69"/>
-      <c r="GL1" s="69"/>
-      <c r="GM1" s="69"/>
-      <c r="GN1" s="69" t="s">
+      <c r="GH1" s="81"/>
+      <c r="GI1" s="81"/>
+      <c r="GJ1" s="81"/>
+      <c r="GK1" s="81"/>
+      <c r="GL1" s="81"/>
+      <c r="GM1" s="81"/>
+      <c r="GN1" s="81" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="69"/>
-      <c r="GP1" s="69"/>
-      <c r="GQ1" s="69"/>
-      <c r="GR1" s="69"/>
-      <c r="GS1" s="69"/>
-      <c r="GT1" s="69"/>
-      <c r="GU1" s="69" t="s">
+      <c r="GO1" s="81"/>
+      <c r="GP1" s="81"/>
+      <c r="GQ1" s="81"/>
+      <c r="GR1" s="81"/>
+      <c r="GS1" s="81"/>
+      <c r="GT1" s="81"/>
+      <c r="GU1" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="69"/>
-      <c r="GW1" s="69"/>
-      <c r="GX1" s="69"/>
-      <c r="GY1" s="69"/>
-      <c r="GZ1" s="69"/>
-      <c r="HA1" s="69"/>
-      <c r="HB1" s="69" t="s">
+      <c r="GV1" s="81"/>
+      <c r="GW1" s="81"/>
+      <c r="GX1" s="81"/>
+      <c r="GY1" s="81"/>
+      <c r="GZ1" s="81"/>
+      <c r="HA1" s="81"/>
+      <c r="HB1" s="81" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="69"/>
-      <c r="HD1" s="69"/>
-      <c r="HE1" s="69"/>
-      <c r="HF1" s="69"/>
-      <c r="HG1" s="69"/>
-      <c r="HH1" s="69"/>
-      <c r="HI1" s="69" t="s">
+      <c r="HC1" s="81"/>
+      <c r="HD1" s="81"/>
+      <c r="HE1" s="81"/>
+      <c r="HF1" s="81"/>
+      <c r="HG1" s="81"/>
+      <c r="HH1" s="81"/>
+      <c r="HI1" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="69"/>
-      <c r="HK1" s="69"/>
-      <c r="HL1" s="69"/>
-      <c r="HM1" s="69"/>
-      <c r="HN1" s="69"/>
-      <c r="HO1" s="69"/>
-      <c r="HP1" s="69" t="s">
+      <c r="HJ1" s="81"/>
+      <c r="HK1" s="81"/>
+      <c r="HL1" s="81"/>
+      <c r="HM1" s="81"/>
+      <c r="HN1" s="81"/>
+      <c r="HO1" s="81"/>
+      <c r="HP1" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="69"/>
-      <c r="HR1" s="69"/>
+      <c r="HQ1" s="81"/>
+      <c r="HR1" s="81"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3" t="s">
@@ -2089,7 +2092,7 @@
       <c r="BM2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="BN2" s="7" t="s">
+      <c r="BN2" s="6" t="s">
         <v>35</v>
       </c>
       <c r="BO2" s="4" t="s">
@@ -2101,7 +2104,7 @@
       <c r="BQ2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="BR2" s="4" t="s">
+      <c r="BR2" s="7" t="s">
         <v>34</v>
       </c>
       <c r="BS2" s="4" t="s">
@@ -2754,7 +2757,7 @@
       <c r="BM3" s="8">
         <v>46309</v>
       </c>
-      <c r="BN3" s="10">
+      <c r="BN3" s="9">
         <v>46310</v>
       </c>
       <c r="BO3" s="8">
@@ -2766,7 +2769,7 @@
       <c r="BQ3" s="8">
         <v>46313</v>
       </c>
-      <c r="BR3" s="8">
+      <c r="BR3" s="10">
         <v>46314</v>
       </c>
       <c r="BS3" s="8">
@@ -3314,11 +3317,11 @@
       <c r="BK4" s="13"/>
       <c r="BL4" s="12"/>
       <c r="BM4" s="12"/>
-      <c r="BN4" s="14"/>
+      <c r="BN4" s="13"/>
       <c r="BO4" s="12"/>
       <c r="BP4" s="12"/>
       <c r="BQ4" s="12"/>
-      <c r="BR4" s="12"/>
+      <c r="BR4" s="14"/>
       <c r="BS4" s="12"/>
       <c r="BT4" s="12"/>
       <c r="BU4" s="12"/>
@@ -3477,20 +3480,20 @@
       <c r="HR4" s="12"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="76" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="71"/>
-      <c r="C5" s="72" t="s">
+      <c r="B5" s="72"/>
+      <c r="C5" s="74" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="73" t="s">
+      <c r="E5" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="74"/>
+      <c r="F5" s="70"/>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
       <c r="I5" s="17"/>
@@ -3542,11 +3545,10 @@
       <c r="BI5" s="21"/>
       <c r="BJ5" s="21"/>
       <c r="BL5" s="17"/>
-      <c r="BM5" s="17"/>
+      <c r="BM5" s="1"/>
       <c r="BO5" s="18"/>
       <c r="BP5" s="19"/>
       <c r="BQ5" s="20"/>
-      <c r="BR5" s="17"/>
       <c r="BS5" s="17"/>
       <c r="BT5" s="17"/>
       <c r="BU5" s="17"/>
@@ -3705,14 +3707,14 @@
       <c r="HR5" s="17"/>
     </row>
     <row r="6" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="70"/>
-      <c r="B6" s="70"/>
-      <c r="C6" s="70"/>
+      <c r="A6" s="76"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="76"/>
       <c r="D6" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
       <c r="G6" s="17"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
@@ -3764,11 +3766,10 @@
       <c r="BI6" s="21"/>
       <c r="BJ6" s="21"/>
       <c r="BL6" s="17"/>
-      <c r="BM6" s="17"/>
+      <c r="BM6" s="1"/>
       <c r="BO6" s="18"/>
       <c r="BP6" s="19"/>
       <c r="BQ6" s="20"/>
-      <c r="BR6" s="17"/>
       <c r="BS6" s="17"/>
       <c r="BT6" s="17"/>
       <c r="BU6" s="17"/>
@@ -3927,18 +3928,18 @@
       <c r="HR6" s="17"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="70"/>
-      <c r="B7" s="71"/>
-      <c r="C7" s="72" t="s">
+      <c r="A7" s="76"/>
+      <c r="B7" s="72"/>
+      <c r="C7" s="74" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="73" t="s">
+      <c r="E7" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="74"/>
+      <c r="F7" s="70"/>
       <c r="G7" s="17"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -3990,11 +3991,10 @@
       <c r="BI7" s="21"/>
       <c r="BJ7" s="21"/>
       <c r="BL7" s="17"/>
-      <c r="BM7" s="17"/>
+      <c r="BM7" s="1"/>
       <c r="BO7" s="18"/>
       <c r="BP7" s="19"/>
       <c r="BQ7" s="20"/>
-      <c r="BR7" s="17"/>
       <c r="BS7" s="17"/>
       <c r="BT7" s="17"/>
       <c r="BU7" s="17"/>
@@ -4153,14 +4153,14 @@
       <c r="HR7" s="17"/>
     </row>
     <row r="8" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="70"/>
-      <c r="B8" s="70"/>
-      <c r="C8" s="70"/>
+      <c r="A8" s="76"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
+      <c r="E8" s="69"/>
+      <c r="F8" s="69"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
@@ -4212,11 +4212,10 @@
       <c r="BI8" s="21"/>
       <c r="BJ8" s="21"/>
       <c r="BL8" s="17"/>
-      <c r="BM8" s="17"/>
+      <c r="BM8" s="1"/>
       <c r="BO8" s="18"/>
       <c r="BP8" s="19"/>
       <c r="BQ8" s="20"/>
-      <c r="BR8" s="17"/>
       <c r="BS8" s="17"/>
       <c r="BT8" s="17"/>
       <c r="BU8" s="17"/>
@@ -4375,18 +4374,18 @@
       <c r="HR8" s="17"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="70"/>
-      <c r="B9" s="71"/>
-      <c r="C9" s="72" t="s">
+      <c r="A9" s="76"/>
+      <c r="B9" s="72"/>
+      <c r="C9" s="74" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="73" t="s">
+      <c r="E9" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="74"/>
+      <c r="F9" s="70"/>
       <c r="G9" s="17"/>
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
@@ -4438,11 +4437,10 @@
       <c r="BI9" s="21"/>
       <c r="BJ9" s="21"/>
       <c r="BL9" s="17"/>
-      <c r="BM9" s="17"/>
+      <c r="BM9" s="1"/>
       <c r="BO9" s="18"/>
       <c r="BP9" s="19"/>
       <c r="BQ9" s="20"/>
-      <c r="BR9" s="17"/>
       <c r="BS9" s="17"/>
       <c r="BT9" s="17"/>
       <c r="BU9" s="17"/>
@@ -4601,14 +4599,14 @@
       <c r="HR9" s="17"/>
     </row>
     <row r="10" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="70"/>
-      <c r="B10" s="70"/>
-      <c r="C10" s="70"/>
+      <c r="A10" s="76"/>
+      <c r="B10" s="76"/>
+      <c r="C10" s="76"/>
       <c r="D10" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="73"/>
-      <c r="F10" s="73"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -4660,11 +4658,10 @@
       <c r="BI10" s="21"/>
       <c r="BJ10" s="21"/>
       <c r="BL10" s="17"/>
-      <c r="BM10" s="17"/>
+      <c r="BM10" s="1"/>
       <c r="BO10" s="18"/>
       <c r="BP10" s="19"/>
       <c r="BQ10" s="20"/>
-      <c r="BR10" s="17"/>
       <c r="BS10" s="17"/>
       <c r="BT10" s="17"/>
       <c r="BU10" s="17"/>
@@ -4823,18 +4820,18 @@
       <c r="HR10" s="17"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70"/>
-      <c r="B11" s="71"/>
-      <c r="C11" s="72" t="s">
+      <c r="A11" s="76"/>
+      <c r="B11" s="72"/>
+      <c r="C11" s="74" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="73" t="s">
+      <c r="E11" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="74"/>
+      <c r="F11" s="70"/>
       <c r="G11" s="17"/>
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
@@ -4886,11 +4883,10 @@
       <c r="BI11" s="21"/>
       <c r="BJ11" s="21"/>
       <c r="BL11" s="17"/>
-      <c r="BM11" s="17"/>
+      <c r="BM11" s="1"/>
       <c r="BO11" s="18"/>
       <c r="BP11" s="19"/>
       <c r="BQ11" s="20"/>
-      <c r="BR11" s="17"/>
       <c r="BS11" s="17"/>
       <c r="BT11" s="17"/>
       <c r="BU11" s="17"/>
@@ -5049,14 +5045,14 @@
       <c r="HR11" s="17"/>
     </row>
     <row r="12" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="70"/>
-      <c r="B12" s="70"/>
-      <c r="C12" s="70"/>
+      <c r="A12" s="76"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
       <c r="D12" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -5108,11 +5104,10 @@
       <c r="BI12" s="21"/>
       <c r="BJ12" s="21"/>
       <c r="BL12" s="17"/>
-      <c r="BM12" s="17"/>
+      <c r="BM12" s="1"/>
       <c r="BO12" s="18"/>
       <c r="BP12" s="19"/>
       <c r="BQ12" s="20"/>
-      <c r="BR12" s="17"/>
       <c r="BS12" s="17"/>
       <c r="BT12" s="17"/>
       <c r="BU12" s="17"/>
@@ -5271,18 +5266,18 @@
       <c r="HR12" s="17"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="70"/>
-      <c r="B13" s="71"/>
-      <c r="C13" s="72" t="s">
+      <c r="A13" s="76"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="74" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="73" t="s">
+      <c r="E13" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="74"/>
+      <c r="F13" s="70"/>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
       <c r="I13" s="17"/>
@@ -5334,11 +5329,10 @@
       <c r="BI13" s="21"/>
       <c r="BJ13" s="21"/>
       <c r="BL13" s="17"/>
-      <c r="BM13" s="17"/>
+      <c r="BM13" s="1"/>
       <c r="BO13" s="18"/>
       <c r="BP13" s="19"/>
       <c r="BQ13" s="20"/>
-      <c r="BR13" s="17"/>
       <c r="BS13" s="17"/>
       <c r="BT13" s="17"/>
       <c r="BU13" s="17"/>
@@ -5497,14 +5491,14 @@
       <c r="HR13" s="17"/>
     </row>
     <row r="14" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="70"/>
-      <c r="B14" s="70"/>
-      <c r="C14" s="70"/>
+      <c r="A14" s="76"/>
+      <c r="B14" s="76"/>
+      <c r="C14" s="76"/>
       <c r="D14" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="69"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -5556,11 +5550,10 @@
       <c r="BI14" s="21"/>
       <c r="BJ14" s="21"/>
       <c r="BL14" s="17"/>
-      <c r="BM14" s="17"/>
+      <c r="BM14" s="1"/>
       <c r="BO14" s="18"/>
       <c r="BP14" s="19"/>
       <c r="BQ14" s="20"/>
-      <c r="BR14" s="17"/>
       <c r="BS14" s="17"/>
       <c r="BT14" s="17"/>
       <c r="BU14" s="17"/>
@@ -5719,18 +5712,18 @@
       <c r="HR14" s="17"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="70"/>
-      <c r="B15" s="71"/>
-      <c r="C15" s="72" t="s">
+      <c r="A15" s="76"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="74" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="73" t="s">
+      <c r="E15" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="74"/>
+      <c r="F15" s="70"/>
       <c r="G15" s="17"/>
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
@@ -5782,11 +5775,10 @@
       <c r="BI15" s="21"/>
       <c r="BJ15" s="21"/>
       <c r="BL15" s="17"/>
-      <c r="BM15" s="17"/>
+      <c r="BM15" s="1"/>
       <c r="BO15" s="18"/>
       <c r="BP15" s="19"/>
       <c r="BQ15" s="20"/>
-      <c r="BR15" s="17"/>
       <c r="BS15" s="17"/>
       <c r="BT15" s="17"/>
       <c r="BU15" s="17"/>
@@ -5945,14 +5937,14 @@
       <c r="HR15" s="17"/>
     </row>
     <row r="16" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="70"/>
-      <c r="B16" s="70"/>
-      <c r="C16" s="70"/>
+      <c r="A16" s="76"/>
+      <c r="B16" s="76"/>
+      <c r="C16" s="76"/>
       <c r="D16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="73"/>
-      <c r="F16" s="73"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -6004,11 +5996,10 @@
       <c r="BI16" s="21"/>
       <c r="BJ16" s="21"/>
       <c r="BL16" s="17"/>
-      <c r="BM16" s="17"/>
+      <c r="BM16" s="1"/>
       <c r="BO16" s="18"/>
       <c r="BP16" s="19"/>
       <c r="BQ16" s="20"/>
-      <c r="BR16" s="17"/>
       <c r="BS16" s="17"/>
       <c r="BT16" s="17"/>
       <c r="BU16" s="17"/>
@@ -6167,18 +6158,18 @@
       <c r="HR16" s="17"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="70"/>
-      <c r="B17" s="71"/>
-      <c r="C17" s="72" t="s">
+      <c r="A17" s="76"/>
+      <c r="B17" s="72"/>
+      <c r="C17" s="74" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="73" t="s">
+      <c r="E17" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="74"/>
+      <c r="F17" s="70"/>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
@@ -6230,11 +6221,10 @@
       <c r="BI17" s="21"/>
       <c r="BJ17" s="21"/>
       <c r="BL17" s="17"/>
-      <c r="BM17" s="17"/>
+      <c r="BM17" s="1"/>
       <c r="BO17" s="18"/>
       <c r="BP17" s="19"/>
       <c r="BQ17" s="20"/>
-      <c r="BR17" s="17"/>
       <c r="BS17" s="17"/>
       <c r="BT17" s="17"/>
       <c r="BU17" s="17"/>
@@ -6393,14 +6383,14 @@
       <c r="HR17" s="17"/>
     </row>
     <row r="18" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="70"/>
-      <c r="B18" s="70"/>
-      <c r="C18" s="70"/>
+      <c r="A18" s="76"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="76"/>
       <c r="D18" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="69"/>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -6452,11 +6442,10 @@
       <c r="BI18" s="21"/>
       <c r="BJ18" s="21"/>
       <c r="BL18" s="17"/>
-      <c r="BM18" s="17"/>
+      <c r="BM18" s="1"/>
       <c r="BO18" s="18"/>
       <c r="BP18" s="19"/>
       <c r="BQ18" s="20"/>
-      <c r="BR18" s="17"/>
       <c r="BS18" s="17"/>
       <c r="BT18" s="17"/>
       <c r="BU18" s="17"/>
@@ -6615,18 +6604,18 @@
       <c r="HR18" s="17"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="70"/>
-      <c r="B19" s="71"/>
-      <c r="C19" s="72" t="s">
+      <c r="A19" s="76"/>
+      <c r="B19" s="72"/>
+      <c r="C19" s="74" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="73" t="s">
+      <c r="E19" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="74"/>
+      <c r="F19" s="70"/>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
@@ -6678,11 +6667,10 @@
       <c r="BI19" s="21"/>
       <c r="BJ19" s="21"/>
       <c r="BL19" s="17"/>
-      <c r="BM19" s="17"/>
+      <c r="BM19" s="1"/>
       <c r="BO19" s="18"/>
       <c r="BP19" s="19"/>
       <c r="BQ19" s="20"/>
-      <c r="BR19" s="17"/>
       <c r="BS19" s="17"/>
       <c r="BT19" s="17"/>
       <c r="BU19" s="17"/>
@@ -6841,14 +6829,14 @@
       <c r="HR19" s="17"/>
     </row>
     <row r="20" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
+      <c r="A20" s="76"/>
+      <c r="B20" s="76"/>
+      <c r="C20" s="76"/>
       <c r="D20" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="73"/>
-      <c r="F20" s="73"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="69"/>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
@@ -6900,11 +6888,10 @@
       <c r="BI20" s="21"/>
       <c r="BJ20" s="21"/>
       <c r="BL20" s="17"/>
-      <c r="BM20" s="17"/>
+      <c r="BM20" s="1"/>
       <c r="BO20" s="18"/>
       <c r="BP20" s="19"/>
       <c r="BQ20" s="20"/>
-      <c r="BR20" s="17"/>
       <c r="BS20" s="17"/>
       <c r="BT20" s="17"/>
       <c r="BU20" s="17"/>
@@ -7063,7 +7050,7 @@
       <c r="HR20" s="17"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="70"/>
+      <c r="A21" s="76"/>
       <c r="B21" s="77"/>
       <c r="C21" s="78" t="s">
         <v>63</v>
@@ -7126,11 +7113,10 @@
       <c r="BI21" s="21"/>
       <c r="BJ21" s="21"/>
       <c r="BL21" s="17"/>
-      <c r="BM21" s="17"/>
+      <c r="BM21" s="1"/>
       <c r="BO21" s="18"/>
       <c r="BP21" s="19"/>
       <c r="BQ21" s="20"/>
-      <c r="BR21" s="17"/>
       <c r="BS21" s="17"/>
       <c r="BT21" s="17"/>
       <c r="BU21" s="17"/>
@@ -7289,9 +7275,9 @@
       <c r="HR21" s="17"/>
     </row>
     <row r="22" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="70"/>
-      <c r="B22" s="70"/>
-      <c r="C22" s="70"/>
+      <c r="A22" s="76"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="76"/>
       <c r="D22" s="29" t="s">
         <v>48</v>
       </c>
@@ -7348,12 +7334,11 @@
       <c r="BI22" s="21"/>
       <c r="BJ22" s="35"/>
       <c r="BL22" s="30"/>
-      <c r="BM22" s="30"/>
-      <c r="BN22" s="67"/>
+      <c r="BM22" s="36"/>
       <c r="BO22" s="31"/>
       <c r="BP22" s="32"/>
       <c r="BQ22" s="33"/>
-      <c r="BR22" s="30"/>
+      <c r="BR22" s="67"/>
       <c r="BS22" s="30"/>
       <c r="BT22" s="30"/>
       <c r="BU22" s="30"/>
@@ -7512,22 +7497,22 @@
       <c r="HR22" s="30"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="71" t="s">
+      <c r="B23" s="72" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="72" t="s">
+      <c r="C23" s="74" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="73" t="s">
+      <c r="E23" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="74" t="s">
+      <c r="F23" s="70" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="17"/>
@@ -7585,11 +7570,11 @@
       <c r="BJ23" s="21"/>
       <c r="BK23" s="38"/>
       <c r="BL23" s="17"/>
-      <c r="BM23" s="17"/>
+      <c r="BM23" s="1"/>
       <c r="BO23" s="18"/>
       <c r="BP23" s="19"/>
       <c r="BQ23" s="20"/>
-      <c r="BR23" s="39"/>
+      <c r="BR23" s="68"/>
       <c r="BS23" s="17"/>
       <c r="BT23" s="17"/>
       <c r="BU23" s="17"/>
@@ -7748,14 +7733,14 @@
       <c r="HR23" s="17"/>
     </row>
     <row r="24" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="75"/>
-      <c r="B24" s="75"/>
-      <c r="C24" s="75"/>
+      <c r="A24" s="71"/>
+      <c r="B24" s="71"/>
+      <c r="C24" s="71"/>
       <c r="D24" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="73"/>
-      <c r="F24" s="73"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
@@ -7811,11 +7796,10 @@
       <c r="BJ24" s="21"/>
       <c r="BK24" s="42"/>
       <c r="BL24" s="17"/>
-      <c r="BM24" s="17"/>
+      <c r="BM24" s="1"/>
       <c r="BO24" s="18"/>
       <c r="BP24" s="19"/>
       <c r="BQ24" s="20"/>
-      <c r="BR24" s="17"/>
       <c r="BS24" s="17"/>
       <c r="BT24" s="17"/>
       <c r="BU24" s="17"/>
@@ -7974,20 +7958,20 @@
       <c r="HR24" s="17"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="75"/>
-      <c r="B25" s="71" t="s">
+      <c r="A25" s="71"/>
+      <c r="B25" s="72" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="72" t="s">
+      <c r="C25" s="74" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="73" t="s">
+      <c r="E25" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="74" t="s">
+      <c r="F25" s="70" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="17"/>
@@ -8036,11 +8020,10 @@
       <c r="BI25" s="21"/>
       <c r="BJ25" s="21"/>
       <c r="BL25" s="17"/>
-      <c r="BM25" s="68"/>
+      <c r="BM25" s="38"/>
       <c r="BO25" s="18"/>
       <c r="BP25" s="19"/>
       <c r="BQ25" s="20"/>
-      <c r="BR25" s="17"/>
       <c r="BS25" s="17"/>
       <c r="BT25" s="17"/>
       <c r="BV25" s="18"/>
@@ -8197,14 +8180,14 @@
       <c r="HS25" s="17"/>
     </row>
     <row r="26" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="75"/>
-      <c r="B26" s="75"/>
-      <c r="C26" s="75"/>
+      <c r="A26" s="71"/>
+      <c r="B26" s="71"/>
+      <c r="C26" s="71"/>
       <c r="D26" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="73"/>
-      <c r="F26" s="73"/>
+      <c r="E26" s="69"/>
+      <c r="F26" s="69"/>
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -8260,7 +8243,6 @@
       <c r="BO26" s="18"/>
       <c r="BP26" s="19"/>
       <c r="BQ26" s="20"/>
-      <c r="BR26" s="17"/>
       <c r="BS26" s="17"/>
       <c r="BT26" s="17"/>
       <c r="BU26" s="17"/>
@@ -8419,20 +8401,20 @@
       <c r="HR26" s="17"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="75"/>
-      <c r="B27" s="71" t="s">
+      <c r="A27" s="71"/>
+      <c r="B27" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="76" t="s">
+      <c r="C27" s="75" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="73" t="s">
+      <c r="E27" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="74"/>
+      <c r="F27" s="70"/>
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -8484,11 +8466,10 @@
       <c r="BI27" s="21"/>
       <c r="BJ27" s="21"/>
       <c r="BL27" s="17"/>
-      <c r="BM27" s="17"/>
+      <c r="BM27" s="1"/>
       <c r="BO27" s="18"/>
       <c r="BP27" s="19"/>
       <c r="BQ27" s="20"/>
-      <c r="BR27" s="17"/>
       <c r="BS27" s="17"/>
       <c r="BT27" s="17"/>
       <c r="BU27" s="17"/>
@@ -8647,14 +8628,14 @@
       <c r="HR27" s="17"/>
     </row>
     <row r="28" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="75"/>
-      <c r="B28" s="75"/>
-      <c r="C28" s="75"/>
+      <c r="A28" s="71"/>
+      <c r="B28" s="71"/>
+      <c r="C28" s="71"/>
       <c r="D28" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="73"/>
-      <c r="F28" s="73"/>
+      <c r="E28" s="69"/>
+      <c r="F28" s="69"/>
       <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -8706,11 +8687,10 @@
       <c r="BI28" s="21"/>
       <c r="BJ28" s="21"/>
       <c r="BL28" s="17"/>
-      <c r="BM28" s="17"/>
+      <c r="BM28" s="1"/>
       <c r="BO28" s="18"/>
       <c r="BP28" s="19"/>
       <c r="BQ28" s="20"/>
-      <c r="BR28" s="17"/>
       <c r="BS28" s="17"/>
       <c r="BT28" s="17"/>
       <c r="BU28" s="17"/>
@@ -8869,22 +8849,22 @@
       <c r="HR28" s="17"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="75" t="s">
+      <c r="A29" s="71" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="71" t="s">
+      <c r="B29" s="72" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="72" t="s">
+      <c r="C29" s="74" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="73" t="s">
+      <c r="E29" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="74" t="s">
+      <c r="F29" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="17"/>
@@ -8937,11 +8917,10 @@
       <c r="BI29" s="21"/>
       <c r="BJ29" s="21"/>
       <c r="BL29" s="17"/>
-      <c r="BM29" s="17"/>
+      <c r="BM29" s="1"/>
       <c r="BO29" s="18"/>
       <c r="BP29" s="19"/>
       <c r="BQ29" s="20"/>
-      <c r="BR29" s="17"/>
       <c r="BS29" s="17"/>
       <c r="BT29" s="17"/>
       <c r="BU29" s="17"/>
@@ -9100,14 +9079,14 @@
       <c r="HR29" s="17"/>
     </row>
     <row r="30" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="75"/>
-      <c r="B30" s="75"/>
-      <c r="C30" s="75"/>
+      <c r="A30" s="71"/>
+      <c r="B30" s="71"/>
+      <c r="C30" s="71"/>
       <c r="D30" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="73"/>
-      <c r="F30" s="73"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="69"/>
       <c r="G30" s="17"/>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -9159,11 +9138,10 @@
       <c r="BI30" s="21"/>
       <c r="BJ30" s="21"/>
       <c r="BL30" s="17"/>
-      <c r="BM30" s="17"/>
+      <c r="BM30" s="1"/>
       <c r="BO30" s="18"/>
       <c r="BP30" s="19"/>
       <c r="BQ30" s="20"/>
-      <c r="BR30" s="17"/>
       <c r="BS30" s="17"/>
       <c r="BT30" s="17"/>
       <c r="BU30" s="17"/>
@@ -9322,20 +9300,20 @@
       <c r="HR30" s="17"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="75"/>
-      <c r="B31" s="71" t="s">
+      <c r="A31" s="71"/>
+      <c r="B31" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="72" t="s">
+      <c r="C31" s="74" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="73" t="s">
+      <c r="E31" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="74" t="s">
+      <c r="F31" s="70" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="17"/>
@@ -9389,11 +9367,10 @@
       <c r="BI31" s="21"/>
       <c r="BJ31" s="21"/>
       <c r="BL31" s="17"/>
-      <c r="BM31" s="17"/>
+      <c r="BM31" s="1"/>
       <c r="BO31" s="18"/>
       <c r="BP31" s="19"/>
       <c r="BQ31" s="20"/>
-      <c r="BR31" s="17"/>
       <c r="BS31" s="17"/>
       <c r="BT31" s="17"/>
       <c r="BU31" s="17"/>
@@ -9552,14 +9529,14 @@
       <c r="HR31" s="17"/>
     </row>
     <row r="32" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="75"/>
-      <c r="B32" s="75"/>
-      <c r="C32" s="75"/>
+      <c r="A32" s="71"/>
+      <c r="B32" s="71"/>
+      <c r="C32" s="71"/>
       <c r="D32" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="73"/>
-      <c r="F32" s="73"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="69"/>
       <c r="G32" s="17"/>
       <c r="H32" s="17"/>
       <c r="I32" s="17"/>
@@ -9611,11 +9588,10 @@
       <c r="BI32" s="21"/>
       <c r="BJ32" s="21"/>
       <c r="BL32" s="17"/>
-      <c r="BM32" s="17"/>
+      <c r="BM32" s="1"/>
       <c r="BO32" s="18"/>
       <c r="BP32" s="19"/>
       <c r="BQ32" s="20"/>
-      <c r="BR32" s="17"/>
       <c r="BS32" s="17"/>
       <c r="BT32" s="17"/>
       <c r="BU32" s="17"/>
@@ -9774,20 +9750,20 @@
       <c r="HR32" s="17"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="75"/>
-      <c r="B33" s="71" t="s">
+      <c r="A33" s="71"/>
+      <c r="B33" s="72" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="72" t="s">
+      <c r="C33" s="74" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="73" t="s">
+      <c r="E33" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="74" t="s">
+      <c r="F33" s="70" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="17"/>
@@ -9841,11 +9817,10 @@
       <c r="BI33" s="21"/>
       <c r="BJ33" s="21"/>
       <c r="BL33" s="17"/>
-      <c r="BM33" s="17"/>
+      <c r="BM33" s="1"/>
       <c r="BO33" s="18"/>
       <c r="BP33" s="19"/>
       <c r="BQ33" s="20"/>
-      <c r="BR33" s="17"/>
       <c r="BS33" s="17"/>
       <c r="BT33" s="17"/>
       <c r="BU33" s="17"/>
@@ -10004,14 +9979,14 @@
       <c r="HR33" s="17"/>
     </row>
     <row r="34" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="75"/>
-      <c r="B34" s="75"/>
-      <c r="C34" s="75"/>
+      <c r="A34" s="71"/>
+      <c r="B34" s="71"/>
+      <c r="C34" s="71"/>
       <c r="D34" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="73"/>
-      <c r="F34" s="73"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="69"/>
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
@@ -10063,11 +10038,10 @@
       <c r="BI34" s="21"/>
       <c r="BJ34" s="21"/>
       <c r="BL34" s="17"/>
-      <c r="BM34" s="17"/>
+      <c r="BM34" s="1"/>
       <c r="BO34" s="18"/>
       <c r="BP34" s="19"/>
       <c r="BQ34" s="20"/>
-      <c r="BR34" s="17"/>
       <c r="BS34" s="17"/>
       <c r="BT34" s="17"/>
       <c r="BU34" s="17"/>
@@ -10226,20 +10200,20 @@
       <c r="HR34" s="17"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="75"/>
-      <c r="B35" s="71" t="s">
+      <c r="A35" s="71"/>
+      <c r="B35" s="72" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="72" t="s">
+      <c r="C35" s="74" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="73" t="s">
+      <c r="E35" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="74" t="s">
+      <c r="F35" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="17"/>
@@ -10294,11 +10268,10 @@
       <c r="BI35" s="21"/>
       <c r="BJ35" s="21"/>
       <c r="BL35" s="17"/>
-      <c r="BM35" s="17"/>
+      <c r="BM35" s="1"/>
       <c r="BO35" s="18"/>
       <c r="BP35" s="19"/>
       <c r="BQ35" s="20"/>
-      <c r="BR35" s="17"/>
       <c r="BS35" s="17"/>
       <c r="BT35" s="17"/>
       <c r="BU35" s="17"/>
@@ -10457,14 +10430,14 @@
       <c r="HR35" s="17"/>
     </row>
     <row r="36" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="75"/>
-      <c r="B36" s="75"/>
-      <c r="C36" s="75"/>
+      <c r="A36" s="71"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="71"/>
       <c r="D36" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="73"/>
-      <c r="F36" s="73"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="69"/>
       <c r="G36" s="17"/>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
@@ -10517,11 +10490,10 @@
       <c r="BI36" s="42"/>
       <c r="BJ36" s="21"/>
       <c r="BL36" s="17"/>
-      <c r="BM36" s="17"/>
+      <c r="BM36" s="1"/>
       <c r="BO36" s="18"/>
       <c r="BP36" s="19"/>
       <c r="BQ36" s="20"/>
-      <c r="BR36" s="17"/>
       <c r="BS36" s="17"/>
       <c r="BT36" s="17"/>
       <c r="BU36" s="17"/>
@@ -10680,20 +10652,20 @@
       <c r="HR36" s="17"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="75"/>
-      <c r="B37" s="71" t="s">
+      <c r="A37" s="71"/>
+      <c r="B37" s="72" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="72" t="s">
+      <c r="C37" s="74" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="73" t="s">
+      <c r="E37" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="74" t="s">
+      <c r="F37" s="70" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="17"/>
@@ -10747,11 +10719,10 @@
       <c r="BI37" s="21"/>
       <c r="BJ37" s="21"/>
       <c r="BL37" s="17"/>
-      <c r="BM37" s="17"/>
+      <c r="BM37" s="1"/>
       <c r="BO37" s="18"/>
       <c r="BP37" s="19"/>
       <c r="BQ37" s="20"/>
-      <c r="BR37" s="17"/>
       <c r="BS37" s="17"/>
       <c r="BT37" s="17"/>
       <c r="BU37" s="17"/>
@@ -10910,14 +10881,14 @@
       <c r="HR37" s="17"/>
     </row>
     <row r="38" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="75"/>
-      <c r="B38" s="75"/>
-      <c r="C38" s="75"/>
+      <c r="A38" s="71"/>
+      <c r="B38" s="71"/>
+      <c r="C38" s="71"/>
       <c r="D38" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="73"/>
-      <c r="F38" s="73"/>
+      <c r="E38" s="69"/>
+      <c r="F38" s="69"/>
       <c r="G38" s="17"/>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -10969,11 +10940,10 @@
       <c r="BI38" s="21"/>
       <c r="BJ38" s="21"/>
       <c r="BL38" s="17"/>
-      <c r="BM38" s="17"/>
+      <c r="BM38" s="1"/>
       <c r="BO38" s="18"/>
       <c r="BP38" s="19"/>
       <c r="BQ38" s="20"/>
-      <c r="BR38" s="17"/>
       <c r="BS38" s="17"/>
       <c r="BT38" s="17"/>
       <c r="BU38" s="17"/>
@@ -11132,20 +11102,20 @@
       <c r="HR38" s="17"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="75"/>
-      <c r="B39" s="71" t="s">
+      <c r="A39" s="71"/>
+      <c r="B39" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="72" t="s">
+      <c r="C39" s="74" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="73" t="s">
+      <c r="E39" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="74" t="s">
+      <c r="F39" s="70" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="17"/>
@@ -11199,12 +11169,12 @@
       <c r="BI39" s="21"/>
       <c r="BJ39" s="21"/>
       <c r="BL39" s="17"/>
-      <c r="BM39" s="39"/>
-      <c r="BN39" s="68"/>
+      <c r="BM39" s="38"/>
+      <c r="BN39" s="38"/>
       <c r="BO39" s="18"/>
       <c r="BP39" s="19"/>
       <c r="BQ39" s="20"/>
-      <c r="BR39" s="39"/>
+      <c r="BR39" s="68"/>
       <c r="BS39" s="17"/>
       <c r="BT39" s="17"/>
       <c r="BU39" s="17"/>
@@ -11363,14 +11333,14 @@
       <c r="HR39" s="17"/>
     </row>
     <row r="40" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="75"/>
-      <c r="B40" s="75"/>
-      <c r="C40" s="75"/>
+      <c r="A40" s="71"/>
+      <c r="B40" s="71"/>
+      <c r="C40" s="71"/>
       <c r="D40" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="73"/>
-      <c r="F40" s="73"/>
+      <c r="E40" s="69"/>
+      <c r="F40" s="69"/>
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
@@ -11423,11 +11393,10 @@
       <c r="BI40" s="21"/>
       <c r="BJ40" s="21"/>
       <c r="BL40" s="17"/>
-      <c r="BM40" s="17"/>
+      <c r="BM40" s="1"/>
       <c r="BO40" s="18"/>
       <c r="BP40" s="19"/>
       <c r="BQ40" s="20"/>
-      <c r="BR40" s="17"/>
       <c r="BS40" s="17"/>
       <c r="BT40" s="17"/>
       <c r="BU40" s="17"/>
@@ -11586,22 +11555,22 @@
       <c r="HR40" s="17"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="75" t="s">
+      <c r="A41" s="71" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="71" t="s">
+      <c r="B41" s="72" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="72" t="s">
+      <c r="C41" s="74" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="73" t="s">
+      <c r="E41" s="69" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="74" t="s">
+      <c r="F41" s="70" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="17"/>
@@ -11655,11 +11624,10 @@
       <c r="BI41" s="21"/>
       <c r="BJ41" s="21"/>
       <c r="BL41" s="17"/>
-      <c r="BM41" s="17"/>
+      <c r="BM41" s="1"/>
       <c r="BO41" s="18"/>
       <c r="BP41" s="19"/>
       <c r="BQ41" s="20"/>
-      <c r="BR41" s="17"/>
       <c r="BS41" s="17"/>
       <c r="BT41" s="17"/>
       <c r="BU41" s="17"/>
@@ -11818,14 +11786,14 @@
       <c r="HR41" s="17"/>
     </row>
     <row r="42" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="75"/>
-      <c r="B42" s="75"/>
-      <c r="C42" s="75"/>
+      <c r="A42" s="71"/>
+      <c r="B42" s="71"/>
+      <c r="C42" s="71"/>
       <c r="D42" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="73"/>
-      <c r="F42" s="73"/>
+      <c r="E42" s="69"/>
+      <c r="F42" s="69"/>
       <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
@@ -11877,11 +11845,10 @@
       <c r="BI42" s="21"/>
       <c r="BJ42" s="21"/>
       <c r="BL42" s="17"/>
-      <c r="BM42" s="17"/>
+      <c r="BM42" s="1"/>
       <c r="BO42" s="18"/>
       <c r="BP42" s="19"/>
       <c r="BQ42" s="20"/>
-      <c r="BR42" s="17"/>
       <c r="BS42" s="17"/>
       <c r="BT42" s="17"/>
       <c r="BU42" s="17"/>
@@ -12040,20 +12007,20 @@
       <c r="HR42" s="17"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="75"/>
-      <c r="B43" s="71" t="s">
+      <c r="A43" s="71"/>
+      <c r="B43" s="72" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="72" t="s">
+      <c r="C43" s="74" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="73" t="s">
+      <c r="E43" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="74" t="s">
+      <c r="F43" s="70" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="17"/>
@@ -12106,11 +12073,10 @@
       <c r="BI43" s="21"/>
       <c r="BJ43" s="21"/>
       <c r="BL43" s="17"/>
-      <c r="BM43" s="17"/>
+      <c r="BM43" s="1"/>
       <c r="BO43" s="18"/>
       <c r="BP43" s="19"/>
       <c r="BQ43" s="20"/>
-      <c r="BR43" s="17"/>
       <c r="BS43" s="17"/>
       <c r="BT43" s="17"/>
       <c r="BU43" s="17"/>
@@ -12269,14 +12235,14 @@
       <c r="HR43" s="17"/>
     </row>
     <row r="44" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="75"/>
-      <c r="B44" s="75"/>
-      <c r="C44" s="75"/>
+      <c r="A44" s="71"/>
+      <c r="B44" s="71"/>
+      <c r="C44" s="71"/>
       <c r="D44" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="73"/>
-      <c r="F44" s="73"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="69"/>
       <c r="G44" s="17"/>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -12330,11 +12296,10 @@
       <c r="BI44" s="21"/>
       <c r="BJ44" s="21"/>
       <c r="BL44" s="17"/>
-      <c r="BM44" s="17"/>
+      <c r="BM44" s="1"/>
       <c r="BO44" s="18"/>
       <c r="BP44" s="19"/>
       <c r="BQ44" s="20"/>
-      <c r="BR44" s="17"/>
       <c r="BS44" s="17"/>
       <c r="BT44" s="17"/>
       <c r="BU44" s="17"/>
@@ -12493,20 +12458,20 @@
       <c r="HR44" s="17"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="75"/>
-      <c r="B45" s="71" t="s">
+      <c r="A45" s="71"/>
+      <c r="B45" s="72" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="72" t="s">
+      <c r="C45" s="74" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="73" t="s">
+      <c r="E45" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="74" t="s">
+      <c r="F45" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="17"/>
@@ -12560,11 +12525,10 @@
       <c r="BI45" s="21"/>
       <c r="BJ45" s="21"/>
       <c r="BL45" s="17"/>
-      <c r="BM45" s="17"/>
+      <c r="BM45" s="1"/>
       <c r="BO45" s="18"/>
       <c r="BP45" s="19"/>
       <c r="BQ45" s="20"/>
-      <c r="BR45" s="17"/>
       <c r="BS45" s="17"/>
       <c r="BT45" s="17"/>
       <c r="BU45" s="17"/>
@@ -12723,14 +12687,14 @@
       <c r="HR45" s="17"/>
     </row>
     <row r="46" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="75"/>
-      <c r="B46" s="75"/>
-      <c r="C46" s="75"/>
+      <c r="A46" s="71"/>
+      <c r="B46" s="71"/>
+      <c r="C46" s="71"/>
       <c r="D46" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="73"/>
-      <c r="F46" s="73"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="69"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
@@ -12783,11 +12747,10 @@
       <c r="BI46" s="21"/>
       <c r="BJ46" s="21"/>
       <c r="BL46" s="17"/>
-      <c r="BM46" s="17"/>
+      <c r="BM46" s="1"/>
       <c r="BO46" s="18"/>
       <c r="BP46" s="19"/>
       <c r="BQ46" s="20"/>
-      <c r="BR46" s="17"/>
       <c r="BS46" s="17"/>
       <c r="BT46" s="17"/>
       <c r="BU46" s="17"/>
@@ -12946,22 +12909,22 @@
       <c r="HR46" s="17"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="75" t="s">
+      <c r="A47" s="71" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="71" t="s">
+      <c r="B47" s="72" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="72" t="s">
+      <c r="C47" s="74" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="73" t="s">
+      <c r="E47" s="69" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="74" t="s">
+      <c r="F47" s="70" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="17"/>
@@ -13018,11 +12981,10 @@
       <c r="BI47" s="21"/>
       <c r="BJ47" s="21"/>
       <c r="BL47" s="17"/>
-      <c r="BM47" s="17"/>
+      <c r="BM47" s="1"/>
       <c r="BO47" s="18"/>
       <c r="BP47" s="19"/>
       <c r="BQ47" s="20"/>
-      <c r="BR47" s="17"/>
       <c r="BS47" s="17"/>
       <c r="BT47" s="17"/>
       <c r="BU47" s="17"/>
@@ -13181,14 +13143,14 @@
       <c r="HR47" s="17"/>
     </row>
     <row r="48" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="75"/>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
+      <c r="A48" s="71"/>
+      <c r="B48" s="71"/>
+      <c r="C48" s="71"/>
       <c r="D48" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="73"/>
-      <c r="F48" s="73"/>
+      <c r="E48" s="69"/>
+      <c r="F48" s="69"/>
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
@@ -13242,11 +13204,10 @@
       <c r="BI48" s="21"/>
       <c r="BJ48" s="21"/>
       <c r="BL48" s="17"/>
-      <c r="BM48" s="17"/>
+      <c r="BM48" s="1"/>
       <c r="BO48" s="18"/>
       <c r="BP48" s="19"/>
       <c r="BQ48" s="20"/>
-      <c r="BR48" s="17"/>
       <c r="BS48" s="17"/>
       <c r="BT48" s="17"/>
       <c r="BU48" s="17"/>
@@ -13405,20 +13366,20 @@
       <c r="HR48" s="17"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="75"/>
-      <c r="B49" s="71" t="s">
+      <c r="A49" s="71"/>
+      <c r="B49" s="72" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="72" t="s">
+      <c r="C49" s="74" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="73" t="s">
+      <c r="E49" s="69" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="74" t="s">
+      <c r="F49" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="17"/>
@@ -13473,11 +13434,10 @@
       <c r="BJ49" s="21"/>
       <c r="BK49" s="27"/>
       <c r="BL49" s="16"/>
-      <c r="BM49" s="17"/>
+      <c r="BM49" s="1"/>
       <c r="BO49" s="18"/>
       <c r="BP49" s="19"/>
       <c r="BQ49" s="20"/>
-      <c r="BR49" s="17"/>
       <c r="BS49" s="17"/>
       <c r="BT49" s="17"/>
       <c r="BU49" s="17"/>
@@ -13636,14 +13596,14 @@
       <c r="HR49" s="17"/>
     </row>
     <row r="50" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="75"/>
-      <c r="B50" s="75"/>
-      <c r="C50" s="75"/>
+      <c r="A50" s="71"/>
+      <c r="B50" s="71"/>
+      <c r="C50" s="71"/>
       <c r="D50" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="73"/>
-      <c r="F50" s="73"/>
+      <c r="E50" s="69"/>
+      <c r="F50" s="69"/>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
@@ -13696,11 +13656,10 @@
       <c r="BJ50" s="21"/>
       <c r="BK50" s="42"/>
       <c r="BL50" s="42"/>
-      <c r="BM50" s="17"/>
+      <c r="BM50" s="1"/>
       <c r="BO50" s="18"/>
       <c r="BP50" s="19"/>
       <c r="BQ50" s="20"/>
-      <c r="BR50" s="17"/>
       <c r="BS50" s="17"/>
       <c r="BT50" s="17"/>
       <c r="BU50" s="17"/>
@@ -13859,22 +13818,22 @@
       <c r="HR50" s="17"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="71" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="71" t="s">
+      <c r="B51" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="72" t="s">
+      <c r="C51" s="74" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="73" t="s">
+      <c r="E51" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="74" t="s">
+      <c r="F51" s="70" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="17"/>
@@ -13928,11 +13887,10 @@
       <c r="BI51" s="21"/>
       <c r="BJ51" s="21"/>
       <c r="BL51" s="17"/>
-      <c r="BM51" s="17"/>
+      <c r="BM51" s="1"/>
       <c r="BO51" s="18"/>
       <c r="BP51" s="19"/>
       <c r="BQ51" s="20"/>
-      <c r="BR51" s="17"/>
       <c r="BS51" s="16"/>
       <c r="BT51" s="16"/>
       <c r="BU51" s="16"/>
@@ -14091,14 +14049,14 @@
       <c r="HR51" s="17"/>
     </row>
     <row r="52" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="75"/>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
+      <c r="A52" s="71"/>
+      <c r="B52" s="71"/>
+      <c r="C52" s="71"/>
       <c r="D52" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="73"/>
-      <c r="F52" s="73"/>
+      <c r="E52" s="69"/>
+      <c r="F52" s="69"/>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
@@ -14154,7 +14112,6 @@
       <c r="BO52" s="18"/>
       <c r="BP52" s="19"/>
       <c r="BQ52" s="20"/>
-      <c r="BR52" s="17"/>
       <c r="BS52" s="17"/>
       <c r="BT52" s="17"/>
       <c r="BU52" s="17"/>
@@ -14313,20 +14270,20 @@
       <c r="HR52" s="17"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="75"/>
-      <c r="B53" s="71" t="s">
+      <c r="A53" s="71"/>
+      <c r="B53" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="72" t="s">
+      <c r="C53" s="74" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="69" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="74" t="s">
+      <c r="F53" s="70" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="17"/>
@@ -14380,11 +14337,10 @@
       <c r="BI53" s="21"/>
       <c r="BJ53" s="21"/>
       <c r="BL53" s="17"/>
-      <c r="BM53" s="17"/>
+      <c r="BM53" s="1"/>
       <c r="BO53" s="18"/>
       <c r="BP53" s="19"/>
       <c r="BQ53" s="20"/>
-      <c r="BR53" s="17"/>
       <c r="BS53" s="17"/>
       <c r="BT53" s="17"/>
       <c r="BU53" s="17"/>
@@ -14543,14 +14499,14 @@
       <c r="HR53" s="17"/>
     </row>
     <row r="54" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="75"/>
-      <c r="B54" s="75"/>
-      <c r="C54" s="75"/>
+      <c r="A54" s="71"/>
+      <c r="B54" s="71"/>
+      <c r="C54" s="71"/>
       <c r="D54" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="73"/>
-      <c r="F54" s="73"/>
+      <c r="E54" s="69"/>
+      <c r="F54" s="69"/>
       <c r="G54" s="17"/>
       <c r="H54" s="17"/>
       <c r="I54" s="17"/>
@@ -14602,11 +14558,10 @@
       <c r="BI54" s="21"/>
       <c r="BJ54" s="21"/>
       <c r="BL54" s="17"/>
-      <c r="BM54" s="17"/>
+      <c r="BM54" s="1"/>
       <c r="BO54" s="18"/>
       <c r="BP54" s="19"/>
       <c r="BQ54" s="20"/>
-      <c r="BR54" s="17"/>
       <c r="BS54" s="17"/>
       <c r="BT54" s="17"/>
       <c r="BU54" s="17"/>
@@ -14765,22 +14720,22 @@
       <c r="HR54" s="17"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="75" t="s">
+      <c r="A55" s="71" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="71" t="s">
+      <c r="B55" s="72" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="72" t="s">
+      <c r="C55" s="74" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="73" t="s">
+      <c r="E55" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="74" t="s">
+      <c r="F55" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="17"/>
@@ -14834,11 +14789,10 @@
       <c r="BI55" s="21"/>
       <c r="BJ55" s="21"/>
       <c r="BL55" s="17"/>
-      <c r="BM55" s="17"/>
+      <c r="BM55" s="1"/>
       <c r="BO55" s="18"/>
       <c r="BP55" s="19"/>
       <c r="BQ55" s="20"/>
-      <c r="BR55" s="17"/>
       <c r="BS55" s="17"/>
       <c r="BT55" s="17"/>
       <c r="BU55" s="17"/>
@@ -14997,14 +14951,14 @@
       <c r="HR55" s="17"/>
     </row>
     <row r="56" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="75"/>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
+      <c r="A56" s="71"/>
+      <c r="B56" s="71"/>
+      <c r="C56" s="71"/>
       <c r="D56" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="73"/>
-      <c r="F56" s="73"/>
+      <c r="E56" s="69"/>
+      <c r="F56" s="69"/>
       <c r="G56" s="17"/>
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
@@ -15056,11 +15010,10 @@
       <c r="BI56" s="21"/>
       <c r="BJ56" s="21"/>
       <c r="BL56" s="17"/>
-      <c r="BM56" s="17"/>
+      <c r="BM56" s="1"/>
       <c r="BO56" s="18"/>
       <c r="BP56" s="19"/>
       <c r="BQ56" s="20"/>
-      <c r="BR56" s="17"/>
       <c r="BS56" s="17"/>
       <c r="BT56" s="17"/>
       <c r="BU56" s="17"/>
@@ -15219,20 +15172,20 @@
       <c r="HR56" s="17"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="75"/>
-      <c r="B57" s="71" t="s">
+      <c r="A57" s="71"/>
+      <c r="B57" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="C57" s="72" t="s">
+      <c r="C57" s="74" t="s">
         <v>124</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="73" t="s">
+      <c r="E57" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="F57" s="74" t="s">
+      <c r="F57" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="17"/>
@@ -15286,11 +15239,10 @@
       <c r="BI57" s="21"/>
       <c r="BJ57" s="21"/>
       <c r="BL57" s="17"/>
-      <c r="BM57" s="17"/>
+      <c r="BM57" s="1"/>
       <c r="BO57" s="18"/>
       <c r="BP57" s="19"/>
       <c r="BQ57" s="20"/>
-      <c r="BR57" s="17"/>
       <c r="BS57" s="17"/>
       <c r="BT57" s="17"/>
       <c r="BU57" s="17"/>
@@ -15449,14 +15401,14 @@
       <c r="HR57" s="17"/>
     </row>
     <row r="58" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="75"/>
-      <c r="B58" s="75"/>
-      <c r="C58" s="75"/>
+      <c r="A58" s="71"/>
+      <c r="B58" s="71"/>
+      <c r="C58" s="71"/>
       <c r="D58" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="73"/>
-      <c r="F58" s="73"/>
+      <c r="E58" s="69"/>
+      <c r="F58" s="69"/>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
@@ -15508,11 +15460,10 @@
       <c r="BI58" s="21"/>
       <c r="BJ58" s="21"/>
       <c r="BL58" s="17"/>
-      <c r="BM58" s="17"/>
+      <c r="BM58" s="1"/>
       <c r="BO58" s="18"/>
       <c r="BP58" s="19"/>
       <c r="BQ58" s="20"/>
-      <c r="BR58" s="17"/>
       <c r="BS58" s="17"/>
       <c r="BT58" s="17"/>
       <c r="BU58" s="17"/>
@@ -15671,20 +15622,20 @@
       <c r="HR58" s="17"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="75"/>
-      <c r="B59" s="71" t="s">
+      <c r="A59" s="71"/>
+      <c r="B59" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="C59" s="72" t="s">
+      <c r="C59" s="74" t="s">
         <v>127</v>
       </c>
       <c r="D59" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="73" t="s">
+      <c r="E59" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="F59" s="74" t="s">
+      <c r="F59" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="17"/>
@@ -15738,11 +15689,10 @@
       <c r="BI59" s="21"/>
       <c r="BJ59" s="21"/>
       <c r="BL59" s="17"/>
-      <c r="BM59" s="17"/>
+      <c r="BM59" s="1"/>
       <c r="BO59" s="18"/>
       <c r="BP59" s="19"/>
       <c r="BQ59" s="20"/>
-      <c r="BR59" s="17"/>
       <c r="BS59" s="17"/>
       <c r="BT59" s="17"/>
       <c r="BU59" s="17"/>
@@ -15901,14 +15851,14 @@
       <c r="HR59" s="17"/>
     </row>
     <row r="60" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="75"/>
-      <c r="B60" s="75"/>
-      <c r="C60" s="75"/>
+      <c r="A60" s="71"/>
+      <c r="B60" s="71"/>
+      <c r="C60" s="71"/>
       <c r="D60" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="73"/>
-      <c r="F60" s="73"/>
+      <c r="E60" s="69"/>
+      <c r="F60" s="69"/>
       <c r="G60" s="17"/>
       <c r="H60" s="17"/>
       <c r="I60" s="17"/>
@@ -15960,11 +15910,10 @@
       <c r="BI60" s="21"/>
       <c r="BJ60" s="21"/>
       <c r="BL60" s="17"/>
-      <c r="BM60" s="17"/>
+      <c r="BM60" s="1"/>
       <c r="BO60" s="18"/>
       <c r="BP60" s="19"/>
       <c r="BQ60" s="20"/>
-      <c r="BR60" s="17"/>
       <c r="BS60" s="17"/>
       <c r="BT60" s="17"/>
       <c r="BU60" s="17"/>
@@ -16123,20 +16072,20 @@
       <c r="HR60" s="17"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="75"/>
-      <c r="B61" s="71" t="s">
+      <c r="A61" s="71"/>
+      <c r="B61" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="C61" s="72" t="s">
+      <c r="C61" s="74" t="s">
         <v>130</v>
       </c>
       <c r="D61" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="73" t="s">
+      <c r="E61" s="69" t="s">
         <v>131</v>
       </c>
-      <c r="F61" s="74" t="s">
+      <c r="F61" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="17"/>
@@ -16190,11 +16139,10 @@
       <c r="BI61" s="21"/>
       <c r="BJ61" s="21"/>
       <c r="BL61" s="17"/>
-      <c r="BM61" s="17"/>
+      <c r="BM61" s="1"/>
       <c r="BO61" s="18"/>
       <c r="BP61" s="19"/>
       <c r="BQ61" s="20"/>
-      <c r="BR61" s="17"/>
       <c r="BS61" s="17"/>
       <c r="BT61" s="17"/>
       <c r="BU61" s="17"/>
@@ -16353,14 +16301,14 @@
       <c r="HR61" s="17"/>
     </row>
     <row r="62" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="75"/>
-      <c r="B62" s="75"/>
-      <c r="C62" s="75"/>
+      <c r="A62" s="71"/>
+      <c r="B62" s="71"/>
+      <c r="C62" s="71"/>
       <c r="D62" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="73"/>
-      <c r="F62" s="73"/>
+      <c r="E62" s="69"/>
+      <c r="F62" s="69"/>
       <c r="G62" s="17"/>
       <c r="H62" s="17"/>
       <c r="I62" s="17"/>
@@ -16412,11 +16360,10 @@
       <c r="BI62" s="21"/>
       <c r="BJ62" s="21"/>
       <c r="BL62" s="17"/>
-      <c r="BM62" s="17"/>
+      <c r="BM62" s="1"/>
       <c r="BO62" s="18"/>
       <c r="BP62" s="19"/>
       <c r="BQ62" s="20"/>
-      <c r="BR62" s="17"/>
       <c r="BS62" s="17"/>
       <c r="BT62" s="17"/>
       <c r="BU62" s="17"/>
@@ -16575,20 +16522,20 @@
       <c r="HR62" s="17"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="75"/>
-      <c r="B63" s="71" t="s">
+      <c r="A63" s="71"/>
+      <c r="B63" s="72" t="s">
         <v>132</v>
       </c>
-      <c r="C63" s="72" t="s">
+      <c r="C63" s="74" t="s">
         <v>133</v>
       </c>
       <c r="D63" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="73" t="s">
+      <c r="E63" s="69" t="s">
         <v>134</v>
       </c>
-      <c r="F63" s="74" t="s">
+      <c r="F63" s="70" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="17"/>
@@ -16642,11 +16589,10 @@
       <c r="BI63" s="21"/>
       <c r="BJ63" s="21"/>
       <c r="BL63" s="17"/>
-      <c r="BM63" s="17"/>
+      <c r="BM63" s="1"/>
       <c r="BO63" s="18"/>
       <c r="BP63" s="19"/>
       <c r="BQ63" s="20"/>
-      <c r="BR63" s="17"/>
       <c r="BS63" s="17"/>
       <c r="BT63" s="17"/>
       <c r="BU63" s="17"/>
@@ -16805,14 +16751,14 @@
       <c r="HR63" s="17"/>
     </row>
     <row r="64" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="75"/>
-      <c r="B64" s="75"/>
-      <c r="C64" s="75"/>
+      <c r="A64" s="71"/>
+      <c r="B64" s="71"/>
+      <c r="C64" s="71"/>
       <c r="D64" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="73"/>
-      <c r="F64" s="73"/>
+      <c r="E64" s="69"/>
+      <c r="F64" s="69"/>
       <c r="G64" s="17"/>
       <c r="H64" s="17"/>
       <c r="I64" s="17"/>
@@ -16864,11 +16810,10 @@
       <c r="BI64" s="21"/>
       <c r="BJ64" s="21"/>
       <c r="BL64" s="17"/>
-      <c r="BM64" s="17"/>
+      <c r="BM64" s="1"/>
       <c r="BO64" s="18"/>
       <c r="BP64" s="19"/>
       <c r="BQ64" s="20"/>
-      <c r="BR64" s="17"/>
       <c r="BS64" s="17"/>
       <c r="BT64" s="17"/>
       <c r="BU64" s="17"/>
@@ -17027,20 +16972,20 @@
       <c r="HR64" s="17"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="75"/>
-      <c r="B65" s="71" t="s">
+      <c r="A65" s="71"/>
+      <c r="B65" s="72" t="s">
         <v>135</v>
       </c>
-      <c r="C65" s="72" t="s">
+      <c r="C65" s="74" t="s">
         <v>136</v>
       </c>
       <c r="D65" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="73" t="s">
+      <c r="E65" s="69" t="s">
         <v>137</v>
       </c>
-      <c r="F65" s="74" t="s">
+      <c r="F65" s="70" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="17"/>
@@ -17094,11 +17039,10 @@
       <c r="BI65" s="21"/>
       <c r="BJ65" s="21"/>
       <c r="BL65" s="17"/>
-      <c r="BM65" s="17"/>
+      <c r="BM65" s="1"/>
       <c r="BO65" s="18"/>
       <c r="BP65" s="19"/>
       <c r="BQ65" s="20"/>
-      <c r="BR65" s="17"/>
       <c r="BS65" s="17"/>
       <c r="BT65" s="17"/>
       <c r="BU65" s="17"/>
@@ -17257,14 +17201,14 @@
       <c r="HR65" s="17"/>
     </row>
     <row r="66" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="75"/>
-      <c r="B66" s="75"/>
-      <c r="C66" s="75"/>
+      <c r="A66" s="71"/>
+      <c r="B66" s="71"/>
+      <c r="C66" s="71"/>
       <c r="D66" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="73"/>
-      <c r="F66" s="73"/>
+      <c r="E66" s="69"/>
+      <c r="F66" s="69"/>
       <c r="G66" s="17"/>
       <c r="H66" s="17"/>
       <c r="I66" s="17"/>
@@ -17316,11 +17260,10 @@
       <c r="BI66" s="21"/>
       <c r="BJ66" s="21"/>
       <c r="BL66" s="17"/>
-      <c r="BM66" s="17"/>
+      <c r="BM66" s="1"/>
       <c r="BO66" s="18"/>
       <c r="BP66" s="19"/>
       <c r="BQ66" s="20"/>
-      <c r="BR66" s="17"/>
       <c r="BS66" s="17"/>
       <c r="BT66" s="17"/>
       <c r="BU66" s="17"/>
@@ -17479,22 +17422,22 @@
       <c r="HR66" s="17"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="75" t="s">
+      <c r="A67" s="71" t="s">
         <v>138</v>
       </c>
-      <c r="B67" s="71" t="s">
+      <c r="B67" s="72" t="s">
         <v>139</v>
       </c>
-      <c r="C67" s="72" t="s">
+      <c r="C67" s="74" t="s">
         <v>140</v>
       </c>
       <c r="D67" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="73" t="s">
+      <c r="E67" s="69" t="s">
         <v>141</v>
       </c>
-      <c r="F67" s="74" t="s">
+      <c r="F67" s="70" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="17"/>
@@ -17548,11 +17491,10 @@
       <c r="BI67" s="21"/>
       <c r="BJ67" s="21"/>
       <c r="BL67" s="17"/>
-      <c r="BM67" s="17"/>
+      <c r="BM67" s="1"/>
       <c r="BO67" s="18"/>
       <c r="BP67" s="19"/>
       <c r="BQ67" s="20"/>
-      <c r="BR67" s="17"/>
       <c r="BS67" s="17"/>
       <c r="BT67" s="17"/>
       <c r="BU67" s="17"/>
@@ -17711,14 +17653,14 @@
       <c r="HR67" s="17"/>
     </row>
     <row r="68" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="75"/>
-      <c r="B68" s="75"/>
-      <c r="C68" s="75"/>
+      <c r="A68" s="71"/>
+      <c r="B68" s="71"/>
+      <c r="C68" s="71"/>
       <c r="D68" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="73"/>
-      <c r="F68" s="73"/>
+      <c r="E68" s="69"/>
+      <c r="F68" s="69"/>
       <c r="G68" s="17"/>
       <c r="H68" s="17"/>
       <c r="I68" s="17"/>
@@ -17771,11 +17713,10 @@
       <c r="BI68" s="21"/>
       <c r="BJ68" s="21"/>
       <c r="BL68" s="17"/>
-      <c r="BM68" s="17"/>
+      <c r="BM68" s="1"/>
       <c r="BO68" s="18"/>
       <c r="BP68" s="19"/>
       <c r="BQ68" s="20"/>
-      <c r="BR68" s="17"/>
       <c r="BS68" s="17"/>
       <c r="BT68" s="17"/>
       <c r="BU68" s="17"/>
@@ -17934,20 +17875,20 @@
       <c r="HR68" s="17"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="75"/>
-      <c r="B69" s="71" t="s">
+      <c r="A69" s="71"/>
+      <c r="B69" s="72" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="72" t="s">
+      <c r="C69" s="74" t="s">
         <v>143</v>
       </c>
       <c r="D69" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="73" t="s">
+      <c r="E69" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="F69" s="74" t="s">
+      <c r="F69" s="70" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="17"/>
@@ -18008,12 +17949,12 @@
       <c r="BJ69" s="21"/>
       <c r="BK69" s="38"/>
       <c r="BL69" s="39"/>
-      <c r="BM69" s="39"/>
-      <c r="BN69" s="68"/>
+      <c r="BM69" s="38"/>
+      <c r="BN69" s="38"/>
       <c r="BO69" s="18"/>
       <c r="BP69" s="19"/>
       <c r="BQ69" s="20"/>
-      <c r="BR69" s="39"/>
+      <c r="BR69" s="68"/>
       <c r="BS69" s="39"/>
       <c r="BT69" s="39"/>
       <c r="BU69" s="39"/>
@@ -18172,14 +18113,14 @@
       <c r="HR69" s="17"/>
     </row>
     <row r="70" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="75"/>
-      <c r="B70" s="75"/>
-      <c r="C70" s="75"/>
+      <c r="A70" s="71"/>
+      <c r="B70" s="71"/>
+      <c r="C70" s="71"/>
       <c r="D70" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="73"/>
-      <c r="F70" s="73"/>
+      <c r="E70" s="69"/>
+      <c r="F70" s="69"/>
       <c r="G70" s="17"/>
       <c r="H70" s="17"/>
       <c r="I70" s="17"/>
@@ -18238,7 +18179,7 @@
       <c r="BO70" s="18"/>
       <c r="BP70" s="19"/>
       <c r="BQ70" s="20"/>
-      <c r="BR70" s="17"/>
+      <c r="BR70" s="84"/>
       <c r="BS70" s="17"/>
       <c r="BT70" s="17"/>
       <c r="BU70" s="17"/>
@@ -18397,20 +18338,20 @@
       <c r="HR70" s="17"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="75"/>
-      <c r="B71" s="71" t="s">
+      <c r="A71" s="71"/>
+      <c r="B71" s="72" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="72" t="s">
+      <c r="C71" s="74" t="s">
         <v>146</v>
       </c>
       <c r="D71" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="73" t="s">
+      <c r="E71" s="69" t="s">
         <v>147</v>
       </c>
-      <c r="F71" s="74" t="s">
+      <c r="F71" s="70" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="17"/>
@@ -18464,11 +18405,10 @@
       <c r="BI71" s="21"/>
       <c r="BJ71" s="21"/>
       <c r="BL71" s="17"/>
-      <c r="BM71" s="17"/>
+      <c r="BM71" s="1"/>
       <c r="BO71" s="18"/>
       <c r="BP71" s="19"/>
       <c r="BQ71" s="20"/>
-      <c r="BR71" s="17"/>
       <c r="BS71" s="17"/>
       <c r="BT71" s="17"/>
       <c r="BU71" s="17"/>
@@ -18627,14 +18567,14 @@
       <c r="HR71" s="17"/>
     </row>
     <row r="72" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="75"/>
-      <c r="B72" s="75"/>
-      <c r="C72" s="75"/>
+      <c r="A72" s="71"/>
+      <c r="B72" s="71"/>
+      <c r="C72" s="71"/>
       <c r="D72" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="73"/>
-      <c r="F72" s="73"/>
+      <c r="E72" s="69"/>
+      <c r="F72" s="69"/>
       <c r="G72" s="17"/>
       <c r="H72" s="17"/>
       <c r="I72" s="17"/>
@@ -18686,11 +18626,10 @@
       <c r="BI72" s="21"/>
       <c r="BJ72" s="21"/>
       <c r="BL72" s="17"/>
-      <c r="BM72" s="17"/>
+      <c r="BM72" s="1"/>
       <c r="BO72" s="18"/>
       <c r="BP72" s="19"/>
       <c r="BQ72" s="20"/>
-      <c r="BR72" s="17"/>
       <c r="BS72" s="17"/>
       <c r="BT72" s="17"/>
       <c r="BU72" s="17"/>
@@ -18849,20 +18788,20 @@
       <c r="HR72" s="17"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="75"/>
-      <c r="B73" s="71" t="s">
+      <c r="A73" s="71"/>
+      <c r="B73" s="72" t="s">
         <v>148</v>
       </c>
-      <c r="C73" s="72" t="s">
+      <c r="C73" s="74" t="s">
         <v>149</v>
       </c>
       <c r="D73" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="73" t="s">
+      <c r="E73" s="69" t="s">
         <v>150</v>
       </c>
-      <c r="F73" s="74" t="s">
+      <c r="F73" s="70" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="17"/>
@@ -18916,11 +18855,10 @@
       <c r="BI73" s="21"/>
       <c r="BJ73" s="21"/>
       <c r="BL73" s="17"/>
-      <c r="BM73" s="17"/>
+      <c r="BM73" s="1"/>
       <c r="BO73" s="18"/>
       <c r="BP73" s="19"/>
       <c r="BQ73" s="20"/>
-      <c r="BR73" s="17"/>
       <c r="BS73" s="17"/>
       <c r="BT73" s="17"/>
       <c r="BU73" s="17"/>
@@ -19079,14 +19017,14 @@
       <c r="HR73" s="17"/>
     </row>
     <row r="74" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="75"/>
-      <c r="B74" s="75"/>
-      <c r="C74" s="75"/>
+      <c r="A74" s="71"/>
+      <c r="B74" s="71"/>
+      <c r="C74" s="71"/>
       <c r="D74" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="73"/>
-      <c r="F74" s="73"/>
+      <c r="E74" s="69"/>
+      <c r="F74" s="69"/>
       <c r="G74" s="17"/>
       <c r="H74" s="17"/>
       <c r="I74" s="17"/>
@@ -19138,11 +19076,10 @@
       <c r="BI74" s="21"/>
       <c r="BJ74" s="21"/>
       <c r="BL74" s="17"/>
-      <c r="BM74" s="17"/>
+      <c r="BM74" s="1"/>
       <c r="BO74" s="18"/>
       <c r="BP74" s="19"/>
       <c r="BQ74" s="20"/>
-      <c r="BR74" s="17"/>
       <c r="BS74" s="17"/>
       <c r="BT74" s="17"/>
       <c r="BU74" s="17"/>
@@ -19301,20 +19238,20 @@
       <c r="HR74" s="17"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="75"/>
-      <c r="B75" s="71" t="s">
+      <c r="A75" s="71"/>
+      <c r="B75" s="72" t="s">
         <v>151</v>
       </c>
-      <c r="C75" s="72" t="s">
+      <c r="C75" s="74" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="73" t="s">
+      <c r="E75" s="69" t="s">
         <v>153</v>
       </c>
-      <c r="F75" s="74" t="s">
+      <c r="F75" s="70" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="17"/>
@@ -19368,11 +19305,10 @@
       <c r="BI75" s="21"/>
       <c r="BJ75" s="21"/>
       <c r="BL75" s="17"/>
-      <c r="BM75" s="17"/>
+      <c r="BM75" s="1"/>
       <c r="BO75" s="18"/>
       <c r="BP75" s="19"/>
       <c r="BQ75" s="20"/>
-      <c r="BR75" s="17"/>
       <c r="BS75" s="17"/>
       <c r="BT75" s="17"/>
       <c r="BU75" s="17"/>
@@ -19531,14 +19467,14 @@
       <c r="HR75" s="17"/>
     </row>
     <row r="76" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="75"/>
-      <c r="B76" s="75"/>
-      <c r="C76" s="75"/>
+      <c r="A76" s="71"/>
+      <c r="B76" s="71"/>
+      <c r="C76" s="71"/>
       <c r="D76" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="73"/>
-      <c r="F76" s="73"/>
+      <c r="E76" s="69"/>
+      <c r="F76" s="69"/>
       <c r="G76" s="17"/>
       <c r="H76" s="17"/>
       <c r="I76" s="17"/>
@@ -19590,11 +19526,10 @@
       <c r="BI76" s="21"/>
       <c r="BJ76" s="21"/>
       <c r="BL76" s="17"/>
-      <c r="BM76" s="17"/>
+      <c r="BM76" s="1"/>
       <c r="BO76" s="18"/>
       <c r="BP76" s="19"/>
       <c r="BQ76" s="20"/>
-      <c r="BR76" s="17"/>
       <c r="BS76" s="17"/>
       <c r="BT76" s="17"/>
       <c r="BU76" s="17"/>
@@ -19753,20 +19688,20 @@
       <c r="HR76" s="17"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="75"/>
-      <c r="B77" s="71" t="s">
+      <c r="A77" s="71"/>
+      <c r="B77" s="72" t="s">
         <v>154</v>
       </c>
-      <c r="C77" s="72" t="s">
+      <c r="C77" s="74" t="s">
         <v>155</v>
       </c>
       <c r="D77" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="73" t="s">
+      <c r="E77" s="69" t="s">
         <v>156</v>
       </c>
-      <c r="F77" s="74" t="s">
+      <c r="F77" s="70" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="17"/>
@@ -19820,11 +19755,10 @@
       <c r="BI77" s="21"/>
       <c r="BJ77" s="21"/>
       <c r="BL77" s="17"/>
-      <c r="BM77" s="17"/>
+      <c r="BM77" s="1"/>
       <c r="BO77" s="18"/>
       <c r="BP77" s="19"/>
       <c r="BQ77" s="20"/>
-      <c r="BR77" s="17"/>
       <c r="BS77" s="17"/>
       <c r="BT77" s="17"/>
       <c r="BU77" s="17"/>
@@ -19983,14 +19917,14 @@
       <c r="HR77" s="17"/>
     </row>
     <row r="78" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="75"/>
-      <c r="B78" s="75"/>
-      <c r="C78" s="75"/>
+      <c r="A78" s="71"/>
+      <c r="B78" s="71"/>
+      <c r="C78" s="71"/>
       <c r="D78" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="73"/>
-      <c r="F78" s="73"/>
+      <c r="E78" s="69"/>
+      <c r="F78" s="69"/>
       <c r="G78" s="17"/>
       <c r="H78" s="17"/>
       <c r="I78" s="17"/>
@@ -20042,11 +19976,10 @@
       <c r="BI78" s="21"/>
       <c r="BJ78" s="21"/>
       <c r="BL78" s="17"/>
-      <c r="BM78" s="17"/>
+      <c r="BM78" s="1"/>
       <c r="BO78" s="18"/>
       <c r="BP78" s="19"/>
       <c r="BQ78" s="20"/>
-      <c r="BR78" s="17"/>
       <c r="BS78" s="17"/>
       <c r="BT78" s="17"/>
       <c r="BU78" s="17"/>
@@ -20205,22 +20138,22 @@
       <c r="HR78" s="17"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="75" t="s">
+      <c r="A79" s="71" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="71" t="s">
+      <c r="B79" s="72" t="s">
         <v>158</v>
       </c>
-      <c r="C79" s="81" t="s">
+      <c r="C79" s="73" t="s">
         <v>159</v>
       </c>
       <c r="D79" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="73" t="s">
+      <c r="E79" s="69" t="s">
         <v>160</v>
       </c>
-      <c r="F79" s="74" t="s">
+      <c r="F79" s="70" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="17"/>
@@ -20274,11 +20207,10 @@
       <c r="BI79" s="21"/>
       <c r="BJ79" s="21"/>
       <c r="BL79" s="17"/>
-      <c r="BM79" s="17"/>
+      <c r="BM79" s="1"/>
       <c r="BO79" s="18"/>
       <c r="BP79" s="19"/>
       <c r="BQ79" s="20"/>
-      <c r="BR79" s="17"/>
       <c r="BS79" s="17"/>
       <c r="BT79" s="17"/>
       <c r="BU79" s="17"/>
@@ -20437,14 +20369,14 @@
       <c r="HR79" s="17"/>
     </row>
     <row r="80" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="75"/>
-      <c r="B80" s="75"/>
-      <c r="C80" s="75"/>
+      <c r="A80" s="71"/>
+      <c r="B80" s="71"/>
+      <c r="C80" s="71"/>
       <c r="D80" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="73"/>
-      <c r="F80" s="73"/>
+      <c r="E80" s="69"/>
+      <c r="F80" s="69"/>
       <c r="G80" s="17"/>
       <c r="H80" s="17"/>
       <c r="I80" s="17"/>
@@ -20496,11 +20428,10 @@
       <c r="BI80" s="21"/>
       <c r="BJ80" s="21"/>
       <c r="BL80" s="17"/>
-      <c r="BM80" s="17"/>
+      <c r="BM80" s="1"/>
       <c r="BO80" s="18"/>
       <c r="BP80" s="19"/>
       <c r="BQ80" s="20"/>
-      <c r="BR80" s="17"/>
       <c r="BS80" s="17"/>
       <c r="BT80" s="17"/>
       <c r="BU80" s="17"/>
@@ -20659,20 +20590,20 @@
       <c r="HR80" s="17"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="75"/>
-      <c r="B81" s="71" t="s">
+      <c r="A81" s="71"/>
+      <c r="B81" s="72" t="s">
         <v>161</v>
       </c>
-      <c r="C81" s="81" t="s">
+      <c r="C81" s="73" t="s">
         <v>162</v>
       </c>
       <c r="D81" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="73" t="s">
+      <c r="E81" s="69" t="s">
         <v>163</v>
       </c>
-      <c r="F81" s="74" t="s">
+      <c r="F81" s="70" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="17"/>
@@ -20726,11 +20657,10 @@
       <c r="BI81" s="21"/>
       <c r="BJ81" s="21"/>
       <c r="BL81" s="17"/>
-      <c r="BM81" s="17"/>
+      <c r="BM81" s="1"/>
       <c r="BO81" s="18"/>
       <c r="BP81" s="19"/>
       <c r="BQ81" s="20"/>
-      <c r="BR81" s="17"/>
       <c r="BS81" s="17"/>
       <c r="BT81" s="17"/>
       <c r="BU81" s="17"/>
@@ -20889,14 +20819,14 @@
       <c r="HR81" s="17"/>
     </row>
     <row r="82" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="75"/>
-      <c r="B82" s="75"/>
-      <c r="C82" s="75"/>
+      <c r="A82" s="71"/>
+      <c r="B82" s="71"/>
+      <c r="C82" s="71"/>
       <c r="D82" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="73"/>
-      <c r="F82" s="73"/>
+      <c r="E82" s="69"/>
+      <c r="F82" s="69"/>
       <c r="G82" s="17"/>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
@@ -20948,11 +20878,10 @@
       <c r="BI82" s="21"/>
       <c r="BJ82" s="21"/>
       <c r="BL82" s="17"/>
-      <c r="BM82" s="17"/>
+      <c r="BM82" s="1"/>
       <c r="BO82" s="18"/>
       <c r="BP82" s="19"/>
       <c r="BQ82" s="20"/>
-      <c r="BR82" s="17"/>
       <c r="BS82" s="17"/>
       <c r="BT82" s="17"/>
       <c r="BU82" s="17"/>
@@ -21111,20 +21040,20 @@
       <c r="HR82" s="17"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="75"/>
-      <c r="B83" s="71" t="s">
+      <c r="A83" s="71"/>
+      <c r="B83" s="72" t="s">
         <v>164</v>
       </c>
-      <c r="C83" s="72" t="s">
+      <c r="C83" s="74" t="s">
         <v>165</v>
       </c>
       <c r="D83" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="73" t="s">
+      <c r="E83" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="F83" s="74" t="s">
+      <c r="F83" s="70" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="17"/>
@@ -21178,11 +21107,10 @@
       <c r="BI83" s="21"/>
       <c r="BJ83" s="21"/>
       <c r="BL83" s="17"/>
-      <c r="BM83" s="17"/>
+      <c r="BM83" s="1"/>
       <c r="BO83" s="18"/>
       <c r="BP83" s="19"/>
       <c r="BQ83" s="20"/>
-      <c r="BR83" s="17"/>
       <c r="BS83" s="17"/>
       <c r="BT83" s="17"/>
       <c r="BU83" s="17"/>
@@ -21341,14 +21269,14 @@
       <c r="HR83" s="17"/>
     </row>
     <row r="84" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="75"/>
-      <c r="B84" s="75"/>
-      <c r="C84" s="75"/>
+      <c r="A84" s="71"/>
+      <c r="B84" s="71"/>
+      <c r="C84" s="71"/>
       <c r="D84" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="73"/>
-      <c r="F84" s="73"/>
+      <c r="E84" s="69"/>
+      <c r="F84" s="69"/>
       <c r="G84" s="17"/>
       <c r="H84" s="17"/>
       <c r="I84" s="17"/>
@@ -21400,11 +21328,10 @@
       <c r="BI84" s="21"/>
       <c r="BJ84" s="21"/>
       <c r="BL84" s="17"/>
-      <c r="BM84" s="17"/>
+      <c r="BM84" s="1"/>
       <c r="BO84" s="18"/>
       <c r="BP84" s="19"/>
       <c r="BQ84" s="20"/>
-      <c r="BR84" s="17"/>
       <c r="BS84" s="17"/>
       <c r="BT84" s="17"/>
       <c r="BU84" s="17"/>
@@ -21563,20 +21490,20 @@
       <c r="HR84" s="17"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="75"/>
-      <c r="B85" s="71" t="s">
+      <c r="A85" s="71"/>
+      <c r="B85" s="72" t="s">
         <v>167</v>
       </c>
-      <c r="C85" s="76" t="s">
+      <c r="C85" s="75" t="s">
         <v>168</v>
       </c>
       <c r="D85" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="73" t="s">
+      <c r="E85" s="69" t="s">
         <v>169</v>
       </c>
-      <c r="F85" s="74"/>
+      <c r="F85" s="70"/>
       <c r="G85" s="17"/>
       <c r="H85" s="17"/>
       <c r="I85" s="17"/>
@@ -21628,11 +21555,10 @@
       <c r="BI85" s="21"/>
       <c r="BJ85" s="21"/>
       <c r="BL85" s="17"/>
-      <c r="BM85" s="17"/>
+      <c r="BM85" s="1"/>
       <c r="BO85" s="18"/>
       <c r="BP85" s="19"/>
       <c r="BQ85" s="20"/>
-      <c r="BR85" s="17"/>
       <c r="BS85" s="17"/>
       <c r="BT85" s="17"/>
       <c r="BU85" s="17"/>
@@ -21791,14 +21717,14 @@
       <c r="HR85" s="49"/>
     </row>
     <row r="86" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="75"/>
-      <c r="B86" s="75"/>
-      <c r="C86" s="75"/>
+      <c r="A86" s="71"/>
+      <c r="B86" s="71"/>
+      <c r="C86" s="71"/>
       <c r="D86" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="73"/>
-      <c r="F86" s="73"/>
+      <c r="E86" s="69"/>
+      <c r="F86" s="69"/>
       <c r="G86" s="17"/>
       <c r="H86" s="17"/>
       <c r="I86" s="17"/>
@@ -21850,11 +21776,10 @@
       <c r="BI86" s="21"/>
       <c r="BJ86" s="21"/>
       <c r="BL86" s="17"/>
-      <c r="BM86" s="17"/>
+      <c r="BM86" s="1"/>
       <c r="BO86" s="18"/>
       <c r="BP86" s="19"/>
       <c r="BQ86" s="20"/>
-      <c r="BR86" s="17"/>
       <c r="BS86" s="17"/>
       <c r="BT86" s="17"/>
       <c r="BU86" s="17"/>
@@ -22014,25 +21939,168 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="GN1:GT1"/>
+    <mergeCell ref="GU1:HA1"/>
+    <mergeCell ref="HB1:HH1"/>
+    <mergeCell ref="HI1:HO1"/>
+    <mergeCell ref="HP1:HR1"/>
+    <mergeCell ref="A5:A22"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="E65:E66"/>
     <mergeCell ref="F65:F66"/>
     <mergeCell ref="A67:A78"/>
     <mergeCell ref="B67:B68"/>
@@ -22057,168 +22125,25 @@
     <mergeCell ref="F75:F76"/>
     <mergeCell ref="B77:B78"/>
     <mergeCell ref="C77:C78"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="GN1:GT1"/>
-    <mergeCell ref="GU1:HA1"/>
-    <mergeCell ref="HB1:HH1"/>
-    <mergeCell ref="HI1:HO1"/>
-    <mergeCell ref="HP1:HR1"/>
-    <mergeCell ref="A5:A22"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="GG1:GM1"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="BK1:BQ1"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="F85:F86"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
edited README and AGENTS.md, sperated nondim from data gen and removed redundancies within, to cheetah and neuralop and resorted repo accordingly + quick tests
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DE7FE1-5042-4E74-9B58-DBD54C08F71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18710F7E-E8DD-4608-B357-988628C4BC57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -398,12 +398,6 @@
     <t>P6</t>
   </si>
   <si>
-    <t>Baselines: Hockney + CNN-Surrogat</t>
-  </si>
-  <si>
-    <t>drei Vergleichsmodelle, exakter Löser liefert Fehler null</t>
-  </si>
-  <si>
     <t>6. Bewertung</t>
   </si>
   <si>
@@ -648,9 +642,6 @@
     <t>Leitfrage 11</t>
   </si>
   <si>
-    <t>drei Vergleichsmodelle</t>
-  </si>
-  <si>
     <t>P2, P5</t>
   </si>
   <si>
@@ -859,6 +850,15 @@
   </si>
   <si>
     <t>Cheetah ist PyTorch, das Skelett ist Python, die Entscheidung ist gefallen. Statt Implementierung ein begründender Absatz im Manuskript.</t>
+  </si>
+  <si>
+    <t>Baselines: Hockney + Poisson-Solver</t>
+  </si>
+  <si>
+    <t>Vergleich, exakter Löser liefert Fehler null</t>
+  </si>
+  <si>
+    <t>Vergleichsmodell</t>
   </si>
 </sst>
 </file>
@@ -1284,6 +1284,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1323,9 +1326,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1618,298 +1618,300 @@
     <col min="64" max="65" width="2.140625" customWidth="1"/>
     <col min="66" max="66" width="2.140625" style="1" customWidth="1"/>
     <col min="67" max="69" width="2.140625" customWidth="1"/>
-    <col min="70" max="70" width="2.140625" style="2" customWidth="1"/>
-    <col min="71" max="226" width="2.140625" customWidth="1"/>
+    <col min="70" max="70" width="2.140625" style="1" customWidth="1"/>
+    <col min="71" max="72" width="2.140625" customWidth="1"/>
+    <col min="73" max="73" width="2.140625" style="2" customWidth="1"/>
+    <col min="74" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="81" t="s">
+      <c r="G1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81" t="s">
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="81"/>
-      <c r="P1" s="81"/>
-      <c r="Q1" s="81"/>
-      <c r="R1" s="81"/>
-      <c r="S1" s="81"/>
-      <c r="T1" s="81"/>
-      <c r="U1" s="81" t="s">
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="81"/>
-      <c r="W1" s="81"/>
-      <c r="X1" s="81"/>
-      <c r="Y1" s="81"/>
-      <c r="Z1" s="81"/>
-      <c r="AA1" s="81"/>
-      <c r="AB1" s="81" t="s">
+      <c r="V1" s="84"/>
+      <c r="W1" s="84"/>
+      <c r="X1" s="84"/>
+      <c r="Y1" s="84"/>
+      <c r="Z1" s="84"/>
+      <c r="AA1" s="84"/>
+      <c r="AB1" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="81"/>
-      <c r="AD1" s="81"/>
-      <c r="AE1" s="81"/>
-      <c r="AF1" s="81"/>
-      <c r="AG1" s="81"/>
-      <c r="AH1" s="81"/>
-      <c r="AI1" s="81" t="s">
+      <c r="AC1" s="84"/>
+      <c r="AD1" s="84"/>
+      <c r="AE1" s="84"/>
+      <c r="AF1" s="84"/>
+      <c r="AG1" s="84"/>
+      <c r="AH1" s="84"/>
+      <c r="AI1" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="81"/>
-      <c r="AK1" s="81"/>
-      <c r="AL1" s="81"/>
-      <c r="AM1" s="81"/>
-      <c r="AN1" s="81"/>
-      <c r="AO1" s="81"/>
-      <c r="AP1" s="81" t="s">
+      <c r="AJ1" s="84"/>
+      <c r="AK1" s="84"/>
+      <c r="AL1" s="84"/>
+      <c r="AM1" s="84"/>
+      <c r="AN1" s="84"/>
+      <c r="AO1" s="84"/>
+      <c r="AP1" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="81"/>
-      <c r="AR1" s="81"/>
-      <c r="AS1" s="81"/>
-      <c r="AT1" s="81"/>
-      <c r="AU1" s="81"/>
-      <c r="AV1" s="81"/>
-      <c r="AW1" s="81" t="s">
+      <c r="AQ1" s="84"/>
+      <c r="AR1" s="84"/>
+      <c r="AS1" s="84"/>
+      <c r="AT1" s="84"/>
+      <c r="AU1" s="84"/>
+      <c r="AV1" s="84"/>
+      <c r="AW1" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="81"/>
-      <c r="AY1" s="81"/>
-      <c r="AZ1" s="81"/>
-      <c r="BA1" s="81"/>
-      <c r="BB1" s="81"/>
-      <c r="BC1" s="81"/>
-      <c r="BD1" s="81" t="s">
+      <c r="AX1" s="84"/>
+      <c r="AY1" s="84"/>
+      <c r="AZ1" s="84"/>
+      <c r="BA1" s="84"/>
+      <c r="BB1" s="84"/>
+      <c r="BC1" s="84"/>
+      <c r="BD1" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="81"/>
-      <c r="BF1" s="81"/>
-      <c r="BG1" s="81"/>
-      <c r="BH1" s="81"/>
-      <c r="BI1" s="81"/>
-      <c r="BJ1" s="81"/>
-      <c r="BK1" s="81" t="s">
+      <c r="BE1" s="84"/>
+      <c r="BF1" s="84"/>
+      <c r="BG1" s="84"/>
+      <c r="BH1" s="84"/>
+      <c r="BI1" s="84"/>
+      <c r="BJ1" s="84"/>
+      <c r="BK1" s="84" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="81"/>
-      <c r="BM1" s="81"/>
-      <c r="BN1" s="81"/>
-      <c r="BO1" s="81"/>
-      <c r="BP1" s="81"/>
-      <c r="BQ1" s="81"/>
-      <c r="BR1" s="81" t="s">
+      <c r="BL1" s="84"/>
+      <c r="BM1" s="84"/>
+      <c r="BN1" s="84"/>
+      <c r="BO1" s="84"/>
+      <c r="BP1" s="84"/>
+      <c r="BQ1" s="84"/>
+      <c r="BR1" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="81"/>
-      <c r="BT1" s="81"/>
-      <c r="BU1" s="81"/>
-      <c r="BV1" s="81"/>
-      <c r="BW1" s="81"/>
-      <c r="BX1" s="81"/>
-      <c r="BY1" s="81" t="s">
+      <c r="BS1" s="84"/>
+      <c r="BT1" s="84"/>
+      <c r="BU1" s="84"/>
+      <c r="BV1" s="84"/>
+      <c r="BW1" s="84"/>
+      <c r="BX1" s="84"/>
+      <c r="BY1" s="84" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="81"/>
-      <c r="CA1" s="81"/>
-      <c r="CB1" s="81"/>
-      <c r="CC1" s="81"/>
-      <c r="CD1" s="81"/>
-      <c r="CE1" s="81"/>
-      <c r="CF1" s="81" t="s">
+      <c r="BZ1" s="84"/>
+      <c r="CA1" s="84"/>
+      <c r="CB1" s="84"/>
+      <c r="CC1" s="84"/>
+      <c r="CD1" s="84"/>
+      <c r="CE1" s="84"/>
+      <c r="CF1" s="84" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="81"/>
-      <c r="CH1" s="81"/>
-      <c r="CI1" s="81"/>
-      <c r="CJ1" s="81"/>
-      <c r="CK1" s="81"/>
-      <c r="CL1" s="81"/>
-      <c r="CM1" s="81" t="s">
+      <c r="CG1" s="84"/>
+      <c r="CH1" s="84"/>
+      <c r="CI1" s="84"/>
+      <c r="CJ1" s="84"/>
+      <c r="CK1" s="84"/>
+      <c r="CL1" s="84"/>
+      <c r="CM1" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="81"/>
-      <c r="CO1" s="81"/>
-      <c r="CP1" s="81"/>
-      <c r="CQ1" s="81"/>
-      <c r="CR1" s="81"/>
-      <c r="CS1" s="81"/>
-      <c r="CT1" s="81" t="s">
+      <c r="CN1" s="84"/>
+      <c r="CO1" s="84"/>
+      <c r="CP1" s="84"/>
+      <c r="CQ1" s="84"/>
+      <c r="CR1" s="84"/>
+      <c r="CS1" s="84"/>
+      <c r="CT1" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="81"/>
-      <c r="CV1" s="81"/>
-      <c r="CW1" s="81"/>
-      <c r="CX1" s="81"/>
-      <c r="CY1" s="81"/>
-      <c r="CZ1" s="81"/>
-      <c r="DA1" s="81" t="s">
+      <c r="CU1" s="84"/>
+      <c r="CV1" s="84"/>
+      <c r="CW1" s="84"/>
+      <c r="CX1" s="84"/>
+      <c r="CY1" s="84"/>
+      <c r="CZ1" s="84"/>
+      <c r="DA1" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="81"/>
-      <c r="DC1" s="81"/>
-      <c r="DD1" s="81"/>
-      <c r="DE1" s="81"/>
-      <c r="DF1" s="81"/>
-      <c r="DG1" s="81"/>
-      <c r="DH1" s="81" t="s">
+      <c r="DB1" s="84"/>
+      <c r="DC1" s="84"/>
+      <c r="DD1" s="84"/>
+      <c r="DE1" s="84"/>
+      <c r="DF1" s="84"/>
+      <c r="DG1" s="84"/>
+      <c r="DH1" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="81"/>
-      <c r="DJ1" s="81"/>
-      <c r="DK1" s="81"/>
-      <c r="DL1" s="81"/>
-      <c r="DM1" s="81"/>
-      <c r="DN1" s="81"/>
-      <c r="DO1" s="81" t="s">
+      <c r="DI1" s="84"/>
+      <c r="DJ1" s="84"/>
+      <c r="DK1" s="84"/>
+      <c r="DL1" s="84"/>
+      <c r="DM1" s="84"/>
+      <c r="DN1" s="84"/>
+      <c r="DO1" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="81"/>
-      <c r="DQ1" s="81"/>
-      <c r="DR1" s="81"/>
-      <c r="DS1" s="81"/>
-      <c r="DT1" s="81"/>
-      <c r="DU1" s="81"/>
-      <c r="DV1" s="81" t="s">
+      <c r="DP1" s="84"/>
+      <c r="DQ1" s="84"/>
+      <c r="DR1" s="84"/>
+      <c r="DS1" s="84"/>
+      <c r="DT1" s="84"/>
+      <c r="DU1" s="84"/>
+      <c r="DV1" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="81"/>
-      <c r="DX1" s="81"/>
-      <c r="DY1" s="81"/>
-      <c r="DZ1" s="81"/>
-      <c r="EA1" s="81"/>
-      <c r="EB1" s="81"/>
-      <c r="EC1" s="81" t="s">
+      <c r="DW1" s="84"/>
+      <c r="DX1" s="84"/>
+      <c r="DY1" s="84"/>
+      <c r="DZ1" s="84"/>
+      <c r="EA1" s="84"/>
+      <c r="EB1" s="84"/>
+      <c r="EC1" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="81"/>
-      <c r="EE1" s="81"/>
-      <c r="EF1" s="81"/>
-      <c r="EG1" s="81"/>
-      <c r="EH1" s="81"/>
-      <c r="EI1" s="81"/>
-      <c r="EJ1" s="81" t="s">
+      <c r="ED1" s="84"/>
+      <c r="EE1" s="84"/>
+      <c r="EF1" s="84"/>
+      <c r="EG1" s="84"/>
+      <c r="EH1" s="84"/>
+      <c r="EI1" s="84"/>
+      <c r="EJ1" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="81"/>
-      <c r="EL1" s="81"/>
-      <c r="EM1" s="81"/>
-      <c r="EN1" s="81"/>
-      <c r="EO1" s="81"/>
-      <c r="EP1" s="81"/>
-      <c r="EQ1" s="81" t="s">
+      <c r="EK1" s="84"/>
+      <c r="EL1" s="84"/>
+      <c r="EM1" s="84"/>
+      <c r="EN1" s="84"/>
+      <c r="EO1" s="84"/>
+      <c r="EP1" s="84"/>
+      <c r="EQ1" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="81"/>
-      <c r="ES1" s="81"/>
-      <c r="ET1" s="81"/>
-      <c r="EU1" s="81"/>
-      <c r="EV1" s="81"/>
-      <c r="EW1" s="81"/>
-      <c r="EX1" s="81" t="s">
+      <c r="ER1" s="84"/>
+      <c r="ES1" s="84"/>
+      <c r="ET1" s="84"/>
+      <c r="EU1" s="84"/>
+      <c r="EV1" s="84"/>
+      <c r="EW1" s="84"/>
+      <c r="EX1" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="81"/>
-      <c r="EZ1" s="81"/>
-      <c r="FA1" s="81"/>
-      <c r="FB1" s="81"/>
-      <c r="FC1" s="81"/>
-      <c r="FD1" s="81"/>
-      <c r="FE1" s="81" t="s">
+      <c r="EY1" s="84"/>
+      <c r="EZ1" s="84"/>
+      <c r="FA1" s="84"/>
+      <c r="FB1" s="84"/>
+      <c r="FC1" s="84"/>
+      <c r="FD1" s="84"/>
+      <c r="FE1" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="81"/>
-      <c r="FG1" s="81"/>
-      <c r="FH1" s="81"/>
-      <c r="FI1" s="81"/>
-      <c r="FJ1" s="81"/>
-      <c r="FK1" s="81"/>
-      <c r="FL1" s="81" t="s">
+      <c r="FF1" s="84"/>
+      <c r="FG1" s="84"/>
+      <c r="FH1" s="84"/>
+      <c r="FI1" s="84"/>
+      <c r="FJ1" s="84"/>
+      <c r="FK1" s="84"/>
+      <c r="FL1" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="81"/>
-      <c r="FN1" s="81"/>
-      <c r="FO1" s="81"/>
-      <c r="FP1" s="81"/>
-      <c r="FQ1" s="81"/>
-      <c r="FR1" s="81"/>
-      <c r="FS1" s="81" t="s">
+      <c r="FM1" s="84"/>
+      <c r="FN1" s="84"/>
+      <c r="FO1" s="84"/>
+      <c r="FP1" s="84"/>
+      <c r="FQ1" s="84"/>
+      <c r="FR1" s="84"/>
+      <c r="FS1" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="81"/>
-      <c r="FU1" s="81"/>
-      <c r="FV1" s="81"/>
-      <c r="FW1" s="81"/>
-      <c r="FX1" s="81"/>
-      <c r="FY1" s="81"/>
-      <c r="FZ1" s="81" t="s">
+      <c r="FT1" s="84"/>
+      <c r="FU1" s="84"/>
+      <c r="FV1" s="84"/>
+      <c r="FW1" s="84"/>
+      <c r="FX1" s="84"/>
+      <c r="FY1" s="84"/>
+      <c r="FZ1" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="81"/>
-      <c r="GB1" s="81"/>
-      <c r="GC1" s="81"/>
-      <c r="GD1" s="81"/>
-      <c r="GE1" s="81"/>
-      <c r="GF1" s="81"/>
-      <c r="GG1" s="81" t="s">
+      <c r="GA1" s="84"/>
+      <c r="GB1" s="84"/>
+      <c r="GC1" s="84"/>
+      <c r="GD1" s="84"/>
+      <c r="GE1" s="84"/>
+      <c r="GF1" s="84"/>
+      <c r="GG1" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="81"/>
-      <c r="GI1" s="81"/>
-      <c r="GJ1" s="81"/>
-      <c r="GK1" s="81"/>
-      <c r="GL1" s="81"/>
-      <c r="GM1" s="81"/>
-      <c r="GN1" s="81" t="s">
+      <c r="GH1" s="84"/>
+      <c r="GI1" s="84"/>
+      <c r="GJ1" s="84"/>
+      <c r="GK1" s="84"/>
+      <c r="GL1" s="84"/>
+      <c r="GM1" s="84"/>
+      <c r="GN1" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="81"/>
-      <c r="GP1" s="81"/>
-      <c r="GQ1" s="81"/>
-      <c r="GR1" s="81"/>
-      <c r="GS1" s="81"/>
-      <c r="GT1" s="81"/>
-      <c r="GU1" s="81" t="s">
+      <c r="GO1" s="84"/>
+      <c r="GP1" s="84"/>
+      <c r="GQ1" s="84"/>
+      <c r="GR1" s="84"/>
+      <c r="GS1" s="84"/>
+      <c r="GT1" s="84"/>
+      <c r="GU1" s="84" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="81"/>
-      <c r="GW1" s="81"/>
-      <c r="GX1" s="81"/>
-      <c r="GY1" s="81"/>
-      <c r="GZ1" s="81"/>
-      <c r="HA1" s="81"/>
-      <c r="HB1" s="81" t="s">
+      <c r="GV1" s="84"/>
+      <c r="GW1" s="84"/>
+      <c r="GX1" s="84"/>
+      <c r="GY1" s="84"/>
+      <c r="GZ1" s="84"/>
+      <c r="HA1" s="84"/>
+      <c r="HB1" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="81"/>
-      <c r="HD1" s="81"/>
-      <c r="HE1" s="81"/>
-      <c r="HF1" s="81"/>
-      <c r="HG1" s="81"/>
-      <c r="HH1" s="81"/>
-      <c r="HI1" s="81" t="s">
+      <c r="HC1" s="84"/>
+      <c r="HD1" s="84"/>
+      <c r="HE1" s="84"/>
+      <c r="HF1" s="84"/>
+      <c r="HG1" s="84"/>
+      <c r="HH1" s="84"/>
+      <c r="HI1" s="84" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="81"/>
-      <c r="HK1" s="81"/>
-      <c r="HL1" s="81"/>
-      <c r="HM1" s="81"/>
-      <c r="HN1" s="81"/>
-      <c r="HO1" s="81"/>
-      <c r="HP1" s="81" t="s">
+      <c r="HJ1" s="84"/>
+      <c r="HK1" s="84"/>
+      <c r="HL1" s="84"/>
+      <c r="HM1" s="84"/>
+      <c r="HN1" s="84"/>
+      <c r="HO1" s="84"/>
+      <c r="HP1" s="84" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="81"/>
-      <c r="HR1" s="81"/>
+      <c r="HQ1" s="84"/>
+      <c r="HR1" s="84"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3" t="s">
@@ -2104,7 +2106,7 @@
       <c r="BQ2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="BR2" s="7" t="s">
+      <c r="BR2" s="6" t="s">
         <v>34</v>
       </c>
       <c r="BS2" s="4" t="s">
@@ -2113,7 +2115,7 @@
       <c r="BT2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="BU2" s="4" t="s">
+      <c r="BU2" s="7" t="s">
         <v>35</v>
       </c>
       <c r="BV2" s="4" t="s">
@@ -2769,7 +2771,7 @@
       <c r="BQ3" s="8">
         <v>46313</v>
       </c>
-      <c r="BR3" s="10">
+      <c r="BR3" s="9">
         <v>46314</v>
       </c>
       <c r="BS3" s="8">
@@ -2778,7 +2780,7 @@
       <c r="BT3" s="8">
         <v>46316</v>
       </c>
-      <c r="BU3" s="8">
+      <c r="BU3" s="10">
         <v>46317</v>
       </c>
       <c r="BV3" s="8">
@@ -3321,10 +3323,10 @@
       <c r="BO4" s="12"/>
       <c r="BP4" s="12"/>
       <c r="BQ4" s="12"/>
-      <c r="BR4" s="14"/>
+      <c r="BR4" s="13"/>
       <c r="BS4" s="12"/>
       <c r="BT4" s="12"/>
-      <c r="BU4" s="12"/>
+      <c r="BU4" s="14"/>
       <c r="BV4" s="12"/>
       <c r="BW4" s="12"/>
       <c r="BX4" s="12"/>
@@ -3480,20 +3482,20 @@
       <c r="HR4" s="12"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="74" t="s">
+      <c r="B5" s="75"/>
+      <c r="C5" s="77" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="69" t="s">
+      <c r="E5" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="70"/>
+      <c r="F5" s="73"/>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
       <c r="I5" s="17"/>
@@ -3548,10 +3550,9 @@
       <c r="BM5" s="1"/>
       <c r="BO5" s="18"/>
       <c r="BP5" s="19"/>
-      <c r="BQ5" s="20"/>
+      <c r="BQ5" s="21"/>
       <c r="BS5" s="17"/>
       <c r="BT5" s="17"/>
-      <c r="BU5" s="17"/>
       <c r="BV5" s="18"/>
       <c r="BW5" s="19"/>
       <c r="BX5" s="20"/>
@@ -3707,14 +3708,14 @@
       <c r="HR5" s="17"/>
     </row>
     <row r="6" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="76"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="76"/>
+      <c r="A6" s="79"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
       <c r="D6" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
       <c r="G6" s="17"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
@@ -3769,10 +3770,9 @@
       <c r="BM6" s="1"/>
       <c r="BO6" s="18"/>
       <c r="BP6" s="19"/>
-      <c r="BQ6" s="20"/>
+      <c r="BQ6" s="21"/>
       <c r="BS6" s="17"/>
       <c r="BT6" s="17"/>
-      <c r="BU6" s="17"/>
       <c r="BV6" s="18"/>
       <c r="BW6" s="19"/>
       <c r="BX6" s="20"/>
@@ -3928,18 +3928,18 @@
       <c r="HR6" s="17"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="76"/>
-      <c r="B7" s="72"/>
-      <c r="C7" s="74" t="s">
+      <c r="A7" s="79"/>
+      <c r="B7" s="75"/>
+      <c r="C7" s="77" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="69" t="s">
+      <c r="E7" s="72" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="70"/>
+      <c r="F7" s="73"/>
       <c r="G7" s="17"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -3994,10 +3994,9 @@
       <c r="BM7" s="1"/>
       <c r="BO7" s="18"/>
       <c r="BP7" s="19"/>
-      <c r="BQ7" s="20"/>
+      <c r="BQ7" s="21"/>
       <c r="BS7" s="17"/>
       <c r="BT7" s="17"/>
-      <c r="BU7" s="17"/>
       <c r="BV7" s="18"/>
       <c r="BW7" s="19"/>
       <c r="BX7" s="20"/>
@@ -4153,14 +4152,14 @@
       <c r="HR7" s="17"/>
     </row>
     <row r="8" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="76"/>
-      <c r="B8" s="76"/>
-      <c r="C8" s="76"/>
+      <c r="A8" s="79"/>
+      <c r="B8" s="79"/>
+      <c r="C8" s="79"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
@@ -4215,10 +4214,9 @@
       <c r="BM8" s="1"/>
       <c r="BO8" s="18"/>
       <c r="BP8" s="19"/>
-      <c r="BQ8" s="20"/>
+      <c r="BQ8" s="21"/>
       <c r="BS8" s="17"/>
       <c r="BT8" s="17"/>
-      <c r="BU8" s="17"/>
       <c r="BV8" s="18"/>
       <c r="BW8" s="19"/>
       <c r="BX8" s="20"/>
@@ -4374,18 +4372,18 @@
       <c r="HR8" s="17"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="76"/>
-      <c r="B9" s="72"/>
-      <c r="C9" s="74" t="s">
+      <c r="A9" s="79"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="77" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="69" t="s">
+      <c r="E9" s="72" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="70"/>
+      <c r="F9" s="73"/>
       <c r="G9" s="17"/>
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
@@ -4440,10 +4438,9 @@
       <c r="BM9" s="1"/>
       <c r="BO9" s="18"/>
       <c r="BP9" s="19"/>
-      <c r="BQ9" s="20"/>
+      <c r="BQ9" s="21"/>
       <c r="BS9" s="17"/>
       <c r="BT9" s="17"/>
-      <c r="BU9" s="17"/>
       <c r="BV9" s="18"/>
       <c r="BW9" s="19"/>
       <c r="BX9" s="20"/>
@@ -4599,14 +4596,14 @@
       <c r="HR9" s="17"/>
     </row>
     <row r="10" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="76"/>
-      <c r="B10" s="76"/>
-      <c r="C10" s="76"/>
+      <c r="A10" s="79"/>
+      <c r="B10" s="79"/>
+      <c r="C10" s="79"/>
       <c r="D10" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="72"/>
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -4661,10 +4658,9 @@
       <c r="BM10" s="1"/>
       <c r="BO10" s="18"/>
       <c r="BP10" s="19"/>
-      <c r="BQ10" s="20"/>
+      <c r="BQ10" s="21"/>
       <c r="BS10" s="17"/>
       <c r="BT10" s="17"/>
-      <c r="BU10" s="17"/>
       <c r="BV10" s="18"/>
       <c r="BW10" s="19"/>
       <c r="BX10" s="20"/>
@@ -4820,18 +4816,18 @@
       <c r="HR10" s="17"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="76"/>
-      <c r="B11" s="72"/>
-      <c r="C11" s="74" t="s">
+      <c r="A11" s="79"/>
+      <c r="B11" s="75"/>
+      <c r="C11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="69" t="s">
+      <c r="E11" s="72" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="70"/>
+      <c r="F11" s="73"/>
       <c r="G11" s="17"/>
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
@@ -4886,10 +4882,9 @@
       <c r="BM11" s="1"/>
       <c r="BO11" s="18"/>
       <c r="BP11" s="19"/>
-      <c r="BQ11" s="20"/>
+      <c r="BQ11" s="21"/>
       <c r="BS11" s="17"/>
       <c r="BT11" s="17"/>
-      <c r="BU11" s="17"/>
       <c r="BV11" s="18"/>
       <c r="BW11" s="19"/>
       <c r="BX11" s="20"/>
@@ -5045,14 +5040,14 @@
       <c r="HR11" s="17"/>
     </row>
     <row r="12" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="76"/>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
+      <c r="A12" s="79"/>
+      <c r="B12" s="79"/>
+      <c r="C12" s="79"/>
       <c r="D12" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -5107,10 +5102,9 @@
       <c r="BM12" s="1"/>
       <c r="BO12" s="18"/>
       <c r="BP12" s="19"/>
-      <c r="BQ12" s="20"/>
+      <c r="BQ12" s="21"/>
       <c r="BS12" s="17"/>
       <c r="BT12" s="17"/>
-      <c r="BU12" s="17"/>
       <c r="BV12" s="18"/>
       <c r="BW12" s="19"/>
       <c r="BX12" s="20"/>
@@ -5266,18 +5260,18 @@
       <c r="HR12" s="17"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="76"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="74" t="s">
+      <c r="A13" s="79"/>
+      <c r="B13" s="75"/>
+      <c r="C13" s="77" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="69" t="s">
+      <c r="E13" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="70"/>
+      <c r="F13" s="73"/>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
       <c r="I13" s="17"/>
@@ -5332,10 +5326,9 @@
       <c r="BM13" s="1"/>
       <c r="BO13" s="18"/>
       <c r="BP13" s="19"/>
-      <c r="BQ13" s="20"/>
+      <c r="BQ13" s="21"/>
       <c r="BS13" s="17"/>
       <c r="BT13" s="17"/>
-      <c r="BU13" s="17"/>
       <c r="BV13" s="18"/>
       <c r="BW13" s="19"/>
       <c r="BX13" s="20"/>
@@ -5491,14 +5484,14 @@
       <c r="HR13" s="17"/>
     </row>
     <row r="14" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="76"/>
-      <c r="B14" s="76"/>
-      <c r="C14" s="76"/>
+      <c r="A14" s="79"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="79"/>
       <c r="D14" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="69"/>
-      <c r="F14" s="69"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="72"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -5553,10 +5546,9 @@
       <c r="BM14" s="1"/>
       <c r="BO14" s="18"/>
       <c r="BP14" s="19"/>
-      <c r="BQ14" s="20"/>
+      <c r="BQ14" s="21"/>
       <c r="BS14" s="17"/>
       <c r="BT14" s="17"/>
-      <c r="BU14" s="17"/>
       <c r="BV14" s="18"/>
       <c r="BW14" s="19"/>
       <c r="BX14" s="20"/>
@@ -5712,18 +5704,18 @@
       <c r="HR14" s="17"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="76"/>
-      <c r="B15" s="72"/>
-      <c r="C15" s="74" t="s">
+      <c r="A15" s="79"/>
+      <c r="B15" s="75"/>
+      <c r="C15" s="77" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="69" t="s">
+      <c r="E15" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="70"/>
+      <c r="F15" s="73"/>
       <c r="G15" s="17"/>
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
@@ -5778,10 +5770,9 @@
       <c r="BM15" s="1"/>
       <c r="BO15" s="18"/>
       <c r="BP15" s="19"/>
-      <c r="BQ15" s="20"/>
+      <c r="BQ15" s="21"/>
       <c r="BS15" s="17"/>
       <c r="BT15" s="17"/>
-      <c r="BU15" s="17"/>
       <c r="BV15" s="18"/>
       <c r="BW15" s="19"/>
       <c r="BX15" s="20"/>
@@ -5937,14 +5928,14 @@
       <c r="HR15" s="17"/>
     </row>
     <row r="16" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="76"/>
-      <c r="B16" s="76"/>
-      <c r="C16" s="76"/>
+      <c r="A16" s="79"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="79"/>
       <c r="D16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="69"/>
-      <c r="F16" s="69"/>
+      <c r="E16" s="72"/>
+      <c r="F16" s="72"/>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -5999,10 +5990,9 @@
       <c r="BM16" s="1"/>
       <c r="BO16" s="18"/>
       <c r="BP16" s="19"/>
-      <c r="BQ16" s="20"/>
+      <c r="BQ16" s="21"/>
       <c r="BS16" s="17"/>
       <c r="BT16" s="17"/>
-      <c r="BU16" s="17"/>
       <c r="BV16" s="18"/>
       <c r="BW16" s="19"/>
       <c r="BX16" s="20"/>
@@ -6158,18 +6148,18 @@
       <c r="HR16" s="17"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="76"/>
-      <c r="B17" s="72"/>
-      <c r="C17" s="74" t="s">
+      <c r="A17" s="79"/>
+      <c r="B17" s="75"/>
+      <c r="C17" s="77" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="69" t="s">
+      <c r="E17" s="72" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="70"/>
+      <c r="F17" s="73"/>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
@@ -6224,10 +6214,9 @@
       <c r="BM17" s="1"/>
       <c r="BO17" s="18"/>
       <c r="BP17" s="19"/>
-      <c r="BQ17" s="20"/>
+      <c r="BQ17" s="21"/>
       <c r="BS17" s="17"/>
       <c r="BT17" s="17"/>
-      <c r="BU17" s="17"/>
       <c r="BV17" s="18"/>
       <c r="BW17" s="19"/>
       <c r="BX17" s="20"/>
@@ -6383,14 +6372,14 @@
       <c r="HR17" s="17"/>
     </row>
     <row r="18" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="76"/>
-      <c r="B18" s="76"/>
-      <c r="C18" s="76"/>
+      <c r="A18" s="79"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
       <c r="D18" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
+      <c r="E18" s="72"/>
+      <c r="F18" s="72"/>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -6445,10 +6434,9 @@
       <c r="BM18" s="1"/>
       <c r="BO18" s="18"/>
       <c r="BP18" s="19"/>
-      <c r="BQ18" s="20"/>
+      <c r="BQ18" s="21"/>
       <c r="BS18" s="17"/>
       <c r="BT18" s="17"/>
-      <c r="BU18" s="17"/>
       <c r="BV18" s="18"/>
       <c r="BW18" s="19"/>
       <c r="BX18" s="20"/>
@@ -6604,18 +6592,18 @@
       <c r="HR18" s="17"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="76"/>
-      <c r="B19" s="72"/>
-      <c r="C19" s="74" t="s">
+      <c r="A19" s="79"/>
+      <c r="B19" s="75"/>
+      <c r="C19" s="77" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="69" t="s">
+      <c r="E19" s="72" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="70"/>
+      <c r="F19" s="73"/>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
@@ -6670,10 +6658,9 @@
       <c r="BM19" s="1"/>
       <c r="BO19" s="18"/>
       <c r="BP19" s="19"/>
-      <c r="BQ19" s="20"/>
+      <c r="BQ19" s="21"/>
       <c r="BS19" s="17"/>
       <c r="BT19" s="17"/>
-      <c r="BU19" s="17"/>
       <c r="BV19" s="18"/>
       <c r="BW19" s="19"/>
       <c r="BX19" s="20"/>
@@ -6829,14 +6816,14 @@
       <c r="HR19" s="17"/>
     </row>
     <row r="20" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="76"/>
-      <c r="B20" s="76"/>
-      <c r="C20" s="76"/>
+      <c r="A20" s="79"/>
+      <c r="B20" s="79"/>
+      <c r="C20" s="79"/>
       <c r="D20" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
+      <c r="E20" s="72"/>
+      <c r="F20" s="72"/>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
@@ -6891,10 +6878,9 @@
       <c r="BM20" s="1"/>
       <c r="BO20" s="18"/>
       <c r="BP20" s="19"/>
-      <c r="BQ20" s="20"/>
+      <c r="BQ20" s="21"/>
       <c r="BS20" s="17"/>
       <c r="BT20" s="17"/>
-      <c r="BU20" s="17"/>
       <c r="BV20" s="18"/>
       <c r="BW20" s="19"/>
       <c r="BX20" s="20"/>
@@ -7050,18 +7036,18 @@
       <c r="HR20" s="17"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="76"/>
-      <c r="B21" s="77"/>
-      <c r="C21" s="78" t="s">
+      <c r="A21" s="79"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="81" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="79" t="s">
+      <c r="E21" s="82" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="80"/>
+      <c r="F21" s="83"/>
       <c r="G21" s="17"/>
       <c r="H21" s="17"/>
       <c r="I21" s="17"/>
@@ -7116,10 +7102,9 @@
       <c r="BM21" s="1"/>
       <c r="BO21" s="18"/>
       <c r="BP21" s="19"/>
-      <c r="BQ21" s="20"/>
+      <c r="BQ21" s="21"/>
       <c r="BS21" s="17"/>
       <c r="BT21" s="17"/>
-      <c r="BU21" s="17"/>
       <c r="BV21" s="18"/>
       <c r="BW21" s="19"/>
       <c r="BX21" s="20"/>
@@ -7275,14 +7260,14 @@
       <c r="HR21" s="17"/>
     </row>
     <row r="22" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="76"/>
-      <c r="B22" s="76"/>
-      <c r="C22" s="76"/>
+      <c r="A22" s="79"/>
+      <c r="B22" s="79"/>
+      <c r="C22" s="79"/>
       <c r="D22" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="79"/>
-      <c r="F22" s="79"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="82"/>
       <c r="G22" s="30"/>
       <c r="H22" s="30"/>
       <c r="I22" s="30"/>
@@ -7337,11 +7322,10 @@
       <c r="BM22" s="36"/>
       <c r="BO22" s="31"/>
       <c r="BP22" s="32"/>
-      <c r="BQ22" s="33"/>
-      <c r="BR22" s="67"/>
+      <c r="BQ22" s="35"/>
       <c r="BS22" s="30"/>
       <c r="BT22" s="30"/>
-      <c r="BU22" s="30"/>
+      <c r="BU22" s="67"/>
       <c r="BV22" s="31"/>
       <c r="BW22" s="32"/>
       <c r="BX22" s="33"/>
@@ -7497,22 +7481,22 @@
       <c r="HR22" s="30"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="71" t="s">
+      <c r="A23" s="74" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="75" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="74" t="s">
+      <c r="C23" s="77" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="69" t="s">
+      <c r="E23" s="72" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="70" t="s">
+      <c r="F23" s="73" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="17"/>
@@ -7573,11 +7557,10 @@
       <c r="BM23" s="1"/>
       <c r="BO23" s="18"/>
       <c r="BP23" s="19"/>
-      <c r="BQ23" s="20"/>
-      <c r="BR23" s="68"/>
+      <c r="BQ23" s="21"/>
+      <c r="BR23" s="38"/>
       <c r="BS23" s="17"/>
       <c r="BT23" s="17"/>
-      <c r="BU23" s="17"/>
       <c r="BV23" s="18"/>
       <c r="BW23" s="19"/>
       <c r="BX23" s="20"/>
@@ -7733,14 +7716,14 @@
       <c r="HR23" s="17"/>
     </row>
     <row r="24" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="71"/>
-      <c r="B24" s="71"/>
-      <c r="C24" s="71"/>
+      <c r="A24" s="74"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
       <c r="D24" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
+      <c r="E24" s="72"/>
+      <c r="F24" s="72"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
@@ -7799,10 +7782,9 @@
       <c r="BM24" s="1"/>
       <c r="BO24" s="18"/>
       <c r="BP24" s="19"/>
-      <c r="BQ24" s="20"/>
+      <c r="BQ24" s="21"/>
       <c r="BS24" s="17"/>
-      <c r="BT24" s="17"/>
-      <c r="BU24" s="17"/>
+      <c r="BU24" s="25"/>
       <c r="BV24" s="18"/>
       <c r="BW24" s="19"/>
       <c r="BX24" s="20"/>
@@ -7958,20 +7940,20 @@
       <c r="HR24" s="17"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="71"/>
-      <c r="B25" s="72" t="s">
+      <c r="A25" s="74"/>
+      <c r="B25" s="75" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="74" t="s">
+      <c r="C25" s="77" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="69" t="s">
+      <c r="E25" s="72" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="70" t="s">
+      <c r="F25" s="73" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="17"/>
@@ -8023,7 +8005,7 @@
       <c r="BM25" s="38"/>
       <c r="BO25" s="18"/>
       <c r="BP25" s="19"/>
-      <c r="BQ25" s="20"/>
+      <c r="BQ25" s="21"/>
       <c r="BS25" s="17"/>
       <c r="BT25" s="17"/>
       <c r="BV25" s="18"/>
@@ -8180,14 +8162,14 @@
       <c r="HS25" s="17"/>
     </row>
     <row r="26" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="71"/>
-      <c r="B26" s="71"/>
-      <c r="C26" s="71"/>
+      <c r="A26" s="74"/>
+      <c r="B26" s="74"/>
+      <c r="C26" s="74"/>
       <c r="D26" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="69"/>
-      <c r="F26" s="69"/>
+      <c r="E26" s="72"/>
+      <c r="F26" s="72"/>
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -8242,10 +8224,9 @@
       <c r="BM26" s="42"/>
       <c r="BO26" s="18"/>
       <c r="BP26" s="19"/>
-      <c r="BQ26" s="20"/>
+      <c r="BQ26" s="21"/>
       <c r="BS26" s="17"/>
       <c r="BT26" s="17"/>
-      <c r="BU26" s="17"/>
       <c r="BV26" s="18"/>
       <c r="BW26" s="19"/>
       <c r="BX26" s="20"/>
@@ -8401,20 +8382,20 @@
       <c r="HR26" s="17"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="71"/>
-      <c r="B27" s="72" t="s">
+      <c r="A27" s="74"/>
+      <c r="B27" s="75" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="75" t="s">
+      <c r="C27" s="78" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="69" t="s">
+      <c r="E27" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="70"/>
+      <c r="F27" s="73"/>
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -8469,10 +8450,9 @@
       <c r="BM27" s="1"/>
       <c r="BO27" s="18"/>
       <c r="BP27" s="19"/>
-      <c r="BQ27" s="20"/>
+      <c r="BQ27" s="21"/>
       <c r="BS27" s="17"/>
       <c r="BT27" s="17"/>
-      <c r="BU27" s="17"/>
       <c r="BV27" s="18"/>
       <c r="BW27" s="19"/>
       <c r="BX27" s="20"/>
@@ -8628,14 +8608,14 @@
       <c r="HR27" s="17"/>
     </row>
     <row r="28" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="71"/>
-      <c r="B28" s="71"/>
-      <c r="C28" s="71"/>
+      <c r="A28" s="74"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="74"/>
       <c r="D28" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="72"/>
       <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -8690,10 +8670,9 @@
       <c r="BM28" s="1"/>
       <c r="BO28" s="18"/>
       <c r="BP28" s="19"/>
-      <c r="BQ28" s="20"/>
+      <c r="BQ28" s="21"/>
       <c r="BS28" s="17"/>
       <c r="BT28" s="17"/>
-      <c r="BU28" s="17"/>
       <c r="BV28" s="18"/>
       <c r="BW28" s="19"/>
       <c r="BX28" s="20"/>
@@ -8849,22 +8828,22 @@
       <c r="HR28" s="17"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="71" t="s">
+      <c r="A29" s="74" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="72" t="s">
+      <c r="B29" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="74" t="s">
+      <c r="C29" s="77" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="69" t="s">
+      <c r="E29" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="70" t="s">
+      <c r="F29" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="17"/>
@@ -8920,10 +8899,9 @@
       <c r="BM29" s="1"/>
       <c r="BO29" s="18"/>
       <c r="BP29" s="19"/>
-      <c r="BQ29" s="20"/>
+      <c r="BQ29" s="21"/>
       <c r="BS29" s="17"/>
       <c r="BT29" s="17"/>
-      <c r="BU29" s="17"/>
       <c r="BV29" s="18"/>
       <c r="BW29" s="19"/>
       <c r="BX29" s="20"/>
@@ -9079,14 +9057,14 @@
       <c r="HR29" s="17"/>
     </row>
     <row r="30" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="71"/>
-      <c r="B30" s="71"/>
-      <c r="C30" s="71"/>
+      <c r="A30" s="74"/>
+      <c r="B30" s="74"/>
+      <c r="C30" s="74"/>
       <c r="D30" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
+      <c r="E30" s="72"/>
+      <c r="F30" s="72"/>
       <c r="G30" s="17"/>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -9141,10 +9119,9 @@
       <c r="BM30" s="1"/>
       <c r="BO30" s="18"/>
       <c r="BP30" s="19"/>
-      <c r="BQ30" s="20"/>
+      <c r="BQ30" s="21"/>
       <c r="BS30" s="17"/>
       <c r="BT30" s="17"/>
-      <c r="BU30" s="17"/>
       <c r="BV30" s="18"/>
       <c r="BW30" s="19"/>
       <c r="BX30" s="20"/>
@@ -9300,20 +9277,20 @@
       <c r="HR30" s="17"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="71"/>
-      <c r="B31" s="72" t="s">
+      <c r="A31" s="74"/>
+      <c r="B31" s="75" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="74" t="s">
+      <c r="C31" s="77" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="69" t="s">
+      <c r="E31" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="70" t="s">
+      <c r="F31" s="73" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="17"/>
@@ -9370,10 +9347,9 @@
       <c r="BM31" s="1"/>
       <c r="BO31" s="18"/>
       <c r="BP31" s="19"/>
-      <c r="BQ31" s="20"/>
+      <c r="BQ31" s="21"/>
       <c r="BS31" s="17"/>
       <c r="BT31" s="17"/>
-      <c r="BU31" s="17"/>
       <c r="BV31" s="18"/>
       <c r="BW31" s="19"/>
       <c r="BX31" s="20"/>
@@ -9529,14 +9505,14 @@
       <c r="HR31" s="17"/>
     </row>
     <row r="32" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="71"/>
-      <c r="B32" s="71"/>
-      <c r="C32" s="71"/>
+      <c r="A32" s="74"/>
+      <c r="B32" s="74"/>
+      <c r="C32" s="74"/>
       <c r="D32" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="72"/>
       <c r="G32" s="17"/>
       <c r="H32" s="17"/>
       <c r="I32" s="17"/>
@@ -9591,10 +9567,9 @@
       <c r="BM32" s="1"/>
       <c r="BO32" s="18"/>
       <c r="BP32" s="19"/>
-      <c r="BQ32" s="20"/>
+      <c r="BQ32" s="21"/>
       <c r="BS32" s="17"/>
       <c r="BT32" s="17"/>
-      <c r="BU32" s="17"/>
       <c r="BV32" s="18"/>
       <c r="BW32" s="19"/>
       <c r="BX32" s="20"/>
@@ -9750,20 +9725,20 @@
       <c r="HR32" s="17"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="71"/>
-      <c r="B33" s="72" t="s">
+      <c r="A33" s="74"/>
+      <c r="B33" s="75" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="74" t="s">
+      <c r="C33" s="77" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="69" t="s">
+      <c r="E33" s="72" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="70" t="s">
+      <c r="F33" s="73" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="17"/>
@@ -9820,10 +9795,9 @@
       <c r="BM33" s="1"/>
       <c r="BO33" s="18"/>
       <c r="BP33" s="19"/>
-      <c r="BQ33" s="20"/>
+      <c r="BQ33" s="21"/>
       <c r="BS33" s="17"/>
       <c r="BT33" s="17"/>
-      <c r="BU33" s="17"/>
       <c r="BV33" s="18"/>
       <c r="BW33" s="19"/>
       <c r="BX33" s="20"/>
@@ -9979,14 +9953,14 @@
       <c r="HR33" s="17"/>
     </row>
     <row r="34" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="71"/>
-      <c r="B34" s="71"/>
-      <c r="C34" s="71"/>
+      <c r="A34" s="74"/>
+      <c r="B34" s="74"/>
+      <c r="C34" s="74"/>
       <c r="D34" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
+      <c r="E34" s="72"/>
+      <c r="F34" s="72"/>
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
@@ -10041,10 +10015,9 @@
       <c r="BM34" s="1"/>
       <c r="BO34" s="18"/>
       <c r="BP34" s="19"/>
-      <c r="BQ34" s="20"/>
+      <c r="BQ34" s="21"/>
       <c r="BS34" s="17"/>
       <c r="BT34" s="17"/>
-      <c r="BU34" s="17"/>
       <c r="BV34" s="18"/>
       <c r="BW34" s="19"/>
       <c r="BX34" s="20"/>
@@ -10200,20 +10173,20 @@
       <c r="HR34" s="17"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="71"/>
-      <c r="B35" s="72" t="s">
+      <c r="A35" s="74"/>
+      <c r="B35" s="75" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="74" t="s">
+      <c r="C35" s="77" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="69" t="s">
+      <c r="E35" s="72" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="70" t="s">
+      <c r="F35" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="17"/>
@@ -10271,10 +10244,9 @@
       <c r="BM35" s="1"/>
       <c r="BO35" s="18"/>
       <c r="BP35" s="19"/>
-      <c r="BQ35" s="20"/>
+      <c r="BQ35" s="21"/>
       <c r="BS35" s="17"/>
       <c r="BT35" s="17"/>
-      <c r="BU35" s="17"/>
       <c r="BV35" s="18"/>
       <c r="BW35" s="19"/>
       <c r="BX35" s="20"/>
@@ -10430,14 +10402,14 @@
       <c r="HR35" s="17"/>
     </row>
     <row r="36" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="71"/>
-      <c r="B36" s="71"/>
-      <c r="C36" s="71"/>
+      <c r="A36" s="74"/>
+      <c r="B36" s="74"/>
+      <c r="C36" s="74"/>
       <c r="D36" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="69"/>
-      <c r="F36" s="69"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
       <c r="G36" s="17"/>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
@@ -10493,10 +10465,9 @@
       <c r="BM36" s="1"/>
       <c r="BO36" s="18"/>
       <c r="BP36" s="19"/>
-      <c r="BQ36" s="20"/>
+      <c r="BQ36" s="21"/>
       <c r="BS36" s="17"/>
       <c r="BT36" s="17"/>
-      <c r="BU36" s="17"/>
       <c r="BV36" s="18"/>
       <c r="BW36" s="19"/>
       <c r="BX36" s="20"/>
@@ -10652,20 +10623,20 @@
       <c r="HR36" s="17"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="71"/>
-      <c r="B37" s="72" t="s">
+      <c r="A37" s="74"/>
+      <c r="B37" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="74" t="s">
+      <c r="C37" s="77" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="69" t="s">
+      <c r="E37" s="72" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="70" t="s">
+      <c r="F37" s="73" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="17"/>
@@ -10722,10 +10693,9 @@
       <c r="BM37" s="1"/>
       <c r="BO37" s="18"/>
       <c r="BP37" s="19"/>
-      <c r="BQ37" s="20"/>
+      <c r="BQ37" s="21"/>
       <c r="BS37" s="17"/>
       <c r="BT37" s="17"/>
-      <c r="BU37" s="17"/>
       <c r="BV37" s="18"/>
       <c r="BW37" s="19"/>
       <c r="BX37" s="20"/>
@@ -10881,14 +10851,14 @@
       <c r="HR37" s="17"/>
     </row>
     <row r="38" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="71"/>
-      <c r="B38" s="71"/>
-      <c r="C38" s="71"/>
+      <c r="A38" s="74"/>
+      <c r="B38" s="74"/>
+      <c r="C38" s="74"/>
       <c r="D38" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="69"/>
-      <c r="F38" s="69"/>
+      <c r="E38" s="72"/>
+      <c r="F38" s="72"/>
       <c r="G38" s="17"/>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -10943,10 +10913,9 @@
       <c r="BM38" s="1"/>
       <c r="BO38" s="18"/>
       <c r="BP38" s="19"/>
-      <c r="BQ38" s="20"/>
+      <c r="BQ38" s="21"/>
       <c r="BS38" s="17"/>
       <c r="BT38" s="17"/>
-      <c r="BU38" s="17"/>
       <c r="BV38" s="18"/>
       <c r="BW38" s="19"/>
       <c r="BX38" s="20"/>
@@ -11102,20 +11071,20 @@
       <c r="HR38" s="17"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="71"/>
-      <c r="B39" s="72" t="s">
+      <c r="A39" s="74"/>
+      <c r="B39" s="75" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="74" t="s">
+      <c r="C39" s="77" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="69" t="s">
+      <c r="E39" s="72" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="70" t="s">
+      <c r="F39" s="73" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="17"/>
@@ -11173,11 +11142,10 @@
       <c r="BN39" s="38"/>
       <c r="BO39" s="18"/>
       <c r="BP39" s="19"/>
-      <c r="BQ39" s="20"/>
-      <c r="BR39" s="68"/>
+      <c r="BQ39" s="21"/>
+      <c r="BR39" s="38"/>
       <c r="BS39" s="17"/>
       <c r="BT39" s="17"/>
-      <c r="BU39" s="17"/>
       <c r="BV39" s="18"/>
       <c r="BW39" s="19"/>
       <c r="BX39" s="20"/>
@@ -11333,14 +11301,14 @@
       <c r="HR39" s="17"/>
     </row>
     <row r="40" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="71"/>
-      <c r="B40" s="71"/>
-      <c r="C40" s="71"/>
+      <c r="A40" s="74"/>
+      <c r="B40" s="74"/>
+      <c r="C40" s="74"/>
       <c r="D40" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="69"/>
-      <c r="F40" s="69"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
@@ -11396,10 +11364,9 @@
       <c r="BM40" s="1"/>
       <c r="BO40" s="18"/>
       <c r="BP40" s="19"/>
-      <c r="BQ40" s="20"/>
+      <c r="BQ40" s="21"/>
       <c r="BS40" s="17"/>
       <c r="BT40" s="17"/>
-      <c r="BU40" s="17"/>
       <c r="BV40" s="18"/>
       <c r="BW40" s="19"/>
       <c r="BX40" s="20"/>
@@ -11555,22 +11522,22 @@
       <c r="HR40" s="17"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="71" t="s">
+      <c r="A41" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="72" t="s">
+      <c r="B41" s="75" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="74" t="s">
+      <c r="C41" s="77" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="69" t="s">
+      <c r="E41" s="72" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="70" t="s">
+      <c r="F41" s="73" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="17"/>
@@ -11627,10 +11594,9 @@
       <c r="BM41" s="1"/>
       <c r="BO41" s="18"/>
       <c r="BP41" s="19"/>
-      <c r="BQ41" s="20"/>
+      <c r="BQ41" s="21"/>
       <c r="BS41" s="17"/>
       <c r="BT41" s="17"/>
-      <c r="BU41" s="17"/>
       <c r="BV41" s="18"/>
       <c r="BW41" s="19"/>
       <c r="BX41" s="20"/>
@@ -11786,14 +11752,14 @@
       <c r="HR41" s="17"/>
     </row>
     <row r="42" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="71"/>
-      <c r="B42" s="71"/>
-      <c r="C42" s="71"/>
+      <c r="A42" s="74"/>
+      <c r="B42" s="74"/>
+      <c r="C42" s="74"/>
       <c r="D42" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="69"/>
-      <c r="F42" s="69"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
       <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
@@ -11848,10 +11814,9 @@
       <c r="BM42" s="1"/>
       <c r="BO42" s="18"/>
       <c r="BP42" s="19"/>
-      <c r="BQ42" s="20"/>
+      <c r="BQ42" s="21"/>
       <c r="BS42" s="17"/>
       <c r="BT42" s="17"/>
-      <c r="BU42" s="17"/>
       <c r="BV42" s="18"/>
       <c r="BW42" s="19"/>
       <c r="BX42" s="20"/>
@@ -12007,20 +11972,20 @@
       <c r="HR42" s="17"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="71"/>
-      <c r="B43" s="72" t="s">
+      <c r="A43" s="74"/>
+      <c r="B43" s="75" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="74" t="s">
+      <c r="C43" s="77" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="69" t="s">
+      <c r="E43" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="70" t="s">
+      <c r="F43" s="73" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="17"/>
@@ -12076,10 +12041,9 @@
       <c r="BM43" s="1"/>
       <c r="BO43" s="18"/>
       <c r="BP43" s="19"/>
-      <c r="BQ43" s="20"/>
+      <c r="BQ43" s="21"/>
       <c r="BS43" s="17"/>
       <c r="BT43" s="17"/>
-      <c r="BU43" s="17"/>
       <c r="BV43" s="18"/>
       <c r="BW43" s="19"/>
       <c r="BX43" s="20"/>
@@ -12235,14 +12199,14 @@
       <c r="HR43" s="17"/>
     </row>
     <row r="44" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="71"/>
-      <c r="B44" s="71"/>
-      <c r="C44" s="71"/>
+      <c r="A44" s="74"/>
+      <c r="B44" s="74"/>
+      <c r="C44" s="74"/>
       <c r="D44" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="69"/>
-      <c r="F44" s="69"/>
+      <c r="E44" s="72"/>
+      <c r="F44" s="72"/>
       <c r="G44" s="17"/>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -12299,10 +12263,9 @@
       <c r="BM44" s="1"/>
       <c r="BO44" s="18"/>
       <c r="BP44" s="19"/>
-      <c r="BQ44" s="20"/>
+      <c r="BQ44" s="21"/>
       <c r="BS44" s="17"/>
       <c r="BT44" s="17"/>
-      <c r="BU44" s="17"/>
       <c r="BV44" s="18"/>
       <c r="BW44" s="19"/>
       <c r="BX44" s="20"/>
@@ -12458,20 +12421,20 @@
       <c r="HR44" s="17"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="71"/>
-      <c r="B45" s="72" t="s">
+      <c r="A45" s="74"/>
+      <c r="B45" s="75" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="74" t="s">
+      <c r="C45" s="77" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="69" t="s">
+      <c r="E45" s="72" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="70" t="s">
+      <c r="F45" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="17"/>
@@ -12528,10 +12491,9 @@
       <c r="BM45" s="1"/>
       <c r="BO45" s="18"/>
       <c r="BP45" s="19"/>
-      <c r="BQ45" s="20"/>
+      <c r="BQ45" s="21"/>
       <c r="BS45" s="17"/>
       <c r="BT45" s="17"/>
-      <c r="BU45" s="17"/>
       <c r="BV45" s="18"/>
       <c r="BW45" s="19"/>
       <c r="BX45" s="20"/>
@@ -12687,14 +12649,14 @@
       <c r="HR45" s="17"/>
     </row>
     <row r="46" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="71"/>
-      <c r="B46" s="71"/>
-      <c r="C46" s="71"/>
+      <c r="A46" s="74"/>
+      <c r="B46" s="74"/>
+      <c r="C46" s="74"/>
       <c r="D46" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="69"/>
-      <c r="F46" s="69"/>
+      <c r="E46" s="72"/>
+      <c r="F46" s="72"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
@@ -12750,10 +12712,9 @@
       <c r="BM46" s="1"/>
       <c r="BO46" s="18"/>
       <c r="BP46" s="19"/>
-      <c r="BQ46" s="20"/>
+      <c r="BQ46" s="21"/>
       <c r="BS46" s="17"/>
       <c r="BT46" s="17"/>
-      <c r="BU46" s="17"/>
       <c r="BV46" s="18"/>
       <c r="BW46" s="19"/>
       <c r="BX46" s="20"/>
@@ -12909,22 +12870,22 @@
       <c r="HR46" s="17"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="71" t="s">
+      <c r="A47" s="74" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="72" t="s">
+      <c r="B47" s="75" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="74" t="s">
+      <c r="C47" s="77" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="69" t="s">
+      <c r="E47" s="72" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="70" t="s">
+      <c r="F47" s="73" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="17"/>
@@ -12984,10 +12945,9 @@
       <c r="BM47" s="1"/>
       <c r="BO47" s="18"/>
       <c r="BP47" s="19"/>
-      <c r="BQ47" s="20"/>
+      <c r="BQ47" s="21"/>
       <c r="BS47" s="17"/>
       <c r="BT47" s="17"/>
-      <c r="BU47" s="17"/>
       <c r="BV47" s="18"/>
       <c r="BW47" s="19"/>
       <c r="BX47" s="20"/>
@@ -13143,14 +13103,14 @@
       <c r="HR47" s="17"/>
     </row>
     <row r="48" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="71"/>
-      <c r="B48" s="71"/>
-      <c r="C48" s="71"/>
+      <c r="A48" s="74"/>
+      <c r="B48" s="74"/>
+      <c r="C48" s="74"/>
       <c r="D48" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="69"/>
-      <c r="F48" s="69"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="72"/>
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
@@ -13207,10 +13167,9 @@
       <c r="BM48" s="1"/>
       <c r="BO48" s="18"/>
       <c r="BP48" s="19"/>
-      <c r="BQ48" s="20"/>
+      <c r="BQ48" s="21"/>
       <c r="BS48" s="17"/>
       <c r="BT48" s="17"/>
-      <c r="BU48" s="17"/>
       <c r="BV48" s="18"/>
       <c r="BW48" s="19"/>
       <c r="BX48" s="20"/>
@@ -13366,20 +13325,20 @@
       <c r="HR48" s="17"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="71"/>
-      <c r="B49" s="72" t="s">
+      <c r="A49" s="74"/>
+      <c r="B49" s="75" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="74" t="s">
+      <c r="C49" s="77" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="69" t="s">
+      <c r="E49" s="72" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="70" t="s">
+      <c r="F49" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="17"/>
@@ -13437,10 +13396,9 @@
       <c r="BM49" s="1"/>
       <c r="BO49" s="18"/>
       <c r="BP49" s="19"/>
-      <c r="BQ49" s="20"/>
+      <c r="BQ49" s="21"/>
       <c r="BS49" s="17"/>
       <c r="BT49" s="17"/>
-      <c r="BU49" s="17"/>
       <c r="BV49" s="18"/>
       <c r="BW49" s="19"/>
       <c r="BX49" s="20"/>
@@ -13596,14 +13554,14 @@
       <c r="HR49" s="17"/>
     </row>
     <row r="50" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="71"/>
-      <c r="B50" s="71"/>
-      <c r="C50" s="71"/>
+      <c r="A50" s="74"/>
+      <c r="B50" s="74"/>
+      <c r="C50" s="74"/>
       <c r="D50" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="69"/>
-      <c r="F50" s="69"/>
+      <c r="E50" s="72"/>
+      <c r="F50" s="72"/>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
@@ -13659,10 +13617,9 @@
       <c r="BM50" s="1"/>
       <c r="BO50" s="18"/>
       <c r="BP50" s="19"/>
-      <c r="BQ50" s="20"/>
+      <c r="BQ50" s="21"/>
       <c r="BS50" s="17"/>
       <c r="BT50" s="17"/>
-      <c r="BU50" s="17"/>
       <c r="BV50" s="18"/>
       <c r="BW50" s="19"/>
       <c r="BX50" s="20"/>
@@ -13818,22 +13775,22 @@
       <c r="HR50" s="17"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="71" t="s">
+      <c r="A51" s="74" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="72" t="s">
+      <c r="B51" s="75" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="74" t="s">
+      <c r="C51" s="77" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="69" t="s">
+      <c r="E51" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="70" t="s">
+      <c r="F51" s="73" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="17"/>
@@ -13890,10 +13847,10 @@
       <c r="BM51" s="1"/>
       <c r="BO51" s="18"/>
       <c r="BP51" s="19"/>
-      <c r="BQ51" s="20"/>
+      <c r="BQ51" s="21"/>
       <c r="BS51" s="16"/>
       <c r="BT51" s="16"/>
-      <c r="BU51" s="16"/>
+      <c r="BU51" s="71"/>
       <c r="BV51" s="18"/>
       <c r="BW51" s="19"/>
       <c r="BX51" s="20"/>
@@ -14049,14 +14006,14 @@
       <c r="HR51" s="17"/>
     </row>
     <row r="52" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="71"/>
-      <c r="B52" s="71"/>
-      <c r="C52" s="71"/>
+      <c r="A52" s="74"/>
+      <c r="B52" s="74"/>
+      <c r="C52" s="74"/>
       <c r="D52" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="69"/>
-      <c r="F52" s="69"/>
+      <c r="E52" s="72"/>
+      <c r="F52" s="72"/>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
@@ -14108,13 +14065,12 @@
       <c r="BI52" s="21"/>
       <c r="BJ52" s="21"/>
       <c r="BL52" s="17"/>
-      <c r="BM52" s="82"/>
+      <c r="BM52" s="69"/>
       <c r="BO52" s="18"/>
       <c r="BP52" s="19"/>
-      <c r="BQ52" s="20"/>
-      <c r="BS52" s="17"/>
-      <c r="BT52" s="17"/>
-      <c r="BU52" s="17"/>
+      <c r="BQ52" s="21"/>
+      <c r="BS52" s="70"/>
+      <c r="BT52" s="70"/>
       <c r="BV52" s="18"/>
       <c r="BW52" s="19"/>
       <c r="BX52" s="20"/>
@@ -14270,20 +14226,20 @@
       <c r="HR52" s="17"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="71"/>
-      <c r="B53" s="72" t="s">
+      <c r="A53" s="74"/>
+      <c r="B53" s="75" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="74" t="s">
-        <v>117</v>
+      <c r="C53" s="77" t="s">
+        <v>268</v>
       </c>
       <c r="D53" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="69" t="s">
-        <v>118</v>
-      </c>
-      <c r="F53" s="70" t="s">
+      <c r="E53" s="72" t="s">
+        <v>269</v>
+      </c>
+      <c r="F53" s="73" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="17"/>
@@ -14340,10 +14296,9 @@
       <c r="BM53" s="1"/>
       <c r="BO53" s="18"/>
       <c r="BP53" s="19"/>
-      <c r="BQ53" s="20"/>
+      <c r="BQ53" s="21"/>
       <c r="BS53" s="17"/>
       <c r="BT53" s="17"/>
-      <c r="BU53" s="17"/>
       <c r="BV53" s="18"/>
       <c r="BW53" s="19"/>
       <c r="BX53" s="20"/>
@@ -14499,14 +14454,14 @@
       <c r="HR53" s="17"/>
     </row>
     <row r="54" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="71"/>
-      <c r="B54" s="71"/>
-      <c r="C54" s="71"/>
+      <c r="A54" s="74"/>
+      <c r="B54" s="74"/>
+      <c r="C54" s="74"/>
       <c r="D54" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="69"/>
-      <c r="F54" s="69"/>
+      <c r="E54" s="72"/>
+      <c r="F54" s="72"/>
       <c r="G54" s="17"/>
       <c r="H54" s="17"/>
       <c r="I54" s="17"/>
@@ -14561,10 +14516,9 @@
       <c r="BM54" s="1"/>
       <c r="BO54" s="18"/>
       <c r="BP54" s="19"/>
-      <c r="BQ54" s="20"/>
+      <c r="BQ54" s="21"/>
       <c r="BS54" s="17"/>
       <c r="BT54" s="17"/>
-      <c r="BU54" s="17"/>
       <c r="BV54" s="18"/>
       <c r="BW54" s="19"/>
       <c r="BX54" s="20"/>
@@ -14720,22 +14674,22 @@
       <c r="HR54" s="17"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="71" t="s">
+      <c r="A55" s="74" t="s">
+        <v>117</v>
+      </c>
+      <c r="B55" s="75" t="s">
+        <v>118</v>
+      </c>
+      <c r="C55" s="77" t="s">
         <v>119</v>
-      </c>
-      <c r="B55" s="72" t="s">
-        <v>120</v>
-      </c>
-      <c r="C55" s="74" t="s">
-        <v>121</v>
       </c>
       <c r="D55" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="69" t="s">
-        <v>122</v>
-      </c>
-      <c r="F55" s="70" t="s">
+      <c r="E55" s="72" t="s">
+        <v>120</v>
+      </c>
+      <c r="F55" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="17"/>
@@ -14792,10 +14746,9 @@
       <c r="BM55" s="1"/>
       <c r="BO55" s="18"/>
       <c r="BP55" s="19"/>
-      <c r="BQ55" s="20"/>
+      <c r="BQ55" s="21"/>
       <c r="BS55" s="17"/>
       <c r="BT55" s="17"/>
-      <c r="BU55" s="17"/>
       <c r="BV55" s="18"/>
       <c r="BW55" s="19"/>
       <c r="BX55" s="20"/>
@@ -14951,14 +14904,14 @@
       <c r="HR55" s="17"/>
     </row>
     <row r="56" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="71"/>
-      <c r="B56" s="71"/>
-      <c r="C56" s="71"/>
+      <c r="A56" s="74"/>
+      <c r="B56" s="74"/>
+      <c r="C56" s="74"/>
       <c r="D56" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="69"/>
-      <c r="F56" s="69"/>
+      <c r="E56" s="72"/>
+      <c r="F56" s="72"/>
       <c r="G56" s="17"/>
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
@@ -15013,10 +14966,9 @@
       <c r="BM56" s="1"/>
       <c r="BO56" s="18"/>
       <c r="BP56" s="19"/>
-      <c r="BQ56" s="20"/>
+      <c r="BQ56" s="21"/>
       <c r="BS56" s="17"/>
       <c r="BT56" s="17"/>
-      <c r="BU56" s="17"/>
       <c r="BV56" s="18"/>
       <c r="BW56" s="19"/>
       <c r="BX56" s="20"/>
@@ -15172,20 +15124,20 @@
       <c r="HR56" s="17"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="71"/>
-      <c r="B57" s="72" t="s">
-        <v>123</v>
-      </c>
-      <c r="C57" s="74" t="s">
-        <v>124</v>
+      <c r="A57" s="74"/>
+      <c r="B57" s="75" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" s="77" t="s">
+        <v>122</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="69" t="s">
-        <v>125</v>
-      </c>
-      <c r="F57" s="70" t="s">
+      <c r="E57" s="72" t="s">
+        <v>123</v>
+      </c>
+      <c r="F57" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="17"/>
@@ -15242,10 +15194,9 @@
       <c r="BM57" s="1"/>
       <c r="BO57" s="18"/>
       <c r="BP57" s="19"/>
-      <c r="BQ57" s="20"/>
+      <c r="BQ57" s="21"/>
       <c r="BS57" s="17"/>
       <c r="BT57" s="17"/>
-      <c r="BU57" s="17"/>
       <c r="BV57" s="18"/>
       <c r="BW57" s="19"/>
       <c r="BX57" s="20"/>
@@ -15401,14 +15352,14 @@
       <c r="HR57" s="17"/>
     </row>
     <row r="58" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="71"/>
-      <c r="B58" s="71"/>
-      <c r="C58" s="71"/>
+      <c r="A58" s="74"/>
+      <c r="B58" s="74"/>
+      <c r="C58" s="74"/>
       <c r="D58" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="69"/>
-      <c r="F58" s="69"/>
+      <c r="E58" s="72"/>
+      <c r="F58" s="72"/>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
@@ -15463,10 +15414,9 @@
       <c r="BM58" s="1"/>
       <c r="BO58" s="18"/>
       <c r="BP58" s="19"/>
-      <c r="BQ58" s="20"/>
+      <c r="BQ58" s="21"/>
       <c r="BS58" s="17"/>
       <c r="BT58" s="17"/>
-      <c r="BU58" s="17"/>
       <c r="BV58" s="18"/>
       <c r="BW58" s="19"/>
       <c r="BX58" s="20"/>
@@ -15622,20 +15572,20 @@
       <c r="HR58" s="17"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="71"/>
-      <c r="B59" s="72" t="s">
-        <v>126</v>
-      </c>
-      <c r="C59" s="74" t="s">
-        <v>127</v>
+      <c r="A59" s="74"/>
+      <c r="B59" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="C59" s="77" t="s">
+        <v>125</v>
       </c>
       <c r="D59" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="69" t="s">
-        <v>128</v>
-      </c>
-      <c r="F59" s="70" t="s">
+      <c r="E59" s="72" t="s">
+        <v>126</v>
+      </c>
+      <c r="F59" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="17"/>
@@ -15692,10 +15642,9 @@
       <c r="BM59" s="1"/>
       <c r="BO59" s="18"/>
       <c r="BP59" s="19"/>
-      <c r="BQ59" s="20"/>
+      <c r="BQ59" s="21"/>
       <c r="BS59" s="17"/>
       <c r="BT59" s="17"/>
-      <c r="BU59" s="17"/>
       <c r="BV59" s="18"/>
       <c r="BW59" s="19"/>
       <c r="BX59" s="20"/>
@@ -15851,14 +15800,14 @@
       <c r="HR59" s="17"/>
     </row>
     <row r="60" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="71"/>
-      <c r="B60" s="71"/>
-      <c r="C60" s="71"/>
+      <c r="A60" s="74"/>
+      <c r="B60" s="74"/>
+      <c r="C60" s="74"/>
       <c r="D60" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="69"/>
-      <c r="F60" s="69"/>
+      <c r="E60" s="72"/>
+      <c r="F60" s="72"/>
       <c r="G60" s="17"/>
       <c r="H60" s="17"/>
       <c r="I60" s="17"/>
@@ -15913,10 +15862,9 @@
       <c r="BM60" s="1"/>
       <c r="BO60" s="18"/>
       <c r="BP60" s="19"/>
-      <c r="BQ60" s="20"/>
+      <c r="BQ60" s="21"/>
       <c r="BS60" s="17"/>
       <c r="BT60" s="17"/>
-      <c r="BU60" s="17"/>
       <c r="BV60" s="18"/>
       <c r="BW60" s="19"/>
       <c r="BX60" s="20"/>
@@ -16072,20 +16020,20 @@
       <c r="HR60" s="17"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="71"/>
-      <c r="B61" s="72" t="s">
-        <v>129</v>
-      </c>
-      <c r="C61" s="74" t="s">
-        <v>130</v>
+      <c r="A61" s="74"/>
+      <c r="B61" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="C61" s="77" t="s">
+        <v>128</v>
       </c>
       <c r="D61" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="69" t="s">
-        <v>131</v>
-      </c>
-      <c r="F61" s="70" t="s">
+      <c r="E61" s="72" t="s">
+        <v>129</v>
+      </c>
+      <c r="F61" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="17"/>
@@ -16142,10 +16090,9 @@
       <c r="BM61" s="1"/>
       <c r="BO61" s="18"/>
       <c r="BP61" s="19"/>
-      <c r="BQ61" s="20"/>
+      <c r="BQ61" s="21"/>
       <c r="BS61" s="17"/>
       <c r="BT61" s="17"/>
-      <c r="BU61" s="17"/>
       <c r="BV61" s="18"/>
       <c r="BW61" s="19"/>
       <c r="BX61" s="20"/>
@@ -16301,14 +16248,14 @@
       <c r="HR61" s="17"/>
     </row>
     <row r="62" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="71"/>
-      <c r="B62" s="71"/>
-      <c r="C62" s="71"/>
+      <c r="A62" s="74"/>
+      <c r="B62" s="74"/>
+      <c r="C62" s="74"/>
       <c r="D62" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="69"/>
-      <c r="F62" s="69"/>
+      <c r="E62" s="72"/>
+      <c r="F62" s="72"/>
       <c r="G62" s="17"/>
       <c r="H62" s="17"/>
       <c r="I62" s="17"/>
@@ -16363,10 +16310,9 @@
       <c r="BM62" s="1"/>
       <c r="BO62" s="18"/>
       <c r="BP62" s="19"/>
-      <c r="BQ62" s="20"/>
+      <c r="BQ62" s="21"/>
       <c r="BS62" s="17"/>
       <c r="BT62" s="17"/>
-      <c r="BU62" s="17"/>
       <c r="BV62" s="18"/>
       <c r="BW62" s="19"/>
       <c r="BX62" s="20"/>
@@ -16522,20 +16468,20 @@
       <c r="HR62" s="17"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="71"/>
-      <c r="B63" s="72" t="s">
-        <v>132</v>
-      </c>
-      <c r="C63" s="74" t="s">
-        <v>133</v>
+      <c r="A63" s="74"/>
+      <c r="B63" s="75" t="s">
+        <v>130</v>
+      </c>
+      <c r="C63" s="77" t="s">
+        <v>131</v>
       </c>
       <c r="D63" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="69" t="s">
-        <v>134</v>
-      </c>
-      <c r="F63" s="70" t="s">
+      <c r="E63" s="72" t="s">
+        <v>132</v>
+      </c>
+      <c r="F63" s="73" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="17"/>
@@ -16592,10 +16538,9 @@
       <c r="BM63" s="1"/>
       <c r="BO63" s="18"/>
       <c r="BP63" s="19"/>
-      <c r="BQ63" s="20"/>
+      <c r="BQ63" s="21"/>
       <c r="BS63" s="17"/>
       <c r="BT63" s="17"/>
-      <c r="BU63" s="17"/>
       <c r="BV63" s="18"/>
       <c r="BW63" s="19"/>
       <c r="BX63" s="20"/>
@@ -16751,14 +16696,14 @@
       <c r="HR63" s="17"/>
     </row>
     <row r="64" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="71"/>
-      <c r="B64" s="71"/>
-      <c r="C64" s="71"/>
+      <c r="A64" s="74"/>
+      <c r="B64" s="74"/>
+      <c r="C64" s="74"/>
       <c r="D64" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="69"/>
-      <c r="F64" s="69"/>
+      <c r="E64" s="72"/>
+      <c r="F64" s="72"/>
       <c r="G64" s="17"/>
       <c r="H64" s="17"/>
       <c r="I64" s="17"/>
@@ -16813,10 +16758,9 @@
       <c r="BM64" s="1"/>
       <c r="BO64" s="18"/>
       <c r="BP64" s="19"/>
-      <c r="BQ64" s="20"/>
+      <c r="BQ64" s="21"/>
       <c r="BS64" s="17"/>
       <c r="BT64" s="17"/>
-      <c r="BU64" s="17"/>
       <c r="BV64" s="18"/>
       <c r="BW64" s="19"/>
       <c r="BX64" s="20"/>
@@ -16972,20 +16916,20 @@
       <c r="HR64" s="17"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="71"/>
-      <c r="B65" s="72" t="s">
-        <v>135</v>
-      </c>
-      <c r="C65" s="74" t="s">
-        <v>136</v>
+      <c r="A65" s="74"/>
+      <c r="B65" s="75" t="s">
+        <v>133</v>
+      </c>
+      <c r="C65" s="77" t="s">
+        <v>134</v>
       </c>
       <c r="D65" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="69" t="s">
-        <v>137</v>
-      </c>
-      <c r="F65" s="70" t="s">
+      <c r="E65" s="72" t="s">
+        <v>135</v>
+      </c>
+      <c r="F65" s="73" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="17"/>
@@ -17042,10 +16986,9 @@
       <c r="BM65" s="1"/>
       <c r="BO65" s="18"/>
       <c r="BP65" s="19"/>
-      <c r="BQ65" s="20"/>
+      <c r="BQ65" s="21"/>
       <c r="BS65" s="17"/>
       <c r="BT65" s="17"/>
-      <c r="BU65" s="17"/>
       <c r="BV65" s="18"/>
       <c r="BW65" s="19"/>
       <c r="BX65" s="20"/>
@@ -17201,14 +17144,14 @@
       <c r="HR65" s="17"/>
     </row>
     <row r="66" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="71"/>
-      <c r="B66" s="71"/>
-      <c r="C66" s="71"/>
+      <c r="A66" s="74"/>
+      <c r="B66" s="74"/>
+      <c r="C66" s="74"/>
       <c r="D66" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="69"/>
-      <c r="F66" s="69"/>
+      <c r="E66" s="72"/>
+      <c r="F66" s="72"/>
       <c r="G66" s="17"/>
       <c r="H66" s="17"/>
       <c r="I66" s="17"/>
@@ -17263,10 +17206,9 @@
       <c r="BM66" s="1"/>
       <c r="BO66" s="18"/>
       <c r="BP66" s="19"/>
-      <c r="BQ66" s="20"/>
+      <c r="BQ66" s="21"/>
       <c r="BS66" s="17"/>
       <c r="BT66" s="17"/>
-      <c r="BU66" s="17"/>
       <c r="BV66" s="18"/>
       <c r="BW66" s="19"/>
       <c r="BX66" s="20"/>
@@ -17422,22 +17364,22 @@
       <c r="HR66" s="17"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="71" t="s">
+      <c r="A67" s="74" t="s">
+        <v>136</v>
+      </c>
+      <c r="B67" s="75" t="s">
+        <v>137</v>
+      </c>
+      <c r="C67" s="77" t="s">
         <v>138</v>
-      </c>
-      <c r="B67" s="72" t="s">
-        <v>139</v>
-      </c>
-      <c r="C67" s="74" t="s">
-        <v>140</v>
       </c>
       <c r="D67" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="69" t="s">
-        <v>141</v>
-      </c>
-      <c r="F67" s="70" t="s">
+      <c r="E67" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="F67" s="73" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="17"/>
@@ -17494,10 +17436,9 @@
       <c r="BM67" s="1"/>
       <c r="BO67" s="18"/>
       <c r="BP67" s="19"/>
-      <c r="BQ67" s="20"/>
+      <c r="BQ67" s="21"/>
       <c r="BS67" s="17"/>
       <c r="BT67" s="17"/>
-      <c r="BU67" s="17"/>
       <c r="BV67" s="18"/>
       <c r="BW67" s="19"/>
       <c r="BX67" s="20"/>
@@ -17653,14 +17594,14 @@
       <c r="HR67" s="17"/>
     </row>
     <row r="68" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="71"/>
-      <c r="B68" s="71"/>
-      <c r="C68" s="71"/>
+      <c r="A68" s="74"/>
+      <c r="B68" s="74"/>
+      <c r="C68" s="74"/>
       <c r="D68" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="69"/>
-      <c r="F68" s="69"/>
+      <c r="E68" s="72"/>
+      <c r="F68" s="72"/>
       <c r="G68" s="17"/>
       <c r="H68" s="17"/>
       <c r="I68" s="17"/>
@@ -17716,10 +17657,9 @@
       <c r="BM68" s="1"/>
       <c r="BO68" s="18"/>
       <c r="BP68" s="19"/>
-      <c r="BQ68" s="20"/>
+      <c r="BQ68" s="21"/>
       <c r="BS68" s="17"/>
       <c r="BT68" s="17"/>
-      <c r="BU68" s="17"/>
       <c r="BV68" s="18"/>
       <c r="BW68" s="19"/>
       <c r="BX68" s="20"/>
@@ -17875,20 +17815,20 @@
       <c r="HR68" s="17"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="71"/>
-      <c r="B69" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="C69" s="74" t="s">
-        <v>143</v>
+      <c r="A69" s="74"/>
+      <c r="B69" s="75" t="s">
+        <v>140</v>
+      </c>
+      <c r="C69" s="77" t="s">
+        <v>141</v>
       </c>
       <c r="D69" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="69" t="s">
-        <v>144</v>
-      </c>
-      <c r="F69" s="70" t="s">
+      <c r="E69" s="72" t="s">
+        <v>142</v>
+      </c>
+      <c r="F69" s="73" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="17"/>
@@ -17953,11 +17893,11 @@
       <c r="BN69" s="38"/>
       <c r="BO69" s="18"/>
       <c r="BP69" s="19"/>
-      <c r="BQ69" s="20"/>
-      <c r="BR69" s="68"/>
+      <c r="BQ69" s="21"/>
+      <c r="BR69" s="38"/>
       <c r="BS69" s="39"/>
       <c r="BT69" s="39"/>
-      <c r="BU69" s="39"/>
+      <c r="BU69" s="68"/>
       <c r="BV69" s="18"/>
       <c r="BW69" s="19"/>
       <c r="BX69" s="20"/>
@@ -18113,14 +18053,14 @@
       <c r="HR69" s="17"/>
     </row>
     <row r="70" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="71"/>
-      <c r="B70" s="71"/>
-      <c r="C70" s="71"/>
+      <c r="A70" s="74"/>
+      <c r="B70" s="74"/>
+      <c r="C70" s="74"/>
       <c r="D70" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="69"/>
-      <c r="F70" s="69"/>
+      <c r="E70" s="72"/>
+      <c r="F70" s="72"/>
       <c r="G70" s="17"/>
       <c r="H70" s="17"/>
       <c r="I70" s="17"/>
@@ -18175,14 +18115,13 @@
       <c r="BI70" s="21"/>
       <c r="BJ70" s="21"/>
       <c r="BL70" s="17"/>
-      <c r="BM70" s="83"/>
+      <c r="BM70" s="70"/>
       <c r="BO70" s="18"/>
       <c r="BP70" s="19"/>
-      <c r="BQ70" s="20"/>
-      <c r="BR70" s="84"/>
-      <c r="BS70" s="17"/>
-      <c r="BT70" s="17"/>
-      <c r="BU70" s="17"/>
+      <c r="BQ70" s="21"/>
+      <c r="BR70" s="70"/>
+      <c r="BS70" s="70"/>
+      <c r="BT70" s="70"/>
       <c r="BV70" s="18"/>
       <c r="BW70" s="19"/>
       <c r="BX70" s="20"/>
@@ -18338,20 +18277,20 @@
       <c r="HR70" s="17"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="71"/>
-      <c r="B71" s="72" t="s">
-        <v>145</v>
-      </c>
-      <c r="C71" s="74" t="s">
-        <v>146</v>
+      <c r="A71" s="74"/>
+      <c r="B71" s="75" t="s">
+        <v>143</v>
+      </c>
+      <c r="C71" s="77" t="s">
+        <v>144</v>
       </c>
       <c r="D71" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="69" t="s">
-        <v>147</v>
-      </c>
-      <c r="F71" s="70" t="s">
+      <c r="E71" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="F71" s="73" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="17"/>
@@ -18408,10 +18347,9 @@
       <c r="BM71" s="1"/>
       <c r="BO71" s="18"/>
       <c r="BP71" s="19"/>
-      <c r="BQ71" s="20"/>
+      <c r="BQ71" s="21"/>
       <c r="BS71" s="17"/>
       <c r="BT71" s="17"/>
-      <c r="BU71" s="17"/>
       <c r="BV71" s="18"/>
       <c r="BW71" s="19"/>
       <c r="BX71" s="20"/>
@@ -18567,14 +18505,14 @@
       <c r="HR71" s="17"/>
     </row>
     <row r="72" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="71"/>
-      <c r="B72" s="71"/>
-      <c r="C72" s="71"/>
+      <c r="A72" s="74"/>
+      <c r="B72" s="74"/>
+      <c r="C72" s="74"/>
       <c r="D72" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="69"/>
-      <c r="F72" s="69"/>
+      <c r="E72" s="72"/>
+      <c r="F72" s="72"/>
       <c r="G72" s="17"/>
       <c r="H72" s="17"/>
       <c r="I72" s="17"/>
@@ -18629,10 +18567,9 @@
       <c r="BM72" s="1"/>
       <c r="BO72" s="18"/>
       <c r="BP72" s="19"/>
-      <c r="BQ72" s="20"/>
+      <c r="BQ72" s="21"/>
       <c r="BS72" s="17"/>
       <c r="BT72" s="17"/>
-      <c r="BU72" s="17"/>
       <c r="BV72" s="18"/>
       <c r="BW72" s="19"/>
       <c r="BX72" s="20"/>
@@ -18788,20 +18725,20 @@
       <c r="HR72" s="17"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="71"/>
-      <c r="B73" s="72" t="s">
-        <v>148</v>
-      </c>
-      <c r="C73" s="74" t="s">
-        <v>149</v>
+      <c r="A73" s="74"/>
+      <c r="B73" s="75" t="s">
+        <v>146</v>
+      </c>
+      <c r="C73" s="77" t="s">
+        <v>147</v>
       </c>
       <c r="D73" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="69" t="s">
-        <v>150</v>
-      </c>
-      <c r="F73" s="70" t="s">
+      <c r="E73" s="72" t="s">
+        <v>148</v>
+      </c>
+      <c r="F73" s="73" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="17"/>
@@ -18858,10 +18795,9 @@
       <c r="BM73" s="1"/>
       <c r="BO73" s="18"/>
       <c r="BP73" s="19"/>
-      <c r="BQ73" s="20"/>
+      <c r="BQ73" s="21"/>
       <c r="BS73" s="17"/>
       <c r="BT73" s="17"/>
-      <c r="BU73" s="17"/>
       <c r="BV73" s="18"/>
       <c r="BW73" s="19"/>
       <c r="BX73" s="20"/>
@@ -19017,14 +18953,14 @@
       <c r="HR73" s="17"/>
     </row>
     <row r="74" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="71"/>
-      <c r="B74" s="71"/>
-      <c r="C74" s="71"/>
+      <c r="A74" s="74"/>
+      <c r="B74" s="74"/>
+      <c r="C74" s="74"/>
       <c r="D74" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="69"/>
-      <c r="F74" s="69"/>
+      <c r="E74" s="72"/>
+      <c r="F74" s="72"/>
       <c r="G74" s="17"/>
       <c r="H74" s="17"/>
       <c r="I74" s="17"/>
@@ -19079,10 +19015,9 @@
       <c r="BM74" s="1"/>
       <c r="BO74" s="18"/>
       <c r="BP74" s="19"/>
-      <c r="BQ74" s="20"/>
+      <c r="BQ74" s="21"/>
       <c r="BS74" s="17"/>
       <c r="BT74" s="17"/>
-      <c r="BU74" s="17"/>
       <c r="BV74" s="18"/>
       <c r="BW74" s="19"/>
       <c r="BX74" s="20"/>
@@ -19238,20 +19173,20 @@
       <c r="HR74" s="17"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="71"/>
-      <c r="B75" s="72" t="s">
-        <v>151</v>
-      </c>
-      <c r="C75" s="74" t="s">
-        <v>152</v>
+      <c r="A75" s="74"/>
+      <c r="B75" s="75" t="s">
+        <v>149</v>
+      </c>
+      <c r="C75" s="77" t="s">
+        <v>150</v>
       </c>
       <c r="D75" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="69" t="s">
-        <v>153</v>
-      </c>
-      <c r="F75" s="70" t="s">
+      <c r="E75" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="F75" s="73" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="17"/>
@@ -19308,10 +19243,9 @@
       <c r="BM75" s="1"/>
       <c r="BO75" s="18"/>
       <c r="BP75" s="19"/>
-      <c r="BQ75" s="20"/>
+      <c r="BQ75" s="21"/>
       <c r="BS75" s="17"/>
       <c r="BT75" s="17"/>
-      <c r="BU75" s="17"/>
       <c r="BV75" s="18"/>
       <c r="BW75" s="19"/>
       <c r="BX75" s="20"/>
@@ -19467,14 +19401,14 @@
       <c r="HR75" s="17"/>
     </row>
     <row r="76" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="71"/>
-      <c r="B76" s="71"/>
-      <c r="C76" s="71"/>
+      <c r="A76" s="74"/>
+      <c r="B76" s="74"/>
+      <c r="C76" s="74"/>
       <c r="D76" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="69"/>
-      <c r="F76" s="69"/>
+      <c r="E76" s="72"/>
+      <c r="F76" s="72"/>
       <c r="G76" s="17"/>
       <c r="H76" s="17"/>
       <c r="I76" s="17"/>
@@ -19529,10 +19463,9 @@
       <c r="BM76" s="1"/>
       <c r="BO76" s="18"/>
       <c r="BP76" s="19"/>
-      <c r="BQ76" s="20"/>
+      <c r="BQ76" s="21"/>
       <c r="BS76" s="17"/>
       <c r="BT76" s="17"/>
-      <c r="BU76" s="17"/>
       <c r="BV76" s="18"/>
       <c r="BW76" s="19"/>
       <c r="BX76" s="20"/>
@@ -19688,20 +19621,20 @@
       <c r="HR76" s="17"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="71"/>
-      <c r="B77" s="72" t="s">
-        <v>154</v>
-      </c>
-      <c r="C77" s="74" t="s">
-        <v>155</v>
+      <c r="A77" s="74"/>
+      <c r="B77" s="75" t="s">
+        <v>152</v>
+      </c>
+      <c r="C77" s="77" t="s">
+        <v>153</v>
       </c>
       <c r="D77" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="F77" s="70" t="s">
+      <c r="E77" s="72" t="s">
+        <v>154</v>
+      </c>
+      <c r="F77" s="73" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="17"/>
@@ -19758,10 +19691,9 @@
       <c r="BM77" s="1"/>
       <c r="BO77" s="18"/>
       <c r="BP77" s="19"/>
-      <c r="BQ77" s="20"/>
+      <c r="BQ77" s="21"/>
       <c r="BS77" s="17"/>
       <c r="BT77" s="17"/>
-      <c r="BU77" s="17"/>
       <c r="BV77" s="18"/>
       <c r="BW77" s="19"/>
       <c r="BX77" s="20"/>
@@ -19917,14 +19849,14 @@
       <c r="HR77" s="17"/>
     </row>
     <row r="78" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="71"/>
-      <c r="B78" s="71"/>
-      <c r="C78" s="71"/>
+      <c r="A78" s="74"/>
+      <c r="B78" s="74"/>
+      <c r="C78" s="74"/>
       <c r="D78" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="69"/>
-      <c r="F78" s="69"/>
+      <c r="E78" s="72"/>
+      <c r="F78" s="72"/>
       <c r="G78" s="17"/>
       <c r="H78" s="17"/>
       <c r="I78" s="17"/>
@@ -19979,10 +19911,9 @@
       <c r="BM78" s="1"/>
       <c r="BO78" s="18"/>
       <c r="BP78" s="19"/>
-      <c r="BQ78" s="20"/>
+      <c r="BQ78" s="21"/>
       <c r="BS78" s="17"/>
       <c r="BT78" s="17"/>
-      <c r="BU78" s="17"/>
       <c r="BV78" s="18"/>
       <c r="BW78" s="19"/>
       <c r="BX78" s="20"/>
@@ -20138,22 +20069,22 @@
       <c r="HR78" s="17"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="71" t="s">
+      <c r="A79" s="74" t="s">
+        <v>155</v>
+      </c>
+      <c r="B79" s="75" t="s">
+        <v>156</v>
+      </c>
+      <c r="C79" s="76" t="s">
         <v>157</v>
-      </c>
-      <c r="B79" s="72" t="s">
-        <v>158</v>
-      </c>
-      <c r="C79" s="73" t="s">
-        <v>159</v>
       </c>
       <c r="D79" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="69" t="s">
-        <v>160</v>
-      </c>
-      <c r="F79" s="70" t="s">
+      <c r="E79" s="72" t="s">
+        <v>158</v>
+      </c>
+      <c r="F79" s="73" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="17"/>
@@ -20210,10 +20141,9 @@
       <c r="BM79" s="1"/>
       <c r="BO79" s="18"/>
       <c r="BP79" s="19"/>
-      <c r="BQ79" s="20"/>
+      <c r="BQ79" s="21"/>
       <c r="BS79" s="17"/>
       <c r="BT79" s="17"/>
-      <c r="BU79" s="17"/>
       <c r="BV79" s="18"/>
       <c r="BW79" s="19"/>
       <c r="BX79" s="20"/>
@@ -20369,14 +20299,14 @@
       <c r="HR79" s="17"/>
     </row>
     <row r="80" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="71"/>
-      <c r="B80" s="71"/>
-      <c r="C80" s="71"/>
+      <c r="A80" s="74"/>
+      <c r="B80" s="74"/>
+      <c r="C80" s="74"/>
       <c r="D80" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="69"/>
-      <c r="F80" s="69"/>
+      <c r="E80" s="72"/>
+      <c r="F80" s="72"/>
       <c r="G80" s="17"/>
       <c r="H80" s="17"/>
       <c r="I80" s="17"/>
@@ -20431,10 +20361,9 @@
       <c r="BM80" s="1"/>
       <c r="BO80" s="18"/>
       <c r="BP80" s="19"/>
-      <c r="BQ80" s="20"/>
+      <c r="BQ80" s="21"/>
       <c r="BS80" s="17"/>
       <c r="BT80" s="17"/>
-      <c r="BU80" s="17"/>
       <c r="BV80" s="18"/>
       <c r="BW80" s="19"/>
       <c r="BX80" s="20"/>
@@ -20590,20 +20519,20 @@
       <c r="HR80" s="17"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="71"/>
-      <c r="B81" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="C81" s="73" t="s">
-        <v>162</v>
+      <c r="A81" s="74"/>
+      <c r="B81" s="75" t="s">
+        <v>159</v>
+      </c>
+      <c r="C81" s="76" t="s">
+        <v>160</v>
       </c>
       <c r="D81" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="69" t="s">
-        <v>163</v>
-      </c>
-      <c r="F81" s="70" t="s">
+      <c r="E81" s="72" t="s">
+        <v>161</v>
+      </c>
+      <c r="F81" s="73" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="17"/>
@@ -20660,10 +20589,9 @@
       <c r="BM81" s="1"/>
       <c r="BO81" s="18"/>
       <c r="BP81" s="19"/>
-      <c r="BQ81" s="20"/>
+      <c r="BQ81" s="21"/>
       <c r="BS81" s="17"/>
       <c r="BT81" s="17"/>
-      <c r="BU81" s="17"/>
       <c r="BV81" s="18"/>
       <c r="BW81" s="19"/>
       <c r="BX81" s="20"/>
@@ -20819,14 +20747,14 @@
       <c r="HR81" s="17"/>
     </row>
     <row r="82" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="71"/>
-      <c r="B82" s="71"/>
-      <c r="C82" s="71"/>
+      <c r="A82" s="74"/>
+      <c r="B82" s="74"/>
+      <c r="C82" s="74"/>
       <c r="D82" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="69"/>
-      <c r="F82" s="69"/>
+      <c r="E82" s="72"/>
+      <c r="F82" s="72"/>
       <c r="G82" s="17"/>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
@@ -20881,10 +20809,9 @@
       <c r="BM82" s="1"/>
       <c r="BO82" s="18"/>
       <c r="BP82" s="19"/>
-      <c r="BQ82" s="20"/>
+      <c r="BQ82" s="21"/>
       <c r="BS82" s="17"/>
       <c r="BT82" s="17"/>
-      <c r="BU82" s="17"/>
       <c r="BV82" s="18"/>
       <c r="BW82" s="19"/>
       <c r="BX82" s="20"/>
@@ -21040,20 +20967,20 @@
       <c r="HR82" s="17"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="71"/>
-      <c r="B83" s="72" t="s">
-        <v>164</v>
-      </c>
-      <c r="C83" s="74" t="s">
-        <v>165</v>
+      <c r="A83" s="74"/>
+      <c r="B83" s="75" t="s">
+        <v>162</v>
+      </c>
+      <c r="C83" s="77" t="s">
+        <v>163</v>
       </c>
       <c r="D83" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="69" t="s">
-        <v>166</v>
-      </c>
-      <c r="F83" s="70" t="s">
+      <c r="E83" s="72" t="s">
+        <v>164</v>
+      </c>
+      <c r="F83" s="73" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="17"/>
@@ -21110,10 +21037,9 @@
       <c r="BM83" s="1"/>
       <c r="BO83" s="18"/>
       <c r="BP83" s="19"/>
-      <c r="BQ83" s="20"/>
+      <c r="BQ83" s="21"/>
       <c r="BS83" s="17"/>
       <c r="BT83" s="17"/>
-      <c r="BU83" s="17"/>
       <c r="BV83" s="18"/>
       <c r="BW83" s="19"/>
       <c r="BX83" s="20"/>
@@ -21269,14 +21195,14 @@
       <c r="HR83" s="17"/>
     </row>
     <row r="84" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="71"/>
-      <c r="B84" s="71"/>
-      <c r="C84" s="71"/>
+      <c r="A84" s="74"/>
+      <c r="B84" s="74"/>
+      <c r="C84" s="74"/>
       <c r="D84" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="69"/>
-      <c r="F84" s="69"/>
+      <c r="E84" s="72"/>
+      <c r="F84" s="72"/>
       <c r="G84" s="17"/>
       <c r="H84" s="17"/>
       <c r="I84" s="17"/>
@@ -21331,10 +21257,9 @@
       <c r="BM84" s="1"/>
       <c r="BO84" s="18"/>
       <c r="BP84" s="19"/>
-      <c r="BQ84" s="20"/>
+      <c r="BQ84" s="21"/>
       <c r="BS84" s="17"/>
       <c r="BT84" s="17"/>
-      <c r="BU84" s="17"/>
       <c r="BV84" s="18"/>
       <c r="BW84" s="19"/>
       <c r="BX84" s="20"/>
@@ -21490,20 +21415,20 @@
       <c r="HR84" s="17"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="71"/>
-      <c r="B85" s="72" t="s">
-        <v>167</v>
-      </c>
-      <c r="C85" s="75" t="s">
-        <v>168</v>
+      <c r="A85" s="74"/>
+      <c r="B85" s="75" t="s">
+        <v>165</v>
+      </c>
+      <c r="C85" s="78" t="s">
+        <v>166</v>
       </c>
       <c r="D85" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="69" t="s">
-        <v>169</v>
-      </c>
-      <c r="F85" s="70"/>
+      <c r="E85" s="72" t="s">
+        <v>167</v>
+      </c>
+      <c r="F85" s="73"/>
       <c r="G85" s="17"/>
       <c r="H85" s="17"/>
       <c r="I85" s="17"/>
@@ -21558,10 +21483,9 @@
       <c r="BM85" s="1"/>
       <c r="BO85" s="18"/>
       <c r="BP85" s="19"/>
-      <c r="BQ85" s="20"/>
+      <c r="BQ85" s="21"/>
       <c r="BS85" s="17"/>
       <c r="BT85" s="17"/>
-      <c r="BU85" s="17"/>
       <c r="BV85" s="18"/>
       <c r="BW85" s="19"/>
       <c r="BX85" s="20"/>
@@ -21717,14 +21641,14 @@
       <c r="HR85" s="49"/>
     </row>
     <row r="86" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="71"/>
-      <c r="B86" s="71"/>
-      <c r="C86" s="71"/>
+      <c r="A86" s="74"/>
+      <c r="B86" s="74"/>
+      <c r="C86" s="74"/>
       <c r="D86" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="69"/>
-      <c r="F86" s="69"/>
+      <c r="E86" s="72"/>
+      <c r="F86" s="72"/>
       <c r="G86" s="17"/>
       <c r="H86" s="17"/>
       <c r="I86" s="17"/>
@@ -21779,10 +21703,9 @@
       <c r="BM86" s="1"/>
       <c r="BO86" s="18"/>
       <c r="BP86" s="19"/>
-      <c r="BQ86" s="20"/>
+      <c r="BQ86" s="21"/>
       <c r="BS86" s="17"/>
       <c r="BT86" s="17"/>
-      <c r="BU86" s="17"/>
       <c r="BV86" s="18"/>
       <c r="BW86" s="19"/>
       <c r="BX86" s="20"/>
@@ -22169,22 +22092,22 @@
         <v>40</v>
       </c>
       <c r="B1" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>171</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>43</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22195,19 +22118,19 @@
         <v>97</v>
       </c>
       <c r="C2" s="51" t="s">
+        <v>173</v>
+      </c>
+      <c r="D2" s="51" t="s">
+        <v>174</v>
+      </c>
+      <c r="E2" s="51" t="s">
         <v>175</v>
-      </c>
-      <c r="D2" s="51" t="s">
-        <v>176</v>
-      </c>
-      <c r="E2" s="51" t="s">
-        <v>177</v>
       </c>
       <c r="F2" s="51" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22215,16 +22138,16 @@
         <v>99</v>
       </c>
       <c r="B3" s="51" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="51" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="51" t="s">
+      <c r="E3" s="51" t="s">
         <v>180</v>
-      </c>
-      <c r="D3" s="51" t="s">
-        <v>181</v>
-      </c>
-      <c r="E3" s="51" t="s">
-        <v>182</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>5</v>
@@ -22241,13 +22164,13 @@
         <v>103</v>
       </c>
       <c r="C4" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="E4" s="51" t="s">
         <v>183</v>
-      </c>
-      <c r="D4" s="51" t="s">
-        <v>184</v>
-      </c>
-      <c r="E4" s="51" t="s">
-        <v>185</v>
       </c>
       <c r="F4" s="51" t="s">
         <v>4</v>
@@ -22264,13 +22187,13 @@
         <v>107</v>
       </c>
       <c r="C5" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>185</v>
+      </c>
+      <c r="E5" s="51" t="s">
         <v>186</v>
-      </c>
-      <c r="D5" s="51" t="s">
-        <v>187</v>
-      </c>
-      <c r="E5" s="51" t="s">
-        <v>188</v>
       </c>
       <c r="F5" s="51" t="s">
         <v>7</v>
@@ -22287,13 +22210,13 @@
         <v>110</v>
       </c>
       <c r="C6" s="51" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="51" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="51" t="s">
         <v>189</v>
-      </c>
-      <c r="D6" s="51" t="s">
-        <v>190</v>
-      </c>
-      <c r="E6" s="51" t="s">
-        <v>191</v>
       </c>
       <c r="F6" s="51" t="s">
         <v>4</v>
@@ -22307,22 +22230,22 @@
         <v>113</v>
       </c>
       <c r="B7" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="51" t="s">
         <v>192</v>
       </c>
-      <c r="C7" s="51" t="s">
+      <c r="E7" s="51" t="s">
         <v>193</v>
-      </c>
-      <c r="D7" s="51" t="s">
-        <v>194</v>
-      </c>
-      <c r="E7" s="51" t="s">
-        <v>195</v>
       </c>
       <c r="F7" s="51" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="51" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22330,160 +22253,160 @@
         <v>116</v>
       </c>
       <c r="B8" s="51" t="s">
+        <v>195</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" s="51" t="s">
         <v>197</v>
       </c>
-      <c r="C8" s="51" t="s">
-        <v>198</v>
-      </c>
-      <c r="D8" s="51" t="s">
-        <v>199</v>
-      </c>
       <c r="E8" s="51" t="s">
-        <v>200</v>
+        <v>270</v>
       </c>
       <c r="F8" s="51" t="s">
         <v>6</v>
       </c>
       <c r="G8" s="51" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C9" s="51" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D9" s="51" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E9" s="51" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F9" s="51" t="s">
         <v>4</v>
       </c>
       <c r="G9" s="51" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="52" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C10" s="51" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D10" s="51" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E10" s="51" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F10" s="51" t="s">
         <v>4</v>
       </c>
       <c r="G10" s="51" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C11" s="51" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E11" s="51" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>4</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C12" s="51" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E12" s="51" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="F12" s="51" t="s">
         <v>4</v>
       </c>
       <c r="G12" s="51" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="52" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C13" s="51" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E13" s="51" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F13" s="51" t="s">
         <v>7</v>
       </c>
       <c r="G13" s="51" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C14" s="51" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E14" s="51" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F14" s="51" t="s">
         <v>5</v>
       </c>
       <c r="G14" s="51" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22494,19 +22417,19 @@
         <v>78</v>
       </c>
       <c r="C15" s="51" t="s">
+        <v>217</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>219</v>
+      </c>
+      <c r="F15" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="D15" s="51" t="s">
-        <v>221</v>
-      </c>
-      <c r="E15" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="F15" s="51" t="s">
-        <v>223</v>
-      </c>
       <c r="G15" s="51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22514,22 +22437,22 @@
         <v>80</v>
       </c>
       <c r="B16" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="C16" s="51" t="s">
+        <v>222</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>223</v>
+      </c>
+      <c r="E16" s="51" t="s">
         <v>224</v>
-      </c>
-      <c r="C16" s="51" t="s">
-        <v>225</v>
-      </c>
-      <c r="D16" s="51" t="s">
-        <v>226</v>
-      </c>
-      <c r="E16" s="51" t="s">
-        <v>227</v>
       </c>
       <c r="F16" s="51" t="s">
         <v>3</v>
       </c>
       <c r="G16" s="51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22540,19 +22463,19 @@
         <v>84</v>
       </c>
       <c r="C17" s="51" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F17" s="51" t="s">
         <v>5</v>
       </c>
       <c r="G17" s="51" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -22563,13 +22486,13 @@
         <v>87</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D18" s="51" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E18" s="51" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="F18" s="51" t="s">
         <v>4</v>
@@ -22586,13 +22509,13 @@
         <v>90</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>3</v>
@@ -22606,16 +22529,16 @@
         <v>92</v>
       </c>
       <c r="B20" s="51" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" s="51" t="s">
+        <v>233</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>234</v>
+      </c>
+      <c r="E20" s="51" t="s">
         <v>235</v>
-      </c>
-      <c r="C20" s="51" t="s">
-        <v>236</v>
-      </c>
-      <c r="D20" s="51" t="s">
-        <v>237</v>
-      </c>
-      <c r="E20" s="51" t="s">
-        <v>238</v>
       </c>
       <c r="F20" s="51" t="s">
         <v>5</v>
@@ -22642,12 +22565,12 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="54" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C3" s="55"/>
     </row>
@@ -22655,42 +22578,42 @@
       <c r="A4" s="56"/>
       <c r="B4" s="57"/>
       <c r="C4" s="55" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="56"/>
       <c r="B5" s="58"/>
       <c r="C5" s="55" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="56"/>
       <c r="B6" s="59"/>
       <c r="C6" s="55" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="56"/>
       <c r="B7" s="60"/>
       <c r="C7" s="55" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="56"/>
       <c r="B8" s="61"/>
       <c r="C8" s="55" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="56"/>
       <c r="B9" s="62"/>
       <c r="C9" s="55" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22699,7 +22622,7 @@
     </row>
     <row r="11" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="54" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C11" s="55"/>
     </row>
@@ -22707,21 +22630,21 @@
       <c r="A12" s="56"/>
       <c r="B12" s="63"/>
       <c r="C12" s="55" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="56"/>
       <c r="B13" s="64"/>
       <c r="C13" s="55" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="56"/>
       <c r="B14" s="65"/>
       <c r="C14" s="55" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22730,48 +22653,48 @@
     </row>
     <row r="16" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="54" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C16" s="55"/>
     </row>
     <row r="17" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="56" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C17" s="55" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="56" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C18" s="55" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="56" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C19" s="55" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="56" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C20" s="55" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="56" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C21" s="55" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22780,7 +22703,7 @@
     </row>
     <row r="23" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="54" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C23" s="55"/>
     </row>
@@ -22789,7 +22712,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="55" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22797,7 +22720,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="55" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22805,7 +22728,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="55" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22813,7 +22736,7 @@
         <v>6</v>
       </c>
       <c r="C27" s="55" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22821,7 +22744,7 @@
         <v>7</v>
       </c>
       <c r="C28" s="55" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -22830,16 +22753,16 @@
     </row>
     <row r="30" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="54" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C30" s="55"/>
     </row>
     <row r="31" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="56" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C31" s="55" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made code base more lean regarding training and evaluating model.
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18710F7E-E8DD-4608-B357-988628C4BC57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B4130B-2A6D-45BA-AE40-7A3022AFABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1287,6 +1287,18 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1296,20 +1308,8 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1323,8 +1323,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1628,290 +1628,290 @@
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="84" t="s">
+      <c r="G1" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84" t="s">
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-      <c r="S1" s="84"/>
-      <c r="T1" s="84"/>
-      <c r="U1" s="84" t="s">
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
+      <c r="Q1" s="72"/>
+      <c r="R1" s="72"/>
+      <c r="S1" s="72"/>
+      <c r="T1" s="72"/>
+      <c r="U1" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="84"/>
-      <c r="W1" s="84"/>
-      <c r="X1" s="84"/>
-      <c r="Y1" s="84"/>
-      <c r="Z1" s="84"/>
-      <c r="AA1" s="84"/>
-      <c r="AB1" s="84" t="s">
+      <c r="V1" s="72"/>
+      <c r="W1" s="72"/>
+      <c r="X1" s="72"/>
+      <c r="Y1" s="72"/>
+      <c r="Z1" s="72"/>
+      <c r="AA1" s="72"/>
+      <c r="AB1" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="84"/>
-      <c r="AD1" s="84"/>
-      <c r="AE1" s="84"/>
-      <c r="AF1" s="84"/>
-      <c r="AG1" s="84"/>
-      <c r="AH1" s="84"/>
-      <c r="AI1" s="84" t="s">
+      <c r="AC1" s="72"/>
+      <c r="AD1" s="72"/>
+      <c r="AE1" s="72"/>
+      <c r="AF1" s="72"/>
+      <c r="AG1" s="72"/>
+      <c r="AH1" s="72"/>
+      <c r="AI1" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="AJ1" s="84"/>
-      <c r="AK1" s="84"/>
-      <c r="AL1" s="84"/>
-      <c r="AM1" s="84"/>
-      <c r="AN1" s="84"/>
-      <c r="AO1" s="84"/>
-      <c r="AP1" s="84" t="s">
+      <c r="AJ1" s="72"/>
+      <c r="AK1" s="72"/>
+      <c r="AL1" s="72"/>
+      <c r="AM1" s="72"/>
+      <c r="AN1" s="72"/>
+      <c r="AO1" s="72"/>
+      <c r="AP1" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="AQ1" s="84"/>
-      <c r="AR1" s="84"/>
-      <c r="AS1" s="84"/>
-      <c r="AT1" s="84"/>
-      <c r="AU1" s="84"/>
-      <c r="AV1" s="84"/>
-      <c r="AW1" s="84" t="s">
+      <c r="AQ1" s="72"/>
+      <c r="AR1" s="72"/>
+      <c r="AS1" s="72"/>
+      <c r="AT1" s="72"/>
+      <c r="AU1" s="72"/>
+      <c r="AV1" s="72"/>
+      <c r="AW1" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="AX1" s="84"/>
-      <c r="AY1" s="84"/>
-      <c r="AZ1" s="84"/>
-      <c r="BA1" s="84"/>
-      <c r="BB1" s="84"/>
-      <c r="BC1" s="84"/>
-      <c r="BD1" s="84" t="s">
+      <c r="AX1" s="72"/>
+      <c r="AY1" s="72"/>
+      <c r="AZ1" s="72"/>
+      <c r="BA1" s="72"/>
+      <c r="BB1" s="72"/>
+      <c r="BC1" s="72"/>
+      <c r="BD1" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="BE1" s="84"/>
-      <c r="BF1" s="84"/>
-      <c r="BG1" s="84"/>
-      <c r="BH1" s="84"/>
-      <c r="BI1" s="84"/>
-      <c r="BJ1" s="84"/>
-      <c r="BK1" s="84" t="s">
+      <c r="BE1" s="72"/>
+      <c r="BF1" s="72"/>
+      <c r="BG1" s="72"/>
+      <c r="BH1" s="72"/>
+      <c r="BI1" s="72"/>
+      <c r="BJ1" s="72"/>
+      <c r="BK1" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="84"/>
-      <c r="BM1" s="84"/>
-      <c r="BN1" s="84"/>
-      <c r="BO1" s="84"/>
-      <c r="BP1" s="84"/>
-      <c r="BQ1" s="84"/>
-      <c r="BR1" s="84" t="s">
+      <c r="BL1" s="72"/>
+      <c r="BM1" s="72"/>
+      <c r="BN1" s="72"/>
+      <c r="BO1" s="72"/>
+      <c r="BP1" s="72"/>
+      <c r="BQ1" s="72"/>
+      <c r="BR1" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="BS1" s="84"/>
-      <c r="BT1" s="84"/>
-      <c r="BU1" s="84"/>
-      <c r="BV1" s="84"/>
-      <c r="BW1" s="84"/>
-      <c r="BX1" s="84"/>
-      <c r="BY1" s="84" t="s">
+      <c r="BS1" s="72"/>
+      <c r="BT1" s="72"/>
+      <c r="BU1" s="72"/>
+      <c r="BV1" s="72"/>
+      <c r="BW1" s="72"/>
+      <c r="BX1" s="72"/>
+      <c r="BY1" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="BZ1" s="84"/>
-      <c r="CA1" s="84"/>
-      <c r="CB1" s="84"/>
-      <c r="CC1" s="84"/>
-      <c r="CD1" s="84"/>
-      <c r="CE1" s="84"/>
-      <c r="CF1" s="84" t="s">
+      <c r="BZ1" s="72"/>
+      <c r="CA1" s="72"/>
+      <c r="CB1" s="72"/>
+      <c r="CC1" s="72"/>
+      <c r="CD1" s="72"/>
+      <c r="CE1" s="72"/>
+      <c r="CF1" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="CG1" s="84"/>
-      <c r="CH1" s="84"/>
-      <c r="CI1" s="84"/>
-      <c r="CJ1" s="84"/>
-      <c r="CK1" s="84"/>
-      <c r="CL1" s="84"/>
-      <c r="CM1" s="84" t="s">
+      <c r="CG1" s="72"/>
+      <c r="CH1" s="72"/>
+      <c r="CI1" s="72"/>
+      <c r="CJ1" s="72"/>
+      <c r="CK1" s="72"/>
+      <c r="CL1" s="72"/>
+      <c r="CM1" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="CN1" s="84"/>
-      <c r="CO1" s="84"/>
-      <c r="CP1" s="84"/>
-      <c r="CQ1" s="84"/>
-      <c r="CR1" s="84"/>
-      <c r="CS1" s="84"/>
-      <c r="CT1" s="84" t="s">
+      <c r="CN1" s="72"/>
+      <c r="CO1" s="72"/>
+      <c r="CP1" s="72"/>
+      <c r="CQ1" s="72"/>
+      <c r="CR1" s="72"/>
+      <c r="CS1" s="72"/>
+      <c r="CT1" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="CU1" s="84"/>
-      <c r="CV1" s="84"/>
-      <c r="CW1" s="84"/>
-      <c r="CX1" s="84"/>
-      <c r="CY1" s="84"/>
-      <c r="CZ1" s="84"/>
-      <c r="DA1" s="84" t="s">
+      <c r="CU1" s="72"/>
+      <c r="CV1" s="72"/>
+      <c r="CW1" s="72"/>
+      <c r="CX1" s="72"/>
+      <c r="CY1" s="72"/>
+      <c r="CZ1" s="72"/>
+      <c r="DA1" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="DB1" s="84"/>
-      <c r="DC1" s="84"/>
-      <c r="DD1" s="84"/>
-      <c r="DE1" s="84"/>
-      <c r="DF1" s="84"/>
-      <c r="DG1" s="84"/>
-      <c r="DH1" s="84" t="s">
+      <c r="DB1" s="72"/>
+      <c r="DC1" s="72"/>
+      <c r="DD1" s="72"/>
+      <c r="DE1" s="72"/>
+      <c r="DF1" s="72"/>
+      <c r="DG1" s="72"/>
+      <c r="DH1" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="DI1" s="84"/>
-      <c r="DJ1" s="84"/>
-      <c r="DK1" s="84"/>
-      <c r="DL1" s="84"/>
-      <c r="DM1" s="84"/>
-      <c r="DN1" s="84"/>
-      <c r="DO1" s="84" t="s">
+      <c r="DI1" s="72"/>
+      <c r="DJ1" s="72"/>
+      <c r="DK1" s="72"/>
+      <c r="DL1" s="72"/>
+      <c r="DM1" s="72"/>
+      <c r="DN1" s="72"/>
+      <c r="DO1" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="DP1" s="84"/>
-      <c r="DQ1" s="84"/>
-      <c r="DR1" s="84"/>
-      <c r="DS1" s="84"/>
-      <c r="DT1" s="84"/>
-      <c r="DU1" s="84"/>
-      <c r="DV1" s="84" t="s">
+      <c r="DP1" s="72"/>
+      <c r="DQ1" s="72"/>
+      <c r="DR1" s="72"/>
+      <c r="DS1" s="72"/>
+      <c r="DT1" s="72"/>
+      <c r="DU1" s="72"/>
+      <c r="DV1" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="DW1" s="84"/>
-      <c r="DX1" s="84"/>
-      <c r="DY1" s="84"/>
-      <c r="DZ1" s="84"/>
-      <c r="EA1" s="84"/>
-      <c r="EB1" s="84"/>
-      <c r="EC1" s="84" t="s">
+      <c r="DW1" s="72"/>
+      <c r="DX1" s="72"/>
+      <c r="DY1" s="72"/>
+      <c r="DZ1" s="72"/>
+      <c r="EA1" s="72"/>
+      <c r="EB1" s="72"/>
+      <c r="EC1" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="ED1" s="84"/>
-      <c r="EE1" s="84"/>
-      <c r="EF1" s="84"/>
-      <c r="EG1" s="84"/>
-      <c r="EH1" s="84"/>
-      <c r="EI1" s="84"/>
-      <c r="EJ1" s="84" t="s">
+      <c r="ED1" s="72"/>
+      <c r="EE1" s="72"/>
+      <c r="EF1" s="72"/>
+      <c r="EG1" s="72"/>
+      <c r="EH1" s="72"/>
+      <c r="EI1" s="72"/>
+      <c r="EJ1" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="EK1" s="84"/>
-      <c r="EL1" s="84"/>
-      <c r="EM1" s="84"/>
-      <c r="EN1" s="84"/>
-      <c r="EO1" s="84"/>
-      <c r="EP1" s="84"/>
-      <c r="EQ1" s="84" t="s">
+      <c r="EK1" s="72"/>
+      <c r="EL1" s="72"/>
+      <c r="EM1" s="72"/>
+      <c r="EN1" s="72"/>
+      <c r="EO1" s="72"/>
+      <c r="EP1" s="72"/>
+      <c r="EQ1" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="ER1" s="84"/>
-      <c r="ES1" s="84"/>
-      <c r="ET1" s="84"/>
-      <c r="EU1" s="84"/>
-      <c r="EV1" s="84"/>
-      <c r="EW1" s="84"/>
-      <c r="EX1" s="84" t="s">
+      <c r="ER1" s="72"/>
+      <c r="ES1" s="72"/>
+      <c r="ET1" s="72"/>
+      <c r="EU1" s="72"/>
+      <c r="EV1" s="72"/>
+      <c r="EW1" s="72"/>
+      <c r="EX1" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="EY1" s="84"/>
-      <c r="EZ1" s="84"/>
-      <c r="FA1" s="84"/>
-      <c r="FB1" s="84"/>
-      <c r="FC1" s="84"/>
-      <c r="FD1" s="84"/>
-      <c r="FE1" s="84" t="s">
+      <c r="EY1" s="72"/>
+      <c r="EZ1" s="72"/>
+      <c r="FA1" s="72"/>
+      <c r="FB1" s="72"/>
+      <c r="FC1" s="72"/>
+      <c r="FD1" s="72"/>
+      <c r="FE1" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="FF1" s="84"/>
-      <c r="FG1" s="84"/>
-      <c r="FH1" s="84"/>
-      <c r="FI1" s="84"/>
-      <c r="FJ1" s="84"/>
-      <c r="FK1" s="84"/>
-      <c r="FL1" s="84" t="s">
+      <c r="FF1" s="72"/>
+      <c r="FG1" s="72"/>
+      <c r="FH1" s="72"/>
+      <c r="FI1" s="72"/>
+      <c r="FJ1" s="72"/>
+      <c r="FK1" s="72"/>
+      <c r="FL1" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="FM1" s="84"/>
-      <c r="FN1" s="84"/>
-      <c r="FO1" s="84"/>
-      <c r="FP1" s="84"/>
-      <c r="FQ1" s="84"/>
-      <c r="FR1" s="84"/>
-      <c r="FS1" s="84" t="s">
+      <c r="FM1" s="72"/>
+      <c r="FN1" s="72"/>
+      <c r="FO1" s="72"/>
+      <c r="FP1" s="72"/>
+      <c r="FQ1" s="72"/>
+      <c r="FR1" s="72"/>
+      <c r="FS1" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="FT1" s="84"/>
-      <c r="FU1" s="84"/>
-      <c r="FV1" s="84"/>
-      <c r="FW1" s="84"/>
-      <c r="FX1" s="84"/>
-      <c r="FY1" s="84"/>
-      <c r="FZ1" s="84" t="s">
+      <c r="FT1" s="72"/>
+      <c r="FU1" s="72"/>
+      <c r="FV1" s="72"/>
+      <c r="FW1" s="72"/>
+      <c r="FX1" s="72"/>
+      <c r="FY1" s="72"/>
+      <c r="FZ1" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="GA1" s="84"/>
-      <c r="GB1" s="84"/>
-      <c r="GC1" s="84"/>
-      <c r="GD1" s="84"/>
-      <c r="GE1" s="84"/>
-      <c r="GF1" s="84"/>
-      <c r="GG1" s="84" t="s">
+      <c r="GA1" s="72"/>
+      <c r="GB1" s="72"/>
+      <c r="GC1" s="72"/>
+      <c r="GD1" s="72"/>
+      <c r="GE1" s="72"/>
+      <c r="GF1" s="72"/>
+      <c r="GG1" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="GH1" s="84"/>
-      <c r="GI1" s="84"/>
-      <c r="GJ1" s="84"/>
-      <c r="GK1" s="84"/>
-      <c r="GL1" s="84"/>
-      <c r="GM1" s="84"/>
-      <c r="GN1" s="84" t="s">
+      <c r="GH1" s="72"/>
+      <c r="GI1" s="72"/>
+      <c r="GJ1" s="72"/>
+      <c r="GK1" s="72"/>
+      <c r="GL1" s="72"/>
+      <c r="GM1" s="72"/>
+      <c r="GN1" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="GO1" s="84"/>
-      <c r="GP1" s="84"/>
-      <c r="GQ1" s="84"/>
-      <c r="GR1" s="84"/>
-      <c r="GS1" s="84"/>
-      <c r="GT1" s="84"/>
-      <c r="GU1" s="84" t="s">
+      <c r="GO1" s="72"/>
+      <c r="GP1" s="72"/>
+      <c r="GQ1" s="72"/>
+      <c r="GR1" s="72"/>
+      <c r="GS1" s="72"/>
+      <c r="GT1" s="72"/>
+      <c r="GU1" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="GV1" s="84"/>
-      <c r="GW1" s="84"/>
-      <c r="GX1" s="84"/>
-      <c r="GY1" s="84"/>
-      <c r="GZ1" s="84"/>
-      <c r="HA1" s="84"/>
-      <c r="HB1" s="84" t="s">
+      <c r="GV1" s="72"/>
+      <c r="GW1" s="72"/>
+      <c r="GX1" s="72"/>
+      <c r="GY1" s="72"/>
+      <c r="GZ1" s="72"/>
+      <c r="HA1" s="72"/>
+      <c r="HB1" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="HC1" s="84"/>
-      <c r="HD1" s="84"/>
-      <c r="HE1" s="84"/>
-      <c r="HF1" s="84"/>
-      <c r="HG1" s="84"/>
-      <c r="HH1" s="84"/>
-      <c r="HI1" s="84" t="s">
+      <c r="HC1" s="72"/>
+      <c r="HD1" s="72"/>
+      <c r="HE1" s="72"/>
+      <c r="HF1" s="72"/>
+      <c r="HG1" s="72"/>
+      <c r="HH1" s="72"/>
+      <c r="HI1" s="72" t="s">
         <v>31</v>
       </c>
-      <c r="HJ1" s="84"/>
-      <c r="HK1" s="84"/>
-      <c r="HL1" s="84"/>
-      <c r="HM1" s="84"/>
-      <c r="HN1" s="84"/>
-      <c r="HO1" s="84"/>
-      <c r="HP1" s="84" t="s">
+      <c r="HJ1" s="72"/>
+      <c r="HK1" s="72"/>
+      <c r="HL1" s="72"/>
+      <c r="HM1" s="72"/>
+      <c r="HN1" s="72"/>
+      <c r="HO1" s="72"/>
+      <c r="HP1" s="72" t="s">
         <v>32</v>
       </c>
-      <c r="HQ1" s="84"/>
-      <c r="HR1" s="84"/>
+      <c r="HQ1" s="72"/>
+      <c r="HR1" s="72"/>
     </row>
     <row r="2" spans="1:226" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3" t="s">
@@ -3482,20 +3482,20 @@
       <c r="HR4" s="12"/>
     </row>
     <row r="5" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="77" t="s">
+      <c r="B5" s="74"/>
+      <c r="C5" s="75" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="72" t="s">
+      <c r="E5" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="73"/>
+      <c r="F5" s="77"/>
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
       <c r="I5" s="17"/>
@@ -3708,14 +3708,14 @@
       <c r="HR5" s="17"/>
     </row>
     <row r="6" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="79"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="79"/>
+      <c r="A6" s="73"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="72"/>
-      <c r="F6" s="72"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
       <c r="G6" s="17"/>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
@@ -3928,18 +3928,18 @@
       <c r="HR6" s="17"/>
     </row>
     <row r="7" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="79"/>
-      <c r="B7" s="75"/>
-      <c r="C7" s="77" t="s">
+      <c r="A7" s="73"/>
+      <c r="B7" s="74"/>
+      <c r="C7" s="75" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="72" t="s">
+      <c r="E7" s="76" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="73"/>
+      <c r="F7" s="77"/>
       <c r="G7" s="17"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -4152,14 +4152,14 @@
       <c r="HR7" s="17"/>
     </row>
     <row r="8" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
+      <c r="A8" s="73"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="73"/>
       <c r="D8" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="72"/>
-      <c r="F8" s="72"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
@@ -4372,18 +4372,18 @@
       <c r="HR8" s="17"/>
     </row>
     <row r="9" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="79"/>
-      <c r="B9" s="75"/>
-      <c r="C9" s="77" t="s">
+      <c r="A9" s="73"/>
+      <c r="B9" s="74"/>
+      <c r="C9" s="75" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="72" t="s">
+      <c r="E9" s="76" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="73"/>
+      <c r="F9" s="77"/>
       <c r="G9" s="17"/>
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
@@ -4596,14 +4596,14 @@
       <c r="HR9" s="17"/>
     </row>
     <row r="10" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="79"/>
-      <c r="B10" s="79"/>
-      <c r="C10" s="79"/>
+      <c r="A10" s="73"/>
+      <c r="B10" s="73"/>
+      <c r="C10" s="73"/>
       <c r="D10" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="72"/>
-      <c r="F10" s="72"/>
+      <c r="E10" s="76"/>
+      <c r="F10" s="76"/>
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -4816,18 +4816,18 @@
       <c r="HR10" s="17"/>
     </row>
     <row r="11" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="79"/>
-      <c r="B11" s="75"/>
-      <c r="C11" s="77" t="s">
+      <c r="A11" s="73"/>
+      <c r="B11" s="74"/>
+      <c r="C11" s="75" t="s">
         <v>53</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="72" t="s">
+      <c r="E11" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="73"/>
+      <c r="F11" s="77"/>
       <c r="G11" s="17"/>
       <c r="H11" s="17"/>
       <c r="I11" s="17"/>
@@ -5040,14 +5040,14 @@
       <c r="HR11" s="17"/>
     </row>
     <row r="12" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="79"/>
-      <c r="B12" s="79"/>
-      <c r="C12" s="79"/>
+      <c r="A12" s="73"/>
+      <c r="B12" s="73"/>
+      <c r="C12" s="73"/>
       <c r="D12" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -5260,18 +5260,18 @@
       <c r="HR12" s="17"/>
     </row>
     <row r="13" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="79"/>
-      <c r="B13" s="75"/>
-      <c r="C13" s="77" t="s">
+      <c r="A13" s="73"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="75" t="s">
         <v>55</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="72" t="s">
+      <c r="E13" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="73"/>
+      <c r="F13" s="77"/>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
       <c r="I13" s="17"/>
@@ -5484,14 +5484,14 @@
       <c r="HR13" s="17"/>
     </row>
     <row r="14" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="79"/>
-      <c r="B14" s="79"/>
-      <c r="C14" s="79"/>
+      <c r="A14" s="73"/>
+      <c r="B14" s="73"/>
+      <c r="C14" s="73"/>
       <c r="D14" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
+      <c r="E14" s="76"/>
+      <c r="F14" s="76"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -5704,18 +5704,18 @@
       <c r="HR14" s="17"/>
     </row>
     <row r="15" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="79"/>
-      <c r="B15" s="75"/>
-      <c r="C15" s="77" t="s">
+      <c r="A15" s="73"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="75" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="72" t="s">
+      <c r="E15" s="76" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="73"/>
+      <c r="F15" s="77"/>
       <c r="G15" s="17"/>
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
@@ -5928,14 +5928,14 @@
       <c r="HR15" s="17"/>
     </row>
     <row r="16" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="79"/>
-      <c r="B16" s="79"/>
-      <c r="C16" s="79"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="73"/>
       <c r="D16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -6148,18 +6148,18 @@
       <c r="HR16" s="17"/>
     </row>
     <row r="17" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="79"/>
-      <c r="B17" s="75"/>
-      <c r="C17" s="77" t="s">
+      <c r="A17" s="73"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="75" t="s">
         <v>59</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="72" t="s">
+      <c r="E17" s="76" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="73"/>
+      <c r="F17" s="77"/>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
@@ -6372,14 +6372,14 @@
       <c r="HR17" s="17"/>
     </row>
     <row r="18" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="79"/>
-      <c r="B18" s="79"/>
-      <c r="C18" s="79"/>
+      <c r="A18" s="73"/>
+      <c r="B18" s="73"/>
+      <c r="C18" s="73"/>
       <c r="D18" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -6592,18 +6592,18 @@
       <c r="HR18" s="17"/>
     </row>
     <row r="19" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="79"/>
-      <c r="B19" s="75"/>
-      <c r="C19" s="77" t="s">
+      <c r="A19" s="73"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="75" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="72" t="s">
+      <c r="E19" s="76" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="73"/>
+      <c r="F19" s="77"/>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
@@ -6816,14 +6816,14 @@
       <c r="HR19" s="17"/>
     </row>
     <row r="20" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="79"/>
-      <c r="B20" s="79"/>
-      <c r="C20" s="79"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="73"/>
+      <c r="C20" s="73"/>
       <c r="D20" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="72"/>
-      <c r="F20" s="72"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
@@ -7036,7 +7036,7 @@
       <c r="HR20" s="17"/>
     </row>
     <row r="21" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="79"/>
+      <c r="A21" s="73"/>
       <c r="B21" s="80"/>
       <c r="C21" s="81" t="s">
         <v>63</v>
@@ -7260,9 +7260,9 @@
       <c r="HR21" s="17"/>
     </row>
     <row r="22" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="79"/>
-      <c r="B22" s="79"/>
-      <c r="C22" s="79"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="73"/>
       <c r="D22" s="29" t="s">
         <v>48</v>
       </c>
@@ -7481,22 +7481,22 @@
       <c r="HR22" s="30"/>
     </row>
     <row r="23" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="78" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="75" t="s">
+      <c r="B23" s="74" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="77" t="s">
+      <c r="C23" s="75" t="s">
         <v>67</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="72" t="s">
+      <c r="E23" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="73" t="s">
+      <c r="F23" s="77" t="s">
         <v>69</v>
       </c>
       <c r="G23" s="17"/>
@@ -7716,14 +7716,14 @@
       <c r="HR23" s="17"/>
     </row>
     <row r="24" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="74"/>
-      <c r="B24" s="74"/>
-      <c r="C24" s="74"/>
+      <c r="A24" s="78"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="78"/>
       <c r="D24" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="72"/>
-      <c r="F24" s="72"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
@@ -7940,20 +7940,20 @@
       <c r="HR24" s="17"/>
     </row>
     <row r="25" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="74"/>
-      <c r="B25" s="75" t="s">
+      <c r="A25" s="78"/>
+      <c r="B25" s="74" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="77" t="s">
+      <c r="C25" s="75" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="72" t="s">
+      <c r="E25" s="76" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="73" t="s">
+      <c r="F25" s="77" t="s">
         <v>69</v>
       </c>
       <c r="G25" s="17"/>
@@ -8162,14 +8162,14 @@
       <c r="HS25" s="17"/>
     </row>
     <row r="26" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="74"/>
-      <c r="B26" s="74"/>
-      <c r="C26" s="74"/>
+      <c r="A26" s="78"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
       <c r="D26" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="72"/>
-      <c r="F26" s="72"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26" s="17"/>
@@ -8382,20 +8382,20 @@
       <c r="HR26" s="17"/>
     </row>
     <row r="27" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="74"/>
-      <c r="B27" s="75" t="s">
+      <c r="A27" s="78"/>
+      <c r="B27" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="78" t="s">
+      <c r="C27" s="79" t="s">
         <v>74</v>
       </c>
       <c r="D27" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="72" t="s">
+      <c r="E27" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="73"/>
+      <c r="F27" s="77"/>
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -8608,14 +8608,14 @@
       <c r="HR27" s="17"/>
     </row>
     <row r="28" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="74"/>
-      <c r="B28" s="74"/>
-      <c r="C28" s="74"/>
+      <c r="A28" s="78"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
       <c r="D28" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="72"/>
-      <c r="F28" s="72"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
       <c r="G28" s="17"/>
       <c r="H28" s="17"/>
       <c r="I28" s="17"/>
@@ -8828,22 +8828,22 @@
       <c r="HR28" s="17"/>
     </row>
     <row r="29" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="74" t="s">
+      <c r="A29" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="75" t="s">
+      <c r="B29" s="74" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="77" t="s">
+      <c r="C29" s="75" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="72" t="s">
+      <c r="E29" s="76" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="73" t="s">
+      <c r="F29" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="17"/>
@@ -9057,14 +9057,14 @@
       <c r="HR29" s="17"/>
     </row>
     <row r="30" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="74"/>
-      <c r="B30" s="74"/>
-      <c r="C30" s="74"/>
+      <c r="A30" s="78"/>
+      <c r="B30" s="78"/>
+      <c r="C30" s="78"/>
       <c r="D30" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="72"/>
-      <c r="F30" s="72"/>
+      <c r="E30" s="76"/>
+      <c r="F30" s="76"/>
       <c r="G30" s="17"/>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
@@ -9277,20 +9277,20 @@
       <c r="HR30" s="17"/>
     </row>
     <row r="31" spans="1:227" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="74"/>
-      <c r="B31" s="75" t="s">
+      <c r="A31" s="78"/>
+      <c r="B31" s="74" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="77" t="s">
+      <c r="C31" s="75" t="s">
         <v>81</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="72" t="s">
+      <c r="E31" s="76" t="s">
         <v>82</v>
       </c>
-      <c r="F31" s="73" t="s">
+      <c r="F31" s="77" t="s">
         <v>3</v>
       </c>
       <c r="G31" s="17"/>
@@ -9505,14 +9505,14 @@
       <c r="HR31" s="17"/>
     </row>
     <row r="32" spans="1:227" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="74"/>
-      <c r="B32" s="74"/>
-      <c r="C32" s="74"/>
+      <c r="A32" s="78"/>
+      <c r="B32" s="78"/>
+      <c r="C32" s="78"/>
       <c r="D32" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E32" s="72"/>
-      <c r="F32" s="72"/>
+      <c r="E32" s="76"/>
+      <c r="F32" s="76"/>
       <c r="G32" s="17"/>
       <c r="H32" s="17"/>
       <c r="I32" s="17"/>
@@ -9725,20 +9725,20 @@
       <c r="HR32" s="17"/>
     </row>
     <row r="33" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="74"/>
-      <c r="B33" s="75" t="s">
+      <c r="A33" s="78"/>
+      <c r="B33" s="74" t="s">
         <v>83</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="75" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E33" s="72" t="s">
+      <c r="E33" s="76" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="73" t="s">
+      <c r="F33" s="77" t="s">
         <v>5</v>
       </c>
       <c r="G33" s="17"/>
@@ -9953,14 +9953,14 @@
       <c r="HR33" s="17"/>
     </row>
     <row r="34" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="74"/>
-      <c r="B34" s="74"/>
-      <c r="C34" s="74"/>
+      <c r="A34" s="78"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="78"/>
       <c r="D34" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="72"/>
-      <c r="F34" s="72"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
@@ -10173,20 +10173,20 @@
       <c r="HR34" s="17"/>
     </row>
     <row r="35" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="74"/>
-      <c r="B35" s="75" t="s">
+      <c r="A35" s="78"/>
+      <c r="B35" s="74" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="75" t="s">
         <v>87</v>
       </c>
       <c r="D35" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="72" t="s">
+      <c r="E35" s="76" t="s">
         <v>88</v>
       </c>
-      <c r="F35" s="73" t="s">
+      <c r="F35" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="17"/>
@@ -10402,14 +10402,14 @@
       <c r="HR35" s="17"/>
     </row>
     <row r="36" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="74"/>
-      <c r="B36" s="74"/>
-      <c r="C36" s="74"/>
+      <c r="A36" s="78"/>
+      <c r="B36" s="78"/>
+      <c r="C36" s="78"/>
       <c r="D36" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
       <c r="G36" s="17"/>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
@@ -10623,20 +10623,20 @@
       <c r="HR36" s="17"/>
     </row>
     <row r="37" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="74"/>
-      <c r="B37" s="75" t="s">
+      <c r="A37" s="78"/>
+      <c r="B37" s="74" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="75" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="72" t="s">
+      <c r="E37" s="76" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="73" t="s">
+      <c r="F37" s="77" t="s">
         <v>3</v>
       </c>
       <c r="G37" s="17"/>
@@ -10851,14 +10851,14 @@
       <c r="HR37" s="17"/>
     </row>
     <row r="38" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="74"/>
-      <c r="B38" s="74"/>
-      <c r="C38" s="74"/>
+      <c r="A38" s="78"/>
+      <c r="B38" s="78"/>
+      <c r="C38" s="78"/>
       <c r="D38" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="72"/>
-      <c r="F38" s="72"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
       <c r="G38" s="17"/>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
@@ -11071,20 +11071,20 @@
       <c r="HR38" s="17"/>
     </row>
     <row r="39" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="74"/>
-      <c r="B39" s="75" t="s">
+      <c r="A39" s="78"/>
+      <c r="B39" s="74" t="s">
         <v>92</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="75" t="s">
         <v>93</v>
       </c>
       <c r="D39" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="72" t="s">
+      <c r="E39" s="76" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="73" t="s">
+      <c r="F39" s="77" t="s">
         <v>5</v>
       </c>
       <c r="G39" s="17"/>
@@ -11301,14 +11301,14 @@
       <c r="HR39" s="17"/>
     </row>
     <row r="40" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="74"/>
-      <c r="B40" s="74"/>
-      <c r="C40" s="74"/>
+      <c r="A40" s="78"/>
+      <c r="B40" s="78"/>
+      <c r="C40" s="78"/>
       <c r="D40" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E40" s="72"/>
-      <c r="F40" s="72"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
       <c r="G40" s="17"/>
       <c r="H40" s="17"/>
       <c r="I40" s="17"/>
@@ -11522,22 +11522,22 @@
       <c r="HR40" s="17"/>
     </row>
     <row r="41" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="74" t="s">
+      <c r="A41" s="78" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="75" t="s">
+      <c r="B41" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="75" t="s">
         <v>97</v>
       </c>
       <c r="D41" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E41" s="72" t="s">
+      <c r="E41" s="76" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="73" t="s">
+      <c r="F41" s="77" t="s">
         <v>5</v>
       </c>
       <c r="G41" s="17"/>
@@ -11752,14 +11752,14 @@
       <c r="HR41" s="17"/>
     </row>
     <row r="42" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="74"/>
-      <c r="B42" s="74"/>
-      <c r="C42" s="74"/>
+      <c r="A42" s="78"/>
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
       <c r="D42" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="72"/>
-      <c r="F42" s="72"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
       <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
@@ -11972,20 +11972,20 @@
       <c r="HR42" s="17"/>
     </row>
     <row r="43" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="74"/>
-      <c r="B43" s="75" t="s">
+      <c r="A43" s="78"/>
+      <c r="B43" s="74" t="s">
         <v>99</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="75" t="s">
         <v>100</v>
       </c>
       <c r="D43" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E43" s="72" t="s">
+      <c r="E43" s="76" t="s">
         <v>101</v>
       </c>
-      <c r="F43" s="73" t="s">
+      <c r="F43" s="77" t="s">
         <v>5</v>
       </c>
       <c r="G43" s="17"/>
@@ -12199,14 +12199,14 @@
       <c r="HR43" s="17"/>
     </row>
     <row r="44" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="74"/>
-      <c r="B44" s="74"/>
-      <c r="C44" s="74"/>
+      <c r="A44" s="78"/>
+      <c r="B44" s="78"/>
+      <c r="C44" s="78"/>
       <c r="D44" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="72"/>
-      <c r="F44" s="72"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
       <c r="G44" s="17"/>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
@@ -12421,20 +12421,20 @@
       <c r="HR44" s="17"/>
     </row>
     <row r="45" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="74"/>
-      <c r="B45" s="75" t="s">
+      <c r="A45" s="78"/>
+      <c r="B45" s="74" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="77" t="s">
+      <c r="C45" s="75" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="72" t="s">
+      <c r="E45" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="F45" s="73" t="s">
+      <c r="F45" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="17"/>
@@ -12649,14 +12649,14 @@
       <c r="HR45" s="17"/>
     </row>
     <row r="46" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="74"/>
-      <c r="B46" s="74"/>
-      <c r="C46" s="74"/>
+      <c r="A46" s="78"/>
+      <c r="B46" s="78"/>
+      <c r="C46" s="78"/>
       <c r="D46" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E46" s="72"/>
-      <c r="F46" s="72"/>
+      <c r="E46" s="76"/>
+      <c r="F46" s="76"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
@@ -12870,22 +12870,22 @@
       <c r="HR46" s="17"/>
     </row>
     <row r="47" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="74" t="s">
+      <c r="A47" s="78" t="s">
         <v>105</v>
       </c>
-      <c r="B47" s="75" t="s">
+      <c r="B47" s="74" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="77" t="s">
+      <c r="C47" s="75" t="s">
         <v>107</v>
       </c>
       <c r="D47" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="72" t="s">
+      <c r="E47" s="76" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="73" t="s">
+      <c r="F47" s="77" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="17"/>
@@ -13103,14 +13103,14 @@
       <c r="HR47" s="17"/>
     </row>
     <row r="48" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="74"/>
-      <c r="B48" s="74"/>
-      <c r="C48" s="74"/>
+      <c r="A48" s="78"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
       <c r="D48" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E48" s="72"/>
-      <c r="F48" s="72"/>
+      <c r="E48" s="76"/>
+      <c r="F48" s="76"/>
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
@@ -13325,20 +13325,20 @@
       <c r="HR48" s="17"/>
     </row>
     <row r="49" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="74"/>
-      <c r="B49" s="75" t="s">
+      <c r="A49" s="78"/>
+      <c r="B49" s="74" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="77" t="s">
+      <c r="C49" s="75" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E49" s="72" t="s">
+      <c r="E49" s="76" t="s">
         <v>111</v>
       </c>
-      <c r="F49" s="73" t="s">
+      <c r="F49" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="17"/>
@@ -13554,14 +13554,14 @@
       <c r="HR49" s="17"/>
     </row>
     <row r="50" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="74"/>
-      <c r="B50" s="74"/>
-      <c r="C50" s="74"/>
+      <c r="A50" s="78"/>
+      <c r="B50" s="78"/>
+      <c r="C50" s="78"/>
       <c r="D50" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E50" s="72"/>
-      <c r="F50" s="72"/>
+      <c r="E50" s="76"/>
+      <c r="F50" s="76"/>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
@@ -13775,22 +13775,22 @@
       <c r="HR50" s="17"/>
     </row>
     <row r="51" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="74" t="s">
+      <c r="A51" s="78" t="s">
         <v>112</v>
       </c>
-      <c r="B51" s="75" t="s">
+      <c r="B51" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="77" t="s">
+      <c r="C51" s="75" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="72" t="s">
+      <c r="E51" s="76" t="s">
         <v>115</v>
       </c>
-      <c r="F51" s="73" t="s">
+      <c r="F51" s="77" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="17"/>
@@ -14006,14 +14006,14 @@
       <c r="HR51" s="17"/>
     </row>
     <row r="52" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="74"/>
-      <c r="B52" s="74"/>
-      <c r="C52" s="74"/>
+      <c r="A52" s="78"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="78"/>
       <c r="D52" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E52" s="72"/>
-      <c r="F52" s="72"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="76"/>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
@@ -14071,6 +14071,7 @@
       <c r="BQ52" s="21"/>
       <c r="BS52" s="70"/>
       <c r="BT52" s="70"/>
+      <c r="BU52" s="70"/>
       <c r="BV52" s="18"/>
       <c r="BW52" s="19"/>
       <c r="BX52" s="20"/>
@@ -14226,20 +14227,20 @@
       <c r="HR52" s="17"/>
     </row>
     <row r="53" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="74"/>
-      <c r="B53" s="75" t="s">
+      <c r="A53" s="78"/>
+      <c r="B53" s="74" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="77" t="s">
+      <c r="C53" s="75" t="s">
         <v>268</v>
       </c>
       <c r="D53" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="72" t="s">
+      <c r="E53" s="76" t="s">
         <v>269</v>
       </c>
-      <c r="F53" s="73" t="s">
+      <c r="F53" s="77" t="s">
         <v>6</v>
       </c>
       <c r="G53" s="17"/>
@@ -14454,14 +14455,14 @@
       <c r="HR53" s="17"/>
     </row>
     <row r="54" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="74"/>
-      <c r="B54" s="74"/>
-      <c r="C54" s="74"/>
+      <c r="A54" s="78"/>
+      <c r="B54" s="78"/>
+      <c r="C54" s="78"/>
       <c r="D54" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E54" s="72"/>
-      <c r="F54" s="72"/>
+      <c r="E54" s="76"/>
+      <c r="F54" s="76"/>
       <c r="G54" s="17"/>
       <c r="H54" s="17"/>
       <c r="I54" s="17"/>
@@ -14674,22 +14675,22 @@
       <c r="HR54" s="17"/>
     </row>
     <row r="55" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="74" t="s">
+      <c r="A55" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="B55" s="75" t="s">
+      <c r="B55" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="C55" s="77" t="s">
+      <c r="C55" s="75" t="s">
         <v>119</v>
       </c>
       <c r="D55" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="72" t="s">
+      <c r="E55" s="76" t="s">
         <v>120</v>
       </c>
-      <c r="F55" s="73" t="s">
+      <c r="F55" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="17"/>
@@ -14904,14 +14905,14 @@
       <c r="HR55" s="17"/>
     </row>
     <row r="56" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="74"/>
-      <c r="B56" s="74"/>
-      <c r="C56" s="74"/>
+      <c r="A56" s="78"/>
+      <c r="B56" s="78"/>
+      <c r="C56" s="78"/>
       <c r="D56" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="72"/>
-      <c r="F56" s="72"/>
+      <c r="E56" s="76"/>
+      <c r="F56" s="76"/>
       <c r="G56" s="17"/>
       <c r="H56" s="17"/>
       <c r="I56" s="17"/>
@@ -15124,20 +15125,20 @@
       <c r="HR56" s="17"/>
     </row>
     <row r="57" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="74"/>
-      <c r="B57" s="75" t="s">
+      <c r="A57" s="78"/>
+      <c r="B57" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="C57" s="77" t="s">
+      <c r="C57" s="75" t="s">
         <v>122</v>
       </c>
       <c r="D57" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="72" t="s">
+      <c r="E57" s="76" t="s">
         <v>123</v>
       </c>
-      <c r="F57" s="73" t="s">
+      <c r="F57" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="17"/>
@@ -15352,14 +15353,14 @@
       <c r="HR57" s="17"/>
     </row>
     <row r="58" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="74"/>
-      <c r="B58" s="74"/>
-      <c r="C58" s="74"/>
+      <c r="A58" s="78"/>
+      <c r="B58" s="78"/>
+      <c r="C58" s="78"/>
       <c r="D58" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="72"/>
-      <c r="F58" s="72"/>
+      <c r="E58" s="76"/>
+      <c r="F58" s="76"/>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
       <c r="I58" s="17"/>
@@ -15572,20 +15573,20 @@
       <c r="HR58" s="17"/>
     </row>
     <row r="59" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="74"/>
-      <c r="B59" s="75" t="s">
+      <c r="A59" s="78"/>
+      <c r="B59" s="74" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="77" t="s">
+      <c r="C59" s="75" t="s">
         <v>125</v>
       </c>
       <c r="D59" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E59" s="72" t="s">
+      <c r="E59" s="76" t="s">
         <v>126</v>
       </c>
-      <c r="F59" s="73" t="s">
+      <c r="F59" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="17"/>
@@ -15800,14 +15801,14 @@
       <c r="HR59" s="17"/>
     </row>
     <row r="60" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="74"/>
-      <c r="B60" s="74"/>
-      <c r="C60" s="74"/>
+      <c r="A60" s="78"/>
+      <c r="B60" s="78"/>
+      <c r="C60" s="78"/>
       <c r="D60" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="72"/>
-      <c r="F60" s="72"/>
+      <c r="E60" s="76"/>
+      <c r="F60" s="76"/>
       <c r="G60" s="17"/>
       <c r="H60" s="17"/>
       <c r="I60" s="17"/>
@@ -16020,20 +16021,20 @@
       <c r="HR60" s="17"/>
     </row>
     <row r="61" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="74"/>
-      <c r="B61" s="75" t="s">
+      <c r="A61" s="78"/>
+      <c r="B61" s="74" t="s">
         <v>127</v>
       </c>
-      <c r="C61" s="77" t="s">
+      <c r="C61" s="75" t="s">
         <v>128</v>
       </c>
       <c r="D61" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E61" s="72" t="s">
+      <c r="E61" s="76" t="s">
         <v>129</v>
       </c>
-      <c r="F61" s="73" t="s">
+      <c r="F61" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="17"/>
@@ -16248,14 +16249,14 @@
       <c r="HR61" s="17"/>
     </row>
     <row r="62" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="74"/>
-      <c r="B62" s="74"/>
-      <c r="C62" s="74"/>
+      <c r="A62" s="78"/>
+      <c r="B62" s="78"/>
+      <c r="C62" s="78"/>
       <c r="D62" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E62" s="72"/>
-      <c r="F62" s="72"/>
+      <c r="E62" s="76"/>
+      <c r="F62" s="76"/>
       <c r="G62" s="17"/>
       <c r="H62" s="17"/>
       <c r="I62" s="17"/>
@@ -16468,20 +16469,20 @@
       <c r="HR62" s="17"/>
     </row>
     <row r="63" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="74"/>
-      <c r="B63" s="75" t="s">
+      <c r="A63" s="78"/>
+      <c r="B63" s="74" t="s">
         <v>130</v>
       </c>
-      <c r="C63" s="77" t="s">
+      <c r="C63" s="75" t="s">
         <v>131</v>
       </c>
       <c r="D63" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E63" s="72" t="s">
+      <c r="E63" s="76" t="s">
         <v>132</v>
       </c>
-      <c r="F63" s="73" t="s">
+      <c r="F63" s="77" t="s">
         <v>7</v>
       </c>
       <c r="G63" s="17"/>
@@ -16696,14 +16697,14 @@
       <c r="HR63" s="17"/>
     </row>
     <row r="64" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="74"/>
-      <c r="B64" s="74"/>
-      <c r="C64" s="74"/>
+      <c r="A64" s="78"/>
+      <c r="B64" s="78"/>
+      <c r="C64" s="78"/>
       <c r="D64" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E64" s="72"/>
-      <c r="F64" s="72"/>
+      <c r="E64" s="76"/>
+      <c r="F64" s="76"/>
       <c r="G64" s="17"/>
       <c r="H64" s="17"/>
       <c r="I64" s="17"/>
@@ -16916,20 +16917,20 @@
       <c r="HR64" s="17"/>
     </row>
     <row r="65" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="74"/>
-      <c r="B65" s="75" t="s">
+      <c r="A65" s="78"/>
+      <c r="B65" s="74" t="s">
         <v>133</v>
       </c>
-      <c r="C65" s="77" t="s">
+      <c r="C65" s="75" t="s">
         <v>134</v>
       </c>
       <c r="D65" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E65" s="72" t="s">
+      <c r="E65" s="76" t="s">
         <v>135</v>
       </c>
-      <c r="F65" s="73" t="s">
+      <c r="F65" s="77" t="s">
         <v>5</v>
       </c>
       <c r="G65" s="17"/>
@@ -17144,14 +17145,14 @@
       <c r="HR65" s="17"/>
     </row>
     <row r="66" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="74"/>
-      <c r="B66" s="74"/>
-      <c r="C66" s="74"/>
+      <c r="A66" s="78"/>
+      <c r="B66" s="78"/>
+      <c r="C66" s="78"/>
       <c r="D66" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E66" s="72"/>
-      <c r="F66" s="72"/>
+      <c r="E66" s="76"/>
+      <c r="F66" s="76"/>
       <c r="G66" s="17"/>
       <c r="H66" s="17"/>
       <c r="I66" s="17"/>
@@ -17364,22 +17365,22 @@
       <c r="HR66" s="17"/>
     </row>
     <row r="67" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="74" t="s">
+      <c r="A67" s="78" t="s">
         <v>136</v>
       </c>
-      <c r="B67" s="75" t="s">
+      <c r="B67" s="74" t="s">
         <v>137</v>
       </c>
-      <c r="C67" s="77" t="s">
+      <c r="C67" s="75" t="s">
         <v>138</v>
       </c>
       <c r="D67" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E67" s="72" t="s">
+      <c r="E67" s="76" t="s">
         <v>139</v>
       </c>
-      <c r="F67" s="73" t="s">
+      <c r="F67" s="77" t="s">
         <v>3</v>
       </c>
       <c r="G67" s="17"/>
@@ -17594,14 +17595,14 @@
       <c r="HR67" s="17"/>
     </row>
     <row r="68" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="74"/>
-      <c r="B68" s="74"/>
-      <c r="C68" s="74"/>
+      <c r="A68" s="78"/>
+      <c r="B68" s="78"/>
+      <c r="C68" s="78"/>
       <c r="D68" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E68" s="72"/>
-      <c r="F68" s="72"/>
+      <c r="E68" s="76"/>
+      <c r="F68" s="76"/>
       <c r="G68" s="17"/>
       <c r="H68" s="17"/>
       <c r="I68" s="17"/>
@@ -17815,20 +17816,20 @@
       <c r="HR68" s="17"/>
     </row>
     <row r="69" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="74"/>
-      <c r="B69" s="75" t="s">
+      <c r="A69" s="78"/>
+      <c r="B69" s="74" t="s">
         <v>140</v>
       </c>
-      <c r="C69" s="77" t="s">
+      <c r="C69" s="75" t="s">
         <v>141</v>
       </c>
       <c r="D69" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E69" s="72" t="s">
+      <c r="E69" s="76" t="s">
         <v>142</v>
       </c>
-      <c r="F69" s="73" t="s">
+      <c r="F69" s="77" t="s">
         <v>69</v>
       </c>
       <c r="G69" s="17"/>
@@ -18053,14 +18054,14 @@
       <c r="HR69" s="17"/>
     </row>
     <row r="70" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="74"/>
-      <c r="B70" s="74"/>
-      <c r="C70" s="74"/>
+      <c r="A70" s="78"/>
+      <c r="B70" s="78"/>
+      <c r="C70" s="78"/>
       <c r="D70" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E70" s="72"/>
-      <c r="F70" s="72"/>
+      <c r="E70" s="76"/>
+      <c r="F70" s="76"/>
       <c r="G70" s="17"/>
       <c r="H70" s="17"/>
       <c r="I70" s="17"/>
@@ -18277,20 +18278,20 @@
       <c r="HR70" s="17"/>
     </row>
     <row r="71" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="74"/>
-      <c r="B71" s="75" t="s">
+      <c r="A71" s="78"/>
+      <c r="B71" s="74" t="s">
         <v>143</v>
       </c>
-      <c r="C71" s="77" t="s">
+      <c r="C71" s="75" t="s">
         <v>144</v>
       </c>
       <c r="D71" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E71" s="72" t="s">
+      <c r="E71" s="76" t="s">
         <v>145</v>
       </c>
-      <c r="F71" s="73" t="s">
+      <c r="F71" s="77" t="s">
         <v>18</v>
       </c>
       <c r="G71" s="17"/>
@@ -18505,14 +18506,14 @@
       <c r="HR71" s="17"/>
     </row>
     <row r="72" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="74"/>
-      <c r="B72" s="74"/>
-      <c r="C72" s="74"/>
+      <c r="A72" s="78"/>
+      <c r="B72" s="78"/>
+      <c r="C72" s="78"/>
       <c r="D72" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E72" s="72"/>
-      <c r="F72" s="72"/>
+      <c r="E72" s="76"/>
+      <c r="F72" s="76"/>
       <c r="G72" s="17"/>
       <c r="H72" s="17"/>
       <c r="I72" s="17"/>
@@ -18725,20 +18726,20 @@
       <c r="HR72" s="17"/>
     </row>
     <row r="73" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="74"/>
-      <c r="B73" s="75" t="s">
+      <c r="A73" s="78"/>
+      <c r="B73" s="74" t="s">
         <v>146</v>
       </c>
-      <c r="C73" s="77" t="s">
+      <c r="C73" s="75" t="s">
         <v>147</v>
       </c>
       <c r="D73" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E73" s="72" t="s">
+      <c r="E73" s="76" t="s">
         <v>148</v>
       </c>
-      <c r="F73" s="73" t="s">
+      <c r="F73" s="77" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="17"/>
@@ -18953,14 +18954,14 @@
       <c r="HR73" s="17"/>
     </row>
     <row r="74" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="74"/>
-      <c r="B74" s="74"/>
-      <c r="C74" s="74"/>
+      <c r="A74" s="78"/>
+      <c r="B74" s="78"/>
+      <c r="C74" s="78"/>
       <c r="D74" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="72"/>
-      <c r="F74" s="72"/>
+      <c r="E74" s="76"/>
+      <c r="F74" s="76"/>
       <c r="G74" s="17"/>
       <c r="H74" s="17"/>
       <c r="I74" s="17"/>
@@ -19173,20 +19174,20 @@
       <c r="HR74" s="17"/>
     </row>
     <row r="75" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="74"/>
-      <c r="B75" s="75" t="s">
+      <c r="A75" s="78"/>
+      <c r="B75" s="74" t="s">
         <v>149</v>
       </c>
-      <c r="C75" s="77" t="s">
+      <c r="C75" s="75" t="s">
         <v>150</v>
       </c>
       <c r="D75" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E75" s="72" t="s">
+      <c r="E75" s="76" t="s">
         <v>151</v>
       </c>
-      <c r="F75" s="73" t="s">
+      <c r="F75" s="77" t="s">
         <v>8</v>
       </c>
       <c r="G75" s="17"/>
@@ -19401,14 +19402,14 @@
       <c r="HR75" s="17"/>
     </row>
     <row r="76" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="74"/>
-      <c r="B76" s="74"/>
-      <c r="C76" s="74"/>
+      <c r="A76" s="78"/>
+      <c r="B76" s="78"/>
+      <c r="C76" s="78"/>
       <c r="D76" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E76" s="72"/>
-      <c r="F76" s="72"/>
+      <c r="E76" s="76"/>
+      <c r="F76" s="76"/>
       <c r="G76" s="17"/>
       <c r="H76" s="17"/>
       <c r="I76" s="17"/>
@@ -19621,20 +19622,20 @@
       <c r="HR76" s="17"/>
     </row>
     <row r="77" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="74"/>
-      <c r="B77" s="75" t="s">
+      <c r="A77" s="78"/>
+      <c r="B77" s="74" t="s">
         <v>152</v>
       </c>
-      <c r="C77" s="77" t="s">
+      <c r="C77" s="75" t="s">
         <v>153</v>
       </c>
       <c r="D77" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E77" s="72" t="s">
+      <c r="E77" s="76" t="s">
         <v>154</v>
       </c>
-      <c r="F77" s="73" t="s">
+      <c r="F77" s="77" t="s">
         <v>6</v>
       </c>
       <c r="G77" s="17"/>
@@ -19849,14 +19850,14 @@
       <c r="HR77" s="17"/>
     </row>
     <row r="78" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="74"/>
-      <c r="B78" s="74"/>
-      <c r="C78" s="74"/>
+      <c r="A78" s="78"/>
+      <c r="B78" s="78"/>
+      <c r="C78" s="78"/>
       <c r="D78" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E78" s="72"/>
-      <c r="F78" s="72"/>
+      <c r="E78" s="76"/>
+      <c r="F78" s="76"/>
       <c r="G78" s="17"/>
       <c r="H78" s="17"/>
       <c r="I78" s="17"/>
@@ -20069,22 +20070,22 @@
       <c r="HR78" s="17"/>
     </row>
     <row r="79" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="74" t="s">
+      <c r="A79" s="78" t="s">
         <v>155</v>
       </c>
-      <c r="B79" s="75" t="s">
+      <c r="B79" s="74" t="s">
         <v>156</v>
       </c>
-      <c r="C79" s="76" t="s">
+      <c r="C79" s="84" t="s">
         <v>157</v>
       </c>
       <c r="D79" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E79" s="72" t="s">
+      <c r="E79" s="76" t="s">
         <v>158</v>
       </c>
-      <c r="F79" s="73" t="s">
+      <c r="F79" s="77" t="s">
         <v>13</v>
       </c>
       <c r="G79" s="17"/>
@@ -20299,14 +20300,14 @@
       <c r="HR79" s="17"/>
     </row>
     <row r="80" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="74"/>
-      <c r="B80" s="74"/>
-      <c r="C80" s="74"/>
+      <c r="A80" s="78"/>
+      <c r="B80" s="78"/>
+      <c r="C80" s="78"/>
       <c r="D80" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E80" s="72"/>
-      <c r="F80" s="72"/>
+      <c r="E80" s="76"/>
+      <c r="F80" s="76"/>
       <c r="G80" s="17"/>
       <c r="H80" s="17"/>
       <c r="I80" s="17"/>
@@ -20519,20 +20520,20 @@
       <c r="HR80" s="17"/>
     </row>
     <row r="81" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="74"/>
-      <c r="B81" s="75" t="s">
+      <c r="A81" s="78"/>
+      <c r="B81" s="74" t="s">
         <v>159</v>
       </c>
-      <c r="C81" s="76" t="s">
+      <c r="C81" s="84" t="s">
         <v>160</v>
       </c>
       <c r="D81" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E81" s="72" t="s">
+      <c r="E81" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="F81" s="73" t="s">
+      <c r="F81" s="77" t="s">
         <v>8</v>
       </c>
       <c r="G81" s="17"/>
@@ -20747,14 +20748,14 @@
       <c r="HR81" s="17"/>
     </row>
     <row r="82" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="74"/>
-      <c r="B82" s="74"/>
-      <c r="C82" s="74"/>
+      <c r="A82" s="78"/>
+      <c r="B82" s="78"/>
+      <c r="C82" s="78"/>
       <c r="D82" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E82" s="72"/>
-      <c r="F82" s="72"/>
+      <c r="E82" s="76"/>
+      <c r="F82" s="76"/>
       <c r="G82" s="17"/>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
@@ -20967,20 +20968,20 @@
       <c r="HR82" s="17"/>
     </row>
     <row r="83" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="74"/>
-      <c r="B83" s="75" t="s">
+      <c r="A83" s="78"/>
+      <c r="B83" s="74" t="s">
         <v>162</v>
       </c>
-      <c r="C83" s="77" t="s">
+      <c r="C83" s="75" t="s">
         <v>163</v>
       </c>
       <c r="D83" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E83" s="72" t="s">
+      <c r="E83" s="76" t="s">
         <v>164</v>
       </c>
-      <c r="F83" s="73" t="s">
+      <c r="F83" s="77" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="17"/>
@@ -21195,14 +21196,14 @@
       <c r="HR83" s="17"/>
     </row>
     <row r="84" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="74"/>
-      <c r="B84" s="74"/>
-      <c r="C84" s="74"/>
+      <c r="A84" s="78"/>
+      <c r="B84" s="78"/>
+      <c r="C84" s="78"/>
       <c r="D84" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E84" s="72"/>
-      <c r="F84" s="72"/>
+      <c r="E84" s="76"/>
+      <c r="F84" s="76"/>
       <c r="G84" s="17"/>
       <c r="H84" s="17"/>
       <c r="I84" s="17"/>
@@ -21415,20 +21416,20 @@
       <c r="HR84" s="17"/>
     </row>
     <row r="85" spans="1:226" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="74"/>
-      <c r="B85" s="75" t="s">
+      <c r="A85" s="78"/>
+      <c r="B85" s="74" t="s">
         <v>165</v>
       </c>
-      <c r="C85" s="78" t="s">
+      <c r="C85" s="79" t="s">
         <v>166</v>
       </c>
       <c r="D85" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="E85" s="72" t="s">
+      <c r="E85" s="76" t="s">
         <v>167</v>
       </c>
-      <c r="F85" s="73"/>
+      <c r="F85" s="77"/>
       <c r="G85" s="17"/>
       <c r="H85" s="17"/>
       <c r="I85" s="17"/>
@@ -21641,14 +21642,14 @@
       <c r="HR85" s="49"/>
     </row>
     <row r="86" spans="1:226" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="74"/>
-      <c r="B86" s="74"/>
-      <c r="C86" s="74"/>
+      <c r="A86" s="78"/>
+      <c r="B86" s="78"/>
+      <c r="C86" s="78"/>
       <c r="D86" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="E86" s="72"/>
-      <c r="F86" s="72"/>
+      <c r="E86" s="76"/>
+      <c r="F86" s="76"/>
       <c r="G86" s="17"/>
       <c r="H86" s="17"/>
       <c r="I86" s="17"/>
@@ -21862,33 +21863,160 @@
     </row>
   </sheetData>
   <mergeCells count="205">
-    <mergeCell ref="G1:M1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="U1:AA1"/>
-    <mergeCell ref="AB1:AH1"/>
-    <mergeCell ref="AI1:AO1"/>
-    <mergeCell ref="AP1:AV1"/>
-    <mergeCell ref="AW1:BC1"/>
-    <mergeCell ref="BD1:BJ1"/>
-    <mergeCell ref="BK1:BQ1"/>
-    <mergeCell ref="BR1:BX1"/>
-    <mergeCell ref="BY1:CE1"/>
-    <mergeCell ref="CF1:CL1"/>
-    <mergeCell ref="CM1:CS1"/>
-    <mergeCell ref="CT1:CZ1"/>
-    <mergeCell ref="DA1:DG1"/>
-    <mergeCell ref="DH1:DN1"/>
-    <mergeCell ref="DO1:DU1"/>
-    <mergeCell ref="DV1:EB1"/>
-    <mergeCell ref="EC1:EI1"/>
-    <mergeCell ref="EJ1:EP1"/>
-    <mergeCell ref="EQ1:EW1"/>
-    <mergeCell ref="EX1:FD1"/>
-    <mergeCell ref="FE1:FK1"/>
-    <mergeCell ref="FL1:FR1"/>
-    <mergeCell ref="FS1:FY1"/>
-    <mergeCell ref="FZ1:GF1"/>
-    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="A79:A86"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="F79:F80"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="E81:E82"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="B85:B86"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="E85:E86"/>
+    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="F67:F68"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="F69:F70"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="E75:E76"/>
+    <mergeCell ref="F75:F76"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="A55:A66"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="F55:F56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="F61:F62"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="A29:A40"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="A41:A46"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
     <mergeCell ref="GN1:GT1"/>
     <mergeCell ref="GU1:HA1"/>
     <mergeCell ref="HB1:HH1"/>
@@ -21913,160 +22041,33 @@
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="C13:C14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="A41:A46"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="A29:A40"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="A51:A54"/>
-    <mergeCell ref="B51:B52"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="F55:F56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="F57:F58"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="F61:F62"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="A67:A78"/>
-    <mergeCell ref="B67:B68"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="F67:F68"/>
-    <mergeCell ref="B69:B70"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="F69:F70"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="B75:B76"/>
-    <mergeCell ref="C75:C76"/>
-    <mergeCell ref="E75:E76"/>
-    <mergeCell ref="F75:F76"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="A79:A86"/>
-    <mergeCell ref="B79:B80"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="E79:E80"/>
-    <mergeCell ref="F79:F80"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="E81:E82"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="B85:B86"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="E85:E86"/>
-    <mergeCell ref="F85:F86"/>
+    <mergeCell ref="EC1:EI1"/>
+    <mergeCell ref="EJ1:EP1"/>
+    <mergeCell ref="EQ1:EW1"/>
+    <mergeCell ref="EX1:FD1"/>
+    <mergeCell ref="FE1:FK1"/>
+    <mergeCell ref="FL1:FR1"/>
+    <mergeCell ref="FS1:FY1"/>
+    <mergeCell ref="FZ1:GF1"/>
+    <mergeCell ref="GG1:GM1"/>
+    <mergeCell ref="BR1:BX1"/>
+    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="CF1:CL1"/>
+    <mergeCell ref="CM1:CS1"/>
+    <mergeCell ref="CT1:CZ1"/>
+    <mergeCell ref="DA1:DG1"/>
+    <mergeCell ref="DH1:DN1"/>
+    <mergeCell ref="DO1:DU1"/>
+    <mergeCell ref="DV1:EB1"/>
+    <mergeCell ref="G1:M1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="AP1:AV1"/>
+    <mergeCell ref="AW1:BC1"/>
+    <mergeCell ref="BD1:BJ1"/>
+    <mergeCell ref="BK1:BQ1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
bugfix on tune script
</commit_message>
<xml_diff>
--- a/Projektplanung/Bearbeitungsplan.xlsx
+++ b/Projektplanung/Bearbeitungsplan.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Masterarbeit NO-Surrogate for SC simulations\Neural Operator for Cheetah\Projektplanung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B4130B-2A6D-45BA-AE40-7A3022AFABF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC4BCEC-C44E-4F7D-A0C9-77A623447573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearbeitungsplan" sheetId="1" r:id="rId1"/>
     <sheet name="Pakete &amp; Leitfragen" sheetId="2" r:id="rId2"/>
     <sheet name="Legende &amp; Regeln" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1620,8 +1620,11 @@
     <col min="67" max="69" width="2.140625" customWidth="1"/>
     <col min="70" max="70" width="2.140625" style="1" customWidth="1"/>
     <col min="71" max="72" width="2.140625" customWidth="1"/>
-    <col min="73" max="73" width="2.140625" style="2" customWidth="1"/>
-    <col min="74" max="226" width="2.140625" customWidth="1"/>
+    <col min="73" max="73" width="2.140625" style="1" customWidth="1"/>
+    <col min="74" max="77" width="2.140625" customWidth="1"/>
+    <col min="78" max="78" width="2.140625" style="1" customWidth="1"/>
+    <col min="79" max="79" width="2.140625" style="2" customWidth="1"/>
+    <col min="80" max="226" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:226" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2115,7 +2118,7 @@
       <c r="BT2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="BU2" s="7" t="s">
+      <c r="BU2" s="6" t="s">
         <v>35</v>
       </c>
       <c r="BV2" s="4" t="s">
@@ -2130,10 +2133,10 @@
       <c r="BY2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="BZ2" s="4" t="s">
+      <c r="BZ2" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="CA2" s="4" t="s">
+      <c r="CA2" s="7" t="s">
         <v>34</v>
       </c>
       <c r="CB2" s="4" t="s">
@@ -2780,7 +2783,7 @@
       <c r="BT3" s="8">
         <v>46316</v>
       </c>
-      <c r="BU3" s="10">
+      <c r="BU3" s="9">
         <v>46317</v>
       </c>
       <c r="BV3" s="8">
@@ -2795,10 +2798,10 @@
       <c r="BY3" s="8">
         <v>46321</v>
       </c>
-      <c r="BZ3" s="8">
+      <c r="BZ3" s="9">
         <v>46322</v>
       </c>
-      <c r="CA3" s="8">
+      <c r="CA3" s="10">
         <v>46323</v>
       </c>
       <c r="CB3" s="8">
@@ -3326,13 +3329,13 @@
       <c r="BR4" s="13"/>
       <c r="BS4" s="12"/>
       <c r="BT4" s="12"/>
-      <c r="BU4" s="14"/>
+      <c r="BU4" s="13"/>
       <c r="BV4" s="12"/>
       <c r="BW4" s="12"/>
       <c r="BX4" s="12"/>
       <c r="BY4" s="12"/>
-      <c r="BZ4" s="12"/>
-      <c r="CA4" s="12"/>
+      <c r="BZ4" s="13"/>
+      <c r="CA4" s="14"/>
       <c r="CB4" s="12"/>
       <c r="CC4" s="12"/>
       <c r="CD4" s="12"/>
@@ -3552,13 +3555,11 @@
       <c r="BP5" s="19"/>
       <c r="BQ5" s="21"/>
       <c r="BS5" s="17"/>
-      <c r="BT5" s="17"/>
+      <c r="BT5" s="1"/>
       <c r="BV5" s="18"/>
       <c r="BW5" s="19"/>
       <c r="BX5" s="20"/>
-      <c r="BY5" s="17"/>
-      <c r="BZ5" s="17"/>
-      <c r="CA5" s="17"/>
+      <c r="BY5" s="1"/>
       <c r="CB5" s="17"/>
       <c r="CC5" s="18"/>
       <c r="CD5" s="19"/>
@@ -3772,13 +3773,11 @@
       <c r="BP6" s="19"/>
       <c r="BQ6" s="21"/>
       <c r="BS6" s="17"/>
-      <c r="BT6" s="17"/>
+      <c r="BT6" s="1"/>
       <c r="BV6" s="18"/>
       <c r="BW6" s="19"/>
       <c r="BX6" s="20"/>
-      <c r="BY6" s="17"/>
-      <c r="BZ6" s="17"/>
-      <c r="CA6" s="17"/>
+      <c r="BY6" s="1"/>
       <c r="CB6" s="17"/>
       <c r="CC6" s="18"/>
       <c r="CD6" s="19"/>
@@ -3996,13 +3995,11 @@
       <c r="BP7" s="19"/>
       <c r="BQ7" s="21"/>
       <c r="BS7" s="17"/>
-      <c r="BT7" s="17"/>
+      <c r="BT7" s="1"/>
       <c r="BV7" s="18"/>
       <c r="BW7" s="19"/>
       <c r="BX7" s="20"/>
-      <c r="BY7" s="17"/>
-      <c r="BZ7" s="17"/>
-      <c r="CA7" s="17"/>
+      <c r="BY7" s="1"/>
       <c r="CB7" s="17"/>
       <c r="CC7" s="18"/>
       <c r="CD7" s="19"/>
@@ -4216,13 +4213,11 @@
       <c r="BP8" s="19"/>
       <c r="BQ8" s="21"/>
       <c r="BS8" s="17"/>
-      <c r="BT8" s="17"/>
+      <c r="BT8" s="1"/>
       <c r="BV8" s="18"/>
       <c r="BW8" s="19"/>
       <c r="BX8" s="20"/>
-      <c r="BY8" s="17"/>
-      <c r="BZ8" s="17"/>
-      <c r="CA8" s="17"/>
+      <c r="BY8" s="1"/>
       <c r="CB8" s="17"/>
       <c r="CC8" s="18"/>
       <c r="CD8" s="19"/>
@@ -4440,13 +4435,11 @@
       <c r="BP9" s="19"/>
       <c r="BQ9" s="21"/>
       <c r="BS9" s="17"/>
-      <c r="BT9" s="17"/>
+      <c r="BT9" s="1"/>
       <c r="BV9" s="18"/>
       <c r="BW9" s="19"/>
       <c r="BX9" s="20"/>
-      <c r="BY9" s="17"/>
-      <c r="BZ9" s="17"/>
-      <c r="CA9" s="17"/>
+      <c r="BY9" s="1"/>
       <c r="CB9" s="17"/>
       <c r="CC9" s="18"/>
       <c r="CD9" s="19"/>
@@ -4660,13 +4653,11 @@
       <c r="BP10" s="19"/>
       <c r="BQ10" s="21"/>
       <c r="BS10" s="17"/>
-      <c r="BT10" s="17"/>
+      <c r="BT10" s="1"/>
       <c r="BV10" s="18"/>
       <c r="BW10" s="19"/>
       <c r="BX10" s="20"/>
-      <c r="BY10" s="17"/>
-      <c r="BZ10" s="17"/>
-      <c r="CA10" s="17"/>
+      <c r="BY10" s="1"/>
       <c r="CB10" s="17"/>
       <c r="CC10" s="18"/>
       <c r="CD10" s="19"/>
@@ -4884,13 +4875,11 @@
       <c r="BP11" s="19"/>
       <c r="BQ11" s="21"/>
       <c r="BS11" s="17"/>
-      <c r="BT11" s="17"/>
+      <c r="BT11" s="1"/>
       <c r="BV11" s="18"/>
       <c r="BW11" s="19"/>
       <c r="BX11" s="20"/>
-      <c r="BY11" s="17"/>
-      <c r="BZ11" s="17"/>
-      <c r="CA11" s="17"/>
+      <c r="BY11" s="1"/>
       <c r="CB11" s="17"/>
       <c r="CC11" s="18"/>
       <c r="CD11" s="19"/>
@@ -5104,13 +5093,11 @@
       <c r="BP12" s="19"/>
       <c r="BQ12" s="21"/>
       <c r="BS12" s="17"/>
-      <c r="BT12" s="17"/>
+      <c r="BT12" s="1"/>
       <c r="BV12" s="18"/>
       <c r="BW12" s="19"/>
       <c r="BX12" s="20"/>
-      <c r="BY12" s="17"/>
-      <c r="BZ12" s="17"/>
-      <c r="CA12" s="17"/>
+      <c r="BY12" s="1"/>
       <c r="CB12" s="17"/>
       <c r="CC12" s="18"/>
       <c r="CD12" s="19"/>
@@ -5328,13 +5315,11 @@
       <c r="BP13" s="19"/>
       <c r="BQ13" s="21"/>
       <c r="BS13" s="17"/>
-      <c r="BT13" s="17"/>
+      <c r="BT13" s="1"/>
       <c r="BV13" s="18"/>
       <c r="BW13" s="19"/>
       <c r="BX13" s="20"/>
-      <c r="BY13" s="17"/>
-      <c r="BZ13" s="17"/>
-      <c r="CA13" s="17"/>
+      <c r="BY13" s="1"/>
       <c r="CB13" s="17"/>
       <c r="CC13" s="18"/>
       <c r="CD13" s="19"/>
@@ -5548,13 +5533,11 @@
       <c r="BP14" s="19"/>
       <c r="BQ14" s="21"/>
       <c r="BS14" s="17"/>
-      <c r="BT14" s="17"/>
+      <c r="BT14" s="1"/>
       <c r="BV14" s="18"/>
       <c r="BW14" s="19"/>
       <c r="BX14" s="20"/>
-      <c r="BY14" s="17"/>
-      <c r="BZ14" s="17"/>
-      <c r="CA14" s="17"/>
+      <c r="BY14" s="1"/>
       <c r="CB14" s="17"/>
       <c r="CC14" s="18"/>
       <c r="CD14" s="19"/>
@@ -5772,13 +5755,11 @@
       <c r="BP15" s="19"/>
       <c r="BQ15" s="21"/>
       <c r="BS15" s="17"/>
-      <c r="BT15" s="17"/>
+      <c r="BT15" s="1"/>
       <c r="BV15" s="18"/>
       <c r="BW15" s="19"/>
       <c r="BX15" s="20"/>
-      <c r="BY15" s="17"/>
-      <c r="BZ15" s="17"/>
-      <c r="CA15" s="17"/>
+      <c r="BY15" s="1"/>
       <c r="CB15" s="17"/>
       <c r="CC15" s="18"/>
       <c r="CD15" s="19"/>
@@ -5992,13 +5973,11 @@
       <c r="BP16" s="19"/>
       <c r="BQ16" s="21"/>
       <c r="BS16" s="17"/>
-      <c r="BT16" s="17"/>
+      <c r="BT16" s="1"/>
       <c r="BV16" s="18"/>
       <c r="BW16" s="19"/>
       <c r="BX16" s="20"/>
-      <c r="BY16" s="17"/>
-      <c r="BZ16" s="17"/>
-      <c r="CA16" s="17"/>
+      <c r="BY16" s="1"/>
       <c r="CB16" s="17"/>
       <c r="CC16" s="18"/>
       <c r="CD16" s="19"/>
@@ -6216,13 +6195,11 @@
       <c r="BP17" s="19"/>
       <c r="BQ17" s="21"/>
       <c r="BS17" s="17"/>
-      <c r="BT17" s="17"/>
+      <c r="BT17" s="1"/>
       <c r="BV17" s="18"/>
       <c r="BW17" s="19"/>
       <c r="BX17" s="20"/>
-      <c r="BY17" s="17"/>
-      <c r="BZ17" s="17"/>
-      <c r="CA17" s="17"/>
+      <c r="BY17" s="1"/>
       <c r="CB17" s="17"/>
       <c r="CC17" s="18"/>
       <c r="CD17" s="19"/>
@@ -6436,13 +6413,11 @@
       <c r="BP18" s="19"/>
       <c r="BQ18" s="21"/>
       <c r="BS18" s="17"/>
-      <c r="BT18" s="17"/>
+      <c r="BT18" s="1"/>
       <c r="BV18" s="18"/>
       <c r="BW18" s="19"/>
       <c r="BX18" s="20"/>
-      <c r="BY18" s="17"/>
-      <c r="BZ18" s="17"/>
-      <c r="CA18" s="17"/>
+      <c r="BY18" s="1"/>
       <c r="CB18" s="17"/>
       <c r="CC18" s="18"/>
       <c r="CD18" s="19"/>
@@ -6660,13 +6635,11 @@
       <c r="BP19" s="19"/>
       <c r="BQ19" s="21"/>
       <c r="BS19" s="17"/>
-      <c r="BT19" s="17"/>
+      <c r="BT19" s="1"/>
       <c r="BV19" s="18"/>
       <c r="BW19" s="19"/>
       <c r="BX19" s="20"/>
-      <c r="BY19" s="17"/>
-      <c r="BZ19" s="17"/>
-      <c r="CA19" s="17"/>
+      <c r="BY19" s="1"/>
       <c r="CB19" s="17"/>
       <c r="CC19" s="18"/>
       <c r="CD19" s="19"/>
@@ -6880,13 +6853,11 @@
       <c r="BP20" s="19"/>
       <c r="BQ20" s="21"/>
       <c r="BS20" s="17"/>
-      <c r="BT20" s="17"/>
+      <c r="BT20" s="1"/>
       <c r="BV20" s="18"/>
       <c r="BW20" s="19"/>
       <c r="BX20" s="20"/>
-      <c r="BY20" s="17"/>
-      <c r="BZ20" s="17"/>
-      <c r="CA20" s="17"/>
+      <c r="BY20" s="1"/>
       <c r="CB20" s="17"/>
       <c r="CC20" s="18"/>
       <c r="CD20" s="19"/>
@@ -7104,13 +7075,11 @@
       <c r="BP21" s="19"/>
       <c r="BQ21" s="21"/>
       <c r="BS21" s="17"/>
-      <c r="BT21" s="17"/>
+      <c r="BT21" s="1"/>
       <c r="BV21" s="18"/>
       <c r="BW21" s="19"/>
       <c r="BX21" s="20"/>
-      <c r="BY21" s="17"/>
-      <c r="BZ21" s="17"/>
-      <c r="CA21" s="17"/>
+      <c r="BY21" s="1"/>
       <c r="CB21" s="17"/>
       <c r="CC21" s="18"/>
       <c r="CD21" s="19"/>
@@ -7324,14 +7293,12 @@
       <c r="BP22" s="32"/>
       <c r="BQ22" s="35"/>
       <c r="BS22" s="30"/>
-      <c r="BT22" s="30"/>
-      <c r="BU22" s="67"/>
+      <c r="BT22" s="36"/>
       <c r="BV22" s="31"/>
       <c r="BW22" s="32"/>
       <c r="BX22" s="33"/>
-      <c r="BY22" s="30"/>
-      <c r="BZ22" s="30"/>
-      <c r="CA22" s="30"/>
+      <c r="BY22" s="36"/>
+      <c r="CA22" s="67"/>
       <c r="CB22" s="30"/>
       <c r="CC22" s="31"/>
       <c r="CD22" s="32"/>
@@ -7560,13 +7527,11 @@
       <c r="BQ23" s="21"/>
       <c r="BR23" s="38"/>
       <c r="BS23" s="17"/>
-      <c r="BT23" s="17"/>
+      <c r="BT23" s="1"/>
       <c r="BV23" s="18"/>
       <c r="BW23" s="19"/>
       <c r="BX23" s="20"/>
-      <c r="BY23" s="39"/>
-      <c r="BZ23" s="17"/>
-      <c r="CA23" s="17"/>
+      <c r="BY23" s="38"/>
       <c r="CB23" s="17"/>
       <c r="CC23" s="18"/>
       <c r="CD23" s="19"/>
@@ -7784,13 +7749,11 @@
       <c r="BP24" s="19"/>
       <c r="BQ24" s="21"/>
       <c r="BS24" s="17"/>
-      <c r="BU24" s="25"/>
+      <c r="BU24" s="45"/>
       <c r="BV24" s="18"/>
       <c r="BW24" s="19"/>
       <c r="BX24" s="20"/>
-      <c r="BY24" s="17"/>
-      <c r="BZ24" s="17"/>
-      <c r="CA24" s="17"/>
+      <c r="BY24" s="70"/>
       <c r="CB24" s="17"/>
       <c r="CC24" s="18"/>
       <c r="CD24" s="19"/>
@@ -8007,13 +7970,12 @@
       <c r="BP25" s="19"/>
       <c r="BQ25" s="21"/>
       <c r="BS25" s="17"/>
-      <c r="BT25" s="17"/>
+      <c r="BT25" s="1"/>
       <c r="BV25" s="18"/>
       <c r="BW25" s="19"/>
       <c r="BX25" s="20"/>
-      <c r="BY25" s="17"/>
-      <c r="BZ25" s="39"/>
-      <c r="CA25" s="17"/>
+      <c r="BY25" s="1"/>
+      <c r="BZ25" s="38"/>
       <c r="CB25" s="17"/>
       <c r="CC25" s="18"/>
       <c r="CD25" s="19"/>
@@ -8226,13 +8188,12 @@
       <c r="BP26" s="19"/>
       <c r="BQ26" s="21"/>
       <c r="BS26" s="17"/>
-      <c r="BT26" s="17"/>
+      <c r="BT26" s="1"/>
       <c r="BV26" s="18"/>
       <c r="BW26" s="19"/>
       <c r="BX26" s="20"/>
-      <c r="BY26" s="17"/>
-      <c r="BZ26" s="17"/>
-      <c r="CA26" s="17"/>
+      <c r="BY26" s="1"/>
+      <c r="BZ26" s="70"/>
       <c r="CB26" s="17"/>
       <c r="CC26" s="18"/>
       <c r="CD26" s="19"/>
@@ -8452,13 +8413,11 @@
       <c r="BP27" s="19"/>
       <c r="BQ27" s="21"/>
       <c r="BS27" s="17"/>
-      <c r="BT27" s="17"/>
+      <c r="BT27" s="1"/>
       <c r="BV27" s="18"/>
       <c r="BW27" s="19"/>
       <c r="BX27" s="20"/>
-      <c r="BY27" s="17"/>
-      <c r="BZ27" s="17"/>
-      <c r="CA27" s="17"/>
+      <c r="BY27" s="1"/>
       <c r="CB27" s="17"/>
       <c r="CC27" s="18"/>
       <c r="CD27" s="19"/>
@@ -8672,13 +8631,11 @@
       <c r="BP28" s="19"/>
       <c r="BQ28" s="21"/>
       <c r="BS28" s="17"/>
-      <c r="BT28" s="17"/>
+      <c r="BT28" s="1"/>
       <c r="BV28" s="18"/>
       <c r="BW28" s="19"/>
       <c r="BX28" s="20"/>
-      <c r="BY28" s="17"/>
-      <c r="BZ28" s="17"/>
-      <c r="CA28" s="17"/>
+      <c r="BY28" s="1"/>
       <c r="CB28" s="17"/>
       <c r="CC28" s="18"/>
       <c r="CD28" s="19"/>
@@ -8901,13 +8858,11 @@
       <c r="BP29" s="19"/>
       <c r="BQ29" s="21"/>
       <c r="BS29" s="17"/>
-      <c r="BT29" s="17"/>
+      <c r="BT29" s="1"/>
       <c r="BV29" s="18"/>
       <c r="BW29" s="19"/>
       <c r="BX29" s="20"/>
-      <c r="BY29" s="17"/>
-      <c r="BZ29" s="17"/>
-      <c r="CA29" s="17"/>
+      <c r="BY29" s="1"/>
       <c r="CB29" s="17"/>
       <c r="CC29" s="18"/>
       <c r="CD29" s="19"/>
@@ -9121,13 +9076,11 @@
       <c r="BP30" s="19"/>
       <c r="BQ30" s="21"/>
       <c r="BS30" s="17"/>
-      <c r="BT30" s="17"/>
+      <c r="BT30" s="1"/>
       <c r="BV30" s="18"/>
       <c r="BW30" s="19"/>
       <c r="BX30" s="20"/>
-      <c r="BY30" s="17"/>
-      <c r="BZ30" s="17"/>
-      <c r="CA30" s="17"/>
+      <c r="BY30" s="1"/>
       <c r="CB30" s="17"/>
       <c r="CC30" s="18"/>
       <c r="CD30" s="19"/>
@@ -9349,13 +9302,11 @@
       <c r="BP31" s="19"/>
       <c r="BQ31" s="21"/>
       <c r="BS31" s="17"/>
-      <c r="BT31" s="17"/>
+      <c r="BT31" s="1"/>
       <c r="BV31" s="18"/>
       <c r="BW31" s="19"/>
       <c r="BX31" s="20"/>
-      <c r="BY31" s="17"/>
-      <c r="BZ31" s="17"/>
-      <c r="CA31" s="17"/>
+      <c r="BY31" s="1"/>
       <c r="CB31" s="17"/>
       <c r="CC31" s="18"/>
       <c r="CD31" s="19"/>
@@ -9569,13 +9520,11 @@
       <c r="BP32" s="19"/>
       <c r="BQ32" s="21"/>
       <c r="BS32" s="17"/>
-      <c r="BT32" s="17"/>
+      <c r="BT32" s="1"/>
       <c r="BV32" s="18"/>
       <c r="BW32" s="19"/>
       <c r="BX32" s="20"/>
-      <c r="BY32" s="17"/>
-      <c r="BZ32" s="17"/>
-      <c r="CA32" s="17"/>
+      <c r="BY32" s="1"/>
       <c r="CB32" s="17"/>
       <c r="CC32" s="18"/>
       <c r="CD32" s="19"/>
@@ -9797,13 +9746,11 @@
       <c r="BP33" s="19"/>
       <c r="BQ33" s="21"/>
       <c r="BS33" s="17"/>
-      <c r="BT33" s="17"/>
+      <c r="BT33" s="1"/>
       <c r="BV33" s="18"/>
       <c r="BW33" s="19"/>
       <c r="BX33" s="20"/>
-      <c r="BY33" s="17"/>
-      <c r="BZ33" s="17"/>
-      <c r="CA33" s="17"/>
+      <c r="BY33" s="1"/>
       <c r="CB33" s="17"/>
       <c r="CC33" s="18"/>
       <c r="CD33" s="19"/>
@@ -10017,13 +9964,11 @@
       <c r="BP34" s="19"/>
       <c r="BQ34" s="21"/>
       <c r="BS34" s="17"/>
-      <c r="BT34" s="17"/>
+      <c r="BT34" s="1"/>
       <c r="BV34" s="18"/>
       <c r="BW34" s="19"/>
       <c r="BX34" s="20"/>
-      <c r="BY34" s="17"/>
-      <c r="BZ34" s="17"/>
-      <c r="CA34" s="17"/>
+      <c r="BY34" s="1"/>
       <c r="CB34" s="17"/>
       <c r="CC34" s="18"/>
       <c r="CD34" s="19"/>
@@ -10246,13 +10191,11 @@
       <c r="BP35" s="19"/>
       <c r="BQ35" s="21"/>
       <c r="BS35" s="17"/>
-      <c r="BT35" s="17"/>
+      <c r="BT35" s="1"/>
       <c r="BV35" s="18"/>
       <c r="BW35" s="19"/>
       <c r="BX35" s="20"/>
-      <c r="BY35" s="17"/>
-      <c r="BZ35" s="17"/>
-      <c r="CA35" s="17"/>
+      <c r="BY35" s="1"/>
       <c r="CB35" s="17"/>
       <c r="CC35" s="18"/>
       <c r="CD35" s="19"/>
@@ -10467,13 +10410,11 @@
       <c r="BP36" s="19"/>
       <c r="BQ36" s="21"/>
       <c r="BS36" s="17"/>
-      <c r="BT36" s="17"/>
+      <c r="BT36" s="1"/>
       <c r="BV36" s="18"/>
       <c r="BW36" s="19"/>
       <c r="BX36" s="20"/>
-      <c r="BY36" s="17"/>
-      <c r="BZ36" s="17"/>
-      <c r="CA36" s="17"/>
+      <c r="BY36" s="1"/>
       <c r="CB36" s="17"/>
       <c r="CC36" s="18"/>
       <c r="CD36" s="19"/>
@@ -10695,13 +10636,11 @@
       <c r="BP37" s="19"/>
       <c r="BQ37" s="21"/>
       <c r="BS37" s="17"/>
-      <c r="BT37" s="17"/>
+      <c r="BT37" s="1"/>
       <c r="BV37" s="18"/>
       <c r="BW37" s="19"/>
       <c r="BX37" s="20"/>
-      <c r="BY37" s="17"/>
-      <c r="BZ37" s="17"/>
-      <c r="CA37" s="17"/>
+      <c r="BY37" s="1"/>
       <c r="CB37" s="17"/>
       <c r="CC37" s="18"/>
       <c r="CD37" s="19"/>
@@ -10915,13 +10854,11 @@
       <c r="BP38" s="19"/>
       <c r="BQ38" s="21"/>
       <c r="BS38" s="17"/>
-      <c r="BT38" s="17"/>
+      <c r="BT38" s="1"/>
       <c r="BV38" s="18"/>
       <c r="BW38" s="19"/>
       <c r="BX38" s="20"/>
-      <c r="BY38" s="17"/>
-      <c r="BZ38" s="17"/>
-      <c r="CA38" s="17"/>
+      <c r="BY38" s="1"/>
       <c r="CB38" s="17"/>
       <c r="CC38" s="18"/>
       <c r="CD38" s="19"/>
@@ -11145,13 +11082,11 @@
       <c r="BQ39" s="21"/>
       <c r="BR39" s="38"/>
       <c r="BS39" s="17"/>
-      <c r="BT39" s="17"/>
+      <c r="BT39" s="1"/>
       <c r="BV39" s="18"/>
       <c r="BW39" s="19"/>
       <c r="BX39" s="20"/>
-      <c r="BY39" s="17"/>
-      <c r="BZ39" s="17"/>
-      <c r="CA39" s="17"/>
+      <c r="BY39" s="1"/>
       <c r="CB39" s="17"/>
       <c r="CC39" s="18"/>
       <c r="CD39" s="19"/>
@@ -11366,13 +11301,11 @@
       <c r="BP40" s="19"/>
       <c r="BQ40" s="21"/>
       <c r="BS40" s="17"/>
-      <c r="BT40" s="17"/>
+      <c r="BT40" s="1"/>
       <c r="BV40" s="18"/>
       <c r="BW40" s="19"/>
       <c r="BX40" s="20"/>
-      <c r="BY40" s="17"/>
-      <c r="BZ40" s="17"/>
-      <c r="CA40" s="17"/>
+      <c r="BY40" s="1"/>
       <c r="CB40" s="17"/>
       <c r="CC40" s="18"/>
       <c r="CD40" s="19"/>
@@ -11596,13 +11529,11 @@
       <c r="BP41" s="19"/>
       <c r="BQ41" s="21"/>
       <c r="BS41" s="17"/>
-      <c r="BT41" s="17"/>
+      <c r="BT41" s="1"/>
       <c r="BV41" s="18"/>
       <c r="BW41" s="19"/>
       <c r="BX41" s="20"/>
-      <c r="BY41" s="17"/>
-      <c r="BZ41" s="17"/>
-      <c r="CA41" s="17"/>
+      <c r="BY41" s="1"/>
       <c r="CB41" s="17"/>
       <c r="CC41" s="18"/>
       <c r="CD41" s="19"/>
@@ -11816,13 +11747,11 @@
       <c r="BP42" s="19"/>
       <c r="BQ42" s="21"/>
       <c r="BS42" s="17"/>
-      <c r="BT42" s="17"/>
+      <c r="BT42" s="1"/>
       <c r="BV42" s="18"/>
       <c r="BW42" s="19"/>
       <c r="BX42" s="20"/>
-      <c r="BY42" s="17"/>
-      <c r="BZ42" s="17"/>
-      <c r="CA42" s="17"/>
+      <c r="BY42" s="1"/>
       <c r="CB42" s="17"/>
       <c r="CC42" s="18"/>
       <c r="CD42" s="19"/>
@@ -12043,13 +11972,11 @@
       <c r="BP43" s="19"/>
       <c r="BQ43" s="21"/>
       <c r="BS43" s="17"/>
-      <c r="BT43" s="17"/>
+      <c r="BT43" s="1"/>
       <c r="BV43" s="18"/>
       <c r="BW43" s="19"/>
       <c r="BX43" s="20"/>
-      <c r="BY43" s="17"/>
-      <c r="BZ43" s="17"/>
-      <c r="CA43" s="17"/>
+      <c r="BY43" s="1"/>
       <c r="CB43" s="17"/>
       <c r="CC43" s="18"/>
       <c r="CD43" s="19"/>
@@ -12265,13 +12192,11 @@
       <c r="BP44" s="19"/>
       <c r="BQ44" s="21"/>
       <c r="BS44" s="17"/>
-      <c r="BT44" s="17"/>
+      <c r="BT44" s="1"/>
       <c r="BV44" s="18"/>
       <c r="BW44" s="19"/>
       <c r="BX44" s="20"/>
-      <c r="BY44" s="17"/>
-      <c r="BZ44" s="17"/>
-      <c r="CA44" s="17"/>
+      <c r="BY44" s="1"/>
       <c r="CB44" s="17"/>
       <c r="CC44" s="18"/>
       <c r="CD44" s="19"/>
@@ -12493,13 +12418,11 @@
       <c r="BP45" s="19"/>
       <c r="BQ45" s="21"/>
       <c r="BS45" s="17"/>
-      <c r="BT45" s="17"/>
+      <c r="BT45" s="1"/>
       <c r="BV45" s="18"/>
       <c r="BW45" s="19"/>
       <c r="BX45" s="20"/>
-      <c r="BY45" s="17"/>
-      <c r="BZ45" s="17"/>
-      <c r="CA45" s="17"/>
+      <c r="BY45" s="1"/>
       <c r="CB45" s="17"/>
       <c r="CC45" s="18"/>
       <c r="CD45" s="19"/>
@@ -12714,13 +12637,11 @@
       <c r="BP46" s="19"/>
       <c r="BQ46" s="21"/>
       <c r="BS46" s="17"/>
-      <c r="BT46" s="17"/>
+      <c r="BT46" s="1"/>
       <c r="BV46" s="18"/>
       <c r="BW46" s="19"/>
       <c r="BX46" s="20"/>
-      <c r="BY46" s="17"/>
-      <c r="BZ46" s="17"/>
-      <c r="CA46" s="17"/>
+      <c r="BY46" s="1"/>
       <c r="CB46" s="17"/>
       <c r="CC46" s="18"/>
       <c r="CD46" s="19"/>
@@ -12947,13 +12868,11 @@
       <c r="BP47" s="19"/>
       <c r="BQ47" s="21"/>
       <c r="BS47" s="17"/>
-      <c r="BT47" s="17"/>
+      <c r="BT47" s="1"/>
       <c r="BV47" s="18"/>
       <c r="BW47" s="19"/>
       <c r="BX47" s="20"/>
-      <c r="BY47" s="17"/>
-      <c r="BZ47" s="17"/>
-      <c r="CA47" s="17"/>
+      <c r="BY47" s="1"/>
       <c r="CB47" s="17"/>
       <c r="CC47" s="18"/>
       <c r="CD47" s="19"/>
@@ -13169,13 +13088,11 @@
       <c r="BP48" s="19"/>
       <c r="BQ48" s="21"/>
       <c r="BS48" s="17"/>
-      <c r="BT48" s="17"/>
+      <c r="BT48" s="1"/>
       <c r="BV48" s="18"/>
       <c r="BW48" s="19"/>
       <c r="BX48" s="20"/>
-      <c r="BY48" s="17"/>
-      <c r="BZ48" s="17"/>
-      <c r="CA48" s="17"/>
+      <c r="BY48" s="1"/>
       <c r="CB48" s="17"/>
       <c r="CC48" s="18"/>
       <c r="CD48" s="19"/>
@@ -13398,13 +13315,11 @@
       <c r="BP49" s="19"/>
       <c r="BQ49" s="21"/>
       <c r="BS49" s="17"/>
-      <c r="BT49" s="17"/>
+      <c r="BT49" s="1"/>
       <c r="BV49" s="18"/>
       <c r="BW49" s="19"/>
       <c r="BX49" s="20"/>
-      <c r="BY49" s="17"/>
-      <c r="BZ49" s="17"/>
-      <c r="CA49" s="17"/>
+      <c r="BY49" s="1"/>
       <c r="CB49" s="17"/>
       <c r="CC49" s="18"/>
       <c r="CD49" s="19"/>
@@ -13619,13 +13534,11 @@
       <c r="BP50" s="19"/>
       <c r="BQ50" s="21"/>
       <c r="BS50" s="17"/>
-      <c r="BT50" s="17"/>
+      <c r="BT50" s="1"/>
       <c r="BV50" s="18"/>
       <c r="BW50" s="19"/>
       <c r="BX50" s="20"/>
-      <c r="BY50" s="17"/>
-      <c r="BZ50" s="17"/>
-      <c r="CA50" s="17"/>
+      <c r="BY50" s="1"/>
       <c r="CB50" s="17"/>
       <c r="CC50" s="18"/>
       <c r="CD50" s="19"/>
@@ -13849,14 +13762,14 @@
       <c r="BP51" s="19"/>
       <c r="BQ51" s="21"/>
       <c r="BS51" s="16"/>
-      <c r="BT51" s="16"/>
-      <c r="BU51" s="71"/>
+      <c r="BT51" s="27"/>
+      <c r="BU51" s="27"/>
       <c r="BV51" s="18"/>
       <c r="BW51" s="19"/>
       <c r="BX51" s="20"/>
-      <c r="BY51" s="16"/>
-      <c r="BZ51" s="16"/>
-      <c r="CA51" s="16"/>
+      <c r="BY51" s="27"/>
+      <c r="BZ51" s="27"/>
+      <c r="CA51" s="71"/>
       <c r="CB51" s="16"/>
       <c r="CC51" s="18"/>
       <c r="CD51" s="19"/>
@@ -14075,9 +13988,9 @@
       <c r="BV52" s="18"/>
       <c r="BW52" s="19"/>
       <c r="BX52" s="20"/>
-      <c r="BY52" s="17"/>
-      <c r="BZ52" s="17"/>
-      <c r="CA52" s="17"/>
+      <c r="BY52" s="70"/>
+      <c r="BZ52" s="70"/>
+      <c r="CA52" s="70"/>
       <c r="CB52" s="17"/>
       <c r="CC52" s="18"/>
       <c r="CD52" s="19"/>
@@ -14299,13 +14212,11 @@
       <c r="BP53" s="19"/>
       <c r="BQ53" s="21"/>
       <c r="BS53" s="17"/>
-      <c r="BT53" s="17"/>
+      <c r="BT53" s="1"/>
       <c r="BV53" s="18"/>
       <c r="BW53" s="19"/>
       <c r="BX53" s="20"/>
-      <c r="BY53" s="17"/>
-      <c r="BZ53" s="17"/>
-      <c r="CA53" s="17"/>
+      <c r="BY53" s="1"/>
       <c r="CB53" s="17"/>
       <c r="CC53" s="18"/>
       <c r="CD53" s="19"/>
@@ -14519,13 +14430,11 @@
       <c r="BP54" s="19"/>
       <c r="BQ54" s="21"/>
       <c r="BS54" s="17"/>
-      <c r="BT54" s="17"/>
+      <c r="BT54" s="1"/>
       <c r="BV54" s="18"/>
       <c r="BW54" s="19"/>
       <c r="BX54" s="20"/>
-      <c r="BY54" s="17"/>
-      <c r="BZ54" s="17"/>
-      <c r="CA54" s="17"/>
+      <c r="BY54" s="1"/>
       <c r="CB54" s="17"/>
       <c r="CC54" s="18"/>
       <c r="CD54" s="19"/>
@@ -14749,13 +14658,11 @@
       <c r="BP55" s="19"/>
       <c r="BQ55" s="21"/>
       <c r="BS55" s="17"/>
-      <c r="BT55" s="17"/>
+      <c r="BT55" s="1"/>
       <c r="BV55" s="18"/>
       <c r="BW55" s="19"/>
       <c r="BX55" s="20"/>
-      <c r="BY55" s="17"/>
-      <c r="BZ55" s="17"/>
-      <c r="CA55" s="17"/>
+      <c r="BY55" s="1"/>
       <c r="CB55" s="17"/>
       <c r="CC55" s="18"/>
       <c r="CD55" s="19"/>
@@ -14969,13 +14876,11 @@
       <c r="BP56" s="19"/>
       <c r="BQ56" s="21"/>
       <c r="BS56" s="17"/>
-      <c r="BT56" s="17"/>
+      <c r="BT56" s="1"/>
       <c r="BV56" s="18"/>
       <c r="BW56" s="19"/>
       <c r="BX56" s="20"/>
-      <c r="BY56" s="17"/>
-      <c r="BZ56" s="17"/>
-      <c r="CA56" s="17"/>
+      <c r="BY56" s="1"/>
       <c r="CB56" s="17"/>
       <c r="CC56" s="18"/>
       <c r="CD56" s="19"/>
@@ -15197,13 +15102,11 @@
       <c r="BP57" s="19"/>
       <c r="BQ57" s="21"/>
       <c r="BS57" s="17"/>
-      <c r="BT57" s="17"/>
+      <c r="BT57" s="1"/>
       <c r="BV57" s="18"/>
       <c r="BW57" s="19"/>
       <c r="BX57" s="20"/>
-      <c r="BY57" s="17"/>
-      <c r="BZ57" s="17"/>
-      <c r="CA57" s="17"/>
+      <c r="BY57" s="1"/>
       <c r="CB57" s="17"/>
       <c r="CC57" s="18"/>
       <c r="CD57" s="19"/>
@@ -15417,13 +15320,11 @@
       <c r="BP58" s="19"/>
       <c r="BQ58" s="21"/>
       <c r="BS58" s="17"/>
-      <c r="BT58" s="17"/>
+      <c r="BT58" s="1"/>
       <c r="BV58" s="18"/>
       <c r="BW58" s="19"/>
       <c r="BX58" s="20"/>
-      <c r="BY58" s="17"/>
-      <c r="BZ58" s="17"/>
-      <c r="CA58" s="17"/>
+      <c r="BY58" s="1"/>
       <c r="CB58" s="17"/>
       <c r="CC58" s="18"/>
       <c r="CD58" s="19"/>
@@ -15645,13 +15546,11 @@
       <c r="BP59" s="19"/>
       <c r="BQ59" s="21"/>
       <c r="BS59" s="17"/>
-      <c r="BT59" s="17"/>
+      <c r="BT59" s="1"/>
       <c r="BV59" s="18"/>
       <c r="BW59" s="19"/>
       <c r="BX59" s="20"/>
-      <c r="BY59" s="17"/>
-      <c r="BZ59" s="17"/>
-      <c r="CA59" s="17"/>
+      <c r="BY59" s="1"/>
       <c r="CB59" s="17"/>
       <c r="CC59" s="18"/>
       <c r="CD59" s="19"/>
@@ -15865,13 +15764,11 @@
       <c r="BP60" s="19"/>
       <c r="BQ60" s="21"/>
       <c r="BS60" s="17"/>
-      <c r="BT60" s="17"/>
+      <c r="BT60" s="1"/>
       <c r="BV60" s="18"/>
       <c r="BW60" s="19"/>
       <c r="BX60" s="20"/>
-      <c r="BY60" s="17"/>
-      <c r="BZ60" s="17"/>
-      <c r="CA60" s="17"/>
+      <c r="BY60" s="1"/>
       <c r="CB60" s="17"/>
       <c r="CC60" s="18"/>
       <c r="CD60" s="19"/>
@@ -16093,13 +15990,11 @@
       <c r="BP61" s="19"/>
       <c r="BQ61" s="21"/>
       <c r="BS61" s="17"/>
-      <c r="BT61" s="17"/>
+      <c r="BT61" s="1"/>
       <c r="BV61" s="18"/>
       <c r="BW61" s="19"/>
       <c r="BX61" s="20"/>
-      <c r="BY61" s="17"/>
-      <c r="BZ61" s="17"/>
-      <c r="CA61" s="17"/>
+      <c r="BY61" s="1"/>
       <c r="CB61" s="17"/>
       <c r="CC61" s="18"/>
       <c r="CD61" s="19"/>
@@ -16313,13 +16208,11 @@
       <c r="BP62" s="19"/>
       <c r="BQ62" s="21"/>
       <c r="BS62" s="17"/>
-      <c r="BT62" s="17"/>
+      <c r="BT62" s="1"/>
       <c r="BV62" s="18"/>
       <c r="BW62" s="19"/>
       <c r="BX62" s="20"/>
-      <c r="BY62" s="17"/>
-      <c r="BZ62" s="17"/>
-      <c r="CA62" s="17"/>
+      <c r="BY62" s="1"/>
       <c r="CB62" s="17"/>
       <c r="CC62" s="18"/>
       <c r="CD62" s="19"/>
@@ -16541,13 +16434,11 @@
       <c r="BP63" s="19"/>
       <c r="BQ63" s="21"/>
       <c r="BS63" s="17"/>
-      <c r="BT63" s="17"/>
+      <c r="BT63" s="1"/>
       <c r="BV63" s="18"/>
       <c r="BW63" s="19"/>
       <c r="BX63" s="20"/>
-      <c r="BY63" s="17"/>
-      <c r="BZ63" s="17"/>
-      <c r="CA63" s="17"/>
+      <c r="BY63" s="1"/>
       <c r="CB63" s="17"/>
       <c r="CC63" s="18"/>
       <c r="CD63" s="19"/>
@@ -16761,13 +16652,11 @@
       <c r="BP64" s="19"/>
       <c r="BQ64" s="21"/>
       <c r="BS64" s="17"/>
-      <c r="BT64" s="17"/>
+      <c r="BT64" s="1"/>
       <c r="BV64" s="18"/>
       <c r="BW64" s="19"/>
       <c r="BX64" s="20"/>
-      <c r="BY64" s="17"/>
-      <c r="BZ64" s="17"/>
-      <c r="CA64" s="17"/>
+      <c r="BY64" s="1"/>
       <c r="CB64" s="17"/>
       <c r="CC64" s="18"/>
       <c r="CD64" s="19"/>
@@ -16989,13 +16878,11 @@
       <c r="BP65" s="19"/>
       <c r="BQ65" s="21"/>
       <c r="BS65" s="17"/>
-      <c r="BT65" s="17"/>
+      <c r="BT65" s="1"/>
       <c r="BV65" s="18"/>
       <c r="BW65" s="19"/>
       <c r="BX65" s="20"/>
-      <c r="BY65" s="17"/>
-      <c r="BZ65" s="17"/>
-      <c r="CA65" s="17"/>
+      <c r="BY65" s="1"/>
       <c r="CB65" s="17"/>
       <c r="CC65" s="18"/>
       <c r="CD65" s="19"/>
@@ -17209,13 +17096,11 @@
       <c r="BP66" s="19"/>
       <c r="BQ66" s="21"/>
       <c r="BS66" s="17"/>
-      <c r="BT66" s="17"/>
+      <c r="BT66" s="1"/>
       <c r="BV66" s="18"/>
       <c r="BW66" s="19"/>
       <c r="BX66" s="20"/>
-      <c r="BY66" s="17"/>
-      <c r="BZ66" s="17"/>
-      <c r="CA66" s="17"/>
+      <c r="BY66" s="1"/>
       <c r="CB66" s="17"/>
       <c r="CC66" s="18"/>
       <c r="CD66" s="19"/>
@@ -17439,13 +17324,11 @@
       <c r="BP67" s="19"/>
       <c r="BQ67" s="21"/>
       <c r="BS67" s="17"/>
-      <c r="BT67" s="17"/>
+      <c r="BT67" s="1"/>
       <c r="BV67" s="18"/>
       <c r="BW67" s="19"/>
       <c r="BX67" s="20"/>
-      <c r="BY67" s="17"/>
-      <c r="BZ67" s="17"/>
-      <c r="CA67" s="17"/>
+      <c r="BY67" s="1"/>
       <c r="CB67" s="17"/>
       <c r="CC67" s="18"/>
       <c r="CD67" s="19"/>
@@ -17660,13 +17543,11 @@
       <c r="BP68" s="19"/>
       <c r="BQ68" s="21"/>
       <c r="BS68" s="17"/>
-      <c r="BT68" s="17"/>
+      <c r="BT68" s="1"/>
       <c r="BV68" s="18"/>
       <c r="BW68" s="19"/>
       <c r="BX68" s="20"/>
-      <c r="BY68" s="17"/>
-      <c r="BZ68" s="17"/>
-      <c r="CA68" s="17"/>
+      <c r="BY68" s="1"/>
       <c r="CB68" s="17"/>
       <c r="CC68" s="18"/>
       <c r="CD68" s="19"/>
@@ -17897,14 +17778,14 @@
       <c r="BQ69" s="21"/>
       <c r="BR69" s="38"/>
       <c r="BS69" s="39"/>
-      <c r="BT69" s="39"/>
-      <c r="BU69" s="68"/>
+      <c r="BT69" s="38"/>
+      <c r="BU69" s="38"/>
       <c r="BV69" s="18"/>
       <c r="BW69" s="19"/>
       <c r="BX69" s="20"/>
-      <c r="BY69" s="39"/>
-      <c r="BZ69" s="39"/>
-      <c r="CA69" s="39"/>
+      <c r="BY69" s="38"/>
+      <c r="BZ69" s="38"/>
+      <c r="CA69" s="68"/>
       <c r="CB69" s="39"/>
       <c r="CC69" s="18"/>
       <c r="CD69" s="19"/>
@@ -18126,9 +18007,7 @@
       <c r="BV70" s="18"/>
       <c r="BW70" s="19"/>
       <c r="BX70" s="20"/>
-      <c r="BY70" s="17"/>
-      <c r="BZ70" s="17"/>
-      <c r="CA70" s="17"/>
+      <c r="BY70" s="1"/>
       <c r="CB70" s="17"/>
       <c r="CC70" s="18"/>
       <c r="CD70" s="19"/>
@@ -18350,13 +18229,11 @@
       <c r="BP71" s="19"/>
       <c r="BQ71" s="21"/>
       <c r="BS71" s="17"/>
-      <c r="BT71" s="17"/>
+      <c r="BT71" s="1"/>
       <c r="BV71" s="18"/>
       <c r="BW71" s="19"/>
       <c r="BX71" s="20"/>
-      <c r="BY71" s="17"/>
-      <c r="BZ71" s="17"/>
-      <c r="CA71" s="17"/>
+      <c r="BY71" s="1"/>
       <c r="CB71" s="17"/>
       <c r="CC71" s="18"/>
       <c r="CD71" s="19"/>
@@ -18570,13 +18447,11 @@
       <c r="BP72" s="19"/>
       <c r="BQ72" s="21"/>
       <c r="BS72" s="17"/>
-      <c r="BT72" s="17"/>
+      <c r="BT72" s="1"/>
       <c r="BV72" s="18"/>
       <c r="BW72" s="19"/>
       <c r="BX72" s="20"/>
-      <c r="BY72" s="17"/>
-      <c r="BZ72" s="17"/>
-      <c r="CA72" s="17"/>
+      <c r="BY72" s="1"/>
       <c r="CB72" s="17"/>
       <c r="CC72" s="18"/>
       <c r="CD72" s="19"/>
@@ -18798,13 +18673,11 @@
       <c r="BP73" s="19"/>
       <c r="BQ73" s="21"/>
       <c r="BS73" s="17"/>
-      <c r="BT73" s="17"/>
+      <c r="BT73" s="1"/>
       <c r="BV73" s="18"/>
       <c r="BW73" s="19"/>
       <c r="BX73" s="20"/>
-      <c r="BY73" s="17"/>
-      <c r="BZ73" s="17"/>
-      <c r="CA73" s="17"/>
+      <c r="BY73" s="1"/>
       <c r="CB73" s="17"/>
       <c r="CC73" s="18"/>
       <c r="CD73" s="19"/>
@@ -19018,13 +18891,11 @@
       <c r="BP74" s="19"/>
       <c r="BQ74" s="21"/>
       <c r="BS74" s="17"/>
-      <c r="BT74" s="17"/>
+      <c r="BT74" s="1"/>
       <c r="BV74" s="18"/>
       <c r="BW74" s="19"/>
       <c r="BX74" s="20"/>
-      <c r="BY74" s="17"/>
-      <c r="BZ74" s="17"/>
-      <c r="CA74" s="17"/>
+      <c r="BY74" s="1"/>
       <c r="CB74" s="17"/>
       <c r="CC74" s="18"/>
       <c r="CD74" s="19"/>
@@ -19246,13 +19117,11 @@
       <c r="BP75" s="19"/>
       <c r="BQ75" s="21"/>
       <c r="BS75" s="17"/>
-      <c r="BT75" s="17"/>
+      <c r="BT75" s="1"/>
       <c r="BV75" s="18"/>
       <c r="BW75" s="19"/>
       <c r="BX75" s="20"/>
-      <c r="BY75" s="17"/>
-      <c r="BZ75" s="17"/>
-      <c r="CA75" s="17"/>
+      <c r="BY75" s="1"/>
       <c r="CB75" s="17"/>
       <c r="CC75" s="18"/>
       <c r="CD75" s="19"/>
@@ -19466,13 +19335,11 @@
       <c r="BP76" s="19"/>
       <c r="BQ76" s="21"/>
       <c r="BS76" s="17"/>
-      <c r="BT76" s="17"/>
+      <c r="BT76" s="1"/>
       <c r="BV76" s="18"/>
       <c r="BW76" s="19"/>
       <c r="BX76" s="20"/>
-      <c r="BY76" s="17"/>
-      <c r="BZ76" s="17"/>
-      <c r="CA76" s="17"/>
+      <c r="BY76" s="1"/>
       <c r="CB76" s="17"/>
       <c r="CC76" s="18"/>
       <c r="CD76" s="19"/>
@@ -19694,13 +19561,11 @@
       <c r="BP77" s="19"/>
       <c r="BQ77" s="21"/>
       <c r="BS77" s="17"/>
-      <c r="BT77" s="17"/>
+      <c r="BT77" s="1"/>
       <c r="BV77" s="18"/>
       <c r="BW77" s="19"/>
       <c r="BX77" s="20"/>
-      <c r="BY77" s="17"/>
-      <c r="BZ77" s="17"/>
-      <c r="CA77" s="17"/>
+      <c r="BY77" s="1"/>
       <c r="CB77" s="17"/>
       <c r="CC77" s="18"/>
       <c r="CD77" s="19"/>
@@ -19914,13 +19779,11 @@
       <c r="BP78" s="19"/>
       <c r="BQ78" s="21"/>
       <c r="BS78" s="17"/>
-      <c r="BT78" s="17"/>
+      <c r="BT78" s="1"/>
       <c r="BV78" s="18"/>
       <c r="BW78" s="19"/>
       <c r="BX78" s="20"/>
-      <c r="BY78" s="17"/>
-      <c r="BZ78" s="17"/>
-      <c r="CA78" s="17"/>
+      <c r="BY78" s="1"/>
       <c r="CB78" s="17"/>
       <c r="CC78" s="18"/>
       <c r="CD78" s="19"/>
@@ -20144,13 +20007,11 @@
       <c r="BP79" s="19"/>
       <c r="BQ79" s="21"/>
       <c r="BS79" s="17"/>
-      <c r="BT79" s="17"/>
+      <c r="BT79" s="1"/>
       <c r="BV79" s="18"/>
       <c r="BW79" s="19"/>
       <c r="BX79" s="20"/>
-      <c r="BY79" s="17"/>
-      <c r="BZ79" s="17"/>
-      <c r="CA79" s="17"/>
+      <c r="BY79" s="1"/>
       <c r="CB79" s="17"/>
       <c r="CC79" s="18"/>
       <c r="CD79" s="19"/>
@@ -20364,13 +20225,11 @@
       <c r="BP80" s="19"/>
       <c r="BQ80" s="21"/>
       <c r="BS80" s="17"/>
-      <c r="BT80" s="17"/>
+      <c r="BT80" s="1"/>
       <c r="BV80" s="18"/>
       <c r="BW80" s="19"/>
       <c r="BX80" s="20"/>
-      <c r="BY80" s="17"/>
-      <c r="BZ80" s="17"/>
-      <c r="CA80" s="17"/>
+      <c r="BY80" s="1"/>
       <c r="CB80" s="17"/>
       <c r="CC80" s="18"/>
       <c r="CD80" s="19"/>
@@ -20592,13 +20451,11 @@
       <c r="BP81" s="19"/>
       <c r="BQ81" s="21"/>
       <c r="BS81" s="17"/>
-      <c r="BT81" s="17"/>
+      <c r="BT81" s="1"/>
       <c r="BV81" s="18"/>
       <c r="BW81" s="19"/>
       <c r="BX81" s="20"/>
-      <c r="BY81" s="17"/>
-      <c r="BZ81" s="17"/>
-      <c r="CA81" s="17"/>
+      <c r="BY81" s="1"/>
       <c r="CB81" s="17"/>
       <c r="CC81" s="18"/>
       <c r="CD81" s="19"/>
@@ -20812,13 +20669,11 @@
       <c r="BP82" s="19"/>
       <c r="BQ82" s="21"/>
       <c r="BS82" s="17"/>
-      <c r="BT82" s="17"/>
+      <c r="BT82" s="1"/>
       <c r="BV82" s="18"/>
       <c r="BW82" s="19"/>
       <c r="BX82" s="20"/>
-      <c r="BY82" s="17"/>
-      <c r="BZ82" s="17"/>
-      <c r="CA82" s="17"/>
+      <c r="BY82" s="1"/>
       <c r="CB82" s="17"/>
       <c r="CC82" s="18"/>
       <c r="CD82" s="19"/>
@@ -21040,13 +20895,11 @@
       <c r="BP83" s="19"/>
       <c r="BQ83" s="21"/>
       <c r="BS83" s="17"/>
-      <c r="BT83" s="17"/>
+      <c r="BT83" s="1"/>
       <c r="BV83" s="18"/>
       <c r="BW83" s="19"/>
       <c r="BX83" s="20"/>
-      <c r="BY83" s="17"/>
-      <c r="BZ83" s="17"/>
-      <c r="CA83" s="17"/>
+      <c r="BY83" s="1"/>
       <c r="CB83" s="17"/>
       <c r="CC83" s="18"/>
       <c r="CD83" s="19"/>
@@ -21260,13 +21113,11 @@
       <c r="BP84" s="19"/>
       <c r="BQ84" s="21"/>
       <c r="BS84" s="17"/>
-      <c r="BT84" s="17"/>
+      <c r="BT84" s="1"/>
       <c r="BV84" s="18"/>
       <c r="BW84" s="19"/>
       <c r="BX84" s="20"/>
-      <c r="BY84" s="17"/>
-      <c r="BZ84" s="17"/>
-      <c r="CA84" s="17"/>
+      <c r="BY84" s="1"/>
       <c r="CB84" s="17"/>
       <c r="CC84" s="18"/>
       <c r="CD84" s="19"/>
@@ -21486,13 +21337,11 @@
       <c r="BP85" s="19"/>
       <c r="BQ85" s="21"/>
       <c r="BS85" s="17"/>
-      <c r="BT85" s="17"/>
+      <c r="BT85" s="1"/>
       <c r="BV85" s="18"/>
       <c r="BW85" s="19"/>
       <c r="BX85" s="20"/>
-      <c r="BY85" s="17"/>
-      <c r="BZ85" s="17"/>
-      <c r="CA85" s="17"/>
+      <c r="BY85" s="1"/>
       <c r="CB85" s="17"/>
       <c r="CC85" s="18"/>
       <c r="CD85" s="19"/>
@@ -21706,13 +21555,11 @@
       <c r="BP86" s="19"/>
       <c r="BQ86" s="21"/>
       <c r="BS86" s="17"/>
-      <c r="BT86" s="17"/>
+      <c r="BT86" s="1"/>
       <c r="BV86" s="18"/>
       <c r="BW86" s="19"/>
       <c r="BX86" s="20"/>
-      <c r="BY86" s="17"/>
-      <c r="BZ86" s="17"/>
-      <c r="CA86" s="17"/>
+      <c r="BY86" s="1"/>
       <c r="CB86" s="17"/>
       <c r="CC86" s="18"/>
       <c r="CD86" s="19"/>

</xml_diff>